<commit_message>
chore: refresh daily snapshot (2026-07-24)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -433,16 +433,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN4"/>
+  <dimension ref="A1:AN21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -450,27 +450,27 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="15" customWidth="1" min="28" max="28"/>
     <col width="13" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
     <col width="22" customWidth="1" min="32" max="32"/>
-    <col width="19" customWidth="1" min="33" max="33"/>
-    <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="15" customWidth="1" min="38" max="38"/>
@@ -707,46 +707,46 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>310.78</v>
+        <v>321.66</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1467473111741109</v>
+        <v>0.1868934297968483</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.007916746472578784</v>
+        <v>-0.03979223260395826</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>313.26</v>
+        <v>334.99</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>195.07</v>
+        <v>201.5</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4564536262656</v>
+        <v>4724335050752</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.5792</v>
+        <v>39.51597</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.346233</v>
+        <v>33.362896</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.111013</v>
+        <v>10.464988</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>42.80716</v>
+        <v>44.305786</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.723816513761468</v>
+        <v>1.812659174311927</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.64035001474781</v>
+        <v>29.63281224396159</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.14918504626253</v>
+        <v>10.50088056711092</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02214699162214073</v>
+        <v>0.02139787827959171</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.166</v>
@@ -787,16 +787,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.0035</v>
+        <v>0.0033</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.6394318133594094</v>
+        <v>0.4599422398417723</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2145492765041057</v>
+        <v>0.3125485356312931</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>13325937518.85484</v>
+        <v>17981600099.16656</v>
       </c>
       <c r="AL2" s="7" t="inlineStr"/>
       <c r="AM2" s="2" t="inlineStr">
@@ -806,130 +806,146 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28 19:03 UTC</t>
+          <t>2026-07-24 06:39 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Banks - Diversified</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>296.37</v>
+        <v>381.58</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>-0.08943716973006643</v>
+        <v>-0.1931746140520755</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1212157153446998</v>
+        <v>-0.3130254748402197</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>337.25</v>
+        <v>555.45</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>260.31</v>
+        <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>794126778368</v>
+        <v>2834542100480</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>14.187171</v>
+        <v>23.252893</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>12.583783</v>
+        <v>19.690578</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>4.5755434</v>
+        <v>8.906008999999999</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>2.3085551</v>
+        <v>6.841171</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.824835523255814</v>
-      </c>
-      <c r="Q3" s="6" t="inlineStr"/>
+        <v>0.993713376068376</v>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>15.62286094549101</v>
+      </c>
       <c r="R3" s="6" t="n">
-        <v>3.231340177534628</v>
-      </c>
-      <c r="S3" s="4" t="inlineStr"/>
+        <v>9.0543217637619</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.0130572240199687</v>
+      </c>
       <c r="T3" s="4" t="n">
-        <v>0.127</v>
+        <v>0.183</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.172</v>
+        <v>0.234</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.127</v>
+        <v>0.183</v>
       </c>
       <c r="W3" s="4" t="n">
-        <v>0.01272</v>
+        <v>0.14814</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>0.16465001</v>
+        <v>0.34013999</v>
       </c>
       <c r="Y3" s="4" t="n">
-        <v>0</v>
+        <v>0.68309</v>
       </c>
       <c r="Z3" s="4" t="n">
-        <v>0.43741</v>
-      </c>
-      <c r="AA3" s="5" t="inlineStr"/>
-      <c r="AB3" s="6" t="inlineStr"/>
-      <c r="AC3" s="6" t="inlineStr"/>
-      <c r="AD3" s="6" t="inlineStr"/>
+        <v>0.46326</v>
+      </c>
+      <c r="AA3" s="5" t="n">
+        <v>37011251200</v>
+      </c>
+      <c r="AB3" s="6" t="n">
+        <v>1.283</v>
+      </c>
+      <c r="AC3" s="6" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="AD3" s="6" t="n">
+        <v>0.30271</v>
+      </c>
       <c r="AE3" s="6" t="inlineStr"/>
-      <c r="AF3" s="6" t="inlineStr"/>
-      <c r="AG3" s="6" t="inlineStr"/>
+      <c r="AF3" s="6" t="n">
+        <v>0.2559078754085186</v>
+      </c>
+      <c r="AG3" s="6" t="n">
+        <v>52.83522012578617</v>
+      </c>
       <c r="AH3" s="4" t="n">
-        <v>0.02</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>1.002591499381793</v>
+        <v>0.4496216130806211</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.2240720916490365</v>
+        <v>0.371636062116977</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>2448255663.165373</v>
+        <v>16130696043.10872</v>
       </c>
       <c r="AL3" s="7" t="inlineStr"/>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>free_cash_flow,current_ratio,quick_ratio,debt_equity,ev_ebitda,fcf_yield,debt_assets,net_debt_ebitda,interest_coverage</t>
+          <t>debt_assets</t>
         </is>
       </c>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28 19:03 UTC</t>
+          <t>2026-07-24 06:39 UTC</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -939,112 +955,112 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Costco</t>
+          <t>Alphabet</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Discount Stores</t>
+          <t>Internet Content &amp; Information</t>
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>997.8099999999999</v>
+        <v>317.69</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1677121123464014</v>
+        <v>0.008059673656062083</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.0900045599635203</v>
+        <v>-0.2225104622990137</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1096.5</v>
+        <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>844.0599999999999</v>
+        <v>187.82</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>442680934400</v>
+        <v>3885328236544</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>51.780487</v>
+        <v>17.153887</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>44.260693</v>
+        <v>21.51217</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>1.5464025</v>
+        <v>8.714117</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>26.766726</v>
+        <v>8.039935</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>1.138032681318681</v>
+        <v>0.05832671540292419</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>32.93956277329332</v>
+        <v>21.83006209362248</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>1.548797377323902</v>
+        <v>8.463649879655318</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.0151133122032192</v>
+        <v>0.006568685734181722</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>0.215</v>
+        <v>0.242</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>0.455</v>
+        <v>2.941</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.215</v>
+        <v>0.242</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>0.08717999999999999</v>
+        <v>0.12958999</v>
       </c>
       <c r="X4" s="4" t="n">
-        <v>0.29650998</v>
+        <v>0.48676</v>
       </c>
       <c r="Y4" s="4" t="n">
-        <v>0.12926</v>
+        <v>0.60897</v>
       </c>
       <c r="Z4" s="4" t="n">
-        <v>0.036730003</v>
+        <v>0.34033</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>6690375168</v>
+        <v>25521500160</v>
       </c>
       <c r="AB4" s="6" t="n">
-        <v>1.058</v>
+        <v>2.724</v>
       </c>
       <c r="AC4" s="6" t="n">
-        <v>0.54</v>
+        <v>2.471</v>
       </c>
       <c r="AD4" s="6" t="n">
-        <v>0.6025699999999999</v>
+        <v>0.17605</v>
       </c>
       <c r="AE4" s="6" t="inlineStr"/>
       <c r="AF4" s="6" t="n">
-        <v>-0.06671618789593939</v>
+        <v>-0.7504005841429527</v>
       </c>
       <c r="AG4" s="6" t="n">
-        <v>71.24675324675324</v>
+        <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.0059</v>
+        <v>0.0026</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>-0.02628485360981389</v>
+        <v>0.8744388338736102</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.2163755304624655</v>
+        <v>0.3669144662079357</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>1922268813.16731</v>
+        <v>12111922489.69289</v>
       </c>
       <c r="AL4" s="7" t="inlineStr"/>
       <c r="AM4" s="2" t="inlineStr">
@@ -1054,7 +1070,2215 @@
       </c>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28 19:03 UTC</t>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Internet Retail</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>233.66</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0.03161147902869765</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>-0.1611860999425617</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>278.56</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>2513506402304</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>29.317442</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>23.585154</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>3.383936</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>5.6861267</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>0.3919444117647059</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>16.7197527593819</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>3.508402696274227</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.003901571429860206</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <v>0.166</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>0.06845</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>0.24285</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>0.50604</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>0.1314</v>
+      </c>
+      <c r="AA5" s="5" t="n">
+        <v>9806624768</v>
+      </c>
+      <c r="AB5" s="6" t="n">
+        <v>1.177</v>
+      </c>
+      <c r="AC5" s="6" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="AD5" s="6" t="n">
+        <v>0.5329999999999999</v>
+      </c>
+      <c r="AE5" s="6" t="inlineStr"/>
+      <c r="AF5" s="6" t="n">
+        <v>0.5931632502890781</v>
+      </c>
+      <c r="AG5" s="6" t="n">
+        <v>43.79287598944591</v>
+      </c>
+      <c r="AH5" s="4" t="inlineStr"/>
+      <c r="AI5" s="6" t="n">
+        <v>0.9068827163075686</v>
+      </c>
+      <c r="AJ5" s="4" t="n">
+        <v>0.3289000957718534</v>
+      </c>
+      <c r="AK5" s="5" t="n">
+        <v>12958042715.31504</v>
+      </c>
+      <c r="AL5" s="7" t="inlineStr"/>
+      <c r="AM5" s="2" t="inlineStr">
+        <is>
+          <t>dividend_yield,debt_assets</t>
+        </is>
+      </c>
+      <c r="AN5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>208.76</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0.105427552306093</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>-0.1174431385812125</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>236.54</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>164.07</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>5056375554048</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>32.466564</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>16.22189</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>19.946962</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>25.86865</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>0.1513592727272727</v>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>30.27921378895412</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>19.77046048042178</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.009163851167444382</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>2.145</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>0.52727</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>1.14288</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <v>0.74144995</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>0.65596</v>
+      </c>
+      <c r="AA6" s="5" t="n">
+        <v>46335873024</v>
+      </c>
+      <c r="AB6" s="6" t="n">
+        <v>3.441</v>
+      </c>
+      <c r="AC6" s="6" t="n">
+        <v>2.139</v>
+      </c>
+      <c r="AD6" s="6" t="n">
+        <v>0.06555</v>
+      </c>
+      <c r="AE6" s="6" t="inlineStr"/>
+      <c r="AF6" s="6" t="n">
+        <v>-0.2438343463332097</v>
+      </c>
+      <c r="AG6" s="6" t="n">
+        <v>547.1389961389962</v>
+      </c>
+      <c r="AH6" s="4" t="n">
+        <v>0.004699999999999999</v>
+      </c>
+      <c r="AI6" s="6" t="n">
+        <v>1.316719271600794</v>
+      </c>
+      <c r="AJ6" s="4" t="n">
+        <v>0.4071538373602223</v>
+      </c>
+      <c r="AK6" s="5" t="n">
+        <v>28367843822.38398</v>
+      </c>
+      <c r="AL6" s="7" t="inlineStr"/>
+      <c r="AM6" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Internet Content &amp; Information</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>606.1</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>-0.06812622034423332</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>-0.2388069073783359</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>796.25</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>520.26</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>1538538340352</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>22.828625</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>16.375778</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>7.157224</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>6.3126864</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>0.3658433493589743</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>14.12638918429391</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>7.183224164081614</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0.01661203286370658</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="V7" s="4" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0.16395001</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>0.32930002</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <v>0.81941</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <v>0.40617</v>
+      </c>
+      <c r="AA7" s="5" t="n">
+        <v>25558249472</v>
+      </c>
+      <c r="AB7" s="6" t="n">
+        <v>2.348</v>
+      </c>
+      <c r="AC7" s="6" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="AD7" s="6" t="n">
+        <v>0.35608</v>
+      </c>
+      <c r="AE7" s="6" t="inlineStr"/>
+      <c r="AF7" s="6" t="n">
+        <v>0.05113075048665012</v>
+      </c>
+      <c r="AG7" s="6" t="n">
+        <v>74.76137339055794</v>
+      </c>
+      <c r="AH7" s="4" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="AI7" s="6" t="n">
+        <v>0.9199131799225191</v>
+      </c>
+      <c r="AJ7" s="4" t="n">
+        <v>0.4905344218933463</v>
+      </c>
+      <c r="AK7" s="5" t="n">
+        <v>11366666189.57662</v>
+      </c>
+      <c r="AL7" s="7" t="inlineStr"/>
+      <c r="AM7" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Auto Manufacturers</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>319.69</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>-0.2702307972355772</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>-0.3591203415993425</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>498.83</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>297.82</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>1262630862848</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>343.7527</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>142.47514</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>12.185322</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>14.599717</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>-114.5842333333333</v>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>93.1023217330783</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>9.663435056784815</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0.003727930265685772</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>0.019299999</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>0.046669997</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <v>0.18852</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>0.014099999</v>
+      </c>
+      <c r="AA8" s="5" t="n">
+        <v>4706999808</v>
+      </c>
+      <c r="AB8" s="6" t="n">
+        <v>1.941</v>
+      </c>
+      <c r="AC8" s="6" t="n">
+        <v>1.344</v>
+      </c>
+      <c r="AD8" s="6" t="n">
+        <v>0.10674</v>
+      </c>
+      <c r="AE8" s="6" t="inlineStr"/>
+      <c r="AF8" s="6" t="n">
+        <v>-3.178242737978831</v>
+      </c>
+      <c r="AG8" s="6" t="n">
+        <v>16.61538461538462</v>
+      </c>
+      <c r="AH8" s="4" t="inlineStr"/>
+      <c r="AI8" s="6" t="n">
+        <v>1.595895714168135</v>
+      </c>
+      <c r="AJ8" s="4" t="n">
+        <v>0.6431593290231431</v>
+      </c>
+      <c r="AK8" s="5" t="n">
+        <v>17424115184.39555</v>
+      </c>
+      <c r="AL8" s="7" t="inlineStr"/>
+      <c r="AM8" s="2" t="inlineStr">
+        <is>
+          <t>dividend_yield,debt_assets</t>
+        </is>
+      </c>
+      <c r="AN8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Broadcom</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>392.47</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0.1290202103238998</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>-0.2071313131313131</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>495</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>281.61</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>1867207540736</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>66.183815</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>20.167343</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>24.742697</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>21.29517</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>0.7749861241217799</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>45.44450398825666</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>25.34269557782883</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0.01457376777584869</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>0.121190004</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>0.37280998</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>0.76284</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>0.48988</v>
+      </c>
+      <c r="AA9" s="5" t="n">
+        <v>27212249088</v>
+      </c>
+      <c r="AB9" s="6" t="n">
+        <v>2.238</v>
+      </c>
+      <c r="AC9" s="6" t="n">
+        <v>1.929</v>
+      </c>
+      <c r="AD9" s="6" t="n">
+        <v>0.7401800000000001</v>
+      </c>
+      <c r="AE9" s="6" t="inlineStr"/>
+      <c r="AF9" s="6" t="n">
+        <v>1.075919658289028</v>
+      </c>
+      <c r="AG9" s="6" t="n">
+        <v>8.080685358255451</v>
+      </c>
+      <c r="AH9" s="4" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="AI9" s="6" t="n">
+        <v>1.631561512053793</v>
+      </c>
+      <c r="AJ9" s="4" t="n">
+        <v>0.6060313747835847</v>
+      </c>
+      <c r="AK9" s="5" t="n">
+        <v>10134305394.62331</v>
+      </c>
+      <c r="AL9" s="7" t="inlineStr"/>
+      <c r="AM9" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Costco</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Discount Stores</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>926.0599999999999</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.08374488004681102</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>-0.1554400364797082</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>1096.5</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>844.0599999999999</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>410687995904</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>46.72351</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>40.891914</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>1.3988631</v>
+      </c>
+      <c r="O10" s="6" t="n">
+        <v>24.841997</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>1.02689032967033</v>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>29.66229906042246</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>1.393260319363755</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0.01693347562470663</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="V10" s="4" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>0.086660005</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>0.29152</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <v>0.12876001</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <v>0.036730003</v>
+      </c>
+      <c r="AA10" s="5" t="n">
+        <v>6954375168</v>
+      </c>
+      <c r="AB10" s="6" t="n">
+        <v>1.072</v>
+      </c>
+      <c r="AC10" s="6" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="AD10" s="6" t="n">
+        <v>0.6025699999999999</v>
+      </c>
+      <c r="AE10" s="6" t="inlineStr"/>
+      <c r="AF10" s="6" t="n">
+        <v>-0.06511964203514763</v>
+      </c>
+      <c r="AG10" s="6" t="n">
+        <v>71.24675324675324</v>
+      </c>
+      <c r="AH10" s="4" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="AI10" s="6" t="n">
+        <v>-0.1425853178542787</v>
+      </c>
+      <c r="AJ10" s="4" t="n">
+        <v>0.231877001079597</v>
+      </c>
+      <c r="AK10" s="5" t="n">
+        <v>2356901527.599284</v>
+      </c>
+      <c r="AL10" s="7" t="inlineStr"/>
+      <c r="AM10" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>-0.2428838156129831</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>-0.4563175755662536</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>126.71</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>65.08</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>286853791744</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>21.528124</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>18.066475</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5.930313</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>9.513878999999999</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>1.939470630630631</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>19.98926724521858</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>6.085919119972625</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0.08850345890026402</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="V11" s="4" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>0.16084999</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>0.49541</v>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <v>0.49118</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <v>0.33381</v>
+      </c>
+      <c r="AA11" s="5" t="n">
+        <v>25387552768</v>
+      </c>
+      <c r="AB11" s="6" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="AC11" s="6" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="AD11" s="6" t="n">
+        <v>0.55236</v>
+      </c>
+      <c r="AE11" s="6" t="inlineStr"/>
+      <c r="AF11" s="6" t="n">
+        <v>0.5110874747049546</v>
+      </c>
+      <c r="AG11" s="6" t="n">
+        <v>17.38427322249553</v>
+      </c>
+      <c r="AH11" s="4" t="inlineStr"/>
+      <c r="AI11" s="6" t="n">
+        <v>0.1831983712919999</v>
+      </c>
+      <c r="AJ11" s="4" t="n">
+        <v>0.3579079483744812</v>
+      </c>
+      <c r="AK11" s="5" t="n">
+        <v>3851660663.514303</v>
+      </c>
+      <c r="AL11" s="7" t="inlineStr"/>
+      <c r="AM11" s="2" t="inlineStr">
+        <is>
+          <t>dividend_yield,debt_assets</t>
+        </is>
+      </c>
+      <c r="AN11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>BRK-B</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Berkshire</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Insurance - Diversified</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>490.85</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>-0.01207609143566268</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>-0.05030473057947182</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>516.85</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>455.19</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>1058691678208</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>14.57826</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>22.815746</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>2.8202147</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>0.00097090466</v>
+      </c>
+      <c r="P12" s="6" t="n">
+        <v>0.1218918060200669</v>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>-2.250111889903251</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>-0.7073160310178424</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0.0578338815240697</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>1.196</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>0.053940002</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>0.10499</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="Z12" s="4" t="n">
+        <v>0.14352</v>
+      </c>
+      <c r="AA12" s="5" t="n">
+        <v>61228249088</v>
+      </c>
+      <c r="AB12" s="6" t="n">
+        <v>2.876</v>
+      </c>
+      <c r="AC12" s="6" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AD12" s="6" t="n">
+        <v>0.17669</v>
+      </c>
+      <c r="AE12" s="6" t="inlineStr"/>
+      <c r="AF12" s="6" t="n">
+        <v>-2.275321290807187</v>
+      </c>
+      <c r="AG12" s="6" t="n">
+        <v>17.26731110672716</v>
+      </c>
+      <c r="AH12" s="4" t="inlineStr"/>
+      <c r="AI12" s="6" t="n">
+        <v>0.04410289618060771</v>
+      </c>
+      <c r="AJ12" s="4" t="n">
+        <v>0.1392153685160389</v>
+      </c>
+      <c r="AK12" s="5" t="n">
+        <v>2368413542.784119</v>
+      </c>
+      <c r="AL12" s="7" t="inlineStr"/>
+      <c r="AM12" s="2" t="inlineStr">
+        <is>
+          <t>dividend_yield,debt_assets</t>
+        </is>
+      </c>
+      <c r="AN12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Banks - Diversified</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>349.9</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0.07502761518186629</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>-0.003815055232889275</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>351.24</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>279.1</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>930104213504</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>14.927474</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>14.144849</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>4.9917574</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>2.6306884</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>0.3182830277185501</v>
+      </c>
+      <c r="Q13" s="6" t="inlineStr"/>
+      <c r="R13" s="6" t="n">
+        <v>2.506070797258559</v>
+      </c>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="U13" s="4" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="V13" s="4" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="W13" s="4" t="n">
+        <v>0.0136</v>
+      </c>
+      <c r="X13" s="4" t="n">
+        <v>0.17789</v>
+      </c>
+      <c r="Y13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="4" t="n">
+        <v>0.5039400000000001</v>
+      </c>
+      <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" s="6" t="inlineStr"/>
+      <c r="AC13" s="6" t="inlineStr"/>
+      <c r="AD13" s="6" t="inlineStr"/>
+      <c r="AE13" s="6" t="inlineStr"/>
+      <c r="AF13" s="6" t="inlineStr"/>
+      <c r="AG13" s="6" t="inlineStr"/>
+      <c r="AH13" s="4" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="AI13" s="6" t="n">
+        <v>0.8050957040535519</v>
+      </c>
+      <c r="AJ13" s="4" t="n">
+        <v>0.2262591689166115</v>
+      </c>
+      <c r="AK13" s="5" t="n">
+        <v>3463644324.26239</v>
+      </c>
+      <c r="AL13" s="7" t="inlineStr"/>
+      <c r="AM13" s="2" t="inlineStr">
+        <is>
+          <t>free_cash_flow,current_ratio,quick_ratio,debt_equity,ev_ebitda,fcf_yield,debt_assets,net_debt_ebitda,interest_coverage</t>
+        </is>
+      </c>
+      <c r="AN13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Credit Services</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>351.6</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0.01477715553949777</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>-0.03708166730569085</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>365.14</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>293.89</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>668653125632</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>30.761154</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>23.641808</v>
+      </c>
+      <c r="N14" s="6" t="n">
+        <v>15.540315</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>18.860638</v>
+      </c>
+      <c r="P14" s="6" t="n">
+        <v>0.8665113802816902</v>
+      </c>
+      <c r="Q14" s="6" t="n">
+        <v>22.33220851755459</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>15.64505434218158</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>0.03116675722154534</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="U14" s="4" t="n">
+        <v>0.355</v>
+      </c>
+      <c r="V14" s="4" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>0.19193001</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>0.60349</v>
+      </c>
+      <c r="Y14" s="4" t="n">
+        <v>0.97778</v>
+      </c>
+      <c r="Z14" s="4" t="n">
+        <v>0.6734599999999999</v>
+      </c>
+      <c r="AA14" s="5" t="n">
+        <v>20839749632</v>
+      </c>
+      <c r="AB14" s="6" t="n">
+        <v>1.088</v>
+      </c>
+      <c r="AC14" s="6" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="AD14" s="6" t="n">
+        <v>0.6723300000000001</v>
+      </c>
+      <c r="AE14" s="6" t="inlineStr"/>
+      <c r="AF14" s="6" t="n">
+        <v>0.3338419984642209</v>
+      </c>
+      <c r="AG14" s="6" t="n">
+        <v>42.07640067911715</v>
+      </c>
+      <c r="AH14" s="4" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="AI14" s="6" t="n">
+        <v>0.3920108403130597</v>
+      </c>
+      <c r="AJ14" s="4" t="n">
+        <v>0.2222949867919922</v>
+      </c>
+      <c r="AK14" s="5" t="n">
+        <v>2977335583.475037</v>
+      </c>
+      <c r="AL14" s="7" t="inlineStr"/>
+      <c r="AM14" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Credit Services</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>530.29</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>-0.05831691545124917</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>-0.1187829237083936</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>601.77</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>464.52</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>468555661312</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>30.670326</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>23.25355</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>13.805819</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>69.99603</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>1.446713490566038</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>22.42128042300872</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>14.1223874784219</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>0.03446362087864594</v>
+      </c>
+      <c r="T15" s="4" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="U15" s="4" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="V15" s="4" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>0.25032</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>2.32076</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="4" t="n">
+        <v>0.60836</v>
+      </c>
+      <c r="AA15" s="5" t="n">
+        <v>16148124672</v>
+      </c>
+      <c r="AB15" s="6" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="AC15" s="6" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="AD15" s="6" t="n">
+        <v>2.82059</v>
+      </c>
+      <c r="AE15" s="6" t="inlineStr"/>
+      <c r="AF15" s="6" t="n">
+        <v>0.5024558851763385</v>
+      </c>
+      <c r="AG15" s="6" t="n">
+        <v>26.73130193905817</v>
+      </c>
+      <c r="AH15" s="4" t="n">
+        <v>0.006500000000000001</v>
+      </c>
+      <c r="AI15" s="6" t="n">
+        <v>0.352652463476208</v>
+      </c>
+      <c r="AJ15" s="4" t="n">
+        <v>0.240481329543966</v>
+      </c>
+      <c r="AK15" s="5" t="n">
+        <v>1884717340.607503</v>
+      </c>
+      <c r="AL15" s="7" t="inlineStr"/>
+      <c r="AM15" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>UnitedHealth</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare Plans</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>423.56</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0.2590963367565819</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>-0.08244876738442874</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>461.62</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>234.6</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>384653623296</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>32.456703</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>18.879059</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0.8545409</v>
+      </c>
+      <c r="O16" s="6" t="n">
+        <v>3.671732</v>
+      </c>
+      <c r="P16" s="6" t="n">
+        <v>0.5277512682926829</v>
+      </c>
+      <c r="Q16" s="6" t="n">
+        <v>17.60196910551248</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>0.948708826705284</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>0.05916946638114946</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="U16" s="4" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>0.04382</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>0.14152999</v>
+      </c>
+      <c r="Y16" s="4" t="n">
+        <v>0.19514</v>
+      </c>
+      <c r="Z16" s="4" t="n">
+        <v>0.07132999600000001</v>
+      </c>
+      <c r="AA16" s="5" t="n">
+        <v>22759749632</v>
+      </c>
+      <c r="AB16" s="6" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="AC16" s="6" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="AD16" s="6" t="n">
+        <v>0.69211</v>
+      </c>
+      <c r="AE16" s="6" t="inlineStr"/>
+      <c r="AF16" s="6" t="n">
+        <v>1.725403043054092</v>
+      </c>
+      <c r="AG16" s="6" t="n">
+        <v>4.672413793103448</v>
+      </c>
+      <c r="AH16" s="4" t="n">
+        <v>0.0215</v>
+      </c>
+      <c r="AI16" s="6" t="n">
+        <v>0.5615307959671498</v>
+      </c>
+      <c r="AJ16" s="4" t="n">
+        <v>0.2708821265478612</v>
+      </c>
+      <c r="AK16" s="5" t="n">
+        <v>2644336932.064413</v>
+      </c>
+      <c r="AL16" s="7" t="inlineStr"/>
+      <c r="AM16" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Exxon</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Oil &amp; Gas Integrated</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>156.89</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0.279168349352988</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>-0.11065132362111</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>176.41</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>105.53</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>650300751872</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>26.368069</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>14.627156</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>1.9947386</v>
+      </c>
+      <c r="O17" s="6" t="n">
+        <v>2.5564191</v>
+      </c>
+      <c r="P17" s="6" t="n">
+        <v>-0.6075591935483871</v>
+      </c>
+      <c r="Q17" s="6" t="n">
+        <v>12.42954882933399</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>2.135351631700753</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>0.01788480146535223</v>
+      </c>
+      <c r="T17" s="4" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="U17" s="4" t="n">
+        <v>-0.434</v>
+      </c>
+      <c r="V17" s="4" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="W17" s="4" t="n">
+        <v>0.04221</v>
+      </c>
+      <c r="X17" s="4" t="n">
+        <v>0.09873</v>
+      </c>
+      <c r="Y17" s="4" t="n">
+        <v>0.29768</v>
+      </c>
+      <c r="Z17" s="4" t="n">
+        <v>0.06355</v>
+      </c>
+      <c r="AA17" s="5" t="n">
+        <v>11630499840</v>
+      </c>
+      <c r="AB17" s="6" t="n">
+        <v>1.036</v>
+      </c>
+      <c r="AC17" s="6" t="n">
+        <v>0.744</v>
+      </c>
+      <c r="AD17" s="6" t="n">
+        <v>0.18261</v>
+      </c>
+      <c r="AE17" s="6" t="inlineStr"/>
+      <c r="AF17" s="6" t="n">
+        <v>0.7003767172527701</v>
+      </c>
+      <c r="AG17" s="6" t="n">
+        <v>69.43781094527363</v>
+      </c>
+      <c r="AH17" s="4" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="AI17" s="6" t="n">
+        <v>-0.4280369953194851</v>
+      </c>
+      <c r="AJ17" s="4" t="n">
+        <v>0.2762722761757503</v>
+      </c>
+      <c r="AK17" s="5" t="n">
+        <v>2424122694.036204</v>
+      </c>
+      <c r="AL17" s="7" t="inlineStr"/>
+      <c r="AM17" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN17" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Johnson &amp; Johnson</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Drug Manufacturers - General</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>259.27</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0.2503978411776089</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>-0.03770923802100745</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>269.43</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>164.23</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>624119119872</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>29.664759</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>20.204672</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>6.3731794</v>
+      </c>
+      <c r="O18" s="6" t="n">
+        <v>7.685489</v>
+      </c>
+      <c r="P18" s="6" t="n">
+        <v>-29.664759</v>
+      </c>
+      <c r="Q18" s="6" t="n">
+        <v>18.85921880435592</v>
+      </c>
+      <c r="R18" s="6" t="n">
+        <v>6.709505192474225</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="U18" s="4" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="V18" s="4" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="W18" s="4" t="inlineStr"/>
+      <c r="X18" s="4" t="inlineStr"/>
+      <c r="Y18" s="4" t="n">
+        <v>0.68097</v>
+      </c>
+      <c r="Z18" s="4" t="n">
+        <v>0.28605</v>
+      </c>
+      <c r="AA18" s="5" t="inlineStr"/>
+      <c r="AB18" s="6" t="inlineStr"/>
+      <c r="AC18" s="6" t="inlineStr"/>
+      <c r="AD18" s="6" t="n">
+        <v>0.6773</v>
+      </c>
+      <c r="AE18" s="6" t="inlineStr"/>
+      <c r="AF18" s="6" t="n">
+        <v>0.9453502579809987</v>
+      </c>
+      <c r="AG18" s="6" t="n">
+        <v>34.55406797116375</v>
+      </c>
+      <c r="AH18" s="4" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="AI18" s="6" t="n">
+        <v>-0.1517102526708811</v>
+      </c>
+      <c r="AJ18" s="4" t="n">
+        <v>0.2732817162462441</v>
+      </c>
+      <c r="AK18" s="5" t="n">
+        <v>2201964419.337616</v>
+      </c>
+      <c r="AL18" s="7" t="inlineStr"/>
+      <c r="AM18" s="2" t="inlineStr">
+        <is>
+          <t>roa,roe,free_cash_flow,current_ratio,quick_ratio,fcf_yield,debt_assets</t>
+        </is>
+      </c>
+      <c r="AN18" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Discount Stores</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>-0.03866621189810682</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>-0.1979875702870671</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>135.16</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>95.34999999999999</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>862655741952</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>38.439716</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>32.99587</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>1.1893697</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>9.149224</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>1.981428659793814</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>20.83315079863233</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>1.287895142399991</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>0.007954795465074212</v>
+      </c>
+      <c r="T19" s="4" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="U19" s="4" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="V19" s="4" t="n">
+        <v>0.073</v>
+      </c>
+      <c r="W19" s="4" t="n">
+        <v>0.06834999999999999</v>
+      </c>
+      <c r="X19" s="4" t="n">
+        <v>0.24132</v>
+      </c>
+      <c r="Y19" s="4" t="n">
+        <v>0.24976</v>
+      </c>
+      <c r="Z19" s="4" t="n">
+        <v>0.042150002</v>
+      </c>
+      <c r="AA19" s="5" t="n">
+        <v>6862249984</v>
+      </c>
+      <c r="AB19" s="6" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="AC19" s="6" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="AD19" s="6" t="n">
+        <v>0.74816</v>
+      </c>
+      <c r="AE19" s="6" t="inlineStr"/>
+      <c r="AF19" s="6" t="n">
+        <v>1.445559661076498</v>
+      </c>
+      <c r="AG19" s="6" t="n">
+        <v>11.52840300107181</v>
+      </c>
+      <c r="AH19" s="4" t="n">
+        <v>0.0091</v>
+      </c>
+      <c r="AI19" s="6" t="n">
+        <v>-0.04634012957674574</v>
+      </c>
+      <c r="AJ19" s="4" t="n">
+        <v>0.236724782033911</v>
+      </c>
+      <c r="AK19" s="5" t="n">
+        <v>2592290752.219925</v>
+      </c>
+      <c r="AL19" s="7" t="inlineStr"/>
+      <c r="AM19" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Procter &amp; Gamble</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Household &amp; Personal Products</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>146.97</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0.03653294984938693</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>-0.121255605381166</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>167.25</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>137.62</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>342234202112</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>21.773333</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>20.837557</v>
+      </c>
+      <c r="N20" s="6" t="n">
+        <v>3.9465642</v>
+      </c>
+      <c r="O20" s="6" t="n">
+        <v>6.367575</v>
+      </c>
+      <c r="P20" s="6" t="n">
+        <v>3.754022931034482</v>
+      </c>
+      <c r="Q20" s="6" t="n">
+        <v>14.69288366203535</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>4.242988120338525</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>0.03720770803565897</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="U20" s="4" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="V20" s="4" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="W20" s="4" t="n">
+        <v>0.10925999</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>0.31112</v>
+      </c>
+      <c r="Y20" s="4" t="n">
+        <v>0.50984</v>
+      </c>
+      <c r="Z20" s="4" t="n">
+        <v>0.23047</v>
+      </c>
+      <c r="AA20" s="5" t="n">
+        <v>12733750272</v>
+      </c>
+      <c r="AB20" s="6" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="AC20" s="6" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="AD20" s="6" t="n">
+        <v>0.6765099999999999</v>
+      </c>
+      <c r="AE20" s="6" t="inlineStr"/>
+      <c r="AF20" s="6" t="n">
+        <v>0.9871416480454489</v>
+      </c>
+      <c r="AG20" s="6" t="n">
+        <v>23.2348401323043</v>
+      </c>
+      <c r="AH20" s="4" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="AI20" s="6" t="n">
+        <v>-0.08229183976326422</v>
+      </c>
+      <c r="AJ20" s="4" t="n">
+        <v>0.251698847524099</v>
+      </c>
+      <c r="AK20" s="5" t="n">
+        <v>1333237928.962504</v>
+      </c>
+      <c r="AL20" s="7" t="inlineStr"/>
+      <c r="AM20" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN20" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>HD</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Home Depot</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Home Improvement Retail</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>324.71</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>-0.0610433372191429</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>-0.2391095489162274</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>426.75</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>289.1</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>323773759488</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>23.529709</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>20.178034</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>1.9435132</v>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>23.333572</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>-5.472025348837209</v>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>15.46956454919042</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>2.316460248846156</v>
+      </c>
+      <c r="S21" s="4" t="n">
+        <v>0.03128187371334946</v>
+      </c>
+      <c r="T21" s="4" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="U21" s="4" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="V21" s="4" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="W21" s="4" t="n">
+        <v>0.12519</v>
+      </c>
+      <c r="X21" s="4" t="n">
+        <v>1.2838</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>0.33126998</v>
+      </c>
+      <c r="Z21" s="4" t="n">
+        <v>0.11926</v>
+      </c>
+      <c r="AA21" s="5" t="n">
+        <v>10128249856</v>
+      </c>
+      <c r="AB21" s="6" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="AC21" s="6" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="AD21" s="6" t="n">
+        <v>4.59356</v>
+      </c>
+      <c r="AE21" s="6" t="inlineStr"/>
+      <c r="AF21" s="6" t="n">
+        <v>2.49057963917238</v>
+      </c>
+      <c r="AG21" s="6" t="n">
+        <v>8.712271973466004</v>
+      </c>
+      <c r="AH21" s="4" t="n">
+        <v>0.0281</v>
+      </c>
+      <c r="AI21" s="6" t="n">
+        <v>0.7044542283994155</v>
+      </c>
+      <c r="AJ21" s="4" t="n">
+        <v>0.285531934146076</v>
+      </c>
+      <c r="AK21" s="5" t="n">
+        <v>1564665388.214823</v>
+      </c>
+      <c r="AL21" s="7" t="inlineStr"/>
+      <c r="AM21" s="2" t="inlineStr">
+        <is>
+          <t>debt_assets</t>
+        </is>
+      </c>
+      <c r="AN21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:39 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore last full snapshot (FMP cap hit mid-run); tighten fail-loud guard to 80%
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,34 +442,34 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="23" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
-    <col width="24" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="21" customWidth="1" min="24" max="24"/>
-    <col width="21" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
     <col width="21" customWidth="1" min="30" max="30"/>
-    <col width="22" customWidth="1" min="31" max="31"/>
-    <col width="23" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
-    <col width="23" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="34" max="34"/>
     <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
@@ -722,74 +722,74 @@
         <v>201.5</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4724334930960</v>
+        <v>4724335050752</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>38.80096501809409</v>
+        <v>39.51597</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>36.71372969764761</v>
+        <v>33.362896</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.46498759743223</v>
+        <v>10.464988</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>44.4342672327239</v>
+        <v>44.305786</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.341345188528735</v>
+        <v>1.812659174311927</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>29.76771905146821</v>
+        <v>29.63281224396159</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.57216194098024</v>
+        <v>10.50088056711092</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02734226126803237</v>
+        <v>0.02139787827959171</v>
       </c>
       <c r="T2" s="4" t="n">
-        <v>0.06425511782832749</v>
+        <v>0.166</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.1744369973190349</v>
+        <v>0.218</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1490094408293905</v>
+        <v>0.166</v>
       </c>
       <c r="W2" s="4" t="n">
-        <v>0.3303178273265747</v>
+        <v>0.26229</v>
       </c>
       <c r="X2" s="4" t="n">
-        <v>1.466892449827072</v>
+        <v>1.4147099</v>
       </c>
       <c r="Y2" s="4" t="n">
-        <v>0.4786240535882794</v>
+        <v>0.47862</v>
       </c>
       <c r="Z2" s="4" t="n">
-        <v>0.3264339605087697</v>
+        <v>0.32275</v>
       </c>
       <c r="AA2" s="5" t="n">
-        <v>98767000000</v>
+        <v>101090746368</v>
       </c>
       <c r="AB2" s="6" t="n">
-        <v>1.07035746912159</v>
+        <v>1.07</v>
       </c>
       <c r="AC2" s="6" t="n">
-        <v>1.0202464331073</v>
+        <v>0.906</v>
       </c>
       <c r="AD2" s="6" t="n">
-        <v>0.7954756740006198</v>
+        <v>0.79548</v>
       </c>
       <c r="AE2" s="6" t="n">
-        <v>0.2282810807314825</v>
+        <v>0.2358054843851342</v>
       </c>
       <c r="AF2" s="6" t="n">
-        <v>0.3017675822667964</v>
+        <v>0.1012901775472749</v>
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003264316358888267</v>
+        <v>0.0033</v>
       </c>
       <c r="AI2" s="6" t="n">
         <v>0.4599422398417723</v>
@@ -812,7 +812,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -858,76 +858,76 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>2834540319400</v>
+        <v>2834542100480</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>22.64569732937685</v>
+        <v>23.252893</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>22.7122435289629</v>
+        <v>19.690578</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>8.906003083516351</v>
+        <v>8.906008999999999</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>6.838413966363151</v>
+        <v>6.841171</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.7620922495041578</v>
+        <v>0.993713376068376</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>14.56947595977289</v>
+        <v>15.62286094549101</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>9.199232480920466</v>
+        <v>9.0543217637619</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.02572410048322561</v>
+        <v>0.0130572240199687</v>
       </c>
       <c r="T3" s="4" t="n">
-        <v>0.1493215623240671</v>
+        <v>0.183</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.2317177419354839</v>
+        <v>0.234</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1693591662194205</v>
+        <v>0.183</v>
       </c>
       <c r="W3" s="4" t="n">
-        <v>0.1803672568666202</v>
+        <v>0.14814</v>
       </c>
       <c r="X3" s="4" t="n">
-        <v>0.3313037398539619</v>
+        <v>0.34013999</v>
       </c>
       <c r="Y3" s="4" t="n">
-        <v>0.6830928165442874</v>
+        <v>0.68309</v>
       </c>
       <c r="Z3" s="4" t="n">
-        <v>0.4680164512855316</v>
+        <v>0.46326</v>
       </c>
       <c r="AA3" s="5" t="n">
-        <v>71611000000</v>
+        <v>37011251200</v>
       </c>
       <c r="AB3" s="6" t="n">
-        <v>1.282948317369257</v>
+        <v>1.283</v>
       </c>
       <c r="AC3" s="6" t="n">
-        <v>1.274028435325367</v>
+        <v>1.142</v>
       </c>
       <c r="AD3" s="6" t="n">
-        <v>0.3027075032519482</v>
+        <v>0.30271</v>
       </c>
       <c r="AE3" s="6" t="n">
-        <v>0.1806783938417926</v>
+        <v>0.202635522632362</v>
       </c>
       <c r="AF3" s="6" t="n">
-        <v>0.4644081628590906</v>
+        <v>0.2559078754085186</v>
       </c>
       <c r="AG3" s="6" t="n">
         <v>52.83522012578617</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.009329629435505006</v>
+        <v>0.009300000000000001</v>
       </c>
       <c r="AI3" s="6" t="n">
         <v>0.4496216130806211</v>
@@ -946,7 +946,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -992,76 +992,76 @@
         <v>187.82</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>3844719734449</v>
+        <v>3885328236544</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>15.77408142999007</v>
+        <v>17.153887</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.49850006530282</v>
+        <v>21.51217</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>8.621723695544631</v>
+        <v>8.714117</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.027122142767924</v>
+        <v>8.039935</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.140279823598786</v>
+        <v>0.05832671540292419</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>11.97750585418783</v>
+        <v>21.83006209362248</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>8.749197716363856</v>
+        <v>8.463649879655318</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.0138561465280992</v>
+        <v>0.006568685734181722</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>0.1512636492980362</v>
+        <v>0.242</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>0.3670037002775208</v>
+        <v>2.941</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2154337191230957</v>
+        <v>0.242</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>0.2648693088701202</v>
+        <v>0.12958999</v>
       </c>
       <c r="X4" s="4" t="n">
-        <v>0.5084008289969907</v>
+        <v>0.48676</v>
       </c>
       <c r="Y4" s="4" t="n">
-        <v>0.6090251023694089</v>
+        <v>0.60897</v>
       </c>
       <c r="Z4" s="4" t="n">
-        <v>0.3312059632142873</v>
+        <v>0.34033</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>73266000000</v>
+        <v>25521500160</v>
       </c>
       <c r="AB4" s="6" t="n">
-        <v>2.723981254609035</v>
+        <v>2.724</v>
       </c>
       <c r="AC4" s="6" t="n">
-        <v>2.644757396262023</v>
+        <v>2.471</v>
       </c>
       <c r="AD4" s="6" t="n">
-        <v>0.1760492130901824</v>
+        <v>0.17605</v>
       </c>
       <c r="AE4" s="6" t="n">
-        <v>0.122297265784727</v>
+        <v>0.1894164247137066</v>
       </c>
       <c r="AF4" s="6" t="n">
-        <v>0.1745098099410268</v>
+        <v>-0.7504005841429527</v>
       </c>
       <c r="AG4" s="6" t="n">
-        <v>1110.671328671329</v>
+        <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002675564229280116</v>
+        <v>0.0026</v>
       </c>
       <c r="AI4" s="6" t="n">
         <v>0.8744388338736102</v>
@@ -1080,7 +1080,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Specialty Retail</t>
+          <t>Internet Retail</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -1126,70 +1126,70 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2513503986000</v>
+        <v>2513506402304</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>27.52179034157833</v>
+        <v>29.317442</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>26.41736405221517</v>
+        <v>23.585154</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.38393268764742</v>
+        <v>3.383936</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.680311961150812</v>
+        <v>5.6861267</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.7773046191067392</v>
+        <v>0.3919444117647059</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>13.91214078901283</v>
+        <v>16.7197527593819</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.529430118905296</v>
+        <v>3.508402696274227</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.0009834875988933482</v>
+        <v>0.003901571429860206</v>
       </c>
       <c r="T5" s="4" t="n">
-        <v>0.1237775468329469</v>
+        <v>0.166</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>0.2336039051603904</v>
+        <v>0.748</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1502617677898912</v>
+        <v>0.166</v>
       </c>
       <c r="W5" s="4" t="n">
-        <v>0.09905632588939921</v>
+        <v>0.06845</v>
       </c>
       <c r="X5" s="4" t="n">
-        <v>0.2333561425996781</v>
+        <v>0.24285</v>
       </c>
       <c r="Y5" s="4" t="n">
-        <v>0.5060408521546199</v>
+        <v>0.50604</v>
       </c>
       <c r="Z5" s="4" t="n">
-        <v>0.115003715790494</v>
+        <v>0.1314</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>7695000000</v>
+        <v>9806624768</v>
       </c>
       <c r="AB5" s="6" t="n">
-        <v>1.177153112255255</v>
+        <v>1.177</v>
       </c>
       <c r="AC5" s="6" t="n">
-        <v>1.008604144752625</v>
+        <v>0.974</v>
       </c>
       <c r="AD5" s="6" t="n">
-        <v>0.474952140009142</v>
+        <v>0.5329999999999999</v>
       </c>
       <c r="AE5" s="6" t="n">
-        <v>0.2289778863881828</v>
+        <v>0.2879314324496786</v>
       </c>
       <c r="AF5" s="6" t="n">
-        <v>0.5735148961462125</v>
+        <v>0.5931632502890781</v>
       </c>
       <c r="AG5" s="6" t="n">
         <v>43.79287598944591</v>
@@ -1214,7 +1214,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1260,76 +1260,76 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5056375960000</v>
+        <v>5056375554048</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>31.82317073170731</v>
+        <v>32.466564</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>23.20561132046109</v>
+        <v>16.22189</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>19.94696442871739</v>
+        <v>19.946962</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>25.93667372642909</v>
+        <v>25.86865</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2921776494080731</v>
+        <v>0.1513592727272727</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>26.2007201119345</v>
+        <v>30.27921378895412</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>19.94529573042041</v>
+        <v>19.77046048042178</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02354967291633117</v>
+        <v>0.009163851167444382</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>0.6547353579009478</v>
+        <v>0.852</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.8359387755102039</v>
+        <v>2.145</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8218445613185266</v>
+        <v>0.852</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>0.6151406306604901</v>
+        <v>0.52727</v>
       </c>
       <c r="X6" s="4" t="n">
-        <v>1.116574996283633</v>
+        <v>1.14288</v>
       </c>
       <c r="Y6" s="4" t="n">
-        <v>0.7414543317119739</v>
+        <v>0.74144995</v>
       </c>
       <c r="Z6" s="4" t="n">
-        <v>0.6402002437956377</v>
+        <v>0.65596</v>
       </c>
       <c r="AA6" s="5" t="n">
-        <v>96676000000</v>
+        <v>46335873024</v>
       </c>
       <c r="AB6" s="6" t="n">
-        <v>3.440775681341719</v>
+        <v>3.441</v>
       </c>
       <c r="AC6" s="6" t="n">
-        <v>2.852930453012487</v>
+        <v>2.139</v>
       </c>
       <c r="AD6" s="6" t="n">
-        <v>0.06555347514247419</v>
+        <v>0.06555</v>
       </c>
       <c r="AE6" s="6" t="n">
-        <v>0.04938452407562993</v>
+        <v>0.06196235126182889</v>
       </c>
       <c r="AF6" s="6" t="n">
-        <v>-0.002192050577810022</v>
+        <v>-0.2438343463332097</v>
       </c>
       <c r="AG6" s="6" t="n">
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.0013412531136233</v>
+        <v>0.004699999999999999</v>
       </c>
       <c r="AI6" s="6" t="n">
         <v>1.316719271600794</v>
@@ -1348,7 +1348,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1394,76 +1394,76 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1538538340310</v>
+        <v>1538538340352</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.67739628040057</v>
+        <v>22.828625</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>18.39831176289885</v>
+        <v>16.375778</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>7.157223988825984</v>
+        <v>7.157224</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6.302737595462922</v>
+        <v>6.3126864</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3.478957744513071</v>
+        <v>0.3658433493589743</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.12182821850784</v>
+        <v>14.12638918429391</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.451893304010457</v>
+        <v>7.183224164081614</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.03136288432713188</v>
+        <v>0.01661203286370658</v>
       </c>
       <c r="T7" s="4" t="n">
-        <v>0.2216703849824622</v>
+        <v>0.331</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.4024367816091956</v>
+        <v>0.624</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2604836918782281</v>
+        <v>0.331</v>
       </c>
       <c r="W7" s="4" t="n">
-        <v>0.1785882352941177</v>
+        <v>0.16395001</v>
       </c>
       <c r="X7" s="4" t="n">
-        <v>0.3321506717172906</v>
+        <v>0.32930002</v>
       </c>
       <c r="Y7" s="4" t="n">
-        <v>0.8194061303573174</v>
+        <v>0.81941</v>
       </c>
       <c r="Z7" s="4" t="n">
-        <v>0.412131390053172</v>
+        <v>0.40617</v>
       </c>
       <c r="AA7" s="5" t="n">
-        <v>46109000000</v>
+        <v>25558249472</v>
       </c>
       <c r="AB7" s="6" t="n">
-        <v>2.347763779864394</v>
+        <v>2.348</v>
       </c>
       <c r="AC7" s="6" t="n">
-        <v>2.347763779864394</v>
+        <v>2.11</v>
       </c>
       <c r="AD7" s="6" t="n">
-        <v>0.3560761815652431</v>
+        <v>0.35608</v>
       </c>
       <c r="AE7" s="6" t="n">
-        <v>0.2195294117647059</v>
+        <v>0.2370601699028198</v>
       </c>
       <c r="AF7" s="6" t="n">
-        <v>0.55841774439537</v>
+        <v>0.05113075048665012</v>
       </c>
       <c r="AG7" s="6" t="n">
-        <v>73.76137339055794</v>
+        <v>74.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003464774789638673</v>
+        <v>0.0033</v>
       </c>
       <c r="AI7" s="6" t="n">
         <v>0.9199131799225191</v>
@@ -1482,7 +1482,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Auto - Manufacturers</t>
+          <t>Auto Manufacturers</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
@@ -1528,70 +1528,70 @@
         <v>297.82</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1200666126800</v>
+        <v>1262630862848</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>270.9237288135594</v>
+        <v>343.7527</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>176.3612291057538</v>
+        <v>142.5819</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>11.58731629141374</v>
+        <v>12.185322</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>11.91411879159087</v>
+        <v>14.271238</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.211913344473619</v>
+        <v>-114.5842333333333</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>114.7842373715054</v>
+        <v>93.1023217330783</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>11.53059889402523</v>
+        <v>9.663435056784815</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004799002713066295</v>
+        <v>0.003727930265685772</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>-0.02930699150373628</v>
+        <v>0.255</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.6784259259259258</v>
+        <v>-0.03</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1082503453763168</v>
+        <v>0.255</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>0.02570628315962403</v>
+        <v>0.019299999</v>
       </c>
       <c r="X8" s="4" t="n">
-        <v>0.04585112154644448</v>
+        <v>0.046669997</v>
       </c>
       <c r="Y8" s="4" t="n">
-        <v>0.1885175498701976</v>
+        <v>0.18852</v>
       </c>
       <c r="Z8" s="4" t="n">
-        <v>0.04219303409606346</v>
+        <v>0.014099999</v>
       </c>
       <c r="AA8" s="5" t="n">
-        <v>6220000000</v>
+        <v>4706999808</v>
       </c>
       <c r="AB8" s="6" t="n">
-        <v>1.940945659844742</v>
+        <v>1.941</v>
       </c>
       <c r="AC8" s="6" t="n">
-        <v>1.552745236414961</v>
+        <v>1.344</v>
       </c>
       <c r="AD8" s="6" t="n">
-        <v>0.1075548596559902</v>
+        <v>0.10674</v>
       </c>
       <c r="AE8" s="6" t="n">
-        <v>0.06289892542619374</v>
+        <v>0.06779095342728184</v>
       </c>
       <c r="AF8" s="6" t="n">
-        <v>-0.564607551157652</v>
+        <v>-3.178242737978831</v>
       </c>
       <c r="AG8" s="6" t="n">
         <v>16.61538461538462</v>
@@ -1616,7 +1616,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1646,39 +1646,93 @@
           <t>Semiconductors</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="n">
+        <v>392.47</v>
+      </c>
       <c r="G9" s="4" t="n">
-        <v>0.1290202138355019</v>
+        <v>0.1290202103238998</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.1850198408297649</v>
-      </c>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="6" t="inlineStr"/>
-      <c r="M9" s="6" t="inlineStr"/>
-      <c r="N9" s="6" t="inlineStr"/>
-      <c r="O9" s="6" t="inlineStr"/>
-      <c r="P9" s="6" t="inlineStr"/>
-      <c r="Q9" s="6" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
-      <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
-      <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" s="4" t="inlineStr"/>
-      <c r="W9" s="4" t="inlineStr"/>
-      <c r="X9" s="4" t="inlineStr"/>
-      <c r="Y9" s="4" t="inlineStr"/>
-      <c r="Z9" s="4" t="inlineStr"/>
-      <c r="AA9" s="5" t="inlineStr"/>
-      <c r="AB9" s="6" t="inlineStr"/>
-      <c r="AC9" s="6" t="inlineStr"/>
-      <c r="AD9" s="6" t="inlineStr"/>
-      <c r="AE9" s="6" t="inlineStr"/>
-      <c r="AF9" s="6" t="inlineStr"/>
-      <c r="AG9" s="6" t="inlineStr"/>
-      <c r="AH9" s="4" t="inlineStr"/>
+        <v>-0.2071313131313131</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>495</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>281.61</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>1867207540736</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>66.183815</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>20.167343</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>24.742697</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>21.29517</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>0.7749861241217799</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>45.44450398825666</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>25.34269557782883</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0.01457376777584869</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>0.479</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>0.121190004</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>0.37280998</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <v>0.76284</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <v>0.48988</v>
+      </c>
+      <c r="AA9" s="5" t="n">
+        <v>27212249088</v>
+      </c>
+      <c r="AB9" s="6" t="n">
+        <v>2.238</v>
+      </c>
+      <c r="AC9" s="6" t="n">
+        <v>1.929</v>
+      </c>
+      <c r="AD9" s="6" t="n">
+        <v>0.7401800000000001</v>
+      </c>
+      <c r="AE9" s="6" t="n">
+        <v>0.3793690053070862</v>
+      </c>
+      <c r="AF9" s="6" t="n">
+        <v>1.075919658289028</v>
+      </c>
+      <c r="AG9" s="6" t="n">
+        <v>8.080685358255451</v>
+      </c>
+      <c r="AH9" s="4" t="n">
+        <v>0.0066</v>
+      </c>
       <c r="AI9" s="6" t="n">
         <v>1.631561512053793</v>
       </c>
@@ -1693,14 +1747,10 @@
           <t>2026-09-03 (C)</t>
         </is>
       </c>
-      <c r="AM9" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1746,76 +1796,76 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>410688162740</v>
+        <v>410687995904</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>46.51230537418382</v>
+        <v>46.72351</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>45.08603767117952</v>
+        <v>40.891914</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.398863582992435</v>
+        <v>1.3988631</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.26832592378167</v>
+        <v>24.841997</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.669073374829594</v>
+        <v>1.02689032967033</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.64161456392537</v>
+        <v>29.66229906042246</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.36237014152534</v>
+        <v>1.393260319363755</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02144205944785152</v>
+        <v>0.01693347562470663</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>0.08167323631476142</v>
+        <v>0.215</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1279428885227898</v>
+        <v>0.455</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.09707374113030687</v>
+        <v>0.215</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>0.1022561610551892</v>
+        <v>0.086660005</v>
       </c>
       <c r="X10" s="4" t="n">
-        <v>0.2826735325396</v>
+        <v>0.29152</v>
       </c>
       <c r="Y10" s="4" t="n">
-        <v>0.1287591071811763</v>
+        <v>0.12876001</v>
       </c>
       <c r="Z10" s="4" t="n">
-        <v>0.03823398174987312</v>
+        <v>0.036730003</v>
       </c>
       <c r="AA10" s="5" t="n">
-        <v>7837000000</v>
+        <v>6954375168</v>
       </c>
       <c r="AB10" s="6" t="n">
-        <v>1.072451038575668</v>
+        <v>1.072</v>
       </c>
       <c r="AC10" s="6" t="n">
-        <v>0.6114896142433235</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="AD10" s="6" t="n">
-        <v>0.2456653436390223</v>
+        <v>0.6025699999999999</v>
       </c>
       <c r="AE10" s="6" t="n">
-        <v>0.09524470669906282</v>
+        <v>0.1326606018755107</v>
       </c>
       <c r="AF10" s="6" t="n">
-        <v>-0.7404284727021424</v>
+        <v>-0.06511964203514763</v>
       </c>
       <c r="AG10" s="6" t="n">
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005982333758071831</v>
+        <v>0.0063</v>
       </c>
       <c r="AI10" s="6" t="n">
         <v>-0.1425853178542787</v>
@@ -1834,7 +1884,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,70 +1930,70 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>286853826531</v>
+        <v>286853791744</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>21.32817337461301</v>
+        <v>21.528124</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.16928462311166</v>
+        <v>18.066475</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5.930314156935789</v>
+        <v>5.930313</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.571523811049412</v>
+        <v>9.513878999999999</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6268402174733824</v>
+        <v>1.939470630630631</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>9.54549589182456</v>
+        <v>19.98926724521858</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.03802537687848</v>
+        <v>6.085919119972625</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03832825984216677</v>
+        <v>0.08850345890026402</v>
       </c>
       <c r="T11" s="4" t="n">
-        <v>0.1585106891967754</v>
+        <v>0.134</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.4204624505928856</v>
+        <v>0.111</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1294454802019058</v>
+        <v>0.134</v>
       </c>
       <c r="W11" s="4" t="n">
-        <v>0.2335250473131588</v>
+        <v>0.16084999</v>
       </c>
       <c r="X11" s="4" t="n">
-        <v>0.4795743488592955</v>
+        <v>0.49541</v>
       </c>
       <c r="Y11" s="4" t="n">
-        <v>0.4911787210969006</v>
+        <v>0.49118</v>
       </c>
       <c r="Z11" s="4" t="n">
-        <v>0.2967601876207703</v>
+        <v>0.33381</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>9461053000</v>
+        <v>25387552768</v>
       </c>
       <c r="AB11" s="6" t="n">
-        <v>1.141608524439184</v>
+        <v>1.142</v>
       </c>
       <c r="AC11" s="6" t="n">
-        <v>1.141608524439184</v>
+        <v>0.917</v>
       </c>
       <c r="AD11" s="6" t="n">
-        <v>0.4745715482316096</v>
+        <v>0.55236</v>
       </c>
       <c r="AE11" s="6" t="n">
-        <v>0.2448109159689659</v>
+        <v>0.2995604565880029</v>
       </c>
       <c r="AF11" s="6" t="n">
-        <v>0.1702803389007786</v>
+        <v>0.5110874747049546</v>
       </c>
       <c r="AG11" s="6" t="n">
         <v>17.38427322249553</v>
@@ -1968,7 +2018,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -1998,39 +2048,93 @@
           <t>Insurance - Diversified</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="n">
+        <v>490.85</v>
+      </c>
       <c r="G12" s="4" t="n">
-        <v>-0.01207607915123976</v>
+        <v>-0.01207609143566268</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.04468576237164368</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
-      <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="6" t="inlineStr"/>
-      <c r="O12" s="6" t="inlineStr"/>
-      <c r="P12" s="6" t="inlineStr"/>
-      <c r="Q12" s="6" t="inlineStr"/>
-      <c r="R12" s="6" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="inlineStr"/>
-      <c r="W12" s="4" t="inlineStr"/>
-      <c r="X12" s="4" t="inlineStr"/>
-      <c r="Y12" s="4" t="inlineStr"/>
-      <c r="Z12" s="4" t="inlineStr"/>
-      <c r="AA12" s="5" t="inlineStr"/>
-      <c r="AB12" s="6" t="inlineStr"/>
-      <c r="AC12" s="6" t="inlineStr"/>
-      <c r="AD12" s="6" t="inlineStr"/>
-      <c r="AE12" s="6" t="inlineStr"/>
-      <c r="AF12" s="6" t="inlineStr"/>
-      <c r="AG12" s="6" t="inlineStr"/>
-      <c r="AH12" s="4" t="inlineStr"/>
+        <v>-0.05030473057947182</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>516.85</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>455.19</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>1058691678208</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>14.57826</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>22.815746</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>2.8202147</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>0.00097090466</v>
+      </c>
+      <c r="P12" s="6" t="n">
+        <v>0.1218918060200669</v>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>-2.250111889903251</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>-0.7073160310178424</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0.0578338815240697</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>1.196</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>0.053940002</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>0.10499</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <v>0.2778</v>
+      </c>
+      <c r="Z12" s="4" t="n">
+        <v>0.14352</v>
+      </c>
+      <c r="AA12" s="5" t="n">
+        <v>61228249088</v>
+      </c>
+      <c r="AB12" s="6" t="n">
+        <v>2.876</v>
+      </c>
+      <c r="AC12" s="6" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AD12" s="6" t="n">
+        <v>0.17669</v>
+      </c>
+      <c r="AE12" s="6" t="n">
+        <v>0.1054561679888985</v>
+      </c>
+      <c r="AF12" s="6" t="n">
+        <v>-2.275321290807187</v>
+      </c>
+      <c r="AG12" s="6" t="n">
+        <v>17.26731110672716</v>
+      </c>
+      <c r="AH12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI12" s="6" t="n">
         <v>0.04410289618060771</v>
       </c>
@@ -2045,14 +2149,10 @@
           <t>2026-08-01 (E)</t>
         </is>
       </c>
-      <c r="AM12" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2098,76 +2198,58 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>937560549000</v>
+        <v>930104213504</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.04299226139295</v>
+        <v>14.927474</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.26146868264625</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>3.150055770025501</v>
-      </c>
+        <v>14.144849</v>
+      </c>
+      <c r="N13" s="6" t="inlineStr"/>
       <c r="O13" s="6" t="n">
-        <v>2.604835396878787</v>
+        <v>2.6306884</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7876397824799048</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>20.5367562608016</v>
-      </c>
+        <v>0.3182830277185501</v>
+      </c>
+      <c r="Q13" s="6" t="inlineStr"/>
       <c r="R13" s="6" t="n">
-        <v>6.268191191836927</v>
-      </c>
-      <c r="S13" s="4" t="n">
-        <v>0.1503316240751935</v>
-      </c>
+        <v>2.506070797258559</v>
+      </c>
+      <c r="S13" s="4" t="inlineStr"/>
       <c r="T13" s="4" t="n">
-        <v>0.03307372160612143</v>
+        <v>0.304</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.2236728179551122</v>
+        <v>0.469</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.263019153357522</v>
+        <v>0.304</v>
       </c>
       <c r="W13" s="4" t="n">
-        <v>0.01297429806050525</v>
+        <v>0.0136</v>
       </c>
       <c r="X13" s="4" t="n">
-        <v>0.1781088712271246</v>
+        <v>0.17789</v>
       </c>
       <c r="Y13" s="4" t="n">
-        <v>0.6260327315855433</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="4" t="n">
-        <v>0.2818840652750199</v>
-      </c>
-      <c r="AA13" s="5" t="n">
-        <v>100867000000</v>
-      </c>
-      <c r="AB13" s="6" t="n">
-        <v>0.8403662699432636</v>
-      </c>
-      <c r="AC13" s="6" t="n">
-        <v>0.8403662699432636</v>
-      </c>
-      <c r="AD13" s="6" t="n">
-        <v>3.304531791413729</v>
-      </c>
+        <v>0.5039400000000001</v>
+      </c>
+      <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" s="6" t="inlineStr"/>
+      <c r="AC13" s="6" t="inlineStr"/>
+      <c r="AD13" s="6" t="inlineStr"/>
       <c r="AE13" s="6" t="n">
-        <v>0.2468303028333209</v>
-      </c>
-      <c r="AF13" s="6" t="n">
-        <v>10.2160870953183</v>
-      </c>
-      <c r="AG13" s="6" t="n">
-        <v>0.7415371100533208</v>
-      </c>
+        <v>0.3014379927989333</v>
+      </c>
+      <c r="AF13" s="6" t="inlineStr"/>
+      <c r="AG13" s="6" t="inlineStr"/>
       <c r="AH13" s="4" t="n">
-        <v>0.01714775650185767</v>
+        <v>0.0172</v>
       </c>
       <c r="AI13" s="6" t="n">
         <v>0.8050957040535519</v>
@@ -2183,10 +2265,14 @@
           <t>2026-10-13 (C)</t>
         </is>
       </c>
-      <c r="AM13" s="2" t="inlineStr"/>
+      <c r="AM13" s="2" t="inlineStr">
+        <is>
+          <t>ps,free_cash_flow,current_ratio,quick_ratio,debt_equity,ev_ebitda,fcf_yield,net_debt_ebitda,interest_coverage</t>
+        </is>
+      </c>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2299,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Financial - Credit Services</t>
+          <t>Credit Services</t>
         </is>
       </c>
       <c r="F14" s="3" t="n">
@@ -2231,77 +2317,69 @@
       <c r="J14" s="3" t="n">
         <v>293.89</v>
       </c>
-      <c r="K14" s="5" t="n">
-        <v>673956148528</v>
-      </c>
+      <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="6" t="n">
-        <v>30.60052219321149</v>
+        <v>30.761154</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>26.73060928455327</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>15.66356354214795</v>
-      </c>
-      <c r="O14" s="6" t="n">
-        <v>18.86569001430134</v>
-      </c>
+        <v>23.641808</v>
+      </c>
+      <c r="N14" s="6" t="inlineStr"/>
+      <c r="O14" s="6" t="inlineStr"/>
       <c r="P14" s="6" t="n">
-        <v>1.992033993754164</v>
+        <v>0.8665113802816902</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.98628931168649</v>
+        <v>22.33220851755459</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.93251094726567</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>0.03143379587272933</v>
-      </c>
+        <v>15.64505434218158</v>
+      </c>
+      <c r="S14" s="4" t="inlineStr"/>
       <c r="T14" s="4" t="n">
-        <v>0.1133997661860491</v>
+        <v>0.171</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2895549019607846</v>
+        <v>0.355</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.13930411415</v>
+        <v>0.171</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>0.2339424928194931</v>
+        <v>0.19193001</v>
       </c>
       <c r="X14" s="4" t="n">
-        <v>0.5889902060114826</v>
+        <v>0.60349</v>
       </c>
       <c r="Y14" s="4" t="n">
-        <v>0.8128616914960374</v>
+        <v>0.97778</v>
       </c>
       <c r="Z14" s="4" t="n">
-        <v>0.6111511376577498</v>
+        <v>0.6734599999999999</v>
       </c>
       <c r="AA14" s="5" t="n">
-        <v>21577000000</v>
+        <v>20839749632</v>
       </c>
       <c r="AB14" s="6" t="n">
-        <v>1.087666804237172</v>
+        <v>1.088</v>
       </c>
       <c r="AC14" s="6" t="n">
-        <v>1.087666804237172</v>
+        <v>0.669</v>
       </c>
       <c r="AD14" s="6" t="n">
-        <v>0.672331118028098</v>
+        <v>0.6723300000000001</v>
       </c>
       <c r="AE14" s="6" t="n">
-        <v>0.2522488400719629</v>
+        <v>0.240657647906692</v>
       </c>
       <c r="AF14" s="6" t="n">
-        <v>0.4048985304408678</v>
+        <v>0.3338419984642209</v>
       </c>
       <c r="AG14" s="6" t="n">
-        <v>42.07640067911715</v>
+        <v>45.08658743633277</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.00739476678043231</v>
+        <v>0.0076</v>
       </c>
       <c r="AI14" s="6" t="n">
         <v>0.3920108403130597</v>
@@ -2317,10 +2395,14 @@
           <t>2026-07-28 (C)</t>
         </is>
       </c>
-      <c r="AM14" s="2" t="inlineStr"/>
+      <c r="AM14" s="2" t="inlineStr">
+        <is>
+          <t>market_cap,ps,pb,fcf_yield</t>
+        </is>
+      </c>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2347,42 +2429,88 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Financial - Credit Services</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
+          <t>Credit Services</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>530.29</v>
+      </c>
       <c r="G15" s="4" t="n">
-        <v>-0.05831695447004781</v>
+        <v>-0.05831691545124917</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.11464879361923</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
+        <v>-0.1187829237083936</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>601.77</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>464.52</v>
+      </c>
       <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="n">
+        <v>30.670326</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>23.256536</v>
+      </c>
       <c r="N15" s="6" t="inlineStr"/>
       <c r="O15" s="6" t="inlineStr"/>
-      <c r="P15" s="6" t="inlineStr"/>
-      <c r="Q15" s="6" t="inlineStr"/>
-      <c r="R15" s="6" t="inlineStr"/>
+      <c r="P15" s="6" t="n">
+        <v>1.446713490566038</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>22.42128042300872</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>14.1223874784219</v>
+      </c>
       <c r="S15" s="4" t="inlineStr"/>
-      <c r="T15" s="4" t="inlineStr"/>
-      <c r="U15" s="4" t="inlineStr"/>
-      <c r="V15" s="4" t="inlineStr"/>
-      <c r="W15" s="4" t="inlineStr"/>
-      <c r="X15" s="4" t="inlineStr"/>
-      <c r="Y15" s="4" t="inlineStr"/>
-      <c r="Z15" s="4" t="inlineStr"/>
-      <c r="AA15" s="5" t="inlineStr"/>
-      <c r="AB15" s="6" t="inlineStr"/>
-      <c r="AC15" s="6" t="inlineStr"/>
-      <c r="AD15" s="6" t="inlineStr"/>
-      <c r="AE15" s="6" t="inlineStr"/>
-      <c r="AF15" s="6" t="inlineStr"/>
-      <c r="AG15" s="6" t="inlineStr"/>
-      <c r="AH15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="U15" s="4" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="V15" s="4" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="W15" s="4" t="n">
+        <v>0.25032</v>
+      </c>
+      <c r="X15" s="4" t="n">
+        <v>2.32076</v>
+      </c>
+      <c r="Y15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="4" t="n">
+        <v>0.60836</v>
+      </c>
+      <c r="AA15" s="5" t="n">
+        <v>16148124672</v>
+      </c>
+      <c r="AB15" s="6" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="AC15" s="6" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="AD15" s="6" t="n">
+        <v>2.82059</v>
+      </c>
+      <c r="AE15" s="6" t="n">
+        <v>0.3500932285023173</v>
+      </c>
+      <c r="AF15" s="6" t="n">
+        <v>0.5024558851763385</v>
+      </c>
+      <c r="AG15" s="6" t="n">
+        <v>26.73130193905817</v>
+      </c>
+      <c r="AH15" s="4" t="n">
+        <v>0.006500000000000001</v>
+      </c>
       <c r="AI15" s="6" t="n">
         <v>0.352652463476208</v>
       </c>
@@ -2399,12 +2527,12 @@
       </c>
       <c r="AM15" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>market_cap,ps,pb,fcf_yield</t>
         </is>
       </c>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2559,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medical - Healthcare Plans</t>
+          <t>Healthcare Plans</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -2450,76 +2578,76 @@
         <v>234.6</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>384653643758</v>
+        <v>384653623296</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>27.23683364413865</v>
+        <v>32.456703</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>21.48384400322998</v>
+        <v>18.879059</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.8545409066245454</v>
+        <v>0.8545409</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.671735471376766</v>
+        <v>3.671732</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.8252831708622166</v>
+        <v>0.5277512682926829</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>16.55527864604278</v>
+        <v>17.60196910551248</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.9475364701185659</v>
+        <v>0.948708826705284</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06139809250021908</v>
+        <v>0.05916946638114946</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>0.118140392427263</v>
+        <v>0.004</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.4901950113378684</v>
+        <v>0.615</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>-0.004122139121070179</v>
+        <v>0.004</v>
       </c>
       <c r="W16" s="4" t="n">
-        <v>0.0455949917185134</v>
+        <v>0.04382</v>
       </c>
       <c r="X16" s="4" t="n">
-        <v>0.1439951464601533</v>
+        <v>0.14152999</v>
       </c>
       <c r="Y16" s="4" t="n">
-        <v>0.2248555414114621</v>
+        <v>0.19514</v>
       </c>
       <c r="Z16" s="4" t="n">
-        <v>0.0481550844313519</v>
+        <v>0.07132999600000001</v>
       </c>
       <c r="AA16" s="5" t="n">
-        <v>16075000000</v>
+        <v>22759749632</v>
       </c>
       <c r="AB16" s="6" t="n">
-        <v>1.240522019786234</v>
+        <v>0.777</v>
       </c>
       <c r="AC16" s="6" t="n">
-        <v>1.240522019786234</v>
+        <v>0.474</v>
       </c>
       <c r="AD16" s="6" t="n">
-        <v>0.7016160669007683</v>
+        <v>0.69211</v>
       </c>
       <c r="AE16" s="6" t="n">
-        <v>0.2367504286032538</v>
+        <v>0.2368620846369771</v>
       </c>
       <c r="AF16" s="6" t="n">
-        <v>1.624810775142646</v>
+        <v>1.725403043054092</v>
       </c>
       <c r="AG16" s="6" t="n">
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.0211304183586741</v>
+        <v>0.0215</v>
       </c>
       <c r="AI16" s="6" t="n">
         <v>0.5615307959671498</v>
@@ -2538,7 +2666,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2583,77 +2711,71 @@
       <c r="J17" s="3" t="n">
         <v>105.53</v>
       </c>
-      <c r="K17" s="5" t="n">
-        <v>650300806372</v>
-      </c>
+      <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="6" t="n">
-        <v>26.59152542372881</v>
+        <v>25.975166</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.27132899192877</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>1.994738798961989</v>
-      </c>
+        <v>14.627156</v>
+      </c>
+      <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="n">
-        <v>2.579873772019136</v>
+        <v>2.5564191</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>-1.216763739085774</v>
+        <v>-0.5985061290322581</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>11.40920653868555</v>
+        <v>12.42954882933399</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2.11506099964418</v>
-      </c>
-      <c r="S17" s="4" t="n">
-        <v>0.02889739612171136</v>
-      </c>
+        <v>2.135351631700753</v>
+      </c>
+      <c r="S17" s="4" t="inlineStr"/>
       <c r="T17" s="4" t="n">
-        <v>-0.04522368657644726</v>
+        <v>0.026</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.6408014925373136</v>
+        <v>-0.434</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.2219833869653138</v>
+        <v>0.026</v>
       </c>
       <c r="W17" s="4" t="n">
-        <v>0.05450787020090007</v>
+        <v>0.04221</v>
       </c>
       <c r="X17" s="4" t="n">
-        <v>0.09765064069490346</v>
+        <v>0.09873</v>
       </c>
       <c r="Y17" s="4" t="n">
-        <v>0.2549231920689063</v>
+        <v>0.29768</v>
       </c>
       <c r="Z17" s="4" t="n">
-        <v>0.09011128561262301</v>
+        <v>0.06355</v>
       </c>
       <c r="AA17" s="5" t="n">
-        <v>23612000000</v>
+        <v>11630499840</v>
       </c>
       <c r="AB17" s="6" t="n">
-        <v>1.03612070609676</v>
+        <v>1.036</v>
       </c>
       <c r="AC17" s="6" t="n">
-        <v>0.7714933565025748</v>
+        <v>0.744</v>
       </c>
       <c r="AD17" s="6" t="n">
-        <v>0.1873606912465947</v>
+        <v>0.18261</v>
       </c>
       <c r="AE17" s="6" t="n">
-        <v>0.1026269890829224</v>
+        <v>0.1061539459575037</v>
       </c>
       <c r="AF17" s="6" t="n">
-        <v>0.6490502349592958</v>
+        <v>0.7003767172527701</v>
       </c>
       <c r="AG17" s="6" t="n">
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02600548154758111</v>
+        <v>0.0267</v>
       </c>
       <c r="AI17" s="6" t="n">
         <v>-0.4280369953194851</v>
@@ -2669,10 +2791,14 @@
           <t>2026-07-31 (C)</t>
         </is>
       </c>
-      <c r="AM17" s="2" t="inlineStr"/>
+      <c r="AM17" s="2" t="inlineStr">
+        <is>
+          <t>market_cap,ps,fcf_yield</t>
+        </is>
+      </c>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2718,76 +2844,64 @@
         <v>164.23</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>624119929400</v>
+        <v>624119119872</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.97341040462427</v>
+        <v>29.664759</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.22304126609707</v>
+        <v>20.204672</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.373188017849666</v>
+        <v>6.3731794</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.445550547951654</v>
+        <v>7.685489</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.711181472467301</v>
+        <v>-29.664759</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.27973712835615</v>
+        <v>18.85921880435592</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.28404179967119</v>
-      </c>
-      <c r="S18" s="4" t="n">
-        <v>0.03623181849318462</v>
-      </c>
+        <v>6.709505192474225</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="n">
-        <v>0.06048119251078021</v>
+        <v>0.066</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.05772620126926564</v>
+        <v>-0.01</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.07475803440807693</v>
-      </c>
-      <c r="W18" s="4" t="n">
-        <v>0.1046299381779659</v>
-      </c>
-      <c r="X18" s="4" t="n">
-        <v>0.2573506474441706</v>
-      </c>
+        <v>0.066</v>
+      </c>
+      <c r="W18" s="4" t="inlineStr"/>
+      <c r="X18" s="4" t="inlineStr"/>
       <c r="Y18" s="4" t="n">
-        <v>0.7045206220833461</v>
+        <v>0.68097</v>
       </c>
       <c r="Z18" s="4" t="n">
-        <v>0.2681126121986337</v>
-      </c>
-      <c r="AA18" s="5" t="n">
-        <v>19698000000</v>
-      </c>
-      <c r="AB18" s="6" t="n">
-        <v>1.088878768558156</v>
-      </c>
-      <c r="AC18" s="6" t="n">
-        <v>0.8130066490572911</v>
-      </c>
+        <v>0.28605</v>
+      </c>
+      <c r="AA18" s="5" t="inlineStr"/>
+      <c r="AB18" s="6" t="inlineStr"/>
+      <c r="AC18" s="6" t="inlineStr"/>
       <c r="AD18" s="6" t="n">
-        <v>0.1375998870202775</v>
+        <v>0.6773</v>
       </c>
       <c r="AE18" s="6" t="n">
-        <v>0.05815150625929445</v>
+        <v>0.2760253092515436</v>
       </c>
       <c r="AF18" s="6" t="n">
-        <v>-0.2735048090479025</v>
+        <v>0.9453502579809987</v>
       </c>
       <c r="AG18" s="6" t="n">
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.0202105912755043</v>
+        <v>0.021</v>
       </c>
       <c r="AI18" s="6" t="n">
         <v>-0.1517102526708811</v>
@@ -2803,10 +2917,14 @@
           <t>2026-10-13 (C)</t>
         </is>
       </c>
-      <c r="AM18" s="2" t="inlineStr"/>
+      <c r="AM18" s="2" t="inlineStr">
+        <is>
+          <t>roa,roe,free_cash_flow,current_ratio,quick_ratio,fcf_yield</t>
+        </is>
+      </c>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2852,76 +2970,76 @@
         <v>95.34999999999999</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>862655872000</v>
+        <v>862655741952</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.03508771929825</v>
+        <v>38.439716</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.36539495636108</v>
+        <v>32.99587</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.189369812699485</v>
+        <v>1.1893697</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>9.157633838651543</v>
+        <v>9.149224</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>1.745139318885448</v>
+        <v>1.981428659793814</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>19.23816182305407</v>
+        <v>20.83315079863233</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.276850251962967</v>
+        <v>1.287895142399991</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.0145504139105889</v>
+        <v>0.007954795465074212</v>
       </c>
       <c r="T19" s="4" t="n">
-        <v>0.04725214211766771</v>
+        <v>0.073</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.06266666666666665</v>
+        <v>0.194</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.05505332192359957</v>
+        <v>0.073</v>
       </c>
       <c r="W19" s="4" t="n">
-        <v>0.07850638969361928</v>
+        <v>0.06834999999999999</v>
       </c>
       <c r="X19" s="4" t="n">
-        <v>0.2392312528442645</v>
+        <v>0.24132</v>
       </c>
       <c r="Y19" s="4" t="n">
-        <v>0.2497638924314599</v>
+        <v>0.24976</v>
       </c>
       <c r="Z19" s="4" t="n">
-        <v>0.04161421746713451</v>
+        <v>0.042150002</v>
       </c>
       <c r="AA19" s="5" t="n">
-        <v>14923000000</v>
+        <v>6862249984</v>
       </c>
       <c r="AB19" s="6" t="n">
-        <v>0.7714407896459335</v>
+        <v>0.771</v>
       </c>
       <c r="AC19" s="6" t="n">
-        <v>0.2253737465418081</v>
+        <v>0.187</v>
       </c>
       <c r="AD19" s="6" t="n">
-        <v>0.7863776105162726</v>
+        <v>0.74816</v>
       </c>
       <c r="AE19" s="6" t="n">
-        <v>0.2561367646500257</v>
+        <v>0.2653793260359436</v>
       </c>
       <c r="AF19" s="6" t="n">
-        <v>1.318058123351129</v>
+        <v>1.445559661076498</v>
       </c>
       <c r="AG19" s="6" t="n">
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.008902214022140221</v>
+        <v>0.0091</v>
       </c>
       <c r="AI19" s="6" t="n">
         <v>-0.04634012957674574</v>
@@ -2940,7 +3058,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -2970,39 +3088,91 @@
           <t>Household &amp; Personal Products</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="n">
+        <v>146.97</v>
+      </c>
       <c r="G20" s="4" t="n">
-        <v>0.03653295845862004</v>
+        <v>0.03653294984938693</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1209927996218887</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="6" t="inlineStr"/>
-      <c r="M20" s="6" t="inlineStr"/>
+        <v>-0.121255605381166</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>167.25</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>137.62</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>342234202112</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>21.773333</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>20.837557</v>
+      </c>
       <c r="N20" s="6" t="inlineStr"/>
-      <c r="O20" s="6" t="inlineStr"/>
-      <c r="P20" s="6" t="inlineStr"/>
-      <c r="Q20" s="6" t="inlineStr"/>
-      <c r="R20" s="6" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="inlineStr"/>
-      <c r="W20" s="4" t="inlineStr"/>
-      <c r="X20" s="4" t="inlineStr"/>
-      <c r="Y20" s="4" t="inlineStr"/>
-      <c r="Z20" s="4" t="inlineStr"/>
-      <c r="AA20" s="5" t="inlineStr"/>
-      <c r="AB20" s="6" t="inlineStr"/>
-      <c r="AC20" s="6" t="inlineStr"/>
-      <c r="AD20" s="6" t="inlineStr"/>
-      <c r="AE20" s="6" t="inlineStr"/>
-      <c r="AF20" s="6" t="inlineStr"/>
-      <c r="AG20" s="6" t="inlineStr"/>
-      <c r="AH20" s="4" t="inlineStr"/>
+      <c r="O20" s="6" t="n">
+        <v>6.367575</v>
+      </c>
+      <c r="P20" s="6" t="n">
+        <v>3.754022931034482</v>
+      </c>
+      <c r="Q20" s="6" t="n">
+        <v>14.69288366203535</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>4.242988120338525</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>0.03720770803565897</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="U20" s="4" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="V20" s="4" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="W20" s="4" t="n">
+        <v>0.10925999</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>0.31112</v>
+      </c>
+      <c r="Y20" s="4" t="n">
+        <v>0.50984</v>
+      </c>
+      <c r="Z20" s="4" t="n">
+        <v>0.23047</v>
+      </c>
+      <c r="AA20" s="5" t="n">
+        <v>12733750272</v>
+      </c>
+      <c r="AB20" s="6" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="AC20" s="6" t="n">
+        <v>0.487</v>
+      </c>
+      <c r="AD20" s="6" t="n">
+        <v>0.6765099999999999</v>
+      </c>
+      <c r="AE20" s="6" t="n">
+        <v>0.29566162448595</v>
+      </c>
+      <c r="AF20" s="6" t="n">
+        <v>0.9871416480454489</v>
+      </c>
+      <c r="AG20" s="6" t="n">
+        <v>23.2348401323043</v>
+      </c>
+      <c r="AH20" s="4" t="n">
+        <v>0.0292</v>
+      </c>
       <c r="AI20" s="6" t="n">
         <v>-0.08229183976326422</v>
       </c>
@@ -3019,12 +3189,12 @@
       </c>
       <c r="AM20" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>ps</t>
         </is>
       </c>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3051,42 +3221,94 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Home Improvement</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
+          <t>Home Improvement Retail</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>324.71</v>
+      </c>
       <c r="G21" s="4" t="n">
-        <v>-0.06104336192830284</v>
+        <v>-0.0610433372191429</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2331255463660392</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="inlineStr"/>
+        <v>-0.2391095489162274</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>426.75</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>289.1</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>323773759488</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>23.529709</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>20.178034</v>
+      </c>
       <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="4" t="inlineStr"/>
-      <c r="T21" s="4" t="inlineStr"/>
-      <c r="U21" s="4" t="inlineStr"/>
-      <c r="V21" s="4" t="inlineStr"/>
-      <c r="W21" s="4" t="inlineStr"/>
-      <c r="X21" s="4" t="inlineStr"/>
-      <c r="Y21" s="4" t="inlineStr"/>
-      <c r="Z21" s="4" t="inlineStr"/>
-      <c r="AA21" s="5" t="inlineStr"/>
-      <c r="AB21" s="6" t="inlineStr"/>
-      <c r="AC21" s="6" t="inlineStr"/>
-      <c r="AD21" s="6" t="inlineStr"/>
-      <c r="AE21" s="6" t="inlineStr"/>
-      <c r="AF21" s="6" t="inlineStr"/>
-      <c r="AG21" s="6" t="inlineStr"/>
-      <c r="AH21" s="4" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>23.333572</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>-5.472025348837209</v>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>15.46956454919042</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>2.316460248846156</v>
+      </c>
+      <c r="S21" s="4" t="n">
+        <v>0.03128187371334946</v>
+      </c>
+      <c r="T21" s="4" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="U21" s="4" t="n">
+        <v>-0.043</v>
+      </c>
+      <c r="V21" s="4" t="n">
+        <v>0.048</v>
+      </c>
+      <c r="W21" s="4" t="n">
+        <v>0.12519</v>
+      </c>
+      <c r="X21" s="4" t="n">
+        <v>1.2838</v>
+      </c>
+      <c r="Y21" s="4" t="n">
+        <v>0.33126998</v>
+      </c>
+      <c r="Z21" s="4" t="n">
+        <v>0.11926</v>
+      </c>
+      <c r="AA21" s="5" t="n">
+        <v>10128249856</v>
+      </c>
+      <c r="AB21" s="6" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="AC21" s="6" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="AD21" s="6" t="n">
+        <v>4.59356</v>
+      </c>
+      <c r="AE21" s="6" t="n">
+        <v>0.6064132384604406</v>
+      </c>
+      <c r="AF21" s="6" t="n">
+        <v>2.49057963917238</v>
+      </c>
+      <c r="AG21" s="6" t="n">
+        <v>8.712271973466004</v>
+      </c>
+      <c r="AH21" s="4" t="n">
+        <v>0.0281</v>
+      </c>
       <c r="AI21" s="6" t="n">
         <v>0.7044542283994155</v>
       </c>
@@ -3103,12 +3325,12 @@
       </c>
       <c r="AM21" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>ps</t>
         </is>
       </c>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3154,70 +3376,68 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>880018514000</v>
+        <v>880018849792</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>175.224025974026</v>
+        <v>185.46048</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>72.05704855696311</v>
-      </c>
-      <c r="N22" s="6" t="n">
-        <v>23.49598211138997</v>
-      </c>
+        <v>40.000534</v>
+      </c>
+      <c r="N22" s="6" t="inlineStr"/>
       <c r="O22" s="6" t="n">
-        <v>13.65508966522913</v>
+        <v>13.6468</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>1.422406799083269</v>
+        <v>2.033557894736842</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>108.6203950037101</v>
+        <v>117.3005204965725</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>23.45021930901907</v>
+        <v>23.26968759880066</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.009742976839234998</v>
+        <v>0.008151387868220651</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>0.3433779329067288</v>
+        <v>0.378</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>1.826324528301887</v>
+        <v>0.912</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.4460310731834061</v>
+        <v>0.378</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>0.06289395042816605</v>
+        <v>0.03647</v>
       </c>
       <c r="X22" s="4" t="n">
-        <v>0.0808176963164943</v>
+        <v>0.08062999999999999</v>
       </c>
       <c r="Y22" s="4" t="n">
-        <v>0.5028034388850323</v>
+        <v>0.5306</v>
       </c>
       <c r="Z22" s="4" t="n">
-        <v>0.1165162599455332</v>
+        <v>0.14396</v>
       </c>
       <c r="AA22" s="5" t="n">
-        <v>6735000000</v>
+        <v>7173374976</v>
       </c>
       <c r="AB22" s="6" t="n">
-        <v>2.724919093851133</v>
+        <v>2.725</v>
       </c>
       <c r="AC22" s="6" t="n">
-        <v>1.959166190748144</v>
+        <v>1.75</v>
       </c>
       <c r="AD22" s="6" t="n">
-        <v>0.06005088269057739</v>
+        <v>0.06005</v>
       </c>
       <c r="AE22" s="6" t="n">
-        <v>0.04860500740815148</v>
+        <v>0.05032108863063203</v>
       </c>
       <c r="AF22" s="6" t="n">
-        <v>-0.2119713084343309</v>
+        <v>-1.140780565004049</v>
       </c>
       <c r="AG22" s="6" t="n">
         <v>32.6030534351145</v>
@@ -3239,10 +3459,14 @@
           <t>2026-08-04 (C)</t>
         </is>
       </c>
-      <c r="AM22" s="2" t="inlineStr"/>
+      <c r="AM22" s="2" t="inlineStr">
+        <is>
+          <t>ps</t>
+        </is>
+      </c>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3269,42 +3493,96 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr"/>
+          <t>Semiconductor Equipment &amp; Materials</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>1803</v>
+      </c>
       <c r="G23" s="4" t="n">
         <v>0.5492618489847474</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.09371478752681706</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="5" t="inlineStr"/>
-      <c r="L23" s="6" t="inlineStr"/>
-      <c r="M23" s="6" t="inlineStr"/>
-      <c r="N23" s="6" t="inlineStr"/>
-      <c r="O23" s="6" t="inlineStr"/>
-      <c r="P23" s="6" t="inlineStr"/>
-      <c r="Q23" s="6" t="inlineStr"/>
-      <c r="R23" s="6" t="inlineStr"/>
-      <c r="S23" s="4" t="inlineStr"/>
-      <c r="T23" s="4" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" s="4" t="inlineStr"/>
-      <c r="W23" s="4" t="inlineStr"/>
-      <c r="X23" s="4" t="inlineStr"/>
-      <c r="Y23" s="4" t="inlineStr"/>
-      <c r="Z23" s="4" t="inlineStr"/>
-      <c r="AA23" s="5" t="inlineStr"/>
-      <c r="AB23" s="6" t="inlineStr"/>
-      <c r="AC23" s="6" t="inlineStr"/>
-      <c r="AD23" s="6" t="inlineStr"/>
-      <c r="AE23" s="6" t="inlineStr"/>
-      <c r="AF23" s="6" t="inlineStr"/>
-      <c r="AG23" s="6" t="inlineStr"/>
-      <c r="AH23" s="4" t="inlineStr"/>
+        <v>-0.09848196963939282</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>1999.96</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>683.48</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>692532281344</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>62.108162</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>31.052652</v>
+      </c>
+      <c r="N23" s="6" t="n">
+        <v>19.603207</v>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>1623.0488</v>
+      </c>
+      <c r="P23" s="6" t="n">
+        <v>2.179233754385965</v>
+      </c>
+      <c r="Q23" s="6" t="n">
+        <v>2851.963075753253</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>1088.908627345221</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>0.01218380028671728</v>
+      </c>
+      <c r="T23" s="4" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="U23" s="4" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="V23" s="4" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="W23" s="4" t="n">
+        <v>0.16454001</v>
+      </c>
+      <c r="X23" s="4" t="n">
+        <v>0.53942</v>
+      </c>
+      <c r="Y23" s="4" t="n">
+        <v>0.5273300400000001</v>
+      </c>
+      <c r="Z23" s="4" t="n">
+        <v>0.37057</v>
+      </c>
+      <c r="AA23" s="5" t="n">
+        <v>8437675008</v>
+      </c>
+      <c r="AB23" s="6" t="n">
+        <v>1.334</v>
+      </c>
+      <c r="AC23" s="6" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="AD23" s="6" t="n">
+        <v>0.09092</v>
+      </c>
+      <c r="AE23" s="6" t="n">
+        <v>0.03924329498127222</v>
+      </c>
+      <c r="AF23" s="6" t="n">
+        <v>-0.4149565363317139</v>
+      </c>
+      <c r="AG23" s="6" t="n">
+        <v>97.4167371090448</v>
+      </c>
+      <c r="AH23" s="4" t="n">
+        <v>0.005</v>
+      </c>
       <c r="AI23" s="6" t="n">
         <v>1.702172886720601</v>
       </c>
@@ -3319,14 +3597,10 @@
           <t>2026-10-14 (C)</t>
         </is>
       </c>
-      <c r="AM23" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM23" s="2" t="inlineStr"/>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3372,70 +3646,66 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>164936427460</v>
+        <v>164936499200</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>86.45867768595038</v>
+        <v>82.6996</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>-1318.731879490735</v>
+        <v>50.978615</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.789208837325349</v>
+        <v>1.7892096</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>28.58696175045933</v>
-      </c>
-      <c r="P24" s="6" t="n">
-        <v>0.4791193213146133</v>
-      </c>
+        <v>27.562902</v>
+      </c>
+      <c r="P24" s="6" t="inlineStr"/>
       <c r="Q24" s="6" t="n">
-        <v>27.67673777444019</v>
+        <v>-59.64360056177035</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.198911171786861</v>
+        <v>2.108592517682061</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.006311522663800032</v>
+        <v>0.01548626287322097</v>
       </c>
       <c r="T24" s="4" t="n">
-        <v>0.3449644451794278</v>
-      </c>
-      <c r="U24" s="4" t="n">
-        <v>-1.063975806451613</v>
-      </c>
+        <v>0.14</v>
+      </c>
+      <c r="U24" s="4" t="inlineStr"/>
       <c r="V24" s="4" t="n">
-        <v>0.09389685671171333</v>
+        <v>0.14</v>
       </c>
       <c r="W24" s="4" t="n">
-        <v>0.01376322161335542</v>
+        <v>-0.02069</v>
       </c>
       <c r="X24" s="4" t="n">
-        <v>-87.23076923076923</v>
+        <v>1.69947</v>
       </c>
       <c r="Y24" s="4" t="n">
-        <v>0.04792588735572333</v>
+        <v>0.048249997</v>
       </c>
       <c r="Z24" s="4" t="n">
-        <v>-0.05889308339842055</v>
+        <v>0.01715</v>
       </c>
       <c r="AA24" s="5" t="n">
-        <v>-1877000000</v>
+        <v>2554249984</v>
       </c>
       <c r="AB24" s="6" t="n">
-        <v>1.176167963087535</v>
+        <v>1.176</v>
       </c>
       <c r="AC24" s="6" t="n">
-        <v>0.3497588751930419</v>
+        <v>0.317</v>
       </c>
       <c r="AD24" s="6" t="n">
-        <v>7.885251377985636</v>
+        <v>8.286960000000001</v>
       </c>
       <c r="AE24" s="6" t="n">
-        <v>0.2864849775771147</v>
+        <v>0.2949089079442447</v>
       </c>
       <c r="AF24" s="6" t="n">
-        <v>5.156744948115784</v>
+        <v>-9.032218373101573</v>
       </c>
       <c r="AG24" s="6" t="n">
         <v>1.950920245398773</v>
@@ -3457,10 +3727,14 @@
           <t>2026-07-28 (C)</t>
         </is>
       </c>
-      <c r="AM24" s="2" t="inlineStr"/>
+      <c r="AM24" s="2" t="inlineStr">
+        <is>
+          <t>fwd_eps_growth,peg</t>
+        </is>
+      </c>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3487,7 +3761,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Financial - Capital Markets</t>
+          <t>Capital Markets</t>
         </is>
       </c>
       <c r="F25" s="3" t="n">
@@ -3506,76 +3780,64 @@
         <v>694.05</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>317049923040</v>
+        <v>317050355712</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>16.37294332723949</v>
+        <v>16.948746</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>15.49433610160704</v>
-      </c>
-      <c r="N25" s="6" t="n">
-        <v>2.688299032873483</v>
-      </c>
+        <v>14.650673</v>
+      </c>
+      <c r="N25" s="6" t="inlineStr"/>
       <c r="O25" s="6" t="n">
-        <v>2.622142048780488</v>
+        <v>2.9327796</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3837591046797189</v>
-      </c>
-      <c r="Q25" s="6" t="n">
-        <v>29.49861188927468</v>
-      </c>
+        <v>0.1836267172264355</v>
+      </c>
+      <c r="Q25" s="6" t="inlineStr"/>
       <c r="R25" s="6" t="n">
-        <v>7.852072912148011</v>
-      </c>
-      <c r="S25" s="4" t="n">
-        <v>-0.1322252331684401</v>
-      </c>
+        <v>2.302078818509192</v>
+      </c>
+      <c r="S25" s="4" t="inlineStr"/>
       <c r="T25" s="4" t="n">
-        <v>-0.01384279441558334</v>
+        <v>0.425</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.3515611847233049</v>
+        <v>0.923</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.4338705009392712</v>
+        <v>0.425</v>
       </c>
       <c r="W25" s="4" t="n">
-        <v>0.009855733082706767</v>
+        <v>0.010720001</v>
       </c>
       <c r="X25" s="4" t="n">
-        <v>0.1695630555791363</v>
+        <v>0.16951999</v>
       </c>
       <c r="Y25" s="4" t="n">
-        <v>0.5729330066052214</v>
+        <v>0.82075995</v>
       </c>
       <c r="Z25" s="4" t="n">
-        <v>0.2480731237864283</v>
-      </c>
-      <c r="AA25" s="5" t="n">
-        <v>-47218000000</v>
-      </c>
+        <v>0.42316002</v>
+      </c>
+      <c r="AA25" s="5" t="inlineStr"/>
       <c r="AB25" s="6" t="n">
-        <v>0.4174107142857143</v>
+        <v>2.567</v>
       </c>
       <c r="AC25" s="6" t="n">
-        <v>0.4174107142857143</v>
+        <v>2.055</v>
       </c>
       <c r="AD25" s="6" t="n">
-        <v>6.471544715447155</v>
+        <v>6.47154</v>
       </c>
       <c r="AE25" s="6" t="n">
-        <v>0.3740601503759399</v>
-      </c>
-      <c r="AF25" s="6" t="n">
-        <v>19.3992291275125</v>
-      </c>
-      <c r="AG25" s="6" t="n">
-        <v>0.327057203580088</v>
-      </c>
+        <v>0.4399442850662127</v>
+      </c>
+      <c r="AF25" s="6" t="inlineStr"/>
+      <c r="AG25" s="6" t="inlineStr"/>
       <c r="AH25" s="4" t="n">
-        <v>0.01581807354473723</v>
+        <v>0.0182</v>
       </c>
       <c r="AI25" s="6" t="n">
         <v>1.56276640457987</v>
@@ -3591,10 +3853,14 @@
           <t>2026-10-13 (C)</t>
         </is>
       </c>
-      <c r="AM25" s="2" t="inlineStr"/>
+      <c r="AM25" s="2" t="inlineStr">
+        <is>
+          <t>ps,free_cash_flow,ev_ebitda,fcf_yield,net_debt_ebitda,interest_coverage</t>
+        </is>
+      </c>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3624,39 +3890,93 @@
           <t>Information Technology Services</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="n">
+        <v>206.65</v>
+      </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2910806384340159</v>
+        <v>-0.2910806174957118</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3723233393049764</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="5" t="inlineStr"/>
-      <c r="L26" s="6" t="inlineStr"/>
-      <c r="M26" s="6" t="inlineStr"/>
-      <c r="N26" s="6" t="inlineStr"/>
-      <c r="O26" s="6" t="inlineStr"/>
-      <c r="P26" s="6" t="inlineStr"/>
-      <c r="Q26" s="6" t="inlineStr"/>
-      <c r="R26" s="6" t="inlineStr"/>
-      <c r="S26" s="4" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr"/>
-      <c r="U26" s="4" t="inlineStr"/>
-      <c r="V26" s="4" t="inlineStr"/>
-      <c r="W26" s="4" t="inlineStr"/>
-      <c r="X26" s="4" t="inlineStr"/>
-      <c r="Y26" s="4" t="inlineStr"/>
-      <c r="Z26" s="4" t="inlineStr"/>
-      <c r="AA26" s="5" t="inlineStr"/>
-      <c r="AB26" s="6" t="inlineStr"/>
-      <c r="AC26" s="6" t="inlineStr"/>
-      <c r="AD26" s="6" t="inlineStr"/>
-      <c r="AE26" s="6" t="inlineStr"/>
-      <c r="AF26" s="6" t="inlineStr"/>
-      <c r="AG26" s="6" t="inlineStr"/>
-      <c r="AH26" s="4" t="inlineStr"/>
+        <v>-0.3784214642362991</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>332.46</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>199.19</v>
+      </c>
+      <c r="K26" s="5" t="n">
+        <v>194692071424</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>18.28761</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>15.829718</v>
+      </c>
+      <c r="N26" s="6" t="n">
+        <v>2.8177447</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>5.890317</v>
+      </c>
+      <c r="P26" s="6" t="n">
+        <v>-10.15978333333334</v>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>15.27846460164561</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>3.643215774168031</v>
+      </c>
+      <c r="S26" s="4" t="n">
+        <v>0.0610142979994801</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="U26" s="4" t="n">
+        <v>-0.018</v>
+      </c>
+      <c r="V26" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="W26" s="4" t="n">
+        <v>0.05298</v>
+      </c>
+      <c r="X26" s="4" t="n">
+        <v>0.34460998</v>
+      </c>
+      <c r="Y26" s="4" t="n">
+        <v>0.58101004</v>
+      </c>
+      <c r="Z26" s="4" t="n">
+        <v>0.16204001</v>
+      </c>
+      <c r="AA26" s="5" t="n">
+        <v>11879000064</v>
+      </c>
+      <c r="AB26" s="6" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="AC26" s="6" t="n">
+        <v>0.593</v>
+      </c>
+      <c r="AD26" s="6" t="n">
+        <v>1.8897</v>
+      </c>
+      <c r="AE26" s="6" t="n">
+        <v>0.4297603404793258</v>
+      </c>
+      <c r="AF26" s="6" t="n">
+        <v>3.4680747681581</v>
+      </c>
+      <c r="AG26" s="6" t="n">
+        <v>6.337467700258398</v>
+      </c>
+      <c r="AH26" s="4" t="n">
+        <v>0.0329</v>
+      </c>
       <c r="AI26" s="6" t="n">
         <v>0.855500584896021</v>
       </c>
@@ -3671,14 +3991,10 @@
           <t>2026-10-21 (C)</t>
         </is>
       </c>
-      <c r="AM26" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3708,39 +4024,89 @@
           <t>Drug Manufacturers - General</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="n">
+        <v>1185.87</v>
+      </c>
       <c r="G27" s="4" t="n">
-        <v>0.09766190084436599</v>
+        <v>0.097661905363982</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.0402166314222856</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="6" t="inlineStr"/>
-      <c r="M27" s="6" t="inlineStr"/>
+        <v>-0.05088639001160522</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>1249.45</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>623.78</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>1057489354752</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>41.31951</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>26.430014</v>
+      </c>
       <c r="N27" s="6" t="inlineStr"/>
-      <c r="O27" s="6" t="inlineStr"/>
-      <c r="P27" s="6" t="inlineStr"/>
-      <c r="Q27" s="6" t="inlineStr"/>
-      <c r="R27" s="6" t="inlineStr"/>
-      <c r="S27" s="4" t="inlineStr"/>
-      <c r="T27" s="4" t="inlineStr"/>
-      <c r="U27" s="4" t="inlineStr"/>
-      <c r="V27" s="4" t="inlineStr"/>
-      <c r="W27" s="4" t="inlineStr"/>
-      <c r="X27" s="4" t="inlineStr"/>
-      <c r="Y27" s="4" t="inlineStr"/>
-      <c r="Z27" s="4" t="inlineStr"/>
-      <c r="AA27" s="5" t="inlineStr"/>
-      <c r="AB27" s="6" t="inlineStr"/>
-      <c r="AC27" s="6" t="inlineStr"/>
-      <c r="AD27" s="6" t="inlineStr"/>
-      <c r="AE27" s="6" t="inlineStr"/>
-      <c r="AF27" s="6" t="inlineStr"/>
+      <c r="O27" s="6" t="n">
+        <v>33.96254</v>
+      </c>
+      <c r="P27" s="6" t="n">
+        <v>0.2431989994114185</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>30.25203196768712</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>15.16391052602099</v>
+      </c>
+      <c r="S27" s="4" t="n">
+        <v>0.008658810385989545</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="U27" s="4" t="n">
+        <v>1.699</v>
+      </c>
+      <c r="V27" s="4" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="W27" s="4" t="n">
+        <v>0.20739001</v>
+      </c>
+      <c r="X27" s="4" t="n">
+        <v>1.07459</v>
+      </c>
+      <c r="Y27" s="4" t="n">
+        <v>0.8283199999999999</v>
+      </c>
+      <c r="Z27" s="4" t="n">
+        <v>0.49386</v>
+      </c>
+      <c r="AA27" s="5" t="n">
+        <v>9156599808</v>
+      </c>
+      <c r="AB27" s="6" t="n">
+        <v>1.497</v>
+      </c>
+      <c r="AC27" s="6" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="AD27" s="6" t="n">
+        <v>1.39015</v>
+      </c>
+      <c r="AE27" s="6" t="n">
+        <v>0.3855933744443259</v>
+      </c>
+      <c r="AF27" s="6" t="n">
+        <v>1.051718883549078</v>
+      </c>
       <c r="AG27" s="6" t="inlineStr"/>
-      <c r="AH27" s="4" t="inlineStr"/>
+      <c r="AH27" s="4" t="n">
+        <v>0.006</v>
+      </c>
       <c r="AI27" s="6" t="n">
         <v>0.4496368562085785</v>
       </c>
@@ -3757,12 +4123,12 @@
       </c>
       <c r="AM27" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>ps,interest_coverage</t>
         </is>
       </c>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3789,42 +4155,78 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Financial - Capital Markets</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr"/>
+          <t>Capital Markets</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>215.18</v>
+      </c>
       <c r="G28" s="4" t="n">
-        <v>0.1829576684770855</v>
+        <v>0.1829577087421708</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.05849927892124673</v>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="6" t="inlineStr"/>
-      <c r="M28" s="6" t="inlineStr"/>
-      <c r="N28" s="6" t="inlineStr"/>
-      <c r="O28" s="6" t="inlineStr"/>
-      <c r="P28" s="6" t="inlineStr"/>
+        <v>-0.07349838536060282</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>232.25</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>136.17</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>338262949888</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>17.637705</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>15.855564</v>
+      </c>
+      <c r="N28" s="6" t="n">
+        <v>4.3462887</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>3.2515335</v>
+      </c>
+      <c r="P28" s="6" t="n">
+        <v>0.2826555288461539</v>
+      </c>
       <c r="Q28" s="6" t="inlineStr"/>
-      <c r="R28" s="6" t="inlineStr"/>
+      <c r="R28" s="6" t="n">
+        <v>3.409029725630936</v>
+      </c>
       <c r="S28" s="4" t="inlineStr"/>
-      <c r="T28" s="4" t="inlineStr"/>
-      <c r="U28" s="4" t="inlineStr"/>
-      <c r="V28" s="4" t="inlineStr"/>
+      <c r="T28" s="4" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="U28" s="4" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="V28" s="4" t="n">
+        <v>0.28</v>
+      </c>
       <c r="W28" s="4" t="inlineStr"/>
       <c r="X28" s="4" t="inlineStr"/>
-      <c r="Y28" s="4" t="inlineStr"/>
-      <c r="Z28" s="4" t="inlineStr"/>
+      <c r="Y28" s="4" t="n">
+        <v>0.87641</v>
+      </c>
+      <c r="Z28" s="4" t="n">
+        <v>0.41567</v>
+      </c>
       <c r="AA28" s="5" t="inlineStr"/>
       <c r="AB28" s="6" t="inlineStr"/>
       <c r="AC28" s="6" t="inlineStr"/>
-      <c r="AD28" s="6" t="inlineStr"/>
-      <c r="AE28" s="6" t="inlineStr"/>
+      <c r="AD28" s="6" t="n">
+        <v>5.02246</v>
+      </c>
+      <c r="AE28" s="6" t="n">
+        <v>0.4080294422440803</v>
+      </c>
       <c r="AF28" s="6" t="inlineStr"/>
       <c r="AG28" s="6" t="inlineStr"/>
-      <c r="AH28" s="4" t="inlineStr"/>
+      <c r="AH28" s="4" t="n">
+        <v>0.0211</v>
+      </c>
       <c r="AI28" s="6" t="n">
         <v>1.355248046188624</v>
       </c>
@@ -3841,12 +4243,12 @@
       </c>
       <c r="AM28" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>roa,roe,free_cash_flow,current_ratio,quick_ratio,ev_ebitda,fcf_yield,net_debt_ebitda,interest_coverage</t>
         </is>
       </c>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3876,39 +4278,87 @@
           <t>Semiconductors</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="n">
+        <v>990.21</v>
+      </c>
       <c r="G29" s="4" t="n">
-        <v>2.139337961506753</v>
+        <v>2.139337891845174</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.1840453095332648</v>
-      </c>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
+        <v>-0.2109880478087649</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>1255</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>103.38</v>
+      </c>
       <c r="K29" s="5" t="inlineStr"/>
-      <c r="L29" s="6" t="inlineStr"/>
-      <c r="M29" s="6" t="inlineStr"/>
+      <c r="L29" s="6" t="n">
+        <v>21.691347</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>6.440829</v>
+      </c>
       <c r="N29" s="6" t="inlineStr"/>
-      <c r="O29" s="6" t="inlineStr"/>
-      <c r="P29" s="6" t="inlineStr"/>
-      <c r="Q29" s="6" t="inlineStr"/>
-      <c r="R29" s="6" t="inlineStr"/>
+      <c r="O29" s="6" t="n">
+        <v>11.099143</v>
+      </c>
+      <c r="P29" s="6" t="n">
+        <v>0.01585045451223968</v>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>16.10463454028702</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>12.17061872860381</v>
+      </c>
       <c r="S29" s="4" t="inlineStr"/>
-      <c r="T29" s="4" t="inlineStr"/>
-      <c r="U29" s="4" t="inlineStr"/>
-      <c r="V29" s="4" t="inlineStr"/>
-      <c r="W29" s="4" t="inlineStr"/>
-      <c r="X29" s="4" t="inlineStr"/>
-      <c r="Y29" s="4" t="inlineStr"/>
-      <c r="Z29" s="4" t="inlineStr"/>
-      <c r="AA29" s="5" t="inlineStr"/>
-      <c r="AB29" s="6" t="inlineStr"/>
-      <c r="AC29" s="6" t="inlineStr"/>
-      <c r="AD29" s="6" t="inlineStr"/>
-      <c r="AE29" s="6" t="inlineStr"/>
-      <c r="AF29" s="6" t="inlineStr"/>
-      <c r="AG29" s="6" t="inlineStr"/>
-      <c r="AH29" s="4" t="inlineStr"/>
+      <c r="T29" s="4" t="n">
+        <v>3.457</v>
+      </c>
+      <c r="U29" s="4" t="n">
+        <v>13.685</v>
+      </c>
+      <c r="V29" s="4" t="n">
+        <v>3.457</v>
+      </c>
+      <c r="W29" s="4" t="n">
+        <v>0.3487</v>
+      </c>
+      <c r="X29" s="4" t="n">
+        <v>0.66638</v>
+      </c>
+      <c r="Y29" s="4" t="n">
+        <v>0.7256899999999999</v>
+      </c>
+      <c r="Z29" s="4" t="n">
+        <v>0.80370003</v>
+      </c>
+      <c r="AA29" s="5" t="n">
+        <v>7639499776</v>
+      </c>
+      <c r="AB29" s="6" t="n">
+        <v>3.425</v>
+      </c>
+      <c r="AC29" s="6" t="n">
+        <v>2.927</v>
+      </c>
+      <c r="AD29" s="6" t="n">
+        <v>0.0633</v>
+      </c>
+      <c r="AE29" s="6" t="n">
+        <v>0.07700669098287398</v>
+      </c>
+      <c r="AF29" s="6" t="n">
+        <v>-0.287971626575836</v>
+      </c>
+      <c r="AG29" s="6" t="n">
+        <v>21.23899371069182</v>
+      </c>
+      <c r="AH29" s="4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
       <c r="AI29" s="6" t="n">
         <v>2.781603638391837</v>
       </c>
@@ -3925,12 +4375,12 @@
       </c>
       <c r="AM29" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>market_cap,ps,fcf_yield</t>
         </is>
       </c>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3960,39 +4410,93 @@
           <t>Software - Application</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="n">
+        <v>91.94</v>
+      </c>
       <c r="G30" s="4" t="n">
-        <v>-0.3764665693843386</v>
+        <v>-0.3764665859418584</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.5385371823670286</v>
-      </c>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="6" t="inlineStr"/>
-      <c r="M30" s="6" t="inlineStr"/>
-      <c r="N30" s="6" t="inlineStr"/>
-      <c r="O30" s="6" t="inlineStr"/>
-      <c r="P30" s="6" t="inlineStr"/>
-      <c r="Q30" s="6" t="inlineStr"/>
-      <c r="R30" s="6" t="inlineStr"/>
-      <c r="S30" s="4" t="inlineStr"/>
-      <c r="T30" s="4" t="inlineStr"/>
-      <c r="U30" s="4" t="inlineStr"/>
-      <c r="V30" s="4" t="inlineStr"/>
-      <c r="W30" s="4" t="inlineStr"/>
-      <c r="X30" s="4" t="inlineStr"/>
-      <c r="Y30" s="4" t="inlineStr"/>
-      <c r="Z30" s="4" t="inlineStr"/>
-      <c r="AA30" s="5" t="inlineStr"/>
-      <c r="AB30" s="6" t="inlineStr"/>
-      <c r="AC30" s="6" t="inlineStr"/>
-      <c r="AD30" s="6" t="inlineStr"/>
-      <c r="AE30" s="6" t="inlineStr"/>
-      <c r="AF30" s="6" t="inlineStr"/>
-      <c r="AG30" s="6" t="inlineStr"/>
-      <c r="AH30" s="4" t="inlineStr"/>
+        <v>-0.5626070409134158</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>210.2</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>81.23999999999999</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>95053275136</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>59.7013</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>18.372715</v>
+      </c>
+      <c r="N30" s="6" t="n">
+        <v>6.4521637</v>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>8.084770000000001</v>
+      </c>
+      <c r="P30" s="6" t="n">
+        <v>-2.776804651162791</v>
+      </c>
+      <c r="Q30" s="6" t="n">
+        <v>33.67923961616968</v>
+      </c>
+      <c r="R30" s="6" t="n">
+        <v>6.691497067538471</v>
+      </c>
+      <c r="S30" s="4" t="n">
+        <v>0.0521983601396272</v>
+      </c>
+      <c r="T30" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U30" s="4" t="n">
+        <v>-0.215</v>
+      </c>
+      <c r="V30" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="W30" s="4" t="n">
+        <v>0.04319</v>
+      </c>
+      <c r="X30" s="4" t="n">
+        <v>0.14244</v>
+      </c>
+      <c r="Y30" s="4" t="n">
+        <v>0.74768996</v>
+      </c>
+      <c r="Z30" s="4" t="n">
+        <v>0.04063</v>
+      </c>
+      <c r="AA30" s="5" t="n">
+        <v>4961625088</v>
+      </c>
+      <c r="AB30" s="6" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="AC30" s="6" t="n">
+        <v>0.5649999999999999</v>
+      </c>
+      <c r="AD30" s="6" t="n">
+        <v>0.67538</v>
+      </c>
+      <c r="AE30" s="6" t="n">
+        <v>0.3246409168138874</v>
+      </c>
+      <c r="AF30" s="6" t="n">
+        <v>1.294499524821329</v>
+      </c>
+      <c r="AG30" s="6" t="n">
+        <v>99.30434782608695</v>
+      </c>
+      <c r="AH30" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI30" s="6" t="n">
         <v>0.7163484028029702</v>
       </c>
@@ -4007,14 +4511,10 @@
           <t>2026-07-22 (C)</t>
         </is>
       </c>
-      <c r="AM30" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4059,77 +4559,71 @@
       <c r="J31" s="3" t="n">
         <v>23.11</v>
       </c>
-      <c r="K31" s="5" t="n">
-        <v>142542994400</v>
-      </c>
+      <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="6" t="n">
-        <v>19.09160305343512</v>
+        <v>18.94697</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>8.50029739145212</v>
-      </c>
-      <c r="N31" s="6" t="n">
-        <v>2.251330559898918</v>
-      </c>
+        <v>8.827225</v>
+      </c>
+      <c r="N31" s="6" t="inlineStr"/>
       <c r="O31" s="6" t="n">
-        <v>1.579692900189787</v>
+        <v>1.5819101</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-3.317166030534352</v>
+        <v>-1.875937623762376</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>12.25788120372582</v>
+        <v>7.639281089278559</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.2424385122009</v>
-      </c>
-      <c r="S31" s="4" t="n">
-        <v>0.06653431155926383</v>
-      </c>
+        <v>3.071880253832314</v>
+      </c>
+      <c r="S31" s="4" t="inlineStr"/>
       <c r="T31" s="4" t="n">
-        <v>-0.01647099501783833</v>
+        <v>0.054</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>1.163419117647059</v>
+        <v>-0.101</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.0129447447226706</v>
+        <v>0.054</v>
       </c>
       <c r="W31" s="4" t="n">
-        <v>0.03608068664566656</v>
+        <v>0.05687</v>
       </c>
       <c r="X31" s="4" t="n">
-        <v>0.08368126052508847</v>
+        <v>0.083100006</v>
       </c>
       <c r="Y31" s="4" t="n">
-        <v>0.6934691621258785</v>
+        <v>0.74801004</v>
       </c>
       <c r="Z31" s="4" t="n">
-        <v>0.234462607596936</v>
+        <v>0.31617</v>
       </c>
       <c r="AA31" s="5" t="n">
-        <v>9076000000</v>
+        <v>12376625152</v>
       </c>
       <c r="AB31" s="6" t="n">
-        <v>1.246710143239781</v>
+        <v>1.247</v>
       </c>
       <c r="AC31" s="6" t="n">
-        <v>0.9361534878304414</v>
+        <v>0.852</v>
       </c>
       <c r="AD31" s="6" t="n">
-        <v>0.7153638694354114</v>
+        <v>0.71602</v>
       </c>
       <c r="AE31" s="6" t="n">
-        <v>0.3104499609860417</v>
+        <v>0.3109675289777095</v>
       </c>
       <c r="AF31" s="6" t="n">
-        <v>3.746835443037975</v>
+        <v>2.028672401334627</v>
       </c>
       <c r="AG31" s="6" t="n">
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06877249100359856</v>
+        <v>0.0693</v>
       </c>
       <c r="AI31" s="6" t="n">
         <v>0.2812004232508987</v>
@@ -4145,10 +4639,14 @@
           <t>2026-08-04 (C)</t>
         </is>
       </c>
-      <c r="AM31" s="2" t="inlineStr"/>
+      <c r="AM31" s="2" t="inlineStr">
+        <is>
+          <t>market_cap,ps,fcf_yield</t>
+        </is>
+      </c>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4178,39 +4676,93 @@
           <t>Semiconductors</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="n">
+        <v>169.5</v>
+      </c>
       <c r="G32" s="4" t="n">
         <v>0.008868552716388756</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1259282095685167</v>
-      </c>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="5" t="inlineStr"/>
-      <c r="L32" s="6" t="inlineStr"/>
-      <c r="M32" s="6" t="inlineStr"/>
-      <c r="N32" s="6" t="inlineStr"/>
-      <c r="O32" s="6" t="inlineStr"/>
-      <c r="P32" s="6" t="inlineStr"/>
-      <c r="Q32" s="6" t="inlineStr"/>
-      <c r="R32" s="6" t="inlineStr"/>
-      <c r="S32" s="4" t="inlineStr"/>
-      <c r="T32" s="4" t="inlineStr"/>
-      <c r="U32" s="4" t="inlineStr"/>
-      <c r="V32" s="4" t="inlineStr"/>
-      <c r="W32" s="4" t="inlineStr"/>
-      <c r="X32" s="4" t="inlineStr"/>
-      <c r="Y32" s="4" t="inlineStr"/>
-      <c r="Z32" s="4" t="inlineStr"/>
-      <c r="AA32" s="5" t="inlineStr"/>
-      <c r="AB32" s="6" t="inlineStr"/>
-      <c r="AC32" s="6" t="inlineStr"/>
-      <c r="AD32" s="6" t="inlineStr"/>
-      <c r="AE32" s="6" t="inlineStr"/>
-      <c r="AF32" s="6" t="inlineStr"/>
-      <c r="AG32" s="6" t="inlineStr"/>
-      <c r="AH32" s="4" t="inlineStr"/>
+        <v>-0.1298767967145791</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>194.8</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>145.57</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>1203203997696</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>23.092642</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>4.1879773</v>
+      </c>
+      <c r="N32" s="6" t="n">
+        <v>0.009109397</v>
+      </c>
+      <c r="O32" s="6" t="n">
+        <v>10.89052</v>
+      </c>
+      <c r="P32" s="6" t="n">
+        <v>0.0582265305093293</v>
+      </c>
+      <c r="Q32" s="6" t="n">
+        <v>-0.3407122419152309</v>
+      </c>
+      <c r="R32" s="6" t="n">
+        <v>-0.2365152323649665</v>
+      </c>
+      <c r="S32" s="4" t="n">
+        <v>21.45027287330613</v>
+      </c>
+      <c r="T32" s="4" t="n">
+        <v>1.981</v>
+      </c>
+      <c r="U32" s="4" t="n">
+        <v>3.966</v>
+      </c>
+      <c r="V32" s="4" t="n">
+        <v>1.981</v>
+      </c>
+      <c r="W32" s="4" t="n">
+        <v>0.27888</v>
+      </c>
+      <c r="X32" s="4" t="n">
+        <v>0.61172</v>
+      </c>
+      <c r="Y32" s="4" t="n">
+        <v>0.68342</v>
+      </c>
+      <c r="Z32" s="4" t="n">
+        <v>0.71535003</v>
+      </c>
+      <c r="AA32" s="5" t="n">
+        <v>25809054072832</v>
+      </c>
+      <c r="AB32" s="6" t="n">
+        <v>2.617</v>
+      </c>
+      <c r="AC32" s="6" t="n">
+        <v>2.174</v>
+      </c>
+      <c r="AD32" s="6" t="n">
+        <v>0.13282</v>
+      </c>
+      <c r="AE32" s="6" t="n">
+        <v>0.1239719822524244</v>
+      </c>
+      <c r="AF32" s="6" t="n">
+        <v>-0.3547735761451565</v>
+      </c>
+      <c r="AG32" s="6" t="n">
+        <v>55.63395918385022</v>
+      </c>
+      <c r="AH32" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="inlineStr"/>
       <c r="AK32" s="5" t="n">
@@ -4223,12 +4775,12 @@
       </c>
       <c r="AM32" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield,vol_2m_annualized,beta</t>
+          <t>vol_2m_annualized,beta</t>
         </is>
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4248,25 +4800,23 @@
           <t>Semiconductor ETF</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Financial Services</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Asset Management</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="3" t="n">
+        <v>580.17</v>
+      </c>
       <c r="G33" s="4" t="n">
-        <v>0.5541655555368437</v>
+        <v>0.5541656013172997</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1326635777565256</v>
-      </c>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
+        <v>-0.1364333239063454</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>671.83</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>279.19</v>
+      </c>
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4290,7 +4840,9 @@
       <c r="AE33" s="6" t="inlineStr"/>
       <c r="AF33" s="6" t="inlineStr"/>
       <c r="AG33" s="6" t="inlineStr"/>
-      <c r="AH33" s="4" t="inlineStr"/>
+      <c r="AH33" s="4" t="n">
+        <v>0.0017</v>
+      </c>
       <c r="AI33" s="6" t="n">
         <v>1.778928160518249</v>
       </c>
@@ -4303,12 +4855,12 @@
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>market_cap,pe_trailing,pe_forward,ps,pb,rev_growth_ttm,fwd_eps_growth,fwd_rev_growth,roa,roe,free_cash_flow,current_ratio,quick_ratio,debt_equity,gross_margin,operating_margin,ev_ebitda,ev_sales,fcf_yield,debt_assets,net_debt_ebitda,interest_coverage,peg</t>
         </is>
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4338,39 +4890,79 @@
           <t>Aerospace &amp; Defense</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="n">
+        <v>118.24</v>
+      </c>
       <c r="G34" s="4" t="n">
-        <v>-0.2653619129810062</v>
+        <v>-0.2653618997083718</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.4406547225262936</v>
-      </c>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="5" t="inlineStr"/>
+        <v>-0.4759794362701648</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>225.64</v>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>110.85</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>1557715877888</v>
+      </c>
       <c r="L34" s="6" t="inlineStr"/>
-      <c r="M34" s="6" t="inlineStr"/>
-      <c r="N34" s="6" t="inlineStr"/>
-      <c r="O34" s="6" t="inlineStr"/>
+      <c r="M34" s="6" t="n">
+        <v>130.9413</v>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>80.70649</v>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>19.85225</v>
+      </c>
       <c r="P34" s="6" t="inlineStr"/>
-      <c r="Q34" s="6" t="inlineStr"/>
-      <c r="R34" s="6" t="inlineStr"/>
+      <c r="Q34" s="6" t="n">
+        <v>177.0892663545757</v>
+      </c>
+      <c r="R34" s="6" t="n">
+        <v>36.24178306415023</v>
+      </c>
       <c r="S34" s="4" t="inlineStr"/>
-      <c r="T34" s="4" t="inlineStr"/>
+      <c r="T34" s="4" t="n">
+        <v>0.154</v>
+      </c>
       <c r="U34" s="4" t="inlineStr"/>
-      <c r="V34" s="4" t="inlineStr"/>
+      <c r="V34" s="4" t="n">
+        <v>0.154</v>
+      </c>
       <c r="W34" s="4" t="inlineStr"/>
       <c r="X34" s="4" t="inlineStr"/>
-      <c r="Y34" s="4" t="inlineStr"/>
-      <c r="Z34" s="4" t="inlineStr"/>
+      <c r="Y34" s="4" t="n">
+        <v>0.48826</v>
+      </c>
+      <c r="Z34" s="4" t="n">
+        <v>-0.41627997</v>
+      </c>
       <c r="AA34" s="5" t="inlineStr"/>
-      <c r="AB34" s="6" t="inlineStr"/>
-      <c r="AC34" s="6" t="inlineStr"/>
-      <c r="AD34" s="6" t="inlineStr"/>
-      <c r="AE34" s="6" t="inlineStr"/>
-      <c r="AF34" s="6" t="inlineStr"/>
-      <c r="AG34" s="6" t="inlineStr"/>
-      <c r="AH34" s="4" t="inlineStr"/>
+      <c r="AB34" s="6" t="n">
+        <v>1.217</v>
+      </c>
+      <c r="AC34" s="6" t="n">
+        <v>1.088</v>
+      </c>
+      <c r="AD34" s="6" t="n">
+        <v>0.7359699999999999</v>
+      </c>
+      <c r="AE34" s="6" t="n">
+        <v>0.3323559096862477</v>
+      </c>
+      <c r="AF34" s="6" t="n">
+        <v>1.753923734556395</v>
+      </c>
+      <c r="AG34" s="6" t="n">
+        <v>-1.169151670951157</v>
+      </c>
+      <c r="AH34" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
         <v>1.06153345183076</v>
@@ -4385,12 +4977,12 @@
       </c>
       <c r="AM34" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield,beta</t>
+          <t>pe_trailing,fwd_eps_growth,roa,roe,free_cash_flow,beta,fcf_yield,peg</t>
         </is>
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4412,20 +5004,30 @@
       </c>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="n">
+        <v>738.1799999999999</v>
+      </c>
       <c r="G35" s="4" t="n">
-        <v>0.08052170198007569</v>
+        <v>0.08052171270100739</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02816068886630918</v>
-      </c>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
+        <v>-0.02922146238821677</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>760.4</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>619.29</v>
+      </c>
       <c r="K35" s="5" t="inlineStr"/>
-      <c r="L35" s="6" t="inlineStr"/>
+      <c r="L35" s="6" t="n">
+        <v>26.552456</v>
+      </c>
       <c r="M35" s="6" t="inlineStr"/>
       <c r="N35" s="6" t="inlineStr"/>
-      <c r="O35" s="6" t="inlineStr"/>
+      <c r="O35" s="6" t="n">
+        <v>1.7198173</v>
+      </c>
       <c r="P35" s="6" t="inlineStr"/>
       <c r="Q35" s="6" t="inlineStr"/>
       <c r="R35" s="6" t="inlineStr"/>
@@ -4444,7 +5046,9 @@
       <c r="AE35" s="6" t="inlineStr"/>
       <c r="AF35" s="6" t="inlineStr"/>
       <c r="AG35" s="6" t="inlineStr"/>
-      <c r="AH35" s="4" t="inlineStr"/>
+      <c r="AH35" s="4" t="n">
+        <v>0.0101</v>
+      </c>
       <c r="AI35" s="6" t="n">
         <v>0.9969070917509125</v>
       </c>
@@ -4457,12 +5061,12 @@
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>market_cap,pe_forward,ps,rev_growth_ttm,fwd_eps_growth,fwd_rev_growth,roa,roe,free_cash_flow,current_ratio,quick_ratio,debt_equity,gross_margin,operating_margin,ev_ebitda,ev_sales,fcf_yield,debt_assets,net_debt_ebitda,interest_coverage,peg</t>
         </is>
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4482,46 +5086,108 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductors</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>415.58</v>
+      </c>
       <c r="G36" s="4" t="n">
-        <v>0.3002722243334752</v>
+        <v>0.3002722663463502</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1298030022850002</v>
-      </c>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="5" t="inlineStr"/>
-      <c r="L36" s="6" t="inlineStr"/>
-      <c r="M36" s="6" t="inlineStr"/>
-      <c r="N36" s="6" t="inlineStr"/>
-      <c r="O36" s="6" t="inlineStr"/>
-      <c r="P36" s="6" t="inlineStr"/>
-      <c r="Q36" s="6" t="inlineStr"/>
-      <c r="R36" s="6" t="inlineStr"/>
-      <c r="S36" s="4" t="inlineStr"/>
-      <c r="T36" s="4" t="inlineStr"/>
-      <c r="U36" s="4" t="inlineStr"/>
-      <c r="V36" s="4" t="inlineStr"/>
-      <c r="W36" s="4" t="inlineStr"/>
-      <c r="X36" s="4" t="inlineStr"/>
-      <c r="Y36" s="4" t="inlineStr"/>
-      <c r="Z36" s="4" t="inlineStr"/>
-      <c r="AA36" s="5" t="inlineStr"/>
-      <c r="AB36" s="6" t="inlineStr"/>
-      <c r="AC36" s="6" t="inlineStr"/>
-      <c r="AD36" s="6" t="inlineStr"/>
-      <c r="AE36" s="6" t="inlineStr"/>
-      <c r="AF36" s="6" t="inlineStr"/>
-      <c r="AG36" s="6" t="inlineStr"/>
-      <c r="AH36" s="4" t="inlineStr"/>
+        <v>-0.1324008350730689</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>479</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>223.7</v>
+      </c>
+      <c r="K36" s="5" t="n">
+        <v>2155394760704</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>37.039215</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>19.519257</v>
+      </c>
+      <c r="N36" s="6" t="n">
+        <v>0.48539543</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>86.56834000000001</v>
+      </c>
+      <c r="P36" s="6" t="n">
+        <v>0.4785428294573643</v>
+      </c>
+      <c r="Q36" s="6" t="n">
+        <v>4.645126008203918</v>
+      </c>
+      <c r="R36" s="6" t="n">
+        <v>3.321545953884065</v>
+      </c>
+      <c r="S36" s="4" t="n">
+        <v>0.3428875327870831</v>
+      </c>
+      <c r="T36" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="U36" s="4" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="V36" s="4" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="W36" s="4" t="n">
+        <v>0.19014</v>
+      </c>
+      <c r="X36" s="4" t="n">
+        <v>0.39969003</v>
+      </c>
+      <c r="Y36" s="4" t="n">
+        <v>0.6423</v>
+      </c>
+      <c r="Z36" s="4" t="n">
+        <v>0.60344005</v>
+      </c>
+      <c r="AA36" s="5" t="n">
+        <v>739057991680</v>
+      </c>
+      <c r="AB36" s="6" t="n">
+        <v>2.458</v>
+      </c>
+      <c r="AC36" s="6" t="n">
+        <v>2.131</v>
+      </c>
+      <c r="AD36" s="6" t="n">
+        <v>0.15174</v>
+      </c>
+      <c r="AE36" s="6" t="n">
+        <v>0.1238455232499574</v>
+      </c>
+      <c r="AF36" s="6" t="n">
+        <v>-0.7985480294951375</v>
+      </c>
+      <c r="AG36" s="6" t="n">
+        <v>166.043547500485</v>
+      </c>
+      <c r="AH36" s="4" t="n">
+        <v>0.009000000000000001</v>
+      </c>
       <c r="AI36" s="6" t="n">
         <v>2.160431722849606</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.5297684711135789</v>
+        <v>0.5297684711135791</v>
       </c>
       <c r="AK36" s="5" t="n">
         <v>6378408983.253886</v>
@@ -4531,14 +5197,10 @@
           <t>2026-10-15 (E)</t>
         </is>
       </c>
-      <c r="AM36" s="2" t="inlineStr">
-        <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+      <c r="AM36" s="2" t="inlineStr"/>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4558,41 +5220,97 @@
           <t>Warner Bros. Discovery</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="3" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>25.95</v>
+      </c>
       <c r="G37" s="4" t="n">
-        <v>-0.08979303561523633</v>
+        <v>-0.08979306237565188</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.1344229099676718</v>
-      </c>
-      <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr"/>
+        <v>-0.135</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>65060200448</v>
+      </c>
       <c r="L37" s="6" t="inlineStr"/>
-      <c r="M37" s="6" t="inlineStr"/>
-      <c r="N37" s="6" t="inlineStr"/>
-      <c r="O37" s="6" t="inlineStr"/>
+      <c r="M37" s="6" t="n">
+        <v>186.56985</v>
+      </c>
+      <c r="N37" s="6" t="n">
+        <v>1.74846</v>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>1.996922</v>
+      </c>
       <c r="P37" s="6" t="inlineStr"/>
-      <c r="Q37" s="6" t="inlineStr"/>
-      <c r="R37" s="6" t="inlineStr"/>
-      <c r="S37" s="4" t="inlineStr"/>
-      <c r="T37" s="4" t="inlineStr"/>
+      <c r="Q37" s="6" t="n">
+        <v>12.57373380590717</v>
+      </c>
+      <c r="R37" s="6" t="n">
+        <v>2.562730276153609</v>
+      </c>
+      <c r="S37" s="4" t="n">
+        <v>0.2838428911198918</v>
+      </c>
+      <c r="T37" s="4" t="n">
+        <v>-0.01</v>
+      </c>
       <c r="U37" s="4" t="inlineStr"/>
-      <c r="V37" s="4" t="inlineStr"/>
-      <c r="W37" s="4" t="inlineStr"/>
-      <c r="X37" s="4" t="inlineStr"/>
-      <c r="Y37" s="4" t="inlineStr"/>
-      <c r="Z37" s="4" t="inlineStr"/>
-      <c r="AA37" s="5" t="inlineStr"/>
-      <c r="AB37" s="6" t="inlineStr"/>
-      <c r="AC37" s="6" t="inlineStr"/>
-      <c r="AD37" s="6" t="inlineStr"/>
-      <c r="AE37" s="6" t="inlineStr"/>
-      <c r="AF37" s="6" t="inlineStr"/>
-      <c r="AG37" s="6" t="inlineStr"/>
-      <c r="AH37" s="4" t="inlineStr"/>
+      <c r="V37" s="4" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="W37" s="4" t="n">
+        <v>0.01391</v>
+      </c>
+      <c r="X37" s="4" t="n">
+        <v>-0.049590003</v>
+      </c>
+      <c r="Y37" s="4" t="n">
+        <v>0.45748</v>
+      </c>
+      <c r="Z37" s="4" t="n">
+        <v>0.08590999000000001</v>
+      </c>
+      <c r="AA37" s="5" t="n">
+        <v>18466875392</v>
+      </c>
+      <c r="AB37" s="6" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="AC37" s="6" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="AD37" s="6" t="n">
+        <v>0.9631799999999999</v>
+      </c>
+      <c r="AE37" s="6" t="n">
+        <v>0.3243842720887246</v>
+      </c>
+      <c r="AF37" s="6" t="n">
+        <v>3.846255257383966</v>
+      </c>
+      <c r="AG37" s="6" t="n">
+        <v>1.786091127098321</v>
+      </c>
+      <c r="AH37" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI37" s="6" t="n">
         <v>0.3849182622219184</v>
       </c>
@@ -4609,12 +5327,12 @@
       </c>
       <c r="AM37" s="2" t="inlineStr">
         <is>
-          <t>last_price,fifty_two_week_high,fifty_two_week_low,market_cap,pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_rev_growth,fwd_eps_growth,pe_forward,dividend_yield</t>
+          <t>pe_trailing,fwd_eps_growth,peg</t>
         </is>
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24 07:22 UTC</t>
+          <t>2026-07-24 07:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-06)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="23" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,55 +699,55 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>308.72</v>
+        <v>314.99</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1391461159201737</v>
+        <v>0.1622817927367695</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.1040427199117741</v>
+        <v>-0.08584612705691141</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>205.59</v>
+        <v>216.58</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4534280544320</v>
+        <v>4626370266440</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>35.24200913242009</v>
+        <v>35.95776255707763</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.57844596844897</v>
+        <v>33.23255636314989</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>9.713061576486162</v>
+        <v>9.910330610188444</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>42.18632097098215</v>
+        <v>43.04311104771206</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.076839167935057</v>
+        <v>1.09870941146626</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>27.17759068599171</v>
+        <v>27.72416263926973</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>9.808950168093688</v>
+        <v>10.00621920179597</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.03164382940083779</v>
+        <v>0.03101394651457711</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08175844748858441</v>
+        <v>0.08200410958904136</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1020173248967291</v>
+        <v>0.1022711330906769</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003401140191759523</v>
+        <v>0.003333439156798628</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.386626448128422</v>
+        <v>0.3846459586013681</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3717022610242396</v>
+        <v>0.3717774222414754</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>19764858860.69354</v>
+        <v>19588034381.74794</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>489.185</v>
+        <v>494.1</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.03434896070269788</v>
+        <v>0.04474139943621136</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.116548074839269</v>
+        <v>-0.1076717474535867</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3632467676750</v>
+        <v>3668964255000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.17694444444444</v>
+        <v>27.45</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.47401614619643</v>
+        <v>24.70764273623628</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>10.94647602789606</v>
+        <v>11.05645887011472</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.214878296604557</v>
+        <v>8.297415837264657</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8632305555555541</v>
+        <v>0.8719037122969822</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.02408916109368</v>
+        <v>18.19996026869829</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.27155324907862</v>
+        <v>11.38153609129729</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01844118277034582</v>
+        <v>0.01825774124365243</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1104407336377475</v>
+        <v>0.1109922663622527</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1966394991521756</v>
+        <v>0.1972693910692456</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007277410386663533</v>
+        <v>0.00720501922687715</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5760777825389296</v>
+        <v>0.5768365695990306</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4927507717255352</v>
+        <v>0.4879930156636278</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>17938591849.67397</v>
+        <v>17759024163.25782</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -953,55 +953,55 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>365.66</v>
+        <v>360.68</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1602729083983623</v>
+        <v>0.1444709090442522</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1051124544186388</v>
+        <v>-0.1173001150241061</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>193.67</v>
+        <v>194.33</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4425258012839</v>
+        <v>4364989498634</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>18.14523386295928</v>
+        <v>17.90863952333664</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.33495045940098</v>
+        <v>21.062096992102</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.917737036312548</v>
+        <v>9.788420480685483</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.933116282335124</v>
+        <v>6.84271590057457</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1613666200946098</v>
+        <v>0.1592625728716992</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.75172651754308</v>
+        <v>13.57469430815894</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>10.04521105713177</v>
+        <v>9.915894501504708</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01204547634332806</v>
+        <v>0.0122046112634799</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1512636492980362</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1495066324391761</v>
+        <v>-0.1497219137271975</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2572752599769641</v>
+        <v>0.2586948649019996</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>1110.671328671329</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002324563802439424</v>
+        <v>0.002356659642896751</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8125247459494371</v>
+        <v>0.8173779763439065</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.4123019863702714</v>
+        <v>0.4159484840293514</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>11777132543.23848</v>
+        <v>11696887640.42406</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>272.6405</v>
+        <v>272.81</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.2037108167770418</v>
+        <v>0.204459161147903</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.05069463788300843</v>
+        <v>-0.05010445682451248</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2932821154065</v>
+        <v>2934644451000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21.63813492063492</v>
+        <v>21.65476190476191</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.91729255620035</v>
+        <v>24.94077378221133</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.780967865698484</v>
+        <v>3.783873162902228</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.316198140023928</v>
+        <v>5.320283165947573</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2449392937716542</v>
+        <v>0.2451275078559343</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>12.11675571758722</v>
+        <v>12.12649651373835</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.967640782281353</v>
+        <v>3.970830413314769</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.003964058382881011</v>
+        <v>-0.003960716863994947</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1316016829745598</v>
+        <v>-0.1317526034333838</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1541565277808283</v>
+        <v>0.1547340207565442</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8821360486545877</v>
+        <v>0.882915211047689</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.493536095433147</v>
+        <v>0.4866525961441048</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>14167995099.53806</v>
+        <v>13894363603.04898</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>219.77</v>
+        <v>222.23</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1637277887062181</v>
+        <v>0.1767539995640115</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.07089709985626103</v>
+        <v>-0.06049716749809764</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5323049170000</v>
+        <v>5382632830000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>33.50449695121952</v>
+        <v>33.86890243902439</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.02578995395998</v>
+        <v>20.23100124330421</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21.00083032336454</v>
+        <v>21.22924198492254</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>27.30699631152993</v>
+        <v>27.60399582553179</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.3076143872129512</v>
+        <v>0.3109600984167737</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>27.58510897807949</v>
+        <v>27.88515717469037</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>20.99916162506756</v>
+        <v>21.22757328662556</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02236790073235206</v>
+        <v>0.02212723790626201</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6730674309601554</v>
+        <v>0.6741090582570088</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9037977138373157</v>
+        <v>0.9050314303479967</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001274059243754835</v>
+        <v>0.001259955901543446</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.282544644026338</v>
+        <v>1.276462202415198</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4235568096513048</v>
+        <v>0.391440497815347</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26875129651.44954</v>
+        <v>26555019214.82043</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>581.89001</v>
+        <v>589.6799999999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.1053488814343643</v>
+        <v>-0.09337183569144958</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.269211918367347</v>
+        <v>-0.2594285714285715</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>796.25</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1482356997534</v>
+        <v>1502201880598</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.62356038647343</v>
+        <v>21.91304347826087</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.43999783250871</v>
+        <v>17.67015309320113</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.494501583952543</v>
+        <v>6.581445973668992</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.664729464438158</v>
+        <v>5.740565421616179</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.432829879227049</v>
+        <v>-4.492173913043474</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.74907536549238</v>
+        <v>14.93441684658921</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6.918847032762609</v>
+        <v>7.005791422479058</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02764246404082574</v>
+        <v>0.02727729243934123</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2398832037792131</v>
+        <v>0.2401162209903129</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2443984577490095</v>
+        <v>0.245005798939522</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003608929460741215</v>
+        <v>0.003561253561253562</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8199909488101941</v>
+        <v>0.8169400510680885</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.5262856144558714</v>
+        <v>0.5074238485513695</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11688743838.74609</v>
+        <v>11640899487.55734</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>322.78</v>
+        <v>318.64001</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.263177130131376</v>
+        <v>-0.272627651579506</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.352925846480765</v>
+        <v>-0.3612252470781628</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1274834907835</v>
+        <v>1258483839479</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>273.542372881356</v>
+        <v>270.033906779661</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>156.6970395775315</v>
+        <v>154.575821071551</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>12.30309989321456</v>
+        <v>12.14529998821645</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>12.02927605977573</v>
+        <v>11.87498805371986</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.281620911912148</v>
+        <v>-7.18822653258534</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>121.9096846800845</v>
+        <v>120.3388259658949</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>12.24638249582606</v>
+        <v>12.08858259082794</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004519800928408345</v>
+        <v>0.00457852522157568</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7456767123287675</v>
+        <v>0.7469349663338753</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1060028584671424</v>
+        <v>0.1063880152747414</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.557573343687068</v>
+        <v>1.557614230413113</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.6464829881077323</v>
+        <v>0.6281992144148159</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>15123233552.99074</v>
+        <v>14852283306.25181</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>419.36</v>
+        <v>416.31</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.2063747940006384</v>
+        <v>0.1976008453128715</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.1528080808080807</v>
+        <v>-0.158969696969697</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>281.87</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1995138748800</v>
+        <v>1980628129800</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>67.74798061389338</v>
+        <v>67.25525040387723</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.81869888553815</v>
+        <v>23.61622568456319</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>26.43793478831246</v>
+        <v>26.24565202146691</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>22.70132533555325</v>
+        <v>22.5362188822114</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.5380564257451242</v>
+        <v>0.534143148135141</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>48.56492760499702</v>
+        <v>48.20718928732897</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>27.04486957662493</v>
+        <v>26.8456520214669</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01641660694245231</v>
+        <v>0.01654121715584654</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.844319118330493</v>
+        <v>1.847840772788634</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.093705193814968</v>
+        <v>1.096218800707032</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006056848531095001</v>
+        <v>0.006101222646585477</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.622088073790489</v>
+        <v>1.619772072184315</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.5202343414861017</v>
+        <v>0.4775931920169154</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8380680740.896036</v>
+        <v>8159807464.14002</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>940.75</v>
+        <v>958.0650000000001</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1009362200117028</v>
+        <v>0.1211995318899941</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1420428636570907</v>
+        <v>-0.1262517099863201</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>417202869250</v>
+        <v>424881708135</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>47.25012556504269</v>
+        <v>48.11978905072828</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.75646340419824</v>
+        <v>42.51393958253504</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.421053620391911</v>
+        <v>1.447208861887618</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.46293718851652</v>
+        <v>12.69232412172849</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.727275530063863</v>
+        <v>3.795878002349864</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.09183616102281</v>
+        <v>28.6225092007602</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.384560178924816</v>
+        <v>1.410715420420523</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02110723738748592</v>
+        <v>0.02072576868195517</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1315643546644834</v>
+        <v>0.1318590919411324</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1085967769350207</v>
+        <v>0.1088329656263007</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005888918416157321</v>
+        <v>0.005782488662042763</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1603271540145831</v>
+        <v>-0.1594268857674613</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2108168929525309</v>
+        <v>0.2149901966734876</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2299169013.684164</v>
+        <v>2272188489.927242</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>73.66</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1904604711576766</v>
+        <v>-0.1878228186064661</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.418672559387578</v>
+        <v>-0.416778470523242</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>306715820326</v>
+        <v>307715165926</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.80185758513932</v>
+        <v>22.87925696594428</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.76220799209567</v>
+        <v>19.82342318957251</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.340073126113948</v>
+        <v>6.361594080382936</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.23287456356204</v>
+        <v>10.26760937199233</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6701521558559241</v>
+        <v>0.6724269425356795</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.19328259572054</v>
+        <v>10.22730500664803</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.447784346056639</v>
+        <v>6.469305300325627</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03585110414838927</v>
+        <v>0.03572982165800696</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1538112337578588</v>
+        <v>0.1541526782306291</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1255506147365801</v>
+        <v>0.1260299792091215</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1457638670350711</v>
+        <v>0.1433494325296332</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3746090169010393</v>
+        <v>0.3746932803131314</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3445169764.092316</v>
+        <v>3379701044.894414</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1961,55 +1961,55 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>514.61</v>
+        <v>520.76001</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.03574518200324661</v>
+        <v>0.04812318326006593</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.01163884994334208</v>
+        <v>-0.007130581506196498</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>520.67</v>
+        <v>524.5</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>461.37</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1109938428523</v>
+        <v>1123203099195</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>15.3228642453111</v>
+        <v>15.50342393569515</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.20755006711678</v>
+        <v>24.49474016530513</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.957217688284842</v>
+        <v>2.992064601978188</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.52684526939216</v>
+        <v>1.544837121613271</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>-1.462885156448024</v>
+        <v>-1.480123323326419</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.88337544909322</v>
+        <v>16.04935963779298</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.191619410209007</v>
+        <v>3.224972418839938</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02150394713197892</v>
+        <v>0.02126411955156703</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.3670212721722104</v>
+        <v>-0.3670713046528036</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05106596532713525</v>
+        <v>0.05099603429197797</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.05787165877034604</v>
@@ -2048,23 +2048,23 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.08023982321606379</v>
+        <v>0.08319064917554425</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1498568873918731</v>
+        <v>0.1422642839035729</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2169158401.045127</v>
+        <v>2140275783.885311</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-08 (E)</t>
+          <t>2026-08-08 (C)</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2087,55 +2087,55 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>359.68</v>
+        <v>360.99</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.105075543379862</v>
+        <v>0.1091003681180394</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.006875224342159814</v>
+        <v>-0.005016399768473789</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>362.17</v>
+        <v>362.81</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>963766156800</v>
+        <v>967276314900</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.46345657781599</v>
+        <v>15.51977644024076</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.47514755423044</v>
+        <v>14.52731244188949</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.238102484603522</v>
+        <v>3.249896062936569</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.677642742353136</v>
+        <v>2.687395055499496</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8096549784577657</v>
+        <v>0.8126038441766816</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.82522766531268</v>
+        <v>20.86386749556928</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.356237906414947</v>
+        <v>6.368031484747995</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.1462439814944122</v>
+        <v>0.1151666781084334</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06827626591597102</v>
+        <v>0.06831710974216465</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2934417624005458</v>
+        <v>-0.2933932569364984</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01668149466192171</v>
+        <v>0.01662095902933599</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7981843719243455</v>
+        <v>0.7957799357438724</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.222696858794364</v>
+        <v>0.2226349461552244</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>3172261189.75626</v>
+        <v>3131909376.559611</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>367.57</v>
+        <v>367.06</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.06086928060765984</v>
+        <v>0.05939733422163851</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01711367221969684</v>
+        <v>-0.01847741797470392</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>373.97</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>686270543347</v>
+        <v>685318349270</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.22939677145284</v>
+        <v>31.18606627017842</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.95465520816218</v>
+        <v>24.91169999074111</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.42596977492807</v>
+        <v>15.40456638351915</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.99338177468873</v>
+        <v>19.96564114105407</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.105929716495999</v>
+        <v>2.103007758350849</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.97998293171352</v>
+        <v>23.9472592367173</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.68444397021669</v>
+        <v>15.66304057880777</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03061911982629737</v>
+        <v>0.03066166260159678</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2514457327079525</v>
+        <v>0.251864235751446</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1238931542079378</v>
+        <v>0.1241986550197929</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.00707348260195337</v>
+        <v>0.007083310630414646</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3408653166646519</v>
+        <v>0.3364477385414529</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2082242464799496</v>
+        <v>0.2075320496787526</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2878908262.693001</v>
+        <v>2844595686.628243</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>569.745</v>
+        <v>569.41998</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.01174683476254135</v>
+        <v>0.0111696678611477</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05321800687970479</v>
+        <v>-0.05375811356498328</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.77</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>499686875820</v>
+        <v>499401824132</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.28747940691927</v>
+        <v>31.26963097199341</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.21831071080503</v>
+        <v>26.19307073811419</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.24299164324602</v>
+        <v>14.23486657731665</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.55891819639993</v>
+        <v>89.5078279023347</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.382794848787949</v>
+        <v>1.382006011708637</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.19763410291192</v>
+        <v>23.18474516784228</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.62357483168486</v>
+        <v>14.61544976575549</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03291661397551892</v>
+        <v>0.03293540232574826</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.19334459614994</v>
+        <v>0.1938130998322463</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1407906596258812</v>
+        <v>0.1411573103619246</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005914926853241362</v>
+        <v>0.005918303042334412</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3304551651152626</v>
+        <v>0.3286303249742201</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2299224286819303</v>
+        <v>0.2268883039685734</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1836771065.424679</v>
+        <v>1809758680.625433</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>412.7</v>
+        <v>407.42</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.2268133397380332</v>
+        <v>0.211117738977634</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1059746111520299</v>
+        <v>-0.1174125904423552</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>239.5</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>374791195531</v>
+        <v>369996193078</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>26.53848627097936</v>
+        <v>26.19895826634944</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.35697010266234</v>
+        <v>19.10269317268544</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.8326306359532489</v>
+        <v>0.8219781286653381</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.577592853520615</v>
+        <v>3.531821856993867</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.8041230631193615</v>
+        <v>-0.7938352759294652</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>16.17246421344564</v>
+        <v>15.97894200027171</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.9256261994472695</v>
+        <v>0.9145500128918598</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06301375347555777</v>
+        <v>0.06386330409215224</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3710041463219123</v>
+        <v>0.3714798237879255</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007257539779290667</v>
+        <v>0.007336070448151988</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02168645505209595</v>
+        <v>0.02196750282264003</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.435298815529077</v>
+        <v>0.4486626012950194</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2477814811074017</v>
+        <v>0.2498294428310391</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2349001522.859894</v>
+        <v>2306768299.693392</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>152.0451</v>
+        <v>152</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.2396665153560458</v>
+        <v>0.2392988023561362</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.1381151862139335</v>
+        <v>-0.1383708406552916</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>105.53</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>630144835146</v>
+        <v>629957920000</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>19.656330749354</v>
+        <v>19.63824289405684</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.12835411837538</v>
+        <v>14.12601110240819</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.746352806735723</v>
+        <v>1.744745804021492</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.44818294062765</v>
+        <v>2.445930110262934</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.008364228738343</v>
+        <v>2.006516121784068</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.412072708152737</v>
+        <v>9.403827253478093</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.834371418600786</v>
+        <v>1.832764415886556</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04845543488740599</v>
+        <v>0.04850006489322334</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3912682669659961</v>
+        <v>0.3902185657144879</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01984632982175727</v>
+        <v>0.01908734320342931</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02683414329037898</v>
+        <v>0.0268421052631579</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4581100821283787</v>
+        <v>-0.458507316328128</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2595765035759439</v>
+        <v>0.2582881962592349</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2153713679.165254</v>
+        <v>2126419801.790039</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>258.32999</v>
+        <v>259.1</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2458643954465745</v>
+        <v>0.2495779714163557</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.06027650054565281</v>
+        <v>-0.05747544561658768</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>274.9</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>169.68</v>
+        <v>169.92</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>622549025446</v>
+        <v>624404679586</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.8647387283237</v>
+        <v>29.95375722543353</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.82988791114603</v>
+        <v>20.8864814482487</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.357146763941222</v>
+        <v>6.376095738606542</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.418555940127455</v>
+        <v>7.440668596344636</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.697726203072717</v>
+        <v>-3.708748098570131</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.40048326846079</v>
+        <v>20.45861961797049</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.649338045379816</v>
+        <v>6.668287020045135</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.03005064538748159</v>
+        <v>0.02996133855435548</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4337445720167865</v>
+        <v>0.4341217451896429</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.07913281819047824</v>
+        <v>0.07933736314218143</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.02028413348368883</v>
+        <v>0.02022385179467387</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1943561851123049</v>
+        <v>-0.1960926818558262</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2769814442102289</v>
+        <v>0.2732207304030316</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>2097948347.005574</v>
+        <v>2073907453.531087</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>112.21</v>
+        <v>113.12</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.004877635028473937</v>
+        <v>0.003192602491569607</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1697987570287067</v>
+        <v>-0.1630659958567623</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>95.42</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>892976156800</v>
+        <v>900218009600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.3719298245614</v>
+        <v>39.69122807017544</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.3101858419722</v>
+        <v>36.59248336110301</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.231173308883849</v>
+        <v>1.241157870964629</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>9.479502703275735</v>
+        <v>9.55637951871091</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>1.806476780185757</v>
+        <v>1.821126934984519</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>19.86801048630009</v>
+        <v>20.01844678119612</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.318653748147331</v>
+        <v>1.328638310228111</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01405636634798892</v>
+        <v>0.01394328914345683</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08432190338860868</v>
+        <v>0.08468254746455184</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06174055560860792</v>
+        <v>0.0618723540079813</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.008599946528829873</v>
+        <v>0.00853076379066478</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.08147538166713757</v>
+        <v>-0.08319584948381982</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.2292292001526385</v>
+        <v>0.2287976431149293</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2527101680.129823</v>
+        <v>2504261192.433465</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>145.51</v>
+        <v>147.67</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.02623603138452935</v>
+        <v>0.04146982856541426</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1299850523168909</v>
+        <v>-0.1170702541106129</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>345907672423</v>
+        <v>351042443727</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.55703703703703</v>
+        <v>21.87703703703703</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.67517227405995</v>
+        <v>20.97876044686285</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.974488376953305</v>
+        <v>4.033487036113154</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.490360608348216</v>
+        <v>6.586705731803869</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.5715724867727</v>
+        <v>20.87694391534414</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.41336559814623</v>
+        <v>17.6967367896396</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.252501061942734</v>
+        <v>4.321702864773877</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04600360520636407</v>
+        <v>0.04533070084361446</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04265332115677301</v>
+        <v>0.04281838254693038</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02190583661317436</v>
+        <v>0.02198523686095011</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3041,28 +3041,28 @@
         <v>0.4661704657052773</v>
       </c>
       <c r="AD20" s="6" t="n">
-        <v>0.6285651157224135</v>
+        <v>0.6449153946714293</v>
       </c>
       <c r="AE20" s="6" t="n">
-        <v>0.2698208202590874</v>
+        <v>0.2768394179622355</v>
       </c>
       <c r="AF20" s="6" t="n">
-        <v>1.138421003105298</v>
+        <v>1.180201373859038</v>
       </c>
       <c r="AG20" s="6" t="n">
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02948663322108446</v>
+        <v>0.02905532606487439</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05520613831183604</v>
+        <v>-0.05605543779365842</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.2428899860935055</v>
+        <v>0.219324067720031</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1322632499.176544</v>
+        <v>1310634670.355571</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>351.55</v>
+        <v>350.0601</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.01656929198549584</v>
+        <v>0.01226098139488485</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.176215582893966</v>
+        <v>-0.1797068541300528</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>350536481350</v>
+        <v>349050876732</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>24.89730878186969</v>
+        <v>24.79179178470255</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>23.52378307666057</v>
+        <v>23.42408720294156</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2.104161552475509</v>
+        <v>2.095243929672493</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>25.18673057517659</v>
+        <v>25.07998698284561</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-5.657434626280245</v>
+        <v>-5.633457917847035</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.81100935137368</v>
+        <v>16.74963341177443</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.44255715370486</v>
+        <v>2.433639530901844</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04083740426922044</v>
+        <v>0.04101121341973023</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.026340492106386</v>
+        <v>0.02645260056773108</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7220084459465473</v>
+        <v>0.7260624375582332</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2996569471214345</v>
+        <v>0.301842018044802</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1425849065.390676</v>
+        <v>1376947977.789716</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>486.59</v>
+        <v>479.98001</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.177428725743974</v>
+        <v>1.147849856258616</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1678381475210782</v>
+        <v>-0.1791424931164811</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>793433654000</v>
+        <v>782655405914</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>123.5</v>
+        <v>121.8223375634518</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>42.81881469740664</v>
+        <v>42.17249294212012</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>19.20914305774119</v>
+        <v>18.94820011896865</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.80572846007378</v>
+        <v>11.64535577040938</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9970642201834861</v>
+        <v>0.9835197895030967</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>73.95257081545064</v>
+        <v>72.94694793804814</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>19.18953284106041</v>
+        <v>18.92858946858734</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01059067756659588</v>
+        <v>0.01073652609927474</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>1.884246116403588</v>
+        <v>1.888668159376955</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.649234157906718</v>
+        <v>0.6511955426850378</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.529291256560551</v>
+        <v>2.53541412085517</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.8700659076653265</v>
+        <v>0.8273160408085457</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>15224639211.32504</v>
+        <v>15142701841.0732</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1691.63</v>
+        <v>1706.23</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4535650702152347</v>
+        <v>0.4661103963356881</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1541680833616672</v>
+        <v>-0.1468679373587471</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>685.4400000000001</v>
+        <v>706.62</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>651984636115</v>
+        <v>657611738784</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.18577648766328</v>
+        <v>53.04789550072569</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.34681265458696</v>
+        <v>36.62999516694403</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.9916691305074</v>
+        <v>15.95021167198358</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.88357235148038</v>
+        <v>25.81647071760425</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.620550167134699</v>
+        <v>3.611164104482828</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.32428978639287</v>
+        <v>41.22763394981413</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.85898213029509</v>
+        <v>15.82188861476187</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01770417963293667</v>
+        <v>0.01774534088210214</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4632858455320772</v>
+        <v>0.4482091864592337</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2322390890642383</v>
+        <v>0.2193109177472146</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004599114463564727</v>
+        <v>0.004559760407447999</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.70456594715301</v>
+        <v>1.705489452032353</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.6375675291706154</v>
+        <v>0.6174333354609256</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3550885471.017611</v>
+        <v>3484057063.506388</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>238.51</v>
+        <v>239.86</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.04715280996654747</v>
+        <v>0.05307984151010903</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.06227639080007863</v>
+        <v>-0.05696874385688999</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>188511148700</v>
+        <v>189578148200</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>89.32958801498124</v>
+        <v>89.83520599250933</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>116.7242816617387</v>
+        <v>116.628471638943</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>2.005544430022873</v>
+        <v>2.016896092345338</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>30.9298507416</v>
+        <v>31.10491802809181</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.478098537009785</v>
+        <v>0.4808046416802945</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>32.68520125179856</v>
+        <v>32.83872635971223</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.416747153571998</v>
+        <v>2.428098815894463</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>0.001299657880658811</v>
+        <v>0.001292343038088606</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2346957570160588</v>
+        <v>-0.2297317736391158</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1341442669625823</v>
+        <v>0.1345562397220488</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.200273481322471</v>
+        <v>1.204606015536247</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.391477855125865</v>
+        <v>0.3913573262511942</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1306310671.122592</v>
+        <v>1313868525.604484</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1069.83</v>
+        <v>1066.46</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.1700570559940167</v>
+        <v>0.166371337441817</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.07292957477967754</v>
+        <v>-0.07584987738195303</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>705.55</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>315607338810</v>
+        <v>314613165220</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>16.29844606946984</v>
+        <v>16.24710542352224</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.91424960024873</v>
+        <v>14.86539563301828</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.676067212240433</v>
+        <v>2.66763751172236</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.615697829593782</v>
+        <v>2.607458294634273</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3820129921835489</v>
+        <v>0.3808096385818939</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>18.03635647469181</v>
+        <v>18.00468783550473</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>4.800998319526527</v>
+        <v>4.792568619008454</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1315400337537544</v>
+        <v>-0.1319556985829558</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09281033282412188</v>
+        <v>0.0929480670823839</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3865530020385158</v>
+        <v>-0.3865077151615542</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.0158903751063253</v>
+        <v>0.01594058848901975</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.582880236068119</v>
+        <v>1.583106477131722</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.4231067486492699</v>
+        <v>0.4027671575275935</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2156307758.22076</v>
+        <v>2125812242.901123</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>235.76</v>
+        <v>232.205</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1912178387650086</v>
+        <v>-0.2034133790737563</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.290862058593515</v>
+        <v>-0.3015550742946519</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>222117511840</v>
+        <v>218768225470</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.59039301310044</v>
+        <v>20.2707423580786</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.39257935158722</v>
+        <v>18.11194947389278</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.214575333806099</v>
+        <v>3.164671424229706</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.431871125043539</v>
+        <v>6.332021072796936</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2509952946751973</v>
+        <v>0.2470987779696016</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.27498377658591</v>
+        <v>17.0565987300413</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.055422259142945</v>
+        <v>4.004154854769382</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06565893827635449</v>
+        <v>0.06672306589669542</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1194945863492254</v>
+        <v>0.1191916357373668</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04285132301333006</v>
+        <v>0.04248944256981679</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02854597896165592</v>
+        <v>0.02898301070175061</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8466461700417585</v>
+        <v>0.8457210471893238</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.8241575705830554</v>
+        <v>0.8143849901380831</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2800726030.910713</v>
+        <v>2761046659.86804</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1150.74</v>
+        <v>1195.23071</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.0651449661249115</v>
+        <v>0.1063263414102265</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.07900276121493455</v>
+        <v>-0.04339452559126011</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1249.45</v>
@@ -3868,95 +3868,95 @@
         <v>623.78</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1083699038340</v>
+        <v>1125597766788</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>40.80638297872341</v>
+        <v>40.0412298157454</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.02121150366913</v>
+        <v>29.08491543594176</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>14.9993984503699</v>
+        <v>14.12899596549586</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>32.99368324892621</v>
+        <v>31.48333438424983</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.3179550976575609</v>
+        <v>0.4244536162662864</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>33.52130256896032</v>
+        <v>33.275271721995</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>15.52657164880034</v>
+        <v>14.70588090231944</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01253106214876924</v>
+        <v>0.01781622227025708</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.456267619741572</v>
+        <v>0.376700919207912</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2958308679570139</v>
+        <v>0.1756814148408745</v>
       </c>
       <c r="W27" s="4" t="n">
-        <v>0.2168113505352731</v>
+        <v>0.1877209505000597</v>
       </c>
       <c r="X27" s="4" t="n">
-        <v>1.013034172618618</v>
+        <v>0.9257633748190075</v>
       </c>
       <c r="Y27" s="4" t="n">
-        <v>0.8350604502453304</v>
+        <v>0.8401195996274436</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>0.458655077197766</v>
+        <v>0.4392022674723658</v>
       </c>
       <c r="AA27" s="5" t="n">
         <v>8972000000</v>
       </c>
       <c r="AB27" s="6" t="n">
-        <v>1.49683354261069</v>
+        <v>1.354642759891917</v>
       </c>
       <c r="AC27" s="6" t="n">
-        <v>1.100234754599552</v>
+        <v>1.00289059718062</v>
       </c>
       <c r="AD27" s="6" t="n">
-        <v>1.390153214949676</v>
+        <v>1.620708993771953</v>
       </c>
       <c r="AE27" s="6" t="n">
-        <v>0.372031979138073</v>
+        <v>0.3859069600725315</v>
       </c>
       <c r="AF27" s="6" t="n">
-        <v>1.138147730906114</v>
+        <v>1.305328334469439</v>
       </c>
       <c r="AG27" s="6" t="n">
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.00561377895962598</v>
+        <v>0.005404814272216951</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3567908317214334</v>
+        <v>0.3512533428522081</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3208420926453294</v>
+        <v>0.3363865686017708</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3295551558.13199</v>
+        <v>3344798444.01119</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05 (C)</t>
+          <t>2026-10-29 (E)</t>
         </is>
       </c>
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3979,55 +3979,55 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>217.575</v>
+        <v>218.84</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1961242842251965</v>
+        <v>0.2030786549918053</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.06318622174381061</v>
+        <v>-0.05773950484391821</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>140.51</v>
+        <v>140.6</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>343176696000</v>
+        <v>345171949424</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.48995176848874</v>
+        <v>17.59163987138264</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.3220160121048</v>
+        <v>16.41427531049305</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.712237479154977</v>
+        <v>2.7280066184353</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.938307085937298</v>
+        <v>2.955390659250917</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4449722771869074</v>
+        <v>0.4475593847619571</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>6.237151872423076</v>
+        <v>6.305140199134494</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>1.446638288455611</v>
+        <v>1.462407427735934</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04331587830194623</v>
+        <v>-0.06818630551896036</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07155585164956157</v>
+        <v>0.07172808659648489</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3334219660070131</v>
+        <v>-0.3333243695006732</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.019073882569229</v>
+        <v>0.0189636263937123</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.367961187392582</v>
+        <v>1.366894486249764</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3206714903423809</v>
+        <v>0.3123405248563712</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1265324272.142854</v>
+        <v>1237367593.739642</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4105,55 +4105,55 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>918.5</v>
+        <v>865.24</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.9119902380907</v>
+        <v>1.743136019167771</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2681274900398406</v>
+        <v>-0.3105657370517928</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>106.75</v>
+        <v>110.79</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1037344715000</v>
+        <v>977193403600</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.49765677304173</v>
+        <v>19.30908279401919</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.14242086972414</v>
+        <v>5.777625734428271</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.49106846932672</v>
+        <v>10.82474913707158</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.28620785512887</v>
+        <v>9.689753385489059</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02921517117830272</v>
+        <v>0.02752110474721247</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>14.8701715858002</v>
+        <v>13.9921527938343</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.28481860779405</v>
+        <v>10.61849927553891</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02522980029835116</v>
+        <v>0.02678282508209923</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.337064849149989</v>
+        <v>2.342044583981682</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.679904342794524</v>
+        <v>1.683548155730969</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005770277626565053</v>
+        <v>0.0006125468078221072</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.876640046436558</v>
+        <v>2.876225958178616</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>1.188889812935463</v>
+        <v>1.136143222280222</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>47485014981.07858</v>
+        <v>45735065097.08406</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>116.185</v>
+        <v>113.58</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.212037962667553</v>
+        <v>-0.2297049687978713</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.4033411049371938</v>
+        <v>-0.4167188767807073</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>120119253946</v>
+        <v>117426047853</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>72.16459627329193</v>
+        <v>70.54658385093168</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>25.06929321175252</v>
+        <v>24.49351317485458</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>8.153628424246538</v>
+        <v>7.970815086410535</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>9.589254154682006</v>
+        <v>9.374252157238734</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>115.4633540372696</v>
+        <v>112.8745341614931</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>36.13334879507022</v>
+        <v>35.36143532616796</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>8.557511128563672</v>
+        <v>8.374697790727668</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03812877494276608</v>
+        <v>0.03900327128213904</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.878605139113418</v>
+        <v>1.880214991916958</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2227776837319932</v>
+        <v>0.2233421701988776</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6330062462221405</v>
+        <v>0.6268059552590223</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6214827323453521</v>
+        <v>0.6105260870819877</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2429901523.696314</v>
+        <v>2418608210.769268</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>25.49</v>
+        <v>25.927</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.01231134595183048</v>
+        <v>0.02966638942695621</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.1133913043478262</v>
+        <v>-0.09819130434782608</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>28.75</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>145278724296</v>
+        <v>147769381141</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>33.68128964059196</v>
+        <v>34.25872093023256</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>8.853623501374688</v>
+        <v>9.006337671392966</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.280813933308214</v>
+        <v>2.319916182193544</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.705217865946707</v>
+        <v>1.734452083577885</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.5633419240771576</v>
+        <v>-0.5729998456472526</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>16.43668601837769</v>
+        <v>16.63398139583333</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.257609964456167</v>
+        <v>3.296712213341497</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.0756201574128393</v>
+        <v>0.07434557765060458</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.804237850792088</v>
+        <v>2.803845933852704</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05332063972929635</v>
+        <v>-0.05342736347492205</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06747744213417027</v>
+        <v>0.06634010876692251</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.2857830801650935</v>
+        <v>0.3020536049117387</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2183833580043137</v>
+        <v>0.219460866094333</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1072929759.190361</v>
+        <v>1042071350.147368</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>154.53</v>
+        <v>141.89</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.08023328937307639</v>
+        <v>-0.1554669088794786</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.2067248459958932</v>
+        <v>-0.2716119096509242</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1096938763062</v>
+        <v>1007213104840</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.287966064992928</v>
+        <v>6.532079896381552</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003549268788162836</v>
+        <v>0.003256154246025604</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.259100855531923</v>
+        <v>5.609925526990542</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.530331253592596</v>
+        <v>4.060458767458592</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01630955802043272</v>
+        <v>0.01461797916099935</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.1418536037656</v>
+        <v>6.19504468936162</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.892384280655851</v>
+        <v>5.243208952114471</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07701093564563066</v>
+        <v>0.0859225690012789</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2052.371130780238</v>
+        <v>2005.072010978741</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2699.235198876185</v>
+        <v>2637.720652891315</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4561,18 +4561,18 @@
         <v>0.05327608051321153</v>
       </c>
       <c r="AF32" s="6" t="n">
-        <v>-0.4444781546983113</v>
+        <v>-0.4332891537291704</v>
       </c>
       <c r="AG32" s="6" t="n">
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.941370607649</v>
+        <v>2.114313905137783</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="inlineStr"/>
       <c r="AK32" s="5" t="n">
-        <v>7862933116.495277</v>
+        <v>7575024105.478096</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4609,13 +4609,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>574.742</v>
+        <v>570.3225</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5396250168611054</v>
+        <v>0.5277860129915124</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1445127487608473</v>
+        <v>-0.1510910498191508</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4624,7 +4624,7 @@
         <v>281.15</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>72440911587</v>
+        <v>71883874501</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4650,13 +4650,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.800997833037191</v>
+        <v>1.800537206549333</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.6220766710224563</v>
+        <v>0.575592087814537</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>7252060453.705945</v>
+        <v>7077401276.224457</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4689,13 +4689,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>114.84</v>
+        <v>109.08</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.2864864729576236</v>
+        <v>-0.3222739852857679</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.4910476865803935</v>
+        <v>-0.5165750753412515</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4704,7 +4704,7 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1501632387359</v>
+        <v>1426315402413</v>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr"/>
@@ -4731,10 +4731,10 @@
       <c r="AH34" s="4" t="inlineStr"/>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>1.001835537752792</v>
+        <v>1.032483558806966</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>10613296047.81738</v>
+        <v>10917159024.08476</v>
       </c>
       <c r="AL34" s="7" t="inlineStr"/>
       <c r="AM34" s="2" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4767,22 +4767,22 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>770.71</v>
+        <v>770.86</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1281379733883246</v>
+        <v>0.128357538070252</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.007903713715646465</v>
+        <v>-0.00643165560353165</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>776.85</v>
+        <v>775.85</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>628.13</v>
+        <v>629.11</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>820989753160</v>
+        <v>821149538894</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4808,13 +4808,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9960370618435733</v>
+        <v>0.9959988058264323</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1599091328017072</v>
+        <v>0.1454717256056127</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>37508392604.9893</v>
+        <v>36820105260.0666</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4847,13 +4847,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>415.97</v>
+        <v>415.9</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3014925035663203</v>
+        <v>0.3012734866294025</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1315866388308976</v>
+        <v>-0.1317327766179541</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4862,40 +4862,40 @@
         <v>223.7</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2157420085600</v>
+        <v>2157057032000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.87759360148371</v>
+        <v>27.41393300104324</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6614860536128594</v>
+        <v>0.6609087692369159</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.04516031106463</v>
+        <v>13.81156097117166</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.694662282328631</v>
+        <v>9.533420498007157</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5236931997876318</v>
+        <v>0.51498312577869</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.47367097003595</v>
+        <v>18.15543701118471</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.56058089959401</v>
+        <v>13.32698155970104</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01793353624589453</v>
+        <v>0.01823685186950374</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.14388716016578</v>
+        <v>40.47914852559047</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.21274280147745</v>
+        <v>40.54984589428122</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4929,16 +4929,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2644421472702358</v>
+        <v>0.2644866554460207</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.186347349716091</v>
+        <v>2.18086664873665</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.5585730619244818</v>
+        <v>0.5326121339106681</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>6243686785.349422</v>
+        <v>6183523647.051966</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -4975,13 +4975,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>25.755</v>
+        <v>26.41</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.09663276768727991</v>
+        <v>-0.07365837292258059</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.1415000000000001</v>
+        <v>-0.1196666666666667</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -4990,38 +4990,38 @@
         <v>10.76</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>64571305760</v>
+        <v>66213480300</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-37.32608695652173</v>
+        <v>-38.27536231884057</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-42.8216578478579</v>
+        <v>-44.17803470488442</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.735321305025531</v>
+        <v>1.779453918301532</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>1.970085947571981</v>
+        <v>2.020189084658359</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.06824186855009465</v>
+        <v>0.06997739267746067</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>7.411651068494233</v>
+        <v>7.538948963738347</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.521275980247245</v>
+        <v>2.564579843671056</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03575039027828587</v>
+        <v>0.03488055208685616</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.005781121027415681</v>
+        <v>0.005853367737572279</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.01774379835849423</v>
@@ -5060,13 +5060,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3239291848549887</v>
+        <v>0.3219221235187428</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2270651449577247</v>
+        <v>0.2211972406426668</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>595171174.3790557</v>
+        <v>577214425.8328384</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -5103,13 +5103,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>347.53</v>
+        <v>348.665</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.06760928887814321</v>
+        <v>-0.06456418929789587</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1031252419417277</v>
+        <v>-0.100196134093783</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5118,40 +5118,40 @@
         <v>290.63</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>234690483476</v>
+        <v>235456961150</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>21.07519708914494</v>
+        <v>21.14402668283809</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>18.17247067015142</v>
+        <v>18.22543498442209</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.791508373389792</v>
+        <v>2.800625184660949</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.873551341890315</v>
+        <v>6.895999708284715</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.306846282383662</v>
+        <v>1.311114318324461</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>10.05082039621421</v>
+        <v>10.08182175821065</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.955722806085188</v>
+        <v>2.964839617356345</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06413553620523882</v>
+        <v>0.06392675725739527</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1597320734027265</v>
+        <v>0.1601383835782586</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.003652557092572284</v>
+        <v>-0.0034187955350935</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5187,16 +5187,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01018617097804506</v>
+        <v>0.01015301220369122</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9802942405456387</v>
+        <v>0.9786850374554003</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.26923703846541</v>
+        <v>0.2687042971159443</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1074827734.09267</v>
+        <v>1061450565.171458</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5206,7 +5206,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>
@@ -5229,13 +5229,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>144.31</v>
+        <v>143.42</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2626335136200534</v>
+        <v>-0.2671810583007974</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5825812796482703</v>
+        <v>-0.5851556172625246</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5244,40 +5244,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>415680625700</v>
+        <v>413117002126</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>24.29461279461279</v>
+        <v>24.15824915824916</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.82616385799618</v>
+        <v>16.7070931876602</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.171213897384127</v>
+        <v>6.136575388224116</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>9.770494495153855</v>
+        <v>9.715653524042533</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7321214396214389</v>
+        <v>0.7280121030121024</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>16.84029710876406</v>
+        <v>16.76940041125339</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.024629833130437</v>
+        <v>7.990846595801538</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05698914417892405</v>
+        <v>-0.05730288232457806</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4438592777085926</v>
+        <v>0.4459875746723172</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4399079299622501</v>
+        <v>0.4423709970555079</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5313,16 +5313,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01385905342665096</v>
+        <v>0.01394505647747873</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>1.975457573426339</v>
+        <v>1.984007587156891</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.6397982487905387</v>
+        <v>0.5995970444910079</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>5157412717.228155</v>
+        <v>5033075057.848439</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5332,7 +5332,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 16:05 UTC</t>
+          <t>2026-08-06 13:44 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-07)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -457,7 +457,7 @@
     <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="23" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
@@ -475,7 +475,7 @@
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
     <col width="19" customWidth="1" min="39" max="39"/>
-    <col width="22" customWidth="1" min="40" max="40"/>
+    <col width="21" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>314.99</v>
+        <v>312.41</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1622817927367695</v>
+        <v>0.1527618491663041</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.08584612705691141</v>
+        <v>-0.09333372028905584</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>216.58</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4626370266440</v>
+        <v>4588476887960</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>35.95776255707763</v>
+        <v>35.66324200913242</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.23255636314989</v>
+        <v>32.95287552101639</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>9.910330610188444</v>
+        <v>9.829157706368365</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>43.04311104771206</v>
+        <v>42.69055627929689</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.09870941146626</v>
+        <v>1.089710172501267</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>27.72416263926973</v>
+        <v>27.49925743361466</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.00621920179597</v>
+        <v>9.925046297975891</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.03101394651457711</v>
+        <v>0.02978831610956815</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08200410958904136</v>
+        <v>0.08224977168949787</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1022711330906769</v>
+        <v>0.1025249412846245</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003333439156798628</v>
+        <v>0.003360967958772126</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3846459586013681</v>
+        <v>0.3838907587299467</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3717774222414754</v>
+        <v>0.3707091338325771</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>19588034381.74794</v>
+        <v>20020748900.26055</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>494.1</v>
+        <v>499.86</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.04474139943621136</v>
+        <v>0.05692053414730758</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1076717474535867</v>
+        <v>-0.09726937802499458</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3668964255000</v>
+        <v>3711735423000</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.45</v>
+        <v>27.77</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.70764273623628</v>
+        <v>24.9832710351277</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.05645887011472</v>
+        <v>11.18535019391934</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.297415837264657</v>
+        <v>8.394143453582496</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8719037122969822</v>
+        <v>0.8820679814385135</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.19996026869829</v>
+        <v>18.40606750707164</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.38153609129729</v>
+        <v>11.5104274151019</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01825774124365243</v>
+        <v>0.01804735315586097</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1109922663622527</v>
+        <v>0.1115437990867578</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1972693910692456</v>
+        <v>0.1978992770141008</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.00720501922687715</v>
+        <v>0.007121994158364342</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5768365695990306</v>
+        <v>0.5710016488474213</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4879930156636278</v>
+        <v>0.4902809155002809</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>17759024163.25782</v>
+        <v>18254306061.37064</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>360.68</v>
+        <v>357.75</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.1444709090442522</v>
+        <v>0.1351737487816935</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1173001150241061</v>
+        <v>-0.1244707667457967</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>194.33</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4364989498634</v>
+        <v>4329530312567</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.90863952333664</v>
+        <v>17.76315789473684</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>21.062096992102</v>
+        <v>20.90859551046429</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.788420480685483</v>
+        <v>9.708903812149332</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.84271590057457</v>
+        <v>6.787128794029479</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1592625728716992</v>
+        <v>0.1579687962871532</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.57469430815894</v>
+        <v>13.46583731420669</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.915894501504708</v>
+        <v>9.836377832968557</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.0122046112634799</v>
+        <v>0.01230456796788522</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1512636492980362</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1497219137271975</v>
+        <v>-0.1504375372393247</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2586948649019996</v>
+        <v>0.2593748100508146</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>1110.671328671329</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002356659642896751</v>
+        <v>0.002375960866526904</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8173779763439065</v>
+        <v>0.8193786772293544</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.4159484840293514</v>
+        <v>0.4169379229761317</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>11696887640.42406</v>
+        <v>11959283622.46055</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>272.81</v>
+        <v>272.26</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.204459161147903</v>
+        <v>0.2020309050772626</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.05010445682451248</v>
+        <v>-0.05201949860724231</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2934644451000</v>
+        <v>2928728046000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21.65476190476191</v>
+        <v>21.60793650793651</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.94077378221133</v>
+        <v>24.89847101110509</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.783873162902228</v>
+        <v>3.775691065903465</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.320283165947573</v>
+        <v>5.308778796997933</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2451275078559343</v>
+        <v>0.2445974538715656</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>12.12649651373835</v>
+        <v>12.10150925404631</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.970830413314769</v>
+        <v>3.962648316316007</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.003960716863994947</v>
+        <v>-0.003969299920447445</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1317526034333838</v>
+        <v>-0.1321580952380953</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1547340207565442</v>
+        <v>0.154972944109169</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.882915211047689</v>
+        <v>0.8862430566271959</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4866525961441048</v>
+        <v>0.486728780274467</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>13894363603.04898</v>
+        <v>14118885807.09914</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>222.23</v>
+        <v>218.99</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1767539995640115</v>
+        <v>0.1595975267269176</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.06049716749809764</v>
+        <v>-0.07419463938445925</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5382632830000</v>
+        <v>5304156790000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>33.86890243902439</v>
+        <v>33.38262195121951</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.23100124330421</v>
+        <v>19.91740692609412</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>21.22924198492254</v>
+        <v>20.92443830352952</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>27.60399582553179</v>
+        <v>27.20766516263033</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.3109600984167737</v>
+        <v>0.3064954179147056</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>27.88515717469037</v>
+        <v>27.48475820075659</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>21.22757328662556</v>
+        <v>20.92276960523253</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02212723790626201</v>
+        <v>0.02244956261935839</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6741090582570088</v>
+        <v>0.6760526144336785</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9050314303479967</v>
+        <v>0.907291481233524</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001259955901543446</v>
+        <v>0.001278597196219005</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.276462202415198</v>
+        <v>1.275912726169961</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.391440497815347</v>
+        <v>0.3904892540988242</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26555019214.82043</v>
+        <v>27272401343.27709</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>589.6799999999999</v>
+        <v>589.9</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.09337183569144958</v>
+        <v>-0.09303358749556723</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2594285714285715</v>
+        <v>-0.2591522762951335</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>796.25</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1502201880598</v>
+        <v>1502762327643</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.91304347826087</v>
+        <v>21.92121887774062</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.67015309320113</v>
+        <v>17.67342471183989</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.581445973668992</v>
+        <v>6.583901403924679</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.740565421616179</v>
+        <v>5.742707133040605</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.492173913043474</v>
+        <v>-4.493849869936823</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.93441684658921</v>
+        <v>14.93965114729341</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.005791422479058</v>
+        <v>7.008246852734745</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02727729243934123</v>
+        <v>0.02726711952133416</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2401162209903129</v>
+        <v>0.2403492382014123</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.245005798939522</v>
+        <v>0.2456131401300341</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003561253561253562</v>
+        <v>0.003559925411086625</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8169400510680885</v>
+        <v>0.8140834077965554</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.5074238485513695</v>
+        <v>0.507434903593638</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11640899487.55734</v>
+        <v>11842498202.69795</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>318.64001</v>
+        <v>319.53</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.272627651579506</v>
+        <v>-0.2705960356616847</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.3612252470781628</v>
+        <v>-0.3594410921556442</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1258483839479</v>
+        <v>1261998878805</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>270.033906779661</v>
+        <v>270.7881355932203</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>154.575821071551</v>
+        <v>154.8959991623313</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>12.14529998821645</v>
+        <v>12.17922271788958</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>11.87498805371986</v>
+        <v>11.9081559556978</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.18822653258534</v>
+        <v>-7.208303891143467</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>120.3388259658949</v>
+        <v>120.6765182827361</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>12.08858259082794</v>
+        <v>12.12250532050107</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00457852522157568</v>
+        <v>0.004565772677592311</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7469349663338753</v>
+        <v>0.7481932203389832</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1063880152747414</v>
+        <v>0.1067731720823402</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.557614230413113</v>
+        <v>1.559871908261978</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.6281992144148159</v>
+        <v>0.6281192841202774</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14852283306.25181</v>
+        <v>15088716873.26146</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>416.31</v>
+        <v>420.565</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.1976008453128715</v>
+        <v>0.2098412229084283</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.158969696969697</v>
+        <v>-0.1503737373737374</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>281.87</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1980628129800</v>
+        <v>2000871632700</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>67.25525040387723</v>
+        <v>67.94264943457189</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.61622568456319</v>
+        <v>23.82813520488734</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>26.24565202146691</v>
+        <v>26.51390224209899</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>22.5362188822114</v>
+        <v>22.76655591793912</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.534143148135141</v>
+        <v>0.5396024911615275</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>48.20718928732897</v>
+        <v>48.68889072456871</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>26.8456520214669</v>
+        <v>27.11390224209899</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01654121715584654</v>
+        <v>0.0163738640023551</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.847840772788634</v>
+        <v>1.851362427246774</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.096218800707032</v>
+        <v>1.098732407599096</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006101222646585477</v>
+        <v>0.006039494489555717</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.619772072184315</v>
+        <v>1.617307716345701</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4775931920169154</v>
+        <v>0.4773164634555489</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8159807464.14002</v>
+        <v>8320062788.725613</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>958.0650000000001</v>
+        <v>949.15</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1211995318899941</v>
+        <v>0.1107665301345817</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1262517099863201</v>
+        <v>-0.1343821249430005</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>424881708135</v>
+        <v>420928092850</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>48.11978905072828</v>
+        <v>47.67202410848819</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.51393958253504</v>
+        <v>42.10737346657685</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.447208861887618</v>
+        <v>1.433742273499848</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.69232412172849</v>
+        <v>12.57421932764332</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.795878002349864</v>
+        <v>3.760556544629408</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.6225092007602</v>
+        <v>28.34928077747063</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.410715420420523</v>
+        <v>1.397248832032753</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02072576868195517</v>
+        <v>0.02092043783625073</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1318590919411324</v>
+        <v>0.1321538292177815</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1088329656263007</v>
+        <v>0.109069154317581</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005782488662042763</v>
+        <v>0.005836801348575041</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1594268857674613</v>
+        <v>-0.1633174446231838</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2149901966734876</v>
+        <v>0.2115690285366796</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2272188489.927242</v>
+        <v>2318432045.685815</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>73.69</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1878228186064661</v>
+        <v>-0.1901307645887753</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.416778470523242</v>
+        <v>-0.4184357982795359</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>307715165926</v>
+        <v>306840738526</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>22.87925696594428</v>
+        <v>22.81424148606811</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.82342318957251</v>
+        <v>19.76392714515986</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.361594080382936</v>
+        <v>6.343516478796986</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.26760937199233</v>
+        <v>10.23843213291089</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.6724269425356795</v>
+        <v>0.6705161217246849</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>10.22730500664803</v>
+        <v>10.19872618146894</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.469305300325627</v>
+        <v>6.451227698739677</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03572982165800696</v>
+        <v>0.03583164364945751</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1541526782306291</v>
+        <v>0.1543374613003097</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1260299792091215</v>
+        <v>0.1263565194297944</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1433494325296332</v>
+        <v>0.1402016748527777</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3746932803131314</v>
+        <v>0.3748256471168486</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3379701044.894414</v>
+        <v>3442524596.671152</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -1961,55 +1961,55 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>520.76001</v>
+        <v>524.61</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.04812318326006593</v>
+        <v>0.05587198058864629</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.007130581506196498</v>
+        <v>-0.001579628501827135</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>524.5</v>
+        <v>525.4400000000001</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>461.37</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1123203099195</v>
+        <v>1131506964473</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>15.50342393569515</v>
+        <v>15.61804108365585</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.49474016530513</v>
+        <v>24.67370517017618</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.992064601978188</v>
+        <v>3.014185001553035</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.544837121613271</v>
+        <v>1.55625813581488</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>-1.480123323326419</v>
+        <v>-1.491065907019766</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>16.04935963779298</v>
+        <v>16.16687830725687</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.224972418839938</v>
+        <v>3.2485867234772</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02126411955156703</v>
+        <v>0.02109752811916487</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.3670713046528036</v>
+        <v>-0.3670167907115213</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05099603429197797</v>
+        <v>0.05109969791792079</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.05787165877034604</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.08319064917554425</v>
+        <v>0.08143344514800227</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1422642839035729</v>
+        <v>0.1440759127855735</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2140275783.885311</v>
+        <v>2211189169.084635</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>360.99</v>
+        <v>356.3</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.1091003681180394</v>
+        <v>0.09469088107830537</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.005016399768473789</v>
+        <v>-0.01794327609492574</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>362.81</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>967276314900</v>
+        <v>954709413000</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.51977644024076</v>
+        <v>15.31814273430783</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.52731244188949</v>
+        <v>14.33802470711677</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.249896062936569</v>
+        <v>3.207673251957948</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.687395055499496</v>
+        <v>2.652480285532758</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8126038441766816</v>
+        <v>0.8020464546944559</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.86386749556928</v>
+        <v>20.72553100403994</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.368031484747995</v>
+        <v>6.325808673769373</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.1151666781084334</v>
+        <v>0.0902002209545618</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06831710974216465</v>
+        <v>0.06835795356835783</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2933932569364984</v>
+        <v>-0.293344751472451</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01662095902933599</v>
+        <v>0.01683974179062588</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7957799357438724</v>
+        <v>0.7968278862993252</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.2226349461552244</v>
+        <v>0.2244212378595976</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>3131909376.559611</v>
+        <v>3194029620.459749</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>367.06</v>
+        <v>370.47</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.05939733422163851</v>
+        <v>0.06923917182229178</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01847741797470392</v>
+        <v>-0.009359039495146715</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>373.97</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>685318349270</v>
+        <v>691684980259</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.18606627017842</v>
+        <v>31.47578589634665</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.91169999074111</v>
+        <v>25.13472790229107</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.40456638351915</v>
+        <v>15.54767533400018</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>19.96564114105407</v>
+        <v>20.15112263261129</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.103007758350849</v>
+        <v>2.122544772615482</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>23.9472592367173</v>
+        <v>24.16605884455976</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.66304057880777</v>
+        <v>15.8061495292888</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03066166260159678</v>
+        <v>0.03037943659284278</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.251864235751446</v>
+        <v>0.2522827387949393</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1241986550197929</v>
+        <v>0.124504155831648</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007083310630414646</v>
+        <v>0.007018112127837611</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3364477385414529</v>
+        <v>0.3356216143173507</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2075320496787526</v>
+        <v>0.2069467950744472</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2844595686.628243</v>
+        <v>2885564932.792234</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>569.41998</v>
+        <v>575.95</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.0111696678611477</v>
+        <v>0.02276560475561129</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.05375811356498328</v>
+        <v>-0.04290675839606484</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.77</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>499401824132</v>
+        <v>505128884200</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.26963097199341</v>
+        <v>31.62822624931356</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.19307073811419</v>
+        <v>26.48305571838122</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.23486657731665</v>
+        <v>14.39810974546076</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>89.5078279023347</v>
+        <v>90.53428978791661</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.382006011708637</v>
+        <v>1.397854642268768</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.18474516784228</v>
+        <v>23.443700678242</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.61544976575549</v>
+        <v>14.77869293389961</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03293540232574826</v>
+        <v>0.03256198668197244</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1938130998322463</v>
+        <v>0.1942816035145525</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1411573103619246</v>
+        <v>0.1415239610979675</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005918303042334412</v>
+        <v>0.005851202361316086</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3286303249742201</v>
+        <v>0.327031343270233</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2268883039685734</v>
+        <v>0.2270215742210439</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1809758680.625433</v>
+        <v>1845493299.287323</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>407.42</v>
+        <v>403.97</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.211117738977634</v>
+        <v>0.2008620907535095</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1174125904423552</v>
+        <v>-0.1248862700922836</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>239.5</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>369996193078</v>
+        <v>366863094884</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>26.19895826634944</v>
+        <v>25.97710758150602</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.10269317268544</v>
+        <v>18.9343659891035</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.8219781286653381</v>
+        <v>0.8150176835618234</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.531821856993867</v>
+        <v>3.501914671763322</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7938352759294652</v>
+        <v>-0.7871131422542489</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.97894200027171</v>
+        <v>15.86473216954547</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.9145500128918598</v>
+        <v>0.908013247055844</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06386330409215224</v>
+        <v>0.06437551318010758</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3714798237879255</v>
+        <v>0.3719555012539388</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007336070448151988</v>
+        <v>0.007414601117013087</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02196750282264003</v>
+        <v>0.0221551105280095</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4486626012950194</v>
+        <v>0.4524435474950426</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2498294428310391</v>
+        <v>0.253321100487149</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2306768299.693392</v>
+        <v>2354369174.31219</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>152</v>
+        <v>154.83</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.2392988023561362</v>
+        <v>0.2623725892684248</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.1383708406552916</v>
+        <v>-0.1223286661753868</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>105.53</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>629957920000</v>
+        <v>641686741800</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>19.63824289405684</v>
+        <v>20.00387596899225</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.12601110240819</v>
+        <v>14.39089779200148</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.744745804021492</v>
+        <v>1.777230216030577</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.445930110262934</v>
+        <v>2.491469466921119</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.006516121784068</v>
+        <v>2.043874283788337</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.403827253478093</v>
+        <v>9.570503230115534</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.832764415886556</v>
+        <v>1.865248827895641</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04850006489322334</v>
+        <v>0.04761357530045823</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3902185657144879</v>
+        <v>0.3900366925064598</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01908734320342931</v>
+        <v>0.01896450366476499</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.0268421052631579</v>
+        <v>0.02635148227087774</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.458507316328128</v>
+        <v>-0.461432298885391</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2582881962592349</v>
+        <v>0.2631517622224404</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2126419801.790039</v>
+        <v>2168180197.097281</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>259.1</v>
+        <v>256.98</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2495779714163557</v>
+        <v>0.2393537132171943</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.05747544561658768</v>
+        <v>-0.06518734085121847</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>274.9</v>
@@ -2732,40 +2732,40 @@
         <v>169.92</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>624404679586</v>
+        <v>619295694944</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>29.95375722543353</v>
+        <v>29.70867052023122</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.8864814482487</v>
+        <v>20.71013797218062</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.376095738606542</v>
+        <v>6.323925445414535</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.440668596344636</v>
+        <v>7.379787788068871</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.708748098570131</v>
+        <v>-3.678402494676003</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.45861961797049</v>
+        <v>20.29855869369341</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.668287020045135</v>
+        <v>6.616116726853129</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02996133855435548</v>
+        <v>0.03020850968726931</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4341217451896429</v>
+        <v>0.4344989183624988</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.07933736314218143</v>
+        <v>0.07954190809388439</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.02022385179467387</v>
+        <v>0.02039069188263678</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1960926818558262</v>
+        <v>-0.1954423826567721</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2732207304030316</v>
+        <v>0.2733414552251205</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>2073907453.531087</v>
+        <v>2107924386.378599</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>113.12</v>
+        <v>112.07</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.003192602491569607</v>
+        <v>-0.006119210031557576</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1630659958567623</v>
+        <v>-0.1708345664397751</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>95.42</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>900218009600</v>
+        <v>891862025600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.69122807017544</v>
+        <v>39.32280701754385</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.59248336110301</v>
+        <v>36.24077578120657</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.241157870964629</v>
+        <v>1.229637222409883</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>9.55637951871091</v>
+        <v>9.467675500901093</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>1.821126934984519</v>
+        <v>1.804222910216717</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.01844678119612</v>
+        <v>19.84486644093147</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.328638310228111</v>
+        <v>1.317117661673365</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01394328914345683</v>
+        <v>0.01407392583124687</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08468254746455184</v>
+        <v>0.085043191540495</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0618723540079813</v>
+        <v>0.06200415240735468</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.00853076379066478</v>
+        <v>0.008610689747479255</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.08319584948381982</v>
+        <v>-0.08279229642429056</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.2287976431149293</v>
+        <v>0.2278871545255647</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2504261192.433465</v>
+        <v>2574961081.092968</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>147.67</v>
+        <v>146.99</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04146982856541426</v>
+        <v>0.03667400352698769</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1170702541106129</v>
+        <v>-0.121136023916293</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>351042443727</v>
+        <v>349425941650</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.87703703703703</v>
+        <v>21.7762962962963</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.97876044686285</v>
+        <v>20.87885135941797</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.033487036113154</v>
+        <v>4.014913384157551</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.586705731803869</v>
+        <v>6.556374859604868</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.87694391534414</v>
+        <v>20.78080846560869</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.6967367896396</v>
+        <v>17.62068042015621</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.321702864773877</v>
+        <v>4.303129212818273</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04533070084361446</v>
+        <v>0.04554040814731249</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04281838254693038</v>
+        <v>0.04298344393708775</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02198523686095011</v>
+        <v>0.02206463710872519</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02905532606487439</v>
+        <v>0.02918974079869379</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05605543779365842</v>
+        <v>-0.05631828247306898</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.219324067720031</v>
+        <v>0.2188479227430429</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1310634670.355571</v>
+        <v>1335460357.347847</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>350.0601</v>
+        <v>349.52</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0.01226098139488485</v>
+        <v>0.01069918627441457</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.1797068541300528</v>
+        <v>-0.1809724663151728</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>349050876732</v>
+        <v>348512333840</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>24.79179178470255</v>
+        <v>24.75354107648725</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>23.42408720294156</v>
+        <v>23.38794669593059</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2.095243929672493</v>
+        <v>2.092011224068383</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>25.07998698284561</v>
+        <v>25.04129162462159</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-5.633457917847035</v>
+        <v>-5.624766179995651</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.74963341177443</v>
+        <v>16.72738417021277</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.433639530901844</v>
+        <v>2.430406825297733</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04101121341973023</v>
+        <v>0.0410745864924595</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02645260056773108</v>
+        <v>0.02649347676813916</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7260624375582332</v>
+        <v>0.7274860428201561</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.301842018044802</v>
+        <v>0.3022299853265483</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1376947977.789716</v>
+        <v>1395144814.310217</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>479.98001</v>
+        <v>489.28</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.147849856258616</v>
+        <v>1.189466135621389</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1791424931164811</v>
+        <v>-0.1632377336548493</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>782655405914</v>
+        <v>797819968000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>121.8223375634518</v>
+        <v>124.1827411167513</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>42.17249294212012</v>
+        <v>42.92390918743777</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.94820011896865</v>
+        <v>19.31533635153129</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.64535577040938</v>
+        <v>11.87099369272879</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9835197895030967</v>
+        <v>1.002576258557258</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>72.94694793804814</v>
+        <v>74.36181824967345</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.92858946858734</v>
+        <v>19.2957261348505</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01073652609927474</v>
+        <v>0.01053245135123016</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>1.888668159376955</v>
+        <v>1.893090202350324</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.6511955426850378</v>
+        <v>0.6531569274633573</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.53541412085517</v>
+        <v>2.532996173749302</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.8273160408085457</v>
+        <v>0.8279219701785322</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>15142701841.0732</v>
+        <v>15477179454.56482</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1706.23</v>
+        <v>1704.37</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4661103963356881</v>
+        <v>0.4645121561586987</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1468679373587471</v>
+        <v>-0.1477979559591193</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>706.62</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>657611738784</v>
+        <v>656894861321</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.04789550072569</v>
+        <v>54.20899854862119</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.62999516694403</v>
+        <v>36.55963097889942</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.95021167198358</v>
+        <v>16.29932711213644</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.81647071760425</v>
+        <v>26.38153710814005</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.611164104482828</v>
+        <v>3.690204632077528</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.22763394981413</v>
+        <v>42.12596466587006</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.82188861476187</v>
+        <v>16.16664011192414</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01774534088210214</v>
+        <v>0.01737000435473076</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4482091864592337</v>
+        <v>0.4827556268253417</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2193109177472146</v>
+        <v>0.2481598887134455</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004559760407447999</v>
+        <v>0.00456473653021351</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.705489452032353</v>
+        <v>1.702105786004374</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.6174333354609256</v>
+        <v>0.6172436522624353</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3484057063.506388</v>
+        <v>3531415810.897111</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>239.86</v>
+        <v>232.19</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0.05307984151010903</v>
+        <v>0.01940552155520803</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.05696874385688999</v>
+        <v>-0.08712404167485743</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>189578148200</v>
+        <v>183516010300</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>89.83520599250933</v>
+        <v>86.96254681647937</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>116.628471638943</v>
+        <v>112.1761270031451</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>2.016896092345338</v>
+        <v>1.952401833076227</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>31.10491802809181</v>
+        <v>30.11027648187541</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4808046416802945</v>
+        <v>0.4654299581078445</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>32.83872635971223</v>
+        <v>31.96647630215827</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.428098815894463</v>
+        <v>2.363604556625353</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>0.001292343038088606</v>
+        <v>0.001335033382643236</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2297317736391158</v>
+        <v>-0.2247677902621725</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1345562397220488</v>
+        <v>0.134968212481515</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.204606015536247</v>
+        <v>1.209475610076213</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3913573262511942</v>
+        <v>0.40129935180787</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1313868525.604484</v>
+        <v>1365305984.290143</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1066.46</v>
+        <v>1032.58</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.166371337441817</v>
+        <v>0.129317288614361</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.07584987738195303</v>
+        <v>-0.1052088839591332</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>705.55</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>314613165220</v>
+        <v>304618328060</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>16.24710542352224</v>
+        <v>15.73095673369896</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.86539563301828</v>
+        <v>14.39132839746458</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.66763751172236</v>
+        <v>2.582890255475381</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.607458294634273</v>
+        <v>2.524622851183783</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3808096385818939</v>
+        <v>0.3687118284857303</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>18.00468783550473</v>
+        <v>17.68630994361801</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>4.792568619008454</v>
+        <v>4.707821362761474</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1319556985829558</v>
+        <v>-0.1362852992608602</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.0929480670823839</v>
+        <v>0.09308580134064592</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3865077151615542</v>
+        <v>-0.3864624282845927</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01594058848901975</v>
+        <v>0.01646361540994402</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.583106477131722</v>
+        <v>1.586795931367534</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.4027671575275935</v>
+        <v>0.4079763259850774</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2125812242.901123</v>
+        <v>2163723946.958618</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>232.205</v>
+        <v>233.43</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2034133790737563</v>
+        <v>-0.1992109777015437</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3015550742946519</v>
+        <v>-0.2978704205017144</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>218768225470</v>
+        <v>219922339620</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.2707423580786</v>
+        <v>20.38689956331878</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.11194947389278</v>
+        <v>18.20419297707924</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.164671424229706</v>
+        <v>3.182805905032057</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.332021072796936</v>
+        <v>6.36830538140021</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2470987779696016</v>
+        <v>0.2485147252970449</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.0565987300413</v>
+        <v>17.13965474508353</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.004154854769382</v>
+        <v>4.023652830368902</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06672306589669542</v>
+        <v>0.06631431815976239</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1191916357373668</v>
+        <v>0.1199013100436681</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04248944256981679</v>
+        <v>0.04307078824840449</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02898301070175061</v>
+        <v>0.02883091290750975</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8457210471893238</v>
+        <v>0.8473541580708447</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.8143849901380831</v>
+        <v>0.8139734974188151</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2761046659.86804</v>
+        <v>2781121348.452158</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1195.23071</v>
+        <v>1192.8</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.1063263414102265</v>
+        <v>0.104076433941459</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.04339452559126011</v>
+        <v>-0.04533994957781429</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1249.45</v>
@@ -3868,40 +3868,40 @@
         <v>623.78</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1125597766788</v>
+        <v>1123308664800</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>40.0412298157454</v>
+        <v>39.95979899497488</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.08491543594176</v>
+        <v>29.0061610856475</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>14.12899596549586</v>
+        <v>14.10026215515315</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>31.48333438424983</v>
+        <v>31.41930753564154</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4244536162662864</v>
+        <v>0.4235904158473524</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>33.275271721995</v>
+        <v>33.21025519200182</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.70588090231944</v>
+        <v>14.67714709197673</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01781622227025708</v>
+        <v>0.0178525285421621</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.376700919207912</v>
+        <v>0.3776314237855947</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1756814148408745</v>
+        <v>0.1761642840767306</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,26 +3937,26 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005404814272216951</v>
+        <v>0.005415828303152247</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3512533428522081</v>
+        <v>0.3481297601332196</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3363865686017708</v>
+        <v>0.3354380070595896</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3344798444.01119</v>
+        <v>3417404135.991699</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
-          <t>2026-10-29 (E)</t>
+          <t>2026-10-29 (C)</t>
         </is>
       </c>
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>218.84</v>
+        <v>213.73</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.2030786549918053</v>
+        <v>0.1749862956104848</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.05773950484391821</v>
+        <v>-0.07974165769644781</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,46 +3994,46 @@
         <v>140.6</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>345171949424</v>
+        <v>337112054400</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.59163987138264</v>
+        <v>17.18086816720257</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.41427531049305</v>
+        <v>16.02841964116978</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.7280066184353</v>
+        <v>2.664306636423271</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>2.955390659250917</v>
+        <v>3.040925129282629</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4475593847619571</v>
+        <v>0.4371086972453532</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>6.305140199134494</v>
+        <v>23.90547771152077</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>1.462407427735934</v>
+        <v>5.544610756427381</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.06818630551896036</v>
+        <v>-0.06981654821536989</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07172808659648489</v>
+        <v>0.07190032154340842</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3333243695006732</v>
+        <v>-0.3332267729943332</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
       </c>
       <c r="X28" s="4" t="n">
-        <v>0.1789084250866303</v>
+        <v>0.1812783863660298</v>
       </c>
       <c r="Y28" s="4" t="n">
         <v>0.5971674477787701</v>
@@ -4045,34 +4045,34 @@
         <v>46100000000</v>
       </c>
       <c r="AB28" s="6" t="n">
-        <v>0</v>
+        <v>1.23600958643505</v>
       </c>
       <c r="AC28" s="6" t="n">
-        <v>0</v>
+        <v>1.23600958643505</v>
       </c>
       <c r="AD28" s="6" t="n">
-        <v>0</v>
+        <v>4.750871695481674</v>
       </c>
       <c r="AE28" s="6" t="n">
-        <v>0</v>
+        <v>0.3131696413913079</v>
       </c>
       <c r="AF28" s="6" t="n">
-        <v>-5.456605445190309</v>
+        <v>12.41837325791393</v>
       </c>
       <c r="AG28" s="6" t="n">
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.0189636263937123</v>
+        <v>0.01941702147569363</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.366894486249764</v>
+        <v>1.36988909207412</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3123405248563712</v>
+        <v>0.3167746002139138</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1237367593.739642</v>
+        <v>1254969280.510813</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>865.24</v>
+        <v>881.47</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.743136019167771</v>
+        <v>1.7945912195643</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.3105657370517928</v>
+        <v>-0.2976334661354582</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>110.79</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>977193403600</v>
+        <v>995523403300</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>19.30908279401919</v>
+        <v>19.6712787324258</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.777625734428271</v>
+        <v>5.877244040879832</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>10.82474913707158</v>
+        <v>11.027797630547</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>9.689753385489059</v>
+        <v>9.871511854175768</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02752110474721247</v>
+        <v>0.02803734016171857</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>13.9921527938343</v>
+        <v>14.25971278244876</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>10.61849927553891</v>
+        <v>10.82154776901433</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02678282508209923</v>
+        <v>0.0262896883320312</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.342044583981682</v>
+        <v>2.347024318813376</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.683548155730969</v>
+        <v>1.687191968667415</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0006125468078221072</v>
+        <v>0.000601268335848072</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.876225958178616</v>
+        <v>2.883159056040856</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>1.136143222280222</v>
+        <v>1.134049849030724</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>45735065097.08406</v>
+        <v>46552661113.19795</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>113.58</v>
+        <v>117.35</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.2297049687978713</v>
+        <v>-0.2041369791198292</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.4167188767807073</v>
+        <v>-0.3973583394102482</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>117426047853</v>
+        <v>121323705700</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>70.54658385093168</v>
+        <v>72.88819875776397</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>24.49351317485458</v>
+        <v>25.29237642297905</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>7.970815086410535</v>
+        <v>8.235385942166712</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>9.374252157238734</v>
+        <v>9.685406679450303</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>112.8745341614931</v>
+        <v>116.6211180124248</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>35.36143532616796</v>
+        <v>36.47856282602465</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>8.374697790727668</v>
+        <v>8.639268646483846</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03900327128213904</v>
+        <v>0.0377502481775909</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.880214991916958</v>
+        <v>1.881824844720497</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2233421701988776</v>
+        <v>0.2239066566657617</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6268059552590223</v>
+        <v>0.6268126947791698</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6105260870819877</v>
+        <v>0.6024067807422786</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2418608210.769268</v>
+        <v>2470352363.433945</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>25.927</v>
+        <v>26.2</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.02966638942695621</v>
+        <v>0.04050832734162269</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.09819130434782608</v>
+        <v>-0.08869565217391306</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>28.75</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>147769381141</v>
+        <v>149325328000</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>34.25872093023256</v>
+        <v>34.61945031712474</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.006337671392966</v>
+        <v>9.102108284516618</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.319916182193544</v>
+        <v>2.34434388344637</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.734452083577885</v>
+        <v>1.752715107406973</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.5729998456472526</v>
+        <v>-0.5790332840651836</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>16.63398139583333</v>
+        <v>16.75723447401774</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.296712213341497</v>
+        <v>3.321139914594323</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.07434557765060458</v>
+        <v>0.07357090821190093</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.803845933852704</v>
+        <v>2.80345401691332</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05342736347492205</v>
+        <v>-0.05353408722054764</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06634010876692251</v>
+        <v>0.06564885496183206</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3020536049117387</v>
+        <v>0.2995193121846252</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.219460866094333</v>
+        <v>0.222239577731794</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1042071350.147368</v>
+        <v>1077010465.095073</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>141.89</v>
+        <v>143.53</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.1554669088794786</v>
+        <v>-0.1457055848295972</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.2716119096509242</v>
+        <v>-0.2631930184804928</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1007213104840</v>
+        <v>1018854725052</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.532079896381552</v>
+        <v>6.676266275365224</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003256154246025604</v>
+        <v>0.003290965132413172</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.609925526990542</v>
+        <v>5.733756659024447</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.060458767458592</v>
+        <v>4.150087623195136</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01461797916099935</v>
+        <v>0.01494065027291438</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.19504468936162</v>
+        <v>6.341355737403089</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.243208952114471</v>
+        <v>5.367040084148376</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.0859225690012789</v>
+        <v>0.08406691142468059</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2005.072010978741</v>
+        <v>2027.665150417351</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2637.720652891315</v>
+        <v>2668.130444642038</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4567,12 +4567,12 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>2.114313905137783</v>
+        <v>2.090155368215704</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="inlineStr"/>
       <c r="AK32" s="5" t="n">
-        <v>7575024105.478096</v>
+        <v>7691585330.374804</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4609,13 +4609,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>570.3225</v>
+        <v>571.48</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5277860129915124</v>
+        <v>0.5308867363717713</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1510910498191508</v>
+        <v>-0.1493681437268357</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4624,7 +4624,7 @@
         <v>281.15</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>71883874501</v>
+        <v>72029766667</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4650,13 +4650,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.800537206549333</v>
+        <v>1.79968732955732</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.575592087814537</v>
+        <v>0.5756347140528623</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>7077401276.224457</v>
+        <v>7177140032.394723</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4689,13 +4689,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>109.08</v>
+        <v>114.92</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.3222739852857679</v>
+        <v>-0.2859894241752883</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.5165750753412515</v>
+        <v>-0.4906931395142705</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4704,7 +4704,7 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1426315402413</v>
+        <v>1502678456595</v>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="6" t="inlineStr"/>
@@ -4731,10 +4731,10 @@
       <c r="AH34" s="4" t="inlineStr"/>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>1.032483558806966</v>
+        <v>1.047595090587305</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>10917159024.08476</v>
+        <v>11580431754.69117</v>
       </c>
       <c r="AL34" s="7" t="inlineStr"/>
       <c r="AM34" s="2" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4767,22 +4767,22 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>770.86</v>
+        <v>768.5599999999999</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.128357538070252</v>
+        <v>0.124990879614032</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.00643165560353165</v>
+        <v>-0.004223782747272864</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>775.85</v>
+        <v>771.8200000000001</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>629.11</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>821149538894</v>
+        <v>818699490975</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4808,13 +4808,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9959988058264323</v>
+        <v>0.9959713951822785</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1454717256056127</v>
+        <v>0.1456140455830462</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>36820105260.0666</v>
+        <v>37593582835.37277</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4847,13 +4847,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>415.9</v>
+        <v>418.2</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3012734866294025</v>
+        <v>0.3084697574138402</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1317327766179541</v>
+        <v>-0.1269311064718163</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4862,13 +4862,13 @@
         <v>223.7</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2157057032000</v>
+        <v>2168985936000</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>27.41393300104324</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6609087692369159</v>
+        <v>0.6640958250067674</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>13.81156097117166</v>
@@ -4892,10 +4892,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.47914852559047</v>
+        <v>40.2800863501346</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.54984589428122</v>
+        <v>40.35335407467702</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4929,16 +4929,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2644866554460207</v>
+        <v>0.2630320420851268</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.18086664873665</v>
+        <v>2.178763454141371</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.5326121339106681</v>
+        <v>0.5330617294883108</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>6183523647.051966</v>
+        <v>6315987218.940943</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -4975,13 +4975,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>26.41</v>
+        <v>26.4</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.07365837292258059</v>
+        <v>-0.07400912704112561</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.1196666666666667</v>
+        <v>-0.12</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -4990,68 +4990,68 @@
         <v>10.76</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>66213480300</v>
+        <v>66188408933</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-38.27536231884057</v>
+        <v>-20.78740157480315</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-44.17803470488442</v>
+        <v>-44.43181802881605</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.779453918301532</v>
+        <v>1.832712416807421</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.020189084658359</v>
+        <v>2.018710031061575</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.06997739267746067</v>
+        <v>0.1546969419520235</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>7.538948963738347</v>
+        <v>13.14913288345942</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.564579843671056</v>
+        <v>1.780767241672435</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03488055208685616</v>
+        <v>0.03293628046274281</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.005853367737572279</v>
+        <v>0.0364250896746503</v>
       </c>
       <c r="W37" s="4" t="n">
-        <v>-0.01774379835849423</v>
+        <v>-0.03256622244159263</v>
       </c>
       <c r="X37" s="4" t="n">
-        <v>-0.04940098460487749</v>
+        <v>-0.09222951082247931</v>
       </c>
       <c r="Y37" s="4" t="n">
-        <v>0.4147809728567589</v>
+        <v>0.4343070746227329</v>
       </c>
       <c r="Z37" s="4" t="n">
-        <v>0.04060736361193228</v>
+        <v>0.05352346670358576</v>
       </c>
       <c r="AA37" s="5" t="n">
         <v>3088000000</v>
       </c>
       <c r="AB37" s="6" t="n">
-        <v>0.7285758609990692</v>
+        <v>0.7767453385368271</v>
       </c>
       <c r="AC37" s="6" t="n">
-        <v>0.7285758609990692</v>
+        <v>0.7767453385368271</v>
       </c>
       <c r="AD37" s="6" t="n">
-        <v>0.9965620971207564</v>
+        <v>0.04546561909982338</v>
       </c>
       <c r="AE37" s="6" t="n">
-        <v>0.3318376483334526</v>
+        <v>0.01535250082263903</v>
       </c>
       <c r="AF37" s="6" t="n">
-        <v>2.306999525991468</v>
+        <v>-0.3835616438356164</v>
       </c>
       <c r="AG37" s="6" t="n">
         <v>1.789928057553957</v>
@@ -5060,13 +5060,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3219221235187428</v>
+        <v>0.3184955010229399</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2211972406426668</v>
+        <v>0.2209357765221306</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>577214425.8328384</v>
+        <v>597043958.0185165</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -5103,13 +5103,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>348.665</v>
+        <v>342.6</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.06456418929789587</v>
+        <v>-0.08083602097560449</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.100196134093783</v>
+        <v>-0.1158481509200237</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5118,40 +5118,40 @@
         <v>290.63</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>235456961150</v>
+        <v>231361206000</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>21.14402668283809</v>
+        <v>20.77622801697999</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>18.22543498442209</v>
+        <v>17.90213520323731</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.800625184660949</v>
+        <v>2.751908531871112</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.895999708284715</v>
+        <v>6.776044340723455</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.311114318324461</v>
+        <v>1.288307588825836</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>10.08182175821065</v>
+        <v>9.916162675942404</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.964839617356345</v>
+        <v>2.916122964566508</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06392675725739527</v>
+        <v>0.06505844372197818</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1601383835782586</v>
+        <v>0.1605446937537904</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.0034187955350935</v>
+        <v>-0.003185033977614715</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5187,16 +5187,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01015301220369122</v>
+        <v>0.01033274956217163</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9786850374554003</v>
+        <v>0.9813231408889448</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2687042971159443</v>
+        <v>0.2735750663526179</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1061450565.171458</v>
+        <v>1079653042.36614</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5206,7 +5206,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>
@@ -5229,13 +5229,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>143.42</v>
+        <v>143.4233</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2671810583007974</v>
+        <v>-0.2671641966182732</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5851556172625246</v>
+        <v>-0.5851460719657526</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5244,40 +5244,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>413117002126</v>
+        <v>413126512951</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>24.15824915824916</v>
+        <v>24.1453367003367</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.7070931876602</v>
+        <v>16.6922061964543</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.136575388224116</v>
+        <v>6.133295420751804</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>9.715653524042533</v>
+        <v>9.710460558012612</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7280121030121024</v>
+        <v>0.7276229843479838</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>16.76940041125339</v>
+        <v>16.762517149609</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.990846595801538</v>
+        <v>7.987566628329225</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05730288232457806</v>
+        <v>-0.0573335267949974</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4459875746723172</v>
+        <v>0.4465036206817026</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4423709970555079</v>
+        <v>0.4432258088083423</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5313,16 +5313,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01394505647747873</v>
+        <v>0.01394473561827123</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>1.984007587156891</v>
+        <v>1.98404501774208</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5995970444910079</v>
+        <v>0.5995628031811445</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>5033075057.848439</v>
+        <v>5124768186.60052</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5332,7 +5332,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06 13:44 UTC</t>
+          <t>2026-08-06 20:26 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-08)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -457,7 +457,7 @@
     <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="23" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
@@ -711,7 +711,7 @@
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>219.25</v>
+        <v>223.78</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>4601989255480</v>
@@ -720,7 +720,7 @@
         <v>35.76826484018265</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.04991673441971</v>
+        <v>33.04241636840295</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.858103082924362</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08224977168949787</v>
+        <v>0.08249543378995439</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1025249412846245</v>
+        <v>0.1027787494785721</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.0033510994797817</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3691288536173068</v>
+        <v>0.369128865381136</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3675205268565243</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>19405603360.9568</v>
+        <v>19406397046.70146</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.77722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.98976850488836</v>
+        <v>24.97737507537381</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18825919949132</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1115437990867578</v>
+        <v>0.1120953318112634</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1978992770141008</v>
+        <v>0.1985291629589558</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007120142402848057</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5730773950114763</v>
+        <v>0.5730774163355732</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4887078823050989</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>17939123937.45356</v>
+        <v>18017125442.5354</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.59185700099305</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.72121526096742</v>
+        <v>20.73859844956407</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.615274970354358</v>
@@ -998,10 +998,10 @@
         <v>0.1512636492980362</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1510219463753723</v>
+        <v>-0.1517335636843464</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2605275172038914</v>
+        <v>0.261211041744337</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002399096810612475</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.814906998178035</v>
+        <v>0.8149070505054825</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4161733495617475</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>11685397595.81362</v>
+        <v>11686393084.29932</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.78412698412698</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>25.10149240846296</v>
+        <v>25.10954183367011</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.806477939356436</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1321580952380953</v>
+        <v>-0.1324363013698632</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.154972944109169</v>
+        <v>0.155381152273339</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8766396327993262</v>
+        <v>0.8766396536786445</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4867091216191816</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>13843294074.55683</v>
+        <v>13865783017.84897</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.14024390243902</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.34913118185881</v>
+        <v>20.33000703681656</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.39932052814499</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6777248914132978</v>
+        <v>0.6793031030738388</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9092650318506463</v>
+        <v>0.9111018286340502</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001250223254152527</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.281155332341915</v>
+        <v>1.281155343251333</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3920089314744357</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27084972842.95662</v>
+        <v>27090520324.85759</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.00297287253809</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.73933678908357</v>
+        <v>17.73600482881467</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.608455706499072</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2403492382014121</v>
+        <v>0.2405822554125112</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2456131401300343</v>
+        <v>0.2462204813205464</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003546698192872825</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8121299533775441</v>
+        <v>0.8121299763581794</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5064928375172059</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11756230821.18639</v>
+        <v>11759928505.27059</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>278.4576271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>162.4280868405468</v>
+        <v>162.3065912214937</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.52417300611857</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7143440677966106</v>
+        <v>0.7156273508242399</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1051525040484853</v>
+        <v>0.1055209982376162</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.55760056611344</v>
+        <v>1.557600576594546</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6212095837082003</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>15146762072.99376</v>
+        <v>15152548990.85927</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>69.10500807754443</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>24.23578546774603</v>
+        <v>24.20588931102079</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.96750044126416</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.851362427246774</v>
+        <v>1.854884081704915</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.098732407599096</v>
+        <v>1.10124601449116</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.005937909107910979</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.613896736761467</v>
+        <v>1.613896771329559</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4744553419374782</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8218402271.672566</v>
+        <v>8251708165.086263</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.605223505776</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.04837035146276</v>
+        <v>42.03742661191326</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431733236757758</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1321538292177815</v>
+        <v>0.1324485664944304</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.109069154317581</v>
+        <v>0.1093053430088609</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005844991665084088</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1720542945133763</v>
+        <v>-0.1720542986099027</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2113923990941288</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2293560101.096612</v>
+        <v>2302209622.137451</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.95356037151703</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.88461878873867</v>
+        <v>19.88143622476718</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.382254196481164</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1543374613003097</v>
+        <v>0.1545222443699903</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1263565194297944</v>
+        <v>0.1266830596504676</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1336707206911988</v>
+        <v>0.1336707122685273</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.37489557524865</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3398842233.110943</v>
+        <v>3398994672.363688</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1967,13 +1967,13 @@
         <v>0.05021635018614878</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0003639916473496818</v>
+        <v>-0.006927527405603096</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>521.99</v>
+        <v>525.4400000000001</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>462.55</v>
+        <v>463.5</v>
       </c>
       <c r="K12" s="5" t="n">
         <v>1125446205871</v>
@@ -1982,7 +1982,7 @@
         <v>15.5343852337005</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.54154392367269</v>
+        <v>24.53943053258187</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.998039941690597</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.3670167907115213</v>
+        <v>-0.3669622767702392</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05109969791792079</v>
+        <v>0.05120336154386385</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.05787165877034604</v>
@@ -2054,7 +2054,7 @@
         <v>0.144793592992015</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2144000281.317013</v>
+        <v>2159906866.931559</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2093,10 +2093,10 @@
         <v>0.09843919113981392</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.004954077372669174</v>
+        <v>-0.01509641873278245</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>359.3</v>
+        <v>363</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>279.1</v>
@@ -2108,7 +2108,7 @@
         <v>15.37059329320722</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.38711926266738</v>
+        <v>14.38656925736971</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.218656584451321</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06835795356835783</v>
+        <v>0.06839879739455124</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.293344751472451</v>
+        <v>-0.2932962460084035</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.2236981109979266</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>3136940945.724731</v>
+        <v>3138267869.246623</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.79864061172472</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.5860966743327</v>
+        <v>24.57789105606379</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.21319488374393</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2526852480767217</v>
+        <v>0.2531034717938572</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1250624930863917</v>
+        <v>0.1253686234309759</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.2125979432658452</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2875125289.91506</v>
+        <v>2887741099.498393</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.91433278418451</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.88529597475946</v>
+        <v>25.87514543666057</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.07312419690448</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1942816035145525</v>
+        <v>0.1947501071968585</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1415239610979675</v>
+        <v>0.1418906118340109</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2334870940204503</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1861609035.521179</v>
+        <v>1861886006.927185</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
         <v>461.62</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>244.37</v>
+        <v>252.14</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>369687423980</v>
@@ -2486,7 +2486,7 @@
         <v>26.17709472059675</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.08013393777818</v>
+        <v>19.0735208631822</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8212921717552079</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3719555012539386</v>
+        <v>0.3724311787199521</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007414601117013087</v>
+        <v>0.007493131785874185</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2502869112012382</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2338873890.456343</v>
+        <v>2338940393.756815</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>19.75968992248062</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.21522901445912</v>
+        <v>14.21708918666403</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.755535679388467</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3900366925064598</v>
+        <v>0.3898548192984317</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01896450366476476</v>
+        <v>0.01884166412610044</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2632994020450284</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2172885877.956724</v>
+        <v>2216342277.831625</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>274.9</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>170.39</v>
+        <v>171.81</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>624742065364</v>
@@ -2738,7 +2738,7 @@
         <v>29.96994219653179</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.00448850833101</v>
+        <v>20.99895898668244</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.379540946645018</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4268351350067303</v>
+        <v>0.4272108543827697</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.07983978976770545</v>
+        <v>0.08004568747237495</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2734884425769581</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>2103204874.126432</v>
+        <v>2104191947.671916</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.24561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.1696330072986</v>
+        <v>36.15761502519362</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.227223372236507</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.085043191540495</v>
+        <v>0.08540383561643816</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06200415240735468</v>
+        <v>0.06213595080672829</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2936,7 +2936,7 @@
         <v>0.226674048718448</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2575114939.973714</v>
+        <v>2575417509.132919</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.59555555555556</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.70671871951385</v>
+        <v>20.70343848785054</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.981590067400496</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0429250451547436</v>
+        <v>0.04309028513444946</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.0222771553881298</v>
+        <v>0.02235718072930504</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.218385915467971</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1332065273.232331</v>
+        <v>1332077922.944082</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.3038639802745476</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1368139854.962272</v>
+        <v>1368427883.450317</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.6802030456853</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.66517529339069</v>
+        <v>39.59839455230968</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.0816321510713</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.092894513594326</v>
+        <v>2.098110527779709</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7539238083429485</v>
+        <v>0.7562504066506923</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.551213500768213</v>
+        <v>2.551213628174088</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.8193034323489479</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>15421082717.71883</v>
+        <v>15438096054.70724</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>710.45</v>
+        <v>716.2</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>671008868151</v>
@@ -3368,7 +3368,7 @@
         <v>54.39042089985486</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.33293202523935</v>
+        <v>37.30190963963538</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.35387639966032</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4569019348141101</v>
+        <v>0.4581135771682308</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2262178086412556</v>
+        <v>0.2270048870614978</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004468721819194826</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.708763115365479</v>
+        <v>1.70876314980093</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5994443606515928</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3458485668.1816</v>
+        <v>3459103777.661133</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>87.79775280898873</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>117.049641990473</v>
+        <v>116.2556604683023</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.971153097505186</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2499101123595507</v>
+        <v>-0.2447872864398956</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1368281139698921</v>
+        <v>0.1372519686949247</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.4017511021464303</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1362680255.941759</v>
+        <v>1364637842.648468</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83805606337599</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.48930728397621</v>
+        <v>14.48748178907374</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.600475061007148</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09308580134064592</v>
+        <v>0.09322353559890817</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3864624282845928</v>
+        <v>-0.3864171414076311</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.4080473481191881</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2146021313.994039</v>
+        <v>2162944258.603922</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.7231441048035</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.49991914861701</v>
+        <v>18.49659587882478</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.235300454723071</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.120174847161572</v>
+        <v>0.1203761081533767</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04307078824840449</v>
+        <v>0.04318052086594171</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.8152301455742935</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2745926223.370859</v>
+        <v>2754396889.956614</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3865,7 +3865,7 @@
         <v>1249.45</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>623.78</v>
+        <v>625.9</v>
       </c>
       <c r="K27" s="5" t="n">
         <v>1116631721110</v>
@@ -3874,7 +3874,7 @@
         <v>39.72227805695143</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.12694932324147</v>
+        <v>28.10861418209978</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.01645023473059</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4122497822445563</v>
+        <v>0.4131709873568759</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.192096985710305</v>
+        <v>0.1925676473681133</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3338491441316793</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3429256447.706755</v>
+        <v>3472721926.789144</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.38424437299035</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.19635621678403</v>
+        <v>16.19383039411742</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.695845006283144</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.0733429260450158</v>
+        <v>0.07351034004316581</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3317936596416632</v>
+        <v>-0.331696626373812</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.3180804393148213</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1260862778.880235</v>
+        <v>1260871547.456309</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>111.67</v>
+        <v>113.46</v>
       </c>
       <c r="K29" s="5" t="n">
         <v>991118782300</v>
@@ -4126,7 +4126,7 @@
         <v>19.58424458826155</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.85123786195431</v>
+        <v>5.842545253106323</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>10.97900594080244</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.347025885855958</v>
+        <v>2.352005631081614</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.687191968667414</v>
+        <v>1.690835781603859</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0006039404264047313</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.884670726814804</v>
+        <v>2.884670860954578</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.109458602054814</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>44262693218.202</v>
+        <v>44278984486.32263</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.56521739130436</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.91502284156086</v>
+        <v>26.89999446729248</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.763826130871573</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.881855900621119</v>
+        <v>1.883465923593976</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2239066615123544</v>
+        <v>0.2244711481436368</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.6199293345286607</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2510592445.07129</v>
+        <v>2515490471.672897</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.33298097251586</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.195917755343192</v>
+        <v>9.196810529787868</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.392662421502135</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.842246300211417</v>
+        <v>2.841873316632396</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.0496125127857322</v>
+        <v>-0.04972484466562921</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2241484475281889</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1069591933.242303</v>
+        <v>1075461313.808505</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>6.21312214893282</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003112045257922633</v>
+        <v>0.003109596471603041</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>5.335996053097357</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1995.475511760466</v>
+        <v>1997.047722806255</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2617.534349826469</v>
+        <v>2620.572703502577</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4572,7 +4572,7 @@
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="inlineStr"/>
       <c r="AK32" s="5" t="n">
-        <v>7553778355.137402</v>
+        <v>7554288858.568101</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4650,13 +4650,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.806971154915171</v>
+        <v>1.806971194618595</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5647683178966268</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6993032335.749827</v>
+        <v>6995008368.60789</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
         <v>1.108725150761214</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12323502561.06727</v>
+        <v>12347379211.79675</v>
       </c>
       <c r="AL34" s="7" t="inlineStr"/>
       <c r="AM34" s="2" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4773,10 +4773,10 @@
         <v>0.1318705729810901</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.0008463461749674828</v>
+        <v>-0.004621226749050744</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>773.915</v>
+        <v>776.85</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>629.28</v>
@@ -4814,7 +4814,7 @@
         <v>0.1461235446452172</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>37510815528.86498</v>
+        <v>37533815555.02279</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
         <v>27.4718905760983</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6668342737881061</v>
+        <v>0.6663645671342884</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>13.84076088865828</v>
@@ -4892,10 +4892,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.19747837800519</v>
+        <v>40.22651763169463</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.25138049626884</v>
+        <v>40.28331659363955</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4938,7 +4938,7 @@
         <v>0.5287271244451457</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>6231001161.750312</v>
+        <v>6231157458.637492</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
         <v>-21.08661417322834</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-45.07136692468539</v>
+        <v>-45.34915420187771</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.859092368268033</v>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03657819536480678</v>
+        <v>0.03665158391250167</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5060,13 +5060,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3211665652162632</v>
+        <v>0.321166558006574</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2226778448203278</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>589699214.1078761</v>
+        <v>589700828.9419174</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
         <v>20.6737416616131</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.81382636350155</v>
+        <v>17.80759187221626</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.73833373496842</v>
@@ -5148,10 +5148,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1605446937537904</v>
+        <v>0.160951003929322</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.003185033977614715</v>
+        <v>-0.002951272420135931</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5196,7 +5196,7 @@
         <v>0.2740445755781122</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1070957661.177271</v>
+        <v>1072169084.875285</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5206,7 +5206,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
         <v>24.73737373737373</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.10149451663011</v>
+        <v>17.08587723135333</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.283682143175272</v>
@@ -5274,10 +5274,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4465036206817024</v>
+        <v>0.4478257921682576</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4432258088083423</v>
+        <v>0.4448847482313887</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5322,7 +5322,7 @@
         <v>0.6052981343869617</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>5028689334.145506</v>
+        <v>5054897781.697133</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5332,7 +5332,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 18:08 ET</t>
+          <t>2026-08-08 08:29 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-09)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.76826484018265</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.04241636840295</v>
+        <v>33.03491940588806</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.858103082924362</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08249543378995439</v>
+        <v>0.08274109589041112</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1027787494785721</v>
+        <v>0.10303255767252</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.77722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.97737507537381</v>
+        <v>24.96499393256436</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18825919949132</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1120953318112634</v>
+        <v>0.1126468645357686</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1985291629589558</v>
+        <v>0.1991590489038111</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.59185700099305</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.73859844956407</v>
+        <v>20.75601082843281</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.615274970354358</v>
@@ -998,10 +998,10 @@
         <v>0.1512636492980362</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1517335636843464</v>
+        <v>-0.1524451809933207</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.261211041744337</v>
+        <v>0.2618945662847831</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.78412698412698</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>25.10954183367011</v>
+        <v>25.11759642303477</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.806477939356436</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1324363013698632</v>
+        <v>-0.1327145075016307</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.155381152273339</v>
+        <v>0.1557893604375093</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.14024390243902</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.33000703681656</v>
+        <v>20.31091880382644</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.39932052814499</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6793031030738388</v>
+        <v>0.6808813147343797</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9111018286340502</v>
+        <v>0.9129386254174543</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.00297287253809</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.73600482881467</v>
+        <v>17.73267411998762</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.608455706499072</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2405822554125112</v>
+        <v>0.240815272623611</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2462204813205464</v>
+        <v>0.2468278225110589</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>278.4576271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>162.3065912214937</v>
+        <v>162.1852772231526</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.52417300611857</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7156273508242399</v>
+        <v>0.7169106338518696</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1055209982376162</v>
+        <v>0.1058894924267473</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>69.10500807754443</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>24.20588931102079</v>
+        <v>24.17606682048807</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.96750044126416</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.854884081704915</v>
+        <v>1.858405736163056</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.10124601449116</v>
+        <v>1.103759621383223</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.605223505776</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.03742661191326</v>
+        <v>42.02648856743691</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431733236757758</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1324485664944304</v>
+        <v>0.1327433037710797</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1093053430088609</v>
+        <v>0.1095415317001411</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.95356037151703</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.88143622476718</v>
+        <v>19.87825467938123</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.382254196481164</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1545222443699903</v>
+        <v>0.1547070274396711</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1266830596504676</v>
+        <v>0.1270095998711409</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>15.5343852337005</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.53943053258187</v>
+        <v>24.53731750544836</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.998039941690597</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.3669622767702392</v>
+        <v>-0.3669077628289569</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05120336154386385</v>
+        <v>0.05130702516980712</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.05787165877034604</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.37059329320722</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.38656925736971</v>
+        <v>14.38601929412275</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.218656584451321</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06839879739455124</v>
+        <v>0.06843964122074486</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2932962460084035</v>
+        <v>-0.2932477405443562</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.79864061172472</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.57789105606379</v>
+        <v>24.56969091322332</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.21319488374393</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2531034717938572</v>
+        <v>0.2535216955109927</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1253686234309759</v>
+        <v>0.1256747537755603</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.91433278418451</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.87514543666057</v>
+        <v>25.86500285620964</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.07312419690448</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1947501071968585</v>
+        <v>0.1952186108791647</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1418906118340109</v>
+        <v>0.1422572625700542</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>26.17709472059675</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.0735208631822</v>
+        <v>19.06691237111206</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8212921717552079</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3724311787199521</v>
+        <v>0.3729068561859654</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007493131785874185</v>
+        <v>0.007571662454735506</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>19.75968992248062</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.21708918666403</v>
+        <v>14.21894984576836</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.755535679388467</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3898548192984317</v>
+        <v>0.3896729460904038</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01884166412610044</v>
+        <v>0.01871882458743612</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>29.96994219653179</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.99895898668244</v>
+        <v>20.99343237560822</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.379540946645018</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4272108543827697</v>
+        <v>0.4275865737588092</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08004568747237495</v>
+        <v>0.080251585177044</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.24561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.15761502519362</v>
+        <v>36.14560502679804</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.227223372236507</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08540383561643816</v>
+        <v>0.08576447969238155</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06213595080672829</v>
+        <v>0.06226774920610167</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.59555555555556</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.70343848785054</v>
+        <v>20.70015929529108</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.981590067400496</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04309028513444946</v>
+        <v>0.04325552511415531</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02235718072930504</v>
+        <v>0.02243720607048005</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.6802030456853</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.59839455230968</v>
+        <v>39.53183829891184</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.0816321510713</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.098110527779709</v>
+        <v>2.103326541965093</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7562504066506923</v>
+        <v>0.7585770049584366</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.39042089985486</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.30190963963538</v>
+        <v>37.27093876830092</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.35387639966032</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4581135771682308</v>
+        <v>0.4593252195223518</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2270048870614978</v>
+        <v>0.22779196548174</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>87.79775280898873</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>116.2556604683023</v>
+        <v>115.47237798336</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.971153097505186</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2447872864398956</v>
+        <v>-0.2396644605202404</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1372519686949247</v>
+        <v>0.1376758234199575</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83805606337599</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.48748178907374</v>
+        <v>14.48565675409828</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.600475061007148</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09322353559890817</v>
+        <v>0.09336126985717041</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3864171414076311</v>
+        <v>-0.3863718545306695</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.7231441048035</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.49659587882478</v>
+        <v>18.49327380278248</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.235300454723071</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1203761081533767</v>
+        <v>0.1205773691451817</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04318052086594171</v>
+        <v>0.04329025348347915</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.72227805695143</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.10861418209978</v>
+        <v>28.09030292967743</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.01645023473059</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4131709873568759</v>
+        <v>0.4140921924691958</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1925676473681133</v>
+        <v>0.1930383090259216</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.38424437299035</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.19383039411742</v>
+        <v>16.19130535913235</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.695845006283144</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07351034004316581</v>
+        <v>0.07367775404131627</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.331696626373812</v>
+        <v>-0.3315995931059608</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>19.58424458826155</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.842545253106323</v>
+        <v>5.833878433454627</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>10.97900594080244</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.352005631081614</v>
+        <v>2.35698537630727</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.690835781603859</v>
+        <v>1.694479594540304</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.56521739130436</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.89999446729248</v>
+        <v>26.88498286625867</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.763826130871573</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.883465923593976</v>
+        <v>1.885075946566835</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2244711481436368</v>
+        <v>0.2250356347749196</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.33298097251586</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.196810529787868</v>
+        <v>9.197703477597205</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.392662421502135</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.841873316632396</v>
+        <v>2.841500333053376</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04972484466562921</v>
+        <v>-0.04983717654552622</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>6.21312214893282</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003109596471603041</v>
+        <v>0.003107151536024117</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>5.335996053097357</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1997.047722806255</v>
+        <v>1998.619933852043</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2620.572703502577</v>
+        <v>2623.611057178686</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
         <v>27.4718905760983</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6663645671342884</v>
+        <v>0.6658955217213655</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>13.84076088865828</v>
@@ -4892,10 +4892,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.22651763169463</v>
+        <v>40.25555688538407</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.28331659363955</v>
+        <v>40.31525269101027</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
         <v>-21.08661417322834</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-45.34915420187771</v>
+        <v>-45.63038687334205</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.859092368268033</v>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03665158391250167</v>
+        <v>0.03672497246019657</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
         <v>20.6737416616131</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.80759187221626</v>
+        <v>17.80136174330457</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.73833373496842</v>
@@ -5148,10 +5148,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.160951003929322</v>
+        <v>0.1613573141048543</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.002951272420135931</v>
+        <v>-0.002717510862657035</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5206,7 +5206,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
         <v>24.73737373737373</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.08587723135333</v>
+        <v>17.07028844382807</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.283682143175272</v>
@@ -5274,10 +5274,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4478257921682576</v>
+        <v>0.4491479636548128</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4448847482313887</v>
+        <v>0.4465436876544344</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5332,7 +5332,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-08 08:29 ET</t>
+          <t>2026-08-09 08:32 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-10)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -447,16 +447,16 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
     <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
@@ -720,7 +720,7 @@
         <v>35.76826484018265</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.03491940588806</v>
+        <v>33.02742584455891</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.858103082924362</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08274109589041112</v>
+        <v>0.08298675799086763</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.10303255767252</v>
+        <v>0.1032863658664678</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,7 +781,7 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.0033510994797817</v>
+        <v>0.003383014712922478</v>
       </c>
       <c r="AI2" s="6" t="n">
         <v>0.369128865381136</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.77722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.96499393256436</v>
+        <v>24.9526250581977</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18825919949132</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1126468645357686</v>
+        <v>0.1131983972602739</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1991590489038111</v>
+        <v>0.1997889348486663</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.59185700099305</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.75601082843281</v>
+        <v>20.77345247116095</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.615274970354358</v>
@@ -995,13 +995,13 @@
         <v>0.01242438382870799</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>0.1512636492980362</v>
+        <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1524451809933207</v>
+        <v>-0.1531567983022949</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2618945662847831</v>
+        <v>0.2625780908252289</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1034,7 +1034,7 @@
         <v>0.1745098099410268</v>
       </c>
       <c r="AG4" s="6" t="n">
-        <v>1110.671328671329</v>
+        <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
         <v>0.002399096810612475</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.78412698412698</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>25.11759642303477</v>
+        <v>25.1256561815282</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.806477939356436</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1327145075016307</v>
+        <v>-0.1329927136333986</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1557893604375093</v>
+        <v>0.1561975686016794</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.14024390243902</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.31091880382644</v>
+        <v>20.2918663818278</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.39932052814499</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6808813147343797</v>
+        <v>0.6824595263949214</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9129386254174543</v>
+        <v>0.9147754222008586</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.00297287253809</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.73267411998762</v>
+        <v>17.72934466189754</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.608455706499072</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.240815272623611</v>
+        <v>0.2410482898347102</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2468278225110589</v>
+        <v>0.247435163701571</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>278.4576271186441</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>162.1852772231526</v>
+        <v>162.0641444385774</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.52417300611857</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7169106338518696</v>
+        <v>0.7181939168794986</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1058894924267473</v>
+        <v>0.1062579866158779</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>69.10500807754443</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>24.17606682048807</v>
+        <v>24.14631772420502</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.96750044126416</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.858405736163056</v>
+        <v>1.861927390621197</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.103759621383223</v>
+        <v>1.106273228275287</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.605223505776</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.02648856743691</v>
+        <v>42.01555621358935</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431733236757758</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1327433037710797</v>
+        <v>0.1330380410477285</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1095415317001411</v>
+        <v>0.1097777203914214</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.95356037151703</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.87825467938123</v>
+        <v>19.8750741520919</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.382254196481164</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1547070274396711</v>
+        <v>0.1548918105093515</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1270095998711409</v>
+        <v>0.1273361400918138</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1979,25 +1979,25 @@
         <v>1125446205871</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>15.5343852337005</v>
+        <v>0.02915758169766638</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.53731750544836</v>
+        <v>24.53520484217817</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.998039941690597</v>
+        <v>2.925615385679786</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.54792225704467</v>
+        <v>0.000998837341054178</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>-1.48307922129375</v>
+        <v>4.760404182984809e-07</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>16.08653099309312</v>
+        <v>19.91270556575665</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.232441663614762</v>
+        <v>2.925615385679786</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>0.02121114263433417</v>
@@ -2006,40 +2006,40 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.3669077628289569</v>
+        <v>-0.9988116022717063</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05130702516980712</v>
+        <v>0.02601144335470584</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>0.05787165877034604</v>
+        <v>0</v>
       </c>
       <c r="X12" s="4" t="n">
-        <v>0.1031342591143128</v>
+        <v>0.1185897214314059</v>
       </c>
       <c r="Y12" s="4" t="n">
-        <v>0.2513572406591474</v>
+        <v>0.1872769290358135</v>
       </c>
       <c r="Z12" s="4" t="n">
-        <v>0.1605832804999547</v>
+        <v>0.1161931648327082</v>
       </c>
       <c r="AA12" s="5" t="n">
         <v>25042000000</v>
       </c>
       <c r="AB12" s="6" t="n">
-        <v>4.274309230860424</v>
+        <v>0</v>
       </c>
       <c r="AC12" s="6" t="n">
-        <v>4.058182957499597</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="6" t="n">
-        <v>0.2009334677336179</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="6" t="n">
-        <v>0.1166800157473901</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="6" t="n">
-        <v>1.16652083996182</v>
+        <v>0</v>
       </c>
       <c r="AG12" s="6" t="n">
         <v>11.61570329453541</v>
@@ -2058,13 +2058,13 @@
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-08 (C)</t>
+          <t>2026-11-07 (E)</t>
         </is>
       </c>
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.37059329320722</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.38601929412275</v>
+        <v>14.38546937292167</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.218656584451321</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06843964122074486</v>
+        <v>0.06848048504693827</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2932477405443562</v>
+        <v>-0.2931992350803088</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.79864061172472</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.56969091322332</v>
+        <v>24.56149624033267</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.21319488374393</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2535216955109927</v>
+        <v>0.2539399192281282</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1256747537755603</v>
+        <v>0.1259808841201444</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.91433278418451</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.86500285620964</v>
+        <v>25.8548682240526</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.07312419690448</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1952186108791647</v>
+        <v>0.1956871145614707</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1422572625700542</v>
+        <v>0.1426239133060971</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>26.17709472059675</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.06691237111206</v>
+        <v>19.06030845680621</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8212921717552079</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3729068561859654</v>
+        <v>0.3733825336519787</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007571662454735506</v>
+        <v>0.007650193123596605</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>19.75968992248062</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.21894984576836</v>
+        <v>14.22081099196334</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.755535679388467</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3896729460904038</v>
+        <v>0.3894910728823755</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01871882458743612</v>
+        <v>0.0185959850487718</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>29.96994219653179</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>20.99343237560822</v>
+        <v>20.98790867281088</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.379540946645018</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4275865737588092</v>
+        <v>0.4279622931348481</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.080251585177044</v>
+        <v>0.08045748288171328</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.24561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.14560502679804</v>
+        <v>36.13360300415901</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.227223372236507</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08576447969238155</v>
+        <v>0.08612512376832471</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06226774920610167</v>
+        <v>0.06239954760547506</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.59555555555556</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.70015929529108</v>
+        <v>20.69688114134179</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.981590067400496</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04325552511415531</v>
+        <v>0.04342076509386095</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02243720607048005</v>
+        <v>0.02251723141165529</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.6802030456853</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.53183829891184</v>
+        <v>39.46550540315224</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.0816321510713</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.103326541965093</v>
+        <v>2.108542556150476</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7585770049584366</v>
+        <v>0.7609036032661807</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>671008868151</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.39042089985486</v>
+        <v>56.16835994194484</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.27093876830092</v>
+        <v>37.24001928302926</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.35387639966032</v>
+        <v>16.88845941739438</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.46982873166127</v>
+        <v>27.33508664216921</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.702554714514199</v>
+        <v>3.823585522393583</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>42.2681056019502</v>
+        <v>43.66108677553549</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.22118939944802</v>
+        <v>16.75577241718208</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.0173120657144548</v>
+        <v>0.01676407397026341</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4593252195223518</v>
+        <v>0.5082795611639617</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.22779196548174</v>
+        <v>0.2687393995732272</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>87.79775280898873</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>115.47237798336</v>
+        <v>114.6995797259019</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.971153097505186</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2396644605202404</v>
+        <v>-0.2345416346005852</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1376758234199575</v>
+        <v>0.1380996781449901</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83805606337599</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.48565675409828</v>
+        <v>14.48383217887603</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.600475061007148</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09336126985717041</v>
+        <v>0.09349900411543244</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3863718545306695</v>
+        <v>-0.3863265676537079</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.7231441048035</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.49327380278248</v>
+        <v>18.489952919847</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.235300454723071</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1205773691451817</v>
+        <v>0.1207786301369862</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04329025348347915</v>
+        <v>0.04339998610101614</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,7 +3811,7 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02836311530681052</v>
+        <v>0.02840525960890088</v>
       </c>
       <c r="AI26" s="6" t="n">
         <v>0.8508796484888125</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.72227805695143</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.09030292967743</v>
+        <v>28.07201551931818</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.01645023473059</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4140921924691958</v>
+        <v>0.4150133975815151</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1930383090259216</v>
+        <v>0.1935089706837299</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.38424437299035</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.19130535913235</v>
+        <v>16.18878111146043</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.695845006283144</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07367775404131627</v>
+        <v>0.07384516803946584</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3315995931059608</v>
+        <v>-0.3315025598381096</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>19.58424458826155</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.833878433454627</v>
+        <v>5.825237288402294</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>10.97900594080244</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.35698537630727</v>
+        <v>2.361965121532926</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.694479594540304</v>
+        <v>1.69812340747675</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.56521739130436</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.88498286625867</v>
+        <v>26.86998801039409</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.763826130871573</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.885075946566835</v>
+        <v>1.886685969539692</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2250356347749196</v>
+        <v>0.2256001214062018</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.33298097251586</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.197703477597205</v>
+        <v>9.198596598821711</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.392662421502135</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.841500333053376</v>
+        <v>2.841127349474355</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04983717654552622</v>
+        <v>-0.04994950842542323</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>978960880178</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.21312214893282</v>
+        <v>6.204383580509567</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003107151536024117</v>
+        <v>0.003104710442110006</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.335996053097357</v>
+        <v>5.328491136004394</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>3.862188874465631</v>
+        <v>3.85675682260281</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01390419154979336</v>
+        <v>0.01388463572482881</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>5.871386916421399</v>
+        <v>5.862519580176463</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>4.969279478221286</v>
+        <v>4.961774561128323</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.09033350257166804</v>
+        <v>0.09046073285698025</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1998.619933852043</v>
+        <v>1997.377528660282</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2623.611057178686</v>
+        <v>2622.953701416179</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4666,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4865,37 +4865,37 @@
         <v>2178529059200</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.4718905760983</v>
+        <v>27.58780572620842</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6658955217213655</v>
+        <v>0.6654271361540031</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.84076088865828</v>
+        <v>13.89916072363153</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.553575721047341</v>
+        <v>9.59388616712771</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5160718850298077</v>
+        <v>0.5182494035320432</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.19521625604111</v>
+        <v>18.27477474575392</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.35618147718766</v>
+        <v>13.41458131216091</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01819837749847103</v>
+        <v>0.01812191372746905</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.25555688538407</v>
+        <v>40.45879274725525</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.31525269101027</v>
+        <v>40.52164950056824</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
         <v>-21.08661417322834</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-45.63038687334205</v>
+        <v>-45.91512943888684</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.859092368268033</v>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03672497246019657</v>
+        <v>0.03679836100789124</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -5124,7 +5124,7 @@
         <v>20.6737416616131</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.80136174330457</v>
+        <v>17.79513597218947</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.73833373496842</v>
@@ -5148,10 +5148,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1613573141048543</v>
+        <v>0.1617636242803857</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.002717510862657035</v>
+        <v>-0.002483749305178362</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5206,7 +5206,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
         <v>24.73737373737373</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.07028844382807</v>
+        <v>17.05472807612323</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.283682143175272</v>
@@ -5274,10 +5274,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4491479636548128</v>
+        <v>0.4504701351413676</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4465436876544344</v>
+        <v>0.4482026270774806</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5332,7 +5332,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 08:32 ET</t>
+          <t>2026-08-10 08:48 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-11)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -457,7 +457,7 @@
     <col width="24" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="23" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
@@ -720,7 +720,7 @@
         <v>35.18949771689498</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.4930083006534</v>
+        <v>32.48563933668847</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.698588888208164</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08298675799086763</v>
+        <v>0.08323242009132437</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1032863658664678</v>
+        <v>0.1035401740604156</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003438655680269902</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3693184231896078</v>
+        <v>0.3693184730345007</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3576838593179019</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>17376039344.64669</v>
+        <v>17390568810.88155</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.11444444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.25555598502275</v>
+        <v>25.24304934845532</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.32408738273681</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1131983972602739</v>
+        <v>0.1137499299847793</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.1997889348486663</v>
+        <v>0.2004188207935214</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007034738963759238</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5719001159182375</v>
+        <v>0.5719000567972845</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4849336598535537</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>16227450567.71487</v>
+        <v>16228584424.67916</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.75173783515392</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.96224873691635</v>
+        <v>20.97987849960508</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.702661889362552</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1531567983022949</v>
+        <v>-0.1538684156112691</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2625780908252286</v>
+        <v>0.2632616153656748</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002377489371223988</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8138560872242853</v>
+        <v>0.8138560399538562</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.416776537443992</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10621782963.98354</v>
+        <v>10622947315.35868</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>22.07063492063492</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>25.45611238531469</v>
+        <v>25.46428338905514</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.85654127862005</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1329927136333987</v>
+        <v>-0.1332709197651665</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1561975686016794</v>
+        <v>0.1566057767658497</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8747500798721349</v>
+        <v>0.8747500115541534</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4870447706456447</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>12259414709.56222</v>
+        <v>12270364857.49069</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>33.16310975609756</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.71108917381067</v>
+        <v>19.69261674289472</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.78684667305743</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6824595263949214</v>
+        <v>0.6840377380554625</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9147754222008586</v>
+        <v>0.9166122189842627</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001287060445874512</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.283736745556912</v>
+        <v>1.283736809032299</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3990951859324948</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26723970977.92529</v>
+        <v>26778992950.24877</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.10776662950576</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.8137843713158</v>
+        <v>17.81044031197182</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.639929857979041</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2410482898347104</v>
+        <v>0.24128130704581</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.247435163701571</v>
+        <v>0.2480425048920836</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003529886371276811</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8118881508141991</v>
+        <v>0.811888107240691</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5065929026370816</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11697784084.9426</v>
+        <v>11710809582.96794</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>280.406779661017</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>163.1985638560974</v>
+        <v>163.0767652378073</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.6118399301962</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7181939168794982</v>
+        <v>0.7194771999071279</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1062579866158782</v>
+        <v>0.1066264808050092</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.555854975911197</v>
+        <v>1.555854906192706</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6186187633879504</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14744956430.70717</v>
+        <v>14752782565.18555</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>68.23909531502423</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.84375492496774</v>
+        <v>23.81445080386515</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.62958711985689</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.861927390621197</v>
+        <v>1.865449045079337</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.106273228275287</v>
+        <v>1.10878683516735</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006013257575757576</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.614640871636319</v>
+        <v>1.614640871972267</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4746954314438966</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8021639287.803991</v>
+        <v>8022794132.437032</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.85283776996484</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.23409632894141</v>
+        <v>42.22311282720936</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.439180267688964</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1330380410477285</v>
+        <v>0.1333327783243776</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1097777203914214</v>
+        <v>0.110013909082701</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005814746785620572</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1731185166096821</v>
+        <v>-0.173118529432724</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2113769769133736</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2083584214.747021</v>
+        <v>2087580969.238688</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>23.61919504643963</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.4514352180077</v>
+        <v>20.44816350511873</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.567334403153112</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1548918105093515</v>
+        <v>0.1550765935790321</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1273361400918136</v>
+        <v>0.1276626803124867</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1298935768479796</v>
+        <v>0.1298934673632423</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3811743479676913</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3282511374.042004</v>
+        <v>3282997378.786723</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -1967,13 +1967,13 @@
         <v>0.06555297070822341</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.01543096514433695</v>
+        <v>-0.01547216126752715</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>537.7175</v>
+        <v>537.74</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>463.5</v>
+        <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
         <v>1141881430265</v>
@@ -1982,7 +1982,7 @@
         <v>0.02958337850206696</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.89349970783052</v>
+        <v>24.89135656179421</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.9683390139646</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.9988116022717063</v>
+        <v>-0.9988114999506505</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02601144335470584</v>
+        <v>0.02611260274713967</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0</v>
@@ -2054,7 +2054,7 @@
         <v>0.1481766708054383</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2126173403.915531</v>
+        <v>2147019822.306722</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.46818572656922</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.47680696376004</v>
+        <v>14.47625359325494</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.239092785074236</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06848048504693827</v>
+        <v>0.06852132887313189</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2931992350803088</v>
+        <v>-0.2931507296162613</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.2237789067436642</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2986239213.27145</v>
+        <v>3008657245.274557</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.69838572642311</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.48154433532966</v>
+        <v>24.47338178420284</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.1636733114323</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2539399192281282</v>
+        <v>0.2543581429452635</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1259808841201444</v>
+        <v>0.1262870144647288</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,7 +2297,7 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007195837484778036</v>
+        <v>0.007417247868925054</v>
       </c>
       <c r="AI14" s="6" t="n">
         <v>0.3243025635854753</v>
@@ -2306,7 +2306,7 @@
         <v>0.2103024325995957</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2791279150.877596</v>
+        <v>2791346455.219828</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.92641405820977</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.86497226705693</v>
+        <v>25.85484161635811</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.07862395234159</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1956871145614707</v>
+        <v>0.1961556182437769</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1426239133060971</v>
+        <v>0.1429905640421405</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2301082377674951</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1746907854.737402</v>
+        <v>1758474164.75708</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
         <v>461.62</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>252.14</v>
+        <v>253.67</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>371194943691</v>
@@ -2486,7 +2486,7 @@
         <v>26.28384026750692</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>19.13803301227025</v>
+        <v>19.13140676003105</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8246412554867604</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3733825336519787</v>
+        <v>0.3738582111179922</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007650193123596605</v>
+        <v>0.007728723792457926</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2474196080887633</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2217386222.15081</v>
+        <v>2231279913.950602</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.64405684754522</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.8572792229035</v>
+        <v>14.8592241758596</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.834106633523514</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3894910728823757</v>
+        <v>0.3893091996743479</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01859598504877202</v>
+        <v>0.0184731455101077</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2790438991997661</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2180548722.934889</v>
+        <v>2218338245.05305</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.26705202312139</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.19597426951325</v>
+        <v>21.19039874176189</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.442785122823678</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4279622931348481</v>
+        <v>0.4283380125108875</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08045748288171328</v>
+        <v>0.08066338058638256</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2703850990757486</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>2016902430.493835</v>
+        <v>2044085605.615438</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.52982456140351</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.39527683905725</v>
+        <v>36.38319592518539</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.236110729693026</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08612512376832493</v>
+        <v>0.08648576784426831</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06239954760547506</v>
+        <v>0.06253134600484866</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2936,7 +2936,7 @@
         <v>0.2271214315905349</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2502387716.620026</v>
+        <v>2506014798.186086</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.68592592592593</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.7834908518187</v>
+        <v>20.78020002232322</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.998251725779024</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04342076509386095</v>
+        <v>0.04358600507356658</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02251723141165529</v>
+        <v>0.02259725675283053</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.2101256912704024</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1270267645.631455</v>
+        <v>1285049893.929749</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.2946524440573409</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1303932886.174366</v>
+        <v>1314600203.184407</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>119.1776649746193</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>38.33875934521715</v>
+        <v>38.27453615383045</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.53684871080983</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.108542556150476</v>
+        <v>2.113758570335859</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7609036032661809</v>
+        <v>0.763230201573925</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.551179397477509</v>
+        <v>2.551179435893698</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.8189214740539928</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>14823592093.01787</v>
+        <v>14829123918.06132</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>668114379039</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.92743105950652</v>
+        <v>56.24818577648766</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.07937933402579</v>
+        <v>37.04864426138122</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.51534229073668</v>
+        <v>16.91246110389923</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.73117193728408</v>
+        <v>27.37393495651855</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.739110958526747</v>
+        <v>3.829019558665718</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>42.68884277276214</v>
+        <v>43.723628787396</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.38265529052438</v>
+        <v>16.77977410368693</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01714281048088179</v>
+        <v>0.01674028287058214</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4813471003572738</v>
+        <v>0.5182252116879664</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2460842665108627</v>
+        <v>0.2768644099179924</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004488081777695734</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.707465804086699</v>
+        <v>1.707465780739648</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5981026803105612</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3352473258.630615</v>
+        <v>3353184549.702962</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>87.18726591760296</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>113.9020355105908</v>
+        <v>113.1448144592746</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.957447016330656</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2345416346005853</v>
+        <v>-0.2294188086809299</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1380996781449901</v>
+        <v>0.1385235328700229</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.4018079101988982</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1302122165.90992</v>
+        <v>1308417113.858948</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.76035953686776</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.41277904922907</v>
+        <v>14.41096388212451</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.587717947463476</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09349900411543244</v>
+        <v>0.09363673837369468</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3863265676537078</v>
+        <v>-0.3862812807767462</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.4070536372001464</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2067406719.028727</v>
+        <v>2089419367.85319</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.63842794759826</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.41436604218242</v>
+        <v>18.41105992259684</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.222074555190529</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1207786301369862</v>
+        <v>0.1209798911287912</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04339998610101614</v>
+        <v>0.04350971871855358</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.8149883025196463</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2702466459.46721</v>
+        <v>2724286582.276662</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>41.25896147403685</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.15800058469767</v>
+        <v>29.13903042947119</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.55868617123032</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4150133975815149</v>
+        <v>0.4159346026938346</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1935089706837299</v>
+        <v>0.1939796323415384</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3459874906097753</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3285024862.074186</v>
+        <v>3285246311.933187</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.30466237942122</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.11467173709464</v>
+        <v>16.1121598283242</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.683503905033629</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07384516803946606</v>
+        <v>0.07401258203761629</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3315025598381095</v>
+        <v>-0.3314055265702582</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.3173823551380288</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1206435006.634154</v>
+        <v>1218311669.260813</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>19.2144610577996</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.71524699489998</v>
+        <v>5.706794087275241</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>10.77170381283647</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.361965121532926</v>
+        <v>2.366944866758582</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.69812340747675</v>
+        <v>1.701767220413196</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0006155632984901278</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885767837522308</v>
+        <v>2.885767847663744</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.109854183057</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>41769244052.72623</v>
+        <v>41815325537.65707</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.1552795031056</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.42081415794861</v>
+        <v>27.40552897220476</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.943481759435244</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.886685969539692</v>
+        <v>1.888295992512551</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2256001214062018</v>
+        <v>0.2261646080374844</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.597752252010406</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2488309271.697828</v>
+        <v>2499158898.467026</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.74260042283299</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.305237023116204</v>
+        <v>9.306140673877975</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.420400841497111</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.841127349474355</v>
+        <v>2.840754365895334</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04994950842542312</v>
+        <v>-0.0500618403053199</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2253678488322476</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1065676184.137108</v>
+        <v>1071819671.346385</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>960362682034</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.204383580509567</v>
+        <v>6.226230001567699</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00304572747235924</v>
+        <v>0.003043336513902098</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.328491136004394</v>
+        <v>5.347253428736805</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>3.85675682260281</v>
+        <v>3.870336952259862</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01388463572482881</v>
+        <v>0.01393352528724018</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>5.862519580176463</v>
+        <v>5.884687920788807</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>4.961774561128323</v>
+        <v>4.980536853860733</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.09046073285698025</v>
+        <v>0.09014332677678032</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2036.07772176465</v>
+        <v>2044.856569960634</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2673.768681811151</v>
+        <v>2686.290609405571</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.497942618736604</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>7316767238.501864</v>
+        <v>7318261698.296634</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.808547917168693</v>
+        <v>1.808547951355199</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5667836233283519</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6857758233.951178</v>
+        <v>6858090194.349263</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4736,7 @@
         <v>1.1003853227048</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12466781161.32763</v>
+        <v>12487850370.26817</v>
       </c>
       <c r="AL34" s="7" t="inlineStr"/>
       <c r="AM34" s="2" t="inlineStr">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4816,7 @@
         <v>0.1458206953958641</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>36631215478.67122</v>
+        <v>36818589189.47103</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4867,37 +4867,37 @@
         <v>2170386285600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.58780572620842</v>
+        <v>27.76167845137359</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6629399430205829</v>
+        <v>0.6624739641493647</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.89916072363153</v>
+        <v>13.98676047609139</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.59388616712771</v>
+        <v>9.654351836248262</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5182494035320432</v>
+        <v>0.5215156812853964</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.27477474575392</v>
+        <v>18.39411248032314</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.41458131216091</v>
+        <v>13.50218106462077</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01812191372746905</v>
+        <v>0.01800841531163939</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.61433628589169</v>
+        <v>40.90606718713902</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.67742886280661</v>
+        <v>40.97249579036279</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4940,7 +4940,7 @@
         <v>0.5287349731143599</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>6135998716.806361</v>
+        <v>6136366745.829875</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -4989,7 +4989,7 @@
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>10.76</v>
+        <v>10.79</v>
       </c>
       <c r="K37" s="5" t="n">
         <v>67366763183</v>
@@ -4998,7 +4998,7 @@
         <v>-21.15748031496063</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-46.069437192789</v>
+        <v>-46.35872472943611</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.865340251502146</v>
@@ -5023,7 +5023,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03679836100789124</v>
+        <v>0.03687174955558636</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5062,13 +5062,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3254051570148393</v>
+        <v>0.3254051480019132</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.222674490586299</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>581915732.3724345</v>
+        <v>586418900.891749</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
         <v>20.54942389326865</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.68812817323083</v>
+        <v>17.68194416670147</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.721867265352729</v>
@@ -5150,10 +5150,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1617636242803857</v>
+        <v>0.162169934455918</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.002483749305178362</v>
+        <v>-0.002249987747699245</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5198,7 +5198,7 @@
         <v>0.2712832767602575</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1021487235.286104</v>
+        <v>1030107347.614136</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5208,7 +5208,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
         <v>25.42760942760942</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.5305983981057</v>
+        <v>17.51463298952873</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.459012868553105</v>
@@ -5276,10 +5276,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4504701351413676</v>
+        <v>0.4517923066279228</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4482026270774806</v>
+        <v>0.4498615665005263</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5324,7 +5324,7 @@
         <v>0.6093429853265822</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4981167943.953258</v>
+        <v>4996165142.220764</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5334,7 +5334,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10 18:09 ET</t>
+          <t>2026-08-11 08:43 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-12)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -457,7 +457,7 @@
     <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="23" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="21" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
@@ -470,7 +470,7 @@
     <col width="23" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -720,7 +720,7 @@
         <v>34.80707762557078</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.13260328991657</v>
+        <v>32.12531771308112</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.593189962705351</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08323242009132459</v>
+        <v>0.0834780821917811</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1035401740604158</v>
+        <v>0.1037939822543636</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003476435669541832</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3620306300548646</v>
+        <v>0.3906505861578045</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3589074024507373</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>17114388854.16568</v>
+        <v>17147253446.78274</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.98944444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.13081589583306</v>
+        <v>25.11837719066761</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.27373920937563</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1137499299847793</v>
+        <v>0.1143014627092844</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2004188207935216</v>
+        <v>0.201048706738377</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007066155892102181</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5727221826551303</v>
+        <v>0.5737593239349764</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4828619792747939</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15985681292.08665</v>
+        <v>15986261966.69617</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.07050645481629</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.17476568629511</v>
+        <v>20.19174743859091</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.33171968350876</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1538684156112691</v>
+        <v>-0.1545800329202432</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2634514444587215</v>
+        <v>0.2641350717117343</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002472367655613729</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8145502630608524</v>
+        <v>0.8049235482471775</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4243070351098869</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10548508281.93058</v>
+        <v>10551931704.68903</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.60873015873016</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.93135473529449</v>
+        <v>24.93935986976656</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.775829745513614</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1332709197651664</v>
+        <v>-0.1335491258969342</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1566057767658497</v>
+        <v>0.1570139849300198</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8791384806184801</v>
+        <v>0.8714578936921219</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4855254718078859</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11917335193.28127</v>
+        <v>11938493974.8025</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>33.15548780487805</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.6880907450223</v>
+        <v>19.66965714252061</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.78206918588826</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6840377380554628</v>
+        <v>0.6856159497160039</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9166122189842625</v>
+        <v>0.918449015767667</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.00128735632183908</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.2835330751076</v>
+        <v>1.287433387926854</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3868971089067414</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26507945570.00901</v>
+        <v>26546254171.25901</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.26384243775548</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.93617797301916</v>
+        <v>17.93281156951709</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.686806253802882</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2412813070458097</v>
+        <v>0.2415143242569089</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2480425048920836</v>
+        <v>0.2486498460825957</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003505140873280812</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8098281895098568</v>
+        <v>0.8120164179498878</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.503225666529087</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11674755727.07027</v>
+        <v>11691759950.77169</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>282.042372881356</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>164.0279806539974</v>
+        <v>163.9056543188001</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.68540391431108</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7194771999071279</v>
+        <v>0.7207604829347574</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.106626480805009</v>
+        <v>0.1069949749941401</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.552462506992225</v>
+        <v>1.519122532459863</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6129670623171438</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>14218903523.49304</v>
+        <v>14220470381.86788</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>67.21809369951535</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.45813610433762</v>
+        <v>23.4293413001227</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.23115200954085</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.865449045079337</v>
+        <v>1.868970699537478</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.10878683516735</v>
+        <v>1.111300442059414</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006104595270140358</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.618305006030362</v>
+        <v>1.631091260127018</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4569115449892051</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7899356931.582938</v>
+        <v>7900124072.123515</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.42943244600703</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.8495197113517</v>
+        <v>41.83863905319986</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.426446297962785</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1333327783243776</v>
+        <v>0.1336275156010265</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.110013909082701</v>
+        <v>0.1102500977739813</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005866655371060657</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1732019038028125</v>
+        <v>-0.1616211432451064</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2086998004899687</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2061502316.719537</v>
+        <v>2066953152.143148</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>23.15479876160991</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.04611546136886</v>
+        <v>20.04290910233618</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.438208677559858</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1550765935790321</v>
+        <v>0.1552613766487128</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1276626803124867</v>
+        <v>0.1279892205331596</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1258126177403212</v>
+        <v>0.1424402182304574</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3831121805480643</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3245337230.368506</v>
+        <v>3248048559.862696</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>0.02885471835385391</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>24.27826432960466</v>
+        <v>24.27617433071322</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.895226663198912</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.9988114999506505</v>
+        <v>-0.9988113976295949</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02611260274713989</v>
+        <v>0.02621376213957394</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.0758810046154518</v>
+        <v>0.08697839480619256</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1603106756359845</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2140864169.778707</v>
+        <v>2142253249.204509</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.56491831470336</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.56678298702582</v>
+        <v>14.56622619850408</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.259348931066111</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06852132887313189</v>
+        <v>0.06856217269932507</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2931507296162613</v>
+        <v>-0.2931022241522139</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01657275439177991</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.794654376709318</v>
+        <v>0.7874721123975421</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.2207674321971328</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2976089578.152963</v>
+        <v>2976183624.079183</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.82582837723024</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.5749816753694</v>
+        <v>24.56679070169642</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.22662446266409</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2543581429452635</v>
+        <v>0.2547763666623992</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1262870144647288</v>
+        <v>0.1265931448093129</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007386582878562373</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3181989387988375</v>
+        <v>0.3295923735042958</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.2091230498372582</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2711634914.500236</v>
+        <v>2711691853.053385</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.83141131246568</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.77541821668076</v>
+        <v>25.76532659465324</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.03537587549525</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1961556182437769</v>
+        <v>0.1966241219260829</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1429905640421405</v>
+        <v>0.1433572147781834</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.006002422342547734</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3079211294101107</v>
+        <v>0.3256516795038522</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2273255569714734</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1710751937.856757</v>
+        <v>1722848331.141357</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
         <v>461.62</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>253.67</v>
+        <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>365246597845</v>
@@ -2486,7 +2486,7 @@
         <v>25.86264548903608</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.82482870484143</v>
+        <v>18.81831315073131</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8114264973929696</v>
@@ -2498,10 +2498,10 @@
         <v>-0.7836449109667459</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.80198726254707</v>
+        <v>15.91389193203431</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.9044220608869901</v>
+        <v>0.9108268915022137</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>0.06466042432521812</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3738582111179922</v>
+        <v>0.3743338885840053</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007728723792457926</v>
+        <v>0.007807254461319246</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2543,7 +2543,7 @@
         <v>0.2367504286032538</v>
       </c>
       <c r="AF16" s="6" t="n">
-        <v>1.624810775142646</v>
+        <v>1.736715444629896</v>
       </c>
       <c r="AG16" s="6" t="n">
         <v>4.672413793103448</v>
@@ -2552,13 +2552,13 @@
         <v>0.02225316392749695</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.458319323100949</v>
+        <v>0.4374242242844034</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2483756006759494</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2204446841.144328</v>
+        <v>2204506365.264689</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.64599483204134</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.86061910255884</v>
+        <v>14.86256474743816</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.834278812385753</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3893091996743476</v>
+        <v>0.3891273264663195</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.0184731455101077</v>
+        <v>0.01835030597144338</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02553191489361702</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4703398158221439</v>
+        <v>-0.4666716542953378</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2779923081361774</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2216796508.465765</v>
+        <v>2237280258.790283</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>274.9</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>171.81</v>
+        <v>172.7</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>626091608477</v>
@@ -2738,7 +2738,7 @@
         <v>30.03468208092486</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.02771320083167</v>
+        <v>21.0221833881708</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.393321778809137</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4283380125108875</v>
+        <v>0.4287137318869267</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08066338058638256</v>
+        <v>0.08086927829105162</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.0201693610469592</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1944390918849237</v>
+        <v>-0.1896726125562956</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2713123307581893</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>2001498497.569615</v>
+        <v>2021403861.694336</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>39.74035087719298</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.57696405544557</v>
+        <v>36.56482686176493</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.242693957438595</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08648576784426831</v>
+        <v>0.08684641192021147</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06253134600484844</v>
+        <v>0.0626631444042216</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,13 +2930,13 @@
         <v>0.008520218965212784</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.1039966308651403</v>
+        <v>-0.08468093795397051</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2243903390386019</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2491907723.673444</v>
+        <v>2492438543.10079</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.51185185185185</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.6133962579686</v>
+        <v>20.61013287773746</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.966157547764041</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04358600507356658</v>
+        <v>0.04375124505327244</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02259725675283053</v>
+        <v>0.02267728209400532</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.0295485692641438</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06328158348376121</v>
+        <v>-0.05919632594530998</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2109117554934247</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1263529765.900081</v>
+        <v>1272070258.562622</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3182,13 +3182,13 @@
         <v>0.02612277138343489</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7302071878552674</v>
+        <v>0.7343849151377686</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2943439675718214</v>
+        <v>0.295356468551779</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1277036354.717337</v>
+        <v>1310329868.951518</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>120.3857868020305</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>38.66253085544949</v>
+        <v>38.59787360867817</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.72475952063915</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.11375857033586</v>
+        <v>2.118974584521243</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7632302015739245</v>
+        <v>0.765556799881669</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.554895924202571</v>
+        <v>2.51525293549024</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.8097512421847737</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>14623724887.19987</v>
+        <v>14635482616.13342</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>693513424646</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>56.38606676342525</v>
+        <v>57.50362844702467</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>38.45708604139888</v>
+        <v>38.42523538957313</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.95391856242304</v>
+        <v>17.28994217357583</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>27.44103659039467</v>
+        <v>27.98491299128538</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.838405621317589</v>
+        <v>3.914482129127487</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>43.83165589883165</v>
+        <v>44.70724406510002</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.82123156221074</v>
+        <v>17.15725517336353</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01669934781593806</v>
+        <v>0.01637480218700104</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.466207468312235</v>
+        <v>0.4965068623269526</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.233116219801663</v>
+        <v>0.2583614877831579</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004323711500627994</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.70410608207412</v>
+        <v>1.705896902464451</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.6019892204222717</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3330279077.22749</v>
+        <v>3331312641.102295</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>87.35580524344566</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>113.3635316142498</v>
+        <v>112.6148676584224</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.961230903771477</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2294188086809299</v>
+        <v>-0.2242959827612748</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1385235328700227</v>
+        <v>0.1389473875950555</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.213704469478871</v>
+        <v>1.265941707272572</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3956350606923887</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1284379714.484576</v>
+        <v>1288106874.223022</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.75883607556368</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.40957085896551</v>
+        <v>14.40775632443047</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.587467807982228</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09363673837369468</v>
+        <v>0.09377447263195671</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3862812807767463</v>
+        <v>-0.3862359938997847</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01643448922574221</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.591435703855653</v>
+        <v>1.568191013115493</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.399907185630438</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2084336444.42255</v>
+        <v>2088316233.588053</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.82270742358079</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.57545134249731</v>
+        <v>18.57211690028577</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.2508442954108</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1209798911287912</v>
+        <v>0.1211811521205957</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04350971871855358</v>
+        <v>0.0436194513360908</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02826944048318094</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8635781874848639</v>
+        <v>0.8546380457079791</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.814699737127365</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2691317138.865739</v>
+        <v>2699865576.637421</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>40.69346733668343</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.73965171785727</v>
+        <v>28.7209658967999</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.35914523798167</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4159346026938349</v>
+        <v>0.4168558078061544</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1939796323415384</v>
+        <v>0.1944502939993467</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005318185560220631</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3555584196308001</v>
+        <v>0.3320741350988915</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3474061035500372</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3197238705.605843</v>
+        <v>3219814061.073405</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.29099678456592</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.09943595982967</v>
+        <v>16.09692681708643</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.681384726031187</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07401258203761629</v>
+        <v>0.0741799960357663</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3314055265702582</v>
+        <v>-0.3313084933024071</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.0192933519293352</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.370243088014204</v>
+        <v>1.352870904051747</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3142738248603538</v>
+        <v>0.322152966023086</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1197072886.030894</v>
+        <v>1194956609.942271</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>19.38228074090605</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.756637399164102</v>
+        <v>5.7481358485949</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>10.86578419921572</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.366944866758582</v>
+        <v>2.371924611984238</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.701767220413196</v>
+        <v>1.705411033349641</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0006102335006678027</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.877981522582489</v>
+        <v>2.868536644271777</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.104036454073715</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>40346255445.32456</v>
+        <v>40352131591.2207</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.21739130434784</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.42703362456838</v>
+        <v>27.41175348951338</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.950499557426012</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.888295992512551</v>
+        <v>1.889906015485408</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2261646080374844</v>
+        <v>0.226729094668767</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6405346345722298</v>
+        <v>0.6383687028847039</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.5969691294717443</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2472450176.80952</v>
+        <v>2472942421.694387</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.17441860465117</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.158205720466976</v>
+        <v>9.159095179092819</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.381924968600854</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.840754365895334</v>
+        <v>2.840381382316314</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05006184030532013</v>
+        <v>-0.05017417218521736</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.06461307287753569</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3187266965253447</v>
+        <v>0.3062990619011497</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2289882825450986</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1059850825.521401</v>
+        <v>1066870911.944052</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1005509453102</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.226230001567699</v>
+        <v>6.571403454286189</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003186404148083614</v>
+        <v>0.00318390471765837</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.347253428736805</v>
+        <v>5.643697653908879</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>3.870336952259862</v>
+        <v>4.084903000841286</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01393352528724018</v>
+        <v>0.01470598037333981</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>5.884687920788807</v>
+        <v>6.234947702463837</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>4.980536853860733</v>
+        <v>5.276981079032808</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.09014332677678032</v>
+        <v>0.08540840469209572</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1952.998837627774</v>
+        <v>2062.944758723554</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2565.632873606331</v>
+        <v>2711.052110962736</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.474187826986787</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>7103438928.15257</v>
+        <v>7105448239.474687</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.809579229548798</v>
+        <v>1.799766393794629</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5606419512382607</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6732044821.662903</v>
+        <v>6733772778.520813</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-86.55194805194805</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>690.082978723404</v>
+        <v>678.5334728033474</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>105.1512582059729</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.71089650612616</v>
+        <v>2.716569350606417</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>1.089993977891825</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12527058247.16339</v>
+        <v>12528220886.90183</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9957568325951488</v>
+        <v>0.9892128145495841</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.1399067487223421</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>36316595101.57367</v>
+        <v>36328345679.20044</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2189005748800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.76167845137359</v>
+        <v>27.99350875159383</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6681572425953612</v>
+        <v>0.6676879263782057</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.98676047609139</v>
+        <v>14.10356014603787</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.654351836248262</v>
+        <v>9.734972728409</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5215156812853964</v>
+        <v>0.5258707182898673</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.39411248032314</v>
+        <v>18.55322945974876</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.50218106462077</v>
+        <v>13.61898073456725</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01800841531163939</v>
+        <v>0.01785927729663617</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.54961838554249</v>
+        <v>40.92603706860675</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.61548195373433</v>
+        <v>40.99538836507539</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.260626451215467</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.194439180183407</v>
+        <v>2.138329927839239</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.5167404863919046</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>6046957901.341457</v>
+        <v>6047074488.38145</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>10.79</v>
+        <v>11.25</v>
       </c>
       <c r="K37" s="5" t="n">
         <v>67868190523</v>
@@ -5046,7 +5046,7 @@
         <v>-21.31496062992126</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-46.70378408730315</v>
+        <v>-46.9989081258263</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.879224436466842</v>
@@ -5058,10 +5058,10 @@
         <v>0.1586229628273211</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>10.90780008644628</v>
+        <v>15.95408107818182</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>1.827279261331856</v>
+        <v>2.672634376934792</v>
       </c>
       <c r="S37" s="4" t="n">
         <v>0.03212108622906654</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03687174955558636</v>
+        <v>0.03694513810328104</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5095,13 +5095,13 @@
         <v>0.7767453385368271</v>
       </c>
       <c r="AD37" s="6" t="n">
-        <v>0.04546561909982338</v>
+        <v>0.97518119252086</v>
       </c>
       <c r="AE37" s="6" t="n">
-        <v>0.01535250082263903</v>
+        <v>0.3292921191181309</v>
       </c>
       <c r="AF37" s="6" t="n">
-        <v>-0.3100826446280991</v>
+        <v>4.736198347107438</v>
       </c>
       <c r="AG37" s="6" t="n">
         <v>1.789928057553957</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3442511134751091</v>
+        <v>0.3204841361180128</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2209874765700913</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>583029041.3562726</v>
+        <v>587880347.1372477</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.66767738023044</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.78369648661255</v>
+        <v>17.77748124105387</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.737530492548143</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.162169934455918</v>
+        <v>0.1625762446314496</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.002249987747699245</v>
+        <v>-0.002016226190220571</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01038701916023591</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9793789980896928</v>
+        <v>0.9785274782874405</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2678941644173603</v>
+        <v>0.2718846023122524</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1012615138.670662</v>
+        <v>1025165057.276611</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.48569023569023</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.86583550822303</v>
+        <v>16.85048948618433</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.219750573799697</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.451792306627923</v>
+        <v>0.4531144781144778</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4498615665005263</v>
+        <v>0.4515205059235725</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.0137509024029702</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>1.998438228448679</v>
+        <v>1.98105773579057</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.6127741281112189</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4939561488.727</v>
+        <v>4966603601.292827</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11 18:20 ET</t>
+          <t>2026-08-12 08:48 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-13)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>34.50342465753425</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>31.84506011209461</v>
+        <v>31.83784136802122</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.509500069619534</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08347808219178088</v>
+        <v>0.08372374429223739</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1037939822543636</v>
+        <v>0.1040477904483113</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003507030603804797</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3744672204061955</v>
+        <v>0.3588762738548325</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3582422766282615</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16911219756.43743</v>
+        <v>16929031762.01243</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.35722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.55100629205544</v>
+        <v>24.53886058006913</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.01908933699776</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1143014627092842</v>
+        <v>0.1148529954337898</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.201048706738377</v>
+        <v>0.2016785926832321</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007229453932538635</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5731733997285215</v>
+        <v>0.568565887274319</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4845166794073197</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15875627704.26795</v>
+        <v>15896670107.81464</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.05759682224429</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.17647735617661</v>
+        <v>20.19347485658569</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.324662536568079</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1545800329202434</v>
+        <v>-0.1552916502292175</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2641350717117341</v>
+        <v>0.2648186989647474</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002474238807707981</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8049849611532941</v>
+        <v>0.8130758820493846</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4241400435149272</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10406739490.53534</v>
+        <v>10419473396.42141</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.21269841269841</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.48228635542368</v>
+        <v>24.49014982472447</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.706628620049505</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1335491258969344</v>
+        <v>-0.133827332028702</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1570139849300198</v>
+        <v>0.1574221930941904</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8581650972141978</v>
+        <v>0.8745641241335206</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4875085829202108</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11675162670.02577</v>
+        <v>11679036394.68542</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.16006097560975</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.26562514513767</v>
+        <v>20.2466685563559</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.41174199478483</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6856159497160037</v>
+        <v>0.6871941613765451</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9184490157676672</v>
+        <v>0.9202858125510713</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.0012494979695658</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.294028039543656</v>
+        <v>1.287236652158015</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3898761610174746</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26232962243.11102</v>
+        <v>26248735467.36425</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.51059085841695</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.32609156265016</v>
+        <v>17.32284027520999</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.460571838723669</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2415143242569089</v>
+        <v>0.2417473414680085</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2486498460825957</v>
+        <v>0.249257187273108</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003627882871210158</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8048669324670079</v>
+        <v>0.8034096217797102</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5105727366532526</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>11657896700.52818</v>
+        <v>11663328339.27409</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>277.5508474576271</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>161.2954564044056</v>
+        <v>161.1752575304113</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.48338882839055</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7207604829347574</v>
+        <v>0.7220437659623871</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1069949749941401</v>
+        <v>0.107363469183271</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.509159391095901</v>
+        <v>1.552301804686668</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6015666534970902</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13915059614.43599</v>
+        <v>13925153483.85396</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>67.21324717285945</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.42765200902723</v>
+        <v>23.3989298803063</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.22926070363745</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.868970699537478</v>
+        <v>1.872492353995618</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.111300442059414</v>
+        <v>1.113814048951478</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006105035452469655</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.626261652060529</v>
+        <v>1.616543287608421</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4494165876705625</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7738945612.091441</v>
+        <v>7760877756.539612</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.69337016574586</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.07146484130618</v>
+        <v>42.06052932174962</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.434384258924952</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1336275156010265</v>
+        <v>0.1339222528776756</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1102500977739813</v>
+        <v>0.1104862864652614</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005834188979280204</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1694329856479229</v>
+        <v>-0.1712013112001938</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.208565608550272</v>
+        <v>0.2085665712381329</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>2018963314.693897</v>
+        <v>2018972649.460856</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>22.97523219814241</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>19.88747539088605</v>
+        <v>19.88429491491145</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.388280063676481</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1552613766487128</v>
+        <v>0.1554461597183934</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1279892205331599</v>
+        <v>0.128315760753833</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1328917565824635</v>
+        <v>0.1255985341204179</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3829973292257892</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3181611695.173342</v>
+        <v>3182135239.295883</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>0.02849374101049069</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.97247533738194</v>
+        <v>23.9704118400292</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.859006894337474</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.9988113976295949</v>
+        <v>-0.9988112953085392</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02621376213957394</v>
+        <v>0.02631492153200798</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.08198416941892493</v>
+        <v>0.07411588932479125</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1637473262717242</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2120716573.819336</v>
+        <v>2121816439.819336</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.69991401547722</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.69256016785361</v>
+        <v>14.69199859319534</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.287617508139218</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06856217269932507</v>
+        <v>0.0686030165255187</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2931022241522139</v>
+        <v>-0.2930537186881665</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01643025357358015</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.790513828080069</v>
+        <v>0.7962276776120267</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.2196341268027958</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2941196067.620506</v>
+        <v>2941250735.065409</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.53695836873407</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.33657437297758</v>
+        <v>24.32846556445131</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.08393518652221</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.254776366662399</v>
+        <v>0.2551945903795345</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1265931448093129</v>
+        <v>0.1268992751538971</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007456457626175505</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3267872206202349</v>
+        <v>0.3166597319173221</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.2080145670684637</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2654446951.902746</v>
+        <v>2666126604.755758</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.73750686436024</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.68685212101962</v>
+        <v>25.67679911046044</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>13.99262777641593</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1966241219260829</v>
+        <v>0.1970926256083891</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1433572147781834</v>
+        <v>0.1437238655142268</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.006020760009290194</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3239985713692412</v>
+        <v>0.3074672293818079</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2268770466106752</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1683493104.442415</v>
+        <v>1700208115.614827</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>26.08128094656292</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.97739782392678</v>
+        <v>18.97083173598898</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8182860664787205</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3743338885840051</v>
+        <v>0.3748095660500184</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007807254461319246</v>
+        <v>0.007885785130180345</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02206661899948224</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4481057505983703</v>
+        <v>0.4599799819776727</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2490283317513428</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2160430154.322404</v>
+        <v>2169315928.119507</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.64082687338501</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.85884445588686</v>
+        <v>14.86079012315726</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.833819668753116</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3891273264663195</v>
+        <v>0.3889454532582917</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01835030597144316</v>
+        <v>0.01822746643277884</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02553830746119179</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4646783504151378</v>
+        <v>-0.4729615580940703</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2687278092920338</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2147101246.177606</v>
+        <v>2175209295.952606</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>274.9</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>172.7</v>
+        <v>172.72</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>628646100798</v>
@@ -2738,7 +2738,7 @@
         <v>30.15722543352601</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.10795519106325</v>
+        <v>21.10240573595613</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.41940692540514</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4287137318869267</v>
+        <v>0.4290894512629662</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08086927829105162</v>
+        <v>0.08107517599572067</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.02008740320478418</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1888679383453603</v>
+        <v>-0.194029611488932</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2712700066143139</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1978087308.133992</v>
+        <v>1989296296.493225</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.70526315789473</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.45263609600344</v>
+        <v>37.44021245391797</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.272867084605787</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08684641192021125</v>
+        <v>0.08720705599615486</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0626631444042216</v>
+        <v>0.06279494280359521</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,13 +2930,13 @@
         <v>0.008318248426859753</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.09797819932034875</v>
+        <v>-0.1011138760750545</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2329152591127281</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2490491172.889397</v>
+        <v>2490727485.263748</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.34666666666667</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.45187181125436</v>
+        <v>20.44863451504199</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.935702221389834</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04375124505327244</v>
+        <v>0.04391648503297807</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02267728209400532</v>
+        <v>0.02275730743518034</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.02977722256922757</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06631685557059426</v>
+        <v>-0.06219609214560512</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2114100351383031</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1252569961.979622</v>
+        <v>1260907943.725586</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3182,13 +3182,13 @@
         <v>0.02696328218268643</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7312307911515228</v>
+        <v>0.7269972980629675</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.3060387693884721</v>
+        <v>0.3017778294722244</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1279175265.323104</v>
+        <v>1268527608.241069</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.5710659898477</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.29851387636817</v>
+        <v>39.23290276866927</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.06465701488924</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.118974584521243</v>
+        <v>2.124190598706627</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.765556799881669</v>
+        <v>0.7678833981894129</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.54596464577007</v>
+        <v>2.5548284002754</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7885838754143993</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>14255370652.09895</v>
+        <v>14267518418.01371</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>697633542969</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>56.8577648766328</v>
+        <v>57.25689404934688</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>38.65351722349067</v>
+        <v>38.62153037675755</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.09574670998514</v>
+        <v>17.21575514253768</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>27.67059481154984</v>
+        <v>27.86483638329652</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.870515835652935</v>
+        <v>3.897686017013613</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>43.41066260255714</v>
+        <v>43.7177796948821</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.96305970977284</v>
+        <v>17.08306814232538</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01656080823609939</v>
+        <v>0.01644536533965003</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4709596683760251</v>
+        <v>0.4825123057216834</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2368797252890718</v>
+        <v>0.2463592901147995</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004298176313623231</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.71145277719301</v>
+        <v>1.702879451057057</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5581428453027781</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3234471371.333114</v>
+        <v>3235311123.116862</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>86.59176029962543</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>111.6298979704479</v>
+        <v>110.8975198001248</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.94407728070642</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2242959827612746</v>
+        <v>-0.2191731568416195</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1389473875950555</v>
+        <v>0.1393712423200881</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.267748928010622</v>
+        <v>1.210422221085799</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3705963642209106</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1263113978.593593</v>
+        <v>1263492345.095266</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.801492992078</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.44675606119675</v>
+        <v>14.4449370731483</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.594471713457185</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09377447263195671</v>
+        <v>0.09391220689021917</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3862359938997846</v>
+        <v>-0.3861907070228232</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01639012350440123</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.570474596224806</v>
+        <v>1.591391812653029</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3913212785971237</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2041744965.146012</v>
+        <v>2041772935.241292</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.60960698689956</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.38204909877291</v>
+        <v>18.37874996603303</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.217575022359871</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1211811521205957</v>
+        <v>0.1213824131124006</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.0436194513360908</v>
+        <v>0.04372918395362801</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02856174252055259</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8531042136046734</v>
+        <v>0.8577427662760566</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8142891128293692</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2664386279.745094</v>
+        <v>2674668785.552927</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>40.88810720268007</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.85834040232423</v>
+        <v>28.83958960408907</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.4278260923759</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4168558078061542</v>
+        <v>0.4177770129184737</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1944502939993467</v>
+        <v>0.1949209556571549</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005292869374277966</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3439141470872392</v>
+        <v>0.3583835671274493</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3439227592081389</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3133101046.958781</v>
+        <v>3149847966.700846</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.5008038585209</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.29224517595484</v>
+        <v>16.28970637902726</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.713920356598092</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07417999603576608</v>
+        <v>0.07434741003391609</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3313084933024071</v>
+        <v>-0.3312114600345559</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01906205502732993</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.355459039959953</v>
+        <v>1.372629679969007</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3201714469451439</v>
+        <v>0.3078235681358153</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1177842799.248734</v>
+        <v>1195280766.007741</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>20.33675518857398</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.031201028722478</v>
+        <v>6.022307130243052</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.40086639674768</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.371924611984238</v>
+        <v>2.376904357209894</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.705411033349641</v>
+        <v>1.709054846286086</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005815931262276553</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.886665981242478</v>
+        <v>2.886991993611568</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.075775443064874</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>39820654453.59482</v>
+        <v>39845047529.587</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.6024844720497</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.85294402524542</v>
+        <v>26.83799205672978</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.768036809666034</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.889906015485408</v>
+        <v>1.891516038458266</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.226729094668767</v>
+        <v>0.2272935813000496</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6343839063554789</v>
+        <v>0.6350462397302735</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.5946020096933298</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2460830644.159185</v>
+        <v>2461262707.510961</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>34.76479915433404</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.052434040643577</v>
+        <v>9.053313311961952</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.354186548605878</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.840381382316314</v>
+        <v>2.840008398737293</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05017417218521725</v>
+        <v>-0.05028650406511415</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.0653743823641201</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3188118301556941</v>
+        <v>0.3174511466549481</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2247612196475463</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1042829807.674739</v>
+        <v>1047251341.650988</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1096086937193</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.571403454286189</v>
+        <v>6.960269749120944</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00347071463080571</v>
+        <v>0.00346799431972323</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.643697653908879</v>
+        <v>5.977666464545775</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.084903000841286</v>
+        <v>4.326629308736814</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01470598037333981</v>
+        <v>0.01557621458426218</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.234947702463837</v>
+        <v>6.629544165363558</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.276981079032808</v>
+        <v>5.610949889669703</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.08540840469209572</v>
+        <v>0.08063668591143248</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1892.386277269551</v>
+        <v>2006.001484845691</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2486.935894813144</v>
+        <v>2637.200833559972</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.473525842204661</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6974388340.245719</v>
+        <v>6974852516.017978</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.80901062480875</v>
+        <v>1.811209404673427</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5389257862039879</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6660494838.088857</v>
+        <v>6672486836.072286</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-94.90259740259741</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>743.9993026499304</v>
+        <v>731.7524005486968</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>115.2963942291403</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.716569350606417</v>
+        <v>2.722242195086675</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>1.10272469013281</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12870111607.21927</v>
+        <v>12873288459.89327</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9890106496280635</v>
+        <v>0.9958477566059306</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.134498422286289</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>35789253954.51804</v>
+        <v>35797588271.77368</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2225777892000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.99350875159383</v>
+        <v>28.22533905181407</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6789041217011965</v>
+        <v>0.678427591551431</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.10356014603787</v>
+        <v>14.22035981598436</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.734972728409</v>
+        <v>9.815593620569736</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5258707182898673</v>
+        <v>0.5302257552943384</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.55322945974876</v>
+        <v>18.71234643917438</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.61898073456725</v>
+        <v>13.73578040451373</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01785927729663617</v>
+        <v>0.01771258918742355</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.23337575480873</v>
+        <v>40.60405532338131</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.30158129643182</v>
+        <v>40.6757388264172</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.2563206338110218</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.147691178230917</v>
+        <v>2.196734241783934</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.5132289272101356</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5927185772.920711</v>
+        <v>5943587528.062439</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-21.77165354330709</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-48.00590357144799</v>
+        <v>-48.31118487282726</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.91948857289215</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03694513810328104</v>
+        <v>0.03701852665097616</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3236868742151141</v>
+        <v>0.3450725059864887</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2194489582757639</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>594691381.7795691</v>
+        <v>594692806.6762161</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.8659793814433</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.94805242047421</v>
+        <v>17.94178192544461</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.763796519691221</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1625762446314496</v>
+        <v>0.1629825548069814</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.002016226190220571</v>
+        <v>-0.001782464632741787</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01028830504533829</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9835116062803617</v>
+        <v>0.9798644967999806</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2689112895493893</v>
+        <v>0.2661835749696821</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>1011703396.396225</v>
+        <v>1006486082.861837</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.79629629629629</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.75241846724208</v>
+        <v>17.7362804377712</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.5526651340598</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4531144781144776</v>
+        <v>0.454436649601033</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4515205059235725</v>
+        <v>0.4531794453466185</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.01305227435880702</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>1.989896702434712</v>
+        <v>2.007822491491851</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5949336314872947</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>5013247436.043003</v>
+        <v>5013724821.489868</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12 18:20 ET</t>
+          <t>2026-08-13 08:50 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-14)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>34.84703196347032</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.15490308023874</v>
+        <v>32.34253063867542</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.604201790742957</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08372374429223739</v>
+        <v>0.07743677675611438</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1040477904483113</v>
+        <v>0.1012921408475342</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003472449714997052</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.358555089992907</v>
+        <v>0.3585550879520824</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3567044161892045</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16839234877.07648</v>
+        <v>16857794217.60488</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.60444444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.76061378271988</v>
+        <v>24.74837043204732</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.1186668354232</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.11485299543379</v>
+        <v>0.1154045281582952</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2016785926832318</v>
+        <v>0.2023084786280869</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007164707776525519</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5670375484984397</v>
+        <v>0.5670375533803765</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4844543351225436</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15662594144.85641</v>
+        <v>15669498358.77492</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.19761668321748</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.35923604624504</v>
+        <v>20.37640197143261</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.401205437987112</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1552916502292174</v>
+        <v>-0.1560032675381916</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2648186989647474</v>
+        <v>0.2655023262177605</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002454094006236286</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8125603066757093</v>
+        <v>0.8125603260385326</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.424457271422282</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10301328943.58323</v>
+        <v>10303810485.87962</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.04206349206349</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.29315108885513</v>
+        <v>24.30095631673304</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.676812503867574</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1338273320287019</v>
+        <v>-0.1341055381604698</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1574221930941901</v>
+        <v>0.1578304012583605</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8730743292693236</v>
+        <v>0.8730743766047532</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4868284168972011</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11514224476.10144</v>
+        <v>11529614592.38454</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.34451219512195</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.35599279640762</v>
+        <v>20.33696947170969</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.52735718427873</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6871941613765451</v>
+        <v>0.6887723730370863</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9202858125510713</v>
+        <v>0.9221226093344757</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001242787394584998</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.288209958725038</v>
+        <v>1.288209998116713</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3899540705771908</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25991157391.50929</v>
+        <v>26028545423.84572</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.10962467484207</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.80525227354528</v>
+        <v>17.80191169718374</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.640487910312467</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2417473414680085</v>
+        <v>0.2419803586791078</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.249257187273108</v>
+        <v>0.2498645284636203</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003529589727213137</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8017336489484927</v>
+        <v>0.8017336284132619</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5147719236148901</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10950558279.68449</v>
+        <v>10954851682.15475</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>288.1016949152543</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>167.3021909255859</v>
+        <v>167.1776086170648</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.95793370003571</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7220437659623871</v>
+        <v>0.7233270489900161</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.107363469183271</v>
+        <v>0.1077319633724021</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.562784047404773</v>
+        <v>1.56278403910487</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6078566119454361</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13734900053.69094</v>
+        <v>13748941353.22601</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>67.49919224555735</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>23.49847586249147</v>
+        <v>23.4697021805701</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>26.34084775193799</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.872492353995618</v>
+        <v>1.876014008453759</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.113814048951478</v>
+        <v>1.116327655843542</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006079172849552439</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.61001393173489</v>
+        <v>1.610013985697339</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4486103128284245</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7652153345.089616</v>
+        <v>7652641553.84084</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.30989452536414</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.60423887331161</v>
+        <v>42.59316774896042</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.452926308555897</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1339222528776756</v>
+        <v>0.1342169901543246</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1104862864652614</v>
+        <v>0.1107224751565417</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.00575973384623382</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1686335302326443</v>
+        <v>-0.1686335588318439</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2104074188876483</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1970851246.805115</v>
+        <v>1971716110.241496</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.22291021671827</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.9641185034722</v>
+        <v>20.96076638297525</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.735197846409869</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1554461597183934</v>
+        <v>0.1556309427880742</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.128315760753833</v>
+        <v>0.1286423009745059</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1388388953091828</v>
+        <v>0.1388388035977539</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.4051753562142125</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3180789099.351001</v>
+        <v>3181458711.156718</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.74654262006537</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.8298573777573</v>
+        <v>23.82780633319064</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.842242635994978</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4651020181109875</v>
+        <v>-0.4650559752825321</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02631492153200798</v>
+        <v>0.02641608092444203</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0</v>
@@ -2054,7 +2054,7 @@
         <v>0.163979830169361</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2133066197.703866</v>
+        <v>2133215843.437703</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.61092003439381</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.60871791767118</v>
+        <v>14.60815956894746</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.268981853826693</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06860301652551892</v>
+        <v>0.06864386035171233</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2930537186881665</v>
+        <v>-0.2930052132241191</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.2153974698854823</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2816942899.171859</v>
+        <v>2833632850.22756</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.04927782497876</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.73662495278151</v>
+        <v>24.72838559497869</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.33699881451178</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2551945903795347</v>
+        <v>0.2556128140966702</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1268992751538971</v>
+        <v>0.1272054054984812</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.2099575503806636</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2551911667.274534</v>
+        <v>2612870398.199056</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.13893465129049</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.01213472137546</v>
+        <v>26.00195838832362</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.17536965025796</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1970926256083891</v>
+        <v>0.1975611292906951</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1437238655142268</v>
+        <v>0.1440905162502699</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2279291470181595</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1660819221.729537</v>
+        <v>1660834456.203613</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.66137225901872</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.66540129826614</v>
+        <v>18.65894539333038</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8051116587911464</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3748095660500184</v>
+        <v>0.3752852435160317</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007885785130180345</v>
+        <v>0.007964315799041666</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2514493312978702</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2144770603.281793</v>
+        <v>2153837472.560323</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.49224806201551</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.75381773556569</v>
+        <v>14.75574990328723</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.820619289314795</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3889454532582917</v>
+        <v>0.3887635800502638</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01822746643277906</v>
+        <v>0.01810462689411474</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2696622355063973</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2163691529.819219</v>
+        <v>2175745900.439606</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
         <v>274.9</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>172.72</v>
+        <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>631586176865</v>
@@ -2738,7 +2738,7 @@
         <v>30.29826589595375</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.20109827217427</v>
+        <v>21.19552579403505</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.449429452613629</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4290894512629662</v>
+        <v>0.4294651706390054</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08107517599572067</v>
+        <v>0.08128107370038995</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2705221613701496</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1963865320.438332</v>
+        <v>1977184190.411937</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.60350877192982</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.34661999109894</v>
+        <v>37.33423562435524</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.269685191195428</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08720705599615486</v>
+        <v>0.08756770007209802</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06279494280359521</v>
+        <v>0.06292674120296882</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2936,7 +2936,7 @@
         <v>0.2325521647708706</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2409071270.667314</v>
+        <v>2409148544.626795</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.37185185185185</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.47276018557816</v>
+        <v>20.46952009584519</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.940345634387352</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04391648503297807</v>
+        <v>0.04408172501268393</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02275730743518034</v>
+        <v>0.02283733277635558</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.2102077291966089</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1249849383.864374</v>
+        <v>1249884410.19104</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.3017730096380883</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1243021771.185335</v>
+        <v>1249159477.924601</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.5913705583756</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.23940191393151</v>
+        <v>39.17399869142732</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.06781517976032</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.124190598706627</v>
+        <v>2.12940661289201</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7678833981894129</v>
+        <v>0.7702099964971572</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.552838788643761</v>
+        <v>2.552838889930714</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7799069001480146</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>14050450542.24095</v>
+        <v>14058657252.61454</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>712213905569</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>58.39622641509434</v>
+        <v>58.12046625544267</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>39.42871048258371</v>
+        <v>39.39610912066787</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.55832466817635</v>
+        <v>17.47541028385819</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.41930777900977</v>
+        <v>28.28510539417376</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.975244534715912</v>
+        <v>3.956472532912996</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>44.59445939476257</v>
+        <v>44.38227076699626</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.42563766796405</v>
+        <v>17.34272328364588</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01612451006958151</v>
+        <v>0.01620101493001883</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4810584901296451</v>
+        <v>0.4752844266275953</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2451370563669339</v>
+        <v>0.2400496336715938</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004210184533795119</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.701487585533064</v>
+        <v>1.701487618225239</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5587856346081734</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3152656840.993636</v>
+        <v>3152720408.754476</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>86.26591760299623</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>110.480215119216</v>
+        <v>109.7601042369432</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.936761764987499</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2191731568416196</v>
+        <v>-0.2140503309219643</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1393712423200884</v>
+        <v>0.1397950970451212</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,17 +3568,17 @@
         <v>0.3694304484461434</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1251658710.705356</v>
+        <v>1255669209.019572</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.88406459475929</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.52041991552011</v>
+        <v>14.51859188263834</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.608029273340851</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09391220689021917</v>
+        <v>0.0940499411484812</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3861907070228232</v>
+        <v>-0.3861454201458615</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3861892608322345</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2023160290.830383</v>
+        <v>2032212161.252441</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.71091703056769</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.46909385094106</v>
+        <v>18.46577969058727</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.233391562007034</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1213824131124006</v>
+        <v>0.1215836741042053</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04372918395362801</v>
+        <v>0.04383891657116523</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.814413350976909</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2645253452.458574</v>
+        <v>2651525180.973765</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>40.53098827470687</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.58770307699827</v>
+        <v>28.56914018752022</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.30181268310869</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4177770129184739</v>
+        <v>0.4186982180307937</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1949209556571549</v>
+        <v>0.1953916173149635</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,7 +3937,7 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005339504897301318</v>
+        <v>0.005529611108815143</v>
       </c>
       <c r="AI27" s="6" t="n">
         <v>0.353427941443768</v>
@@ -3946,7 +3946,7 @@
         <v>0.3389829771227302</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3102550041.789225</v>
+        <v>3119488534.789225</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.55466237942122</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.33983776148074</v>
+        <v>16.33729194498051</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.722272415019482</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07434741003391609</v>
+        <v>0.07451482403206611</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3312114600345559</v>
+        <v>-0.3311144267667047</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.3075523667243538</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1181101983.400409</v>
+        <v>1188447828.166656</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.19683106449453</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.277000714941193</v>
+        <v>6.267757978231452</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.88302837694131</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.376904357209894</v>
+        <v>2.38188410243555</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.709054846286086</v>
+        <v>1.712698659222532</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005579945885053115</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.891687497409799</v>
+        <v>2.891687545379202</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.080534272329429</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>39234046731.38277</v>
+        <v>39239356787.75431</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.03726708074535</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.33419632798835</v>
+        <v>27.31898486360753</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.930147943252782</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.891516038458266</v>
+        <v>1.893126061431124</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2272935813000494</v>
+        <v>0.2278580679313318</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.594523666023931</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2465114612.699979</v>
+        <v>2466128672.191645</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.41226215644821</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.22192309998405</v>
+        <v>9.222818920943952</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.398031147952776</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.840008398737293</v>
+        <v>2.839635415158273</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05028650406511403</v>
+        <v>-0.05039883594501093</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2291893923898994</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1034660004.485401</v>
+        <v>1039535060.133286</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1176016597920</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.960269749120944</v>
+        <v>7.18747252812552</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003720889961456819</v>
+        <v>0.003717975849527797</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.977666464545775</v>
+        <v>6.172794308962837</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.326629308736814</v>
+        <v>4.467862657170157</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01557621458426218</v>
+        <v>0.01608466603334042</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.629544165363558</v>
+        <v>6.860094907731933</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.610949889669703</v>
+        <v>5.806077734086766</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.08063668591143248</v>
+        <v>0.07808768428991608</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1869.592740236755</v>
+        <v>1932.168158969717</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2457.891716725141</v>
+        <v>2541.082737562446</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.460979414009908</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6909303867.419021</v>
+        <v>6910028010.981018</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.80792977401632</v>
+        <v>1.807929832235032</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5374386488538413</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6527418184.498853</v>
+        <v>6528187909.047139</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-91.74675324675324</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>707.4190672153634</v>
+        <v>695.9628879892038</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>111.4623848144796</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.722242195086675</v>
+        <v>2.727915039566934</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>1.091917546418777</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12858715940.07777</v>
+        <v>12867571615.37397</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>0.1348585334943447</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>35413479490.9603</v>
+        <v>35551119445.93628</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2232727775200</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.22533905181407</v>
+        <v>27.76167845137359</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6805459487055238</v>
+        <v>0.6800686011950002</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.22035981598436</v>
+        <v>13.98676047609139</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.815593620569736</v>
+        <v>9.654351836248262</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5302257552943384</v>
+        <v>0.5215156812853964</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.71234643917438</v>
+        <v>18.39411248032314</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.73578040451373</v>
+        <v>13.50218106462077</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01771258918742355</v>
+        <v>0.01800841531163939</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.47455304891888</v>
+        <v>39.82187944362001</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.54601342042077</v>
+        <v>39.8950222675423</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.5130305966717054</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5786299679.856009</v>
+        <v>5786637801.044006</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-21.8503937007874</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-48.48590886875069</v>
+        <v>-48.79621596022223</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.926430665402187</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03701852665097616</v>
+        <v>0.03709191519867083</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3334052691096194</v>
+        <v>0.3334052818137015</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2193693361780137</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>604479103.12165</v>
+        <v>604535344.0466499</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.83990297149788</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.91935991245943</v>
+        <v>17.91310162815691</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.760342577284027</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1629825548069814</v>
+        <v>0.1633888649825135</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.001782464632741787</v>
+        <v>-0.001548703075262892</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.2616091516837668</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>990304383.4347646</v>
+        <v>994429821.4264933</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>26.31481481481481</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>18.09278858727414</v>
+        <v>18.07635607878727</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.684376996050951</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4544366496010332</v>
+        <v>0.4557588210875883</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4531794453466185</v>
+        <v>0.4548383847696644</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5372,7 +5372,7 @@
         <v>0.5975973394850834</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4929072936.041052</v>
+        <v>4929314618.797607</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13 18:21 ET</t>
+          <t>2026-08-14 08:44 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-15)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>34.92351598173516</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.41351765147733</v>
+        <v>32.40689375063213</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.62528157584352</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07743677675611438</v>
+        <v>0.07765700256458374</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1012921408475342</v>
+        <v>0.1015382957273441</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -790,7 +790,7 @@
         <v>0.3541994996991685</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16348280502.73323</v>
+        <v>16370362031.63625</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.52222222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.67465527297585</v>
+        <v>24.6624604560597</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.08554892583452</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1154045281582952</v>
+        <v>0.1159560608828007</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2023084786280869</v>
+        <v>0.2029383645729421</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -920,7 +920,7 @@
         <v>0.4829771386370983</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15358563950.0182</v>
+        <v>15389097499.29535</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.17477656405164</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.34934011409672</v>
+        <v>20.36651217416417</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.388719716478233</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1560032675381916</v>
+        <v>-0.1567148848471658</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2655023262177605</v>
+        <v>0.2661859534707733</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1046,7 +1046,7 @@
         <v>0.4188406779370541</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10187453368.12771</v>
+        <v>10197387419.94242</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.84523809523809</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.07364755625517</v>
+        <v>24.08138474501521</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.642419960550743</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1341055381604699</v>
+        <v>-0.1343837442922377</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1578304012583605</v>
+        <v>0.1582386094225305</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1172,7 +1172,7 @@
         <v>0.482398518582443</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11367071838.08923</v>
+        <v>11377917102.8422</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.32317073170731</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.32433220705794</v>
+        <v>20.30535620387122</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.51398022020506</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6887723730370863</v>
+        <v>0.6903505846976274</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9221226093344757</v>
+        <v>0.9239594061178797</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1298,7 +1298,7 @@
         <v>0.3813410411393719</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25670013872.60815</v>
+        <v>25674533961.38438</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1337,10 +1337,10 @@
         <v>-0.09311046208554041</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.259215070643642</v>
+        <v>-0.2541097622660596</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>796.25</v>
+        <v>790.8</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>520.26</v>
@@ -1352,7 +1352,7 @@
         <v>21.91936083240431</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.64871777498669</v>
+        <v>17.64540718835541</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.583343351595633</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2419803586791078</v>
+        <v>0.2422133758902074</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2498645284636203</v>
+        <v>0.2504718696541324</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1424,7 +1424,7 @@
         <v>0.5029497839348533</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10698293100.2583</v>
+        <v>10705468044.51762</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>290.0593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>168.3135666000788</v>
+        <v>168.1883244283675</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.04598178465339</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7233270489900161</v>
+        <v>0.7246103320176458</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1077319633724021</v>
+        <v>0.1081004575615332</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1550,7 +1550,7 @@
         <v>0.6072060681422552</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13292984150.59671</v>
+        <v>13301320810.17558</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>63.48788368336026</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>22.07495634469926</v>
+        <v>22.04795880845553</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>24.77547689922481</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.876014008453759</v>
+        <v>1.8795356629119</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.116327655843542</v>
+        <v>1.118841262735605</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1676,7 +1676,7 @@
         <v>0.4687631189585583</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7713800297.403812</v>
+        <v>7716967634.244893</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.2722250125565</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.55995583877513</v>
+        <v>42.54889909500164</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.451793393099831</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1342169901543246</v>
+        <v>0.1345117274309735</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1107224751565417</v>
+        <v>0.1109586638478215</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1802,7 +1802,7 @@
         <v>0.2103189011222713</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1916239131.906185</v>
+        <v>1920721253.678996</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.19814241486068</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.93933410651005</v>
+        <v>20.93598648426654</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.728311141043793</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1556309427880744</v>
+        <v>0.155815725857755</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1286423009745061</v>
+        <v>0.1289688411951793</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1928,7 +1928,7 @@
         <v>0.4029103956078296</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3105094645.700845</v>
+        <v>3108114934.479014</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.67362333417148</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.69149434067441</v>
+        <v>23.68945538055917</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.825982987436539</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4650559752825321</v>
+        <v>-0.4650099324540767</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02641608092444203</v>
+        <v>0.02651724031687608</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.07572599545342923</v>
+        <v>0.06337194040170699</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1619784056065648</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2125464096.920893</v>
+        <v>2125574429.087626</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.59931212381771</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.59729728731485</v>
+        <v>14.5967393964131</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.266551116307667</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0686438603517121</v>
+        <v>0.06868470417790573</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2930052132241191</v>
+        <v>-0.2929567077600717</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01653621430933745</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7852155663688458</v>
+        <v>0.7926174781125103</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.2148730588593354</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2800989237.299885</v>
+        <v>2801020468.033651</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.93882752761257</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.64042034317004</v>
+        <v>24.63221576232971</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.28244115010789</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.25561281409667</v>
+        <v>0.2560310378138055</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1272054054984812</v>
+        <v>0.1275115358430654</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007359604558561034</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.325243314078175</v>
+        <v>0.320613700447486</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.210531830388713</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2540386160.035753</v>
+        <v>2592814872.986857</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.26249313563975</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.10513348421408</v>
+        <v>26.09492476246978</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.23161714904655</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1975611292906951</v>
+        <v>0.1980296329730014</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1440905162502699</v>
+        <v>0.1444571669863131</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.005919654306241108</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3169291182853491</v>
+        <v>0.311293425421233</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2278688170133619</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1637640640.379195</v>
+        <v>1637644321.78772</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.83306539772362</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.7837872321521</v>
+        <v>18.77729262674758</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.810498438045538</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3752852435160317</v>
+        <v>0.3757609209820452</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.007964315799041888</v>
+        <v>0.008042846467902987</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02227864486097627</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4309474178129207</v>
+        <v>0.4273424181534725</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2515375816636645</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2144728048.138379</v>
+        <v>2144747224.050903</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.68346253229974</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.89343674432414</v>
+        <v>14.89538745209014</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.837607603722373</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3887635800502636</v>
+        <v>0.3885817068422355</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01810462689411474</v>
+        <v>0.01798178735545042</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02548566431382348</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4726315108722751</v>
+        <v>-0.482021854902214</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2464029004481813</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2167610164.095443</v>
+        <v>2167732042.893423</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.09826589595376</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.05561332599598</v>
+        <v>21.05008054122516</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.406856524686252</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4294651706390054</v>
+        <v>0.429840890015045</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08128107370038995</v>
+        <v>0.08148697140505923</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.02012675244862685</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1900767091553943</v>
+        <v>-0.1888776125070776</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2647682899247202</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1941143118.082886</v>
+        <v>1950438995.783234</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.44561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.18905409971853</v>
+        <v>37.17672607083396</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.264747770386251</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08756770007209802</v>
+        <v>0.0879283441480414</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06292674120296882</v>
+        <v>0.0630585396023422</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,13 +2930,13 @@
         <v>0.008371649171510367</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.1009676663757074</v>
+        <v>-0.09581012521430746</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2326489209441878</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2353240820.147439</v>
+        <v>2354887473.072993</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.41481481481481</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.51066913804536</v>
+        <v>20.50742356236667</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.948266750654932</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0440817250126837</v>
+        <v>0.04424696499238956</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02283733277635558</v>
+        <v>0.02291735811753082</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.02968246281563473</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06591646084753192</v>
+        <v>-0.06325592238672778</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2096994686128575</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1238097254.488559</v>
+        <v>1238108541.86498</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3182,13 +3182,13 @@
         <v>0.02732691967184088</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7292705810665301</v>
+        <v>0.7113728343167208</v>
       </c>
       <c r="AJ21" s="4" t="n">
         <v>0.302494737801638</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1238927272.37616</v>
+        <v>1246762957.724101</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>130.5558375634518</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.71903933020704</v>
+        <v>41.64961882036091</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>20.30660535044183</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.12940661289201</v>
+        <v>2.134622627077393</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7702099964971572</v>
+        <v>0.7725365948049012</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3314,7 +3314,7 @@
         <v>0.7775434718225019</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13999931378.51288</v>
+        <v>14010778736.37207</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>57.31494920174165</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>39.31466903362801</v>
+        <v>39.28218882215359</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>17.23321091455665</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4578514994674636</v>
+        <v>0.4590569140948249</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2253963958120258</v>
+        <v>0.2261794287238537</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3438,7 +3438,7 @@
         <v>0.5574069555414716</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3046808660.644991</v>
+        <v>3050719892.762451</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>86.76779026217224</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>110.3986599599385</v>
+        <v>109.6837405052561</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.948029340922389</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2140503309219643</v>
+        <v>-0.2089275050023091</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1397950970451212</v>
+        <v>0.140218951770154</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.264244272361418</v>
+        <v>1.194686973677663</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3535881126457306</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1230414128.973859</v>
+        <v>1230438659.650218</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83516148689823</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.47389272767132</v>
+        <v>14.47207078165253</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599999795992776</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.0940499411484812</v>
+        <v>0.09418767540674344</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3861454201458615</v>
+        <v>-0.3861001332689</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01635527505724346</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.572566233242105</v>
+        <v>1.580334748130775</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3848500054748674</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2034718101.748641</v>
+        <v>2034892303.452555</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.4646288209607</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.24619000210175</v>
+        <v>18.24291642783489</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.194941008726862</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1215836741042056</v>
+        <v>0.1217849350960103</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04383891657116523</v>
+        <v>0.04394864918870267</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02876408330488221</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8698463489755045</v>
+        <v>0.8664545533513828</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8143375055874656</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2617834963.739296</v>
+        <v>2629521002.387238</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.53634840871023</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.86804685184434</v>
+        <v>27.84996300006564</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.95084287812336</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4186982180307934</v>
+        <v>0.419619423143113</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1953916173149635</v>
+        <v>0.1958622789727718</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005668722885032538</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3411157118196864</v>
+        <v>0.3529040073765982</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3446181444999699</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3069319724.708968</v>
+        <v>3075578226.455892</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.47186495176849</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.26023630479675</v>
+        <v>16.25770328519866</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.70943268341645</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07451482403206633</v>
+        <v>0.07468223803021634</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3311144267667047</v>
+        <v>-0.3310173934988535</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01909362778927997</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.351549649644295</v>
+        <v>1.36637449424097</v>
       </c>
       <c r="AJ28" s="4" t="n">
         <v>0.3045258496970822</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1186419702.405075</v>
+        <v>1186419890.783742</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.68399910734211</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.411810236703802</v>
+        <v>6.402382877692578</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.15613673261404</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.38188410243555</v>
+        <v>2.386863847661206</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.712698659222531</v>
+        <v>1.716342472158976</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4198,7 +4198,7 @@
         <v>1.050687251493404</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>38139635488.1471</v>
+        <v>38152585758.48775</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.01863354037268</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.62125047612836</v>
+        <v>26.60644400549233</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.70206950855281</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.893126061431124</v>
+        <v>1.894736084403982</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2278580679313318</v>
+        <v>0.2284225545626144</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6417550071938375</v>
+        <v>0.6485303200215876</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.5982244735138025</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2454649190.530744</v>
+        <v>2456647014.064077</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.39904862579282</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.219377570600315</v>
+        <v>9.220273231291374</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.397136360211002</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.839635415158273</v>
+        <v>2.839262431579253</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05039883594501116</v>
+        <v>-0.05051116782490817</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.06420306084359836</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3207204238114388</v>
+        <v>0.3208469192009179</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2281935388440251</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1012927014.667162</v>
+        <v>1017187998.246778</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.18747252812552</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00373278760820884</v>
+        <v>0.003729866466096307</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.172794308962837</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1924.497317961359</v>
+        <v>1926.005321358852</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2530.995714135663</v>
+        <v>2533.909984251388</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.430291791726731</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6776585754.310918</v>
+        <v>6778361160.750463</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
         <v>0.5259440508918425</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6214946752.773335</v>
+        <v>6216314955.651958</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-90.90909090909091</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>689.608636977058</v>
+        <v>678.6188579017263</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>110.4447156488688</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.727915039566934</v>
+        <v>2.733587884047191</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.9917175357859459</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12978521028.7073</v>
+        <v>12988067724.2408</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9891942385995555</v>
+        <v>0.9964541428148497</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.128640414015669</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34899714071.58089</v>
+        <v>34937487814.2275</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.76167845137359</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6735284167332304</v>
+        <v>0.673056322584938</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>13.98676047609139</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.21827344126651</v>
+        <v>40.24718470031183</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.29212650628424</v>
+        <v>40.32392184075995</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.2580039873343497</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.158356594349318</v>
+        <v>2.207244908647239</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.5035963642370442</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5610093350.278818</v>
+        <v>5610601770.845032</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.03937007874016</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-49.21823728744577</v>
+        <v>-49.53526016825236</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.943091687359823</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03709191519867083</v>
+        <v>0.03716530374636595</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5116,7 +5116,7 @@
         <v>0.2196391625615738</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>602499645.3661188</v>
+        <v>603079066.6113981</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.7689508793208</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.85211420227318</v>
+        <v>17.84588158006442</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.750944640966779</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1633888649825135</v>
+        <v>0.1637951751580453</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.001548703075262892</v>
+        <v>-0.001314941517783996</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01033637000700771</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9803042152526011</v>
+        <v>0.9680213288500964</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2622922822554877</v>
+        <v>0.2516285048311834</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>983021716.4662832</v>
+        <v>983257475.4817709</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.3063973063973</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.38364689247842</v>
+        <v>17.36787277808759</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.428223082633094</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4557588210875883</v>
+        <v>0.457080992574143</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4548383847696644</v>
+        <v>0.4564973241927106</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.01330494944119212</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>1.999609042574185</v>
+        <v>2.031736199265938</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5900110526330925</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4832666951.987203</v>
+        <v>4832803017.053731</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14 17:52 ET</t>
+          <t>2026-08-15 08:20 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-16)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>34.92351598173516</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.40689375063213</v>
+        <v>32.4002725565032</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.62528157584352</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07765700256458374</v>
+        <v>0.07787722837305311</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1015382957273441</v>
+        <v>0.1017844506071541</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,7 +784,7 @@
         <v>0.003464844899159939</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3586790971624771</v>
+        <v>0.3654802030955034</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3541994996991685</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.52222222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.6624604560597</v>
+        <v>24.6502776871415</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.08554892583452</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1159560608828007</v>
+        <v>0.1165075936073059</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2029383645729421</v>
+        <v>0.2035682505177971</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,7 +914,7 @@
         <v>0.007186112232539362</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.566891268453768</v>
+        <v>0.575210297885807</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4829771386370983</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.17477656405164</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.36651217416417</v>
+        <v>20.38371324044938</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.388719716478233</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1567148848471658</v>
+        <v>-0.15742650215614</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2661859534707733</v>
+        <v>0.2668695807237869</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,7 +1040,7 @@
         <v>0.002457357617808615</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.812536262534543</v>
+        <v>0.800936970610205</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4188406779370541</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.84523809523809</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.08138474501521</v>
+        <v>24.0891269087867</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.642419960550743</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1343837442922377</v>
+        <v>-0.1346619504240053</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1582386094225305</v>
+        <v>0.1586468175867009</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,10 +1166,10 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8737784119386238</v>
+        <v>0.8558725183414375</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.482398518582443</v>
+        <v>0.4823985185824431</v>
       </c>
       <c r="AK5" s="5" t="n">
         <v>11377917102.8422</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.32317073170731</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.30535620387122</v>
+        <v>20.28641560187817</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.51398022020506</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6903505846976274</v>
+        <v>0.6919287963581691</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9239594061178797</v>
+        <v>0.9257962029012841</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,7 +1292,7 @@
         <v>0.001243560135015101</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.28800087491103</v>
+        <v>1.291456316257423</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3813410411393719</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.91936083240431</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.64540718835541</v>
+        <v>17.64209784350595</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.583343351595633</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2422133758902074</v>
+        <v>0.2424463931013066</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2504718696541324</v>
+        <v>0.2510792108446449</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,7 +1418,7 @@
         <v>0.00356022717640078</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8019174703197121</v>
+        <v>0.8108184213878351</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5029497839348533</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>290.0593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>168.1883244283675</v>
+        <v>168.0632685035394</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.04598178465339</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7246103320176458</v>
+        <v>0.7258936150452751</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1081004575615332</v>
+        <v>0.1084689517506641</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.562132021823696</v>
+        <v>1.512227202443606</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6072060681422552</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>63.48788368336026</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>22.04795880845553</v>
+        <v>22.02102722719182</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>24.77547689922481</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.8795356629119</v>
+        <v>1.88305731737004</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.118841262735605</v>
+        <v>1.121354869627669</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,7 +1670,7 @@
         <v>0.006463268785465279</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.613252892265167</v>
+        <v>1.628221427995763</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4687631189585583</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.2722250125565</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.54889909500164</v>
+        <v>42.53784809464723</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.451793393099831</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1345117274309735</v>
+        <v>0.1348064647076226</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1109586638478215</v>
+        <v>0.1111948525391018</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,7 +1796,7 @@
         <v>0.005764228488190615</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1687586565188836</v>
+        <v>-0.1669479354783426</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2103189011222713</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.19814241486068</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.93598648426654</v>
+        <v>20.93263993223696</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.728311141043793</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.155815725857755</v>
+        <v>0.1560005089274357</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1289688411951793</v>
+        <v>0.1292953814158522</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1385539394457838</v>
+        <v>0.1417915381918108</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.4029103956078296</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.67362333417148</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.68945538055917</v>
+        <v>23.6874167713716</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.825982987436539</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4650099324540767</v>
+        <v>-0.4649638896256213</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02651724031687608</v>
+        <v>0.02661839970931013</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06337194040170699</v>
+        <v>0.07572599545342923</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1619784056065648</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.59931212381771</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.5967393964131</v>
+        <v>14.59618154815354</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.266551116307667</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06868470417790573</v>
+        <v>0.06872554800409914</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2929567077600717</v>
+        <v>-0.2929082022960243</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,7 +2174,7 @@
         <v>0.01653621430933745</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7926174781125103</v>
+        <v>0.7852155663688458</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.2148730588593354</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.93882752761257</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.63221576232971</v>
+        <v>24.62401664346927</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.28244115010789</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2560310378138055</v>
+        <v>0.2564492615309411</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1275115358430654</v>
+        <v>0.1278176661876498</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,7 +2300,7 @@
         <v>0.007359604558561034</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.320613700447486</v>
+        <v>0.325243314078175</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.210531830388713</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.26249313563975</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.09492476246978</v>
+        <v>26.08472402208746</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.23161714904655</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1980296329730014</v>
+        <v>0.1984981366553076</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1444571669863131</v>
+        <v>0.1448238177223564</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,7 +2426,7 @@
         <v>0.005919654306241108</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.311293425421233</v>
+        <v>0.3169291182853491</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2278688170133619</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.83306539772362</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.77729262674758</v>
+        <v>18.77080251088717</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.810498438045538</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3757609209820452</v>
+        <v>0.3762365984480582</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008042846467902987</v>
+        <v>0.008121377136764085</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,7 +2552,7 @@
         <v>0.02227864486097627</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4273424181534725</v>
+        <v>0.4309474178129207</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2515375816636645</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.68346253229974</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.89538745209014</v>
+        <v>14.89733867092142</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.837607603722373</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3885817068422355</v>
+        <v>0.3883998336342074</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01798178735545042</v>
+        <v>0.0178589478167861</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,7 +2678,7 @@
         <v>0.02548566431382348</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.482021854902214</v>
+        <v>-0.4726315108722751</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2464029004481813</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.09826589595376</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.05008054122516</v>
+        <v>21.04455066339086</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.406856524686252</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.429840890015045</v>
+        <v>0.430216609391084</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08148697140505923</v>
+        <v>0.08169286910972806</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,7 +2804,7 @@
         <v>0.02012675244862685</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1888776125070776</v>
+        <v>-0.1900767091553943</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2647682899247202</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.44561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.17672607083396</v>
+        <v>37.16440621262949</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.264747770386251</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.0879283441480414</v>
+        <v>0.08828898822398457</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0630585396023422</v>
+        <v>0.06319033800171536</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,7 +2930,7 @@
         <v>0.008371649171510367</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.09581012521430746</v>
+        <v>-0.1009676663757074</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2326489209441878</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.41481481481481</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.50742356236667</v>
+        <v>20.50417901367495</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.948266750654932</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04424696499238956</v>
+        <v>0.04441220497209519</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02291735811753082</v>
+        <v>0.02299738345870583</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,7 +3056,7 @@
         <v>0.02968246281563473</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06325592238672778</v>
+        <v>-0.06591646084753192</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2096994686128575</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3182,13 +3182,13 @@
         <v>0.02732691967184088</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7113728343167208</v>
+        <v>0.7292705810665301</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.302494737801638</v>
+        <v>0.3026649267504622</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1246762957.724101</v>
+        <v>1249466616.124675</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>130.5558375634518</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.64961882036091</v>
+        <v>41.58042895826804</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>20.30660535044183</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.134622627077393</v>
+        <v>2.139838641262777</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7725365948049012</v>
+        <v>0.7748631931126455</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.549679313510372</v>
+        <v>2.535974518596775</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7775434718225019</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>57.31494920174165</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>39.28218882215359</v>
+        <v>39.24976223408813</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>17.23321091455665</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4590569140948249</v>
+        <v>0.4602623287221861</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2261794287238537</v>
+        <v>0.2269624616356813</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,7 +3432,7 @@
         <v>0.004218905904299163</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.701859350747158</v>
+        <v>1.711158171331724</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5574069555414716</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>86.76779026217224</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>109.6837405052561</v>
+        <v>108.9780208230836</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.948029340922389</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2089275050023091</v>
+        <v>-0.2038046790826539</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.140218951770154</v>
+        <v>0.1406428064951866</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,7 +3562,7 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.194686973677663</v>
+        <v>1.264244272361418</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3535881126457306</v>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83516148689823</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.47207078165253</v>
+        <v>14.4702492942622</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599999795992776</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09418767540674344</v>
+        <v>0.09432540966500547</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3861001332689</v>
+        <v>-0.3860548463919383</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,7 +3688,7 @@
         <v>0.01635527505724346</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.580334748130775</v>
+        <v>1.572566233242105</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3848500054748674</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.4646288209607</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.24291642783489</v>
+        <v>18.23964402799033</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.194941008726862</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1217849350960103</v>
+        <v>0.121986196087815</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04394864918870267</v>
+        <v>0.04405838180623989</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,7 +3814,7 @@
         <v>0.02876408330488221</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8664545533513828</v>
+        <v>0.8698463489755045</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8143375055874656</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.53634840871023</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.84996300006564</v>
+        <v>27.83190260264844</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.95084287812336</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.419619423143113</v>
+        <v>0.4205406282554325</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1958622789727718</v>
+        <v>0.19633294063058</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,7 +3940,7 @@
         <v>0.005668722885032538</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3529040073765982</v>
+        <v>0.3411157118196864</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3446181444999699</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.47186495176849</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.25770328519866</v>
+        <v>16.25517105466523</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.70943268341645</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07468223803021634</v>
+        <v>0.07484965202836613</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3310173934988535</v>
+        <v>-0.3309203602310022</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01909362778927997</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.36637449424097</v>
+        <v>1.351549649644295</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3045258496970822</v>
+        <v>0.3126999356772434</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1186419890.783742</v>
+        <v>1162637898.926748</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.68399910734211</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.402382877692578</v>
+        <v>6.392983200291511</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.15613673261404</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.386863847661206</v>
+        <v>2.391843592886862</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.716342472158976</v>
+        <v>1.719986285095422</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,7 +4192,7 @@
         <v>0.000545458287878476</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.889941370587172</v>
+        <v>2.878930119561414</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.050687251493404</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.01863354037268</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.60644400549233</v>
+        <v>26.59165399611956</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.70206950855281</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.894736084403982</v>
+        <v>1.89634610737684</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2284225545626144</v>
+        <v>0.228987041193897</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,7 +4318,7 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6485303200215876</v>
+        <v>0.6417550071938375</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.5982244735138025</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.39904862579282</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.220273231291374</v>
+        <v>9.221169066025857</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.397136360211002</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.839262431579253</v>
+        <v>2.838889448000232</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05051116782490817</v>
+        <v>-0.05062349970480517</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,7 +4444,7 @@
         <v>0.06420306084359836</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3208469192009179</v>
+        <v>0.3207204238114388</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2281935388440251</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.18747252812552</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003729866466096307</v>
+        <v>0.003726949892365204</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.172794308962837</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1926.005321358852</v>
+        <v>1927.513324756344</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2533.909984251388</v>
+        <v>2536.824254367113</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.808024874240311</v>
+        <v>1.806747078820497</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5259440508918425</v>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-90.90909090909091</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>678.6188579017263</v>
+        <v>667.9738562091503</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>110.4447156488688</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.733587884047191</v>
+        <v>2.739260728527449</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4858,7 +4858,7 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9964541428148497</v>
+        <v>0.9891942385995555</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.128640414015669</v>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.76167845137359</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.673056322584938</v>
+        <v>0.6725848897800161</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>13.98676047609139</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.24718470031183</v>
+        <v>40.27609595935715</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.32392184075995</v>
+        <v>40.35571717523568</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,7 +4982,7 @@
         <v>0.2580039873343497</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.207244908647239</v>
+        <v>2.158356594349318</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.5035963642370442</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.03937007874016</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-49.53526016825236</v>
+        <v>-49.85639351985908</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.943091687359823</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03716530374636595</v>
+        <v>0.03723869229406085</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,7 +5110,7 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3341525451416469</v>
+        <v>0.3462505543057409</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2196391625615738</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.7689508793208</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.84588158006442</v>
+        <v>17.83965330826726</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.750944640966779</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1637951751580453</v>
+        <v>0.1642014853335771</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.001314941517783996</v>
+        <v>-0.001081179960305101</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01033637000700771</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9680213288500964</v>
+        <v>0.9803042152526011</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2516285048311834</v>
+        <v>0.2622922822554877</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>983257475.4817709</v>
+        <v>983165569.4868978</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.3063973063973</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.36787277808759</v>
+        <v>17.35212726495707</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.428223082633094</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.457080992574143</v>
+        <v>0.4584031640606983</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4564973241927106</v>
+        <v>0.4581562636157563</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,7 +5366,7 @@
         <v>0.01330494944119212</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.031736199265938</v>
+        <v>1.999609042574185</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5900110526330925</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15 08:20 ET</t>
+          <t>2026-08-16 08:21 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-17)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>34.92351598173516</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.4002725565032</v>
+        <v>32.39365406743182</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.62528157584352</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07787722837305311</v>
+        <v>0.07809745418152247</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1017844506071541</v>
+        <v>0.102030605486964</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,7 +784,7 @@
         <v>0.003464844899159939</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3654802030955034</v>
+        <v>0.3586790971624771</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3541994996991685</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.52222222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.6502776871415</v>
+        <v>24.63810694837564</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.08554892583452</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1165075936073059</v>
+        <v>0.1170591263318113</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2035682505177971</v>
+        <v>0.2041981364626524</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,7 +914,7 @@
         <v>0.007186112232539362</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.575210297885807</v>
+        <v>0.566891268453768</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4829771386370983</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.17477656405164</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.38371324044938</v>
+        <v>20.40094338650832</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.388719716478233</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.15742650215614</v>
+        <v>-0.1581381194651141</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2668695807237869</v>
+        <v>0.2675532079767995</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,7 +1040,7 @@
         <v>0.002457357617808615</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.800936970610205</v>
+        <v>0.812536262534543</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4188406779370541</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.84523809523809</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.0891269087867</v>
+        <v>24.09687405236959</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.642419960550743</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1346619504240053</v>
+        <v>-0.1349401565557732</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1586468175867009</v>
+        <v>0.1590550257508709</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,10 +1166,10 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8558725183414375</v>
+        <v>0.8737784119386238</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4823985185824431</v>
+        <v>0.482398518582443</v>
       </c>
       <c r="AK5" s="5" t="n">
         <v>11377917102.8422</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.32317073170731</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.28641560187817</v>
+        <v>20.26751030210565</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.51398022020506</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6919287963581691</v>
+        <v>0.69350700801871</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9257962029012841</v>
+        <v>0.9276329996846879</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,7 +1292,7 @@
         <v>0.001243560135015101</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.291456316257423</v>
+        <v>1.28800087491103</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3813410411393719</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.91936083240431</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.64209784350595</v>
+        <v>17.63878973973975</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.583343351595633</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2424463931013066</v>
+        <v>0.2426794103124061</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2510792108446449</v>
+        <v>0.251686552035157</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,7 +1418,7 @@
         <v>0.00356022717640078</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8108184213878351</v>
+        <v>0.8019174703197121</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5029497839348533</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>290.0593220338983</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>168.0632685035394</v>
+        <v>167.9383984104533</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.04598178465339</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7258936150452751</v>
+        <v>0.7271768980729043</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1084689517506641</v>
+        <v>0.1088374459397949</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.512227202443606</v>
+        <v>1.562132021823696</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6072060681422552</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>63.48788368336026</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>22.02102722719182</v>
+        <v>21.99416135951097</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>24.77547689922481</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.88305731737004</v>
+        <v>1.88657897182818</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.121354869627669</v>
+        <v>1.123868476519732</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,7 +1670,7 @@
         <v>0.006463268785465279</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.628221427995763</v>
+        <v>1.613252892265167</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4687631189585583</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.2722250125565</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.53784809464723</v>
+        <v>42.52680283323792</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.451793393099831</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1348064647076226</v>
+        <v>0.1351012019842719</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1111948525391018</v>
+        <v>0.1114310412303821</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,7 +1796,7 @@
         <v>0.005764228488190615</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1669479354783426</v>
+        <v>-0.1687586565188836</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2103189011222713</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.19814241486068</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.93263993223696</v>
+        <v>20.92929444990816</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.728311141043793</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1560005089274357</v>
+        <v>0.1561852919971163</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1292953814158522</v>
+        <v>0.1296219216365253</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1417915381918108</v>
+        <v>0.1385539394457838</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.4029103956078296</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.67362333417148</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.6874167713716</v>
+        <v>23.68537851302113</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.825982987436539</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4649638896256213</v>
+        <v>-0.464917846797166</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02661839970931013</v>
+        <v>0.02671955910174395</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.59931212381771</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.59618154815354</v>
+        <v>14.59562374253129</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.266551116307667</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06872554800409914</v>
+        <v>0.06876639183029254</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2929082022960243</v>
+        <v>-0.2928596968319769</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.93882752761257</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.62401664346927</v>
+        <v>24.61582298113628</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.28244115010789</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2564492615309411</v>
+        <v>0.2568674852480766</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1278176661876498</v>
+        <v>0.1281237965322342</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.26249313563975</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.08472402208746</v>
+        <v>26.07453125371081</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.23161714904655</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1984981366553076</v>
+        <v>0.1989666403376136</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1448238177223564</v>
+        <v>0.1451904684583993</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.83306539772362</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.77080251088717</v>
+        <v>18.76431687991719</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.810498438045538</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3762365984480582</v>
+        <v>0.3767122759140717</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008121377136764085</v>
+        <v>0.008199907805625184</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.68346253229974</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.89733867092142</v>
+        <v>14.89929040101885</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.837607603722373</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3883998336342074</v>
+        <v>0.3882179604261793</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.0178589478167861</v>
+        <v>0.01773610827812178</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,7 +2675,7 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02548566431382348</v>
+        <v>0.02573552376788057</v>
       </c>
       <c r="AI17" s="6" t="n">
         <v>-0.4726315108722751</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.09826589595376</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.04455066339086</v>
+        <v>21.0390236902027</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.406856524686252</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.430216609391084</v>
+        <v>0.4305923287671234</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08169286910972806</v>
+        <v>0.08189876681439734</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.44561403508771</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.16440621262949</v>
+        <v>37.15209451698484</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.264747770386251</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08828898822398457</v>
+        <v>0.08864963229992795</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06319033800171536</v>
+        <v>0.06332213640108897</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.41481481481481</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.50417901367495</v>
+        <v>20.50093549148282</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.948266750654932</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04441220497209519</v>
+        <v>0.04457744495180083</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02299738345870583</v>
+        <v>0.02307740879988085</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>130.5558375634518</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>41.58042895826804</v>
+        <v>41.51146859635353</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>20.30660535044183</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.139838641262777</v>
+        <v>2.14505465544816</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7748631931126455</v>
+        <v>0.7771897914203891</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.535974518596775</v>
+        <v>2.549679313510372</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7775434718225019</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>710741608843</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>57.31494920174165</v>
+        <v>58.58490566037735</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>39.24976223408813</v>
+        <v>39.21738913674629</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.23321091455665</v>
+        <v>17.61505592722384</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>27.89308970282331</v>
+        <v>28.51113106747184</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.901638043393348</v>
+        <v>3.988088620450051</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>43.76245127197653</v>
+        <v>44.73964202028324</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.10052391434435</v>
+        <v>17.48236892701154</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01642870758796575</v>
+        <v>0.0160725792802868</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4602623287221861</v>
+        <v>0.4938502269005944</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2269624616356813</v>
+        <v>0.2549492754471894</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,7 +3432,7 @@
         <v>0.004218905904299163</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.711158171331724</v>
+        <v>1.701859350747158</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5574069555414716</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>86.76779026217224</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>108.9780208230836</v>
+        <v>108.2813244710181</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.948029340922389</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.2038046790826539</v>
+        <v>-0.1986818531629987</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1406428064951866</v>
+        <v>0.1410666612202194</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83516148689823</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.4702492942622</v>
+        <v>14.46842826532716</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599999795992776</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09432540966500547</v>
+        <v>0.09446314392326771</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3860548463919383</v>
+        <v>-0.3860095595149767</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.4646288209607</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.23964402799033</v>
+        <v>18.23637280193618</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.194941008726862</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.121986196087815</v>
+        <v>0.1221874570796198</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04405838180623989</v>
+        <v>0.04416811442377711</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.53634840871023</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.83190260264844</v>
+        <v>27.81386561399262</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.95084287812336</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4205406282554325</v>
+        <v>0.421461833367752</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.19633294063058</v>
+        <v>0.1968036022883886</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.47186495176849</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.25517105466523</v>
+        <v>16.25263961282781</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.70943268341645</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07484965202836613</v>
+        <v>0.07501706602651614</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3309203602310022</v>
+        <v>-0.3308233269631511</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.68399910734211</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.392983200291511</v>
+        <v>6.383611082756827</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.15613673261404</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.391843592886862</v>
+        <v>2.396823338112518</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.719986285095422</v>
+        <v>1.723630098031867</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,7 +4192,7 @@
         <v>0.000545458287878476</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.878930119561414</v>
+        <v>2.889941370587172</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.050687251493404</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>77.01863354037268</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.59165399611956</v>
+        <v>26.57688042057379</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.70206950855281</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.89634610737684</v>
+        <v>1.897956130349698</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.228987041193897</v>
+        <v>0.2295515278251796</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.39904862579282</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.221169066025857</v>
+        <v>9.222065074854495</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.397136360211002</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.838889448000232</v>
+        <v>2.838516464421212</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05062349970480517</v>
+        <v>-0.05073583158470196</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.18747252812552</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003726949892365204</v>
+        <v>0.00372403787630715</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.172794308962837</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1927.513324756344</v>
+        <v>1929.021328153837</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2536.824254367113</v>
+        <v>2539.738524482838</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.806747078820497</v>
+        <v>1.808024874240311</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5259440508918425</v>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-90.90909090909091</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>667.9738562091503</v>
+        <v>657.6576576576579</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>110.4447156488688</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.739260728527449</v>
+        <v>2.744933573007707</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2211255748000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.76167845137359</v>
+        <v>27.81963602642865</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6725848897800161</v>
+        <v>0.6721141169297518</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.98676047609139</v>
+        <v>14.01596039357801</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.654351836248262</v>
+        <v>9.674507059288446</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5215156812853964</v>
+        <v>0.5226044405365141</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.39411248032314</v>
+        <v>18.43389172517954</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.50218106462077</v>
+        <v>13.53138098210739</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01800841531163939</v>
+        <v>0.01797089777974014</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.27609595935715</v>
+        <v>40.39123896624881</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.35571717523568</v>
+        <v>40.47391650242479</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.03937007874016</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-49.85639351985908</v>
+        <v>-50.18171780753171</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.943091687359823</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03723869229406085</v>
+        <v>0.03731208084175552</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,7 +5110,7 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3462505543057409</v>
+        <v>0.3341525451416469</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2196391625615738</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.7689508793208</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.83965330826726</v>
+        <v>17.83342938232836</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.750944640966779</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1642014853335771</v>
+        <v>0.1646077955091092</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.001081179960305101</v>
+        <v>-0.0008474184028264276</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.3063973063973</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.35212726495707</v>
+        <v>17.33641027536862</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.428223082633094</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4584031640606983</v>
+        <v>0.4597253355472533</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4581562636157563</v>
+        <v>0.4598152030388025</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16 08:21 ET</t>
+          <t>2026-08-17 08:25 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-18)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -464,7 +464,7 @@
     <col width="22" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="21" customWidth="1" min="29" max="29"/>
     <col width="21" customWidth="1" min="30" max="30"/>
     <col width="22" customWidth="1" min="31" max="31"/>
     <col width="23" customWidth="1" min="32" max="32"/>
@@ -720,7 +720,7 @@
         <v>34.88470319634703</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.35765288290291</v>
+        <v>32.35104444978663</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.614584371464129</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07809745418152247</v>
+        <v>0.07831767998999184</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.102030605486964</v>
+        <v>0.1022767603667742</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003468699892012174</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.358643242936049</v>
+        <v>0.3586790971624771</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3535466889728263</v>
+        <v>0.3541994996991685</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16145387799.88844</v>
+        <v>16370797471.99249</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.68611111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.88961379219265</v>
+        <v>23.87782444169262</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.74877558846308</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1170591263318113</v>
+        <v>0.1176106590563166</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2041981364626526</v>
+        <v>0.2048280224075079</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007411262621005516</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5691348388238667</v>
+        <v>0.566891268453768</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4885748932400781</v>
+        <v>0.4829771386370983</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15400241543.96546</v>
+        <v>15389302264.62616</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.08043694141013</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.28888269719243</v>
+        <v>20.30604719292914</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.33714825807696</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1581381194651141</v>
+        <v>-0.1588497367740883</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2675532079767995</v>
+        <v>0.268236835229813</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.00247093023255814</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8131084558775542</v>
+        <v>0.812536262534543</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.4178408185119522</v>
+        <v>0.4188406779370541</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10077465113.3422</v>
+        <v>10198025028.93117</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.73888888888889</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.97393549828555</v>
+        <v>23.98164807631733</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.623836892790842</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1349401565557732</v>
+        <v>-0.1352183626875408</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1590550257508712</v>
+        <v>0.1594632339150415</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8753316115120231</v>
+        <v>0.8737784119386238</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4826611104345527</v>
+        <v>0.4823985185824431</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11413528910.49439</v>
+        <v>11378501936.82861</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>34.30030487804878</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.25400823004437</v>
+        <v>20.23515070501244</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>21.49964775869755</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.69350700801871</v>
+        <v>0.6950852196792514</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9276329996846877</v>
+        <v>0.9294697964680922</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001244389138260522</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.288035152145797</v>
+        <v>1.28800087491103</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.3760372658184665</v>
+        <v>0.3813410411393719</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25574885812.78591</v>
+        <v>25675861654.87264</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.14344109996284</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.01439721661393</v>
+        <v>17.01120741232832</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.350300698069644</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2426794103124064</v>
+        <v>0.2429124275235057</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.251686552035157</v>
+        <v>0.2522938932256698</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003690880011248396</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8044218325303526</v>
+        <v>0.8019174703197121</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.5096547700246357</v>
+        <v>0.5029497839348533</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10675764045.17704</v>
+        <v>10705987112.49613</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>287.542372881356</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>166.4811364731551</v>
+        <v>166.3575337317136</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.93277710443066</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7271768980729043</v>
+        <v>0.728460181100534</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1088374459397952</v>
+        <v>0.109205940128926</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.562080812117329</v>
+        <v>1.562132021823696</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.6066206851424251</v>
+        <v>0.6072060681422552</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12823040986.3711</v>
+        <v>13302028168.15287</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>63.39741518578352</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>21.96282028121043</v>
+        <v>21.93605807672067</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>24.74017252236136</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.88657897182818</v>
+        <v>1.890100626286321</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.123868476519732</v>
+        <v>1.126382083411797</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006472491909385114</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.613513533883012</v>
+        <v>1.613252892265167</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.455207695458853</v>
+        <v>0.4687631189585583</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7672448591.156697</v>
+        <v>7718024777.318624</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.89050728277248</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.19051763759479</v>
+        <v>42.17956540688926</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.44031318314503</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1351012019842719</v>
+        <v>0.1353959392609208</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1114310412303821</v>
+        <v>0.1116672299216621</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005810173046670163</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1683376826378394</v>
+        <v>-0.1687586565188836</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2101668219868918</v>
+        <v>0.2103189011222713</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1882112426.378996</v>
+        <v>1920721253.678996</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>23.53560371517028</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.35625593758979</v>
+        <v>20.35300309359074</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.544091772542605</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1561852919971161</v>
+        <v>0.1563700750667969</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1296219216365251</v>
+        <v>0.1299484618571982</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1413974969890907</v>
+        <v>0.1385539394457838</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3985713496149972</v>
+        <v>0.4029103956078296</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3071444798.734314</v>
+        <v>3108234519.284617</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.52778476238371</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.41282490435593</v>
+        <v>23.41081044746742</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.793463690317063</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.464917846797166</v>
+        <v>-0.4648718039687104</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02671955910174395</v>
+        <v>0.026820718494178</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06762595448095293</v>
+        <v>0.06337194040170699</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1645850887197225</v>
+        <v>0.1619784056065648</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2115972532.682383</v>
+        <v>2125710517.187297</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.51848667239897</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.51999874904667</v>
+        <v>14.5194438760205</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.249625980990011</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06876639183029254</v>
+        <v>0.06880723565648617</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2928596968319769</v>
+        <v>-0.2928111913679294</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01662234042553191</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7934532933202095</v>
+        <v>0.7926174781125103</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1990457609183193</v>
+        <v>0.2148730588593354</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2741513857.983324</v>
+        <v>2801027724.833578</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.48768054375531</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.25687743663584</v>
+        <v>24.24880862508783</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.0595940746943</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2568674852480766</v>
+        <v>0.2572857089652121</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1281237965322342</v>
+        <v>0.1284299268768183</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.00746850964218036</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3255801038951567</v>
+        <v>0.320613700447486</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2047654329367929</v>
+        <v>0.210531830388713</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2585944693.351003</v>
+        <v>2592830652.819926</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>30.87644151565074</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>25.75254429677571</v>
+        <v>25.7424852603268</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.05587496394265</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1989666403376136</v>
+        <v>0.1994351440199198</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1451904684583993</v>
+        <v>0.1455571191944427</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.005993668409632555</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3154072545494951</v>
+        <v>0.311293425421233</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2265555937072982</v>
+        <v>0.2278688170133619</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1614365350.003491</v>
+        <v>1637644321.78772</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.44016461963861</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.4789262540334</v>
+        <v>18.47254367655471</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7981713888907401</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3767122759140717</v>
+        <v>0.377187953380085</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008199907805625184</v>
+        <v>0.008278438474486505</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02262271877053738</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4325468458589652</v>
+        <v>0.4273424181534725</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2534537841039565</v>
+        <v>0.2515375816636645</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2107591344.29703</v>
+        <v>2144761954.151306</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.86821705426356</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.03237794723321</v>
+        <v>15.03434762714768</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.854021988589154</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3882179604261793</v>
+        <v>0.3880360872181514</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01773610827812178</v>
+        <v>0.01761326873945745</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02550767706785537</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4835514350574072</v>
+        <v>-0.482021854902214</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2466057625451323</v>
+        <v>0.2464029004481813</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2173039942.801291</v>
+        <v>2167747519.227346</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.33179190751445</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.20226097790852</v>
+        <v>21.19669404699376</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.456565954987798</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4305923287671234</v>
+        <v>0.4309680481431624</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08189876681439734</v>
+        <v>0.08210466451906662</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.01997179555589435</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1906902521484739</v>
+        <v>-0.1888776125070776</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2648490759957333</v>
+        <v>0.2647682899247202</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1939834128.175995</v>
+        <v>1950438995.783234</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.11578947368421</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.84912784008742</v>
+        <v>36.83692463140565</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.254434046918193</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08864963229992795</v>
+        <v>0.08901027637587133</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06332213640108919</v>
+        <v>0.06345393480046257</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,13 +2930,13 @@
         <v>0.008440479314265722</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.09244880166315837</v>
+        <v>-0.09581012521430746</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.2331695921052838</v>
+        <v>0.2326489209441878</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2307342606.628863</v>
+        <v>2354938960.33816</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.20444444444444</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.29954269730844</v>
+        <v>20.29633205408335</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.909480595102951</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04457744495180083</v>
+        <v>0.04474268493150668</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02307740879988085</v>
+        <v>0.02315743414105587</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.02997694403688955</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05987407033040303</v>
+        <v>-0.06325592238672778</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.2076630623474862</v>
+        <v>0.2096994686128575</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1228374064.995831</v>
+        <v>1238108541.86498</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3113,67 +3113,67 @@
         <v>336905891960</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>23.92917847025496</v>
+        <v>23.59497206703911</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>22.60906222711441</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2.022341360689589</v>
+        <v>1.991452049699721</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>24.20734611503532</v>
+        <v>20.21139315159174</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-5.437445630856404</v>
+        <v>-8.093624139275077</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.24787820532948</v>
+        <v>16.42027564122935</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.36073696191894</v>
+        <v>2.321197403650636</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04248961013035529</v>
+        <v>0.04482260583852569</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.05838881019830033</v>
+        <v>0.04360684357541889</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.02625862135636758</v>
+        <v>0.01058351213529107</v>
       </c>
       <c r="W21" s="4" t="n">
-        <v>0.1298561684460261</v>
+        <v>0.1300647261025379</v>
       </c>
       <c r="X21" s="4" t="n">
-        <v>1.133015282606938</v>
+        <v>1.02684951281126</v>
       </c>
       <c r="Y21" s="4" t="n">
-        <v>0.3312704091432962</v>
+        <v>0.3320624674894784</v>
       </c>
       <c r="Z21" s="4" t="n">
-        <v>0.1244837687283903</v>
+        <v>0.1242611245093867</v>
       </c>
       <c r="AA21" s="5" t="n">
         <v>12646000000</v>
       </c>
       <c r="AB21" s="6" t="n">
-        <v>1.044744238336144</v>
+        <v>1.078083914484966</v>
       </c>
       <c r="AC21" s="6" t="n">
-        <v>0.2780213603147836</v>
+        <v>0.3107636904081399</v>
       </c>
       <c r="AD21" s="6" t="n">
-        <v>4.178679544471674</v>
+        <v>3.482578082686405</v>
       </c>
       <c r="AE21" s="6" t="n">
-        <v>0.537283140569395</v>
+        <v>0.5290536093030059</v>
       </c>
       <c r="AF21" s="6" t="n">
-        <v>2.329022929146871</v>
+        <v>2.332636420656492</v>
       </c>
       <c r="AG21" s="6" t="n">
         <v>8.712271973466004</v>
@@ -3182,13 +3182,13 @@
         <v>0.02740617970877235</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.710221362814863</v>
+        <v>0.7113728343167208</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2978910214423897</v>
+        <v>0.302494737801638</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1242831414.330986</v>
+        <v>1246769734.923808</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>128.4263959390863</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>40.83439240606327</v>
+        <v>40.76678146326567</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.97539280958722</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.14505465544816</v>
+        <v>2.150270669633545</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7771897914203891</v>
+        <v>0.7795163897281334</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.549836524193336</v>
+        <v>2.549679313510372</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7559388660361674</v>
+        <v>0.7775434718225019</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13782983860.99084</v>
+        <v>14012309903.98234</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>725788327212</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>58.8243831640058</v>
+        <v>56.93759071117562</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>40.04763883952414</v>
+        <v>40.01463487730252</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>17.68706098673838</v>
+        <v>17.11974839648999</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>28.62767601051985</v>
+        <v>27.70944312589918</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>4.004390729266458</v>
+        <v>3.875949871925071</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>44.92391227563476</v>
+        <v>43.47208602100764</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>17.55437398652608</v>
+        <v>16.98706139627769</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01600714687020482</v>
+        <v>0.01653759017714525</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4688602092054019</v>
+        <v>0.4229191615958565</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2339557353733854</v>
+        <v>0.1951383484088118</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004131441437614173</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.700251770540371</v>
+        <v>1.701859350747158</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.5468501564222554</v>
+        <v>0.5574069555414716</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>3008667726.382939</v>
+        <v>3050775215.161133</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>84.62546816479397</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>105.6078269272091</v>
+        <v>104.9369650397583</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.899931927230172</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1986818531629986</v>
+        <v>-0.1935590272433433</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1410666612202194</v>
+        <v>0.1414905159452522</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.201136872662814</v>
+        <v>1.194686973677663</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3586477375822985</v>
+        <v>0.3535881126457306</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1213077341.113911</v>
+        <v>1230458737.716726</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>16.01630103595368</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.63393365494323</v>
+        <v>14.63209225865204</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.629741380313218</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09446314392326771</v>
+        <v>0.09460087818152996</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3860095595149767</v>
+        <v>-0.3859642726380151</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01617030181392739</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.573331506361317</v>
+        <v>1.580334748130775</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3844251539557897</v>
+        <v>0.3848500054748674</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2012402724.511947</v>
+        <v>2034892303.452555</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>19.98689956331878</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.81066027536316</v>
+        <v>17.80746655905614</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.120357843321707</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1221874570796195</v>
+        <v>0.1223887180714245</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04416811442377711</v>
+        <v>0.04427784704131432</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02945160585536378</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8728794078896674</v>
+        <v>0.8664545533513828</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.8153522600966761</v>
+        <v>0.8143375055874656</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2614372880.770444</v>
+        <v>2629549120.788116</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.70385259631492</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.93170499854214</v>
+        <v>27.91361505459289</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.00994860479654</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4214618333677522</v>
+        <v>0.422383038480072</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1968036022883886</v>
+        <v>0.1972742639461968</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005644807452158358</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3530552551820408</v>
+        <v>0.3529040073765982</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3441683304404431</v>
+        <v>0.3446181444999699</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3031230280.78018</v>
+        <v>3075672639.258626</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.54099678456592</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.3169472735917</v>
+        <v>16.3144066069141</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.72015323601704</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07501706602651614</v>
+        <v>0.07518448002466638</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3308233269631512</v>
+        <v>-0.3307262936952998</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01901837679299757</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.362684301016988</v>
+        <v>1.36637449424097</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3029403337467731</v>
+        <v>0.3045258496970822</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1170283211.678737</v>
+        <v>1186419890.783742</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>22.57866547645615</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.646994332358252</v>
+        <v>6.637264098867182</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.65769028180872</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.396823338112518</v>
+        <v>2.401803083338174</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.723630098031868</v>
+        <v>1.727273910968313</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005238448233259204</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.887308826486797</v>
+        <v>2.889941370587172</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>1.044435021815946</v>
+        <v>1.050687251493404</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>38049455698.71275</v>
+        <v>38156112884.19027</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>73.10559006211182</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>25.22660343146399</v>
+        <v>25.21259602176744</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.259948235134402</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.897956130349698</v>
+        <v>1.899566153322557</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2295515278251798</v>
+        <v>0.2301160144564625</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6650135292540603</v>
+        <v>0.6485303200215876</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6091993735458735</v>
+        <v>0.5982244735138025</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2466909737.475126</v>
+        <v>2456763987.39741</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>35.50475687103594</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.249603902998892</v>
+        <v>9.25050276214407</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.404294662145189</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.838516464421212</v>
+        <v>2.838143480842192</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05073583158470196</v>
+        <v>-0.05084816346459897</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.06401190919240789</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3191277360920765</v>
+        <v>0.3208469192009179</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2282530427257863</v>
+        <v>0.2281935388440251</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>992327321.2885374</v>
+        <v>1017193713.446973</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1216549312196</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.18747252812552</v>
+        <v>7.26175035972317</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003837104618779049</v>
+        <v>0.003834108875091841</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.172794308962837</v>
+        <v>6.236586104253031</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.467862657170157</v>
+        <v>4.514035098004133</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01608466603334042</v>
+        <v>0.01625089054553907</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.860094907731933</v>
+        <v>6.951251471526091</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.806077734086766</v>
+        <v>5.883228575653781</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07808768428991608</v>
+        <v>0.07728895346384594</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1872.150002986508</v>
+        <v>1892.986476727066</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2464.871389759911</v>
+        <v>2493.212185008512</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4540,7 +4540,7 @@
         <v>1.001212727821457</v>
       </c>
       <c r="Y32" s="4" t="n">
-        <v>0.7626812917006164</v>
+        <v>0.7617145295002609</v>
       </c>
       <c r="Z32" s="4" t="n">
         <v>0.6803691736161032</v>
@@ -4555,13 +4555,13 @@
         <v>15.52297494663521</v>
       </c>
       <c r="AD32" s="6" t="n">
-        <v>0.07075179011241259</v>
+        <v>0.08037191322189781</v>
       </c>
       <c r="AE32" s="6" t="n">
-        <v>0.05327608051321153</v>
+        <v>0.06052003084314141</v>
       </c>
       <c r="AF32" s="6" t="n">
-        <v>-0.4332891537291704</v>
+        <v>-0.4175049480169813</v>
       </c>
       <c r="AG32" s="6" t="n">
         <v>55.63395918385022</v>
@@ -4571,10 +4571,10 @@
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.404567699335458</v>
+        <v>1.430291791726731</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6678823550.595737</v>
+        <v>6779020083.450024</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.807238689513244</v>
+        <v>1.808024874240311</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.513373786626932</v>
+        <v>0.5259440508918425</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6168647569.891911</v>
+        <v>6216375697.052714</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-94.95454545454545</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>686.9234234234235</v>
+        <v>676.4759188846639</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>115.3595054952639</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.744933573007707</v>
+        <v>2.750606417487965</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.9676068730234598</v>
+        <v>0.9917175357859459</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12538372889.40363</v>
+        <v>12990280657.57413</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>772.66</v>
+        <v>772.67</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1309923142533804</v>
+        <v>0.1310069518988421</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.00860951794398046</v>
+        <v>-0.008596687067759956</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>823066967701</v>
+        <v>823077620083</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9962736258373266</v>
+        <v>0.9964541428148497</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1282816494286649</v>
+        <v>0.128640414015669</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34525789016.79326</v>
+        <v>34938403895.45919</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2235217285600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.81963602642865</v>
+        <v>27.58780572620842</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6793972580584382</v>
+        <v>0.6789220495409314</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.01596039357801</v>
+        <v>13.89916072363153</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.674507059288446</v>
+        <v>9.59388616712771</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5226044405365141</v>
+        <v>0.5182494035320432</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.43389172517954</v>
+        <v>18.27477474575392</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.53138098210739</v>
+        <v>13.41458131216091</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01797089777974014</v>
+        <v>0.01812191372746905</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>39.94752473086336</v>
+        <v>39.63471755684255</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>40.02931596354458</v>
+        <v>39.71866248458279</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.2552381836322714</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.199316053549032</v>
+        <v>2.207244908647239</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.4965398911177071</v>
+        <v>0.5035963642370442</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5522137048.822072</v>
+        <v>5610853317.348633</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-21.99212598425197</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-50.07414713699038</v>
+        <v>-50.40303840666584</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.938926431870414</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03731208084175552</v>
+        <v>0.03738546938945042</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3333667339870736</v>
+        <v>0.3341525451416469</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2184671560926791</v>
+        <v>0.2196391625615738</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>599722993.5359167</v>
+        <v>603079533.1113943</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.38872043662826</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.50694140572476</v>
+        <v>17.50083568700352</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.700581341215373</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1646077955091092</v>
+        <v>0.165014105684641</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.0008474184028264276</v>
+        <v>-0.0006136568453474212</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01052913357722852</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9728639825385216</v>
+        <v>0.9680213288500964</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2528006917971722</v>
+        <v>0.2516285048311834</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>960686252.7042582</v>
+        <v>983257475.4817709</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.6986531986532</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.92006886308761</v>
+        <v>16.9047570867808</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.273846517117492</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4597253355472533</v>
+        <v>0.4610475070338085</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4598152030388027</v>
+        <v>0.4614741424618487</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.01363233590075659</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.036418375103719</v>
+        <v>2.031736199265938</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.590666987439879</v>
+        <v>0.5900110526330925</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4757612074.260573</v>
+        <v>4833171289.330852</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17 17:53 ET</t>
+          <t>2026-08-18 08:27 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-19)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.39155251141553</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.82108154968209</v>
+        <v>32.74727214633685</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.754277275712635</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07831767998999184</v>
+        <v>0.0807481109651591</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1022767603667742</v>
+        <v>0.1048535834353748</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003419023965422702</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3488249768106958</v>
+        <v>0.3537361217363841</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3539369074027918</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16242688521.78174</v>
+        <v>16312642243.89964</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.75722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.9414522449306</v>
+        <v>23.92964314023871</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.77741810486411</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1176106590563166</v>
+        <v>0.1181621917808218</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2048280224075076</v>
+        <v>0.2054579083523629</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007391566139982974</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5629878212885915</v>
+        <v>0.5689889537086364</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4763742845412415</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15423612508.94156</v>
+        <v>15429149182.98869</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.09036742800397</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.31785303432037</v>
+        <v>20.33505659340307</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.342576832645159</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1588497367740883</v>
+        <v>-0.1595613540830625</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2682368352298128</v>
+        <v>0.2689204624828256</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002469494479953515</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.808328289387685</v>
+        <v>0.7954108970003755</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4136043675218524</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10004753204.17674</v>
+        <v>10005092814.85545</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.59126984126984</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.81094712563825</v>
+        <v>23.81860973431582</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.598042485303218</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1352183626875408</v>
+        <v>-0.1354965688193087</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1594632339150412</v>
+        <v>0.1598714420792113</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8724784012183031</v>
+        <v>0.8554101556434207</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4744105561616347</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11374515531.55847</v>
+        <v>11388472385.51514</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>33.4969512195122</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.7612195721054</v>
+        <v>19.7428379729154</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.99610061106706</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6950852196792516</v>
+        <v>0.6966634313397928</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9294697964680922</v>
+        <v>0.9313065932514963</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001274233184672795</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.288470457413049</v>
+        <v>1.295541754286085</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3794513653003851</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25602870448.21643</v>
+        <v>25605754418.59386</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.2032701597919</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.25478168244465</v>
+        <v>16.25173485963666</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.067926218464127</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2429124275235057</v>
+        <v>0.2431454447346051</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2522938932256698</v>
+        <v>0.2529012344161818</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003862637261574117</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8195267685601331</v>
+        <v>0.8194826576872534</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5033950026993275</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10779328706.64039</v>
+        <v>10787549467.96265</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>285.4830508474577</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>165.1661137288605</v>
+        <v>165.0435782923155</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>12.84015509334196</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.728460181100534</v>
+        <v>0.7297434641281635</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.109205940128926</v>
+        <v>0.1095744343180569</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.55175464735351</v>
+        <v>1.512148986964324</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6052668151168374</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12622842815.05256</v>
+        <v>12632007329.58272</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>61.38933764135703</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>21.24124574867838</v>
+        <v>21.21539430003386</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.95654144305307</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.890100626286321</v>
+        <v>1.893622280744462</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.126382083411797</v>
+        <v>1.128895690303861</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.00668421052631579</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.614370563313218</v>
+        <v>1.627567434167704</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4503109121932953</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7665148995.466878</v>
+        <v>7665485308.133545</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.28478151682572</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.52682244773256</v>
+        <v>42.51578578071421</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.452171031585186</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1353959392609208</v>
+        <v>0.1356906765375698</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1116672299216621</v>
+        <v>0.111903418612942</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005762729494981017</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1714751632862794</v>
+        <v>-0.1694593505587476</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2046517411605224</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1884301752.006913</v>
+        <v>1884327035.511271</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.07739938080496</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.82153447235665</v>
+        <v>20.81820781039315</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.694738452384172</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1563700750667969</v>
+        <v>0.1565548581364775</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1299484618571982</v>
+        <v>0.1302750020778711</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1302115160076528</v>
+        <v>0.1299738644347</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3988264705822719</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3076439917.559065</v>
+        <v>3081097466.741689</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.64671863213477</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.63306349007127</v>
+        <v>23.63103025863161</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.819983737794622</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4648718039687103</v>
+        <v>-0.4648257611402551</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.026820718494178</v>
+        <v>0.02692187788661182</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06215898489957017</v>
+        <v>0.06795041236467576</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1649913072007667</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2128935722.870228</v>
+        <v>2129016313.826192</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.61693895098882</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.61155803403271</v>
+        <v>14.61099968346053</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.270242236243965</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06880723565648617</v>
+        <v>0.06884807948267957</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2928111913679294</v>
+        <v>-0.2927626859038821</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01651754989676531</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7858123495244972</v>
+        <v>0.7798286744831684</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.1989521993103648</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2735856094.403129</v>
+        <v>2753334449.353129</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>30.94732370433305</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.61439232440152</v>
+        <v>24.60620731170861</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.28663789352185</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2572857089652121</v>
+        <v>0.2577039326823476</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1284299268768183</v>
+        <v>0.1287360572214025</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007357584076870282</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3171122982211614</v>
+        <v>0.3225882249535397</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.205673125647146</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2617430407.82227</v>
+        <v>2637046897.305603</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.53816584294343</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.29418189068809</v>
+        <v>26.28391529881415</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.35711156856597</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1994351440199198</v>
+        <v>0.1999036477022258</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1455571191944427</v>
+        <v>0.1459237699304856</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.005867911058487577</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3038234020135107</v>
+        <v>0.3113663361261061</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.225555477055968</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1643132553.599955</v>
+        <v>1643134659.40328</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.3314899363385</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.3936331088044</v>
+        <v>18.38728218497069</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7947617795520839</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.377187953380085</v>
+        <v>0.3776636308460983</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008278438474486505</v>
+        <v>0.008356969143347825</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02271977254842231</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4602320783450616</v>
+        <v>0.4195303892535209</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2489286281489237</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2080667550.204449</v>
+        <v>2090237304.647522</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.39793281653747</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.41597730317111</v>
+        <v>15.41799751049456</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.901084210934471</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3880360872181514</v>
+        <v>0.3878542140101231</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01761326873945723</v>
+        <v>0.01749042920079291</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02487622267842048</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4954047615479182</v>
+        <v>-0.4898220761019505</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2507661945179219</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2208892006.085795</v>
+        <v>2208945128.770345</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.34219653179191</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.90279270907679</v>
+        <v>21.89704335396245</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.671645371258769</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4309680481431624</v>
+        <v>0.431343767519202</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08210466451906662</v>
+        <v>0.08231056222373589</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.01932794806536092</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.2027708397341194</v>
+        <v>-0.202217850837891</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2743265640505719</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1909371897.325153</v>
+        <v>1929700636.763763</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>40.42105263157895</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>37.117237099081</v>
+        <v>37.10494917086129</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.263979727149268</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08901027637587133</v>
+        <v>0.08937092045181427</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06345393480046235</v>
+        <v>0.06358573319983574</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07850638969361928</v>
@@ -2930,13 +2930,13 @@
         <v>0.008376736111111111</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.09743450203231394</v>
+        <v>-0.09859235481036054</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2269103883965658</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2315480830.601602</v>
+        <v>2320334778.633016</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.25333333333333</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.34312720239501</v>
+        <v>20.33991017451539</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.918494279138708</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0447426849315069</v>
+        <v>0.04490792491121254</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02315743414105587</v>
+        <v>0.0232374594822311</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.02990798828941866</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05993900485756402</v>
+        <v>-0.06231077276105747</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2059257553365873</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1241535720.770363</v>
+        <v>1263657316.939748</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3182,23 +3182,23 @@
         <v>0.02743785001037068</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7081664261683188</v>
+        <v>0.7173585711763895</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.288918262326767</v>
+        <v>0.2979462289187499</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1281333127.052291</v>
+        <v>1297308041.624858</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18 (C)</t>
+          <t>2026-11-17 (E)</t>
         </is>
       </c>
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.9416243654822</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>39.02573374108944</v>
+        <v>38.96122426880031</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>19.12229352378647</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.150270669633545</v>
+        <v>2.155486683818927</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7795163897281334</v>
+        <v>0.7818429880358773</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.549582155956617</v>
+        <v>2.545359930796348</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.76292295710798</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13663897711.65586</v>
+        <v>13665946229.32047</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>694900929413</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>55.94339622641509</v>
+        <v>56.11756095791001</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>38.31173073998412</v>
+        <v>38.28018336884436</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.82081830087043</v>
+        <v>16.87318535053429</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>27.2256050290029</v>
+        <v>27.31036463441677</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.80827142017211</v>
+        <v>3.820127449910985</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>42.70708526379079</v>
+        <v>42.84109931333985</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.68813130065813</v>
+        <v>16.74049835032199</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01683148690229538</v>
+        <v>0.01677924926653082</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4602158437084034</v>
+        <v>0.465968969301835</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2264645799095073</v>
+        <v>0.2310669953706495</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004315078370253691</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.706112444261097</v>
+        <v>1.716398540887444</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5507270273890214</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2992540901.363737</v>
+        <v>2995182507.432455</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>83.54307116104866</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>103.5947750465523</v>
+        <v>102.9408548007073</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.875630961221342</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1935590272433433</v>
+        <v>-0.1884362013236882</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1414905159452522</v>
+        <v>0.1419143706702848</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.205768381374729</v>
+        <v>1.260020249999911</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3594718417852168</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1206288012.55073</v>
+        <v>1215024536.557109</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.8511578305911</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.48122155440326</v>
+        <v>14.4793996032207</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.602626260545885</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09460087818152996</v>
+        <v>0.09473861243979198</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3859642726380151</v>
+        <v>-0.3859189857610535</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01633876997895182</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.569318420824454</v>
+        <v>1.555577833758965</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3844899016450891</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2025036512.158203</v>
+        <v>2043141730.118408</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.32052401746725</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.10471157655928</v>
+        <v>18.10146571451152</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.17244334457357</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1223887180714245</v>
+        <v>0.122589979063229</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04427784704131432</v>
+        <v>0.04438757965885154</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.0289680663600808</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8652758038288617</v>
+        <v>0.8719524027390428</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8138370418137757</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2552371233.11635</v>
+        <v>2563653300.503896</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>41.09447236180905</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.89128402833159</v>
+        <v>28.87258472446301</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.50064434763726</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.422383038480072</v>
+        <v>0.4233042435923913</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1972742639461968</v>
+        <v>0.1977449256040054</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005453789527745848</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3414274341654803</v>
+        <v>0.3263399204216609</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3529961835785302</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3006175173.241292</v>
+        <v>3034561813.001302</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.4935691318328</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.27029543007491</v>
+        <v>16.26776242183438</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.712798438302682</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07518448002466638</v>
+        <v>0.07535189402281639</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3307262936952998</v>
+        <v>-0.3306292604274488</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01906993842477714</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.355002650746833</v>
+        <v>1.341612704405342</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2992918815090388</v>
+        <v>0.3079790494861182</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1153197942.67497</v>
+        <v>1146970647.321421</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>20.9944208881946</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.17155678146804</v>
+        <v>6.162535724956983</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.76955642156102</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.401803083338174</v>
+        <v>2.406782828563829</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.727273910968312</v>
+        <v>1.730917723904757</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005633742931247077</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.896190230998804</v>
+        <v>2.898759875507753</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.05778912477339</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>37576221088.7263</v>
+        <v>37585831077.66073</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>74.21739130434783</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>25.59603312354283</v>
+        <v>25.58182847038194</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.385566819169156</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.899566153322557</v>
+        <v>1.901176176295414</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2301160144564625</v>
+        <v>0.2306805010877451</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6601932980125627</v>
+        <v>0.6522145379937044</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.588819221877288</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2451866024.339063</v>
+        <v>2463009426.542841</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.0068710359408</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.381324907645176</v>
+        <v>9.382236655792312</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.43829659633258</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.838143480842191</v>
+        <v>2.83777049726317</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05084816346459897</v>
+        <v>-0.0509604953444962</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.06311926605504586</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3120589672541382</v>
+        <v>0.3123399211941842</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2301262221072392</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>988855694.5298622</v>
+        <v>993169379.5215288</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1104676181374</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.26175035972317</v>
+        <v>6.553926317439683</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003481526567521253</v>
+        <v>0.003478810554851782</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.236586104253031</v>
+        <v>5.628687819722952</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.514035098004133</v>
+        <v>4.074038897115644</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01625089054553907</v>
+        <v>0.01466686872341071</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.951251471526091</v>
+        <v>6.614757970857151</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.883228575653781</v>
+        <v>5.59843551547369</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07728895346384594</v>
+        <v>0.0856361604379413</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2084.794900279428</v>
+        <v>1882.956086168342</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2745.806864586213</v>
+        <v>2480.907841956402</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4561,7 +4561,7 @@
         <v>0.06052003084314141</v>
       </c>
       <c r="AF32" s="6" t="n">
-        <v>-0.4175049480169813</v>
+        <v>-0.03574421284598284</v>
       </c>
       <c r="AG32" s="6" t="n">
         <v>55.63395918385022</v>
@@ -4574,7 +4574,7 @@
         <v>1.408959728584181</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6564698269.565048</v>
+        <v>6568120603.361238</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.810671488784057</v>
+        <v>1.812588331805092</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5217678249949264</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6099224513.595179</v>
+        <v>6103290848.270569</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-93.07792207792208</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>663.1064638783268</v>
+        <v>653.1722846441949</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>113.0796110079035</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.750606417487965</v>
+        <v>2.756279261968222</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.9424218149439709</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12531977943.04971</v>
+        <v>12532603650.80172</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9963486973618474</v>
+        <v>0.98941789718341</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.1253531096535055</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34570840785.10037</v>
+        <v>34586091679.65128</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2144142696800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.58780572620842</v>
+        <v>27.24006027587806</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6512591700134962</v>
+        <v>0.6508039612502213</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.89916072363153</v>
+        <v>13.7239612187118</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.59388616712771</v>
+        <v>9.472954828886603</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5182494035320432</v>
+        <v>0.5117168480253368</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.27477474575392</v>
+        <v>18.0360992766155</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.41458131216091</v>
+        <v>13.23938180724118</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01812191372746905</v>
+        <v>0.01835325730696866</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.36071750918564</v>
+        <v>40.8560148643668</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.44822808103492</v>
+        <v>40.94534082516599</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.2660796787692605</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.210886655085341</v>
+        <v>2.174311244519919</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.5055563014328557</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5532268221.498685</v>
+        <v>5532665191.564534</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.4251968503937</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-51.39557944224286</v>
+        <v>-51.73538184317033</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.977107940551018</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.03738546938945042</v>
+        <v>0.0374588579371451</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3238582353809497</v>
+        <v>0.3239118571123482</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2197506188270884</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>617215089.6853863</v>
+        <v>618195886.7576218</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.52880533656762</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.62107878041829</v>
+        <v>17.61493539772575</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.719136241123785</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.165014105684641</v>
+        <v>0.1654204158601726</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.0006136568453474212</v>
+        <v>-0.0003798952878687478</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01045728465083304</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9655220914255007</v>
+        <v>0.9703864806273597</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2534073224668002</v>
+        <v>0.2538702029992585</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>957839832.2314585</v>
+        <v>973532136.817627</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.01851851851852</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.43924540638686</v>
+        <v>16.42438220055317</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.101081607232993</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4610475070338085</v>
+        <v>0.4623696785203633</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4614741424618485</v>
+        <v>0.4631330818848947</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.01401836405691456</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.045759897911939</v>
+        <v>2.021778644323258</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5908476317642759</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4617061122.434979</v>
+        <v>4626345094.574788</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18 17:50 ET</t>
+          <t>2026-08-19 08:27 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-20)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -470,7 +470,7 @@
     <col width="23" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -720,7 +720,7 @@
         <v>36.16780821917808</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.46552989750639</v>
+        <v>33.45870121571161</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.968221363300437</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.0807481109651591</v>
+        <v>0.08096868393069379</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.104853583435375</v>
+        <v>0.1051046048970836</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003345642773727236</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3469499428829872</v>
+        <v>0.3469498640635618</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3572620713342697</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16409663392.98399</v>
+        <v>16414087173.91551</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.90611111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.06279814224407</v>
+        <v>24.05093503524188</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.83738837357875</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1181621917808218</v>
+        <v>0.1187137245053274</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2054579083523629</v>
+        <v>0.2060877942972179</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007350663831017324</v>
+        <v>0.007515847287894117</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5622577579865001</v>
+        <v>0.5622577262636583</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4762456759113857</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15419044140.81387</v>
+        <v>15419567340.90424</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>196.6</v>
+        <v>199.43</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>4171839802510</v>
@@ -974,7 +974,7 @@
         <v>17.11618669314796</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.36577777128968</v>
+        <v>20.207614144365</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.356691126524277</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1595613540830626</v>
+        <v>-0.1529832977377537</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2689204624828259</v>
+        <v>0.2732064614883774</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002465769320027848</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8081036905136584</v>
+        <v>0.808103675689741</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.4124065319915229</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9964274599.161686</v>
+        <v>9965059262.319132</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.09841269841269</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>24.4052388196975</v>
+        <v>24.41309520584558</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.686658756188119</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1354965688193087</v>
+        <v>-0.1357747749510765</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1598714420792116</v>
+        <v>0.1602796502433819</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8703350717029998</v>
+        <v>0.8703349700664186</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4730591404137224</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11435924526.4075</v>
+        <v>11463880313.59039</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>33.16463414634146</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.54697291975732</v>
+        <v>19.52880750689196</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.78780217049126</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6966634313397926</v>
+        <v>0.698241643000334</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9313065932514963</v>
+        <v>0.9331433900349009</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001287001287001287</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.289235055848763</v>
+        <v>1.289235065607851</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3741448183896907</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25307726465.2261</v>
+        <v>25304357410.87591</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.29096989966555</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.32228150423493</v>
+        <v>16.47374355891992</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.094266288497599</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2431454447346049</v>
+        <v>0.2317157801499672</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2529012344161818</v>
+        <v>0.2557151368250732</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003845942530630185</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8183930780179269</v>
+        <v>0.8183930415195237</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5015954488438872</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10813213254.02693</v>
+        <v>10822990176.5155</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>297.5593220338984</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>172.0251171371681</v>
+        <v>172.2792091406913</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.38330886209093</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7297434641281637</v>
+        <v>0.7271922916182965</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1095744343180567</v>
+        <v>0.1107019069069288</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.548256940733343</v>
+        <v>1.548256762501951</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6144786764165941</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12601588295.696</v>
+        <v>12616690692.33398</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
         <v>495</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>281.87</v>
+        <v>286.17</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>1724527598400</v>
@@ -1604,7 +1604,7 @@
         <v>58.55896607431341</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.2372529628323</v>
+        <v>20.21265335241905</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>22.8520187954681</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.893622280744462</v>
+        <v>1.897143935202602</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.128895690303861</v>
+        <v>1.131409297195924</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.007007283160450232</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.617805107798043</v>
+        <v>1.61780523645709</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4487239278959511</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7676616489.586105</v>
+        <v>7679287423.547058</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.06579608237067</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.32296440868122</v>
+        <v>42.29241342792474</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.44558501640059</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1356906765375698</v>
+        <v>0.1365110710526134</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.111903418612942</v>
+        <v>0.1103936033299036</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005788984210911295</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1708904863167022</v>
+        <v>-0.1708904669239098</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2016671114969098</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1880508366.498258</v>
+        <v>1884420828.675334</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.8359133126935</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.47404694033353</v>
+        <v>21.47161840819544</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.905643804178905</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1565548581364773</v>
+        <v>0.1566856694516308</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1302750020778713</v>
+        <v>0.1348951687653812</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1276115601254718</v>
+        <v>0.1276114429109569</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.4057333899097348</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3077822648.145301</v>
+        <v>3078627674.575552</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.56726175509178</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>23.48256108490552</v>
+        <v>22.67890587893788</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.802266327640393</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4648257611402552</v>
+        <v>-0.4458611970887398</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.02692187788661182</v>
+        <v>0.05947089950481366</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06170933171846876</v>
+        <v>0.06519695450224021</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.165618060053194</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2115017368.306926</v>
+        <v>2115227541.784871</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.35941530524506</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.37006399700787</v>
+        <v>14.28207262039292</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.216315874247815</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.06884807948267957</v>
+        <v>0.0754332171168095</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2927626859038821</v>
+        <v>-0.2911021491870769</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01679449140681856</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7844334026612091</v>
+        <v>0.7799132426022436</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.1929062674211035</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2608415595.359607</v>
+        <v>2629132531.7099</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.05692438402719</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.69335077754829</v>
+        <v>24.66551836454355</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.34077588358659</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2577039326823476</v>
+        <v>0.2591231177476983</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1287360572214025</v>
+        <v>0.1297380983430965</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007331618974667615</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3170847998795436</v>
+        <v>0.3203812395061349</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.2035163329267589</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2563181106.64325</v>
+        <v>2590174871.591593</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.50576606260297</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.25691331377767</v>
+        <v>26.14204491313168</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.34236222443919</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.1999036477022258</v>
+        <v>0.2051760360482349</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1459237699304856</v>
+        <v>0.1473724901802731</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.005873945478630691</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3039243085842712</v>
+        <v>0.3103942386430582</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2244362706176763</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1642945969.213981</v>
+        <v>1654314670.285441</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.98938974985532</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.13896308963892</v>
+        <v>18.132702259586</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7840285714495178</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3776636308460983</v>
+        <v>0.3781393083121116</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008356969143347825</v>
+        <v>0.008435499812209146</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02303080208949847</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4596556014390018</v>
+        <v>0.4126878910371898</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2508171639218384</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2103520570.905347</v>
+        <v>2103707608.891296</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.2906976744186</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.34073064698948</v>
+        <v>15.00174185850283</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.891556980557248</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.3878542140101233</v>
+        <v>0.419215040175569</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.01749042920079313</v>
+        <v>0.07925402163176298</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02500151708234723</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4959087059729074</v>
+        <v>-0.4923357567155885</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.243910744406078</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2197772148.434934</v>
+        <v>2197803097.73407</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.60809248554914</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.08281001588607</v>
+        <v>22.16776734902661</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.728245217647479</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.431343767519202</v>
+        <v>0.4258581835458071</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08231056222373589</v>
+        <v>0.08243262050364408</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.01916535605866647</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.2024007242691897</v>
+        <v>-0.2028840222218334</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2649759781917974</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1927381606.34005</v>
+        <v>1940697338.816071</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2861,67 +2861,67 @@
         <v>909608544000</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>40.10526315789473</v>
+        <v>41.26353790613719</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>36.81506675546393</v>
+        <v>36.83164820784825</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.254104885530915</v>
+        <v>1.236149902152642</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>9.656065938725751</v>
+        <v>9.254486044096987</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>1.840123839009287</v>
+        <v>9.978273711847727</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.21351802073163</v>
+        <v>22.11378578742576</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.341585324794397</v>
+        <v>1.320714481409002</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01379934267635903</v>
+        <v>0.03044166656376526</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.08937092045181427</v>
+        <v>0.1203283022600268</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.06358573319983596</v>
+        <v>0.04792906633305849</v>
       </c>
       <c r="W19" s="4" t="n">
-        <v>0.07850638969361928</v>
+        <v>0.07511040644542281</v>
       </c>
       <c r="X19" s="4" t="n">
-        <v>0.2392312528442645</v>
+        <v>0.2274240945299643</v>
       </c>
       <c r="Y19" s="4" t="n">
-        <v>0.2497638924314599</v>
+        <v>0.2523062078712764</v>
       </c>
       <c r="Z19" s="4" t="n">
-        <v>0.04161421746713451</v>
+        <v>0.04386823222439661</v>
       </c>
       <c r="AA19" s="5" t="n">
         <v>14923000000</v>
       </c>
       <c r="AB19" s="6" t="n">
-        <v>0.7714407896459335</v>
+        <v>0.7671279079823575</v>
       </c>
       <c r="AC19" s="6" t="n">
-        <v>0.2253737465418081</v>
+        <v>0.2343941883594223</v>
       </c>
       <c r="AD19" s="6" t="n">
-        <v>0.7863776105162726</v>
+        <v>0.7507787210651683</v>
       </c>
       <c r="AE19" s="6" t="n">
-        <v>0.2561367646500257</v>
+        <v>0.2509407513762529</v>
       </c>
       <c r="AF19" s="6" t="n">
-        <v>1.318058123351129</v>
+        <v>1.415932828179398</v>
       </c>
       <c r="AG19" s="6" t="n">
         <v>11.52840300107181</v>
@@ -2930,13 +2930,13 @@
         <v>0.008442694663167103</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.0978111152988374</v>
+        <v>-0.0953722323130108</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.2268642395322842</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2375513015.647097</v>
+        <v>2375733184.122976</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.39259259259259</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.47318436637406</v>
+        <v>20.52125817949645</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.944169621552992</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04490792491121254</v>
+        <v>0.04246008726534756</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.0232374594822311</v>
+        <v>0.02329388733336324</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.02971329639889197</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05891475892258414</v>
+        <v>-0.06211434366480952</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2067683356121111</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1250176272.93433</v>
+        <v>1260179251.746623</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>24.04329608938547</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>23.0386531454821</v>
+        <v>22.96904415953846</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>2.029291288953516</v>
@@ -3140,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04360684357541889</v>
+        <v>0.04676955307262554</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01058351213529107</v>
+        <v>0.01351098766373471</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3182,13 +3182,13 @@
         <v>0.02689514957885565</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7092684365564549</v>
+        <v>0.7149167198287663</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2886791886851872</v>
+        <v>0.2927736543609129</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1289080966.659153</v>
+        <v>1313038155.55837</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>118.3807106598985</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>37.51583274521325</v>
+        <v>37.45392147595687</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.4128907396199</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.155486683818927</v>
+        <v>2.160702698004311</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7818429880358773</v>
+        <v>0.7841695863436213</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.552141834950708</v>
+        <v>2.552141924999353</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7579855596883514</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13543533860.0816</v>
+        <v>13554067691.78019</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>675148257374</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.70246734397677</v>
+        <v>54.12191582002902</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.19206292510496</v>
+        <v>37.10133126409674</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.44770117421272</v>
+        <v>16.2731434541363</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.62169032411776</v>
+        <v>26.33915712884987</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.723796856305274</v>
+        <v>3.684276592507925</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.75223030403129</v>
+        <v>41.30551453337679</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.31501417400042</v>
+        <v>16.140456453924</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01721331023212383</v>
+        <v>0.01739795287339078</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.470810249330164</v>
+        <v>0.4587594023183543</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2351325283748391</v>
+        <v>0.2306064514535573</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004441323719979677</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.708437628580227</v>
+        <v>1.708437703223695</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5483624975385101</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2984558640.127978</v>
+        <v>2996653401.387125</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>83.22097378277149</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>102.5439699485213</v>
+        <v>101.9007429244268</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.868399531889994</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1884362013236883</v>
+        <v>-0.1833133754040329</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1419143706702846</v>
+        <v>0.1423382253953176</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,23 +3562,23 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.20473869529085</v>
+        <v>1.259543936310741</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3581820889076676</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1222505475.221931</v>
+        <v>1222516096.381785</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>705.55</v>
+        <v>712.97</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>301393901550</v>
@@ -3622,7 +3622,7 @@
         <v>15.56444241316271</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.2174965204479</v>
+        <v>14.15903319342078</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.555550010174924</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09473861243979198</v>
+        <v>0.09925884066681689</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3859189857610535</v>
+        <v>-0.383421507698108</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01663974942494984</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.56750119647536</v>
+        <v>1.554299618321783</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3867222481542269</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2075064737.093872</v>
+        <v>2078266928.820394</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.71266375545852</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.45078269159562</v>
+        <v>18.46669292932874</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.233664260966468</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1225899790632292</v>
+        <v>0.1216227959562126</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04438757965885154</v>
+        <v>0.04320487652819227</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02841963231573621</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8667135889614276</v>
+        <v>0.8704068751778097</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8061168994181661</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2531012234.637095</v>
+        <v>2531197614.706625</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>42.90586264656617</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>30.14525027921833</v>
+        <v>29.82788498590782</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>15.13981367588099</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4233042435923913</v>
+        <v>0.4384480383653431</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.1977449256040054</v>
+        <v>0.2163686147984576</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005223542639411591</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3445491068407581</v>
+        <v>0.3253461459545689</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3651487881153955</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3089124933.691406</v>
+        <v>3122624602.117106</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.22668810289389</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.01958223967975</v>
+        <v>16.01555639306635</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.671412118960871</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07535189402281639</v>
+        <v>0.07562220631634609</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3306292604274488</v>
+        <v>-0.3305322271595974</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4066,13 +4066,13 @@
         <v>0.01936537564162389</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.353448962893439</v>
+        <v>1.340308691581038</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3009261286003964</v>
+        <v>0.3063945887261881</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1162576080.537266</v>
+        <v>1141960893.200429</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>113.46</v>
+        <v>114.25</v>
       </c>
       <c r="K29" s="5" t="n">
         <v>1058357015950</v>
@@ -4126,7 +4126,7 @@
         <v>20.91285427359964</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.138593308108139</v>
+        <v>6.13550657397766</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.7238298507876</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.406782828563829</v>
+        <v>2.408496759223877</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.730917723904757</v>
+        <v>1.731843871801404</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005655716275123919</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.8968820088699</v>
+        <v>2.896881555171403</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>1.035586871686965</v>
+        <v>1.035586892302971</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>37040382427.35501</v>
+        <v>37070631563.74715</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.00621118012424</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.23247620246533</v>
+        <v>27.21738805358678</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.926639044257399</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.901176176295415</v>
+        <v>1.902784463541225</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2306805010877448</v>
+        <v>0.2312449873733073</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6671016484260096</v>
+        <v>0.6560038057662955</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.6045984947101118</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2504019941.74769</v>
+        <v>2504249830.302175</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.31501057082453</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.723095895764216</v>
+        <v>9.662410691412996</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.526880582768149</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.837770497263171</v>
+        <v>2.861873787251297</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.05096049534449609</v>
+        <v>-0.04795738436051544</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4444,13 +4444,13 @@
         <v>0.06090651558073654</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3148614885657931</v>
+        <v>0.3123561367188902</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2335064772181578</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1018714479.274884</v>
+        <v>1018752308.637244</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1108509397786</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.553926317439683</v>
+        <v>7.388459601860337</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003490881996180789</v>
+        <v>0.003488160807999701</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.628687819722952</v>
+        <v>6.345407402101007</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.074038897115644</v>
+        <v>4.592799850015036</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01466686872341071</v>
+        <v>0.01653445000752501</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>6.614757970857151</v>
+        <v>7.461588582248683</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.59843551547369</v>
+        <v>6.315155097851746</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.0856361604379413</v>
+        <v>0.07596347762088229</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1876.441381464635</v>
+        <v>2117.153378971446</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2472.325424981083</v>
+        <v>2790.453059770463</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.382750936619185</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6521607337.42915</v>
+        <v>6524185738.328237</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>281.15</v>
+        <v>281.74</v>
       </c>
       <c r="K33" s="5" t="n">
         <v>70698776368</v>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.811780135234249</v>
+        <v>1.811780159525724</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.5018450356600513</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6076906159.080064</v>
+        <v>6077171829.481303</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-90.68181818181819</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>636.3576779026218</v>
+        <v>152.1514283155727</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>110.1686038597285</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>2.756279261968222</v>
+        <v>3.862239302464928</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.9408147440670116</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12570432953.83047</v>
+        <v>12586062218.05738</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.996341987671325</v>
+        <v>0.9893811419452287</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.1241890315225673</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34521112983.8774</v>
+        <v>34532309420.75785</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4909,43 +4909,43 @@
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>223.7</v>
+        <v>225.63</v>
       </c>
       <c r="K36" s="5" t="n">
         <v>2137296543200</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.24006027587806</v>
+        <v>27.52984815115336</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6487259727428066</v>
+        <v>0.6456486418697348</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.7239612187118</v>
+        <v>13.8699608061449</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.472954828886603</v>
+        <v>9.573730944087526</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5117168480253368</v>
+        <v>0.5171606442809255</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.0360992766155</v>
+        <v>18.23499550089752</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.23938180724118</v>
+        <v>13.38538139467429</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01835325730696866</v>
+        <v>0.01816006512479004</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>40.99008737187964</v>
+        <v>41.63905530944761</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.07969946014674</v>
+        <v>41.75742887609249</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4982,13 +4982,13 @@
         <v>0.2669319808779635</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.210667060391127</v>
+        <v>2.176542048017721</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.4757968675882759</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5482072644.359024</v>
+        <v>5482166834.395854</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.46456692913386</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-51.82620940960848</v>
+        <v>-69.56983223271484</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.980578986792192</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.0374588579371451</v>
+        <v>0.0220433448930073</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3238075709544639</v>
+        <v>0.3238075711481519</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2195785437911515</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>624190190.5402787</v>
+        <v>628012705.6512769</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.61249241964827</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.68674389013051</v>
+        <v>17.68057976311738</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.730220986523616</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1654204158601726</v>
+        <v>0.1658267260357047</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>-0.0003798952878687478</v>
+        <v>-0.0001461337303898524</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5240,13 +5240,13 @@
         <v>0.01041482789055605</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9659826167095512</v>
+        <v>0.9691930283192182</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.252928986671957</v>
+        <v>0.2540775957839826</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>957103837.6170136</v>
+        <v>968400267.2697958</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.21212121212121</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.5567719077841</v>
+        <v>16.53598069635157</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.150259737521898</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.462369678520363</v>
+        <v>0.4642083621604167</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4631330818848949</v>
+        <v>0.4653802445684823</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5366,13 +5366,13 @@
         <v>0.01390627172854958</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.04655141801548</v>
+        <v>2.028594101872035</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5912067324046106</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4578762668.075004</v>
+        <v>4591739976.794026</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19 17:53 ET</t>
+          <t>2026-08-20 08:29 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-21)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -470,7 +470,7 @@
     <col width="23" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="23" customWidth="1" min="35" max="35"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -711,7 +711,7 @@
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>223.78</v>
+        <v>224.69</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>4572173922800</v>
@@ -720,7 +720,7 @@
         <v>35.5365296803653</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.87470785105901</v>
+        <v>32.86800109573792</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.794234480306239</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08096868393069379</v>
+        <v>0.08118925689622825</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1051046048970834</v>
+        <v>0.105355626358792</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003405075489881143</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3555033504342336</v>
+        <v>0.3513033229741481</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3601361946228768</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16303847968.12281</v>
+        <v>16331997196.88232</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.73055555555555</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.76450426911686</v>
+        <v>23.75232527676675</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.76667716121372</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1248101476407915</v>
+        <v>0.125386893455099</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.209475906310483</v>
+        <v>0.2101125270553508</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007565208354982854</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5687437376079219</v>
+        <v>0.5604030559783857</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.467677354993122</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15276176620.32986</v>
+        <v>15343436882.70498</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>199.43</v>
+        <v>201.3</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>4122826251802</v>
@@ -974,7 +974,7 @@
         <v>16.91509433962264</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>19.97020164353917</v>
+        <v>19.95953726708458</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.246762491509799</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1529832977377535</v>
+        <v>-0.1525307368965189</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2732064614883771</v>
+        <v>0.274813818124257</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002495083218363812</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7969120002264451</v>
+        <v>0.8097780820773571</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3941904494545274</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9880263624.424618</v>
+        <v>9880525792.711283</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.64365079365079</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.88688757896665</v>
+        <v>22.92325960345977</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.60719533957302</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1357747749510765</v>
+        <v>-0.09944522939769529</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1602796502433819</v>
+        <v>0.1677128038541102</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.857825211032913</v>
+        <v>0.872473367675124</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4597852974834055</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11394660582.76501</v>
+        <v>11396910785.57795</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>33.05640243902439</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.47730044936906</v>
+        <v>19.45934259546436</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.71996185268905</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6971757726361509</v>
+        <v>0.6987419938189108</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9358238619328036</v>
+        <v>0.9376688193594942</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001291215125662901</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.2947123230566</v>
+        <v>1.281296859329106</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3733649386978485</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>25064213437.26144</v>
+        <v>25081863488.12322</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.28353771832033</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.46770955215879</v>
+        <v>16.46464957166182</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.092034079172655</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2317157801499672</v>
+        <v>0.2319446964259351</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2557151368250734</v>
+        <v>0.2563297465338952</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003847351739552608</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8172865684160164</v>
+        <v>0.8138670010556266</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.498518180141499</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>10513545164.82197</v>
+        <v>10516876456.38794</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>292.4830508474577</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>169.340178431097</v>
+        <v>169.2135903984835</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.15499369894517</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.727192291618296</v>
+        <v>0.7284843974924542</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1107019069069288</v>
+        <v>0.1110701441424438</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.508989588126892</v>
+        <v>1.551232982574169</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6143275747529169</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12449535548.86336</v>
+        <v>12458523746.57186</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
         <v>495</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>286.17</v>
+        <v>287.17</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>1731901847400</v>
@@ -1604,7 +1604,7 @@
         <v>58.80936995153473</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.29908463882451</v>
+        <v>20.26327845072171</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>22.94973626714371</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.897143935202602</v>
+        <v>1.902263327948304</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.131409297195924</v>
+        <v>1.141535181588816</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006977446913715903</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.627656138652846</v>
+        <v>1.6093442605739</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4346532178060927</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7540152281.522736</v>
+        <v>7543878419.784241</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>46.88648920140633</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.25475800071267</v>
+        <v>41.24396850757104</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.410117209856022</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1365110710526134</v>
+        <v>0.1368083843047136</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1103936033299036</v>
+        <v>0.1106243150558017</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005934590952426862</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.163794582599252</v>
+        <v>-0.1656926236896975</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.210748372996102</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1818701329.039046</v>
+        <v>1823992806.061401</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.81114551083591</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.45020567480407</v>
+        <v>21.44678406495388</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.898757098812829</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1566856694516308</v>
+        <v>0.1568702065397174</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.134895168765381</v>
+        <v>0.1352233527003812</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1276886102676244</v>
+        <v>0.1189104457545514</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.376075351218768</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3054940709.261726</v>
+        <v>3059797703.449402</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.49585114407845</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.55003814645251</v>
+        <v>22.54993313273961</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.786343085602061</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4458611970887398</v>
+        <v>-0.4458586164969122</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05947089950481366</v>
+        <v>0.0595163034341637</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06819447553262896</v>
+        <v>0.07040144744848219</v>
       </c>
       <c r="AJ12" s="4" t="n">
         <v>0.1662054713708828</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2098134037.400134</v>
+        <v>2113620484.101562</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.11392949269132</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.05380571488308</v>
+        <v>14.05334932798813</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.16491027708621</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0754332171168095</v>
+        <v>0.07546814214537267</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2911021491870769</v>
+        <v>-0.2910518201599754</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2174,13 +2174,13 @@
         <v>0.01706727350305788</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7855488424481497</v>
+        <v>0.7903705505982586</v>
       </c>
       <c r="AJ13" s="4" t="n">
         <v>0.1932887103652243</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2534395085.588593</v>
+        <v>2534701297.346293</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.07306711979609</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>24.67833898195687</v>
+        <v>24.67011791380668</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.34874969607535</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2591231177476985</v>
+        <v>0.2595427078362684</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1297380983430965</v>
+        <v>0.1300450035937042</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2300,13 +2300,13 @@
         <v>0.007327810133158341</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.318823226028293</v>
+        <v>0.315644414471675</v>
       </c>
       <c r="AJ14" s="4" t="n">
         <v>0.203263018356845</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2565350373.774937</v>
+        <v>2588494329.656168</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.51290499725425</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.14796847486686</v>
+        <v>26.14048909569872</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.34561207992475</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2051760360482349</v>
+        <v>0.2055208638938413</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1473724901802731</v>
+        <v>0.1477001847265524</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2426,13 +2426,13 @@
         <v>0.005872614794807005</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3089721702806651</v>
+        <v>0.3039078919834984</v>
       </c>
       <c r="AJ15" s="4" t="n">
         <v>0.2212611921544708</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1635105837.783866</v>
+        <v>1654706697.501628</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>24.74760465564916</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>17.9573001601752</v>
+        <v>17.95110447836283</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7764426950474197</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3781361582702254</v>
+        <v>0.3786118110714809</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008419709500780304</v>
+        <v>0.008498174326312613</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2552,13 +2552,13 @@
         <v>0.02325581395348837</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4168557806015787</v>
+        <v>0.4586125692674896</v>
       </c>
       <c r="AJ16" s="4" t="n">
         <v>0.2489071650790178</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2067513420.898727</v>
+        <v>2081335578.262939</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.48901808785529</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.1414813678954</v>
+        <v>15.14467928037889</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.909176617459702</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4192150401755688</v>
+        <v>0.4189153622880601</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.07925402163176298</v>
+        <v>0.07911482879399956</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2678,13 +2678,13 @@
         <v>0.02477078009920337</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.4935897641807037</v>
+        <v>-0.4963941280109144</v>
       </c>
       <c r="AJ17" s="4" t="n">
         <v>0.2441137742456344</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2207697052.393677</v>
+        <v>2209644274.938812</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.90982658959538</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.67805111776908</v>
+        <v>21.67245414612168</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.579609099306641</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4258581835458071</v>
+        <v>0.4262264153931425</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08243262050364408</v>
+        <v>0.082639686278275</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2804,13 +2804,13 @@
         <v>0.01959830945880241</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.188317288989263</v>
+        <v>-0.1854224297134863</v>
       </c>
       <c r="AJ18" s="4" t="n">
         <v>0.2719612703397984</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1921806068.450979</v>
+        <v>1942883825.522715</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.48736462093864</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.46105293003467</v>
+        <v>33.56998672987502</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.123025422918026</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1203283022600268</v>
+        <v>0.1166928638544089</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04792906633305849</v>
+        <v>0.04896578106968619</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,26 +2927,26 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009293143297380586</v>
+        <v>0.009413520801232665</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.04270740072606952</v>
+        <v>-0.04289677276046609</v>
       </c>
       <c r="AJ19" s="4" t="n">
         <v>0.3256317038750667</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2587289062.473754</v>
+        <v>2588488566.730118</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-20 (C)</t>
+          <t>2026-11-19 (E)</t>
         </is>
       </c>
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.18666666666666</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.32371975242235</v>
+        <v>20.32045619840998</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.906202891809909</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04246008726534733</v>
+        <v>0.04262751090816841</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02329388733336324</v>
+        <v>0.02337378423366876</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3056,13 +3056,13 @@
         <v>0.03000209775540173</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05663545905880082</v>
+        <v>-0.04634117165808813</v>
       </c>
       <c r="AJ20" s="4" t="n">
         <v>0.2035102773401885</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1282547913.359699</v>
+        <v>1297517544.446513</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>23.35824022346369</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.3145965173512</v>
+        <v>22.31233398660286</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.971471516822717</v>
@@ -3140,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04676955307262554</v>
+        <v>0.04687569832402216</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01351098766373471</v>
+        <v>0.01378773042866599</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3182,13 +3182,13 @@
         <v>0.02768393673951389</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7265802042931603</v>
+        <v>0.736176023309619</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2976963542611242</v>
+        <v>0.2919129440608622</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1310969099.802336</v>
+        <v>1313976628.522542</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>119.1510152284264</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>37.6976345493232</v>
+        <v>36.44527165510803</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.53270361941654</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.160702698004311</v>
+        <v>2.269313406578124</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.7841695863436215</v>
+        <v>0.8253059761884947</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.543109466580352</v>
+        <v>2.538904909509764</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7547920930154839</v>
+        <v>0.7547929899433202</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13302334922.17287</v>
+        <v>13302703326.65619</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>674600963827</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.62264150943396</v>
+        <v>54.93468795355587</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.07125591550133</v>
+        <v>37.04035053187791</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.42369948767957</v>
+        <v>16.51752426223197</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.58284200976843</v>
+        <v>26.73470360222493</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.71836282003314</v>
+        <v>3.739604961824214</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.69080688550834</v>
+        <v>41.93091661226411</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.29101248746727</v>
+        <v>16.38483726201967</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01723846586022694</v>
+        <v>0.01714054590882942</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4734499859928814</v>
+        <v>0.4831038898046502</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2429993978254252</v>
+        <v>0.2509068921207229</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004444926898663665</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.71672418304472</v>
+        <v>1.712750481680561</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5483506754652504</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2949200614.290039</v>
+        <v>2951828821.530355</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>80.56179775280896</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>98.64468858255717</v>
+        <v>97.08459456808532</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.808698196712591</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1833133754040327</v>
+        <v>-0.1701896875480995</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1423382253953178</v>
+        <v>0.1427578770417255</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.270995235458507</v>
+        <v>1.206937526886893</v>
       </c>
       <c r="AJ24" s="4" t="n">
         <v>0.3663736817188189</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1252977533.774078</v>
+        <v>1253005425.07487</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>712.97</v>
+        <v>718.58</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>295582263650</v>
@@ -3622,7 +3622,7 @@
         <v>15.26432053625838</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.88601116639549</v>
+        <v>13.88440335785933</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.506272532368977</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09925884066681689</v>
+        <v>0.09938613441519939</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.383421507698108</v>
+        <v>-0.3833788024082512</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3688,13 +3688,13 @@
         <v>0.01696691451669245</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.557754291758406</v>
+        <v>1.569242318676463</v>
       </c>
       <c r="AJ25" s="4" t="n">
         <v>0.3881896311739879</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2093198628.003017</v>
+        <v>2093205073.881429</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.40960698689956</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.19649802097669</v>
+        <v>18.19325446935294</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.186350991504697</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1216227959562124</v>
+        <v>0.1218227624573787</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04320487652819227</v>
+        <v>0.04331239982561752</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3814,13 +3814,13 @@
         <v>0.02884162779750952</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8740683164108131</v>
+        <v>0.8758258669664725</v>
       </c>
       <c r="AJ26" s="4" t="n">
         <v>0.8060449632631772</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2459787158.600978</v>
+        <v>2463333879.557699</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>41.73165829145729</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.01158552719171</v>
+        <v>28.99254722625216</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.72548253190202</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4384480383653429</v>
+        <v>0.4393926123769534</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2163686147984576</v>
+        <v>0.2168357011352939</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3940,13 +3940,13 @@
         <v>0.005370517544493413</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3419119572038311</v>
+        <v>0.363029635524021</v>
       </c>
       <c r="AJ27" s="4" t="n">
         <v>0.3735316832344959</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3146644343.741455</v>
+        <v>3146665083.741862</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>16.68649517684888</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.51334202553763</v>
+        <v>15.51092035084966</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.587642219570217</v>
@@ -4011,20 +4011,30 @@
       <c r="P28" s="6" t="n">
         <v>0.4245310596275227</v>
       </c>
-      <c r="Q28" s="6" t="inlineStr"/>
-      <c r="R28" s="6" t="inlineStr"/>
-      <c r="S28" s="4" t="inlineStr"/>
+      <c r="Q28" s="6" t="n">
+        <v>23.57494062084711</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>5.467946339574327</v>
+      </c>
+      <c r="S28" s="4" t="n">
+        <v>-0.04790297980430896</v>
+      </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07562220631634609</v>
+        <v>0.07579014006959439</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3305322271595973</v>
-      </c>
-      <c r="W28" s="4" t="inlineStr"/>
-      <c r="X28" s="4" t="inlineStr"/>
+        <v>-0.3304351938917462</v>
+      </c>
+      <c r="W28" s="4" t="n">
+        <v>0.01207481297651363</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>0.1812783863660298</v>
+      </c>
       <c r="Y28" s="4" t="n">
         <v>0.5971674477787701</v>
       </c>
@@ -4046,7 +4056,9 @@
       <c r="AE28" s="6" t="n">
         <v>0.3131696413913079</v>
       </c>
-      <c r="AF28" s="6" t="inlineStr"/>
+      <c r="AF28" s="6" t="n">
+        <v>12.41837325791393</v>
+      </c>
       <c r="AG28" s="6" t="n">
         <v>0.4478854275047432</v>
       </c>
@@ -4054,27 +4066,23 @@
         <v>0.01999229212833606</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.352030104640574</v>
+        <v>1.366138171814245</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.3152951361437119</v>
+        <v>0.306752441902052</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1145804528.81653</v>
+        <v>1166136901.081187</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
           <t>2026-10-14 (C)</t>
         </is>
       </c>
-      <c r="AM28" s="2" t="inlineStr">
-        <is>
-          <t>roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda</t>
-        </is>
-      </c>
+      <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4126,7 @@
         <v>21.74358402142379</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.379229777051295</v>
+        <v>6.369939370227888</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.18954027405454</v>
@@ -4142,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.408496759223877</v>
+        <v>2.41346797161837</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.731843871801404</v>
+        <v>1.735480524237321</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763496182295395</v>
@@ -4184,13 +4192,13 @@
         <v>0.0005439635441790769</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.887138248103706</v>
+        <v>2.893589209167899</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>1.026332605006858</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>36528633146.19776</v>
+        <v>36532955891.22925</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4200,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4252,7 @@
         <v>80.59006211180125</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.76301965371765</v>
+        <v>27.7476280293149</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.105592893021994</v>
@@ -4268,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.902784463541224</v>
+        <v>1.904394639666468</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2312449873733073</v>
+        <v>0.2318094740051477</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4310,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6406739233296107</v>
+        <v>0.6513588243883968</v>
       </c>
       <c r="AJ30" s="4" t="n">
         <v>0.6010900894209663</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2526017464.035215</v>
+        <v>2526050178.335215</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4326,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4378,7 @@
         <v>36.75343551797041</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.516995516347469</v>
+        <v>9.517719445120418</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.488852103742778</v>
@@ -4394,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.861873787251297</v>
+        <v>2.861580048654754</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04795738436051555</v>
+        <v>-0.04806618126821594</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4436,13 +4444,13 @@
         <v>0.06183713823476541</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3199662139350291</v>
+        <v>0.327178109118475</v>
       </c>
       <c r="AJ31" s="4" t="n">
         <v>0.2372580664543968</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1022365641.384645</v>
+        <v>1022371021.528823</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4452,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4493,37 +4501,37 @@
         <v>1157631356243</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.388459601860337</v>
+        <v>7.558861686113768</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003584550101192597</v>
+        <v>0.003567056385607636</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.345407402101007</v>
+        <v>6.491753285413805</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.592799850015036</v>
+        <v>4.698724861340043</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01653445000752501</v>
+        <v>0.01691578859433369</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.461588582248683</v>
+        <v>7.634501639024965</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.315155097851746</v>
+        <v>6.461500981164543</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07596347762088229</v>
+        <v>0.07425100616006471</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2060.19579676182</v>
+        <v>2118.075469794162</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2691.073796582972</v>
+        <v>2757.407862423892</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4566,7 +4574,7 @@
         <v>1.364580280055541</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>6424295180.073595</v>
+        <v>6425648994.144795</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4580,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4644,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.810468529090777</v>
+        <v>1.810027289631095</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.500255195717265</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6006624895.482007</v>
+        <v>6011779201.070659</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4660,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4712,7 @@
         <v>-87.01298701298701</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>145.9956419211367</v>
+        <v>136.7499860202427</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>105.7113706924887</v>
@@ -4729,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.862239302464928</v>
+        <v>3.930091944048431</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4772,7 +4780,7 @@
         <v>0.8403138488945874</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12878174035.13754</v>
+        <v>12887586833.87087</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4786,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4850,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9892503623153246</v>
+        <v>0.9963717956836434</v>
       </c>
       <c r="AJ35" s="4" t="n">
         <v>0.1258596746409782</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34650290237.17126</v>
+        <v>34651616347.6888</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4866,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -4907,37 +4915,37 @@
         <v>2157575680000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.52984815115336</v>
+        <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6517746973180851</v>
+        <v>0.6497940021162968</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.8699608061449</v>
+        <v>14.07436022855125</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.573730944087526</v>
+        <v>9.714817505368815</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5171606442809255</v>
+        <v>0.5247819590387496</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.23499550089752</v>
+        <v>18.51345021489235</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.38538139467429</v>
+        <v>13.58978081708063</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01816006512479004</v>
+        <v>0.01789632973916031</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.23828918863045</v>
+        <v>41.9913958663149</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.3555501575696</v>
+        <v>42.01922532757949</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4974,13 +4982,13 @@
         <v>0.2644230769230769</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.160789760286776</v>
+        <v>2.185215131129227</v>
       </c>
       <c r="AJ36" s="4" t="n">
         <v>0.4753632337725694</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5460292451.389408</v>
+        <v>5460362991.122742</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4994,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5038,7 +5046,7 @@
         <v>-22.22834645669291</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-68.83828825550439</v>
+        <v>-69.37756415105972</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.959752709317458</v>
@@ -5063,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.0220433448930073</v>
+        <v>0.02212403877901448</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5102,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3263364402574147</v>
+        <v>0.3181249171304611</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2115480692694484</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>629417189.6963819</v>
+        <v>632639632.8521284</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5122,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5174,7 @@
         <v>20.08186779866586</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.23142809247742</v>
+        <v>17.2253424790519</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.659937274749325</v>
@@ -5190,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1654209790906902</v>
+        <v>0.1658327155519743</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.0002156581788592682</v>
+        <v>0.0004504109104790377</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5232,13 +5240,13 @@
         <v>0.01069001962856712</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9790114515673115</v>
+        <v>0.9768865335179416</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2614012736027859</v>
+        <v>0.2609508606326678</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>971187353.254954</v>
+        <v>959832295.0286865</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5248,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>
@@ -5292,7 +5300,7 @@
         <v>23.91414141414142</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.33247154718913</v>
+        <v>16.31766688449992</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.074568180468541</v>
@@ -5316,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4642083621604169</v>
+        <v>0.4655368064203678</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.465380244568482</v>
+        <v>0.4670424379858267</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5358,13 +5366,13 @@
         <v>0.01407954945441746</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.023947556791989</v>
+        <v>2.02444578801389</v>
       </c>
       <c r="AJ39" s="4" t="n">
         <v>0.5803990821440267</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4494366803.176778</v>
+        <v>4494381635.285542</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5374,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-20 17:55 ET</t>
+          <t>2026-08-21 08:29 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-22)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.31392694063928</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.66211416307911</v>
+        <v>32.7129571056517</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.732882866953855</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08118925689622847</v>
+        <v>0.07950885719647238</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.105355626358792</v>
+        <v>0.1037998404184812</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -790,7 +790,7 @@
         <v>0.3596991676175606</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16409227011.03204</v>
+        <v>16456166172.33816</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.84666666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.85549967108961</v>
+        <v>23.84328030706784</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.81344502002477</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1253868934550988</v>
+        <v>0.1259636392694061</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2101125270553508</v>
+        <v>0.2107491478002186</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -920,7 +920,7 @@
         <v>0.4668257055831498</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15379372779.19473</v>
+        <v>15389562925.3008</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>201.3</v>
+        <v>205.28</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>4173050013639</v>
@@ -974,7 +974,7 @@
         <v>17.12115193644489</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.20268189284676</v>
+        <v>20.22053542132392</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.359405413809499</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1525307368965189</v>
+        <v>-0.1532790017820462</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.274813818124257</v>
+        <v>0.2755078001268267</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1046,7 +1046,7 @@
         <v>0.3946452532388603</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9903684981.673088</v>
+        <v>9903963987.035013</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.52619047619048</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.79282853885972</v>
+        <v>22.80401219994041</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.58667075727104</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.09944522939769518</v>
+        <v>-0.09988688410524027</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1677128038541102</v>
+        <v>0.1681400235647383</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1172,7 +1172,7 @@
         <v>0.4601697648890013</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11444210953.00845</v>
+        <v>11446039234.37597</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>32.73170731707317</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.23161557773916</v>
+        <v>19.21382588987824</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.51644089928242</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7019738765452725</v>
+        <v>0.7035496992983632</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9501401994478635</v>
+        <v>0.952029926048938</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1298,7 +1298,7 @@
         <v>0.3585649135905839</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>24694990183.62466</v>
+        <v>24744765772.68631</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.43478260869565</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.58741879240209</v>
+        <v>16.6152392409601</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.13745953893572</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2319446964259351</v>
+        <v>0.2298819362359565</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2563297465338952</v>
+        <v>0.2566335033965461</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1424,7 +1424,7 @@
         <v>0.4988883384652686</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9853117040.462797</v>
+        <v>9862058836.449789</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>307.5084745762712</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.9064219627205</v>
+        <v>177.773529688822</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.83079133544041</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7284843974924542</v>
+        <v>0.7297765033666128</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1110701441424438</v>
+        <v>0.1114383813779594</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1550,7 +1550,7 @@
         <v>0.611850585080307</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12704443323.94502</v>
+        <v>12718612135.50903</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>59.52342487883683</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.50931226868229</v>
+        <v>20.48443222068591</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.22838867024448</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.902263327948304</v>
+        <v>1.905788368336026</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.141535181588816</v>
+        <v>1.144070801184837</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1676,7 +1676,7 @@
         <v>0.4296133661701584</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7582832781.71288</v>
+        <v>7583098692.08669</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.60120542440984</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.87267272269754</v>
+        <v>41.86172448760554</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431612392442445</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1368083843047136</v>
+        <v>0.1371056975568139</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1106243150558017</v>
+        <v>0.1108550267816999</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1802,7 +1802,7 @@
         <v>0.2135130002947417</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1828869823.633309</v>
+        <v>1834570416.491903</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.64086687306502</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.29959500536161</v>
+        <v>21.30467666633804</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.851410999421056</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1568702065397176</v>
+        <v>0.1565942660842277</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1352233527003812</v>
+        <v>0.1355544048504347</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1928,7 +1928,7 @@
         <v>0.3766737779099306</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>3006620674.400589</v>
+        <v>3008298548.255386</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.46718632134775</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.49820477679281</v>
+        <v>22.35200028154181</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.779951361686254</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4458586164969122</v>
+        <v>-0.4422339761849815</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.0595163034341637</v>
+        <v>0.05956170736351374</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1650843383128798</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2145092970.486847</v>
+        <v>2145165641.172587</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.11521926053311</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.0545485897712</v>
+        <v>14.05409219357306</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.165180359032768</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0754681421453729</v>
+        <v>0.07550306717393651</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2910518201599754</v>
+        <v>-0.2910014911328739</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1926001760985463</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2529500364.060603</v>
+        <v>2558722579.207865</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.52421410365336</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.02830107111484</v>
+        <v>25.01972001481664</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.57159677146646</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2595427078362684</v>
+        <v>0.2599746953596909</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1300450035937042</v>
+        <v>0.1303790397451798</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.2051636433303028</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2592520308.233508</v>
+        <v>2616270430.764465</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2345,10 +2345,10 @@
         <v>0.03107629670848255</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.03512970071622046</v>
+        <v>-0.03488913267511051</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>601.77</v>
+        <v>601.62</v>
       </c>
       <c r="J15" s="3" t="n">
         <v>464.52</v>
@@ -2360,7 +2360,7 @@
         <v>31.88522789676002</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.44933725474522</v>
+        <v>26.43569379877291</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.51510454294102</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2055208638938413</v>
+        <v>0.2061430329564518</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1477001847265524</v>
+        <v>0.1481248585501544</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2218410096444005</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1668901230.433407</v>
+        <v>1668902507.819417</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.08584656935246</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.19645411992757</v>
+        <v>18.19017808987016</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7870548519291136</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3786118110714811</v>
+        <v>0.3790874638727371</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008498174326312613</v>
+        <v>0.008576639151844923</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2509048795578694</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2091031519.418424</v>
+        <v>2091044692.132263</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2609,10 +2609,10 @@
         <v>684291790600</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.33204134366925</v>
+        <v>21.24967824967825</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.03404777383652</v>
+        <v>15.03722366687584</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.895230129618346</v>
@@ -2621,7 +2621,7 @@
         <v>2.656891582273113</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.179578137287944</v>
+        <v>2.080697661947664</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>9.969673381134703</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4189153622880601</v>
+        <v>0.413138403765801</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.07911482879399956</v>
+        <v>0.0789756359562368</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2451798826150538</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2242830880.628749</v>
+        <v>2243243771.207275</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2738,13 +2738,13 @@
         <v>31.24161849710983</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.90509035586611</v>
+        <v>21.89943622565933</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.650235864146474</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.760580013416342</v>
+        <v>7.760443257111249</v>
       </c>
       <c r="P18" s="6" t="n">
         <v>-3.868205658655315</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4262264153931425</v>
+        <v>0.4265946472404782</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.082639686278275</v>
+        <v>0.08284675205290615</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.262293274102694</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1942593353.258331</v>
+        <v>1942598037.418162</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.43682310469315</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.52472673235785</v>
+        <v>33.70674751192277</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.121511328549685</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1166928638544089</v>
+        <v>0.1106625785074924</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04896578106968619</v>
+        <v>0.04785574493170053</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3210384069276272</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2694021402.002074</v>
+        <v>2695055339.36498</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.43407407407408</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.55774842868301</v>
+        <v>20.55444782468496</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.951817595884273</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04262751090816841</v>
+        <v>0.04279493455098926</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02337378423366876</v>
+        <v>0.02345368113397428</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1984773897731298</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1275219238.650132</v>
+        <v>1283589222.182414</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.2914177937939828</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1308626263.323983</v>
+        <v>1320493365.284017</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>120.1142131979695</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.73988946923534</v>
+        <v>36.65574715207108</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.68251906548844</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.269313406578124</v>
+        <v>2.276818030734997</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8253059761884944</v>
+        <v>0.8291973630995617</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3314,7 +3314,7 @@
         <v>0.7422839987287737</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>13142120042.32907</v>
+        <v>13143929135.10406</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.644412191582</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.32498166273687</v>
+        <v>37.29389067405498</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.43024540219376</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4640171209015183</v>
+        <v>0.4652376355465004</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2348083767479885</v>
+        <v>0.2358462634671634</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3438,7 +3438,7 @@
         <v>0.5115820229194993</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2929336477.062842</v>
+        <v>2936032180.395915</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>80.22471910112355</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>96.67838287533182</v>
+        <v>96.08847528594903</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.801130421830948</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1701896875480996</v>
+        <v>-0.1650953055256277</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1427578770417253</v>
+        <v>0.1431824643765223</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,17 +3568,17 @@
         <v>0.3636468032817798</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1269159878.21896</v>
+        <v>1269207694.798279</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>718.58</v>
+        <v>721.16</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>306594874960</v>
@@ -3622,7 +3622,7 @@
         <v>15.83302864107252</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.40169940791061</v>
+        <v>14.39024718763068</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599649600719028</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.09938613441519939</v>
+        <v>0.100261061163841</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3833788024082513</v>
+        <v>-0.3833128107861627</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3990489279135445</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2142048413.930339</v>
+        <v>2149248545.973307</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.58340611353712</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.3481801246827</v>
+        <v>18.34491011839173</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.213484537968363</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1218227624573787</v>
+        <v>0.1220227289585452</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04331239982561752</v>
+        <v>0.04341992312304277</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.7963160021596862</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2451912196.485464</v>
+        <v>2458631158.116659</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>42.03584589614741</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.20387775697358</v>
+        <v>29.21555114750615</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.83281853154051</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4393926123769534</v>
+        <v>0.4388174874371862</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2168357011352939</v>
+        <v>0.2170698723767857</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3737932909435933</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3145691378.589746</v>
+        <v>3171675313.521729</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.21864951768489</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.00558405989014</v>
+        <v>16.00308593485209</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.670165543077081</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07579014006959439</v>
+        <v>0.07595807382284292</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3304351938917462</v>
+        <v>-0.3303381606238949</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.3178658012200694</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1162953376.285189</v>
+        <v>1171897339.997762</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.57509484490069</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.320579253793804</v>
+        <v>6.30627631159537</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.09508456698496</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.41346797161837</v>
+        <v>2.421209883434777</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.735480524237321</v>
+        <v>1.741829319938931</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4198,7 +4198,7 @@
         <v>0.9679567165909377</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>36177480883.28703</v>
+        <v>36201689538.61063</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.80124223602485</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.47603274918211</v>
+        <v>27.46080866844116</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.016466858539234</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.904394639666468</v>
+        <v>1.906004815791713</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2318094740051475</v>
+        <v>0.2323739606369883</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5997728336907299</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2530581693.324819</v>
+        <v>2539629622.933273</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.09038054968288</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.604975186932595</v>
+        <v>9.605705863630638</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.511669191158</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.861580048654754</v>
+        <v>2.861286310058212</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04806618126821582</v>
+        <v>-0.04817497817591598</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.234096834597786</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1034924294.423277</v>
+        <v>1034932846.416518</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.558861686113768</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003574274490876525</v>
+        <v>0.003565298722522418</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.491753285413805</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2113.796081109063</v>
+        <v>2119.120156654345</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2751.837367383911</v>
+        <v>2756.326031517468</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.34087574829858</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>5907249567.502287</v>
+        <v>5907574252.285563</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
         <v>0.4698050852213885</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6056313523.653601</v>
+        <v>6056619737.132263</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-88.94155844155844</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.7809372029302</v>
+        <v>139.0925910469354</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>108.0543764459125</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.930091944048431</v>
+        <v>3.940039257009442</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.8420151073298282</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13015744262.49574</v>
+        <v>13020765445.77049</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>0.1201842836610447</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34575727757.49226</v>
+        <v>34587128919.47205</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6544019163139965</v>
+        <v>0.6539594505576378</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.07436022855125</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.68867569014679</v>
+        <v>41.71755863871658</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.71630919267947</v>
+        <v>41.74933466957107</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.4456280842784813</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5425227883.909221</v>
+        <v>5446450076.077576</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.48031496062992</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-70.16399066641002</v>
+        <v>-70.71799207279864</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.981967405288661</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02212403877901448</v>
+        <v>0.02220473266502188</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5116,7 +5116,7 @@
         <v>0.2127800295994011</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>635661355.3460509</v>
+        <v>635710218.6697451</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.37598544572468</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.47762365381682</v>
+        <v>17.47145327083883</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.69889453213279</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1658327155519743</v>
+        <v>0.1662444520132584</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.0004504109104790377</v>
+        <v>0.0006851636420992513</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.2635312010075681</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>956402281.3118652</v>
+        <v>956507090.9118652</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.65824915824916</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.825404213817</v>
+        <v>16.81016654175486</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.263583255144155</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4655368064203678</v>
+        <v>0.466865250680319</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4670424379858267</v>
+        <v>0.4687046314031711</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5372,7 +5372,7 @@
         <v>0.5709504350446908</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4436156341.00444</v>
+        <v>4450228714.900055</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21 17:52 ET</t>
+          <t>2026-08-22 08:20 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-23)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.31392694063928</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.7129571056517</v>
+        <v>32.70641624240266</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.732882866953855</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07950885719647238</v>
+        <v>0.0797247451053984</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1037998404184812</v>
+        <v>0.1040464878800533</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.84666666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.84328030706784</v>
+        <v>23.82918888268729</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.81344502002477</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1259636392694061</v>
+        <v>0.1266294794520546</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2107491478002186</v>
+        <v>0.2113734123326352</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.12115193644489</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.22053542132392</v>
+        <v>20.23801507801613</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.359405413809499</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1532790017820462</v>
+        <v>-0.1540103181836733</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2755078001268267</v>
+        <v>0.2762017897689619</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.52619047619048</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.80401219994041</v>
+        <v>22.8152068412884</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.58667075727104</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.09988688410524027</v>
+        <v>-0.1003285388127854</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1681400235647383</v>
+        <v>0.1685672432753658</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>32.73170731707317</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.21382588987824</v>
+        <v>19.18085031959008</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.51644089928242</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7035496992983632</v>
+        <v>0.7064784288339461</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.952029926048938</v>
+        <v>0.9549655142156033</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.43478260869565</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.6152392409601</v>
+        <v>16.6122309905875</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.13745953893572</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2298819362359565</v>
+        <v>0.2301046512219829</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2566335033965461</v>
+        <v>0.2572471081025542</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>307.5084745762712</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.773529688822</v>
+        <v>177.6408358020779</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.83079133544041</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7297765033666128</v>
+        <v>0.731068609240771</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1114383813779594</v>
+        <v>0.1118066186134745</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>59.52342487883683</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.48443222068591</v>
+        <v>20.45961246401035</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.22838867024448</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.905788368336026</v>
+        <v>1.909313408723748</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.144070801184837</v>
+        <v>1.146606420780857</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.60120542440984</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.86172448760554</v>
+        <v>41.85078197617585</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431612392442445</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1371056975568139</v>
+        <v>0.1374030108089141</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1108550267816999</v>
+        <v>0.1110857385075981</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.64086687306502</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.30467666633804</v>
+        <v>21.30131423859113</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.851410999421056</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1565942660842277</v>
+        <v>0.1567768353195642</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1355544048504347</v>
+        <v>0.1358825914395911</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.46718632134775</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.35200028154181</v>
+        <v>22.3519741655507</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.779951361686254</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422339761849815</v>
+        <v>-0.4422333244925445</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05956170736351374</v>
+        <v>0.05960711129286356</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.11521926053311</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.05409219357306</v>
+        <v>14.05294142975869</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.165180359032768</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07550306717393651</v>
+        <v>0.07559113770480241</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2910014911328739</v>
+        <v>-0.2909319594096048</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.52421410365336</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.01972001481664</v>
+        <v>25.01139935336542</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.57159677146646</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2599746953596909</v>
+        <v>0.2603938571478452</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1303790397451798</v>
+        <v>0.1306854677942397</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.88522789676002</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.43569379877291</v>
+        <v>26.42534620353858</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.51510454294102</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2061430329564518</v>
+        <v>0.206615332535939</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1481248585501544</v>
+        <v>0.1484922714021817</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.08584656935246</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.19017808987016</v>
+        <v>18.18390638757599</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7870548519291136</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3790874638727371</v>
+        <v>0.3795631166739928</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008576639151844923</v>
+        <v>0.008655103977377454</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.24967824967825</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.03722366687584</v>
+        <v>15.04040090199255</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.895230129618346</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.413138403765801</v>
+        <v>0.4128398829357733</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.0789756359562368</v>
+        <v>0.07883644311847382</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.24161849710983</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.89943622565933</v>
+        <v>21.89378501358146</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.650235864146474</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4265946472404782</v>
+        <v>0.4269628790878139</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08284675205290615</v>
+        <v>0.08305381782753707</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.43682310469315</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.70674751192277</v>
+        <v>33.696571942121</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.121511328549685</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1106625785074924</v>
+        <v>0.1109979724049257</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04785574493170053</v>
+        <v>0.04798030108309348</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.43407407407408</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.55444782468496</v>
+        <v>20.55114828035918</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.951817595884273</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04279493455098926</v>
+        <v>0.04296235819381033</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02345368113397428</v>
+        <v>0.02353357803428002</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>23.43645251396648</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.38704418441145</v>
+        <v>22.38581971280836</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.978072754823379</v>
@@ -3140,7 +3140,7 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04687569832402216</v>
+        <v>0.04693296089385468</v>
       </c>
       <c r="V21" s="4" t="n">
         <v>0.01378773042866599</v>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>120.1142131979695</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.65574715207108</v>
+        <v>36.57614004643607</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.68251906548844</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.276818030734997</v>
+        <v>2.283949947847854</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8291973630995617</v>
+        <v>0.833835415135519</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.644412191582</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.29389067405498</v>
+        <v>37.26285143864953</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.43024540219376</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4652376355465004</v>
+        <v>0.4664581501914824</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2358462634671634</v>
+        <v>0.2366425825778211</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>80.22471910112355</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>96.08847528594903</v>
+        <v>95.49917259823697</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.801130421830948</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1650953055256277</v>
+        <v>-0.159943307167411</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1431824643765223</v>
+        <v>0.143607066512573</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83302864107252</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.39024718763068</v>
+        <v>14.38855251754607</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599649600719028</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.100261061163841</v>
+        <v>0.1003906488692996</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3833128107861627</v>
+        <v>-0.3832700059820655</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.58340611353712</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.34491011839173</v>
+        <v>18.34164127745184</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.213484537968363</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1220227289585452</v>
+        <v>0.1222226954597119</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04341992312304277</v>
+        <v>0.0435274464204678</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>42.03584589614741</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.21555114750615</v>
+        <v>29.19651131973573</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.83281853154051</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4388174874371862</v>
+        <v>0.4397557788944726</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2170698723767857</v>
+        <v>0.2175367740960465</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
         <v>232.25</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>144.67</v>
+        <v>145.66</v>
       </c>
       <c r="K28" s="5" t="n">
         <v>337853376000</v>
@@ -4000,7 +4000,7 @@
         <v>17.21864951768489</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.00308593485209</v>
+        <v>15.99997298650046</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.670165543077081</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07595807382284292</v>
+        <v>0.076167411795798</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3303381606238949</v>
+        <v>-0.3302218211312649</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.57509484490069</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.30627631159537</v>
+        <v>6.266880505213346</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.09508456698496</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.421209883434777</v>
+        <v>2.442716807341805</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.741829319938931</v>
+        <v>1.74547407708723</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.80124223602485</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.46080866844116</v>
+        <v>27.44560144925267</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.016466858539234</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.906004815791713</v>
+        <v>1.907614991916958</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2323739606369883</v>
+        <v>0.2329384472688285</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.09038054968288</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.605705863630638</v>
+        <v>9.606783891268108</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.511669191158</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.861286310058212</v>
+        <v>2.860853014857077</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04817497817591598</v>
+        <v>-0.04828377508361636</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.558861686113768</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003565298722522418</v>
+        <v>0.003561938248463475</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.491753285413805</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2119.120156654345</v>
+        <v>2121.120362242231</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2756.326031517468</v>
+        <v>2760.44775222109</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-88.94155844155844</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.0925910469354</v>
+        <v>138.4109911406423</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>108.0543764459125</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.940039257009442</v>
+        <v>3.949986569970455</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6539594505576378</v>
+        <v>0.6535002167216367</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.07436022855125</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.71755863871658</v>
+        <v>41.74757752442817</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.74933466957107</v>
+        <v>41.78236014646265</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.48031496062992</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-70.71799207279864</v>
+        <v>-71.28081168363011</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.981967405288661</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02220473266502188</v>
+        <v>0.02228542655102905</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.37598544572468</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.47145327083883</v>
+        <v>17.46528724316564</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.69889453213279</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1662444520132584</v>
+        <v>0.1666561884745426</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.0006851636420992513</v>
+        <v>0.0009199163737190208</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.65824915824916</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.81016654175486</v>
+        <v>16.7949564442533</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.263583255144155</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.466865250680319</v>
+        <v>0.4681936949402703</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4687046314031711</v>
+        <v>0.4703668248205155</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22 08:20 ET</t>
+          <t>2026-08-23 08:21 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-24)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.31392694063928</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.70641624240266</v>
+        <v>32.69987799428496</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.732882866953855</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.0797247451053984</v>
+        <v>0.07994063301432441</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1040464878800533</v>
+        <v>0.104293135341625</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>26.84666666666666</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>23.82918888268729</v>
+        <v>23.81706559550955</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.81344502002477</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1266294794520546</v>
+        <v>0.1272029528158292</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2113734123326352</v>
+        <v>0.2120066281068302</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.12115193644489</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.23801507801613</v>
+        <v>20.25588569367279</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.359405413809499</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1540103181836733</v>
+        <v>-0.1547566867543633</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2762017897689619</v>
+        <v>0.2768957794110971</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.52619047619048</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.8152068412884</v>
+        <v>22.82641247908251</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.58667075727104</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1003285388127854</v>
+        <v>-0.1007701935203306</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1685672432753658</v>
+        <v>0.1689944629859936</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>32.73170731707317</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.18085031959008</v>
+        <v>19.1420084563231</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.51644089928242</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7064784288339461</v>
+        <v>0.709941116772469</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9549655142156033</v>
+        <v>0.9587814224078313</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.43478260869565</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.6122309905875</v>
+        <v>16.60922382932737</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.13745953893572</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2301046512219829</v>
+        <v>0.2303273662080094</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2572471081025542</v>
+        <v>0.2578607128085628</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>307.5084745762712</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>177.6408358020779</v>
+        <v>177.5083398585786</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.83079133544041</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.731068609240771</v>
+        <v>0.7323607151149294</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1118066186134745</v>
+        <v>0.1121748558489895</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>59.52342487883683</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.45961246401035</v>
+        <v>20.43485277976669</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.22838867024448</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.909313408723748</v>
+        <v>1.91283844911147</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.146606420780857</v>
+        <v>1.149142040376878</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.60120542440984</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.85078197617585</v>
+        <v>41.83984518392123</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.431612392442445</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1374030108089141</v>
+        <v>0.1377003240610142</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1110857385075981</v>
+        <v>0.1113164502334958</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.64086687306502</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.30131423859113</v>
+        <v>21.29795287203247</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.851410999421056</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1567768353195642</v>
+        <v>0.1569594045549008</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1358825914395911</v>
+        <v>0.1362107780287474</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.46718632134775</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.3519741655507</v>
+        <v>22.35194804962063</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.779951361686254</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422333244925445</v>
+        <v>-0.4422326728001076</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05960711129286356</v>
+        <v>0.0596525152222136</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.11521926053311</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.05294142975869</v>
+        <v>14.05248218338871</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.165180359032768</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07559113770480241</v>
+        <v>0.07562628888443945</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2909319594096048</v>
+        <v>-0.2908818131196602</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.52421410365336</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.01139935336542</v>
+        <v>25.00308422438139</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.57159677146646</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2603938571478452</v>
+        <v>0.2608130189359994</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1306854677942397</v>
+        <v>0.1309918958432996</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.88522789676002</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.42534620353858</v>
+        <v>26.4150067057526</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.51510454294102</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.206615332535939</v>
+        <v>0.2070876321154265</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1484922714021817</v>
+        <v>0.1488596842542089</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.08584656935246</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.18390638757599</v>
+        <v>18.17763900857017</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7870548519291136</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3795631166739928</v>
+        <v>0.3800387694752487</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008655103977377454</v>
+        <v>0.008733568802909764</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.24967824967825</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.04040090199255</v>
+        <v>15.04357948003752</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.895230129618346</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4128398829357733</v>
+        <v>0.4125413621057457</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.07883644311847382</v>
+        <v>0.0786972502807104</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.24161849710983</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.89378501358146</v>
+        <v>21.88813671737397</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.650235864146474</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4269628790878139</v>
+        <v>0.4273311109351492</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08305381782753707</v>
+        <v>0.08326088360216799</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.43682310469315</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.696571942121</v>
+        <v>33.68640251417391</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.121511328549685</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1109979724049257</v>
+        <v>0.111333366302359</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04798030108309348</v>
+        <v>0.04810485723448665</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.43407407407408</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.55114828035918</v>
+        <v>20.54784979519543</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.951817595884273</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04296235819381033</v>
+        <v>0.04312978183663119</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02353357803428002</v>
+        <v>0.02361347493458554</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>120.1142131979695</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.57614004643607</v>
+        <v>36.51344960282042</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.68251906548844</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.283949947847854</v>
+        <v>2.289588206661567</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.833835415135519</v>
+        <v>0.8363474169875618</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>679784835806</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.644412191582</v>
+        <v>54.65166908563135</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>37.26285143864953</v>
+        <v>37.23186382740717</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.43024540219376</v>
+        <v>16.43242737368905</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.59343700459098</v>
+        <v>26.59696866953183</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.71984482992554</v>
+        <v>3.720338833223007</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.70755872693687</v>
+        <v>41.71314267405556</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.29755840198146</v>
+        <v>16.29974037347675</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01723159794552971</v>
+        <v>0.01722930985657728</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4664581501914824</v>
+        <v>0.4678735756817278</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2366425825778211</v>
+        <v>0.2376032362035492</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>80.22471910112355</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>95.49917259823697</v>
+        <v>94.9170541397247</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.801130421830948</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.159943307167411</v>
+        <v>-0.1547913088091943</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.143607066512573</v>
+        <v>0.1440316686486234</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3572,13 +3572,13 @@
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (E)</t>
+          <t>2026-10-28 (C)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.83302864107252</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.38855251754607</v>
+        <v>14.38685824656072</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.599649600719028</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1003906488692996</v>
+        <v>0.1005202365747582</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3832700059820655</v>
+        <v>-0.3832272011779682</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.58340611353712</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.34164127745184</v>
+        <v>18.3383736012402</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.213484537968363</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1222226954597119</v>
+        <v>0.1224226619608781</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.0435274464204678</v>
+        <v>0.04363496971789305</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>42.03584589614741</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.19651131973573</v>
+        <v>29.17749629238355</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.83281853154051</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4397557788944726</v>
+        <v>0.4406940703517588</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2175367740960465</v>
+        <v>0.2180036758153074</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.21864951768489</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.99997298650046</v>
+        <v>15.9974739938842</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.670165543077081</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.076167411795798</v>
+        <v>0.07633552173721547</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3302218211312649</v>
+        <v>-0.3301247057092656</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>21.57509484490069</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.266880505213346</v>
+        <v>6.257749525572894</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.09508456698496</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.442716807341805</v>
+        <v>2.447740238999979</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.74547407708723</v>
+        <v>1.749118834235528</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.80124223602485</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.44560144925267</v>
+        <v>27.43041106361941</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.016466858539234</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.907614991916958</v>
+        <v>1.909225168042202</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2329384472688285</v>
+        <v>0.2335029339006689</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.09038054968288</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.606783891268108</v>
+        <v>9.607513942267483</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.511669191158</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.860853014857077</v>
+        <v>2.860559638275073</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04828377508361636</v>
+        <v>-0.04839257199131664</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1159973877383</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.558861686113768</v>
+        <v>7.301073917627807</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003561938248463475</v>
+        <v>0.003559198896763882</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.491753285413805</v>
+        <v>6.270358231171368</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.698724861340043</v>
+        <v>4.538479331386828</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01691578859433369</v>
+        <v>0.01633889175787954</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.634501639024965</v>
+        <v>7.372915219799308</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.461500981164543</v>
+        <v>6.240105926922107</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07425100616006471</v>
+        <v>0.07687267543800835</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2121.120362242231</v>
+        <v>2050.325067634219</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2760.44775222109</v>
+        <v>2669.378811967969</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-88.94155844155844</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.4109911406423</v>
+        <v>137.7360387910847</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>108.0543764459125</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.949986569970455</v>
+        <v>3.959933882931465</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2172875796000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.93555117653877</v>
+        <v>27.52984815115336</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6535002167216367</v>
+        <v>0.6530416274140427</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.07436022855125</v>
+        <v>13.8699608061449</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.714817505368815</v>
+        <v>9.573730944087526</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5247819590387496</v>
+        <v>0.5171606442809255</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.51345021489235</v>
+        <v>18.23499550089752</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.58978081708063</v>
+        <v>13.38538139467429</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01789632973916031</v>
+        <v>0.01816006512479004</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.74757752442817</v>
+        <v>41.15634500999249</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.78236014646265</v>
+        <v>41.19358541720595</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.48031496062992</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-71.28081168363011</v>
+        <v>-71.85266173094175</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.981967405288661</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02228542655102905</v>
+        <v>0.02236612043703623</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.37598544572468</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.46528724316564</v>
+        <v>17.45912556618767</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.69889453213279</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1666561884745426</v>
+        <v>0.1670679249358267</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.0009199163737190208</v>
+        <v>0.00115466910533879</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>24.65824915824916</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.7949564442533</v>
+        <v>16.77977384653032</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.263583255144155</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4681936949402703</v>
+        <v>0.4695221392002211</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4703668248205155</v>
+        <v>0.4720290182378597</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-23 08:21 ET</t>
+          <t>2026-08-24 08:30 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-25)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.4269406392694</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.80452606027604</v>
+        <v>32.79796951000089</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.764030609117373</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.07994063301432419</v>
+        <v>0.08015652092325043</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.104293135341625</v>
+        <v>0.1045397828031971</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003415608687246247</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3452666595895402</v>
+        <v>0.3452666434899563</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3594787818193289</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16354277399.00305</v>
+        <v>16358243722.55025</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.07277777777778</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.01766044894412</v>
+        <v>24.00548996298323</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>10.90451927139366</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1272029528158294</v>
+        <v>0.1277744307458144</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2120066281068302</v>
+        <v>0.2126398612860827</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007469577886766125</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5558182531536007</v>
+        <v>0.5558182176773362</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4611181625229751</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15284874574.10936</v>
+        <v>15292718812.83844</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>205.28</v>
+        <v>205.65</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>4212260854205</v>
@@ -974,7 +974,7 @@
         <v>17.28202581926514</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.44621418287731</v>
+        <v>20.46428459953414</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.447348321820183</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1547566867543633</v>
+        <v>-0.1555030553250534</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2768957794110973</v>
+        <v>0.2775897690532323</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002442107682583463</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.8050426180681493</v>
+        <v>0.8050425756461549</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3952707227995144</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10022003706.33341</v>
+        <v>10022867833.36233</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.79920634920635</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.13002327028246</v>
+        <v>23.14138911176892</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.634376543162129</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1007701935203307</v>
+        <v>-0.1012118482278759</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1689944629859936</v>
+        <v>0.1694216826966213</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.862824995917596</v>
+        <v>0.8628249418251438</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4609101386527416</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11404895126.81194</v>
+        <v>11405920815.08113</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>31.78048780487805</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>18.5660344618559</v>
+        <v>18.54879074182914</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>19.92021050057004</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.711754218175743</v>
+        <v>0.7133455354159706</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.960414396856369</v>
+        <v>0.9623172680346763</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001343054489639294</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.286712617360347</v>
+        <v>1.286712621615805</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.3662849193753829</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>24855104374.87707</v>
+        <v>24860134313.70931</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>20.77369007803791</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>16.8846850428634</v>
+        <v>16.88162911490821</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.23924828415145</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2303273662080096</v>
+        <v>0.2305500811940362</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2578607128085628</v>
+        <v>0.258474317514571</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003756574004507889</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8062416636512205</v>
+        <v>0.8062416029613436</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.5002209555840639</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9667512114.210644</v>
+        <v>9672159357.838949</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>295.7203389830509</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.703674126801</v>
+        <v>170.5764472579555</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.30059702502437</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7323607151149294</v>
+        <v>0.7336528209890878</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1121748558489895</v>
+        <v>0.1125430930845046</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.558663640802493</v>
+        <v>1.558663650760562</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6178588313732408</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12740778315.8204</v>
+        <v>12744796851.95841</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>57.95799676898223</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.89742918515158</v>
+        <v>19.87337894527509</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>22.61749686344663</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.91283844911147</v>
+        <v>1.916363489499192</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.149142040376878</v>
+        <v>1.151677659972899</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.00707994202252202</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.612468539541932</v>
+        <v>1.612468527349244</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4339821034458192</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7533352469.863107</v>
+        <v>7534241392.944641</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.78955298844802</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.88436239017144</v>
+        <v>42.87315842205375</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.467352098696468</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1377003240610142</v>
+        <v>0.1379976373131142</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1113164502334958</v>
+        <v>0.111547161959394</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005703108914968088</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1727808459486644</v>
+        <v>-0.1727808829994832</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2219156320150146</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1832594415.463643</v>
+        <v>1832668727.565511</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.77089783281734</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.41034312465533</v>
+        <v>21.40696508629781</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.887566202592955</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1569594045549005</v>
+        <v>0.1571419737902371</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1362107780287476</v>
+        <v>0.1365389646179043</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1160527916210732</v>
+        <v>0.1160527756161532</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3746782167372559</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2977700329.011438</v>
+        <v>2978427789.392115</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.68091526276087</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.73513460607615</v>
+        <v>22.73510804249445</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.827608952291083</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422326728001076</v>
+        <v>-0.4422320211076706</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.0596525152222136</v>
+        <v>0.05969791915156364</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1699420110841808</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2145213897.062329</v>
+        <v>2145741843.267415</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.32201203783319</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.24473555190256</v>
+        <v>14.24427005296431</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.208483497797623</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07562628888443923</v>
+        <v>0.07566144006407627</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2908818131196602</v>
+        <v>-0.2908316668297156</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1947677221167146</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2529649556.137081</v>
+        <v>2531981661.725973</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2219,10 +2219,10 @@
         <v>0.1037000342715</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.002647193062528475</v>
+        <v>-0.002660198732493457</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>383.425</v>
+        <v>383.43</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>293.89</v>
@@ -2234,7 +2234,7 @@
         <v>32.49022939677145</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.7692686455522</v>
+        <v>25.76070440742857</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>16.04876649790955</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2608130189359994</v>
+        <v>0.2612321807241536</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1309918958432998</v>
+        <v>0.1312983238923597</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.2148866280122805</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2605407614.531381</v>
+        <v>2605505269.299316</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>32.94124107633169</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.28985054598067</v>
+        <v>27.27917696813261</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.99583316592082</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2070876321154265</v>
+        <v>0.2075599316949139</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1488596842542089</v>
+        <v>0.1492270971062362</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2316419571789821</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1679841708.64906</v>
+        <v>1679867082.72644</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.64208089511929</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.58069603716244</v>
+        <v>18.57429410468225</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8045064026956716</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3800387694752487</v>
+        <v>0.3805144222765044</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008733568802909764</v>
+        <v>0.008812033628442073</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2564368765951148</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2097988771.555392</v>
+        <v>2098039161.528625</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>21.11325611325611</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.94700026467298</v>
+        <v>14.95015977151913</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.883062823353459</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4125413621057457</v>
+        <v>0.4122428412757178</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.07869725028071062</v>
+        <v>0.07855805744294764</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2389167834326707</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2209600127.651132</v>
+        <v>2212414076.672363</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.56531791907515</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.11492321385358</v>
+        <v>22.10921933854546</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.719140024967068</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4273311109351492</v>
+        <v>0.4276993427824844</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08326088360216799</v>
+        <v>0.08346794937679891</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,7 +2801,7 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.0191913272780545</v>
+        <v>0.01933782595956636</v>
       </c>
       <c r="AI18" s="6" t="n">
         <v>-0.1849466073313465</v>
@@ -2810,7 +2810,7 @@
         <v>0.262629033740609</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1946552646.498362</v>
+        <v>1946869684.827118</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.44404332129964</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.59271941884648</v>
+        <v>34.58228268858645</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.151685066318765</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1113333663023588</v>
+        <v>0.1116687601997923</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04810485723448665</v>
+        <v>0.0482294133858796</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3292894789695507</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2748880331.059629</v>
+        <v>2756341710.318451</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.71703703703704</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.81911322558541</v>
+        <v>20.82314512018614</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>4.00398770653323</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04312978183663119</v>
+        <v>0.04292780517503814</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02361347493458577</v>
+        <v>0.02369345835535874</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.2003750898144018</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1279061283.468772</v>
+        <v>1279442062.324626</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         <v>0.2578999005085725</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1316475709.155613</v>
+        <v>1316923290.412598</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>115.9251269035533</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>35.24001170383563</v>
+        <v>35.17971469279065</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.03095017552354</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.289588206661567</v>
+        <v>2.295226465475279</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8363474169875618</v>
+        <v>0.8388594188396044</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.543023055968455</v>
+        <v>2.543020053155943</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7467117086309402</v>
+        <v>0.746708784786794</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12986529677.65714</v>
+        <v>12987564140.1944</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>670677408679</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.0566037735849</v>
+        <v>54.94920174165457</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.73304939560147</v>
+        <v>36.70252774689444</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.25350571062204</v>
+        <v>16.52188820522256</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.30737214438223</v>
+        <v>26.74176693210662</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.679830562830723</v>
+        <v>3.740592968419148</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.25525900916368</v>
+        <v>41.9420845065015</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.12081871040974</v>
+        <v>16.38920120501026</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01741897335612748</v>
+        <v>0.01713601855915579</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4716067591180659</v>
+        <v>0.497150335818602</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2407507824085273</v>
+        <v>0.2620500457316022</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004470930332791228</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.713284066388405</v>
+        <v>1.713284032278255</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5121887872683704</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2916647609.47404</v>
+        <v>2924065667.676188</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>78.82397003745315</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>93.25977224204698</v>
+        <v>92.69474824765997</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.769682112878344</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1547913088091943</v>
+        <v>-0.1496393104509779</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1440316686486234</v>
+        <v>0.1444562607764766</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,17 +3568,17 @@
         <v>0.3636614867046326</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1285113620.764015</v>
+        <v>1285554871.214091</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.78732480195003</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.34532894287001</v>
+        <v>14.34363996039734</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.592145416281574</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1005202365747582</v>
+        <v>0.100649824280217</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.383227201177968</v>
+        <v>-0.3831843963738708</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3973208386843363</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2155130730.45638</v>
+        <v>2155164927.697347</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.17816593886463</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.97733298044185</v>
+        <v>17.97413077848612</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.150218379379713</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1224226619608781</v>
+        <v>0.1226226284620446</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04363496971789305</v>
+        <v>0.0437424930153183</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.7973436266697537</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>2440193148.320086</v>
+        <v>2441816304.752146</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>41.80636515912899</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>29.01821144368393</v>
+        <v>28.9993248394257</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.75184368599826</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.440694070351759</v>
+        <v>0.4416323618090454</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2180036758153074</v>
+        <v>0.2184705775345683</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3742151485185202</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3159089241.629211</v>
+        <v>3159207907.80599</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.20900321543408</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.98851182357951</v>
+        <v>15.98601501102178</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.668669652016534</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07633552173721525</v>
+        <v>0.0765036316786325</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3301247057092656</v>
+        <v>-0.3300275902872664</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.3108882899350973</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1162875320.801541</v>
+        <v>1163038776.128693</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>20.3175630439634</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>5.893008647848869</v>
+        <v>5.884434899678653</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.39010720362452</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.447740238999979</v>
+        <v>2.452763670658152</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.749118834235528</v>
+        <v>1.752763591383827</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005821425040914733</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.896428330581974</v>
+        <v>2.89642834052833</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.978349923575576</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>35995964735.77262</v>
+        <v>36000401774.56869</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>79.53416149068325</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.33860629433737</v>
+        <v>27.32348349763202</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.98629032717893</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.909225168042202</v>
+        <v>1.910835344167447</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2335029339006689</v>
+        <v>0.2340674205325095</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5957962668149512</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2516156231.112478</v>
+        <v>2516391207.986196</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.95824524312896</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.573286959929515</v>
+        <v>9.574014520676997</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.502721313740266</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.860559638275073</v>
+        <v>2.86026626169307</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04839257199131664</v>
+        <v>-0.04850136889901702</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2215989677204972</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1022079852.00668</v>
+        <v>1022118855.426489</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1102901544147</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.301073917627807</v>
+        <v>7.331658907109192</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003384081345022976</v>
+        <v>0.003379852481997177</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.270358231171368</v>
+        <v>6.296625440996742</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.538479331386828</v>
+        <v>4.557491512906701</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01633889175787954</v>
+        <v>0.01640733714525545</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.372915219799308</v>
+        <v>7.40395089665659</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.240105926922107</v>
+        <v>6.26637313674748</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07687267543800835</v>
+        <v>0.07655199085632416</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2156.475891755858</v>
+        <v>2168.224528632938</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2807.564083565228</v>
+        <v>2823.686205023801</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645611932511996</v>
@@ -4574,7 +4574,7 @@
         <v>1.325879570870433</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>5702187004.299691</v>
+        <v>5702860734.978333</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.812333719244707</v>
+        <v>1.812333698768389</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.4728929160153765</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>6025605517.159327</v>
+        <v>6027536594.058533</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-87.66233766233766</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>135.755021076122</v>
+        <v>135.0962329330482</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>106.500261518552</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.959933882931465</v>
+        <v>3.969881195892477</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.8423069447382688</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12959014536.22428</v>
+        <v>12960689501.80133</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>0.1205254342477912</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34300252914.39732</v>
+        <v>34316027158.87146</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -4915,37 +4915,37 @@
         <v>2127079177600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.52984815115336</v>
+        <v>27.81963602642865</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6392777950472543</v>
+        <v>0.6388142573358058</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.8699608061449</v>
+        <v>14.01596039357801</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.573730944087526</v>
+        <v>9.674507059288446</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5171606442809255</v>
+        <v>0.5226044405365141</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.23499550089752</v>
+        <v>18.43389172517954</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.38538139467429</v>
+        <v>13.53138098210739</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01816006512479004</v>
+        <v>0.01797089777974014</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.06398308284491</v>
+        <v>42.54886527181045</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.10202528659521</v>
+        <v>42.58932735513012</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.4474638900881592</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5390302490.202454</v>
+        <v>5390593182.098287</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.59842519685039</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-72.2301713372339</v>
+        <v>-72.81432398126468</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.992380544012183</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02236612043703623</v>
+        <v>0.02244681432304363</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.316895006748855</v>
+        <v>0.3168949925639272</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2114077991180071</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>615110254.0706714</v>
+        <v>615292378.7182173</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.45664038811401</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.52823460488716</v>
+        <v>17.52205290123321</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.709577656322482</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1670679249358267</v>
+        <v>0.167479661397111</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.00115466910533879</v>
+        <v>0.001389421836958782</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.2613434681062255</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>952507180.330892</v>
+        <v>952523821.9435629</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>23.97979797979798</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.31809235133323</v>
+        <v>16.30335416081867</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.091245981175213</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4695221392002209</v>
+        <v>0.4708505834601724</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4720290182378597</v>
+        <v>0.4736912116552041</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5372,7 +5372,7 @@
         <v>0.563580571975006</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4268709683.435678</v>
+        <v>4269134931.884664</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24 17:56 ET</t>
+          <t>2026-08-25 08:30 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-26)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -455,7 +455,7 @@
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
     <col width="23" customWidth="1" min="19" max="19"/>
-    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
@@ -474,7 +474,7 @@
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
-    <col width="28" customWidth="1" min="39" max="39"/>
+    <col width="19" customWidth="1" min="39" max="39"/>
     <col width="21" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
@@ -711,7 +711,7 @@
         <v>344.57</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>224.69</v>
+        <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>4551611624400</v>
@@ -720,7 +720,7 @@
         <v>35.37671232876712</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>32.75146855432518</v>
+        <v>32.74492391656634</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.75018716815581</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08015652092325043</v>
+        <v>0.08037240883217622</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1045397828031971</v>
+        <v>0.1047864302647692</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003420458212326557</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3421738945909705</v>
+        <v>0.3421738830354458</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3211721708300478</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>16242200915.6821</v>
+        <v>16244017177.56632</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.31722222222222</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.22223937472755</v>
+        <v>24.20997143888356</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.00297792152218</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1277744307458144</v>
+        <v>0.1283459086757992</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2123381108156632</v>
+        <v>0.2129657895236123</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007402737385857518</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5574877895979143</v>
+        <v>0.5574877946576324</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.4489091304400483</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15249209466.42283</v>
+        <v>15255024477.95278</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.227408142999</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.40078701554449</v>
+        <v>20.41880806909727</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.417491161693958</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1555517868074168</v>
+        <v>-0.1562970725469659</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2815789985431982</v>
+        <v>0.2822781350065597</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002449850126815771</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7968553478675923</v>
+        <v>0.7968553227354308</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3951804914384784</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>10042652631.78848</v>
+        <v>10042873876.6097</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.71904761904762</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.05220376814742</v>
+        <v>23.06353693897489</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.620369902537129</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1012118482278759</v>
+        <v>-0.1016535029354209</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1694216826966211</v>
+        <v>0.1697164229855448</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8547133194715718</v>
+        <v>0.8547132946930575</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4532335293977366</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11379433240.22162</v>
+        <v>11379856679.53766</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>32.47713414634146</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>18.99422502965892</v>
+        <v>18.97671371951496</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>20.35687282783215</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.7098425492816571</v>
+        <v>0.7114203558302703</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9599058400458194</v>
+        <v>0.9617995902769882</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6151406306604901</v>
@@ -1292,13 +1292,13 @@
         <v>0.001314245482281155</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.289593488552541</v>
+        <v>1.289593500673863</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.36693837279253</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>24840066479.21801</v>
+        <v>24849164147.54999</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.18357487922705</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.21471982568321</v>
+        <v>17.21403659920117</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.362354628426099</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.230550081194036</v>
+        <v>0.2305989218246514</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.258474317514571</v>
+        <v>0.2590552739452594</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.00368388737830015</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.8046018773285951</v>
+        <v>0.8046018981760402</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.497767322915995</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9488810235.466211</v>
+        <v>9489400275.206909</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>296.8220338983051</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>171.2119233474679</v>
+        <v>171.0844127109872</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.35014789516402</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7336528209890878</v>
+        <v>0.7349449268632462</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1125430930845048</v>
+        <v>0.11291133032002</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.543041201340273</v>
+        <v>1.54304117700517</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.6180025622027738</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12783799937.1156</v>
+        <v>12784390575.3656</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>57.63166397415186</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.76148178430548</v>
+        <v>19.73762470185254</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>22.49014893261777</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.916363489499192</v>
+        <v>1.919888529886915</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.151677659972899</v>
+        <v>1.154213279568919</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.007120031395414027</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.613746921811361</v>
+        <v>1.61374687828798</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4337746326063504</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7487037875.759746</v>
+        <v>7487675132.295634</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.21747865394274</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.36789077795346</v>
+        <v>42.35681962079933</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.450146889303682</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1380665350240464</v>
+        <v>0.1383640010182807</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1116784686300123</v>
+        <v>0.1119094394037641</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.00577077322111228</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1708921207903663</v>
+        <v>-0.1708921384360023</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2183015951116987</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1800978338.9528</v>
+        <v>1802163311.308187</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>25.45820433436533</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>22.0009341213132</v>
+        <v>21.99746344945764</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7.078672276460219</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1571419737902371</v>
+        <v>0.1573245430255736</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.136538964617904</v>
+        <v>0.1368671512070605</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1207679456442953</v>
+        <v>0.1207679948037887</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3773630646905634</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2977449736.551013</v>
+        <v>2977515981.041718</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -1978,29 +1978,75 @@
       <c r="K12" s="5" t="n">
         <v>1087744405030</v>
       </c>
-      <c r="L12" s="6" t="inlineStr"/>
-      <c r="M12" s="6" t="inlineStr"/>
-      <c r="N12" s="6" t="inlineStr"/>
-      <c r="O12" s="6" t="inlineStr"/>
-      <c r="P12" s="6" t="inlineStr"/>
-      <c r="Q12" s="6" t="inlineStr"/>
-      <c r="R12" s="6" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="inlineStr"/>
-      <c r="W12" s="4" t="inlineStr"/>
-      <c r="X12" s="4" t="inlineStr"/>
-      <c r="Y12" s="4" t="inlineStr"/>
-      <c r="Z12" s="4" t="inlineStr"/>
-      <c r="AA12" s="5" t="inlineStr"/>
-      <c r="AB12" s="6" t="inlineStr"/>
-      <c r="AC12" s="6" t="inlineStr"/>
-      <c r="AD12" s="6" t="inlineStr"/>
-      <c r="AE12" s="6" t="inlineStr"/>
-      <c r="AF12" s="6" t="inlineStr"/>
-      <c r="AG12" s="6" t="inlineStr"/>
-      <c r="AH12" s="4" t="inlineStr"/>
+      <c r="L12" s="6" t="n">
+        <v>12.68091526276087</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>22.73508147897482</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>2.827608952291083</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>1.448511682549585</v>
+      </c>
+      <c r="P12" s="6" t="n">
+        <v>0.3489644322780516</v>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>15.37634165028622</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>3.058344589315469</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0.02226166357466316</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>2.961503151310829e-05</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <v>-0.4422313694152336</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0.05974332308091368</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>0.06790433791924602</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>0.1185897214314059</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <v>0.2351704112694216</v>
+      </c>
+      <c r="Z12" s="4" t="n">
+        <v>0.1625113403884197</v>
+      </c>
+      <c r="AA12" s="5" t="n">
+        <v>25042000000</v>
+      </c>
+      <c r="AB12" s="6" t="n">
+        <v>7.291819852941177</v>
+      </c>
+      <c r="AC12" s="6" t="n">
+        <v>6.884727328431373</v>
+      </c>
+      <c r="AD12" s="6" t="n">
+        <v>0.1724526345115886</v>
+      </c>
+      <c r="AE12" s="6" t="n">
+        <v>0.1024249626505557</v>
+      </c>
+      <c r="AF12" s="6" t="n">
+        <v>1.160062210837232</v>
+      </c>
+      <c r="AG12" s="6" t="n">
+        <v>11.61570329453541</v>
+      </c>
+      <c r="AH12" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AI12" s="6" t="n">
         <v>0.06771254785976095</v>
       </c>
@@ -2008,17 +2054,17 @@
         <v>0.165902004607791</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2129360039.636379</v>
-      </c>
-      <c r="AL12" s="7" t="inlineStr"/>
-      <c r="AM12" s="2" t="inlineStr">
-        <is>
-          <t>pe_trailing,ps,pb,current_ratio,quick_ratio,debt_equity,debt_assets,gross_margin,operating_margin,peg,roa,roe,ev_ebitda,ev_sales,fcf_yield,net_debt_ebitda,free_cash_flow,rev_growth_ttm,interest_coverage,fwd_eps_growth,fwd_rev_growth,pe_forward,dividend_yield</t>
-        </is>
-      </c>
+        <v>2129442630.442912</v>
+      </c>
+      <c r="AL12" s="7" t="inlineStr">
+        <is>
+          <t>2026-11-07 (E)</t>
+        </is>
+      </c>
+      <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2108,7 @@
         <v>15.33490971625108</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.25626051570426</v>
+        <v>14.25579465536928</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.211184317263207</v>
@@ -2086,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07566144006407627</v>
+        <v>0.07569659124371309</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2908316668297156</v>
+        <v>-0.2907815205397711</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2134,7 +2180,7 @@
         <v>0.1945862118968186</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2415197575.807037</v>
+        <v>2416920091.277161</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2144,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2234,7 @@
         <v>32.63721325403568</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.8772442955718</v>
+        <v>25.86849525844681</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>16.12137015900917</v>
@@ -2212,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2612321807241533</v>
+        <v>0.2616587446607928</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1312983239104033</v>
+        <v>0.1316047519595864</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2260,7 +2306,7 @@
         <v>0.2138359840418237</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2613538757.937927</v>
+        <v>2613581282.237549</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2270,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2360,7 @@
         <v>32.91433278418451</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.25689377419672</v>
+        <v>27.24623725433375</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.98358371062908</v>
@@ -2338,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2075599316949137</v>
+        <v>0.208032231274401</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1492270971062362</v>
+        <v>0.1495945099867673</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2386,7 +2432,7 @@
         <v>0.2286798480713376</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1687590956.949975</v>
+        <v>1687605261.913859</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2396,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2486,7 @@
         <v>25.50254002958009</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.441573346157</v>
+        <v>18.43526063321433</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8001283836011454</v>
@@ -2464,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3828830952156539</v>
+        <v>0.3833566303713019</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008812031257462438</v>
+        <v>0.008890496076299659</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2512,7 +2558,7 @@
         <v>0.2494363637874038</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>2060318913.596488</v>
+        <v>2060346265.086568</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2522,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2612,7 @@
         <v>20.67310167310167</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.65337975468682</v>
+        <v>14.65667793839407</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.843806042762976</v>
@@ -2590,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4108077466899385</v>
+        <v>0.4104902734436979</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08554458332905623</v>
+        <v>0.08538314513109402</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2638,7 +2684,7 @@
         <v>0.2468226127661523</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2226987549.683435</v>
+        <v>2228317632.814382</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2648,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2738,7 @@
         <v>31.57687861271676</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.11731676725134</v>
+        <v>22.11161374552043</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.721600887847318</v>
@@ -2716,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4276993427824844</v>
+        <v>0.4280675746298204</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08346801202702481</v>
+        <v>0.0836750773004542</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2764,7 +2810,7 @@
         <v>0.2606558308780918</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1909937553.128147</v>
+        <v>1915329364.331309</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2774,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2855,7 @@
         <v>135.16</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>95.42</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>838622470400</v>
@@ -2818,7 +2864,7 @@
         <v>38.04332129963899</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.22181378273303</v>
+        <v>34.20692523108575</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.139680460969776</v>
@@ -2842,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1116687601997923</v>
+        <v>0.1121526136195043</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0482294133858796</v>
+        <v>0.04808878360281188</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2890,7 +2936,7 @@
         <v>0.3240221700961246</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2794147059.138859</v>
+        <v>2795722251.236471</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2900,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2990,7 @@
         <v>21.54074074074074</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.65410533102575</v>
+        <v>20.65075372994244</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.971483815608052</v>
@@ -2968,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04292780517503814</v>
+        <v>0.0430970715372907</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02369345835535852</v>
+        <v>0.02377335448214923</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3016,7 +3062,7 @@
         <v>0.1930887718374205</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1284887000.153996</v>
+        <v>1286332751.06664</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3026,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3116,7 @@
         <v>23.59497206703911</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.5372329923533</v>
+        <v>22.53621081108482</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.991452049699721</v>
@@ -3094,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04693296089385468</v>
+        <v>0.04698044692737424</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01378773042866599</v>
+        <v>0.01393283308507121</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3142,7 +3188,7 @@
         <v>0.2574081715354979</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1312054781.044804</v>
+        <v>1313791855.937907</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3152,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3242,7 @@
         <v>121.6192893401015</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.90771806257633</v>
+        <v>36.89498227485868</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.91661803655732</v>
@@ -3220,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.295226465475279</v>
+        <v>2.296363945483624</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8388594188396044</v>
+        <v>0.8398442459572872</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3262,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.553820183076856</v>
+        <v>2.553820211471331</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7542243169739438</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12902998113.78429</v>
+        <v>12903624354.11672</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3278,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3319,37 +3365,37 @@
         <v>672230643183</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.46298984034833</v>
+        <v>54.15820029027576</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.75421960770574</v>
+        <v>36.72383382638135</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.37569611466987</v>
+        <v>16.28405331164107</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.50514538106976</v>
+        <v>26.35681545355411</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.707494747488868</v>
+        <v>3.686746608995259</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.56796004860734</v>
+        <v>41.33343426904271</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.24300911445757</v>
+        <v>16.15136631142877</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01728899833841955</v>
+        <v>0.01738629673452345</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4818159770947723</v>
+        <v>0.4747425485671939</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2489958815401292</v>
+        <v>0.242803397145066</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3386,13 +3432,13 @@
         <v>0.004460599944959178</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.71247833918571</v>
+        <v>1.712478303369909</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.5003244986727934</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2820424004.191716</v>
+        <v>2821401664.029541</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3496,7 @@
         <v>79.05617977528087</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>92.9678202989455</v>
+        <v>92.40795711477834</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.774895468907921</v>
@@ -3474,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1496393104509779</v>
+        <v>-0.1444873120927612</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1444562607764768</v>
+        <v>0.1448808629282963</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3522,17 +3568,17 @@
         <v>0.363135549052766</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1291896100.455359</v>
+        <v>1291941081.60375</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 (C)</t>
+          <t>2026-10-28 (E)</t>
         </is>
       </c>
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3622,7 @@
         <v>16.13162705667276</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.65645721355767</v>
+        <v>14.65473180278074</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.648676939043727</v>
@@ -3600,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.100649824280217</v>
+        <v>0.1007794119856753</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3831843963738708</v>
+        <v>-0.3831415915697736</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3648,7 +3694,7 @@
         <v>0.400234253168411</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2092337016.296204</v>
+        <v>2099190828.903809</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3658,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3748,7 @@
         <v>20.45327510917031</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.21919012730984</v>
+        <v>18.21594542265196</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.193168465490543</v>
@@ -3726,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1226226284620446</v>
+        <v>0.1228225949632114</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.0437424930153183</v>
+        <v>0.04385001631274354</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3774,7 +3820,7 @@
         <v>0.7974599560643318</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1977303636.152726</v>
+        <v>1977433400.833079</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3784,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3874,7 @@
         <v>41.32294807370184</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>28.66399865070133</v>
+        <v>28.64535472154284</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.58126455881947</v>
@@ -3852,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4416323618090452</v>
+        <v>0.4425706532663316</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2184705775345683</v>
+        <v>0.2189374792538294</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3900,7 +3946,7 @@
         <v>0.3752251041830481</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3145397015.681189</v>
+        <v>3145719288.804118</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3910,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -3954,7 +4000,7 @@
         <v>17.42524115755627</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.18688562191326</v>
+        <v>16.18435822541121</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.702202543290471</v>
@@ -3978,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07650363167863272</v>
+        <v>0.07667174162005019</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3300275902872665</v>
+        <v>-0.3299304748652673</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4026,7 +4072,7 @@
         <v>0.312221073298894</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1116034144.416576</v>
+        <v>1116044845.62912</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4036,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4126,7 @@
         <v>20.82057576433832</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.030118985922249</v>
+        <v>6.021358501334825</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.6720981489687</v>
@@ -4104,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.452763670658151</v>
+        <v>2.457787102316324</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.752763591383827</v>
+        <v>1.756408348532125</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4146,13 +4192,13 @@
         <v>0.0005680782876191088</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.909621645702002</v>
+        <v>2.909621616191935</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.9068030268131854</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>35585303861.14005</v>
+        <v>35587994017.85258</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4162,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4252,7 @@
         <v>78.88198757763976</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>27.09943306676506</v>
+        <v>27.08445086029021</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.912603448275862</v>
@@ -4230,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.910835344167447</v>
+        <v>1.912445520292692</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2340674205325095</v>
+        <v>0.2346319071643501</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4278,7 +4324,7 @@
         <v>0.5816035306760755</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2487190598.601501</v>
+        <v>2487328059.168167</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4288,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4332,7 +4378,7 @@
         <v>37.75105708245243</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.779392022014367</v>
+        <v>9.780135303040137</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.556408578246672</v>
@@ -4356,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.860266261693071</v>
+        <v>2.859972885111067</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04850136889901702</v>
+        <v>-0.04861016580671718</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4404,7 +4450,7 @@
         <v>0.2203878412950987</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1019437868.272913</v>
+        <v>1019475953.03484</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4414,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4455,37 +4501,37 @@
         <v>1132431507612</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.331658907109192</v>
+        <v>7.375351749225457</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00347034734152674</v>
+        <v>0.003460827438346635</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.296625440996742</v>
+        <v>6.334150026461562</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.562917656148448</v>
+        <v>4.59011025243062</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01640733714525545</v>
+        <v>0.01650511627007819</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.40395089665659</v>
+        <v>7.448287577881277</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.26637313674748</v>
+        <v>6.3038977222123</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07655199085632416</v>
+        <v>0.07609848380148812</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2111.658528262394</v>
+        <v>2130.094913171671</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2750.027992695942</v>
+        <v>2773.595844160914</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4528,7 +4574,7 @@
         <v>1.306845992079737</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>5298636738.270755</v>
+        <v>5298852491.958771</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4542,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4606,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.8157095354047</v>
+        <v>1.815709524379658</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.4688046868911466</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5984854403.754008</v>
+        <v>5987928755.37852</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4622,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4712,7 @@
         <v>-89.57792207792207</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.0483358008444</v>
+        <v>137.3816539794276</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>108.8274894554449</v>
@@ -4691,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.969881195892477</v>
+        <v>3.979828508853489</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4734,7 +4780,7 @@
         <v>0.8442994651428137</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12992167387.11419</v>
+        <v>12992749434.93797</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4748,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4864,7 @@
         <v>0.1206442607872523</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>34126757115.57496</v>
+        <v>34135881988.28267</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4828,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -4869,37 +4915,37 @@
         <v>2164888616800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.81963602642865</v>
+        <v>27.99350875159383</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6501693630023864</v>
+        <v>0.6496884234388629</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.01596039357801</v>
+        <v>14.10356014603787</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.674507059288446</v>
+        <v>9.734972728409</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5226044405365141</v>
+        <v>0.5258707182898673</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.43389172517954</v>
+        <v>18.55322945974876</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.53138098210739</v>
+        <v>13.61898073456725</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01797089777974014</v>
+        <v>0.01785927729663617</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.78829118917827</v>
+        <v>42.08759051519114</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.82804660857661</v>
+        <v>42.12893799194023</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4942,7 +4988,7 @@
         <v>0.4489463308487254</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>5288446585.206067</v>
+        <v>5288556614.483032</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -4956,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5046,7 @@
         <v>-22.75590551181102</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-73.32174087312018</v>
+        <v>-73.91955620992736</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>2.006264729004569</v>
@@ -5025,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02124113161358587</v>
+        <v>0.02131770779249686</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5064,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3052159745685355</v>
+        <v>0.3052159742417161</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.210509806852791</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>618868633.5266134</v>
+        <v>618868937.9399427</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5084,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5174,7 @@
         <v>20.37295330503336</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.45037106740965</v>
+        <v>17.44421899364272</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.698492910922651</v>
@@ -5152,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.167479661397111</v>
+        <v>0.1678913978583949</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.001389421836958782</v>
+        <v>0.001624174568578773</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5200,7 +5246,7 @@
         <v>0.2615031583955741</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>932297518.479421</v>
+        <v>933319243.2515463</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5210,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>
@@ -5254,7 +5300,7 @@
         <v>24.36195286195286</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.56317312982358</v>
+        <v>16.54822708599563</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.188319334006354</v>
@@ -5278,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4708505834601726</v>
+        <v>0.4721790277201234</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4736912116552041</v>
+        <v>0.4753534050725483</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5326,7 +5372,7 @@
         <v>0.5601111765225609</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>4108553110.904281</v>
+        <v>4108689286.631114</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5336,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 17:55 ET</t>
+          <t>2026-08-26 08:33 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-27)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>35.78196347031964</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.12002711083485</v>
+        <v>33.11341014726224</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>9.86187856682297</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08037240883217645</v>
+        <v>0.08058829674110246</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1047864302647692</v>
+        <v>0.1050330777263413</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.57611111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.43941250557979</v>
+        <v>24.42704084310524</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.10725458279467</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1283459086757992</v>
+        <v>0.128917386605784</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2129657895236123</v>
+        <v>0.2135934682315617</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.9811320754717</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.12690903744313</v>
+        <v>20.14470387972763</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.282862512390466</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1562970725469658</v>
+        <v>-0.157042358286515</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.28227813500656</v>
+        <v>0.2829772877038739</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.65714285714285</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.99462726758746</v>
+        <v>23.00593769259232</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.609552892945545</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1016535029354207</v>
+        <v>-0.1020951576429658</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.169716422985545</v>
+        <v>0.1701438734137755</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>26.37232704402515</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>18.6670272289754</v>
+        <v>18.64981599348954</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>16.76136786271863</v>
@@ -1238,10 +1238,10 @@
         <v>0.2116962306935352</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>21.80060881510868</v>
+        <v>21.80278712869168</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>16.81387488488921</v>
+        <v>16.81555492476128</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>0.02501016674325389</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.4127759455500988</v>
+        <v>0.4140797449814766</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.6415585754605029</v>
+        <v>0.6431435833864554</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1277,13 +1277,13 @@
         <v>3.85497105929938</v>
       </c>
       <c r="AD6" s="6" t="n">
-        <v>0.1674833176117109</v>
+        <v>0.1697061803444782</v>
       </c>
       <c r="AE6" s="6" t="n">
-        <v>0.1197450916720787</v>
+        <v>0.1213343657890793</v>
       </c>
       <c r="AF6" s="6" t="n">
-        <v>0.06807978875921718</v>
+        <v>0.07025810234222205</v>
       </c>
       <c r="AG6" s="6" t="n">
         <v>547.1389961389962</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.40988480118915</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.39793885845761</v>
+        <v>17.39479805614872</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.430325402369353</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2305989218246516</v>
+        <v>0.230821118594198</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2590552739452592</v>
+        <v>0.2596687999278604</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>293.0677966101695</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>168.9205184973978</v>
+        <v>168.7948080154182</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.18129377617039</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7349449268632462</v>
+        <v>0.7362370327374046</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1129113303200198</v>
+        <v>0.1132795675555351</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>57.44588045234249</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.68512729609787</v>
+        <v>19.66141474818179</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>22.41764887298748</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.918237692256623</v>
+        <v>1.921757217783876</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.153031796835075</v>
+        <v>1.155563438374752</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>48.02209944751381</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>42.18518804578979</v>
+        <v>42.17416751047921</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.444270834471554</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1383640010182807</v>
+        <v>0.1386614670125152</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1119094394037641</v>
+        <v>0.1121404101775159</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>25.21981424148607</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.79147966183655</v>
+        <v>21.78804257385966</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7.012387737332411</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1573245430255736</v>
+        <v>0.1575071122609102</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1368671512070605</v>
+        <v>0.137195337796217</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.69575056575308</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.76167907191699</v>
+        <v>22.76165247738306</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.830916949756555</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422313694152336</v>
+        <v>-0.4422307177227965</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05974332308091368</v>
+        <v>0.05978872701026372</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.32674118658642</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.24820094378633</v>
+        <v>14.24773536203288</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.209473798268337</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07569659124371309</v>
+        <v>0.07573174242335035</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2907815205397711</v>
+        <v>-0.2907313742498265</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>32.61682242990654</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.85233334127592</v>
+        <v>25.84374711162488</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>16.11129797480219</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.261658744660793</v>
+        <v>0.2620779134321061</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1316047519595864</v>
+        <v>0.1319111800087693</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>32.86490939044481</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.20532494052275</v>
+        <v>27.19469273915222</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.96108471111364</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2080322312744012</v>
+        <v>0.2085045308538889</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1495945099867673</v>
+        <v>0.1499619228387943</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.78676612436499</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.64072181982723</v>
+        <v>18.63434312009353</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8090458234150654</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3833566303713019</v>
+        <v>0.3838301655269494</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008890496076299659</v>
+        <v>0.008968960895136879</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.36036036036036</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.43495268538842</v>
+        <v>14.43820243697044</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.815913067080264</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4104902734436979</v>
+        <v>0.4101728001974576</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08538314513109402</v>
+        <v>0.08522170693313225</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.21387283236994</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.85742004572936</v>
+        <v>21.85178549209739</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.644329793217535</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4280675746298204</v>
+        <v>0.4284358064771556</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.0836750773004542</v>
+        <v>0.08388214257388316</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.66787003610109</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.86933553436598</v>
+        <v>33.85915317399166</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.128432902804958</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1121526136195043</v>
+        <v>0.1124870678997083</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.0480887836028121</v>
+        <v>0.04821286396859659</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.48592592592593</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.598203668869</v>
+        <v>20.59486168142312</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.961377563804118</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.0430970715372907</v>
+        <v>0.04326633789954348</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02377335448214923</v>
+        <v>0.02385325060893995</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>122.0634517766497</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>37.02972541727072</v>
+        <v>36.96671692666353</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.98570289311222</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.296363945483624</v>
+        <v>2.301982483832835</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8398442459572872</v>
+        <v>0.8423499739938611</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.33962264150943</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.75499568886131</v>
+        <v>36.7246343665155</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.33860259916496</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4784282142625087</v>
+        <v>0.4796504738262226</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.245909402225873</v>
+        <v>0.2467086273933092</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>79.43445692883893</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>92.85012139697432</v>
+        <v>92.29431414633284</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.783388194052875</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1444873120927611</v>
+        <v>-0.1393353137345446</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1448808629282963</v>
+        <v>0.1453054650801158</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.8510054844607</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.39980191477906</v>
+        <v>14.39810691792671</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.602601246597759</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1007794119856753</v>
+        <v>0.1009089996911339</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3831415915697737</v>
+        <v>-0.3830987867656764</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.07598253275109</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.87992388362017</v>
+        <v>17.87674016679842</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.134265490252833</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1228225949632114</v>
+        <v>0.1230225614643776</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04385001631274354</v>
+        <v>0.04395753961016879</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.86700167504188</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.63608256189967</v>
+        <v>27.61811890446929</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>14.06751758257621</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4425706532663316</v>
+        <v>0.443508944723618</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2189374792538294</v>
+        <v>0.2194043809730903</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.20498392282958</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.97978590665111</v>
+        <v>15.97729123590807</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.668046364074639</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07667174162005019</v>
+        <v>0.07683985156146766</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3299304748652672</v>
+        <v>-0.3298333594432679</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>20.94175407275162</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.056403160842602</v>
+        <v>6.047617253404043</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>11.74003119392073</v>
@@ -4150,10 +4150,10 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.457787323035159</v>
+        <v>2.462810755916152</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.756408348532125</v>
+        <v>1.760053105680423</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4202,13 +4202,13 @@
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23 (E)</t>
+          <t>2026-09-30 (C)</t>
         </is>
       </c>
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>78.13664596273293</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>26.82853478916935</v>
+        <v>26.81371054739322</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>8.828389872386641</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.912445520292692</v>
+        <v>1.914055696417936</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2346319071643501</v>
+        <v>0.2351963937961905</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.39429175475687</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.687708403081411</v>
+        <v>9.688444771676902</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.532249309218789</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.859972885111066</v>
+        <v>2.859679508529062</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04861016580671729</v>
+        <v>-0.04871896271441756</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4501,37 +4501,37 @@
         <v>1121712698758</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.375351749225457</v>
+        <v>7.604739170335846</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.00342806965340397</v>
+        <v>0.003425427786260174</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.334150026461562</v>
+        <v>6.531154100151865</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.59011025243062</v>
+        <v>4.732871382912022</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01650511627007819</v>
+        <v>0.01701845667539757</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.448287577881277</v>
+        <v>7.681055154310886</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.3038977222123</v>
+        <v>6.500901795902603</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07609848380148812</v>
+        <v>0.07380306846131109</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2150.459128580411</v>
+        <v>2219.084510565197</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2800.109195158539</v>
+        <v>2890.598176090773</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-90.66883116883116</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.0547324766036</v>
+        <v>138.3864179428695</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>110.1528260431976</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.979828508853489</v>
+        <v>3.989775821814501</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.99350875159383</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6501242365687899</v>
+        <v>0.6496689764985476</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.10356014603787</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.05870659327716</v>
+        <v>42.08888028249017</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.10002635259588</v>
+        <v>42.1332201781286</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.63779527559055</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-73.53589069326684</v>
+        <v>-74.1403806590933</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.995851590281047</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02131770779249686</v>
+        <v>0.02139428397140786</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.38508186779867</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.45460400271767</v>
+        <v>17.44845260529855</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.700099395763206</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1678913978583949</v>
+        <v>0.1683031343196792</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.001624174568578773</v>
+        <v>0.001858927300198543</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.05723905723906</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.02051081113668</v>
+        <v>17.00516592804756</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.364932967130853</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4721790277201234</v>
+        <v>0.4735074719800745</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4753534050725483</v>
+        <v>0.4770155984898927</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26 17:01 ET</t>
+          <t>2026-08-26 21:00 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-28)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -446,7 +446,7 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>314.58</v>
+        <v>319.7</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1607689334871993</v>
+        <v>0.1796612246037816</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.08703601590388022</v>
+        <v>-0.07217691615636879</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4620348450480</v>
+        <v>4695547713200</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>35.91095890410959</v>
+        <v>36.49543378995434</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.23278533777557</v>
+        <v>33.76692495113887</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>9.897431040201532</v>
+        <v>10.05851835320882</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>42.98708490234375</v>
+        <v>43.68672847377233</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.097279299847792</v>
+        <v>1.115138254693048</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>27.68842188953385</v>
+        <v>28.13474539843073</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>9.993319631809058</v>
+        <v>10.15440694481634</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02958283373320041</v>
+        <v>0.02910906423456423</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08058829674110224</v>
+        <v>0.08080418465002825</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1050330777263413</v>
+        <v>0.1052797251879132</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003369572127916587</v>
+        <v>0.003315608382858931</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3403660487563715</v>
+        <v>0.3366059664559604</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3132692946696073</v>
+        <v>0.3093319618130679</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15572991244.22676</v>
+        <v>15279100169.37729</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>505.06</v>
+        <v>513.53</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.06791558631704708</v>
+        <v>0.08582483475506497</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.08787835006862676</v>
+        <v>-0.07258181030123534</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3750348283000</v>
+        <v>3813242691500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.05888888888889</v>
+        <v>28.52944444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.85468752788994</v>
+        <v>25.25872130325989</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.30171041679851</v>
+        <v>11.49124331829592</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.481466996091656</v>
+        <v>8.623703612447922</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8912440577468403</v>
+        <v>0.9061904743490573</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.59213654171425</v>
+        <v>18.89521437314174</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.62678763798107</v>
+        <v>11.81632053947848</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01786154110103486</v>
+        <v>0.01756693854008269</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.128917386605784</v>
+        <v>0.1294888645357686</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2135934682315617</v>
+        <v>0.2142211469395108</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007207064507187265</v>
+        <v>0.007088193484314452</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5610036030830456</v>
+        <v>0.5564237721699398</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4309381351573677</v>
+        <v>0.431384309336069</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15107157560.16489</v>
+        <v>15169480217.37055</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>340.65</v>
+        <v>346.59</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08091387148143636</v>
+        <v>0.09976203938573613</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1663199628007147</v>
+        <v>-0.1517828736447958</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>206.2</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4122584209576</v>
+        <v>4194470750615</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.91410129096326</v>
+        <v>17.2090367428004</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.06518531178134</v>
+        <v>20.43313259504467</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.246219634052306</v>
+        <v>9.407448298741553</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.462712574943792</v>
+        <v>6.575404524731451</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1504180865275156</v>
+        <v>0.1530409646545476</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.79059490380037</v>
+        <v>13.01059423369895</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.373712810268533</v>
+        <v>9.53494147495778</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01292223452373797</v>
+        <v>0.01270076802709592</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.157042358286515</v>
+        <v>-0.1577876440260642</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2829772877038736</v>
+        <v>0.2836764404011871</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002495229707911346</v>
+        <v>0.002452465449089703</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7935027558318022</v>
+        <v>0.7890007459280095</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3763138795893953</v>
+        <v>0.3779469495109017</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9704395470.835485</v>
+        <v>9650478848.543863</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>256.26</v>
+        <v>266.43</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1313907284768212</v>
+        <v>0.1762913907284769</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1077298050139276</v>
+        <v>-0.07231894150417817</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2756614446000</v>
+        <v>2866014153000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.33809523809524</v>
+        <v>21.1452380952381</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.65061315930424</v>
+        <v>23.5611202623461</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.553803689665842</v>
+        <v>3.694840853186881</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.996795910228055</v>
+        <v>5.195100032631159</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2302231085327532</v>
+        <v>0.2393598017887358</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.42388865222818</v>
+        <v>11.85460124725883</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.740760940078383</v>
+        <v>3.881798103599423</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.00421712946359565</v>
+        <v>-0.004056155824573139</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.102095157642966</v>
+        <v>-0.102536812350511</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1701438734137752</v>
+        <v>0.1705713238420059</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8450139813156574</v>
+        <v>0.8354206364838515</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.446483023664843</v>
+        <v>0.455093526265724</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11110514812.83328</v>
+        <v>11190094542.38074</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>227.98</v>
+        <v>217.55</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2072014436421876</v>
+        <v>0.1519724276882091</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03618838251458523</v>
+        <v>-0.08028240466728664</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5521903580000</v>
+        <v>5269278550000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.67672955974842</v>
+        <v>27.36477987421383</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>20.27942883809856</v>
+        <v>19.33382649687764</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.22596892751404</v>
+        <v>17.39213764444547</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.08393686895154</v>
+        <v>22.98210573664536</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2301941556496812</v>
+        <v>0.2196628588542335</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.70176610304408</v>
+        <v>22.62063342277686</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.28015598955669</v>
+        <v>17.44632470648812</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02300040161150369</v>
+        <v>0.02410310990296765</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.4140797449814766</v>
+        <v>0.415383544412854</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.6431435833864554</v>
+        <v>0.6447285913124072</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001228177910343013</v>
+        <v>0.001287060445874512</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.315003539939778</v>
+        <v>1.32268345257298</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4173397848022767</v>
+        <v>0.4313667636147622</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26634872181.43882</v>
+        <v>27074416690.97906</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>571.1</v>
+        <v>578.02</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.1219384333255101</v>
+        <v>-0.111298990073212</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2778199291856347</v>
+        <v>-0.269069296914517</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1454869580127</v>
+        <v>1472498187191</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.22259383128949</v>
+        <v>21.47974730583426</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.24263055831315</v>
+        <v>17.44840903464677</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.374073727379868</v>
+        <v>6.451308170021205</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.55968815677147</v>
+        <v>5.627054716121599</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.350631735414341</v>
+        <v>-4.40334819769602</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.49235635952443</v>
+        <v>14.65699890906119</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6.798419176189934</v>
+        <v>6.875653618831271</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02816472387609003</v>
+        <v>0.02782753850323412</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.230821118594198</v>
+        <v>0.2310433153637441</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2596687999278604</v>
+        <v>0.2602823259104612</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003677114340745929</v>
+        <v>0.003633092280543926</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7982373253422315</v>
+        <v>0.7943674066257901</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4950843506490172</v>
+        <v>0.4959095475370009</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9599777348.865683</v>
+        <v>9420927424.287313</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>354.81</v>
+        <v>348.75</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1900609627049802</v>
+        <v>-0.2038943680938019</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2887155944911092</v>
+        <v>-0.3008640218110378</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1401338910865</v>
+        <v>1377404653658</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>300.6864406779661</v>
+        <v>295.5508474576271</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.182828731567</v>
+        <v>170.0983545483433</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.52395710115905</v>
+        <v>13.29297381424256</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.22296127011905</v>
+        <v>12.99711886066914</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.004188350441629</v>
+        <v>-7.867480305562183</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>116.0177844084636</v>
+        <v>114.0279060241104</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.46723970377055</v>
+        <v>13.23625641685405</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004111781921793144</v>
+        <v>0.004183229659270967</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7362370327374046</v>
+        <v>0.7375291386115626</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1132795675555351</v>
+        <v>0.1136478047910503</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.546813718890179</v>
+        <v>1.548041761178965</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5856167218320338</v>
+        <v>0.5832359100438107</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12672767620.20612</v>
+        <v>12656491900.70394</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>371.54</v>
+        <v>368.79</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.06881078539440399</v>
+        <v>0.06089984805297477</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2494141414141414</v>
+        <v>-0.254969696969697</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>287.17</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1767631273200</v>
+        <v>1754547928200</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>60.02261712439419</v>
+        <v>59.578352180937</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.54332809004602</v>
+        <v>20.36674045187947</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>23.42319317829458</v>
+        <v>23.249823470483</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>20.11267268020663</v>
+        <v>19.96380620588202</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4767013649879423</v>
+        <v>0.4731729999297605</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>43.13885242593695</v>
+        <v>42.82752952290303</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>24.02319317829457</v>
+        <v>23.84982347048301</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01853440844633275</v>
+        <v>0.01867261616136683</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.921757217783875</v>
+        <v>1.925276743311129</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.155563438374752</v>
+        <v>1.15809507991443</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006836410615276955</v>
+        <v>0.006887388486672632</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.62162018727273</v>
+        <v>1.6206286440273</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4353397048392953</v>
+        <v>0.4342226581384321</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7470489318.635706</v>
+        <v>7387256584.972611</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>934.66</v>
+        <v>945.47</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.09380924517261557</v>
+        <v>0.1064599180807491</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1475968992248062</v>
+        <v>-0.1377382580939353</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>414502082140</v>
+        <v>419296090130</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>46.9442491210447</v>
+        <v>47.48719236564541</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.22757332274661</v>
+        <v>41.69350710502219</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.411854346888656</v>
+        <v>1.428183434995419</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.38225763764959</v>
+        <v>12.52546715240682</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.703146794503843</v>
+        <v>3.745976290629264</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.90518881409814</v>
+        <v>28.23649551693158</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.375360905421562</v>
+        <v>1.391689993528324</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02124476662345385</v>
+        <v>0.02100186528634159</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1386614670125152</v>
+        <v>0.1389589330067496</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1121404101775159</v>
+        <v>0.1123713809512674</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005927289067682366</v>
+        <v>0.005859519604006473</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1799039870830309</v>
+        <v>-0.1821889678506964</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2235863604600854</v>
+        <v>0.2234699502450108</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1750448535.27195</v>
+        <v>1716103675.54248</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>79.84</v>
+        <v>81.72</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1225409179640089</v>
+        <v>-0.1018793063128609</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3698997711309289</v>
+        <v>-0.3550627416936311</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>332448969520</v>
+        <v>340277176718</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>24.71826625386997</v>
+        <v>25.30030959752322</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.35474243919661</v>
+        <v>21.85413760000352</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.872931953690044</v>
+        <v>7.034769529751484</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.09290842029591</v>
+        <v>11.35411417969165</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7264758740466664</v>
+        <v>0.7435822698784266</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.03567749008907</v>
+        <v>11.29152602019843</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6.980643173632735</v>
+        <v>7.142480749694175</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03307156588836582</v>
+        <v>0.03231074180773408</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1575071122609102</v>
+        <v>0.1576896814962467</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1371953377962172</v>
+        <v>0.1375235243853736</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1145522315513156</v>
+        <v>0.1091416067064795</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3711953175656678</v>
+        <v>0.3643511406552154</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2839014071.739907</v>
+        <v>2591821421.794762</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>503.7</v>
+        <v>505</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01378684474657565</v>
+        <v>0.01640332856267768</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.0633019674935843</v>
+        <v>-0.06088444229553314</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1086407155802</v>
+        <v>1089211065475</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.66532562232839</v>
+        <v>12.69801357807392</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.70710493525152</v>
+        <v>22.76568313337069</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.824132751566858</v>
+        <v>2.831421559540614</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.446730913904319</v>
+        <v>1.450464783644393</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3485354230219991</v>
+        <v>0.3494349585588833</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.3588644666597</v>
+        <v>15.39551017428183</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.054868388591244</v>
+        <v>3.062157196564999</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02228906526496889</v>
+        <v>0.02223168747320791</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422307177227965</v>
+        <v>-0.4422300660303596</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05978872701026372</v>
+        <v>0.05983413093961354</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06223410101262753</v>
+        <v>0.06100543137216175</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1566665279614262</v>
+        <v>0.1553396173775642</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2123182772.967977</v>
+        <v>2123359959.79598</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>354.22</v>
+        <v>357.62</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.08830031966196272</v>
+        <v>0.0987464296694458</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.0335061391541609</v>
+        <v>-0.02422919508867671</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>949136032200</v>
+        <v>958246366200</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.22871883061049</v>
+        <v>15.37489251934652</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.15661380067121</v>
+        <v>14.29202981684305</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.188947570329903</v>
+        <v>3.219556857606515</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.636995696720218</v>
+        <v>2.662307043817639</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7973642862247269</v>
+        <v>0.8050178308387071</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.15023649849721</v>
+        <v>20.24802883426363</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.307082992141329</v>
+        <v>6.337692279417941</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.09072988178564274</v>
+        <v>0.08986728573936126</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07573174242335035</v>
+        <v>0.07576689360298738</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2907313742498265</v>
+        <v>-0.290681227959882</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01693862571283383</v>
+        <v>0.01677758514624462</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7765311397591226</v>
+        <v>0.7742646257140239</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1893537996915995</v>
+        <v>0.1892102857984039</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2280760395.171466</v>
+        <v>2222240774.296281</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>379.66</v>
+        <v>381.6</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.09576306846452143</v>
+        <v>0.1013622370701717</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01532795601317527</v>
+        <v>-0.01029644422543241</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>708843144128</v>
+        <v>712465215718</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>32.25658453695837</v>
+        <v>32.4214103653356</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.55831473925371</v>
+        <v>25.68038439245415</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.93335605394713</v>
+        <v>16.01477287623629</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.65099797202797</v>
+        <v>20.75652116663824</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.175197312525154</v>
+        <v>2.186312212136119</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.75572699594474</v>
+        <v>24.88020536524847</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.19183024923575</v>
+        <v>16.27324707152491</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02964407594835333</v>
+        <v>0.02949336969219439</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2620779134321061</v>
+        <v>0.2624970822034196</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1319111800087693</v>
+        <v>0.1322176080579525</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007058947479323605</v>
+        <v>0.007023060796645702</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.294154609127498</v>
+        <v>0.2933733536069152</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2116376618750014</v>
+        <v>0.2116927394260224</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2560126582.105615</v>
+        <v>2530558444.684012</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>591.73</v>
+        <v>595.3</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.0507875532633697</v>
+        <v>0.05712711956075234</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.01643894817326552</v>
+        <v>-0.01050496991456407</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>518968512280</v>
+        <v>522099530800</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32.49478308621637</v>
+        <v>32.69082921471718</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.88842470723435</v>
+        <v>27.03995147245589</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.79259220363139</v>
+        <v>14.88183823504261</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>93.01476742113705</v>
+        <v>93.57594011762609</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.436153359614026</v>
+        <v>1.444817898329018</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>24.0694751437873</v>
+        <v>24.21104769397721</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>15.17317539207023</v>
+        <v>15.26242142348146</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03169363768861141</v>
+        <v>0.03150357169407363</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2085045308538889</v>
+        <v>0.2089825400765799</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1499619228387943</v>
+        <v>0.1503465872348118</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2396,10 +2396,10 @@
         <v>2.324587116608279</v>
       </c>
       <c r="Y15" s="4" t="n">
-        <v>0.8273522788815095</v>
+        <v>1</v>
       </c>
       <c r="Z15" s="4" t="n">
-        <v>0.5943334378473905</v>
+        <v>0.5983524784083459</v>
       </c>
       <c r="AA15" s="5" t="n">
         <v>16912000000</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005695165024588917</v>
+        <v>0.005661011254829498</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2876668721989412</v>
+        <v>0.2865377405887672</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2249632247851309</v>
+        <v>0.2248056471103976</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1703054347.405811</v>
+        <v>1682014347.824178</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>395.05</v>
+        <v>392.95</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1743460379537438</v>
+        <v>0.1681034694694941</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1442095229842728</v>
+        <v>-0.1487587192929249</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>358762446800</v>
+        <v>356855343552</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.4035110282297</v>
+        <v>25.26847148093371</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.35739071243347</v>
+        <v>18.2535605940184</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7970214023091158</v>
+        <v>0.7927846096385702</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.424589427631012</v>
+        <v>3.406385054012419</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7697330169258634</v>
+        <v>-0.7656412833844272</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.66220730504988</v>
+        <v>15.58818241478089</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8964217964183601</v>
+        <v>0.8921850037478145</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06582907495099624</v>
+        <v>0.06618087812536452</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3838301655269496</v>
+        <v>0.3843037006825973</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.008968960895136879</v>
+        <v>0.0090474257139741</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.0226553600810024</v>
+        <v>0.02277643466089833</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4441012578348895</v>
+        <v>0.4441678495401687</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2379497362229291</v>
+        <v>0.2371849768606844</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1874336679.952108</v>
+        <v>1754286074.600732</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>156.45</v>
+        <v>156.7</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.2755809054514309</v>
+        <v>0.2776192258500429</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.1131455132928972</v>
+        <v>-0.1117283600702909</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>648400767000</v>
+        <v>649436882000</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.13513513513513</v>
+        <v>20.16731016731017</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.27848780824289</v>
+        <v>14.3045245719797</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.795825533152384</v>
+        <v>1.798695180856367</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.517537932569974</v>
+        <v>2.521560843935538</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>1.971565315315316</v>
+        <v>1.974715787215788</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.469972391228682</v>
+        <v>9.48439793943613</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.883844145017449</v>
+        <v>1.886713792721431</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04712054882563086</v>
+        <v>0.04704537245545595</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4101728001974574</v>
+        <v>0.4098553269512173</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08522170693313202</v>
+        <v>0.08506026873517003</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02633429210610419</v>
+        <v>0.02629227823867263</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5206064777833972</v>
+        <v>-0.5214199114687725</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2517870463621718</v>
+        <v>0.2517873811071983</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2250612740.875606</v>
+        <v>2215146616.465059</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>265.77</v>
+        <v>268.04</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2817458026373014</v>
+        <v>0.2926934753316865</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03870221000470231</v>
+        <v>-0.03049155423734951</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>276.47</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>640478702020</v>
+        <v>645949171425</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.72485549132948</v>
+        <v>30.98728323699422</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.50944085272119</v>
+        <v>21.68756694818131</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.540235293120526</v>
+        <v>6.596096880648225</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.632078909274928</v>
+        <v>7.697266173164962</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.804222239123827</v>
+        <v>-3.836714937633106</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.83554790762481</v>
+        <v>19.99772238304874</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.832426574559119</v>
+        <v>6.888288162086818</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02920940218776519</v>
+        <v>0.02896203111264793</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4284358064771556</v>
+        <v>0.4288040383244913</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08388214257388316</v>
+        <v>0.08408920784731255</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01986680212213568</v>
+        <v>0.01969855245485748</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1932066728305555</v>
+        <v>-0.1944663493133095</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2472231408609359</v>
+        <v>0.2435592487244984</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1865634223.848373</v>
+        <v>1831381850.863892</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2843,55 +2843,55 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>102.63</v>
+        <v>103.09</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.08983683881091065</v>
+        <v>-0.08575737808649286</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2406777153003847</v>
+        <v>-0.2372743415211601</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>95.7</v>
+        <v>95.8</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>816737750400</v>
+        <v>820398467200</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.05054151624549</v>
+        <v>37.21660649819495</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.30424468321606</v>
+        <v>33.44346398449514</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.10993932159165</v>
+        <v>1.114914203087628</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.309605447993647</v>
+        <v>8.346850098739795</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>8.959494584837552</v>
+        <v>8.99965211683624</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.51784006162609</v>
+        <v>20.60329296202059</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.194503900848011</v>
+        <v>1.199478782343988</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01654019297306133</v>
+        <v>0.01646638863929852</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1124870678997083</v>
+        <v>0.112821522179912</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04821286396859659</v>
+        <v>0.04833694433438107</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009524505505212902</v>
+        <v>0.009482006014162382</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05991517117899932</v>
+        <v>-0.06068402732597815</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3259358147378019</v>
+        <v>0.3255647402781208</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2854901112.381141</v>
+        <v>2813847739.28701</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>143.14</v>
+        <v>143.76</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.009521170588835837</v>
+        <v>0.01389383459446036</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1441554559043349</v>
+        <v>-0.1404484304932736</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>340273687242</v>
+        <v>341747556783</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.20592592592592</v>
+        <v>21.29777777777777</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.32647384043925</v>
+        <v>20.41120476509464</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.90975373703925</v>
+        <v>3.926688537354077</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.384648597889929</v>
+        <v>6.412303216659608</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.23651216931238</v>
+        <v>20.32416507936529</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.19006715168909</v>
+        <v>17.25941266505128</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.197969565699973</v>
+        <v>4.2149043660148</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04676529686729141</v>
+        <v>0.04656361013900182</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04326633789954326</v>
+        <v>0.04343560426179605</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02385325060893995</v>
+        <v>0.02393314673573066</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02997484979740115</v>
+        <v>0.02984557595993323</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05763558130105116</v>
+        <v>-0.05922023214247132</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1950897225816267</v>
+        <v>0.1933771736825277</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1300123886.318818</v>
+        <v>1283685708.290853</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>328.61</v>
+        <v>330.19</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.04976579422741068</v>
+        <v>-0.04519694347691416</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2299707088459285</v>
+        <v>-0.2262683069712946</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>327662617370</v>
+        <v>329238062230</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22.94762569832402</v>
+        <v>23.05796089385475</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.91791237904162</v>
+        <v>22.02329657781489</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.936815017319242</v>
+        <v>1.946127478070175</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.65687789613047</v>
+        <v>19.75139074441837</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.871569280239088</v>
+        <v>-7.909416818240907</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.23017425757892</v>
+        <v>16.29605110725486</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.294324356705443</v>
+        <v>2.303636817456377</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04608703953233638</v>
+        <v>0.04586650734644011</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02817930069078847</v>
+        <v>0.02804445925073442</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6969599695718738</v>
+        <v>0.6952918696801946</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2596517473824705</v>
+        <v>0.2595703065254926</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1305949958.020776</v>
+        <v>1290941579.850724</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>476.67</v>
+        <v>465.58</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.133037980025032</v>
+        <v>1.083411632240448</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.1848032425221897</v>
+        <v>-0.2037692610264568</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>777258102000</v>
+        <v>759174748000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>120.9822335025381</v>
+        <v>118.1675126903553</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.6392717389905</v>
+        <v>35.72604794165878</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.81753061372715</v>
+        <v>18.37973000847355</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.56504775080329</v>
+        <v>11.2959803046531</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9767372980021422</v>
+        <v>0.9540129464909419</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>72.44337581638365</v>
+        <v>70.75618100391864</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.79792039704636</v>
+        <v>18.36011979179276</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01081108061579267</v>
+        <v>0.01106859787175113</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.301982483832835</v>
+        <v>2.307601022182046</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8423499739938611</v>
+        <v>0.8448557020304353</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.534249787416535</v>
+        <v>2.53603055845523</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7477529796640676</v>
+        <v>0.7238675915754516</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12451378549.3144</v>
+        <v>12158324144.49397</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1735.01</v>
+        <v>1696.16</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4908401556334034</v>
+        <v>0.4574575583882248</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1324776495529911</v>
+        <v>-0.1519030380607612</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>716.2</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>668704068565</v>
+        <v>653730579615</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.93323657474601</v>
+        <v>54.22351233671989</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>36.50100127875624</v>
+        <v>35.65422605764373</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.21641219508881</v>
+        <v>16.30369105512703</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.2473338403878</v>
+        <v>26.38860043802175</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.671432506773787</v>
+        <v>3.691192638672462</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.16033190785613</v>
+        <v>41.38368979318338</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.08372519487651</v>
+        <v>16.17100405491473</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01745881761705185</v>
+        <v>0.01736535499597549</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4775823863806008</v>
+        <v>0.5208158564164145</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2449661196120889</v>
+        <v>0.2811564967036335</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004484124010812618</v>
+        <v>0.004586831430997075</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.701198303696669</v>
+        <v>1.703723359846175</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4813878229254439</v>
+        <v>0.4621705225616071</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2520118811.442489</v>
+        <v>2466493813.674959</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>209.89</v>
+        <v>209.82</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.0785002587569551</v>
+        <v>-0.07880758631847307</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1747985059956753</v>
+        <v>-0.1750737173186554</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>165890759300</v>
+        <v>165835433400</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.61048689138573</v>
+        <v>78.58426966292132</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>91.33694939022961</v>
+        <v>90.76317315030494</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.764889188786638</v>
+        <v>1.764300584073621</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.21842426797377</v>
+        <v>27.20934670497049</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4207291179949846</v>
+        <v>0.4205888014565137</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.43046896402878</v>
+        <v>29.4225084028777</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.176091912335762</v>
+        <v>2.175503307622746</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001265893295600824</v>
+        <v>-0.00126631562202677</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1393353137345446</v>
+        <v>-0.134183315376328</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1453054650801158</v>
+        <v>0.145730067231935</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.185945448834664</v>
+        <v>1.185044133411448</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3630380795341275</v>
+        <v>0.3623681161035353</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1295981186.282844</v>
+        <v>1297785322.02537</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1040.87</v>
+        <v>1033.99</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.1383839375157661</v>
+        <v>0.1308593845071211</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.09802511286926241</v>
+        <v>-0.10398703628281</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>721.16</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>307063936090</v>
+        <v>305034287930</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.85725167580743</v>
+        <v>15.75243753808653</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.40378058518576</v>
+        <v>14.30688962076542</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.603626818470878</v>
+        <v>2.586417222160984</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.544891618191002</v>
+        <v>2.528070253051115</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3716720069301576</v>
+        <v>0.369215308776037</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.44790036281974</v>
+        <v>27.38324747332208</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.306205313769215</v>
+        <v>7.288995717459321</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1351998561883608</v>
+        <v>-0.1360994538736149</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1009089996911339</v>
+        <v>0.1010385873965924</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3830987867656763</v>
+        <v>-0.3830559819615791</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01633249108918501</v>
+        <v>0.01644116480817029</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.563504055705266</v>
+        <v>1.564427864553645</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3877117558577918</v>
+        <v>0.3874434741487459</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>2012605724.658077</v>
+        <v>1971922033.129745</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>238.79</v>
+        <v>235.59</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1808233276157805</v>
+        <v>-0.1918010291595197</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2817481802322084</v>
+        <v>-0.2913733983035552</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>224972177860</v>
+        <v>221957349060</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.85502183406114</v>
+        <v>20.57554585152839</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.57043887601599</v>
+        <v>18.31831657507457</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.255889226160325</v>
+        <v>3.212257392650911</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.514533873214909</v>
+        <v>6.42723328108673</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2542210994888461</v>
+        <v>0.2508143089265767</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.45096959866839</v>
+        <v>17.26510998458788</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.096736151497171</v>
+        <v>4.053104317987756</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.0605897143800713</v>
+        <v>0.0614126995917366</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1230225614643776</v>
+        <v>0.1232225279655439</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04395753961016879</v>
+        <v>0.04406506290759382</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.0282256375895138</v>
+        <v>0.0286090241521287</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8925206935420051</v>
+        <v>0.8939393766754512</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7912416348277762</v>
+        <v>0.7906766049060748</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1683767913.282338</v>
+        <v>1621571116.299121</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1175.49</v>
+        <v>1172.86</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.08805399675875725</v>
+        <v>0.08561962299847381</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.09063551618767651</v>
+        <v>-0.09267009631377421</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1107007128090</v>
+        <v>1104530349260</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.37989949748744</v>
+        <v>39.29179229480737</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.28067577373227</v>
+        <v>27.20195747592293</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.89563812941061</v>
+        <v>13.86454851718052</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.9633482688391</v>
+        <v>30.89407196198234</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4174432410499701</v>
+        <v>0.4165092682182476</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.74895274057032</v>
+        <v>32.67860569359237</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.47327621250273</v>
+        <v>14.44218660027264</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01811542084159878</v>
+        <v>0.01815604253286066</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4435089447236182</v>
+        <v>0.4444472361809046</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2194043809730903</v>
+        <v>0.2198712826923515</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005691243651583596</v>
+        <v>0.005704005593165425</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.347390515064774</v>
+        <v>0.3483695509148373</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3457167142666453</v>
+        <v>0.3404165787178404</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3161258465.698324</v>
+        <v>3151997782.253336</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>214.83</v>
+        <v>214.767</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1810335745379708</v>
+        <v>0.1806872303812148</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.07500538213132391</v>
+        <v>-0.07527664155005387</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>145.66</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>338847062400</v>
+        <v>338747693760</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.26929260450161</v>
+        <v>17.26422829581994</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.03701105550685</v>
+        <v>16.02980564018207</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.678018971144955</v>
+        <v>2.677233628338167</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.056575799016456</v>
+        <v>3.055679442477155</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.439358356006266</v>
+        <v>0.4392295119135955</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.96459816676321</v>
+        <v>23.96121217705387</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.558323091149065</v>
+        <v>5.557537748342278</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04628636851360822</v>
+        <v>-0.04629994621044413</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07683985156146766</v>
+        <v>0.07700796150288514</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.329833359443268</v>
+        <v>-0.3297362440212688</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01931759996276125</v>
+        <v>0.01932326660986092</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.367058922375227</v>
+        <v>1.366702314359371</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2964586926517028</v>
+        <v>0.2946456949941399</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1030287023.441925</v>
+        <v>1000620872.160711</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>935.39</v>
+        <v>932.86</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.965537886562504</v>
+        <v>1.957516835607284</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2546693227091633</v>
+        <v>-0.2566852589641434</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,40 +4120,40 @@
         <v>114.25</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1056420112100</v>
+        <v>1053562755400</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.87458156661459</v>
+        <v>20.81812095514394</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.028218992606147</v>
+        <v>6.003205407685578</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.70237401798967</v>
+        <v>11.6707219731041</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.4753576108971</v>
+        <v>10.44702434375124</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02975239953018246</v>
+        <v>0.02967192660358354</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.18451865654171</v>
+        <v>15.14271143007637</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.49612415645701</v>
+        <v>11.46447211157144</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02477423489029768</v>
+        <v>0.02484142483763431</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.462810755916152</v>
+        <v>2.467834188797144</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.760053105680423</v>
+        <v>1.763697862828721</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.000566608580378238</v>
+        <v>0.0005681452736745064</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.892343224369627</v>
+        <v>2.890084036332151</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8924047513250013</v>
+        <v>0.8918592028125559</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>34085064158.55794</v>
+        <v>33006220046.03546</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>138.43</v>
+        <v>144.71</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.06117325964685083</v>
+        <v>-0.01858255005053655</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2891036636093793</v>
+        <v>-0.2568532193954582</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>143117516660</v>
+        <v>149610170020</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>85.98136645962734</v>
+        <v>89.88198757763976</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.5057388797746</v>
+        <v>30.82725919456624</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.714737758620689</v>
+        <v>10.15545547244094</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.42523090444231</v>
+        <v>11.94354666027485</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>137.5701863354067</v>
+        <v>143.8111801242267</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.72499760963026</v>
+        <v>44.58588994554314</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.11862046293782</v>
+        <v>10.55933817675808</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03200167321852411</v>
+        <v>0.03061289215424154</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.914055696417936</v>
+        <v>1.915665872543181</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2351963937961905</v>
+        <v>0.2357608804280309</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6851410507884158</v>
+        <v>0.6730351447188559</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5844094081493592</v>
+        <v>0.5899717374953706</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2552872768.330767</v>
+        <v>2636713544.359764</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.01</v>
+        <v>27.96</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1123907728564448</v>
+        <v>0.1104050699416705</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.0257391304347826</v>
+        <v>-0.02747826086956517</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>28.75</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>159641314400</v>
+        <v>159356342400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.01109936575053</v>
+        <v>36.94503171247358</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.589163888857598</v>
+        <v>9.572774127639521</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.50630046470736</v>
+        <v>2.501826525998493</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.873799624369058</v>
+        <v>1.870454748209884</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6190352017811371</v>
+        <v>-0.6179301764298678</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.57440703422053</v>
+        <v>17.55183320659062</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.483096495855313</v>
+        <v>3.478622557146446</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06881677240813297</v>
+        <v>0.06893983530585852</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.859679508529062</v>
+        <v>2.859386131947059</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04871896271441734</v>
+        <v>-0.04882775962211783</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06140664048554088</v>
+        <v>0.06151645207439198</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3268326070158217</v>
+        <v>0.3266580984528082</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2188310131914338</v>
+        <v>0.2159139583501666</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1003250803.331423</v>
+        <v>990474907.272971</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>161.61</v>
+        <v>161.04</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.03809293920651557</v>
+        <v>-0.04148559451653544</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1703798767967145</v>
+        <v>-0.1733059548254621</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1147196489345</v>
+        <v>1143150316466</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.558861686113768</v>
+        <v>7.222426801818531</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003503248857976881</v>
+        <v>0.003488204655462377</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.491753285413805</v>
+        <v>6.202813977334693</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.704319156815743</v>
+        <v>4.494936165443018</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01691578859433369</v>
+        <v>0.01616288933319861</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.634501639024965</v>
+        <v>7.29310919359487</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.461500981164543</v>
+        <v>6.172561673085431</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07425100616006471</v>
+        <v>0.07770976446274165</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2156.671918996641</v>
+        <v>2069.528399332455</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2809.307515718858</v>
+        <v>2696.868588886155</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.856320772229441</v>
+        <v>1.862891207153502</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.268537072657392</v>
+        <v>1.249759359915266</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>4690831577.080143</v>
+        <v>4373631026.801108</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>573</v>
+        <v>553.11</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.5349585286292171</v>
+        <v>0.481676983891983</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1471056666120895</v>
+        <v>-0.1767113704359734</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>281.74</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>72221348604</v>
+        <v>69714398126</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817632884153544</v>
+        <v>1.822484444101408</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.458412896134327</v>
+        <v>0.4544132725217073</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5732058251.723661</v>
+        <v>5440081695.83549</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>140.87</v>
+        <v>141.5</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1247592254052633</v>
+        <v>-0.1208449662443726</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3756869349406133</v>
+        <v>-0.3728948767948945</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1841997164815</v>
+        <v>1850234960043</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-91.47402597402598</v>
+        <v>-91.88311688311688</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.6153741718258</v>
+        <v>139.5689771652479</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>111.1310506675716</v>
+        <v>111.6280518879638</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.492970508709049</v>
+        <v>6.522008426083129</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9147402597402597</v>
+        <v>-0.9188311688311689</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>429.0470757895368</v>
+        <v>431.0239884912407</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>107.8635996871795</v>
+        <v>108.3606009075716</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0154305340653739</v>
+        <v>-0.01536183274763084</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.989775821814501</v>
+        <v>3.999723134775511</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.8264438873693197</v>
+        <v>0.8195228575355898</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13019040872.47394</v>
+        <v>12932608883.7583</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>771.1</v>
+        <v>769.35</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1287088415613358</v>
+        <v>0.1261472536055164</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01061113463438412</v>
+        <v>-0.01285653797297814</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>821405196069</v>
+        <v>819541029173</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9957670725761122</v>
+        <v>0.9957371613519083</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1134925619735879</v>
+        <v>0.1124484247221805</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>33480822590.33699</v>
+        <v>32873022737.20056</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -4897,13 +4897,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>427.3</v>
+        <v>417.52</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3369419592131371</v>
+        <v>0.3063421643123543</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1079331941544885</v>
+        <v>-0.1283507306889353</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4912,40 +4912,40 @@
         <v>225.63</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2216182904000</v>
+        <v>2165459129600</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.93555117653877</v>
+        <v>28.0514663266489</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6646162313146817</v>
+        <v>0.6489501230825194</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.07436022855125</v>
+        <v>14.13276006352449</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.714817505368815</v>
+        <v>9.755127951449184</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5247819590387496</v>
+        <v>0.5269594775409852</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.51345021489235</v>
+        <v>18.59300870460516</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.58978081708063</v>
+        <v>13.64818065205387</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01789632973916031</v>
+        <v>0.01782237796337865</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.03260447202632</v>
+        <v>42.22592034254367</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.07585742460906</v>
+        <v>42.2733977517231</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2574303767844606</v>
+        <v>0.2634604330331481</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.203492657968162</v>
+        <v>2.207519375116576</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.4336034214599973</v>
+        <v>0.4182944075005067</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4995825518.300403</v>
+        <v>4840567328.569606</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -5025,13 +5025,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.88</v>
+        <v>28.77</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.01297789435804142</v>
+        <v>0.009119599054046024</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.03733333333333333</v>
+        <v>-0.04100000000000004</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5040,38 +5040,38 @@
         <v>11.25</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>72406107954</v>
+        <v>72130322917</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.74015748031496</v>
+        <v>-22.65354330708661</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-74.47562411946485</v>
+        <v>-74.80689462536287</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>2.004876310508099</v>
+        <v>1.997240008777516</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.208346427918875</v>
+        <v>2.199935136122785</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1692290789232742</v>
+        <v>0.1685845083318074</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.70415007504132</v>
+        <v>16.65856577140496</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.798286250976049</v>
+        <v>2.790649949245466</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03010795720970068</v>
+        <v>0.03022307279157082</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02139428397140786</v>
+        <v>0.02147086015031885</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3059095691029505</v>
+        <v>0.3064953553260474</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2072350655406984</v>
+        <v>0.2021918699847645</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>600613831.2081285</v>
+        <v>585011656.335789</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>334.16</v>
+        <v>333.2</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1034797570613193</v>
+        <v>-0.1060553478957135</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1376293581769852</v>
+        <v>-0.1401068414668766</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>225661589600</v>
+        <v>225013292000</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>20.26440266828381</v>
+        <v>20.20618556701031</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.34515818112915</v>
+        <v>17.28923458765273</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.684114871599681</v>
+        <v>2.676403744365016</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.609115519253209</v>
+        <v>6.590128354725787</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.256569947116291</v>
+        <v>1.252959978391035</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.685632972011001</v>
+        <v>9.659411583886103</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.848329304295077</v>
+        <v>2.840618177060412</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06670164836949283</v>
+        <v>0.06689382598784431</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1683031343196792</v>
+        <v>0.1687148707809631</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.001858927300198543</v>
+        <v>0.002093680031818312</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01059372755566196</v>
+        <v>0.01062424969987995</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9515853473858182</v>
+        <v>0.9512041130609026</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2614417396495906</v>
+        <v>0.2608809026673605</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>914769865.3014883</v>
+        <v>905018766.4876893</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>151.92</v>
+        <v>150.72</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2237494517993107</v>
+        <v>-0.2298809727171676</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5605692467893093</v>
+        <v>-0.5640402637972927</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>437601002400</v>
+        <v>434144438400</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>25.57575757575757</v>
+        <v>25.37373737373737</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.35705998245757</v>
+        <v>17.20444769098494</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.496644829122005</v>
+        <v>6.445328519255322</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>10.28572880398984</v>
+        <v>10.20448292086196</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7707289107289099</v>
+        <v>0.7646410046410039</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>17.52503356700003</v>
+        <v>17.41734238090787</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.350916036699427</v>
+        <v>8.299599726832744</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05412693268547229</v>
+        <v>-0.0545578796017579</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4735074719800745</v>
+        <v>0.474835916240026</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4770155984898927</v>
+        <v>0.4786777919072371</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01316482359136388</v>
+        <v>0.01326963906581741</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.057408419218062</v>
+        <v>2.056899797826053</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5630489862277076</v>
+        <v>0.5629553223339963</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3911481705.923538</v>
+        <v>3833023048.165332</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02 ET</t>
+          <t>2026-08-28 17:36 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-29)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>36.49543378995434</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.76692495113887</v>
+        <v>33.76018144007593</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.05851835320882</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08080418465002825</v>
+        <v>0.08102007255895427</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1052797251879132</v>
+        <v>0.1055263726494853</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003315608382858931</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3366059664559604</v>
+        <v>0.3366060014141145</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.3093319618130679</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15279678996.55258</v>
+        <v>15280847127.11385</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.52944444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.25872130325989</v>
+        <v>25.24594782451542</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.49124331829592</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1294888645357686</v>
+        <v>0.1300603424657536</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2142211469395108</v>
+        <v>0.2148488256474601</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007088193484314452</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5564237721699398</v>
+        <v>0.556423816066045</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.431384309336069</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15170145213.034</v>
+        <v>15173994137.72125</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.2090367428004</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.43313259504467</v>
+        <v>20.43785894218623</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.407448298741553</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1577876440260642</v>
+        <v>-0.1579824094353226</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2836764404011871</v>
+        <v>0.2859759413617506</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002452465449089703</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7890007459280095</v>
+        <v>0.789000793952618</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.3779469495109017</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9650922829.03591</v>
+        <v>9651806414.019571</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.1452380952381</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.5611202623461</v>
+        <v>23.57272074159521</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.694840853186881</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.102536812350511</v>
+        <v>-0.1029784670580559</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1705713238420059</v>
+        <v>0.1710006496606318</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8354206364838515</v>
+        <v>0.8354207266950323</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.455093526265724</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11190734338.20512</v>
+        <v>11192090431.34384</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>27.36477987421383</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.33382649687764</v>
+        <v>19.31603327517455</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.39213764444547</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.415383544412854</v>
+        <v>0.4166873438442316</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.6447285913124072</v>
+        <v>0.6463135992383597</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.001287060445874512</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.32268345257298</v>
+        <v>1.322683408248895</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.4313667636147622</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27079573598.48242</v>
+        <v>27083565002.89174</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.47974730583426</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.44840903464677</v>
+        <v>17.48519900773532</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.451308170021205</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2310433153637441</v>
+        <v>0.228453121770692</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2602823259104612</v>
+        <v>0.2615201003801682</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003633092280543926</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7943674066257901</v>
+        <v>0.7943674507329229</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.4959095475370009</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9421496620.596313</v>
+        <v>9430063166.295776</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>295.5508474576271</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.0983545483433</v>
+        <v>169.9732515997364</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.29297381424256</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7375291386115626</v>
+        <v>0.7388079869979107</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1136478047910503</v>
+        <v>0.1140160420265657</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.548041761178965</v>
+        <v>1.548041773634103</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.5832359100438107</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12657369464.0979</v>
+        <v>12658473199.7229</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>59.578352180937</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.36674045187947</v>
+        <v>20.33395789405199</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.249823470483</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.925276743311129</v>
+        <v>1.929992896186956</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.15809507991443</v>
+        <v>1.161592384970988</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1670,13 +1670,13 @@
         <v>0.006887388486672632</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.6206286440273</v>
+        <v>1.620628673731938</v>
       </c>
       <c r="AJ9" s="4" t="n">
         <v>0.4342226581384321</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7387987280.32275</v>
+        <v>7389106975.960693</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.48719236564541</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.69350710502219</v>
+        <v>41.6826207053013</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.428183434995419</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1389589330067496</v>
+        <v>0.1392563990009839</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1123713809512674</v>
+        <v>0.112602351725019</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.005859519604006473</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1821889678506964</v>
+        <v>-0.1821889529918093</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2234699502450108</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1716103675.54248</v>
+        <v>1716132260.251261</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>25.30030959752322</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.85413760000352</v>
+        <v>21.85069171623866</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7.034769529751484</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1576896814962467</v>
+        <v>0.1578722507315833</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1375235243853736</v>
+        <v>0.1378517109745303</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1091416067064795</v>
+        <v>0.1091416527536769</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3643511406552154</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2591965133.78817</v>
+        <v>2592020640.737</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.69801357807392</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.76568313337069</v>
+        <v>22.7656565342206</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.831421559540614</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422300660303596</v>
+        <v>-0.4422294143379225</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05983413093961354</v>
+        <v>0.05987953486896358</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1553396173775642</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2123359959.79598</v>
+        <v>2123413220.462646</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.37489251934652</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.29202981684305</v>
+        <v>14.29156283343295</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.219556857606515</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07576689360298738</v>
+        <v>0.0758020447826242</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.290681227959882</v>
+        <v>-0.2906310816699373</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1892102857984039</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2222240774.296281</v>
+        <v>2222282222.453715</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>32.4214103653356</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.68038439245415</v>
+        <v>25.65772664134541</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>16.01477287623629</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2624970822034196</v>
+        <v>0.2636119644789983</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1322176080579525</v>
+        <v>0.1326270024585359</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.2116927394260224</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2530558444.684012</v>
+        <v>2530782838.207601</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>32.69082921471718</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.03995147245589</v>
+        <v>27.02939243988374</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.88183823504261</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2089825400765799</v>
+        <v>0.2094548291244462</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1503465872348118</v>
+        <v>0.1507140655266435</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2248056471103976</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1682014347.824178</v>
+        <v>1682099436.035767</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.26847148093371</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.2535605940184</v>
+        <v>18.24731864951403</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7927846096385702</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3843037006825973</v>
+        <v>0.3847772358382453</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.0090474257139741</v>
+        <v>0.00912589053281132</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2371849768606844</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1754286074.600732</v>
+        <v>1754314052.641602</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.16731016731017</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.3045245719797</v>
+        <v>14.30774641085395</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.798695180856367</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4098553269512173</v>
+        <v>0.409537853704977</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08506026873517003</v>
+        <v>0.08489883053720826</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2517873811071983</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2215146616.465059</v>
+        <v>2216454053.27474</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.98728323699422</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.68756694818131</v>
+        <v>21.68190318861996</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.596096880648225</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4288040383244913</v>
+        <v>0.4291772713595692</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08408920784731255</v>
+        <v>0.08429627312074151</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2435592487244984</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1831381850.863892</v>
+        <v>1831419072.686412</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
         <v>135.16</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>95.8</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>820398467200</v>
@@ -2864,7 +2864,7 @@
         <v>37.21660649819495</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.44346398449514</v>
+        <v>33.43280375488809</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.114914203087628</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.112821522179912</v>
+        <v>0.1131763513179369</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04833694433438107</v>
+        <v>0.04816880120010092</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3255647402781208</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2814044446.781745</v>
+        <v>2814190631.832886</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.29777777777777</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.41120476509464</v>
+        <v>20.4078941918336</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.926688537354077</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04343560426179605</v>
+        <v>0.04360487062404861</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02393314673573066</v>
+        <v>0.02401304286252115</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1933771736825277</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1283736284.42397</v>
+        <v>1283798924.576772</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>23.05796089385475</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.02329657781489</v>
+        <v>22.0135325322796</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.946127478070175</v>
@@ -3140,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04698044692737424</v>
+        <v>0.04744483240223452</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01393283308507121</v>
+        <v>0.01436683199153554</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3188,7 +3188,7 @@
         <v>0.2595703065254926</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1290941579.850724</v>
+        <v>1296188122.888184</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>118.1675126903553</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>35.72604794165878</v>
+        <v>35.62775850430868</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.37973000847355</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.307601022182046</v>
+        <v>2.316725992629164</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8448557020304353</v>
+        <v>0.8491804527777822</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.53603055845523</v>
+        <v>2.536030579442794</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.7238675915754516</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12158931104.31107</v>
+        <v>12159786002.28241</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.22351233671989</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.65422605764373</v>
+        <v>35.62482259903076</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.30369105512703</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5208158564164145</v>
+        <v>0.5220710836099751</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2811564967036335</v>
+        <v>0.2819772791247528</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.004586831430997075</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.703723359846175</v>
+        <v>1.703723361984467</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.4621705225616071</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2466493813.674959</v>
+        <v>2466968399.252523</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>78.58426966292132</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>90.76317315030494</v>
+        <v>90.22628620110262</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.764300584073621</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.134183315376328</v>
+        <v>-0.1290313170181113</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.145730067231935</v>
+        <v>0.1461546693837545</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.3623681161035353</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1297785322.02537</v>
+        <v>1297816375.386454</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.75243753808653</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.30688962076542</v>
+        <v>14.30520595696172</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.586417222160984</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1010385873965924</v>
+        <v>0.101168175102051</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3830559819615791</v>
+        <v>-0.3830131771574816</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3874434741487459</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1971922033.129745</v>
+        <v>1972253909.450277</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.57554585152839</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.31831657507457</v>
+        <v>18.31505595879635</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.212257392650911</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1232225279655439</v>
+        <v>0.1234224944667108</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04406506290759382</v>
+        <v>0.04417258620501929</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.7906766049060748</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1621571116.299121</v>
+        <v>1621611747.72049</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.29179229480737</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.20195747592293</v>
+        <v>27.18429895933128</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.86454851718052</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4444472361809046</v>
+        <v>0.4453855276381913</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2198712826923515</v>
+        <v>0.2203381844116126</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3404165787178404</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3151997782.253336</v>
+        <v>3152132627.479655</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.26422829581994</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.02980564018207</v>
+        <v>16.02730394175175</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.677233628338167</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07700796150288514</v>
+        <v>0.07717607144430261</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3297362440212688</v>
+        <v>-0.3296391285992696</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.2946456949941399</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1000620872.160711</v>
+        <v>1000631660.773926</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4192,13 +4192,13 @@
         <v>0.0005681452736745064</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.890084036332151</v>
+        <v>2.890084094900321</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.8918592028125559</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>33010800339.14052</v>
+        <v>33012654398.36141</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>89.88198757763976</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.82725919456624</v>
+        <v>30.81024424091299</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>10.15545547244094</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.915665872543181</v>
+        <v>1.917276048668425</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2357608804280309</v>
+        <v>0.2363253670598717</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.5899717374953706</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2636956258.280256</v>
+        <v>2637400889.423218</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.94503171247358</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.572774127639521</v>
+        <v>9.573501870643353</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.501826525998493</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.859386131947059</v>
+        <v>2.859092755365056</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04882775962211783</v>
+        <v>-0.04893655652981799</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2159139583501666</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>990497323.2733372</v>
+        <v>990507848.3489927</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.222426801818531</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003488204655462377</v>
+        <v>0.003460544213149107</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.202813977334693</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2069.528399332455</v>
+        <v>2086.078319755406</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2696.868588886155</v>
+        <v>2711.674749178965</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4574,7 +4574,7 @@
         <v>1.249759359915266</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>4374082996.102816</v>
+        <v>4374228082.400767</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.822484444101408</v>
+        <v>1.822484429593136</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.4544132725217073</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5440081695.83549</v>
+        <v>5443038714.002177</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-91.88311688311688</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.5689771652479</v>
+        <v>138.9045774837286</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>111.6280518879638</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>3.999723134775511</v>
+        <v>4.009670447736523</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.8195228575355898</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12933421234.06348</v>
+        <v>12933850229.04681</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>0.1124484247221805</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32874420998.48962</v>
+        <v>32883917752.00826</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>28.0514663266489</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6489501230825194</v>
+        <v>0.6499395027631194</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.13276006352449</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.22592034254367</v>
+        <v>42.16011906860921</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.2733977517231</v>
+        <v>42.27564946127661</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.4182944075005067</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4840846497.894963</v>
+        <v>4841104706.173503</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.65354330708661</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-74.80689462536287</v>
+        <v>-75.43211166697981</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.997240008777516</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02147086015031885</v>
+        <v>0.02154743632922984</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3064953553260474</v>
+        <v>0.3064953506989899</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.2021918699847645</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>585011656.335789</v>
+        <v>585012103.2297961</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.20618556701031</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.28923458765273</v>
+        <v>17.28314576183751</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.676403744365016</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1687148707809631</v>
+        <v>0.1691266072422475</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.002093680031818312</v>
+        <v>0.002328432763438304</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.2608809026673605</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>905018766.4876893</v>
+        <v>905021309.9144491</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.37373737373737</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.20444769098494</v>
+        <v>17.1758300072142</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.445328519255322</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.474835916240026</v>
+        <v>0.4772932290945988</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4786777919072371</v>
+        <v>0.4804921389467931</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5372,7 +5372,7 @@
         <v>0.5629553223339963</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3833545215.307055</v>
+        <v>3833669711.817093</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28 19:11 ET</t>
+          <t>2026-08-29 11:58 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-30)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>36.49543378995434</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.76018144007593</v>
+        <v>33.75344062193582</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.05851835320882</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08102007255895427</v>
+        <v>0.08123596046788006</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1055263726494853</v>
+        <v>0.1057730201110572</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>28.52944444444444</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.24594782451542</v>
+        <v>25.23318725848235</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.49124331829592</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1300603424657536</v>
+        <v>0.1306318203957382</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2148488256474601</v>
+        <v>0.2154765043554092</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>17.2090367428004</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.43785894218623</v>
+        <v>20.45593255507941</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.407448298741553</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1579824094353226</v>
+        <v>-0.1587263647617365</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2859759413617506</v>
+        <v>0.2866805595837703</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>21.1452380952381</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.57272074159521</v>
+        <v>23.5843326496225</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.694840853186881</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1029784670580559</v>
+        <v>-0.1034201217656013</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1710006496606318</v>
+        <v>0.1714280950148874</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>27.36477987421383</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>19.31603327517455</v>
+        <v>16.7482514968441</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>17.39213764444547</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.4166873438442316</v>
+        <v>0.6338887602308949</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.6463135992383597</v>
+        <v>0.8772916918275875</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>21.47974730583426</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.48519900773532</v>
+        <v>17.49727323550747</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.451308170021205</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.228453121770692</v>
+        <v>0.2276054112388834</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2615201003801682</v>
+        <v>0.2621348599632796</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>295.5508474576271</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>169.9732515997364</v>
+        <v>169.847074754195</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.29297381424256</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7388079869979107</v>
+        <v>0.7400997213837939</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1140160420265657</v>
+        <v>0.1143842792620808</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>59.578352180937</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.33395789405199</v>
+        <v>20.30294926675432</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>23.249823470483</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.929992896186956</v>
+        <v>1.934467864651338</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.161592384970988</v>
+        <v>1.164840685100795</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>47.48719236564541</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.6826207053013</v>
+        <v>41.67173998909185</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.428183434995419</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1392563990009839</v>
+        <v>0.1395538649952182</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.112602351725019</v>
+        <v>0.1128333224987708</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>25.30030959752322</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.85069171623866</v>
+        <v>21.84724691897222</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7.034769529751484</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1578722507315833</v>
+        <v>0.1580548199669196</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1378517109745303</v>
+        <v>0.1381798975636865</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.69801357807392</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.7656565342206</v>
+        <v>22.76562993513267</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.831421559540614</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422294143379225</v>
+        <v>-0.4422287626454856</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05987953486896358</v>
+        <v>0.05992493879831362</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.37489251934652</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.29156283343295</v>
+        <v>14.29109588053865</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.219556857606515</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.0758020447826242</v>
+        <v>0.07583719596226102</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2906310816699373</v>
+        <v>-0.290580935379993</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>32.4214103653356</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.65772664134541</v>
+        <v>25.64920574390395</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>16.01477287623629</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2636119644789983</v>
+        <v>0.264031747768299</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1326270024585359</v>
+        <v>0.1329330686200743</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>32.69082921471718</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.02939243988374</v>
+        <v>27.01884165064354</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.88183823504261</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2094548291244462</v>
+        <v>0.2099271181723124</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1507140655266435</v>
+        <v>0.1510831904628513</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.26847148093371</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.24731864951403</v>
+        <v>18.24110076135842</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.7927846096385702</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3847772358382453</v>
+        <v>0.3852492682054542</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.00912589053281132</v>
+        <v>0.009204369005926027</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.16731016731017</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.30774641085395</v>
+        <v>14.31096970137857</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.798695180856367</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.409537853704977</v>
+        <v>0.4092203804587364</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08489883053720826</v>
+        <v>0.08473739233924604</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>30.98728323699422</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.68190318861996</v>
+        <v>21.67631841176311</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.596096880648225</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4291772713595692</v>
+        <v>0.4295454905376515</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08429627312074151</v>
+        <v>0.08450333839417068</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>37.21660649819495</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.43280375488809</v>
+        <v>33.4228322324975</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.114914203087628</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1131763513179369</v>
+        <v>0.1135084615004203</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04816880120010092</v>
+        <v>0.04877177918438935</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.29777777777777</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.4078941918336</v>
+        <v>20.40458469230809</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.926688537354077</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04360487062404861</v>
+        <v>0.04377413698630139</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02401304286252115</v>
+        <v>0.02409293898931208</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>23.05796089385475</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.0135325322796</v>
+        <v>22.02016820396815</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.946127478070175</v>
@@ -3140,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04744483240223452</v>
+        <v>0.04712918994413395</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01436683199153554</v>
+        <v>0.01431960424055423</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>118.1675126903553</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>35.62775850430868</v>
+        <v>35.56735166403298</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.37973000847355</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.316725992629164</v>
+        <v>2.322359050135596</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8491804527777822</v>
+        <v>0.8516936045558186</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>54.22351233671989</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.62482259903076</v>
+        <v>35.59546759756133</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.30369105512703</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5220710836099751</v>
+        <v>0.5233263108035353</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2819772791247528</v>
+        <v>0.2827980615458721</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>78.58426966292132</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>90.22628620110262</v>
+        <v>89.6957135433895</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.764300584073621</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1290313170181113</v>
+        <v>-0.1238793186598948</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1461546693837545</v>
+        <v>0.146579271535574</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.75243753808653</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.30520595696172</v>
+        <v>14.30352268938534</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.586417222160984</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.101168175102051</v>
+        <v>0.1012977628075096</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3830131771574816</v>
+        <v>-0.3829703723533845</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.57554585152839</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.31505595879635</v>
+        <v>18.31179650307526</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.212257392650911</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1234224944667108</v>
+        <v>0.1236224609678771</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04417258620501929</v>
+        <v>0.04428010950244454</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>39.29179229480737</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.18429895933128</v>
+        <v>27.16666335439337</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.86454851718052</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4453855276381913</v>
+        <v>0.4463238190954775</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2203381844116126</v>
+        <v>0.2208050861308735</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.26422829581994</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.02730394175175</v>
+        <v>16.02480302405685</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.677233628338167</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07717607144430261</v>
+        <v>0.07734418138572008</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3296391285992696</v>
+        <v>-0.3295420131772705</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>89.88198757763976</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.81024424091299</v>
+        <v>30.79324805953796</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>10.15545547244094</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.917276048668425</v>
+        <v>1.91888622479367</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2363253670598717</v>
+        <v>0.2368898536917119</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>36.94503171247358</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.573501870643353</v>
+        <v>9.574229724304796</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.501826525998493</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.859092755365056</v>
+        <v>2.858799378783052</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04893655652981799</v>
+        <v>-0.04904535343751848</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.222426801818531</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003460544213149107</v>
+        <v>0.003457139953852709</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.202813977334693</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2086.078319755406</v>
+        <v>2088.133473977444</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2711.674749178965</v>
+        <v>2715.29142948499</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-91.88311688311688</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.9045774837286</v>
+        <v>138.2464734066758</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>111.6280518879638</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.009670447736523</v>
+        <v>4.019617760697535</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>28.0514663266489</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6499395027631194</v>
+        <v>0.6494840269862829</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.13276006352449</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.16011906860921</v>
+        <v>42.19038677026824</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.27564946127661</v>
+        <v>42.30891968599801</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.65354330708661</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-75.43211166697981</v>
+        <v>-76.06786760072919</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.997240008777516</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02154743632922984</v>
+        <v>0.02162401250814083</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>20.20618556701031</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.28314576183751</v>
+        <v>17.27706122316962</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.676403744365016</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1691266072422475</v>
+        <v>0.1695383437035314</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.002328432763438304</v>
+        <v>0.002563185495058073</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>25.37373737373737</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.1758300072142</v>
+        <v>17.16036032751456</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.445328519255322</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4772932290945988</v>
+        <v>0.4786249757852497</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4804921389467931</v>
+        <v>0.4821555132075719</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29 11:58 ET</t>
+          <t>2026-08-30 11:46 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-08-31)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>319.7</v>
+        <v>315.685</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1796612246037816</v>
+        <v>0.1648462736598211</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.07217691615636879</v>
+        <v>-0.08382912035290357</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4695547713200</v>
+        <v>4636577978860</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>36.49543378995434</v>
+        <v>36.037100456621</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.75344062193582</v>
+        <v>33.32288951256638</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.05851835320882</v>
+        <v>9.932196954434549</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>43.68672847377233</v>
+        <v>43.13808219656809</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.115138254693048</v>
+        <v>1.101133625063418</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.13474539843073</v>
+        <v>27.78474756870007</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.15440694481634</v>
+        <v>10.02808554604207</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02910906423456423</v>
+        <v>0.02947928420986169</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08123596046788006</v>
+        <v>0.08145184837680608</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1057730201110572</v>
+        <v>0.106019667572629</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003315608382858931</v>
+        <v>0.003357777531399971</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3366060014141145</v>
+        <v>0.3367145211153043</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3093319618130679</v>
+        <v>0.309176597887675</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15280847127.11385</v>
+        <v>14896948341.10478</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>513.53</v>
+        <v>511.0642</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.08582483475506497</v>
+        <v>0.08061106559349906</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.07258181030123534</v>
+        <v>-0.07703496351946837</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3813242691500</v>
+        <v>3794932770310</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.52944444444444</v>
+        <v>28.39245555555556</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.23318725848235</v>
+        <v>25.09933943578383</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.49124331829592</v>
+        <v>11.43606619568526</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.623703612447922</v>
+        <v>8.582295460309638</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9061904743490573</v>
+        <v>0.9018392495488512</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.89521437314174</v>
+        <v>18.80698186821448</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.81632053947848</v>
+        <v>11.76114341686782</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01756693854008269</v>
+        <v>0.01765169610488988</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1306318203957382</v>
+        <v>0.131203298325723</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2154765043554092</v>
+        <v>0.2161041830633579</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007088193484314452</v>
+        <v>0.007122392842229998</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.556423816066045</v>
+        <v>0.5563290318956275</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.431384309336069</v>
+        <v>0.428832921628053</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15173994137.72125</v>
+        <v>14967591403.43832</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>346.59</v>
+        <v>338.05</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09976203938573613</v>
+        <v>0.07266383165800572</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1517828736447958</v>
+        <v>-0.1726829984581875</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>206.2</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4194470750615</v>
+        <v>4091118720232</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.2090367428004</v>
+        <v>16.7850049652433</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.45593255507941</v>
+        <v>19.96955653844801</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.407448298741553</v>
+        <v>9.175648164658966</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.575404524731451</v>
+        <v>6.413386132275794</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1530409646545476</v>
+        <v>0.1492700253944713</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>13.01059423369895</v>
+        <v>12.69525445345791</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.53494147495778</v>
+        <v>9.303841626994149</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01270076802709592</v>
+        <v>0.01302062789028958</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1587263647617365</v>
+        <v>-0.1594703200881502</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2866805595837703</v>
+        <v>0.2873851778057901</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002452465449089703</v>
+        <v>0.002514420943647389</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.789000793952618</v>
+        <v>0.7888461080625434</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3779469495109017</v>
+        <v>0.3813561687369495</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9651806414.019571</v>
+        <v>9492078741.425358</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>266.43</v>
+        <v>257.765</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1762913907284769</v>
+        <v>0.1380353200883002</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.07231894150417817</v>
+        <v>-0.1024895543175488</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2866014153000</v>
+        <v>2772803881500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>21.1452380952381</v>
+        <v>20.45753968253968</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>23.5843326496225</v>
+        <v>22.82855383852138</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.694840853186881</v>
+        <v>3.574674970993193</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.195100032631159</v>
+        <v>5.026141800514846</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2393598017887358</v>
+        <v>0.2315751953911852</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.85460124725883</v>
+        <v>11.48762734008669</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.881798103599423</v>
+        <v>3.761632221405735</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004056155824573139</v>
+        <v>-0.004192507114391098</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1034201217656013</v>
+        <v>-0.1038617764731465</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1714280950148874</v>
+        <v>0.1718555403691431</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8354207266950323</v>
+        <v>0.8367295359482756</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.455093526265724</v>
+        <v>0.4624230930396683</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11192090431.34384</v>
+        <v>11109013778.14427</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>217.55</v>
+        <v>218.93</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1519724276882091</v>
+        <v>0.1592798142669714</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.08028240466728664</v>
+        <v>-0.07444829627124372</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5269278550000</v>
+        <v>5302703530000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.36477987421383</v>
+        <v>27.53836477987421</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.7482514968441</v>
+        <v>16.83230540131734</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.39213764444547</v>
+        <v>17.50246239714294</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>22.98210573664536</v>
+        <v>23.1278897215526</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2196628588542335</v>
+        <v>0.22105626149831</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.62063342277686</v>
+        <v>22.7636787821986</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.44632470648812</v>
+        <v>17.55664945918559</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02410310990296765</v>
+        <v>0.02395117873014485</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6338887602308949</v>
+        <v>0.636042367536831</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8772916918275875</v>
+        <v>0.8847629049148795</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001287060445874512</v>
+        <v>0.001278947608824739</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.322683408248895</v>
+        <v>1.324089650323722</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4313667636147622</v>
+        <v>0.4299077324501831</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27083565002.89174</v>
+        <v>26966746622.08807</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>578.02</v>
+        <v>571.665</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.111298990073212</v>
+        <v>-0.1210697504588124</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.269069296914517</v>
+        <v>-0.2771054628224583</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1472498187191</v>
+        <v>1456308910039</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.47974730583426</v>
+        <v>21.24358974358974</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.49727323550747</v>
+        <v>17.30135961114968</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.451308170021205</v>
+        <v>6.380379718722618</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.627054716121599</v>
+        <v>5.565188461111473</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.40334819769602</v>
+        <v>-4.354935897435894</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.65699890906119</v>
+        <v>14.50579899543298</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6.875653618831271</v>
+        <v>6.804725167532684</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02782753850323412</v>
+        <v>0.02813688752264975</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2276054112388834</v>
+        <v>0.2278566668193831</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2621348599632796</v>
+        <v>0.262749619546391</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003633092280543926</v>
+        <v>0.003673480097609614</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7943674507329229</v>
+        <v>0.7946736602383492</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4959095475370009</v>
+        <v>0.4497229519665484</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9430063166.295776</v>
+        <v>9331550890.6339</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>348.75</v>
+        <v>367.29</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.2038943680938019</v>
+        <v>-0.1615723654685949</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.3008640218110378</v>
+        <v>-0.263697051099573</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1377404653658</v>
+        <v>1450629262342</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>295.5508474576271</v>
+        <v>311.2627118644068</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>169.847074754195</v>
+        <v>178.7436769791843</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.29297381424256</v>
+        <v>13.99964545442438</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>12.99711886066914</v>
+        <v>13.68806246977826</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-7.867480305562183</v>
+        <v>-8.285725710193361</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>114.0279060241104</v>
+        <v>120.1157517743598</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.23625641685405</v>
+        <v>13.94292805703587</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004183229659270967</v>
+        <v>0.003972069328518449</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7400997213837939</v>
+        <v>0.7413914557696775</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1143842792620808</v>
+        <v>0.1147525164975958</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.548041773634103</v>
+        <v>1.546643755401861</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5832359100438107</v>
+        <v>0.5982180302510033</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12658473199.7229</v>
+        <v>12758300803.33565</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>368.79</v>
+        <v>371.23</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.06089984805297477</v>
+        <v>0.06791900700318831</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.254969696969697</v>
+        <v>-0.250040404040404</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>287.17</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1754547928200</v>
+        <v>1766156423400</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>59.578352180937</v>
+        <v>59.97253634894992</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.30294926675432</v>
+        <v>20.41275362634286</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>23.249823470483</v>
+        <v>23.40364968395945</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>19.96380620588202</v>
+        <v>20.0958913685555</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4731729999297605</v>
+        <v>0.4763036220177472</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>42.82752952290303</v>
+        <v>43.09017284473528</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>23.84982347048301</v>
+        <v>23.99608446034586</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01867261616136683</v>
+        <v>0.01855588400784261</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.934467864651338</v>
+        <v>1.937993445017373</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.164840685100795</v>
+        <v>1.167377175775252</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006887388486672632</v>
+        <v>0.006842119440777954</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.620628673731938</v>
+        <v>1.617569269880087</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4342226581384321</v>
+        <v>0.4310362044822887</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7389106975.960693</v>
+        <v>7316515905.756067</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>945.47</v>
+        <v>942.255</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1064599180807491</v>
+        <v>0.1026974839087185</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1377382580939353</v>
+        <v>-0.1406703146374829</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>419296090130</v>
+        <v>417870305145</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>47.48719236564541</v>
+        <v>47.32571572074335</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.67173998909185</v>
+        <v>41.51920029751781</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.428183434995419</v>
+        <v>1.42332700407375</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.52546715240682</v>
+        <v>12.4828752384434</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.745976290629264</v>
+        <v>3.733238378506857</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.23649551693158</v>
+        <v>28.13796165480304</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.391689993528324</v>
+        <v>1.386833562606655</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02100186528634159</v>
+        <v>0.02107352422887369</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1395538649952182</v>
+        <v>0.1398513309894525</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1128333224987708</v>
+        <v>0.1130642932725223</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005859519604006473</v>
+        <v>0.005879512446206176</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1821889529918093</v>
+        <v>-0.1814044937310335</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2234699502450108</v>
+        <v>0.2217079911636664</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1716132260.251261</v>
+        <v>1688203366.262179</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>81.72</v>
+        <v>81.51000000000001</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1018793063128609</v>
+        <v>-0.1041872522951699</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3550627416936311</v>
+        <v>-0.356720069449925</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>340277176718</v>
+        <v>339402749318</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>25.30030959752322</v>
+        <v>25.23529411764706</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.84724691897222</v>
+        <v>21.78767008637844</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7.034769529751484</v>
+        <v>7.016691928165534</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.35411417969165</v>
+        <v>11.32493694061021</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7435822698784266</v>
+        <v>0.7416714490674321</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.29152602019843</v>
+        <v>11.26294719501933</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.142480749694175</v>
+        <v>7.124403148108225</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03231074180773408</v>
+        <v>0.03239398626585288</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1580548199669196</v>
+        <v>0.1582373892022564</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1381798975636865</v>
+        <v>0.1385080841528432</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1091416527536769</v>
+        <v>0.1082531964759029</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3643511406552154</v>
+        <v>0.3537312760727187</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2592020640.737</v>
+        <v>2482088656.920186</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>505</v>
+        <v>504.89</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01640332856267768</v>
+        <v>0.01618193377823829</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06088444229553314</v>
+        <v>-0.06108900211998369</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1089211065475</v>
+        <v>1088973811580</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.69801357807392</v>
+        <v>12.69524767412623</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.76562993513267</v>
+        <v>22.76064449181586</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.831421559540614</v>
+        <v>2.830804814251586</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.450464783644393</v>
+        <v>1.450148840820233</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3494349585588833</v>
+        <v>0.3493588440134547</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.39551017428183</v>
+        <v>15.39240938364221</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.062157196564999</v>
+        <v>3.061540451275973</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02223168747320791</v>
+        <v>0.02223653107402673</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422287626454856</v>
+        <v>-0.4422281109530485</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05992493879831362</v>
+        <v>0.05997034272766366</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06100543137216175</v>
+        <v>0.05980177153665873</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1553396173775642</v>
+        <v>0.1552975923189197</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2123413220.462646</v>
+        <v>2091734024.509595</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>357.62</v>
+        <v>355.83</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.0987464296694458</v>
+        <v>0.09324685998903548</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.02422919508867671</v>
+        <v>-0.0291132332878582</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>958246366200</v>
+        <v>953450043300</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.37489251934652</v>
+        <v>15.29793637145314</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.29109588053865</v>
+        <v>14.21909988865573</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.219556857606515</v>
+        <v>3.203441968128534</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.662307043817639</v>
+        <v>2.648981364022232</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8050178308387071</v>
+        <v>0.8009884647036998</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.24802883426363</v>
+        <v>20.19654404572778</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.337692279417941</v>
+        <v>6.321577389939959</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.08986728573936126</v>
+        <v>0.09031936240932573</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07583719596226102</v>
+        <v>0.07587234714189806</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.290580935379993</v>
+        <v>-0.2905307890900483</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01677758514624462</v>
+        <v>0.01686198465559396</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7742646257140239</v>
+        <v>0.7743852485934481</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1892102857984039</v>
+        <v>0.1842973622688814</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2222282222.453715</v>
+        <v>2163925145.076166</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>381.6</v>
+        <v>380.65</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.1013622370701717</v>
+        <v>0.0986203761550335</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01029644422543241</v>
+        <v>-0.01276032886376022</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>712465215718</v>
+        <v>710691520867</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>32.4214103653356</v>
+        <v>32.34069668649108</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.64920574390395</v>
+        <v>25.57685754822172</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>16.01477287623629</v>
+        <v>15.97490381377001</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.75652116663824</v>
+        <v>20.70484743731878</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.186312212136119</v>
+        <v>2.180869348924564</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.88020536524847</v>
+        <v>24.81924946274658</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.27324707152491</v>
+        <v>16.23337800905862</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02949336969219439</v>
+        <v>0.02956697720885347</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.264031747768299</v>
+        <v>0.2644515310575994</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1329330686200743</v>
+        <v>0.1332391347816126</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007023060796645702</v>
+        <v>0.007040588467095758</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2933733536069152</v>
+        <v>0.2942095090130602</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2116927394260224</v>
+        <v>0.2056577932453457</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2530782838.207601</v>
+        <v>2463037011.039962</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>595.3</v>
+        <v>591.42</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.05712711956075234</v>
+        <v>0.05023705871093598</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.01050496991456407</v>
+        <v>-0.01695422359629006</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>522099530800</v>
+        <v>518696631120</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32.69082921471718</v>
+        <v>32.47775947281713</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>27.01884165064354</v>
+        <v>26.83226650565373</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.88183823504261</v>
+        <v>14.78484254824274</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>93.57594011762609</v>
+        <v>92.96603813936909</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.444817898329018</v>
+        <v>1.435400976700399</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>24.21104769397721</v>
+        <v>24.05718172906493</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>15.26242142348146</v>
+        <v>15.16542573668158</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03150357169407363</v>
+        <v>0.0317102502950222</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2099271181723124</v>
+        <v>0.2103994072201787</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1510831904628513</v>
+        <v>0.1514506553673307</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005661011254829498</v>
+        <v>0.005698150214737412</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2865377405887672</v>
+        <v>0.2882698547676688</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2248056471103976</v>
+        <v>0.2235187174491093</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1682099436.035767</v>
+        <v>1653143951.060852</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>392.95</v>
+        <v>390.75</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1681034694694941</v>
+        <v>0.1615636358193275</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1487587192929249</v>
+        <v>-0.1535245439972271</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>356855343552</v>
+        <v>354857425863</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.26847148093371</v>
+        <v>25.12700147900457</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.24110076135842</v>
+        <v>18.13277618446684</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7927846096385702</v>
+        <v>0.7883460649347187</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.406385054012419</v>
+        <v>3.387313805459608</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7656412833844272</v>
+        <v>-0.761354705388637</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.58818241478089</v>
+        <v>15.51063252971316</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8921850037478145</v>
+        <v>0.8877464590439629</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06618087812536452</v>
+        <v>0.0665534895953335</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3852492682054542</v>
+        <v>0.3857228051228705</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009204369005926027</v>
+        <v>0.009282833922202638</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02277643466089833</v>
+        <v>0.02290467050543826</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4441678495401687</v>
+        <v>0.4466964656552516</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2371849768606844</v>
+        <v>0.2272901903063554</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1754314052.641602</v>
+        <v>1701079496.394043</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>156.7</v>
+        <v>160.49</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.2776192258500429</v>
+        <v>0.3085201630930019</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.1117283600702909</v>
+        <v>-0.09024431721557724</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>649436882000</v>
+        <v>665144385400</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.16731016731017</v>
+        <v>20.65508365508366</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.31096970137857</v>
+        <v>14.66040246588006</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.798695180856367</v>
+        <v>1.842199040048745</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.521560843935538</v>
+        <v>2.582548180237489</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>1.974715787215788</v>
+        <v>2.022476941226943</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.48439793943613</v>
+        <v>9.703089250261051</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.886713792721431</v>
+        <v>1.930217651913809</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04704537245545595</v>
+        <v>0.04593438758657828</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4092203804587364</v>
+        <v>0.4089029072124961</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08473739233924604</v>
+        <v>0.08457595414128427</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02629227823867263</v>
+        <v>0.02567138139447941</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5214199114687725</v>
+        <v>-0.5280703554663262</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2517873811071983</v>
+        <v>0.2562267441309772</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2216454053.27474</v>
+        <v>2191248377.79423</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>268.04</v>
+        <v>266.295</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2926934753316865</v>
+        <v>0.2842777533705845</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03049155423734951</v>
+        <v>-0.03680326979419113</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>276.47</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>645949171425</v>
+        <v>641743898689</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.98728323699422</v>
+        <v>30.78554913294798</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.67631841176311</v>
+        <v>21.5296551979127</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.596096880648225</v>
+        <v>6.553154823280131</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.697266173164962</v>
+        <v>7.64715525885302</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.836714937633106</v>
+        <v>-3.811737070276854</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.99772238304874</v>
+        <v>19.87305522023598</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.888288162086818</v>
+        <v>6.845346104718725</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02896203111264793</v>
+        <v>0.02915181591631495</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4295454905376515</v>
+        <v>0.4299137097157337</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08450333839417068</v>
+        <v>0.08471040366759963</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01969855245485748</v>
+        <v>0.01982763476595505</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1944663493133095</v>
+        <v>-0.19050164786551</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2435592487244984</v>
+        <v>0.2442819054606212</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1831419072.686412</v>
+        <v>1781231618.814524</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>103.09</v>
+        <v>104.62</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.08575737808649286</v>
+        <v>-0.07218873698136474</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2372743415211601</v>
+        <v>-0.225954424385913</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>96.51000000000001</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>820398467200</v>
+        <v>832574329600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.21660649819495</v>
+        <v>37.76895306859206</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.4228322324975</v>
+        <v>33.90876039963859</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.114914203087628</v>
+        <v>1.131461091541639</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.346850098739795</v>
+        <v>8.470729045786763</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>8.99965211683624</v>
+        <v>9.133219560223178</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.60329296202059</v>
+        <v>20.88844557529354</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.199478782343988</v>
+        <v>1.216079745596869</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01646638863929852</v>
+        <v>0.01622480291350332</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1135084615004203</v>
+        <v>0.1138405716829038</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04877177918438935</v>
+        <v>0.04889636152208499</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009482006014162382</v>
+        <v>0.009343337793920856</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.06068402732597815</v>
+        <v>-0.0647865460076697</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3255647402781208</v>
+        <v>0.3139512581536252</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2814190631.832886</v>
+        <v>2789985783.103643</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>143.76</v>
+        <v>145.72</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.01389383459446036</v>
+        <v>0.02771709499933772</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1404484304932736</v>
+        <v>-0.128729446935725</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>341747556783</v>
+        <v>346406886300</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.29777777777777</v>
+        <v>21.58814814814815</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.40458469230809</v>
+        <v>20.67942388342316</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.926688537354077</v>
+        <v>3.98022435770751</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.412303216659608</v>
+        <v>6.499727495350849</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.32416507936529</v>
+        <v>20.60126137566159</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.25941266505128</v>
+        <v>17.47863396537122</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.2149043660148</v>
+        <v>4.268440186368233</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04656361013900182</v>
+        <v>0.04593730849281907</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04377413698630139</v>
+        <v>0.04394340334855396</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02409293898931208</v>
+        <v>0.02417283511610258</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02984557595993323</v>
+        <v>0.02944413944551194</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05922023214247132</v>
+        <v>-0.06193747396928009</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1933771736825277</v>
+        <v>0.1958673293128494</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1283798924.576772</v>
+        <v>1274230732.629063</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>330.19</v>
+        <v>328.41</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.04519694347691416</v>
+        <v>-0.05034412976544822</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2262683069712946</v>
+        <v>-0.230439367311072</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,40 +3110,40 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>329238062230</v>
+        <v>327463193970</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>23.05796089385475</v>
+        <v>22.93645251396648</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22.02016820396815</v>
+        <v>21.9014610977473</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.946127478070175</v>
+        <v>1.935871983319147</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.75139074441837</v>
+        <v>19.64730697478486</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.909416818240907</v>
+        <v>-7.867736618162954</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.29605110725486</v>
+        <v>16.22350318419402</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.303636817456377</v>
+        <v>2.293381322705348</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04586650734644011</v>
+        <v>0.04610949021379528</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04712918994413395</v>
+        <v>0.04725672920176249</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01431960424055423</v>
+        <v>0.01444314732441154</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02804445925073442</v>
+        <v>0.02819646173989829</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6952918696801946</v>
+        <v>0.6961032774303664</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2595703065254926</v>
+        <v>0.2595776037019503</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1296188122.888184</v>
+        <v>1263422330.918032</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>465.58</v>
+        <v>468.7758</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.083411632240448</v>
+        <v>1.097712433164701</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.2037692610264568</v>
+        <v>-0.1983038325380945</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>759174748000</v>
+        <v>764385819480</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>118.1675126903553</v>
+        <v>118.9786294416244</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>35.56735166403298</v>
+        <v>35.75087487990587</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.37973000847355</v>
+        <v>18.50589079966106</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.2959803046531</v>
+        <v>11.37351734202071</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9540129464909419</v>
+        <v>0.9605614120057746</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>70.75618100391864</v>
+        <v>71.24237912670274</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.36011979179276</v>
+        <v>18.48628058298027</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01106859787175113</v>
+        <v>0.01099313957147509</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.322359050135596</v>
+        <v>2.327992107642028</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8516936045558186</v>
+        <v>0.8542067563338547</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.536030579442794</v>
+        <v>2.536580435834404</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7238675915754516</v>
+        <v>0.7051031286250898</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12159786002.28241</v>
+        <v>11885734217.76869</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1696.16</v>
+        <v>1688.77</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4574575583882248</v>
+        <v>0.4511075611258857</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1519030380607612</v>
+        <v>-0.1555981119622393</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,40 +3362,40 @@
         <v>716.2</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>653730579615</v>
+        <v>650882340661</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>54.22351233671989</v>
+        <v>52.677793904209</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.59546759756133</v>
+        <v>35.41120271657555</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.30369105512703</v>
+        <v>15.83893112544052</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>26.38860043802175</v>
+        <v>25.63635580562097</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.691192638672462</v>
+        <v>3.585969936312018</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>41.38368979318338</v>
+        <v>40.19430905385925</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>16.17100405491473</v>
+        <v>15.70624412522822</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01736535499597549</v>
+        <v>0.01787490460528893</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5233263108035353</v>
+        <v>0.4876025060722144</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2827980615458721</v>
+        <v>0.252484410665841</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004586831430997075</v>
+        <v>0.004606903249110299</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.703723361984467</v>
+        <v>1.706580145462919</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4621705225616071</v>
+        <v>0.424747428004508</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2466968399.252523</v>
+        <v>2417356852.075212</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>209.82</v>
+        <v>206.75</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.07880758631847307</v>
+        <v>-0.09228609508790531</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1750737173186554</v>
+        <v>-0.1871436996264989</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>165835433400</v>
+        <v>163408997500</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.58426966292132</v>
+        <v>77.43445692883893</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>89.6957135433895</v>
+        <v>87.86662597477361</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.764300584073621</v>
+        <v>1.738486063088462</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.20934670497049</v>
+        <v>26.81123072754098</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4205888014565137</v>
+        <v>0.4144349189835774</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.4225084028777</v>
+        <v>29.0733809352518</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.175503307622746</v>
+        <v>2.149688786637587</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.00126631562202677</v>
+        <v>-0.001285118954358679</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1238793186598948</v>
+        <v>-0.118727320301678</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.146579271535574</v>
+        <v>0.1470038736873935</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.185044133411448</v>
+        <v>1.187635552875871</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3623681161035353</v>
+        <v>0.3629835773700484</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1297816375.386454</v>
+        <v>1272719103.242902</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1033.99</v>
+        <v>1027.22</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.1308593845071211</v>
+        <v>0.123455136851812</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.10398703628281</v>
+        <v>-0.1098536382464319</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>721.16</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>305034287930</v>
+        <v>303037090540</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.75243753808653</v>
+        <v>15.64929920780012</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.30352268938534</v>
+        <v>14.20819920670371</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.586417222160984</v>
+        <v>2.569482779280463</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.528070253051115</v>
+        <v>2.511517834156197</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.369215308776037</v>
+        <v>0.3667978892261248</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.38324747332208</v>
+        <v>27.3196282782786</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.288995717459321</v>
+        <v>7.2720612745788</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1360994538736149</v>
+        <v>-0.1369964314467972</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1012977628075096</v>
+        <v>0.1014273505129684</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3829703723533845</v>
+        <v>-0.3829275675492871</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01644116480817029</v>
+        <v>0.01654952201086428</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.564427864553645</v>
+        <v>1.565084740420895</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3874434741487459</v>
+        <v>0.3873454371707339</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1972253909.450277</v>
+        <v>1927400563.185368</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>235.59</v>
+        <v>235.16</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1918010291595197</v>
+        <v>-0.1932761578044597</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2913733983035552</v>
+        <v>-0.2926667869818925</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>221957349060</v>
+        <v>221552234890</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.57554585152839</v>
+        <v>20.53799126637555</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.31179650307526</v>
+        <v>18.27512137538408</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.212257392650911</v>
+        <v>3.206394414952892</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.42723328108673</v>
+        <v>6.415502264019506</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2508143089265767</v>
+        <v>0.2503565214447718</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.26510998458788</v>
+        <v>17.24013531163307</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.053104317987756</v>
+        <v>4.047241340289738</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.0614126995917366</v>
+        <v>0.06152499435073516</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1236224609678771</v>
+        <v>0.1238224274690438</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04428010950244454</v>
+        <v>0.04438763279986979</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.0286090241521287</v>
+        <v>0.02866133696206838</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8939393766754512</v>
+        <v>0.8931663884698617</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7906766049060748</v>
+        <v>0.7887834866735925</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1621611747.72049</v>
+        <v>1568213677.824716</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1172.86</v>
+        <v>1155.25</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.08561962299847381</v>
+        <v>0.06931950059596792</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.09267009631377421</v>
+        <v>-0.1062932735079102</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1104530349260</v>
+        <v>1087946290250</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>39.29179229480737</v>
+        <v>38.70184254606366</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>27.16666335439337</v>
+        <v>26.74141903105717</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.86454851718052</v>
+        <v>13.65637814783759</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.89407196198234</v>
+        <v>30.43021045485404</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4165092682182476</v>
+        <v>0.410255556595954</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.67860569359237</v>
+        <v>32.20757470603272</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.44218660027264</v>
+        <v>14.23401623092971</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01815604253286066</v>
+        <v>0.01843280332836265</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4463238190954775</v>
+        <v>0.4472621105527641</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2208050861308735</v>
+        <v>0.2212719878501344</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005704005593165425</v>
+        <v>0.005790954338887687</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3483695509148373</v>
+        <v>0.3541799864407826</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3404165787178404</v>
+        <v>0.3424168134924933</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3152132627.479655</v>
+        <v>3098262968.986133</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>214.767</v>
+        <v>213.84</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1806872303812148</v>
+        <v>0.1755910235032336</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.07527664155005387</v>
+        <v>-0.07926803013993544</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>145.66</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>338747693760</v>
+        <v>337285555200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.26422829581994</v>
+        <v>17.18971061093248</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.02480302405685</v>
+        <v>15.95314573141478</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.677233628338167</v>
+        <v>2.665677869895439</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.055679442477155</v>
+        <v>3.042490196256011</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4392295119135955</v>
+        <v>0.4373336631214445</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.96121217705387</v>
+        <v>23.91138975704501</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.557537748342278</v>
+        <v>5.545981989899549</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04629994621044413</v>
+        <v>-0.04650065725672678</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07734418138572008</v>
+        <v>0.07751229132713755</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3295420131772705</v>
+        <v>-0.3294448977552711</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01932326660986092</v>
+        <v>0.01940703329592219</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.366702314359371</v>
+        <v>1.366473882433483</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2946456949941399</v>
+        <v>0.2931254632769064</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>1000631660.773926</v>
+        <v>960908244.4760051</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>932.86</v>
+        <v>947.6900000000001</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.957516835607284</v>
+        <v>2.004533509783534</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2566852589641434</v>
+        <v>-0.2448685258964143</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>114.25</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1053562755400</v>
+        <v>1070311609100</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.81812095514394</v>
+        <v>21.1490738674403</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.003205407685578</v>
+        <v>6.098640452811296</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.6707219731041</v>
+        <v>11.8562555010302</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.44702434375124</v>
+        <v>10.61310432468925</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02967192660358354</v>
+        <v>0.03014363154487285</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.14271143007637</v>
+        <v>15.38777118046411</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.46447211157144</v>
+        <v>11.65000563949753</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02484142483763431</v>
+        <v>0.02445269188662489</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005681452736745064</v>
+        <v>0.0005592546085745339</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.890084094900321</v>
+        <v>2.887579954825612</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8918592028125559</v>
+        <v>0.8519159031593102</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>33012654398.36141</v>
+        <v>32381355611.12071</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>144.71</v>
+        <v>148.28</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.01858255005053655</v>
+        <v>0.005629047602145221</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2568532193954582</v>
+        <v>-0.2385197662356336</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>149610170020</v>
+        <v>153301057360</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>89.88198757763976</v>
+        <v>92.09937888198759</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.79324805953796</v>
+        <v>31.53552213007663</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>10.15545547244094</v>
+        <v>10.40599086071138</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.94354666027485</v>
+        <v>12.23819431128156</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>143.8111801242267</v>
+        <v>147.3590062111833</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>44.58588994554314</v>
+        <v>45.64375390083118</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.55933817675808</v>
+        <v>10.80987356502851</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03061289215424154</v>
+        <v>0.02987585394955687</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.91888622479367</v>
+        <v>1.920496400918915</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2368898536917119</v>
+        <v>0.2374543403235525</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6730351447188559</v>
+        <v>0.6582172436732332</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5899717374953706</v>
+        <v>0.5752842863169193</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2637400889.423218</v>
+        <v>2639158211.969902</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>27.96</v>
+        <v>28.555</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1104050699416705</v>
+        <v>0.1340349346274823</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.02747826086956517</v>
+        <v>-0.00678260869565217</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>28.75</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>159356342400</v>
+        <v>162747509200</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>36.94503171247358</v>
+        <v>37.73123678646935</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.574229724304796</v>
+        <v>9.778716623725844</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.501826525998493</v>
+        <v>2.555066396634011</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.870454748209884</v>
+        <v>1.91025877450405</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6179301764298678</v>
+        <v>-0.631079978109974</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.55183320659062</v>
+        <v>17.82046175538656</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.478622557146446</v>
+        <v>3.531862427781964</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06893983530585852</v>
+        <v>0.06750333724923147</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858799378783052</v>
+        <v>2.858506002201049</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04904535343751848</v>
+        <v>-0.04915415034521853</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06151645207439198</v>
+        <v>0.06023463491507617</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3266580984528082</v>
+        <v>0.3232392122974059</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2159139583501666</v>
+        <v>0.2179557999249083</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>990507848.3489927</v>
+        <v>978712398.5011922</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>161.04</v>
+        <v>163.1133</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.04148559451653544</v>
+        <v>-0.02914525722835315</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1733059548254621</v>
+        <v>-0.1626627310061601</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1143150316466</v>
+        <v>1157867737922</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.222426801818531</v>
+        <v>7.314181770262687</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003457139953852709</v>
+        <v>0.003498973524835673</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.202813977334693</v>
+        <v>6.281615606810814</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.494936165443018</v>
+        <v>4.552040617635579</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01616288933319861</v>
+        <v>0.01636822549532636</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.29310919359487</v>
+        <v>7.386216224166715</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.172561673085431</v>
+        <v>6.251363302561552</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07770976446274165</v>
+        <v>0.07673491078668575</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2088.133473977444</v>
+        <v>2089.379283623242</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2715.29142948499</v>
+        <v>2718.024246602104</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.862891207153502</v>
+        <v>1.839212375692233</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.249759359915266</v>
+        <v>1.232307604251599</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>4374228082.400767</v>
+        <v>4229671107.300415</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>553.11</v>
+        <v>555.34</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.481676983891983</v>
+        <v>0.4876507317433674</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1767113704359734</v>
+        <v>-0.1733920783531548</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>281.74</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>69714398126</v>
+        <v>69995468994</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.822484429593136</v>
+        <v>1.823064851727479</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4544132725217073</v>
+        <v>0.4359932833833187</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5443038714.002177</v>
+        <v>5360621808.507344</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>141.5</v>
+        <v>142.28</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1208449662443726</v>
+        <v>-0.115998740616603</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3728948767948945</v>
+        <v>-0.369438042900195</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1850234960043</v>
+        <v>1860434135088</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-91.88311688311688</v>
+        <v>-92.3896103896104</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.2464734066758</v>
+        <v>138.3530477408354</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>111.6280518879638</v>
+        <v>112.2433867323077</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.522008426083129</v>
+        <v>6.557960133308181</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9188311688311689</v>
+        <v>-0.923896103896104</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>431.0239884912407</v>
+        <v>433.4715946935445</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>108.3606009075716</v>
+        <v>108.9759357519155</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01536183274763084</v>
+        <v>-0.01527761690883809</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.019617760697535</v>
+        <v>4.029565073658547</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.8195228575355898</v>
+        <v>0.7968685001994</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12933850229.04681</v>
+        <v>12901149010.44839</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>769.35</v>
+        <v>766.3200000000001</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1261472536055164</v>
+        <v>0.1217120470305835</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01285653797297814</v>
+        <v>-0.01674429346780082</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>819541029173</v>
+        <v>816313357348</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9957371613519083</v>
+        <v>0.9956634284005813</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1124484247221805</v>
+        <v>0.112923999795694</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32883917752.00826</v>
+        <v>32040959852.9495</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -4897,13 +4897,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>417.52</v>
+        <v>416.04889</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3063421643123543</v>
+        <v>0.3017393356542264</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1283507306889353</v>
+        <v>-0.1314219415448853</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4912,40 +4912,40 @@
         <v>225.63</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2165459129600</v>
+        <v>2157829242651</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.0514663266489</v>
+        <v>27.87759360148371</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6494840269862829</v>
+        <v>0.6467423685701239</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.13276006352449</v>
+        <v>14.04516031106463</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.755127951449184</v>
+        <v>9.694662282328631</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5269594775409852</v>
+        <v>0.5236931997876318</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.59300870460516</v>
+        <v>18.47367097003595</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.64818065205387</v>
+        <v>13.56058089959401</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01782237796337865</v>
+        <v>0.01793353624589453</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.19038677026824</v>
+        <v>42.10463479162189</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.30891968599801</v>
+        <v>42.22584407313282</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2634604330331481</v>
+        <v>0.2643920045069704</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.207519375116576</v>
+        <v>2.208079755303055</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.4182944075005067</v>
+        <v>0.3806199457930494</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4841104706.173503</v>
+        <v>4744190114.109697</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -5025,13 +5025,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.77</v>
+        <v>28.565</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.009119599054046024</v>
+        <v>0.001929139623872977</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.04100000000000004</v>
+        <v>-0.04783333333333328</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5040,38 +5040,38 @@
         <v>11.25</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>72130322917</v>
+        <v>71616359893</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.65354330708661</v>
+        <v>-22.49212598425197</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-76.06786760072919</v>
+        <v>-76.16780417678686</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.997240008777516</v>
+        <v>1.983008719174858</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.199935136122785</v>
+        <v>2.184259546866436</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1685845083318074</v>
+        <v>0.1673832631386194</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.65856577140496</v>
+        <v>16.57361320545455</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.790649949245466</v>
+        <v>2.776418659642808</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03022307279157082</v>
+        <v>0.03043997214124087</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02162401250814083</v>
+        <v>0.02170058868705182</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3064953506989899</v>
+        <v>0.3087974275185777</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2021918699847645</v>
+        <v>0.2031330585927424</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>585012103.2297961</v>
+        <v>553075022.083438</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>333.2</v>
+        <v>330.85</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1060553478957135</v>
+        <v>-0.1123601796257406</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1401068414668766</v>
+        <v>-0.1461715141035898</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>225013292000</v>
+        <v>223426313500</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>20.20618556701031</v>
+        <v>20.06488781079442</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.27706122316962</v>
+        <v>17.14917182764878</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.676403744365016</v>
+        <v>2.657688195972548</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.590128354725787</v>
+        <v>6.544044924154026</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.252959978391035</v>
+        <v>1.244198283464111</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.659411583886103</v>
+        <v>9.595770089791296</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.840618177060412</v>
+        <v>2.821902628667943</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06689382598784431</v>
+        <v>0.06736489503173368</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1695383437035314</v>
+        <v>0.1700208040626645</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.002563185495058073</v>
+        <v>0.002858557718183441</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01062424969987995</v>
+        <v>0.01069971286081306</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9512041130609026</v>
+        <v>0.95028555459996</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2608809026673605</v>
+        <v>0.2511228769639241</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>905021309.9144491</v>
+        <v>888261846.349703</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>150.72</v>
+        <v>150.38</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2298809727171676</v>
+        <v>-0.2316182369772271</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5640402637972927</v>
+        <v>-0.5650237186162212</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>434144438400</v>
+        <v>433165092665</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>25.37373737373737</v>
+        <v>25.31649831649831</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.16036032751456</v>
+        <v>17.10624231913009</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.445328519255322</v>
+        <v>6.430789106936072</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>10.20448292086196</v>
+        <v>10.18146325397572</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7646410046410039</v>
+        <v>0.7629160979160973</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>17.41734238090787</v>
+        <v>17.3886247312833</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.299599726832744</v>
+        <v>8.285915377534963</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.0545578796017579</v>
+        <v>-0.05467396019665526</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4786249757852497</v>
+        <v>0.4799567224759003</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4821555132075719</v>
+        <v>0.4838188874683502</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01326963906581741</v>
+        <v>0.01329964090969544</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.056899797826053</v>
+        <v>2.052431556064581</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5629553223339963</v>
+        <v>0.5584350966982112</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3833669711.817093</v>
+        <v>3727321366.766129</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30 11:46 ET</t>
+          <t>2026-08-31 14:29 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-01)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,7 +442,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -454,7 +454,7 @@
     <col width="21" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>315.8497</v>
+        <v>316.85</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1654540002900751</v>
+        <v>0.1691450078689654</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.08335113329657262</v>
+        <v>-0.08044809472676084</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4638996986393</v>
+        <v>4653688748600</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>36.04908675799087</v>
+        <v>36.17009132420092</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.34027481722995</v>
+        <v>33.4391884964629</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>9.935500502845832</v>
+        <v>9.968850610616871</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>43.15243035574778</v>
+        <v>43.2972784388951</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.101499873160831</v>
+        <v>1.105197234906138</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>27.79390068753487</v>
+        <v>27.88630360148618</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.03138909445336</v>
+        <v>10.0647392022244</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02946948236419832</v>
+        <v>0.02937089422689028</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08124743888916663</v>
+        <v>0.08166773628573232</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.105810614424442</v>
+        <v>0.1062663150342011</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003356026616457132</v>
+        <v>0.003345431592236074</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3388683428257555</v>
+        <v>0.3358825958320216</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.3074282102969242</v>
+        <v>0.3082595845328544</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15093640739.65532</v>
+        <v>15128292500.53618</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>509.5</v>
+        <v>507.29</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.07730366932351695</v>
+        <v>0.0726307721513777</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.07985985696742037</v>
+        <v>-0.08385104384887665</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3783317725000</v>
+        <v>3766907259500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.30555555555555</v>
+        <v>28.18277777777778</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.02251858481157</v>
+        <v>24.90140120547297</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.40106414556457</v>
+        <v>11.35161105084092</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.556027867003325</v>
+        <v>8.518915361436932</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.899079015210104</v>
+        <v>0.8951791827790652</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.75101087129372</v>
+        <v>18.6719315315706</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.72614136674713</v>
+        <v>11.67668827202348</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01770588802451161</v>
+        <v>0.0177830234155782</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.131203298325723</v>
+        <v>0.1317747762557078</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2161041830633579</v>
+        <v>0.2167318617713074</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007144259077526987</v>
+        <v>0.007175382917069132</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5572735451366373</v>
+        <v>0.5561146595901971</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4308106283244855</v>
+        <v>0.4303995339795346</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>14876725862.83981</v>
+        <v>15250076065.82969</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -953,13 +953,13 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>338.77</v>
+        <v>339.35</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.07494845807064787</v>
+        <v>0.07678885156972104</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1709209270453489</v>
+        <v>-0.169501480629451</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
@@ -968,40 +968,40 @@
         <v>206.2</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4099832240358</v>
+        <v>4106851464904</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.82075471698113</v>
+        <v>16.84955312810328</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.01208894699019</v>
+        <v>20.06410996855315</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.195191033106285</v>
+        <v>9.210933899355636</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.427045762553085</v>
+        <v>6.438049353609793</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1495879500159298</v>
+        <v>0.1498440559609935</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.72096548625588</v>
+        <v>12.74244690230691</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.32268420932251</v>
+        <v>9.338427075571863</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01299394630726358</v>
+        <v>0.0129717377059424</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1594703200881502</v>
+        <v>-0.1602142754145639</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2873851778057901</v>
+        <v>0.2880897960278097</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002509076954866133</v>
+        <v>0.002504788566376897</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.793551365502721</v>
+        <v>0.7872895379001923</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3753838432687253</v>
+        <v>0.3800630215209703</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9516857956.253744</v>
+        <v>9738420777.37315</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>259.43</v>
+        <v>259.77</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1453863134657838</v>
+        <v>0.146887417218543</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.09669220055710304</v>
+        <v>-0.09550835654596102</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2790714453000</v>
+        <v>2794371867000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.58968253968254</v>
+        <v>20.61666666666666</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.97601195789809</v>
+        <v>23.0174675044733</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.597765126082921</v>
+        <v>3.602480232827971</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.058607519669337</v>
+        <v>5.065237156013197</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2330710257030054</v>
+        <v>0.2333764805414552</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.55856574683953</v>
+        <v>11.57254167175203</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.784861056105611</v>
+        <v>3.789437483240512</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004165439393852225</v>
+        <v>-0.004160147808988802</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1038617764731465</v>
+        <v>-0.1043034311806915</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1718555403691431</v>
+        <v>0.172282985723399</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8400815135764711</v>
+        <v>0.8347530088682033</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4466500103571434</v>
+        <v>0.4592387735213114</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>10984779222.78754</v>
+        <v>11315358887.17889</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>219.68</v>
+        <v>220.78</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1632512200162988</v>
+        <v>0.1690759484486455</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.07127758518643779</v>
+        <v>-0.06662720892872243</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5320869280000</v>
+        <v>5347512380000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.63270440251572</v>
+        <v>27.77106918238993</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.88996871402454</v>
+        <v>16.95222647892013</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.56242150186983</v>
+        <v>17.65036152213593</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.20712014813262</v>
+        <v>23.32332477378332</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2218135455440037</v>
+        <v>0.2229242288110212</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.84142082536259</v>
+        <v>22.95544248866977</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.61660856391248</v>
+        <v>17.70454858417858</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02386940804529594</v>
+        <v>0.02375048264965401</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.636042367536831</v>
+        <v>0.6381959748427668</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8847629049148795</v>
+        <v>0.8872362080226031</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001274581209031318</v>
+        <v>0.001268230818008878</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.321297040462333</v>
+        <v>1.324604717909381</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4251949425488812</v>
+        <v>0.4308750567158028</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>26259958471.53905</v>
+        <v>27395329973.83073</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>572.4773</v>
+        <v>572.34</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.1198208458701069</v>
+        <v>-0.1200319434941735</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2760782751643904</v>
+        <v>-0.2762518968133535</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1458378233380</v>
+        <v>1458028463474</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.27377554812337</v>
+        <v>21.26867335562988</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.32594375468154</v>
+        <v>17.31824456768273</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.38944583689671</v>
+        <v>6.387913425195402</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.57309624379357</v>
+        <v>5.57175962116369</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.361123987365288</v>
+        <v>-4.360078037904121</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.525125461185</v>
+        <v>14.5218587816983</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6.813791285706776</v>
+        <v>6.812258874005468</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02809696350516167</v>
+        <v>0.02810370375237239</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2278566668193829</v>
+        <v>0.2281079223998819</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2627496195463912</v>
+        <v>0.2633643791295024</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.00366826771996025</v>
+        <v>0.003669147709403501</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7957129651739591</v>
+        <v>0.7941639390363734</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4951059291372276</v>
+        <v>0.4495885078754943</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9274017500.816952</v>
+        <v>9463197349.872856</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>367.67001</v>
+        <v>367.95</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.160704901379188</v>
+        <v>-0.1600657569609015</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2629352484814466</v>
+        <v>-0.2623739550548283</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1452130143385</v>
+        <v>1453235963622</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>311.6</v>
+        <v>311.8220338983051</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>178.9286109133749</v>
+        <v>178.9321407699298</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.01481564389736</v>
+        <v>14.02480205002944</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.70289502406226</v>
+        <v>13.71265916783716</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.29470422535211</v>
+        <v>-8.30061470518023</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>120.2464401567177</v>
+        <v>120.3324712023612</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.95809824650885</v>
+        <v>13.96808465264093</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.00396776980394071</v>
+        <v>0.003964944540485339</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7414766616103423</v>
+        <v>0.7426831901555608</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1148070506615788</v>
+        <v>0.1151207537331111</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.534351525695682</v>
+        <v>1.550200404454444</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5904894043160188</v>
+        <v>0.5992685959790698</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12854890199.54324</v>
+        <v>12990936492.25119</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>369.57501</v>
+        <v>370.34</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.06315808984293669</v>
+        <v>0.06535874000905273</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2533838181818181</v>
+        <v>-0.2518383838383839</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>287.17</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1758282686576</v>
+        <v>1761922177200</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>59.70517124394185</v>
+        <v>59.82875605815832</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.32175100499205</v>
+        <v>20.33940815676351</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>23.29931341119724</v>
+        <v>23.34754094215862</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>20.0063013589764</v>
+        <v>20.04771276413771</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4741802006040599</v>
+        <v>0.4751617147807357</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>42.91809618560381</v>
+        <v>43.00300243188578</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>23.90025829457364</v>
+        <v>23.94754094215862</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01863219814970771</v>
+        <v>0.01859446485432433</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.937993445017373</v>
+        <v>1.941519025383407</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.167377175775252</v>
+        <v>1.16991366644971</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006872759064526576</v>
+        <v>0.006858562402116974</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.619321127753445</v>
+        <v>1.618200211325754</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4340483793479238</v>
+        <v>0.4308421547694293</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7311912636.807963</v>
+        <v>7475638932.061221</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>943.1508</v>
+        <v>943.89</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1037458162668228</v>
+        <v>0.104610883557636</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1398533515731875</v>
+        <v>-0.1391792065663475</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>418267573633</v>
+        <v>418595393310</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>47.37070818684078</v>
+        <v>47.40783525866399</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.55867252067026</v>
+        <v>41.59124437527429</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.424680158293794</v>
+        <v>1.425796759767973</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.49474268370885</v>
+        <v>12.50453551195201</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.736787560988739</v>
+        <v>3.739716290270507</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.16541628424326</v>
+        <v>28.1880714105045</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.388186716826699</v>
+        <v>1.389303318300878</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02105350869901915</v>
+        <v>0.02103702080992211</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005873928114146752</v>
+        <v>0.005869327993728083</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1818846754016071</v>
+        <v>-0.1816712207877005</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2227719813725588</v>
+        <v>0.2215442051757468</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1695137124.491549</v>
+        <v>1744088776.159326</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>81.36</v>
+        <v>81.05</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1058357851396765</v>
+        <v>-0.1092427530183232</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3579038749901349</v>
+        <v>-0.3603504064399021</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>338778158319</v>
+        <v>337487336919</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>25.18885448916409</v>
+        <v>25.09287925696594</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.74757499972702</v>
+        <v>21.66129741998723</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7.003779355624816</v>
+        <v>6.977093372331271</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.30409605555204</v>
+        <v>11.26102489309849</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7403065770595789</v>
+        <v>0.7374858415766822</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.24253374849552</v>
+        <v>11.20034595894544</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.111490575567506</v>
+        <v>7.084804592273962</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.0324537096917779</v>
+        <v>0.03257783862462017</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1582373892022564</v>
+        <v>0.1584199584375927</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1385080841528432</v>
+        <v>0.1388362707419997</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1092090135095534</v>
+        <v>0.1082254330773223</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3629988129500539</v>
+        <v>0.3544855803856646</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2545143898.212287</v>
+        <v>2532911397.44292</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>504.18</v>
+        <v>504.03</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01475293107867492</v>
+        <v>0.01445102909989382</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06240934280507304</v>
+        <v>-0.06268828802023285</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1087442445527</v>
+        <v>1087118917488</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.67739502137289</v>
+        <v>12.67362333417148</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.72863740593738</v>
+        <v>22.72184879766798</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.826824003740704</v>
+        <v>2.825982987436539</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.448109573500654</v>
+        <v>1.447678742376799</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3488675592202333</v>
+        <v>0.3487637666582851</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.37239518946859</v>
+        <v>15.36816683859163</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.057559640765089</v>
+        <v>3.056718624460925</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02226784516238452</v>
+        <v>0.02227447210278842</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422281109530485</v>
+        <v>-0.4422274592606116</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.05997034272766366</v>
+        <v>0.06001574665701348</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06097128891173814</v>
+        <v>0.0602257652088585</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1552388901332344</v>
+        <v>0.1553845113762773</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2071177146.828511</v>
+        <v>2152366461.077631</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>355.91</v>
+        <v>356.02</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.09349265081274116</v>
+        <v>0.09383061319533592</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.02889495225102312</v>
+        <v>-0.02859481582537526</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>953664404100</v>
+        <v>953959150200</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.30137575236458</v>
+        <v>15.3061049011178</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.22229671857758</v>
+        <v>14.22622755673329</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.204162186652689</v>
+        <v>3.205152487123403</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.649576925130407</v>
+        <v>2.650395821654147</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8011685481063818</v>
+        <v>0.8014161627850693</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.20028316444826</v>
+        <v>20.20200891155002</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.322747745041712</v>
+        <v>6.323287908934829</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.09028637691344638</v>
+        <v>0.09027116096317726</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07587234714189806</v>
+        <v>0.07590749832153509</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2905307890900483</v>
+        <v>-0.2904806428001039</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.0168581944873704</v>
+        <v>0.01685298578731532</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7722713662903462</v>
+        <v>0.7742974247094891</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.188426584703087</v>
+        <v>0.184185884261664</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2209285659.261324</v>
+        <v>2226921013.938838</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>379.66</v>
+        <v>379.37</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.09576306846452143</v>
+        <v>0.09492607934305819</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01532795601317527</v>
+        <v>-0.01608008921855952</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>708843144128</v>
+        <v>708301700437</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>32.25658453695837</v>
+        <v>32.23194562446899</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.51033688889494</v>
+        <v>25.48239117993718</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.93335605394713</v>
+        <v>15.92118549804442</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.65099797202797</v>
+        <v>20.63522388623572</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.175197312525154</v>
+        <v>2.173535806913206</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.75572699594474</v>
+        <v>24.73711940466699</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.19183024923575</v>
+        <v>16.17965969333303</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02964407594835333</v>
+        <v>0.02966673662795901</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2644515310575994</v>
+        <v>0.2648713143468999</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1332391347816126</v>
+        <v>0.133545200943151</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007058947479323605</v>
+        <v>0.007064343516883254</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.2938298127839107</v>
+        <v>0.2950142956159523</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.211694852352617</v>
+        <v>0.2062636822981946</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2500987469.667658</v>
+        <v>2524254104.439449</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>588.41998</v>
+        <v>589.3099999999999</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.04490965655870238</v>
+        <v>0.04649014417662856</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.02194079319171571</v>
+        <v>-0.02046142083042457</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>516065508132</v>
+        <v>516846085160</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32.31301372872048</v>
+        <v>32.36188907193849</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.69615792602793</v>
+        <v>26.72610910939543</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.70984545597583</v>
+        <v>14.73209489382322</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>92.49446130101586</v>
+        <v>92.63436464088397</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.428119803188985</v>
+        <v>1.430279918804424</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.93821252179417</v>
+        <v>23.97350719659974</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>15.09042864441467</v>
+        <v>15.11267808226206</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03187192273232278</v>
+        <v>0.03182378753030159</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2103994072201787</v>
+        <v>0.2108716962680446</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1514506553673307</v>
+        <v>0.1518181202718094</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005727201853342913</v>
+        <v>0.005718552205121244</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2894781718098139</v>
+        <v>0.2889375699579723</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2258120363330918</v>
+        <v>0.2245938102132268</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1669596539.890153</v>
+        <v>1697021571.12912</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>390.56</v>
+        <v>389.41</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.160998832004086</v>
+        <v>0.1575802825960444</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1539361379489623</v>
+        <v>-0.1564273644989385</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>354684878426</v>
+        <v>353640512362</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.1147836152016</v>
+        <v>25.04083338692046</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.1239592235582</v>
+        <v>18.06442033317147</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7879627360734367</v>
+        <v>0.7856425877070795</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.385666743084592</v>
+        <v>3.375697681341078</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7609845009253643</v>
+        <v>-0.7587437897002922</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.50393503963048</v>
+        <v>15.46339759973606</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8873631301826809</v>
+        <v>0.8850429818163237</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06658586660025134</v>
+        <v>0.06678250702177677</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3857228051228707</v>
+        <v>0.3861963420402867</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009282833922202638</v>
+        <v>0.009361298838479026</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02291581319131503</v>
+        <v>0.02298348784057934</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4471898683075785</v>
+        <v>0.4474091914599684</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.238226139112006</v>
+        <v>0.2277731438229457</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1745425434.803818</v>
+        <v>1759496645.182897</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>160.44</v>
+        <v>160.98</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3081124990132795</v>
+        <v>0.3125152710742816</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.09052774786009865</v>
+        <v>-0.08746669689926878</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>664937162400</v>
+        <v>667175170800</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.64864864864865</v>
+        <v>20.71814671814672</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.65583507773566</v>
+        <v>14.70847718466684</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.841625110507949</v>
+        <v>1.847823549548551</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.581743597964377</v>
+        <v>2.590433086513995</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.021846846846848</v>
+        <v>2.028651866151867</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.70193527683954</v>
+        <v>9.731363324747651</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.929988094109012</v>
+        <v>1.935842161413615</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04594011221843604</v>
+        <v>0.04579456990787643</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4089029072124961</v>
+        <v>0.4085854339662556</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08457595414128405</v>
+        <v>0.08441451594332183</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02567938170032411</v>
+        <v>0.02559324139644677</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.530677559549498</v>
+        <v>-0.5279981585317083</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.25753737191427</v>
+        <v>0.2576578945092202</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2197890056.152976</v>
+        <v>2252912919.928731</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>266.15</v>
+        <v>265.85</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.2835784526918681</v>
+        <v>0.2821316237014209</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.03732773899518949</v>
+        <v>-0.03841284768691</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>276.47</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>641394463418</v>
+        <v>640671493894</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>30.76878612716763</v>
+        <v>30.73410404624278</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.51793210884344</v>
+        <v>21.48814399830432</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.549586572087941</v>
+        <v>6.54220398343698</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.642991314683832</v>
+        <v>7.634376257782067</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.809661545482208</v>
+        <v>-3.805367356251908</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>19.86269605769003</v>
+        <v>19.84126330766038</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.841777853526534</v>
+        <v>6.834395264875573</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02916769798776373</v>
+        <v>0.02920061244849964</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4299137097157337</v>
+        <v>0.4302819288938158</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08471040366759963</v>
+        <v>0.08491746894102903</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01983843697163254</v>
+        <v>0.01986082377280421</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1924719394814994</v>
+        <v>-0.1904984860025334</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2428848379956363</v>
+        <v>0.2446526693066723</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1800416386.991852</v>
+        <v>1832718316.395295</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>104.89</v>
+        <v>104.87</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.06979427090398915</v>
+        <v>-0.06997163876157253</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2239567919502812</v>
+        <v>-0.2241047647232909</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>96.51000000000001</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>834723011200</v>
+        <v>834563849600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>37.86642599277979</v>
+        <v>37.85920577617329</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>33.99627106019969</v>
+        <v>33.97965718634212</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.134381130680583</v>
+        <v>1.134164831485105</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.49259003644211</v>
+        <v>8.490970703800972</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.156790285526755</v>
+        <v>9.155044305874638</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>20.93767387660776</v>
+        <v>20.93395853311235</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.218945709936943</v>
+        <v>1.218729410741465</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01618381165816841</v>
+        <v>0.01618689811028211</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1138405716829041</v>
+        <v>0.1141726818653876</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04889636152208499</v>
+        <v>0.0490209438597804</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009319286871961102</v>
+        <v>0.009321064174692476</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.06918265081123934</v>
+        <v>-0.06478809405779103</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3305030499143676</v>
+        <v>0.3147368899221482</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2797469139.435469</v>
+        <v>2866126010.709811</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>145.5</v>
+        <v>145.12</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.02616550454572897</v>
+        <v>0.02348548467131395</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1300448430493274</v>
+        <v>-0.1323168908819132</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>345883900334</v>
+        <v>344980560937</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.55555555555555</v>
+        <v>21.49925925925926</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.64820323248744</v>
+        <v>20.59093801171288</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.974215235017005</v>
+        <v>3.963835841265282</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.489914566109996</v>
+        <v>6.472964961057612</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.57015873015895</v>
+        <v>20.5164359788362</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.45402749289546</v>
+        <v>17.41152540401807</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.262431063677728</v>
+        <v>4.252051669926004</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04600676696612285</v>
+        <v>0.04612723672539339</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04394340334855396</v>
+        <v>0.04411266971080652</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02417283511610258</v>
+        <v>0.02425273124289351</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02948865979381443</v>
+        <v>0.02956587651598677</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06545482494078865</v>
+        <v>-0.06033009602373817</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1973927722769822</v>
+        <v>0.1943360563400797</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1280377468.365578</v>
+        <v>1311998857.473692</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>328.24</v>
+        <v>327.83</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.05083571497278017</v>
+        <v>-0.05202130282575723</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.230837727006444</v>
+        <v>-0.2317984768599883</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>327293684080</v>
+        <v>326884866110</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22.92178770949721</v>
+        <v>22.893156424581</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.89012390220935</v>
+        <v>21.86278125414724</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.934634251194023</v>
+        <v>1.932217726568781</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.63474514051875</v>
+        <v>19.61021965457062</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.86270624918803</v>
+        <v>-7.852885052617936</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16.21474740037633</v>
+        <v>16.19765277482751</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.292143590580224</v>
+        <v>2.289727065954982</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04613898994857744</v>
+        <v>0.04619669359339005</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02821106507433585</v>
+        <v>0.02824634719214227</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.6948781003261235</v>
+        <v>0.6966243977485421</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2590810248754111</v>
+        <v>0.2597822369828832</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1278252612.963029</v>
+        <v>1290113661.321519</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>468.45</v>
+        <v>470.72</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.096254519358731</v>
+        <v>1.106412482340787</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.198861012775127</v>
+        <v>-0.1949788791408</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>763854570000</v>
+        <v>767556032000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>118.8959390862944</v>
+        <v>119.4720812182741</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>35.72602795940384</v>
+        <v>35.83848672229277</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.49302917322358</v>
+        <v>18.58264210144051</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.36561272759729</v>
+        <v>11.42068784957753</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9598938201462299</v>
+        <v>0.9645452428631304</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>71.19281302481807</v>
+        <v>71.53816309012876</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.47341895654279</v>
+        <v>18.56303188475971</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01100078513636437</v>
+        <v>0.01094773495311415</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.327992107642027</v>
+        <v>2.333625165148459</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8542067563338545</v>
+        <v>0.856719908111891</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.533866464625572</v>
+        <v>2.537135416875415</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7230591770296156</v>
+        <v>0.7055039023776581</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>12055560805.04792</v>
+        <v>11958552234.80343</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3347,13 +3347,13 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1692.4912</v>
+        <v>1696.01</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4543050726025588</v>
+        <v>0.4573286680513706</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1537374747494951</v>
+        <v>-0.1519780395607913</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
@@ -3362,13 +3362,13 @@
         <v>716.2</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>652316558089</v>
+        <v>653672766916</v>
       </c>
       <c r="L23" s="6" t="n">
         <v>52.677793904209</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.48923120331378</v>
+        <v>35.53375977982921</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>15.83893112544052</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.484331785110359</v>
+        <v>0.4824717178988647</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2497306326913287</v>
+        <v>0.2479352070364185</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004596774269786455</v>
+        <v>0.004587237103554814</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.704098733360151</v>
+        <v>1.706356147864655</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.462745241956569</v>
+        <v>0.4247375441625872</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2447497732.285026</v>
+        <v>2439705814.951546</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>207.355</v>
+        <v>207.78</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.08962990687764272</v>
+        <v>-0.08776398953985476</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1847650874778848</v>
+        <v>-0.1830941615883624</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>163887171350</v>
+        <v>164223078600</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>77.66104868913854</v>
+        <v>77.82022471910109</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>88.12374475936727</v>
+        <v>87.79113064600118</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.743573289536677</v>
+        <v>1.747146961008564</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>26.8896868077836</v>
+        <v>26.94480058316066</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4156476547803613</v>
+        <v>0.4164995766210772</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.15071210071942</v>
+        <v>29.19051490647482</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.155406660992606</v>
+        <v>2.158349684557689</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001280906058977279</v>
+        <v>-0.001278748406072081</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1187273203016782</v>
+        <v>-0.1135753219434616</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1470038736873935</v>
+        <v>0.147428475839213</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.18708993879337</v>
+        <v>1.186254060752734</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3633737215181797</v>
+        <v>0.3620576711904705</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1285840517.475244</v>
+        <v>1292721574.320933</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1027.47</v>
+        <v>1025.9</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.1237285581093934</v>
+        <v>0.1220114726117811</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1096369985875094</v>
+        <v>-0.1109974956455427</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>721.16</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>303110842290</v>
+        <v>302647681300</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.65310786106033</v>
+        <v>15.62918951858623</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.21165713178468</v>
+        <v>14.18827205052485</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.570108127983584</v>
+        <v>2.566180938127983</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.512129075622036</v>
+        <v>2.508290479216568</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3668871587811437</v>
+        <v>0.3663265459756249</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.32197758385628</v>
+        <v>27.30722394482847</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.272686623281921</v>
+        <v>7.268759433426321</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.136963098008486</v>
+        <v>-0.1371727013459197</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1014273505129684</v>
+        <v>0.1015569382184267</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3829275675492871</v>
+        <v>-0.3828847627451899</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01654549524560328</v>
+        <v>0.01657081586899308</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.565287292138259</v>
+        <v>1.565645635728434</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3885043494438919</v>
+        <v>0.3874958509425507</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1955394265.480473</v>
+        <v>1958130705.804211</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>235.315</v>
+        <v>233.87</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.1927444253859348</v>
+        <v>-0.1977015437392796</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2922005654815617</v>
+        <v>-0.2965469530169043</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>221698264510</v>
+        <v>220336878580</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.55152838427948</v>
+        <v>20.42532751091703</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.28716697758337</v>
+        <v>18.17163752296057</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.208507815245235</v>
+        <v>3.188805282139601</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.419730886450715</v>
+        <v>6.380309212817834</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2505215378626317</v>
+        <v>0.2489831589993569</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.24913781579434</v>
+        <v>17.1652104420196</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.04935474058208</v>
+        <v>4.029652207476446</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06148446867695329</v>
+        <v>0.06186436010098442</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1238224274690438</v>
+        <v>0.1240223939702099</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04438763279987001</v>
+        <v>0.04449515609729504</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02864245798185411</v>
+        <v>0.02881942959763972</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8955247627696769</v>
+        <v>0.8947620175211669</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7907660012059975</v>
+        <v>0.7887762342380554</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1609253190.314244</v>
+        <v>1600910833.31618</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1160.24182</v>
+        <v>1157.83</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07394001604237777</v>
+        <v>0.07170759348628386</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1024315785402082</v>
+        <v>-0.1042973736123468</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1092647293023</v>
+        <v>1090375982030</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.86907269681743</v>
+        <v>38.78827470686767</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.85696834968743</v>
+        <v>26.78377567982369</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.71538719278536</v>
+        <v>13.68687670280095</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.56169899253224</v>
+        <v>30.49816972165648</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4120282654403832</v>
+        <v>0.4111717732901912</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.34109557552261</v>
+        <v>32.2765843566803</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.29302527587748</v>
+        <v>14.26451478589307</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01835349808492855</v>
+        <v>0.01839172939472198</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4472621105527641</v>
+        <v>0.4482004020100503</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2212719878501344</v>
+        <v>0.2217388895693952</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005766039358932952</v>
+        <v>0.005778050318267795</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3536655920196939</v>
+        <v>0.3532013780018772</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3419295785425133</v>
+        <v>0.3420660841772869</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3114858505.854932</v>
+        <v>3167756947.91613</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>213.58</v>
+        <v>213.44</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1741616666658279</v>
+        <v>0.1733920129841477</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.08038751345532824</v>
+        <v>-0.08099031216361685</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>145.66</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>336875462400</v>
+        <v>336654643200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.16881028938907</v>
+        <v>17.15755627009646</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.93374890252323</v>
+        <v>15.92082054187868</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.662436772597586</v>
+        <v>2.660691566360281</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.038790947046198</v>
+        <v>3.036799043625529</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4368019255961378</v>
+        <v>0.4365156053902035</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.89741583126044</v>
+        <v>23.88989140968413</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.542740892601697</v>
+        <v>5.540995686364391</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04655726448065575</v>
+        <v>-0.04658780241650325</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07751229132713733</v>
+        <v>0.0776804012685548</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3294448977552712</v>
+        <v>-0.329347782333272</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01943065830133908</v>
+        <v>0.01944340329835083</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.366208372122312</v>
+        <v>1.367332780534712</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2950828807786875</v>
+        <v>0.2934188278182759</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>985046275.9182591</v>
+        <v>981176068.9368185</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4105,13 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>945.8108999999999</v>
+        <v>958.73</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.998576056483156</v>
+        <v>2.039534459406311</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2463658167330678</v>
+        <v>-0.2360717131474104</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
@@ -4120,31 +4120,31 @@
         <v>114.25</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1068189372351</v>
+        <v>1082780074700</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>21.10713903146619</v>
+        <v>21.39544744476679</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.086547938091421</v>
+        <v>6.169685826930508</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.8327466640561</v>
+        <v>11.99437351507632</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.59206043445455</v>
+        <v>10.73674039950757</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03008386210757165</v>
+        <v>0.03049478613366812</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.35761379378457</v>
+        <v>15.57020271413104</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.62717363083501</v>
+        <v>11.78812365354366</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02449987215304038</v>
+        <v>0.02417111342508896</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005603657136960464</v>
+        <v>0.00055281466106203</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885107848555588</v>
+        <v>2.888414684894863</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8927227174626965</v>
+        <v>0.8538983120639434</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>32837560703.50714</v>
+        <v>32638999293.26419</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>149.1</v>
+        <v>147.99</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>0.01119025490612247</v>
+        <v>0.003662279165372651</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2343087209720325</v>
+        <v>-0.2400090383410536</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>154148824200</v>
+        <v>153001237380</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>92.60869565217392</v>
+        <v>91.91925465838511</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>31.70991603449167</v>
+        <v>31.4565031202132</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>10.46353680423568</v>
+        <v>10.38563924653815</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>12.30587248322148</v>
+        <v>12.21425934803452</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>148.1739130434814</v>
+        <v>147.0708074534193</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>45.89266306678131</v>
+        <v>45.55782097449126</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.86882306815096</v>
+        <v>10.78952195085528</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.02970756185381097</v>
+        <v>0.02993439842989589</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.920496400918915</v>
+        <v>1.922106577044159</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2374543403235527</v>
+        <v>0.2380188269553931</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6465476363151583</v>
+        <v>0.660038133031976</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6053777558464245</v>
+        <v>0.5749625578803566</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2587350206.353087</v>
+        <v>2693216271.193902</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.669</v>
+        <v>28.46</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1385623372731672</v>
+        <v>0.1302620990894114</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.002817391304347772</v>
+        <v>-0.01008695652173908</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>28.75</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>163397245360</v>
+        <v>162206062400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.8818710359408</v>
+        <v>37.60570824524314</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.817756150782568</v>
+        <v>9.746924779504434</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.565266976890229</v>
+        <v>2.546565913087164</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.917885092146966</v>
+        <v>1.90390350980162</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6335994359108683</v>
+        <v>-0.6289804299425622</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.87193008238276</v>
+        <v>17.77757148288973</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.542063008038181</v>
+        <v>3.523361944235117</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06723491559356114</v>
+        <v>0.06772866462234028</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858506002201049</v>
+        <v>2.858212625619045</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04915415034521853</v>
+        <v>-0.04926294725291902</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.05999511667654958</v>
+        <v>0.06043569922698524</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3154425646430467</v>
+        <v>0.3250888534795566</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2205305669275092</v>
+        <v>0.2165251373763786</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>990544065.1657573</v>
+        <v>1001701835.612195</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>163.22</v>
+        <v>164.58</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.02851017596242489</v>
+        <v>-0.02041541943325498</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1621149897330596</v>
+        <v>-0.1551334702258726</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,13 +4498,13 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1158625153090</v>
+        <v>1168279179608</v>
       </c>
       <c r="L32" s="6" t="n">
         <v>7.314181770262687</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003501262366242842</v>
+        <v>0.003527740869810874</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.281615606810814</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2088.012763162744</v>
+        <v>2072.33305936805</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2716.246769045153</v>
+        <v>2696.953922599575</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.838010047788261</v>
+        <v>1.822821728034998</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.250089076155815</v>
+        <v>1.233272555151941</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>4362892337.018143</v>
+        <v>4249913978.192619</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4611,13 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>555.45</v>
+        <v>556.63</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4879454009198929</v>
+        <v>0.4911063975408048</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1732283464566929</v>
+        <v>-0.1714719497491926</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
@@ -4626,7 +4626,7 @@
         <v>281.74</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>70009333477</v>
+        <v>70158061559</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.821709830202796</v>
+        <v>1.823443357096683</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.452768815330494</v>
+        <v>0.4362465239922472</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5380917547.426866</v>
+        <v>5392250385.431046</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>142.455</v>
+        <v>143.69</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1149114464052443</v>
+        <v>-0.1072382558279427</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3686624711930507</v>
+        <v>-0.3631891508597767</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1862722411540</v>
+        <v>1878871105361</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-92.50324675324676</v>
+        <v>-93.3051948051948</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>138.5232177109974</v>
+        <v>139.0683583910057</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>112.3814426268477</v>
+        <v>113.3557227970437</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.566026221467649</v>
+        <v>6.622949757907313</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9250324675324676</v>
+        <v>-0.933051948051948</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>434.0207371106312</v>
+        <v>437.8961135975522</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>109.1139916464555</v>
+        <v>110.0882718166516</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01525884899645427</v>
+        <v>-0.01512770084062733</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.029565073658547</v>
+        <v>4.039512386619558</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.8201398327787764</v>
+        <v>0.7978344941609902</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12892413081.41169</v>
+        <v>13005980475.6423</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>766.63</v>
+        <v>767.05</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1221658140399</v>
+        <v>0.1227805951492964</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.0163465363049643</v>
+        <v>-0.01580763950370179</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>816643581198</v>
+        <v>817090981253</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9955221199801183</v>
+        <v>0.9955996348636899</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1133565438265974</v>
+        <v>0.1127049040687387</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32453750955.4978</v>
+        <v>32624730430.68662</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -4897,13 +4897,13 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>415.595</v>
+        <v>415.32</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3003191985471185</v>
+        <v>0.2994587748663704</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1323695198329853</v>
+        <v>-0.1329436325678497</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
@@ -4912,13 +4912,13 @@
         <v>225.63</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2155475155600</v>
+        <v>2154048873600</v>
       </c>
       <c r="L36" s="6" t="n">
         <v>27.87759360148371</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6460368027082123</v>
+        <v>0.6451575109854464</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.04516031106463</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.15171130285415</v>
+        <v>42.21052320835893</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.27305287511633</v>
+        <v>42.33494484425928</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2646807589119214</v>
+        <v>0.2648560146393142</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.210114709465739</v>
+        <v>2.209079795546562</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.4197998216084086</v>
+        <v>0.3806996315702489</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4783986757.94904</v>
+        <v>4776626496.386209</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -5025,13 +5025,13 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.595</v>
+        <v>28.53</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.002981401979508025</v>
+        <v>0.0007015002089654221</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.04683333333333339</v>
+        <v>-0.04899999999999993</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
@@ -5040,38 +5040,38 @@
         <v>11.25</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>71691573994</v>
+        <v>71528610108</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.51574803149606</v>
+        <v>-22.46456692913386</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-76.24779836986592</v>
+        <v>-76.72664063579992</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.985091346919563</v>
+        <v>1.980578986792192</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.186553535538096</v>
+        <v>2.181583226749498</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1675590551181103</v>
+        <v>0.1671781724958799</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.58604528826446</v>
+        <v>16.55910910876033</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.778501287387512</v>
+        <v>2.773988927260141</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03040803651740787</v>
+        <v>0.03047731525481133</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02170058868705182</v>
+        <v>0.02177716486596282</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.308092453870339</v>
+        <v>0.3081680947970383</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2037820980318145</v>
+        <v>0.2034762496937432</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>584600977.3994473</v>
+        <v>570134183.4238789</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>331.295</v>
+        <v>330.17</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1111662859577142</v>
+        <v>-0.1141845564667698</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1450230973702546</v>
+        <v>-0.1479263981005962</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>223726826450</v>
+        <v>222967102700</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>20.09066100667071</v>
+        <v>20.02243784111583</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.17223781363429</v>
+        <v>17.10790420251081</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.661101976258728</v>
+        <v>2.652065499030604</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.552450700116687</v>
+        <v>6.530200116686115</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.245796446701855</v>
+        <v>1.241566014601945</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.607378516825756</v>
+        <v>9.576650327616891</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.825316408954123</v>
+        <v>2.816279931726</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06727847634026993</v>
+        <v>0.06750771668882613</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1699500801648157</v>
+        <v>0.1703618166260996</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.002797938226678065</v>
+        <v>0.003032690958297835</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01068534085935496</v>
+        <v>0.0107217494018233</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9520650383382436</v>
+        <v>0.950834925831435</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2615896214207884</v>
+        <v>0.2514690247573396</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>896816288.3192037</v>
+        <v>904950526.8828114</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>149.97</v>
+        <v>149.07</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2337131732908282</v>
+        <v>-0.238311813979221</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5662096494272822</v>
+        <v>-0.5688129121832697</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>431984085900</v>
+        <v>429391662900</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>25.24747474747474</v>
+        <v>25.09595959595959</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.05960340869757</v>
+        <v>16.94197998454674</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.413255825588646</v>
+        <v>6.374768593188634</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>10.15370424390703</v>
+        <v>10.09276983156112</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7608360633360626</v>
+        <v>0.7562701337701331</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>17.35003538960028</v>
+        <v>17.26926700003116</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.267527033166068</v>
+        <v>8.229039800766056</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05483072356856005</v>
+        <v>-0.05516176033794157</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4799567224759003</v>
+        <v>0.4812884691665511</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4838188874683502</v>
+        <v>0.4854822617291292</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01333600053344002</v>
+        <v>0.0134165157308647</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.055820037350564</v>
+        <v>2.05517645380122</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5636412102141967</v>
+        <v>0.5592225486762452</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3796323753.188751</v>
+        <v>3762642485.660867</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:35 ET</t>
+          <t>2026-08-31 20:02 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-02)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>325.13</v>
+        <v>325.865</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1996973849090633</v>
+        <v>0.2024094618564634</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.0564181443538323</v>
+        <v>-0.05428505093304692</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4775300056280</v>
+        <v>4786095262940</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.11529680365297</v>
+        <v>37.19920091324201</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.31340191845227</v>
+        <v>34.37871616077117</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.22935899962084</v>
+        <v>10.25248383849982</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>44.42873327706474</v>
+        <v>44.52917039132255</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.13407851344495</v>
+        <v>1.136642250126838</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.60809240103035</v>
+        <v>28.67521474042353</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.32524759122837</v>
+        <v>10.349473420879</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02862291340629959</v>
+        <v>0.02855528692874742</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08165599236879983</v>
+        <v>0.08204159629699137</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1062662899133076</v>
+        <v>0.107043275770738</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003260234367791345</v>
+        <v>0.003252880794193915</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3303635228013043</v>
+        <v>0.3307612779529245</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2928724957568901</v>
+        <v>0.2914090115468013</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15251421637.28593</v>
+        <v>14976121907.58242</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>501.02</v>
+        <v>495.67</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05937327655440328</v>
+        <v>0.04806105941822891</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.09517445640395872</v>
+        <v>-0.1048363793975294</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3720349061000</v>
+        <v>3680622368500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.83444444444444</v>
+        <v>27.53333388888889</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.59362501126785</v>
+        <v>24.31872947027598</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.21130747440777</v>
+        <v>11.09002445560046</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.413623320757615</v>
+        <v>8.32260548861065</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8841149523072941</v>
+        <v>0.8745506750322232</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.44757521479961</v>
+        <v>18.25363424709063</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.53638469559033</v>
+        <v>11.41510167678302</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01800556853716152</v>
+        <v>0.01820248151208522</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1317747762557078</v>
+        <v>0.1321863637054728</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2167318617713074</v>
+        <v>0.2171876363138756</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007265179034769071</v>
+        <v>0.007343595537353481</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5637281020202041</v>
+        <v>0.563922101532554</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4322154578135036</v>
+        <v>0.4325025820054645</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15259844174.10402</v>
+        <v>15013994600.22096</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -953,55 +953,55 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>335.02</v>
+        <v>337.0872</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.06304936217146873</v>
+        <v>0.06960877844954427</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1800983823205502</v>
+        <v>-0.1750392795085779</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>206.2</v>
+        <v>224.79</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4054449323036</v>
+        <v>4079466807486</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.63455809334657</v>
+        <v>16.73719960278054</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>19.80809819261728</v>
+        <v>19.94795046062082</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.09340525994523</v>
+        <v>9.149515006685849</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.355901854858856</v>
+        <v>6.395120171121659</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1479320926125005</v>
+        <v>0.1488448895256656</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.58207702041266</v>
+        <v>12.65863975016985</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.220898436161455</v>
+        <v>9.277008182902076</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.0131393922467648</v>
+        <v>0.01305881442698387</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1602142754145639</v>
+        <v>-0.1609564282896437</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2880897960278099</v>
+        <v>0.2887944220759853</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002537161960479972</v>
+        <v>0.002521602718821717</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7963503175593711</v>
+        <v>0.8013908496021929</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3810516581329303</v>
+        <v>0.3783381122307395</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9705132742.325422</v>
+        <v>9382822578.452536</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>254.92</v>
+        <v>255.025</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1254746136865341</v>
+        <v>0.1259381898454746</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1123955431754875</v>
+        <v>-0.1120299442896935</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2742199932000</v>
+        <v>2743329427500</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.23174603174603</v>
+        <v>20.24007936507936</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.58841885542202</v>
+        <v>22.56025436213956</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.535220621905941</v>
+        <v>3.5366767578125</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.970667343461078</v>
+        <v>4.972714731155505</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2290192571106277</v>
+        <v>0.2291135887519136</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.36713792682591</v>
+        <v>11.37222008133954</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.722177872318482</v>
+        <v>3.723842027640264</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004239297020010283</v>
+        <v>-0.004237302369593089</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.104331021961296</v>
+        <v>-0.102843476842792</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1722662372499426</v>
+        <v>0.1728287394827941</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8506013389380439</v>
+        <v>0.850369530653322</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4619422654825733</v>
+        <v>0.4617783350798591</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11359887463.36619</v>
+        <v>11163633800.95411</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>217.44</v>
+        <v>226.45</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1513899548449744</v>
+        <v>0.1990997759135598</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.08074744229305819</v>
+        <v>-0.04265663312758938</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5266614240000</v>
+        <v>5484845376083</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>27.35094339622641</v>
+        <v>28.48490566037735</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>16.69577011312797</v>
+        <v>17.31988053983072</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.38334364241886</v>
+        <v>18.10405208123603</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>22.97048527408028</v>
+        <v>23.92283500157216</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.2195517905275317</v>
+        <v>0.2286543447567706</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>22.60923125644614</v>
+        <v>23.54213577441401</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.43753070446151</v>
+        <v>18.15703996118415</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02411530334524748</v>
+        <v>0.02315682546984019</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6381959748427668</v>
+        <v>0.6446363815772465</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8867365359439416</v>
+        <v>0.893902735711656</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001287711552612215</v>
+        <v>0.001236476043276662</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.312059712922509</v>
+        <v>1.307166794685703</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4311771723267008</v>
+        <v>0.4410854715126115</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27428233226.15511</v>
+        <v>26990170627.85485</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>578.54</v>
+        <v>593.7289</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.1104994943374902</v>
+        <v>-0.08714668514459556</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2684117349519474</v>
+        <v>-0.2492047293879616</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1473822880208</v>
+        <v>1512516398971</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>21.49907097733185</v>
+        <v>22.06350427350427</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.50583936816132</v>
+        <v>17.96172918655641</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.45711191426869</v>
+        <v>6.626635935346641</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.632116943124787</v>
+        <v>5.779981673372355</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.407309550353025</v>
+        <v>-4.523018376068372</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>14.66937089255828</v>
+        <v>15.03074939266101</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6.881457363078757</v>
+        <v>7.050981384156707</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02780252671489065</v>
+        <v>0.02709127651632533</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2281085485357075</v>
+        <v>0.2283619268693717</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2633644030509952</v>
+        <v>0.2639791625992733</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003629826805406714</v>
+        <v>0.003536967797929325</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7906036937577582</v>
+        <v>0.7894580502743576</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4336253718548668</v>
+        <v>0.432198020224356</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9565963612.63349</v>
+        <v>9499950691.291113</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>356.09</v>
+        <v>354.0724</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.1871390552961203</v>
+        <v>-0.1917447118493357</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2861495900406953</v>
+        <v>-0.2901942545556602</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1406394331529</v>
+        <v>1398425724707</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>301.771186440678</v>
+        <v>300.0613559322034</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.1646854375983</v>
+        <v>172.0560036212107</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.57274565020894</v>
+        <v>13.49584269976549</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.27066395726358</v>
+        <v>13.19547259665201</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.033063977082833</v>
+        <v>-7.987548770589636</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>116.4380887536581</v>
+        <v>115.7755840295145</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.51602825282043</v>
+        <v>13.43912530237698</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004097001723361388</v>
+        <v>0.004120347543811997</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7426831901555608</v>
+        <v>0.7439749245414444</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1151207537331109</v>
+        <v>0.1154889909686263</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.541163743600746</v>
+        <v>1.535608437502632</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5745367878700262</v>
+        <v>0.5493044939305041</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13012477293.51283</v>
+        <v>12831641165.57021</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1583,55 +1583,55 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>369.68</v>
+        <v>370.96</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.06346011504710991</v>
+        <v>0.06714229679148409</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2531717171717172</v>
+        <v>-0.2505858585858586</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>287.17</v>
+        <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1758782174400</v>
+        <v>1764871876800</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>59.7221324717286</v>
+        <v>59.92891760904685</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.30316035910875</v>
+        <v>20.34906958354759</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>23.30593221228384</v>
+        <v>23.38662793082886</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>20.0119848102998</v>
+        <v>20.08127538743998</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4743149071667721</v>
+        <v>0.4759572007211257</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>42.92828493515765</v>
+        <v>43.07319159547888</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>23.90593221228384</v>
+        <v>23.98662793082886</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.01862766207030532</v>
+        <v>0.01856338719579058</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.941519025383407</v>
+        <v>1.945044605749441</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>1.16991366644971</v>
+        <v>1.172450157124168</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.1636376829390817</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.00687080718459208</v>
+        <v>0.006847099417726979</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.609389729946287</v>
+        <v>1.603662859864755</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4265013898893932</v>
+        <v>0.4169085337845793</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7486778268.044932</v>
+        <v>7360915367.377526</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>939.96</v>
+        <v>932.8543</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1000117027501464</v>
+        <v>0.09169607957870096</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1427633378932969</v>
+        <v>-0.1492436844505244</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,31 +1724,31 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>416852520840</v>
+        <v>413701292110</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>47.21044701155198</v>
+        <v>46.85355600200904</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>41.418074206722</v>
+        <v>41.10497108542885</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.419860282778188</v>
+        <v>1.409126739637654</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.45247136828912</v>
+        <v>12.35833595209943</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.724145529884484</v>
+        <v>3.695992564979913</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>28.06762410780926</v>
+        <v>27.84984741603317</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.383366841311094</v>
+        <v>1.372633298170559</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02112497720358034</v>
+        <v>0.02128588952450879</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.00589386782416273</v>
+        <v>0.005938762355493243</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1787493202257051</v>
+        <v>-0.1803837475494556</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2213029344755717</v>
+        <v>0.2103770311338914</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1746617633.765015</v>
+        <v>1707906327.221568</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>80.81</v>
+        <v>82.3828</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.1118804055695336</v>
+        <v>-0.09459498918393483</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.362244495304238</v>
+        <v>-0.3498318996132901</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>336487991319</v>
+        <v>343037036150</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>25.01857585139319</v>
+        <v>25.50551083591332</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>21.59715539184662</v>
+        <v>22.01403002903983</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6.956433256233042</v>
+        <v>7.091825883709425</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.22767947700541</v>
+        <v>11.44620310380203</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7353020463641171</v>
+        <v>0.749613184323794</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.16768444445505</v>
+        <v>11.38172623604938</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.064144476175733</v>
+        <v>7.199537103652116</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03267459250745387</v>
+        <v>0.03205078997706936</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1584199584375927</v>
+        <v>0.1586025276729295</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1388362707419997</v>
+        <v>0.1391644573311563</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1146826964306175</v>
+        <v>0.1098216379088069</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3374245382787057</v>
+        <v>0.3356765575952403</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2465161407.827324</v>
+        <v>2384799763.566264</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>502.33</v>
+        <v>507.15</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01102947334037596</v>
+        <v>0.02073059025853863</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06584966712537665</v>
+        <v>-0.05688622754491024</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1083452266376</v>
+        <v>1093848300704</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.63087754588886</v>
+        <v>12.75207442796077</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.64521220271126</v>
+        <v>22.86247277744424</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.816451469314014</v>
+        <v>2.843476126575632</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.442795989639778</v>
+        <v>1.456640029752978</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3475874509562056</v>
+        <v>0.3509226519468073</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.32024552860914</v>
+        <v>15.45611653689521</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.0471871063384</v>
+        <v>3.074211763600017</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02234985402817594</v>
+        <v>0.02213743897066462</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422274592606116</v>
+        <v>-0.4422268075681746</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06001574665701348</v>
+        <v>0.06006115058636352</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06134992242713064</v>
+        <v>0.06713928947968452</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1554360546171267</v>
+        <v>0.1521804515928159</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2142200896.007302</v>
+        <v>2097784524.62683</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>354.95</v>
+        <v>358.38501</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.09054316092827519</v>
+        <v>0.1010968351449826</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.03151432469304227</v>
+        <v>-0.02214185538881308</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>951092074500</v>
+        <v>960296217517</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.26010318142735</v>
+        <v>15.40778202923474</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.18347135347026</v>
+        <v>14.32026329319512</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.195519564362823</v>
+        <v>3.226444035160752</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.642430191832311</v>
+        <v>2.668002171359698</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.7990075472741991</v>
+        <v>0.806739900887278</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.17123308823529</v>
+        <v>20.27003239069343</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.313654986174248</v>
+        <v>6.344579456972177</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.09054328419808529</v>
+        <v>0.08967545474943571</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07590749832153509</v>
+        <v>0.07594264950117213</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2904806428001039</v>
+        <v>-0.2904304965101593</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01690378926609382</v>
+        <v>0.01674177164943366</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7711795114447989</v>
+        <v>0.7752808388049121</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1830527146838056</v>
+        <v>0.1841453839601632</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2242526498.243172</v>
+        <v>2190688985.781352</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>372.67</v>
+        <v>379.28</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.07558874446787445</v>
+        <v>0.0946663240984662</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.03345695982571251</v>
+        <v>-0.01631350986850644</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>695792484123</v>
+        <v>708133666188</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>31.66270178419711</v>
+        <v>32.22429906542056</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.0323502676205</v>
+        <v>25.48851989973036</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.64000368915213</v>
+        <v>15.91740842896961</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.27078811103531</v>
+        <v>20.63032848030019</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.135149297947504</v>
+        <v>2.173020167240532</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.30721988188192</v>
+        <v>24.73134463495773</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>15.89847788444075</v>
+        <v>16.17588262425823</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.03020009626359429</v>
+        <v>0.02967377629864209</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2648713143468999</v>
+        <v>0.2642671756613635</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.133545200943151</v>
+        <v>0.1338512671046894</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007191348914589315</v>
+        <v>0.00706601982704071</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3020709532900788</v>
+        <v>0.3101743644077155</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.210918661256638</v>
+        <v>0.2016301631788038</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2535338904.984746</v>
+        <v>2482937536.902624</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>581.1</v>
+        <v>588.615</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.0319109174815273</v>
+        <v>0.04525597090584954</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.03410790864665403</v>
+        <v>-0.02161663508526979</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>509645619600</v>
+        <v>516236545140</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>31.91103789126853</v>
+        <v>32.32372322899506</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.35377306251326</v>
+        <v>26.68418188460748</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.52685402046575</v>
+        <v>14.71472066641963</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>91.3438246301907</v>
+        <v>92.52511673498485</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.4103539068016</v>
+        <v>1.428593124852906</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.64792998733948</v>
+        <v>23.94594615391572</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>14.9074372089046</v>
+        <v>15.09530385485848</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03227340600495961</v>
+        <v>0.03186136308025114</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2108716962680446</v>
+        <v>0.2113439853159109</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1518181202718094</v>
+        <v>0.1521855851762886</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005799346067802444</v>
+        <v>0.005725304316063981</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2945730197856485</v>
+        <v>0.3025976452454281</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2266498070222247</v>
+        <v>0.2160093790181953</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1723618175.366557</v>
+        <v>1684023603.606299</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>396.3</v>
+        <v>400.66</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.178061852527702</v>
+        <v>0.1910226137616682</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1415016680386465</v>
+        <v>-0.132056669988302</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>359897627305</v>
+        <v>363857136907</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.48389171114398</v>
+        <v>25.76233039675905</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.38404195587132</v>
+        <v>18.57995181413678</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.7995433027087789</v>
+        <v>0.808279165694723</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.435425364308746</v>
+        <v>3.472961048960416</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7721685726052896</v>
+        <v>-0.7806053374788219</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.70626973974304</v>
+        <v>15.85890201354656</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.8989436968180232</v>
+        <v>0.9076795598039672</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.0656214384541787</v>
+        <v>0.06491220342795662</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3861963420402865</v>
+        <v>0.3865660500345043</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009361298838478804</v>
+        <v>0.009364180485202267</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02258390108503659</v>
+        <v>0.02233814206559177</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4398711849632869</v>
+        <v>0.4538890665971236</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2340655106562975</v>
+        <v>0.2360994298408964</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1777362601.623405</v>
+        <v>1691719098.761708</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>164.57</v>
+        <v>163.37</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3417855519983508</v>
+        <v>0.3320016140850131</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.06711637662264047</v>
+        <v>-0.07391871209115131</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>682053782200</v>
+        <v>677080430200</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.18018018018018</v>
+        <v>21.02574002574003</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.0364895656642</v>
+        <v>14.93021258183708</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.889031690577743</v>
+        <v>1.875257381598626</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.648202093723494</v>
+        <v>2.628892119168787</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.073892642642644</v>
+        <v>2.058770377520379</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.938514197006613</v>
+        <v>9.869271565610861</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.977050302442807</v>
+        <v>1.96327599346369</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04479558767557847</v>
+        <v>0.04512462425029044</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4085854339662558</v>
+        <v>0.4082679607200155</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08441451594332183</v>
+        <v>0.08425307774536028</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02503493953940572</v>
+        <v>0.02521882842627165</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5399618440265002</v>
+        <v>-0.5405995684318105</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2623209021937768</v>
+        <v>0.2638438564778737</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2255002713.532426</v>
+        <v>2209672319.518654</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2717,55 +2717,55 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>271.19</v>
+        <v>274.795</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3078851797313835</v>
+        <v>0.3252712414332593</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.01909791297428298</v>
+        <v>-0.02232539936670574</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>276.47</v>
+        <v>281.07</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>653540351435</v>
+        <v>662228035225</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.3514450867052</v>
+        <v>31.76820809248555</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>21.91976592401786</v>
+        <v>22.20543445600581</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.673614061565011</v>
+        <v>6.762328168622165</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.78772427063351</v>
+        <v>7.891248537736404</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.881803924551269</v>
+        <v>-3.933405765135388</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.22276625859718</v>
+        <v>20.48067368424641</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>6.965805343003605</v>
+        <v>7.05464249320426</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02862562343537355</v>
+        <v>0.02824957357873411</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4302819288938158</v>
+        <v>0.4306501480718981</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08491746894102903</v>
+        <v>0.0851245342144582</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01946974445960397</v>
+        <v>0.01921432340471988</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1955234527979963</v>
+        <v>-0.1920420508179143</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2343157339533922</v>
+        <v>0.2344665190527604</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1822927009.082621</v>
+        <v>1801240484.992812</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2843,55 +2843,55 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>105.92</v>
+        <v>105.9338</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.06065982623844535</v>
+        <v>-0.06053744241671277</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2163361941402782</v>
+        <v>-0.2162340929269014</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>96.51000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>842919833600</v>
+        <v>843029655104</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.23826714801444</v>
+        <v>38.24324909747293</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.30327427826553</v>
+        <v>34.29448741773891</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.145520539247663</v>
+        <v>1.145669785692542</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.575985667460657</v>
+        <v>8.577103006983041</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.246708237610772</v>
+        <v>9.247912963570732</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.12901406662154</v>
+        <v>21.13157765363337</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.230085118504023</v>
+        <v>1.230234364948902</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01602643509087315</v>
+        <v>0.01602434732658778</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.11471187379457</v>
+        <v>0.1151427525839475</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04921059132838201</v>
+        <v>0.04933020365737639</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009228663141993958</v>
+        <v>0.009227460923708958</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.07078697263836657</v>
+        <v>-0.06728357020486131</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.307946188431454</v>
+        <v>0.3070550904374058</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2861442837.942438</v>
+        <v>2792470569.241409</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.21</v>
+        <v>147.37</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03117291010055689</v>
+        <v>0.0393540234014027</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1257997010463378</v>
+        <v>-0.118863976083707</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>347571718679</v>
+        <v>350329281046</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.66074074074074</v>
+        <v>21.83259259259259</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.74559706927053</v>
+        <v>20.90672104476824</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>3.993608312792996</v>
+        <v>4.025292777897785</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.52158356502366</v>
+        <v>6.573324464657252</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.67053544973567</v>
+        <v>20.83453121693144</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.53343929043945</v>
+        <v>17.66318250898654</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.281824141453718</v>
+        <v>4.313508606558507</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04578335677160332</v>
+        <v>0.04542298021018273</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04411266971080674</v>
+        <v>0.04428583257229834</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02425273124289351</v>
+        <v>0.02433254703733612</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02934546200670269</v>
+        <v>0.02911447377349529</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.06603947522871999</v>
+        <v>-0.05956730932319696</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1965853340458698</v>
+        <v>0.1859723755958249</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1326551486.961515</v>
+        <v>1299873187.263528</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>319.77</v>
+        <v>319.5</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.07532822500867031</v>
+        <v>-0.07610897798502092</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2506854130052725</v>
+        <v>-0.2513181019332161</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>318848103090</v>
+        <v>318578881500</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22.33030726256983</v>
+        <v>22.31145251396648</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.32526480687754</v>
+        <v>21.30725867278786</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.884712388814016</v>
+        <v>1.883121018938857</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.12808449178552</v>
+        <v>19.1119335620148</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.659814700532707</v>
+        <v>-7.653347083279233</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.86159745306293</v>
+        <v>15.8503400167259</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.242221728200218</v>
+        <v>2.240630358325058</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04736110973737705</v>
+        <v>0.04740113321039455</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02895831378803515</v>
+        <v>0.02898278560250391</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7048501383405112</v>
+        <v>0.705482031627267</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2651181757932175</v>
+        <v>0.2592775289006641</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1293083664.792889</v>
+        <v>1267530198.892944</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>459.61</v>
+        <v>458.4861</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.056696637084996</v>
+        <v>1.051667326690488</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.2139791014656337</v>
+        <v>-0.2159011851623827</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>749440066000</v>
+        <v>747607434660</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>116.6522842639594</v>
+        <v>116.3670304568528</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>34.99262169109657</v>
+        <v>34.84827485829913</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.14405195496913</v>
+        <v>18.09968368623653</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.15113516006188</v>
+        <v>11.12386690913959</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9417799096539839</v>
+        <v>0.939476943137894</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>69.84792554581078</v>
+        <v>69.67693922933383</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.12444173828834</v>
+        <v>18.08007346955575</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01121237091692933</v>
+        <v>0.01123985612023983</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.333625165148459</v>
+        <v>2.339247952159099</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8567199081118908</v>
+        <v>0.8592330598899269</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.528671010922055</v>
+        <v>2.52583514583559</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.7002272867255939</v>
+        <v>0.6798523207329189</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>11682170744.7521</v>
+        <v>11317267206.72933</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1665.14</v>
+        <v>1675.78</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4308030367268232</v>
+        <v>0.4399456579543315</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1674133482669653</v>
+        <v>-0.1620932418648373</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>716.2</v>
+        <v>729.5599999999999</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>641774913534</v>
+        <v>645875760958</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>52.08272859216255</v>
+        <v>52.27140783744557</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>34.86895497071953</v>
+        <v>35.02110681735682</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.6600094623452</v>
+        <v>15.71674072139268</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.34675928047137</v>
+        <v>25.43858256893344</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.545461665919734</v>
+        <v>3.558305751653873</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>39.73642538889492</v>
+        <v>39.87602406722446</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.5273224621329</v>
+        <v>15.58187174965678</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01807913230178801</v>
+        <v>0.01801637496944352</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.493670476671811</v>
+        <v>0.4925686989292788</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2572722695527565</v>
+        <v>0.2559520925200618</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004672279808304407</v>
+        <v>0.004642614185632959</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.705710283227658</v>
+        <v>1.702803320714526</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4266194987997516</v>
+        <v>0.4161001381906129</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2419647345.744682</v>
+        <v>2345506440.459701</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>205.66</v>
+        <v>209.47</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.09707162426011418</v>
+        <v>-0.08034422412606301</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1914291330843326</v>
+        <v>-0.1764497739335561</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>162547494200</v>
+        <v>165558804865</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>77.02621722846439</v>
+        <v>78.45318352059923</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>86.89538901076428</v>
+        <v>87.99375936579946</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.729320646842917</v>
+        <v>1.761357570775041</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>26.66988010363279</v>
+        <v>27.1639588899541</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4122499900273883</v>
+        <v>0.4198872187641595</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>28.94942362589928</v>
+        <v>29.38270573597122</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.140523370392042</v>
+        <v>2.172560294324166</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.00129193009731429</v>
+        <v>-0.001268431480713081</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1135753219434615</v>
+        <v>-0.1084233235852448</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.147428475839213</v>
+        <v>0.1478530779910325</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.186957952516927</v>
+        <v>1.192026025484229</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3627737119913853</v>
+        <v>0.3543426697670881</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1295082241.479945</v>
+        <v>1240831117.350391</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3601,55 +3601,55 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1002.56</v>
+        <v>1005.23</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.09648486400396461</v>
+        <v>0.09940500303493582</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1312229742025495</v>
+        <v>-0.1289092626452569</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>721.16</v>
+        <v>722.3</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>295762217920</v>
+        <v>296549886610</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.27361365021328</v>
+        <v>15.3142900670323</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.86547814306871</v>
+        <v>13.90076914500663</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.507798383204592</v>
+        <v>2.514477107353926</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.451224975965847</v>
+        <v>2.457753034821006</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3579923403190588</v>
+        <v>0.3589457391666609</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.08789277609658</v>
+        <v>27.11298335966617</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.210376878502929</v>
+        <v>7.217055602652263</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1403661370000589</v>
+        <v>-0.1399933093031237</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1015569382184267</v>
+        <v>0.1016865259238855</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3828847627451899</v>
+        <v>-0.3828419579410927</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01795403766358123</v>
+        <v>0.01790634979059519</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.572247710805858</v>
+        <v>1.570845494788868</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3924443282067089</v>
+        <v>0.3924895315405574</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1983134669.091528</v>
+        <v>1943431259.763835</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>231.4</v>
+        <v>230.6</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2061749571183533</v>
+        <v>-0.2089193825042882</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3039764182157252</v>
+        <v>-0.3063827227335619</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>218009807600</v>
+        <v>217256100400</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.20960698689957</v>
+        <v>20.13973799126638</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.97971917224559</v>
+        <v>17.91437236920102</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.155126960649522</v>
+        <v>3.144219002272168</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.312924068268897</v>
+        <v>6.291098920236852</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2463535425341052</v>
+        <v>0.2455018448935379</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.02175005240121</v>
+        <v>16.97528514888108</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>3.995973885986367</v>
+        <v>3.985065927609014</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.0625247100121747</v>
+        <v>0.06274162140857427</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1240223939702099</v>
+        <v>0.1242223604713766</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04449515609729504</v>
+        <v>0.04460267939472029</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02912705272255834</v>
+        <v>0.02922810060711188</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8994964851217339</v>
+        <v>0.8955746974934872</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7895768244663467</v>
+        <v>0.7885179414609703</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1594885754.716293</v>
+        <v>1519034716.107802</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1159.9312</v>
+        <v>1171.03003</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07365250076579244</v>
+        <v>0.08392577092619025</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1026718756043786</v>
+        <v>-0.09408576954318659</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1092354768219</v>
+        <v>1102806990820</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.85866666666667</v>
+        <v>39.23048676716918</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.83238218462875</v>
+        <v>27.07158876097833</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.71171529337558</v>
+        <v>13.8429161675399</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.55351701289884</v>
+        <v>30.8458690862186</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.41191795721187</v>
+        <v>0.4158594042399711</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.33278710006248</v>
+        <v>32.6296577715292</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.28935337646769</v>
+        <v>14.42055425063202</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01835841302061265</v>
+        <v>0.0181844150127202</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4482004020100503</v>
+        <v>0.4491386934673371</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2217388895693952</v>
+        <v>0.2222057912886561</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005767583456673982</v>
+        <v>0.005712919249389361</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.353654034684814</v>
+        <v>0.3559700953723587</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3425210823491776</v>
+        <v>0.3401475485834055</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3164924664.735026</v>
+        <v>3113579501.360417</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -3979,55 +3979,55 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>211.16</v>
+        <v>213.165</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1608576530253591</v>
+        <v>0.1718801932522762</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.09080731969860067</v>
+        <v>-0.08217438105489783</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>145.66</v>
+        <v>146.29</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>333058444800</v>
+        <v>336220891200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>16.97427652733119</v>
+        <v>17.1354501607717</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.75075180670494</v>
+        <v>15.89782792531371</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.632269636209881</v>
+        <v>2.65726348267986</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.004359473631778</v>
+        <v>3.032886376192072</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4318526763221296</v>
+        <v>0.4359531906999753</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.76735082972706</v>
+        <v>23.87511129587352</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.512573756213991</v>
+        <v>5.53756760268397</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04709083419103265</v>
+        <v>-0.04664790442980064</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07768040126855458</v>
+        <v>0.07784851120997227</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3293477823332721</v>
+        <v>-0.3292506669112728</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01965334343625687</v>
+        <v>0.01946848685290737</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.367783172140879</v>
+        <v>1.372763245188019</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2946929322718856</v>
+        <v>0.2948246217062868</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>979826272.8748901</v>
+        <v>937155088.2895844</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4105,55 +4105,55 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>933.4400000000001</v>
+        <v>943.58</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>1.959355653612829</v>
+        <v>1.991503264951141</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2562231075697211</v>
+        <v>-0.2481434262948207</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>114.25</v>
+        <v>117.3</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1054217801600</v>
+        <v>1065669816200</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>20.83106449453247</v>
+        <v>21.0550095960723</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.006937863934595</v>
+        <v>6.072191495598436</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.6779781731174</v>
+        <v>11.80352263860026</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.45351971724713</v>
+        <v>10.56590065366745</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.02969037494248764</v>
+        <v>0.03000956237685981</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.15229569543206</v>
+        <v>15.31811960724841</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.47172831158473</v>
+        <v>11.59727277706759</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02482598943053173</v>
+        <v>0.02456193558249261</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.467834188797144</v>
+        <v>2.467448220520466</v>
       </c>
       <c r="V29" s="4" t="n">
-        <v>1.763697862828721</v>
+        <v>1.763390251657762</v>
       </c>
       <c r="W29" s="4" t="n">
         <v>0.3763197924123121</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005677922523140213</v>
+        <v>0.000561690582674495</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.881986673522564</v>
+        <v>2.883191551541208</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8452331888279956</v>
+        <v>0.8453364963310421</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>31908653661.12205</v>
+        <v>31245563511.85334</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>142.9</v>
+        <v>137.38</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.03085789788004756</v>
+        <v>-0.06829431777999262</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2661483315016998</v>
+        <v>-0.2944958557152101</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>147738879800</v>
+        <v>142031966608</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>88.75776397515529</v>
+        <v>85.32919254658385</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.37458136278442</v>
+        <v>29.18517754980342</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>10.02843332880804</v>
+        <v>9.641051222373065</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.79415947587088</v>
+        <v>11.33856983061681</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>142.0124223602515</v>
+        <v>136.5267080745371</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>44.04954995700773</v>
+        <v>42.41386259902551</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.43231603312517</v>
+        <v>10.0449339266902</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03100064117313011</v>
+        <v>0.0322462619463725</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.922106577044159</v>
+        <v>1.923716753169404</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2380188269553929</v>
+        <v>0.2385833135872333</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6784891035772674</v>
+        <v>0.6626141263121342</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5845080542725847</v>
+        <v>0.5948405458051468</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2708254922.262723</v>
+        <v>2596678768.610263</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.55</v>
+        <v>28.84</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1338363643360048</v>
+        <v>0.1453534412416946</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.01856308009625296</v>
+        <v>-0.008594018563080064</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.09</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>162719012000</v>
+        <v>164371850470</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>37.72463002114165</v>
+        <v>38.107822410148</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.777747802348967</v>
+        <v>9.877817535880233</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.554619002763125</v>
+        <v>2.580567860933182</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.909924286888133</v>
+        <v>1.929324568611339</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6309694755748471</v>
+        <v>-0.6373786226122098</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.81820437262357</v>
+        <v>17.94913264179341</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.531415033911077</v>
+        <v>3.557363892081135</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06751515919971293</v>
+        <v>0.06683626161405956</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.858212625619045</v>
+        <v>2.857919249037042</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04926294725291902</v>
+        <v>-0.04937174416061918</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.06024518388791594</v>
+        <v>0.05963938973647712</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3201014553015608</v>
+        <v>0.3260157384742168</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2152062621165819</v>
+        <v>0.2128294043765254</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1015439102.791748</v>
+        <v>1007107103.291278</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>160.78</v>
+        <v>161.6744</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.04303312150005312</v>
+        <v>-0.03770962867675209</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.174640657084189</v>
+        <v>-0.1700492813141685</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1141304693750</v>
+        <v>1147653635895</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.397198170283589</v>
+        <v>7.047655433353473</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003446288595504875</v>
+        <v>0.003435337347870945</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.352912319193972</v>
+        <v>6.052715635475415</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.603706550571706</v>
+        <v>4.386165780314331</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01655400583248956</v>
+        <v>0.01577177283390766</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.470455918493621</v>
+        <v>7.11576246869612</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.322660014944709</v>
+        <v>6.022463331226152</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07587373931300175</v>
+        <v>0.07963685099622564</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2145.424469480599</v>
+        <v>2050.517717094441</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2792.065152187342</v>
+        <v>2665.085898103323</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.865903719368081</v>
+        <v>1.855581341263676</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.21747637549716</v>
+        <v>1.201020048996448</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>4085305419.395833</v>
+        <v>3962723565.224841</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>545.22</v>
+        <v>551.89</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4605411675030049</v>
+        <v>0.4784088348432436</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1884554128276499</v>
+        <v>-0.1785273060149145</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>281.74</v>
+        <v>283.78</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>68719936625</v>
+        <v>69560628414</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.821403281526887</v>
+        <v>1.818958605996238</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.435283431850093</v>
+        <v>0.4228005799564486</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5384499236.760575</v>
+        <v>5283633759.980894</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>142.23</v>
+        <v>141.1</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1163093961055627</v>
+        <v>-0.1233302101560493</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3696596348165219</v>
+        <v>-0.3746676121255097</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1859780341816</v>
+        <v>1845004613866</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-92.35714285714285</v>
+        <v>-91.62337662337661</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>137.6553177949248</v>
+        <v>135.9237265769332</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>112.2039421910106</v>
+        <v>111.3124955575264</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.55565553669119</v>
+        <v>6.503571653147205</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9235714285714285</v>
+        <v>-0.9162337662337662</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>433.3146968600912</v>
+        <v>429.7688058233742</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>108.9364912106184</v>
+        <v>108.0450445771342</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.01528298765231925</v>
+        <v>-0.01540538152934089</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.039512386619558</v>
+        <v>4.04945969958057</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.7944501473614949</v>
+        <v>0.7943627941505259</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12929939482.72425</v>
+        <v>12696474646.90762</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>761.78</v>
+        <v>765.7701</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1150665559909148</v>
+        <v>0.1209071229066374</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.02256951127192475</v>
+        <v>-0.01744986335116827</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>811477175802</v>
+        <v>815727582848</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9945165588160644</v>
+        <v>0.9944879297731887</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1141284666360961</v>
+        <v>0.1129162506357109</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32792217056.48495</v>
+        <v>32249994300.53522</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -4897,55 +4897,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>414</v>
+        <v>414.285</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.2953287411987802</v>
+        <v>0.2962204530133736</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1356993736951984</v>
+        <v>-0.1351043841336116</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>225.63</v>
+        <v>228.6</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2147202720000</v>
+        <v>2148680866800</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>28.28329662686913</v>
+        <v>27.64576330126348</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6411926834108234</v>
+        <v>0.6408864417144891</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>14.24955973347098</v>
+        <v>13.92836064111815</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.83574884360992</v>
+        <v>9.614041390167893</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5313145145454561</v>
+        <v>0.5193381627831609</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.75212568403078</v>
+        <v>18.31455399061033</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.76498032200035</v>
+        <v>13.44378122964753</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01767629289810506</v>
+        <v>0.01808392229407813</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>43.11044816733745</v>
+        <v>42.13675793687564</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>43.16193336122117</v>
+        <v>42.16985541392097</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2657004830917875</v>
+        <v>0.2655176991684468</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.197719349561458</v>
+        <v>2.185600597624338</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3769547430374206</v>
+        <v>0.3627552150702786</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4629911607.080888</v>
+        <v>4520557514.501959</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -5025,53 +5025,53 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.32</v>
+        <v>28.4489</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.006664336280480132</v>
+        <v>-0.00214311569243486</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.05599999999999994</v>
+        <v>-0.05170333333333343</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>11.25</v>
+        <v>11.45</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>71002111401</v>
+        <v>71325281322</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.2992125984252</v>
+        <v>-22.40070866141732</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-76.16188092554692</v>
+        <v>-77.17009118897035</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.966000592579261</v>
+        <v>1.974948949799252</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.165525306047872</v>
+        <v>2.175381810707107</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1659476286394434</v>
+        <v>0.1667029481779894</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.47208452909091</v>
+        <v>16.52550104495868</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.75941053304721</v>
+        <v>2.768358890267202</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.0307033122957143</v>
+        <v>0.03056419770934135</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02177716486596282</v>
+        <v>0.02185374104487381</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.3120924508957708</v>
+        <v>0.300251691712329</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.2055662776467251</v>
+        <v>0.2027890490966311</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>574227043.0057274</v>
+        <v>552928427.5290267</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>324.19</v>
+        <v>329.19</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1302283410393498</v>
+        <v>-0.1168138054435471</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1633590544272111</v>
+        <v>-0.1504554956256936</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>218928748900</v>
+        <v>222305298900</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>19.65979381443299</v>
+        <v>19.9630078835658</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.79804786446975</v>
+        <v>17.05112643766374</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.604031602298003</v>
+        <v>2.644193723311884</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.411925904317386</v>
+        <v>6.510817386231039</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.219078917750869</v>
+        <v>1.237880838194912</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.413312930755541</v>
+        <v>9.549882660572724</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.768246034993398</v>
+        <v>2.80840815600728</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.068752962210894</v>
+        <v>0.06770868744235768</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1703618166260996</v>
+        <v>0.170773553087384</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.003032690958297835</v>
+        <v>0.003267443689917826</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01091952250223634</v>
+        <v>0.01075366809441356</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9558903343246893</v>
+        <v>0.9688856938525349</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.2528229513732891</v>
+        <v>0.2569361930358967</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>903948608.2901551</v>
+        <v>892013402.8720948</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>141.261</v>
+        <v>144.69</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.278212686352175</v>
+        <v>-0.2606918653293987</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5914005553627213</v>
+        <v>-0.5814821242624089</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>406898072670</v>
+        <v>416775204300</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>23.78131313131313</v>
+        <v>24.35858585858585</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.05447799421116</v>
+        <v>16.42941705371427</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.040827706731197</v>
+        <v>6.187464062175242</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>9.564062247106428</v>
+        <v>9.79622235814435</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7166530849030842</v>
+        <v>0.7340492765492759</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>16.56846660653644</v>
+        <v>16.87619417079478</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>7.895098914308619</v>
+        <v>8.041735269752664</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05821113834375342</v>
+        <v>-0.05683159591939285</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4812884691665509</v>
+        <v>0.4826202158572019</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4854822617291292</v>
+        <v>0.4871456359899078</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01415818945073304</v>
+        <v>0.01382265533208929</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.070309145793718</v>
+        <v>2.05604099806373</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5737897342206658</v>
+        <v>0.5735485568908285</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3766237771.907195</v>
+        <v>3721545443.935913</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01 18:47 ET</t>
+          <t>2026-09-02 11:41 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-03)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -462,7 +462,7 @@
     <col width="21" customWidth="1" min="24" max="24"/>
     <col width="21" customWidth="1" min="25" max="25"/>
     <col width="22" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="27" max="27"/>
     <col width="20" customWidth="1" min="28" max="28"/>
     <col width="21" customWidth="1" min="29" max="29"/>
     <col width="21" customWidth="1" min="30" max="30"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>324.96</v>
+        <v>329.99</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1990701018055829</v>
+        <v>0.2176303018673815</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.05691151290013641</v>
+        <v>-0.04231360826537423</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4772803205760</v>
+        <v>4846680606440</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.0958904109589</v>
+        <v>37.67009132420092</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.28323877557946</v>
+        <v>34.80645787582248</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.22401039743115</v>
+        <v>10.38226609751447</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>44.40550292410715</v>
+        <v>45.0928480733817</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.133485540334854</v>
+        <v>1.151030568239471</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.59327306577401</v>
+        <v>29.03175104424106</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.31989898903867</v>
+        <v>10.478154689122</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02863788723470638</v>
+        <v>0.02820136318006662</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08204159629699137</v>
+        <v>0.08227304997810725</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.107043275770738</v>
+        <v>0.1072914127062383</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.00326193993106844</v>
+        <v>0.003212218552077336</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3234527973862911</v>
+        <v>0.3315443722273647</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.29141139845766</v>
+        <v>0.2929291563851946</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15202997037.57178</v>
+        <v>14915885839.7699</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>496.82</v>
+        <v>512.9215</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.05049265749422904</v>
+        <v>0.08453820220789465</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.1027595174456405</v>
+        <v>-0.07368074116882173</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3689161751000</v>
+        <v>3808724244325</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>27.60111111111111</v>
+        <v>28.49563888888889</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.37515115988967</v>
+        <v>25.15243435697176</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.1173242174669</v>
+        <v>11.47762693452246</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.343092767192525</v>
+        <v>8.613485078675458</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.8767035060582609</v>
+        <v>0.9051166969579774</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.29728868681904</v>
+        <v>18.87344071783788</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.44240143864947</v>
+        <v>11.80270415570502</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.0181577833993975</v>
+        <v>0.01758777892618786</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1323462541856926</v>
+        <v>0.1329177321156774</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2173595404792559</v>
+        <v>0.2179872191872054</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.0073265971579244</v>
+        <v>0.007096602501552382</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.558392900020248</v>
+        <v>0.5717019171942199</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4319529799545624</v>
+        <v>0.436579821005558</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15178737495.48513</v>
+        <v>14937564020.23822</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -953,55 +953,55 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>337.12</v>
+        <v>342.78</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.06971285587500908</v>
+        <v>0.08767255795217022</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1749590073664374</v>
+        <v>-0.1611071682044004</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>224.79</v>
+        <v>226.11</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4079863756736</v>
+        <v>4148361706615</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>16.73882820258192</v>
+        <v>17.01986097318768</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>19.94989147996272</v>
+        <v>20.30283786548074</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.150405292914703</v>
+        <v>9.30403395320802</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.395742443167625</v>
+        <v>6.503122314514115</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1488593727584209</v>
+        <v>0.1513586135326635</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.65985456128389</v>
+        <v>12.86837244467465</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.277898469130928</v>
+        <v>9.430712843240247</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01305754387313654</v>
+        <v>0.01284306109558254</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1609564282896438</v>
+        <v>-0.1617003944987826</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2887944220759855</v>
+        <v>0.2894990403021651</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002521357380161367</v>
+        <v>0.002479724604702725</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7931707340049563</v>
+        <v>0.8026175202573731</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3783828308594888</v>
+        <v>0.3810313344060888</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9534232846.39229</v>
+        <v>8885488945.234741</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>254.98</v>
+        <v>258.73</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.1257395143487858</v>
+        <v>0.1422958057395145</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.1121866295264624</v>
+        <v>-0.09912952646239548</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2742845358000</v>
+        <v>2783184483000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.23650793650793</v>
+        <v>20.53412698412698</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.55627353105909</v>
+        <v>22.89963875456104</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.536052699566832</v>
+        <v>3.588057553372525</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>4.971837279286465</v>
+        <v>5.044958268373155</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2290731609056482</v>
+        <v>0.2324421480944324</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.36967900408273</v>
+        <v>11.52849633263385</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.723009949979373</v>
+        <v>3.775014803785066</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004238299460118524</v>
+        <v>-0.004176870082097249</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.102843476842792</v>
+        <v>-0.1032990867579908</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1728287394827941</v>
+        <v>0.172964637968436</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8350404983747306</v>
+        <v>0.8496676248500586</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4617796690036123</v>
+        <v>0.4627235253255302</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11286046299.82586</v>
+        <v>11008791324.65442</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>224.41</v>
+        <v>227.75</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.1882975522753896</v>
+        <v>0.2059835458790606</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.05128096727826159</v>
+        <v>-0.03716073391392571</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5435434610000</v>
+        <v>5516332750000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.22767295597484</v>
+        <v>28.64779874213836</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.1638524704942</v>
+        <v>17.39625384612775</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>17.94056358901406</v>
+        <v>18.20758146873112</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>23.70680003843063</v>
+        <v>24.05963953813367</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.226589483592179</v>
+        <v>0.2299619218756685</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.33171397758348</v>
+        <v>23.67792520980712</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>17.99475065105671</v>
+        <v>18.26176853077378</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02336630078601939</v>
+        <v>0.02302362923991487</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6446000689239249</v>
+        <v>0.6467797604893597</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8938608938735855</v>
+        <v>0.8963443512833744</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001247716233679426</v>
+        <v>0.001229418221734358</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.316889047595176</v>
+        <v>1.304710125527702</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4369667044530559</v>
+        <v>0.4377862509320758</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27642432961.89283</v>
+        <v>27289592957.53905</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>592.85</v>
+        <v>618.23</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.08849798668714526</v>
+        <v>-0.04947644481672231</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2503161355589276</v>
+        <v>-0.2182220536165907</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1510277413025</v>
+        <v>1574932622171</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>22.03084355258268</v>
+        <v>22.97064288368636</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>17.93514034477684</v>
+        <v>18.69912143784212</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.616826491469805</v>
+        <v>6.899089360607761</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.771425536231773</v>
+        <v>6.017624999521479</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.516322928279446</v>
+        <v>-4.708981791155701</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>15.0098383613363</v>
+        <v>15.61154501998655</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.041171940279871</v>
+        <v>7.323434809417827</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02713143932804199</v>
+        <v>0.02602140907502018</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2283619268693717</v>
+        <v>0.2284343390165811</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2639791625992733</v>
+        <v>0.2644098264989343</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.003542211351944</v>
+        <v>0.003396794073403102</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7855943629230826</v>
+        <v>0.7999782553723747</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4317108267134282</v>
+        <v>0.4395812903118277</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9668450710.775581</v>
+        <v>9541353980.865295</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>357.01</v>
+        <v>381.26</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.185038934346002</v>
+        <v>-0.1296824853890837</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2843052743419602</v>
+        <v>-0.2356915181524768</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1410027915132</v>
+        <v>1505804439436</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>302.5508474576271</v>
+        <v>323.1016949152543</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>173.4834848827766</v>
+        <v>185.1302740830667</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>13.60781241984578</v>
+        <v>14.53212672807111</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>13.30495026364871</v>
+        <v>14.20869257869166</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.053818333731197</v>
+        <v>-8.600876104082117</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>116.7401825018291</v>
+        <v>124.7407413856834</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>13.55109502245727</v>
+        <v>14.47979267689323</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.004086443919417431</v>
+        <v>0.003825372254791314</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7439749245414444</v>
+        <v>0.7452666589273276</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1154889909686263</v>
+        <v>0.1158572282041415</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.548942341098291</v>
+        <v>1.549942560627468</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5495280161723051</v>
+        <v>0.5673196622451324</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>13034479952.70655</v>
+        <v>12241754126.69464</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>367.24</v>
+        <v>348.11</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.05644095609689637</v>
+        <v>0.001409599245427051</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2581010101010101</v>
+        <v>-0.2967474747474748</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1747173679200</v>
+        <v>1656161173800</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>45.56327543424317</v>
+        <v>43.18982630272953</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>20.14500839406409</v>
+        <v>19.19613579492991</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.60825192135033</v>
+        <v>18.58683306922248</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.55708536463035</v>
+        <v>16.64251439462333</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.453377146647667</v>
+        <v>0.4297601528142886</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>35.68661273222293</v>
+        <v>33.86461350496477</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>20.00603428802298</v>
+        <v>18.98461543589513</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02255242307567382</v>
+        <v>0.02379176654020411</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.261765026003603</v>
+        <v>1.249922940956525</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8399168511781214</v>
+        <v>0.8363526329837443</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1667,16 +1667,16 @@
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.006916457902189304</v>
+        <v>0.007296544195800178</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.608800197160063</v>
+        <v>1.587103971919628</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4170972003250273</v>
+        <v>0.4366230040411669</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>7646377250.435527</v>
+        <v>7857839550.175766</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>928.48</v>
+        <v>927.87</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.08657694558221185</v>
+        <v>0.0858630778232885</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1532330141358869</v>
+        <v>-0.1537893296853625</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>411761381920</v>
+        <v>411490859730</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>46.63385233550979</v>
+        <v>46.6049070818684</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.91222343446236</v>
+        <v>40.87018111374514</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.402519123530674</v>
+        <v>1.401648591293211</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.30038577814915</v>
+        <v>12.29275102853263</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.678661476644906</v>
+        <v>3.676378161324177</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.71578313199724</v>
+        <v>27.69812059239807</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.366025682063579</v>
+        <v>1.365155149826116</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02138617263945091</v>
+        <v>0.02139945510756327</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1398513309894525</v>
+        <v>0.1403156485204469</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1130642932725223</v>
+        <v>0.1142113311475084</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005966741340685852</v>
+        <v>0.005970663993878453</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.182565431746724</v>
+        <v>-0.1817159995183528</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2121206223965534</v>
+        <v>0.211558205790487</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1747158065.568514</v>
+        <v>1726383415.124247</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>82.73</v>
+        <v>82.48999999999999</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.0907791851598504</v>
+        <v>-0.09341683771106091</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3470917843895509</v>
+        <v>-0.3489858732538869</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>344482756117</v>
+        <v>343483410518</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>25.61300309597523</v>
+        <v>25.53869969040248</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>22.10680754116715</v>
+        <v>22.03920274651601</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7.121714184977521</v>
+        <v>7.101054068899966</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.49444280575</v>
+        <v>11.46109738965693</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7527724080646382</v>
+        <v>0.750588612852073</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.4289765603128</v>
+        <v>11.39631504585509</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.229425404920212</v>
+        <v>7.208765288842658</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03191627971144598</v>
+        <v>0.03200913832612547</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1586025276729295</v>
+        <v>0.158785096908266</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1391644573311561</v>
+        <v>0.1394926439203128</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1052506280837404</v>
+        <v>0.1110197773019693</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3371405993584717</v>
+        <v>0.3373555988742467</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2423990919.517314</v>
+        <v>2338517051.665696</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>505.09</v>
+        <v>508.37</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.01658446974994621</v>
+        <v>0.02318605968595744</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.06071707516643743</v>
+        <v>-0.05461747312827758</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1089405182299</v>
+        <v>1096479662090</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.70027659039477</v>
+        <v>12.78275081719889</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.76960736499913</v>
+        <v>22.91744396381397</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.831926169324672</v>
+        <v>2.850316392521712</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.450723282318706</v>
+        <v>1.460144122893664</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3494972340960522</v>
+        <v>0.3517668314506525</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.39804718481585</v>
+        <v>15.49050712405573</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.062661806349058</v>
+        <v>3.081052029546099</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02222772609627068</v>
+        <v>0.02208431294917389</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422268075681746</v>
+        <v>-0.4422261558757375</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06006115058636352</v>
+        <v>0.06010655451571356</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06431852594660128</v>
+        <v>0.06728511279110221</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1510932357306426</v>
+        <v>0.1516637421326966</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2165062101.991264</v>
+        <v>2102071916.511963</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>356.22</v>
+        <v>361.8</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.09444509025459991</v>
+        <v>0.1115890002080573</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.02804911323328774</v>
+        <v>-0.01282401091405183</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>954495052200</v>
+        <v>969446718000</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.31470335339639</v>
+        <v>15.55460017196905</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.23375433671728</v>
+        <v>14.4562463669112</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.206953033433793</v>
+        <v>3.257188275493645</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.651884724424583</v>
+        <v>2.693425111719764</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8018663712917741</v>
+        <v>0.8144271886288357</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.20776140188922</v>
+        <v>20.36825588235294</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.325088455245218</v>
+        <v>6.37532369730507</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.09022047814864513</v>
+        <v>0.08882901803789489</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07594264950117213</v>
+        <v>0.07597780068080895</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2904304965101593</v>
+        <v>-0.2903803502202146</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2150,7 +2150,7 @@
         <v>0.2818840652750199</v>
       </c>
       <c r="AA13" s="5" t="n">
-        <v>100867000000</v>
+        <v>-147782000000</v>
       </c>
       <c r="AB13" s="6" t="n">
         <v>0.8403662699432636</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01684352366515075</v>
+        <v>0.01658374792703151</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.775580001592568</v>
+        <v>0.7777696991993061</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1831254518063516</v>
+        <v>0.1852882111330811</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2237108907.825361</v>
+        <v>2164880839.140082</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>378.4</v>
+        <v>379.35</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.09212649504023296</v>
+        <v>0.09486835595537113</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.01859584511243095</v>
+        <v>-0.01613196047410315</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>706490664642</v>
+        <v>708264359493</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>32.14953271028037</v>
+        <v>32.23024638912489</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.42938180251521</v>
+        <v>25.48481406454033</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.88047708689984</v>
+        <v>15.92034614936612</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.58246228893058</v>
+        <v>20.63413601825004</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.167978357107724</v>
+        <v>2.173421220319279</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.67488022001512</v>
+        <v>24.73583612251701</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.13895128218845</v>
+        <v>16.17882034465474</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02974278508074543</v>
+        <v>0.02966830071054518</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2642671756613633</v>
+        <v>0.2646843844927316</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1338512671046894</v>
+        <v>0.1341573332662278</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007082452431289642</v>
+        <v>0.007064715961513115</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3088558887285578</v>
+        <v>0.3066421493972804</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.2006332931458161</v>
+        <v>0.1972723552258211</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2537353724.343595</v>
+        <v>2495451124.820871</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>588.14</v>
+        <v>586.55</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.04441247118841063</v>
+        <v>0.04158896687108893</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.022406170007646</v>
+        <v>-0.02504903427412664</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>515819953040</v>
+        <v>514425465800</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32.29763866007688</v>
+        <v>32.2103239978034</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.66264830765957</v>
+        <v>26.58172723120263</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.70284619445315</v>
+        <v>14.66309796197589</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>92.45045090001783</v>
+        <v>92.20051684191766</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.427440280065897</v>
+        <v>1.423581283831489</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.92710947006692</v>
+        <v>23.8640561493941</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>15.083429382892</v>
+        <v>15.04368115041473</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03188709529955797</v>
+        <v>0.03197353376435432</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2113439853159109</v>
+        <v>0.2117468408897714</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1521855851762886</v>
+        <v>0.1524203980450276</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005729928248376238</v>
+        <v>0.005745460745034525</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.3014651276664039</v>
+        <v>0.2965753014032813</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2157709093333069</v>
+        <v>0.2133448735150242</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1715999427.03787</v>
+        <v>1687843301.277771</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>399.66</v>
+        <v>404.61</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1880499621025016</v>
+        <v>0.2027645878153759</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.134222953944803</v>
+        <v>-0.1234998483601231</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>362948992503</v>
+        <v>367444307302</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.69995498681757</v>
+        <v>26.01826249115813</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.53357845065119</v>
+        <v>18.75674457691351</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.8063221709843178</v>
+        <v>0.8163088965652068</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.464552362098495</v>
+        <v>3.507462671342321</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7787153462715872</v>
+        <v>-0.7883601467621151</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.82470956422001</v>
+        <v>15.99919680557389</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.905722565093562</v>
+        <v>0.9157092906744511</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06506974943539702</v>
+        <v>0.06427368591831073</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3866698789577028</v>
+        <v>0.3871416963891676</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009439763754755637</v>
+        <v>0.00951823030784138</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02239403492969023</v>
+        <v>0.02212006623662292</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4503163480289218</v>
+        <v>0.4562231540146999</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2306600451603952</v>
+        <v>0.2342384798606088</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1693488412.357012</v>
+        <v>1672950175.002156</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>164.17</v>
+        <v>164.52</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3385242393605714</v>
+        <v>0.3413778879186284</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.06938382177881075</v>
+        <v>-0.06739980726716166</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>680395998200</v>
+        <v>681846559200</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>21.12870012870013</v>
+        <v>21.17374517374517</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>15.0033237409573</v>
+        <v>15.0387001262639</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.884440254251371</v>
+        <v>1.888457761036947</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.641765435538592</v>
+        <v>2.647397511450382</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.068851887601889</v>
+        <v>2.07326254826255</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.915433319874696</v>
+        <v>9.935629087365124</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.972458866116435</v>
+        <v>1.976476372902011</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04490473206901351</v>
+        <v>0.04480920170052242</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4082679607200155</v>
+        <v>0.4079504874737749</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08425307774536028</v>
+        <v>0.08409163954739807</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02509593713833222</v>
+        <v>0.02504254801847799</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5361595737298586</v>
+        <v>-0.5366576136909386</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.261008017874156</v>
+        <v>0.2619153965860521</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2241575762.256608</v>
+        <v>2199674737.212023</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>275.21</v>
+        <v>278.34</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3272726882033778</v>
+        <v>0.342367937337045</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.02084889885082009</v>
+        <v>-0.009712882911730225</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>663228143067</v>
+        <v>670771125109</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>31.81618497109826</v>
+        <v>32.17803468208092</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.23896947410746</v>
+        <v>22.48610878693204</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.772540749594094</v>
+        <v>6.849565757936873</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.90316603311718</v>
+        <v>7.993049793458944</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.939346060237304</v>
+        <v>-3.984148767873446</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.50996510930274</v>
+        <v>20.73358013485711</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>7.064732031032687</v>
+        <v>7.141757039375466</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02820748817064311</v>
+        <v>0.02789028820666656</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4306501480718981</v>
+        <v>0.4310183672499801</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.0851245342144582</v>
+        <v>0.08533159948788738</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01918534936957233</v>
+        <v>0.0189696055184307</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1932506045492204</v>
+        <v>-0.1850146057998956</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.2349763036852026</v>
+        <v>0.2331177262248448</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1844568152.504904</v>
+        <v>1780024640.394238</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2843,55 +2843,55 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>106.09</v>
+        <v>108.92</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.05915219944898664</v>
+        <v>-0.03405464760093913</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.2150784255696951</v>
+        <v>-0.1941402781888132</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>97.5</v>
+        <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>844272707200</v>
+        <v>866794073600</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>38.29963898916968</v>
+        <v>39.32129963898917</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.34505483752987</v>
+        <v>35.25064272053409</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.147359082409219</v>
+        <v>1.177965418569254</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.589749994910319</v>
+        <v>8.818885563631181</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.261549064653765</v>
+        <v>9.508605185428298</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.16059448633255</v>
+        <v>21.68605551688882</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.23192366166558</v>
+        <v>1.262514856881931</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01600075412221024</v>
+        <v>0.01558521689431635</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1151427525839477</v>
+        <v>0.1154775233667971</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04933020365737639</v>
+        <v>0.04945453700575531</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009213875011782448</v>
+        <v>0.008974476680132208</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.06149000306391298</v>
+        <v>-0.04727164707200158</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3071107247847898</v>
+        <v>0.3135978563482321</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2864449487.50757</v>
+        <v>2818710927.070473</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>147.64</v>
+        <v>147.255</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.04125824804901312</v>
+        <v>0.03854296475519803</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1172496263079223</v>
+        <v>-0.1195515695067265</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>350971127459</v>
+        <v>350055902018</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.87259259259259</v>
+        <v>21.81555555555556</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.94502473400002</v>
+        <v>20.88701975427124</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.032667610292766</v>
+        <v>4.022151645578638</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.585367605089208</v>
+        <v>6.568194978917714</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.87270264550287</v>
+        <v>20.81827301587324</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.693381361579</v>
+        <v>17.65032003472287</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.320883438953489</v>
+        <v>4.31036747423936</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04533991190445982</v>
+        <v>0.04545845365915798</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04428583257229834</v>
+        <v>0.04445515981735171</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02433254703733612</v>
+        <v>0.02441244393764164</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02906123001896506</v>
+        <v>0.02913721096057859</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.057813732509269</v>
+        <v>-0.05823490777328469</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1865040566213673</v>
+        <v>0.183552804568943</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1328716942.894674</v>
+        <v>1310043784.470195</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>318.51</v>
+        <v>318.85</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.07897173889830678</v>
+        <v>-0.07798856848364288</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2536379613356766</v>
+        <v>-0.2528412419449326</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>317591735670</v>
+        <v>317930755450</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22.24231843575419</v>
+        <v>22.26606145251397</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.2412361811257</v>
+        <v>21.2639105722016</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.877285996063271</v>
+        <v>1.879289943313472</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.05271348618884</v>
+        <v>19.07305169404826</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.629632486683156</v>
+        <v>-7.63777689359494</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.80906275015681</v>
+        <v>15.82323878109973</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.234795335449473</v>
+        <v>2.236799282699674</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04754846648683262</v>
+        <v>0.04749776402923336</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.0290728705535148</v>
+        <v>0.02913595734671475</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7081832424517087</v>
+        <v>0.7046871463078951</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2563168683373866</v>
+        <v>0.2555625780408174</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1298234906.43479</v>
+        <v>1273244263.503544</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>457.06</v>
+        <v>456.659</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.045285709506034</v>
+        <v>1.043491285208322</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.2183400885878953</v>
+        <v>-0.2190258751902588</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>745282036000</v>
+        <v>744628165400</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>116.005076142132</v>
+        <v>115.9032994923858</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>34.73988089657288</v>
+        <v>34.65094868257331</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.04338544970343</v>
+        <v>18.02755514828713</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.08926663096513</v>
+        <v>11.07953750148756</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.936554743165836</v>
+        <v>0.9357330601220136</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>69.45997723455869</v>
+        <v>69.39572995148349</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>18.02377523302264</v>
+        <v>18.00710407020942</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01127492626160655</v>
+        <v>0.01128535334933995</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.339247952159099</v>
+        <v>2.344880988804673</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8592330598899265</v>
+        <v>0.8617462116679628</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.535423676416555</v>
+        <v>2.519727357519701</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6798439737942396</v>
+        <v>0.6613287690453237</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>11408119066.35942</v>
+        <v>11024860366.67969</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1682.3</v>
+        <v>1654.5347</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4455480912629175</v>
+        <v>0.4216902321305736</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1588331766635334</v>
+        <v>-0.1727161043220865</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>729.5599999999999</v>
+        <v>735.4299999999999</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>648388686259</v>
+        <v>637687440114</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>52.46008708272859</v>
+        <v>51.50217779390421</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.15736433114095</v>
+        <v>34.54867899727669</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.77347198041186</v>
+        <v>15.4854520086335</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.53040585739551</v>
+        <v>25.06422643836997</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.571149837388012</v>
+        <v>3.505941451522715</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>40.02679063986381</v>
+        <v>39.2897102999022</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.64078498019956</v>
+        <v>15.3527650084212</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01794908459396766</v>
+        <v>0.01828292663069475</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4921507365744593</v>
+        <v>0.4907133728025863</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2556003896508678</v>
+        <v>0.2541607280853724</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004624621054508709</v>
+        <v>0.004702228366682186</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.700305523988325</v>
+        <v>1.689289776496114</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.4086625203368899</v>
+        <v>0.4103945991331352</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2382747215.787012</v>
+        <v>2345906397.343307</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>208.87</v>
+        <v>207.595</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.08297846036764589</v>
+        <v>-0.08857621238100943</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1788087281305287</v>
+        <v>-0.1838215057990957</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>165084581900</v>
+        <v>164076860150</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.22846441947563</v>
+        <v>77.75093632958799</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>87.74171250649034</v>
+        <v>86.70508540308748</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.756312377254109</v>
+        <v>1.745591362838449</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.08615120706886</v>
+        <v>26.92080988093771</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4186845055772663</v>
+        <v>0.4161287400551185</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.31447221582734</v>
+        <v>29.16947628057554</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.167515100803234</v>
+        <v>2.156794086387574</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001272075184629946</v>
+        <v>-0.001279887973282868</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1084233235852448</v>
+        <v>-0.1032713252270281</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1478530779910328</v>
+        <v>0.1482776801428523</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.20013185700927</v>
+        <v>1.190010375711335</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.3411035675317026</v>
+        <v>0.3411975328069975</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1261121991.17122</v>
+        <v>1243121938.648869</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3601,55 +3601,55 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1004.42</v>
+        <v>1039.37</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.09851911816037151</v>
+        <v>0.1367434099702767</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1296111751401658</v>
+        <v>-0.09932495082279758</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>722.3</v>
+        <v>727.15</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>296310930940</v>
+        <v>306621425590</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.30195003046923</v>
+        <v>15.8273942717855</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>13.88956810344654</v>
+        <v>14.37118186998394</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.512450977555813</v>
+        <v>2.598724475482673</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.455772612471688</v>
+        <v>2.540099876293363</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3586565058083996</v>
+        <v>0.3709721907513245</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.1053716095945</v>
+        <v>27.42948327541172</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.215029472854151</v>
+        <v>7.30130297078101</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1401062048851865</v>
+        <v>-0.135454902875012</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1016865259238855</v>
+        <v>0.1013286461041207</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3828419579410927</v>
+        <v>-0.3830722185050527</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01792079010772386</v>
+        <v>0.01731818313016539</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.571814096250298</v>
+        <v>1.578024897075941</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3924597405276543</v>
+        <v>0.3928451392083565</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1991288101.813061</v>
+        <v>1958169225.79882</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>231.7</v>
+        <v>235.36</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.2051457975986278</v>
+        <v>-0.1925900514579759</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.3030740540215364</v>
+        <v>-0.2920652108524333</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>218292447800</v>
+        <v>221740658240</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.23580786026201</v>
+        <v>20.54934497816594</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>17.99982687746694</v>
+        <v>18.2809056901498</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.159217445041029</v>
+        <v>3.208166908259404</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.321108498780913</v>
+        <v>6.419048850574713</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.246672929149318</v>
+        <v>0.2504949223113639</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.03917439122126</v>
+        <v>17.24768564576783</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.000064370377875</v>
+        <v>4.049013833596249</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06244375441008729</v>
+        <v>0.0614910021540109</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1242223604713766</v>
+        <v>0.1240879049684298</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04460267939472029</v>
+        <v>0.04439948840684438</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02908933966335779</v>
+        <v>0.02863698164513936</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8939166872200316</v>
+        <v>0.9009998806334287</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7818710040805544</v>
+        <v>0.7843901124023464</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1477884086.736617</v>
+        <v>1454436786.739461</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1160.06</v>
+        <v>1154.39</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07377172028682843</v>
+        <v>0.0685234696325292</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1025722353305226</v>
+        <v>-0.1069585734730979</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1092476064460</v>
+        <v>1087136392990</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.86298157453937</v>
+        <v>38.67303182579565</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.81798626296588</v>
+        <v>26.66099627211939</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.71323785689719</v>
+        <v>13.6462119628498</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.55690970807875</v>
+        <v>30.40755736591989</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4119636970220319</v>
+        <v>0.4099501510312083</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.33623223301522</v>
+        <v>32.18457148915019</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.29087593998931</v>
+        <v>14.22385004594192</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01835637470914518</v>
+        <v>0.01844653543870872</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4491386934673371</v>
+        <v>0.4505471375140544</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2222057912886561</v>
+        <v>0.2229077529986656</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005766943089150562</v>
+        <v>0.00579526849678185</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3511426584534518</v>
+        <v>0.3491635311446447</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3391726722968073</v>
+        <v>0.3383166262200302</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3182788087.194315</v>
+        <v>3146806522.111918</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>211.88</v>
+        <v>217.34</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1648158719597135</v>
+        <v>0.1948323655452338</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.0877072120559742</v>
+        <v>-0.0641980624327233</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>146.29</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>334194086400</v>
+        <v>342806035200</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.03215434083601</v>
+        <v>17.47106109324759</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>15.80199273246297</v>
+        <v>16.20654077052252</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.641244982573165</v>
+        <v>2.709308025828071</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.014603548366646</v>
+        <v>3.092287781772734</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4333251802383635</v>
+        <v>0.4444916682698033</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>23.80604785497666</v>
+        <v>24.09950029645279</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.521549102577275</v>
+        <v>5.589612145832181</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04693081247771595</v>
+        <v>-0.04575181994928892</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07784851120997227</v>
+        <v>0.07802530722811962</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3292506669112728</v>
+        <v>-0.3291535514892736</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01958655842929961</v>
+        <v>0.01909450630348762</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.370857626398377</v>
+        <v>1.377082304102873</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2781214989296588</v>
+        <v>0.2857793715740013</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>955597855.8695313</v>
+        <v>937073986.5051636</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4105,46 +4105,46 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>956.08</v>
+        <v>950.5601</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.031132963346496</v>
+        <v>2.013632805572694</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2381832669322709</v>
+        <v>-0.242581593625498</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>117.3</v>
+        <v>118.52</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1079787191200</v>
+        <v>1073553071339</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>21.33630885962955</v>
+        <v>21.21312430261102</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.152632363034139</v>
+        <v>6.117110319501473</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.96122018742938</v>
+        <v>11.89216243147529</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.70706326198324</v>
+        <v>10.64524634446607</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03041049630936491</v>
+        <v>0.03023492219571536</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.5264125362128</v>
+        <v>15.43519842183888</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.75497032589671</v>
+        <v>11.68591256994262</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.024238109336076</v>
+        <v>0.02437885997322583</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005543469165760188</v>
+        <v>0.0005575660076622194</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.891286633394994</v>
+        <v>2.873336427879375</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8470927117875043</v>
+        <v>0.8387801420679375</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>31580887482.72587</v>
+        <v>30647682709.27636</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>136.72</v>
+        <v>143.86011</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.07277041146368168</v>
+        <v>-0.02434647014270419</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2978852336103037</v>
+        <v>-0.2612177623943388</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>141349612640</v>
+        <v>148731498379</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>84.9192546583851</v>
+        <v>89.35410559006212</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.04496633141013</v>
+        <v>30.5449981317497</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>9.594733412978551</v>
+        <v>10.09581172814282</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>11.28409715564078</v>
+        <v>11.87340153643336</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>135.870807453419</v>
+        <v>142.9665689441024</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>42.21828966466036</v>
+        <v>44.33404940642018</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>9.998616117295683</v>
+        <v>10.49969443245995</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03240192820099688</v>
+        <v>0.03079374611240163</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.923716753169404</v>
+        <v>1.925326929294648</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2385833135872333</v>
+        <v>0.2391478002190741</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6595099492401759</v>
+        <v>0.6920174895309401</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.5974008082238925</v>
+        <v>0.6057554811947137</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2637089721.392606</v>
+        <v>2516453657.061295</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4357,55 +4357,55 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>29.02</v>
+        <v>28.695</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1525019717348812</v>
+        <v>0.1395949027888497</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.002406325197662484</v>
+        <v>-0.01763094830537493</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>29.09</v>
+        <v>29.21</v>
       </c>
       <c r="J31" s="3" t="n">
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>165397748800</v>
+        <v>163545429061</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>38.34566596194503</v>
+        <v>37.91622621564483</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.939468269460624</v>
+        <v>9.828338343417171</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.596674026626476</v>
+        <v>2.567593397717282</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.941366122784364</v>
+        <v>1.919624427749736</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6413567138767797</v>
+        <v>-0.6341740490935285</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>18.03039835234474</v>
+        <v>17.88366833499683</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.573470057774428</v>
+        <v>3.544389428865235</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06642170210722965</v>
+        <v>0.0671739960149078</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857919249037042</v>
+        <v>2.857847063338064</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04937174416061907</v>
+        <v>-0.0494803444525882</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.05926946933149552</v>
+        <v>0.05994075622930824</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.329865708698279</v>
+        <v>0.3230794338970157</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2144851992323479</v>
+        <v>0.2054533826139834</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1032505776.351425</v>
+        <v>1015258947.938517</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>164.98</v>
+        <v>161.27</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.01803460868938167</v>
+        <v>-0.04011662833880814</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1530800821355237</v>
+        <v>-0.1721252566735113</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1171118599172</v>
+        <v>1144782982716</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>7.047655433353473</v>
+        <v>6.973377601755823</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003505576366151651</v>
+        <v>0.003426855897584164</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>6.052715635475415</v>
+        <v>5.988923840185221</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.386165780314331</v>
+        <v>4.339938366634638</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.01577177283390766</v>
+        <v>0.015605548321709</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.11576246869612</v>
+        <v>7.040390110614151</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>6.022463331226152</v>
+        <v>5.958671535935959</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.07963685099622564</v>
+        <v>0.08048511319355385</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2009.412753064696</v>
+        <v>2033.91999960426</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2611.667219810149</v>
+        <v>2647.170176592263</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.818402230573403</v>
+        <v>1.860234389533081</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.20291887132289</v>
+        <v>1.188322793079931</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3997675836.407492</v>
+        <v>3838515444.217027</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>550.48</v>
+        <v>550.325</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4746317117623235</v>
+        <v>0.4742164961044921</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1806260512331989</v>
+        <v>-0.1808567643600315</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>283.78</v>
+        <v>284.3</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>69382910959</v>
+        <v>69363374643</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.820284454120215</v>
+        <v>1.81257713974366</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4221597192572309</v>
+        <v>0.4188776350986283</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5357574574.696733</v>
+        <v>5290842573.533297</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>140.71</v>
+        <v>149.02</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.1257533229699339</v>
+        <v>-0.07412238070485078</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3763960290728593</v>
+        <v>-0.3395674525793299</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1839905026344</v>
+        <v>1948565524033</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-91.37012987012987</v>
+        <v>-96.76623376623377</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>135.5480337820005</v>
+        <v>142.8857015262563</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>111.0048281353846</v>
+        <v>117.5605142704676</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.485595799534679</v>
+        <v>6.868619757278501</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9137012987012987</v>
+        <v>-0.9676623376623377</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>428.5450027223422</v>
+        <v>454.6841817796977</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>107.7373771549925</v>
+        <v>114.3088377361086</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0154480799786053</v>
+        <v>-0.01458467078495308</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.04945969958057</v>
+        <v>4.05940701254158</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.7945024223792098</v>
+        <v>0.78952941474297</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>12811348413.71411</v>
+        <v>12785796469.68667</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>765.16</v>
+        <v>772.96503</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1200140801570115</v>
+        <v>0.1314388063529024</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.01823267510938331</v>
+        <v>-0.008218137726625385</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>815077681006</v>
+        <v>823391893968</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9953952364099921</v>
+        <v>0.9942391541816716</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1127260732152532</v>
+        <v>0.114401062914581</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32743999194.55756</v>
+        <v>31786011608.50663</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -4897,55 +4897,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>415.5</v>
+        <v>411.7</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3000219612755872</v>
+        <v>0.2881324704143424</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1325678496868476</v>
+        <v>-0.1405010438413361</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>228.6</v>
+        <v>230.3</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2154982440000</v>
+        <v>2135273816000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.64576330126348</v>
+        <v>27.70372087631853</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6427660101919456</v>
+        <v>0.6355453561214504</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.92836064111815</v>
+        <v>13.95756055860477</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.614041390167893</v>
+        <v>9.634196613208077</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5193381627831609</v>
+        <v>0.5204269220342786</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.31455399061033</v>
+        <v>18.35433323546673</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.44378122964753</v>
+        <v>13.47298114713415</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01808392229407813</v>
+        <v>0.01804608982065956</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.01061795879308</v>
+        <v>42.59047015210108</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.04361865260228</v>
+        <v>42.59495905769823</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2647412755716005</v>
+        <v>0.2671848433325237</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.195525901920805</v>
+        <v>2.169713248298459</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3629626082742914</v>
+        <v>0.348305007780893</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4572780277.969775</v>
+        <v>4468028174.153398</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -5025,53 +5025,53 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.39</v>
+        <v>28.345</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.004209057450665021</v>
+        <v>-0.005787450984117704</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.05366666666666664</v>
+        <v>-0.0551666666666667</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>11.45</v>
+        <v>11.54</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>71177610970</v>
+        <v>71064789818</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.35433070866141</v>
+        <v>-22.31889763779527</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-77.0103198666686</v>
+        <v>-77.55889109682697</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.970860057316904</v>
+        <v>1.967736115686003</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.170877946281747</v>
+        <v>2.167436963274255</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1663578099249222</v>
+        <v>0.1660941219556858</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.50109272231405</v>
+        <v>16.48244459801653</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.764269997784854</v>
+        <v>2.761146056153953</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03062760846130152</v>
+        <v>0.03067623228863512</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02185374104487381</v>
+        <v>0.0219303172237848</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2980452966836984</v>
+        <v>0.2970566979565227</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1980670952355524</v>
+        <v>0.1991916915854715</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>563257687.7653129</v>
+        <v>556783519.3529153</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>329.98</v>
+        <v>330.71</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1146943088194103</v>
+        <v>-0.1127357866224232</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1484167333350538</v>
+        <v>-0.1465328137500324</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>222838793800</v>
+        <v>223331770100</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>20.01091570648878</v>
+        <v>20.05518496058217</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.09204624046988</v>
+        <v>17.12383611675204</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.650539338432077</v>
+        <v>2.656403008100103</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.526442240373396</v>
+        <v>6.540880396732788</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.240851541625071</v>
+        <v>1.243596622009901</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.571460677883838</v>
+        <v>9.591399858437146</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.814753771127473</v>
+        <v>2.820617440795499</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06754658712391576</v>
+        <v>0.0673974866776019</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.170773553087384</v>
+        <v>0.1711852895486679</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.003267443689917826</v>
+        <v>0.003502196421537818</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01072792290441845</v>
+        <v>0.01070424238759034</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.968676276005502</v>
+        <v>0.9678387713391668</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.257970111754726</v>
+        <v>0.2560823591417925</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>908038644.1913503</v>
+        <v>886656094.1407267</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>145.75</v>
+        <v>152.7</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2552756885186251</v>
+        <v>-0.2197639632027036</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.5784160592386903</v>
+        <v>-0.5583130857341201</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>419828502500</v>
+        <v>439847769000</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>24.53703703703703</v>
+        <v>25.7070707070707</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>16.54977908341181</v>
+        <v>17.32335130597424</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.232793469224146</v>
+        <v>6.530000430535348</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>9.867989554907313</v>
+        <v>10.33853862802296</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7394269269269262</v>
+        <v>0.7746860496860489</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>16.97132138517619</v>
+        <v>17.60131482381531</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.087064676801567</v>
+        <v>8.38726508952166</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05641827522179726</v>
+        <v>-0.05382577478285626</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4826202158572022</v>
+        <v>0.4839548221945482</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.487145635989908</v>
+        <v>0.4888090421977518</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.0137221269296741</v>
+        <v>0.01309757694826457</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.065053777228375</v>
+        <v>2.080556779548588</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5756374944858818</v>
+        <v>0.5854354501043408</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3784879042.655848</v>
+        <v>3706944296.952924</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 18:48 ET</t>
+          <t>2026-09-03 11:31 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-04)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -442,11 +442,11 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
@@ -470,7 +470,7 @@
     <col width="22" customWidth="1" min="32" max="32"/>
     <col width="20" customWidth="1" min="33" max="33"/>
     <col width="23" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="23" customWidth="1" min="35" max="35"/>
     <col width="21" customWidth="1" min="36" max="36"/>
     <col width="20" customWidth="1" min="37" max="37"/>
     <col width="16" customWidth="1" min="38" max="38"/>
@@ -699,13 +699,13 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="3" t="n">
-        <v>328.21</v>
+        <v>319.31</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.2110622787838823</v>
+        <v>0.1782221633663856</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>-0.04747946716197005</v>
+        <v>-0.07330876164494871</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>344.57</v>
@@ -714,40 +714,40 @@
         <v>225.95</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>4820537112760</v>
+        <v>4689819608502</v>
       </c>
       <c r="L2" s="6" t="n">
-        <v>37.46689497716895</v>
+        <v>36.45091324200914</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>34.61870826214036</v>
+        <v>33.63515294578257</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>10.32626308635179</v>
+        <v>10.0462479537255</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>44.84961261300224</v>
+        <v>43.63343531110492</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>1.14482179096905</v>
+        <v>1.113777904616945</v>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>28.87658388685113</v>
+        <v>28.10074788707667</v>
       </c>
       <c r="R2" s="6" t="n">
-        <v>10.42215167795931</v>
+        <v>10.14213654533303</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0.02835430924039543</v>
+        <v>0.02914461779131386</v>
       </c>
       <c r="T2" s="4" t="n">
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08227304997810725</v>
+        <v>0.08371480577969614</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1072914127062383</v>
+        <v>0.1089653641838908</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -781,16 +781,16 @@
       </c>
       <c r="AG2" s="6" t="inlineStr"/>
       <c r="AH2" s="4" t="n">
-        <v>0.003229639560037781</v>
+        <v>0.003319658012589646</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3186279644011144</v>
+        <v>0.3192971051387462</v>
       </c>
       <c r="AJ2" s="4" t="n">
-        <v>0.2916369511575955</v>
+        <v>0.2993259508347068</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15173304263.96715</v>
+        <v>14809995934.92528</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -827,13 +827,13 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="3" t="n">
-        <v>510.12</v>
+        <v>500.77</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.0786146178514473</v>
+        <v>0.05884466827701185</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-0.07874015748031504</v>
+        <v>-0.09562594813263026</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>553.72</v>
@@ -842,40 +842,40 @@
         <v>349.2</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>3787921566000</v>
+        <v>3718492673500</v>
       </c>
       <c r="L3" s="6" t="n">
-        <v>28.34</v>
+        <v>27.82055555555555</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>25.01505554783419</v>
+        <v>24.54417325634252</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>11.41493786444631</v>
+        <v>11.20571323292319</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>8.566439520148647</v>
+        <v>8.409425073521598</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.9001730858468662</v>
+        <v>0.8836737947924707</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>18.77319602542418</v>
+        <v>18.4386295881341</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>11.74001508562887</v>
+        <v>11.53079045410576</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0.01768436828293081</v>
+        <v>0.0180145574784605</v>
       </c>
       <c r="T3" s="4" t="n">
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1329177321156774</v>
+        <v>0.1334892100456622</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2179872191872054</v>
+        <v>0.2186149345582133</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -911,16 +911,16 @@
         <v>55.38675843985578</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>0.007135575942915392</v>
+        <v>0.007268806038700402</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.564813883253538</v>
+        <v>0.5653853291601371</v>
       </c>
       <c r="AJ3" s="4" t="n">
-        <v>0.4348430953694607</v>
+        <v>0.4361759126353973</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15203550913.91745</v>
+        <v>14940294292.07424</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -953,55 +953,55 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="3" t="n">
-        <v>342.48</v>
+        <v>337.7601</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.08672063028023591</v>
+        <v>0.07174395221769303</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>-0.1618413646264164</v>
+        <v>-0.1733924769339957</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>226.11</v>
+        <v>231.9</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>4144731073229</v>
+        <v>4087610318170</v>
       </c>
       <c r="L4" s="6" t="n">
-        <v>17.00496524329692</v>
+        <v>16.77061072492552</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.28506888432769</v>
+        <v>20.0367316513445</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>9.295891091354594</v>
+        <v>9.167779445821287</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>6.497430801898576</v>
+        <v>6.407886233918312</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>0.1512261449403892</v>
+        <v>0.1491420165781369</v>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>12.85837247513144</v>
+        <v>12.68281745430563</v>
       </c>
       <c r="R4" s="6" t="n">
-        <v>9.423384267570821</v>
+        <v>9.294727050295267</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0.01285318614375071</v>
+        <v>0.01303357372686403</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1617003944987826</v>
+        <v>-0.1630066711104461</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2894990403021651</v>
+        <v>0.2895004357856084</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1037,16 +1037,16 @@
         <v>216.7961956521739</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>0.002481896753095071</v>
+        <v>0.002546185887557471</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7794591474858877</v>
+        <v>0.7802242373772644</v>
       </c>
       <c r="AJ4" s="4" t="n">
-        <v>0.3807963280117856</v>
+        <v>0.3807855964975712</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>9037288460.22608</v>
+        <v>8780084436.692057</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1079,13 +1079,13 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="3" t="n">
-        <v>258.9</v>
+        <v>255.95</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0.143046357615894</v>
+        <v>0.1300220750551875</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>-0.09853760445682458</v>
+        <v>-0.1088091922005571</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>287.2</v>
@@ -1094,40 +1094,40 @@
         <v>196</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>2785013190000</v>
+        <v>2753279745000</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>20.54761904761904</v>
+        <v>20.31349206349206</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.91468509085089</v>
+        <v>22.65537250005575</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>3.59041510674505</v>
+        <v>3.549504621751238</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>5.048273086545085</v>
+        <v>4.990751241796889</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>0.2325948755136572</v>
+        <v>0.2299446055918137</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11.53569605152817</v>
+        <v>11.41203452682512</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>3.777372357157591</v>
+        <v>3.736879297790326</v>
       </c>
       <c r="S5" s="4" t="n">
-        <v>-0.004174127448207885</v>
+        <v>-0.004221740660078738</v>
       </c>
       <c r="T5" s="4" t="n">
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1032990867579909</v>
+        <v>-0.1033697608175691</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.172964637968436</v>
+        <v>0.173391249565207</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8373056543606789</v>
+        <v>0.8299690414036144</v>
       </c>
       <c r="AJ5" s="4" t="n">
-        <v>0.4628431787348057</v>
+        <v>0.4631367298186026</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11149656040.69295</v>
+        <v>10968742815.88841</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="3" t="n">
-        <v>228.45</v>
+        <v>231.85</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.2096901912450992</v>
+        <v>0.2276938973087166</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>-0.03420140356810686</v>
+        <v>-0.01982751331698651</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>236.54</v>
@@ -1220,40 +1220,40 @@
         <v>164.07</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>5533287450000</v>
+        <v>5615638850000</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>28.73584905660377</v>
+        <v>29.16352201257861</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.44972202479861</v>
+        <v>17.68601524812359</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>18.26354329980955</v>
+        <v>18.53535790790477</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.13358793627502</v>
+        <v>24.49276587010446</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>0.230668720318316</v>
+        <v>0.234101741325461</v>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>23.75048445009351</v>
+        <v>24.10291504577026</v>
       </c>
       <c r="R6" s="6" t="n">
-        <v>18.3177303618522</v>
+        <v>18.58954496994742</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0.02295308189709176</v>
+        <v>0.02261648289579733</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6467797604893595</v>
+        <v>0.6489594520547943</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.8963443512833744</v>
+        <v>0.9012376830240194</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1289,16 +1289,16 @@
         <v>547.1389961389962</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>0.001225651127161305</v>
+        <v>0.001207677377614837</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.319691597318945</v>
+        <v>1.32054676429171</v>
       </c>
       <c r="AJ6" s="4" t="n">
-        <v>0.4383378111093153</v>
+        <v>0.4317778435528599</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>27901456266.45962</v>
+        <v>27611364582.45171</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1331,13 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="3" t="n">
-        <v>610.6799999999999</v>
+        <v>612.34</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-0.06108450790268349</v>
+        <v>-0.05853227151557139</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-0.2277693474962064</v>
+        <v>-0.2256702073849266</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>790.8</v>
@@ -1346,40 +1346,40 @@
         <v>520.26</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>1555699098568</v>
+        <v>1559927926274</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>22.69342251950948</v>
+        <v>22.75510962467484</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>18.47076246649536</v>
+        <v>18.5171841519619</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6.815827952788196</v>
+        <v>6.834355290184361</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.945001512129576</v>
+        <v>5.961161698332064</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-4.652151616499438</v>
+        <v>-4.664797473058339</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>15.43405464143754</v>
+        <v>15.47354981950463</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>7.240173401598262</v>
+        <v>7.258700738994428</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0.02633928375848379</v>
+        <v>0.02626788027179828</v>
       </c>
       <c r="T7" s="4" t="n">
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2286131967033695</v>
+        <v>0.2288644665373669</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2645939221475511</v>
+        <v>0.2650237051818187</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1415,16 +1415,16 @@
         <v>73.76137339055794</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>0.00343878954607978</v>
+        <v>0.003429467289414378</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7922193469194103</v>
+        <v>0.7899715646321138</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>0.4334697486246399</v>
+        <v>0.4305095519557905</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9758755852.047087</v>
+        <v>9643384803.507463</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1457,13 +1457,13 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="3" t="n">
-        <v>376.365</v>
+        <v>353.16</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-0.14085649848781</v>
+        <v>-0.1938274839742138</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-0.2455044804843333</v>
+        <v>-0.2920233346029709</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>498.83</v>
@@ -1472,40 +1472,40 @@
         <v>297.38</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>1486471404943</v>
+        <v>1394822157665</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>318.9533898305085</v>
+        <v>299.2881355932204</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>182.7533851053701</v>
+        <v>170.173813773925</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>14.34554864400351</v>
+        <v>13.46106561214642</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.02626706808814</v>
+        <v>13.16146952497179</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>-8.490449391262828</v>
+        <v>-7.966965862974454</v>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>123.0956439094613</v>
+        <v>115.4759858384603</v>
       </c>
       <c r="R8" s="6" t="n">
-        <v>14.288831246615</v>
+        <v>13.40434821475791</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0.003876293873423652</v>
+        <v>0.004130992591661913</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7452666589273276</v>
+        <v>0.7587202693289992</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1158572282041415</v>
+        <v>0.1168689092940987</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.558741390314899</v>
+        <v>1.561010339993693</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>0.5585073610096054</v>
+        <v>0.5768528101800358</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12593178765.41164</v>
+        <v>12355976978.32685</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1583,13 +1583,13 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="3" t="n">
-        <v>357.16</v>
+        <v>356.19</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.02744377485994853</v>
+        <v>0.02465337150678981</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>-0.2784646464646464</v>
+        <v>-0.2804242424242425</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>495</v>
@@ -1598,40 +1598,40 @@
         <v>289.96</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>1699217272800</v>
+        <v>1694602420200</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>44.31265508684864</v>
+        <v>44.18610421836228</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.69518790186196</v>
+        <v>19.77589658200599</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>19.07004481055845</v>
+        <v>19.01558337672832</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>17.07517865382686</v>
+        <v>17.02641428428127</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>0.4409328550721075</v>
+        <v>0.4396736112817234</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>34.72656295643818</v>
+        <v>33.09814861756883</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>19.4678271772311</v>
+        <v>19.41336574340097</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0.02318891211308784</v>
+        <v>0.02325532613666101</v>
       </c>
       <c r="T9" s="4" t="n">
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.249922940956525</v>
+        <v>1.234341388019142</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8363526329837438</v>
+        <v>0.8338156854346666</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1661,22 +1661,22 @@
         <v>0.3158098943384995</v>
       </c>
       <c r="AF9" s="6" t="n">
-        <v>0.7095611787315823</v>
+        <v>0.6781853318791496</v>
       </c>
       <c r="AG9" s="6" t="n">
         <v>8.080685358255451</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>0.007111658640385261</v>
+        <v>0.007131025576237402</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.595720636413219</v>
+        <v>1.596254174885275</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4220684542205427</v>
+        <v>0.4044752988131968</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8246770402.908705</v>
+        <v>8202662230.823149</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1709,13 +1709,13 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="3" t="n">
-        <v>925.41</v>
+        <v>916.72</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.08298420128730255</v>
+        <v>0.07281451141018147</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>-0.1560328317373462</v>
+        <v>-0.1639580483356133</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1096.5</v>
@@ -1724,40 +1724,40 @@
         <v>844.0599999999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>410399901390</v>
+        <v>406546068880</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>46.47965846308387</v>
+        <v>46.04319437468609</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.76182472164299</v>
+        <v>40.40170770286464</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>1.397881722930511</v>
+        <v>1.384755009179562</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.25971480587305</v>
+        <v>12.14459078337163</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>3.666498058226308</v>
+        <v>3.632068056253143</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>27.62169325431928</v>
+        <v>27.35536066897028</v>
       </c>
       <c r="R10" s="6" t="n">
-        <v>1.361388281463416</v>
+        <v>1.348261567712467</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>0.02145712016541574</v>
+        <v>0.02166052183030519</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1402742340532397</v>
+        <v>0.1396348568558514</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1141708647487798</v>
+        <v>0.1141161844836454</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1793,16 +1793,16 @@
         <v>71.24675324675324</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>0.005986535697690754</v>
+        <v>0.006043284754341565</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1852983164375997</v>
+        <v>-0.1867199324069447</v>
       </c>
       <c r="AJ10" s="4" t="n">
-        <v>0.2121511746098779</v>
+        <v>0.2126071463403524</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1759134798.335028</v>
+        <v>1725807903.57981</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1835,13 +1835,13 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="3" t="n">
-        <v>82.67</v>
+        <v>79.515</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-0.091438598297653</v>
+        <v>-0.1261127391271063</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3475653066056349</v>
+        <v>-0.372464683134717</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>126.71</v>
@@ -1850,40 +1850,40 @@
         <v>65.08</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>344232919717</v>
+        <v>331095686479</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>25.59442724458205</v>
+        <v>24.61764705882353</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>22.0872941090372</v>
+        <v>21.24101282371175</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7.116549155952964</v>
+        <v>6.844954660608628</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>11.48610645172674</v>
+        <v>11.04775316933654</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>0.7522264592614969</v>
+        <v>0.7235186513629844</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>11.4208111816902</v>
+        <v>10.99144827283608</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7.224260375895655</v>
+        <v>6.952665880551319</v>
       </c>
       <c r="S11" s="4" t="n">
-        <v>0.03193944381914101</v>
+        <v>0.03320673886428702</v>
       </c>
       <c r="T11" s="4" t="n">
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.158785096908266</v>
+        <v>0.1589676661436026</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1394926439203128</v>
+        <v>0.1398208305094693</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.1031865540721662</v>
+        <v>0.09876506134673883</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>0.3372071964773972</v>
+        <v>0.3510195225927256</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2386878968.761574</v>
+        <v>2334662547.279826</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -1961,13 +1961,13 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="3" t="n">
-        <v>507.94</v>
+        <v>506.37</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0.0223206073467852</v>
+        <v>0.01916069996887737</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>-0.05541711607840227</v>
+        <v>-0.05833674266374089</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>537.74</v>
@@ -1976,40 +1976,40 @@
         <v>464.01</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1095552215044</v>
+        <v>1092165954900</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>12.77193864722152</v>
+        <v>12.73246165451345</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.898059458622</v>
+        <v>22.8272568036128</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>2.847905479114189</v>
+        <v>2.839102841790858</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>1.458909073671947</v>
+        <v>1.454399707908933</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>0.3514692927730677</v>
+        <v>0.3503829306246767</v>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>15.47838585153044</v>
+        <v>15.43412911231932</v>
       </c>
       <c r="R12" s="6" t="n">
-        <v>3.078641116138575</v>
+        <v>3.069838478815245</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>0.02210300857182555</v>
+        <v>0.02217153894182423</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422261558757375</v>
+        <v>-0.4422255041833006</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06010655451571356</v>
+        <v>0.0601519584450636</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2048,13 +2048,13 @@
         <v>0</v>
       </c>
       <c r="AI12" s="6" t="n">
-        <v>0.06724006786338242</v>
+        <v>0.06358180459102618</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>0.1511957847235217</v>
+        <v>0.1441489762039075</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2183146565.369246</v>
+        <v>2134271324.979162</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2087,13 +2087,13 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="3" t="n">
-        <v>362.06</v>
+        <v>355.495</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.1123878203851001</v>
+        <v>0.09221761091476877</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-0.0121145975443383</v>
+        <v>-0.0300272851296044</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>366.5</v>
@@ -2102,40 +2102,40 @@
         <v>279.1</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>970143390600</v>
+        <v>952552394366</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>15.56577815993121</v>
+        <v>15.2835339638865</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.4666350458924</v>
+        <v>14.20385687501344</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3.259528985697151</v>
+        <v>3.200426009098453</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2.695360685321331</v>
+        <v>2.646487451881751</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>0.8150124596875519</v>
+        <v>0.8002343654549694</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>20.3757341197939</v>
+        <v>20.18690848396307</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6.377664407508576</v>
+        <v>6.318561430909878</v>
       </c>
       <c r="S13" s="4" t="n">
-        <v>0.08876522876349327</v>
+        <v>-0.1706299841996402</v>
       </c>
       <c r="T13" s="4" t="n">
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07597780068080895</v>
+        <v>0.07601295186044599</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2903803502202146</v>
+        <v>-0.2903302039302701</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2171,16 +2171,16 @@
         <v>0.7415371100533208</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>0.01657183892172568</v>
+        <v>0.016877874513003</v>
       </c>
       <c r="AI13" s="6" t="n">
-        <v>0.7815359821724135</v>
+        <v>0.7829981646916716</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>0.1869514303997223</v>
+        <v>0.1811657040472596</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2128562539.052266</v>
+        <v>2057715817.144755</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2213,13 +2213,13 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="3" t="n">
-        <v>378.75</v>
+        <v>374.6051</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0.0931366543247576</v>
+        <v>0.08117377084354138</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>-0.0176880981404155</v>
+        <v>-0.02843815649557802</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>385.57</v>
@@ -2228,40 +2228,40 @@
         <v>293.89</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>707144131166</v>
+        <v>699405407181</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>32.17926932880204</v>
+        <v>31.82711129991504</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.44450593632437</v>
+        <v>25.15069679986761</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>15.89516568885992</v>
+        <v>15.72121487099892</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>20.60149997867986</v>
+        <v>20.37604477798908</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2.169983622501454</v>
+        <v>2.146236123842956</v>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>24.69733765777717</v>
+        <v>24.43138384703416</v>
       </c>
       <c r="R14" s="6" t="n">
-        <v>16.15363988414854</v>
+        <v>15.97968906628754</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.02971529999881631</v>
+        <v>0.03004409143002525</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2646843844927316</v>
+        <v>0.2654564425460595</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1341573332662278</v>
+        <v>0.1344633994277662</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2297,16 +2297,16 @@
         <v>42.07640067911715</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>0.007075907590759076</v>
+        <v>0.007154200516757514</v>
       </c>
       <c r="AI14" s="6" t="n">
-        <v>0.3059802668322294</v>
+        <v>0.310400170607982</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>0.194316063042982</v>
+        <v>0.1932800424713141</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2541795901.85787</v>
+        <v>2500028819.762655</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2339,13 +2339,13 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="3" t="n">
-        <v>585.71</v>
+        <v>580.08</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.04009730421288138</v>
+        <v>0.03009961282513229</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>-0.0264452644526445</v>
+        <v>-0.03580333100628297</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>601.62</v>
@@ -2354,40 +2354,40 @@
         <v>464.52</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>513688755560</v>
+        <v>508751042880</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32.16419549697968</v>
+        <v>31.85502471169687</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.54365946055357</v>
+        <v>26.27829833612504</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>14.64209889576148</v>
+        <v>14.50135515434826</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>92.06847620744966</v>
+        <v>91.18348957405098</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1.421542568839726</v>
+        <v>1.407878324311602</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>23.83074496111412</v>
+        <v>23.60748068728522</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>15.02268208420032</v>
+        <v>14.88193834278711</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.03201938882635097</v>
+        <v>0.0323301548570577</v>
       </c>
       <c r="T15" s="4" t="n">
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2117468408897714</v>
+        <v>0.2122179413689604</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1524203980450276</v>
+        <v>0.1527873237135888</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2423,16 +2423,16 @@
         <v>26.73130193905817</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>0.005753700636833928</v>
+        <v>0.005809543511239829</v>
       </c>
       <c r="AI15" s="6" t="n">
-        <v>0.2953640136919465</v>
+        <v>0.2973451624970729</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>0.2150318203930366</v>
+        <v>0.2082374535025665</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1719478519.295687</v>
+        <v>1682747835.859172</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="n">
-        <v>400.94</v>
+        <v>397.47</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.1918549562262346</v>
+        <v>0.1815398549689269</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.1314501104804818</v>
+        <v>-0.1389671158095402</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>461.62</v>
@@ -2480,40 +2480,40 @@
         <v>255.97</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>364111417340</v>
+        <v>360960157366</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>25.78226480612179</v>
+        <v>25.55912803035175</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.58661222082426</v>
+        <v>18.41946344297264</v>
       </c>
       <c r="N16" s="6" t="n">
-        <v>0.8089045969933063</v>
+        <v>0.8019038039450912</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.475648361256495</v>
+        <v>3.445567801039105</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>-0.7812093552873196</v>
+        <v>-0.7744482527212325</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>15.86982949734115</v>
+        <v>15.74751222163568</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0.9083049911025506</v>
+        <v>0.9013041980543355</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0.06486201441452442</v>
+        <v>0.06542827378051382</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3871416963891676</v>
+        <v>0.3876152315448156</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.00951823030784138</v>
+        <v>0.009596695305573943</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2549,16 +2549,16 @@
         <v>4.672413793103448</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>0.02232254202623834</v>
+        <v>0.02251742269856844</v>
       </c>
       <c r="AI16" s="6" t="n">
-        <v>0.4504607441891266</v>
+        <v>0.4514190203223158</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>0.2221615484033596</v>
+        <v>0.2225811641902752</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1698075315.897207</v>
+        <v>1652932050.859612</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2591,13 +2591,13 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="3" t="n">
-        <v>162.24</v>
+        <v>160.41</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.3227884058832864</v>
+        <v>0.3078679005654461</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>-0.08032424465733223</v>
+        <v>-0.09069780624681145</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>176.41</v>
@@ -2606,40 +2606,40 @@
         <v>108.35</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>672397190400</v>
+        <v>664812828600</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>20.88030888030888</v>
+        <v>20.64864864864865</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.83028633895608</v>
+        <v>14.52659372863773</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1.862286573976624</v>
+        <v>1.841625110507949</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2.610708559796437</v>
+        <v>2.581743597964377</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2.044530244530246</v>
+        <v>2.021846846846848</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>9.804068087713192</v>
+        <v>9.700204140619562</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1.950305185841688</v>
+        <v>1.929643722373013</v>
       </c>
       <c r="S17" s="4" t="n">
-        <v>0.04543891681317769</v>
+        <v>0.04594870271609292</v>
       </c>
       <c r="T17" s="4" t="n">
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4079504874737749</v>
+        <v>0.4214377461346563</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08409163954739807</v>
+        <v>0.0841329187987252</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2675,16 +2675,16 @@
         <v>69.43781094527363</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>0.02539447731755424</v>
+        <v>0.02568418427778817</v>
       </c>
       <c r="AI17" s="6" t="n">
-        <v>-0.5347963570637113</v>
+        <v>-0.5325856171137178</v>
       </c>
       <c r="AJ17" s="4" t="n">
-        <v>0.2501156810565711</v>
+        <v>0.2520003467982942</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2233231122.294317</v>
+        <v>2185200238.471715</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2717,13 +2717,13 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="3" t="n">
-        <v>278.43</v>
+        <v>276.56</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.3428019860341793</v>
+        <v>0.333783418660391</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.009392677980574193</v>
+        <v>-0.01604582488348094</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>281.07</v>
@@ -2732,40 +2732,40 @@
         <v>173.33</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>670988015967</v>
+        <v>666481505929</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>32.18843930635838</v>
+        <v>31.97225433526011</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.49337957011385</v>
+        <v>22.3038622500684</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>6.85178053454033</v>
+        <v>6.805762398564266</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>7.995634310529474</v>
+        <v>7.94193378917513</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-3.985437024642537</v>
+        <v>-3.95866991177366</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>20.74000995988972</v>
+        <v>20.60641248455472</v>
       </c>
       <c r="R18" s="6" t="n">
-        <v>7.143971815978923</v>
+        <v>7.097953680002859</v>
       </c>
       <c r="S18" s="4" t="n">
-        <v>0.02788127292115465</v>
+        <v>0.02806979613623811</v>
       </c>
       <c r="T18" s="4" t="n">
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4310183672499801</v>
+        <v>0.4334851057090825</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08533159948788738</v>
+        <v>0.0864773700708803</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2801,16 +2801,16 @@
         <v>34.55406797116375</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>0.01896347376360306</v>
+        <v>0.01909169800404975</v>
       </c>
       <c r="AI18" s="6" t="n">
-        <v>-0.1841029868977979</v>
+        <v>-0.1825808175733511</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>0.223981199313451</v>
+        <v>0.2214933992875132</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1803740917.020087</v>
+        <v>1758370585.903526</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2843,13 +2843,13 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="3" t="n">
-        <v>108.42</v>
+        <v>107.605</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-0.03848884404052344</v>
+        <v>-0.04571658423704594</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>-0.1978395975140573</v>
+        <v>-0.2038694880142053</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>135.16</v>
@@ -2858,40 +2858,40 @@
         <v>98.88</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>862815033600</v>
+        <v>856329198400</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>39.14079422382672</v>
+        <v>38.84657039711192</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>35.08882375835756</v>
+        <v>34.81461048671868</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1.172557938682322</v>
+        <v>1.163743746466623</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8.778402247602759</v>
+        <v>8.712414442476435</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>9.464955694125377</v>
+        <v>9.393807023301616</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>21.59343200354817</v>
+        <v>21.44203175611009</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1.257122517938682</v>
+        <v>1.248308325722983</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0.01565688991722269</v>
+        <v>0.01577547516216983</v>
       </c>
       <c r="T19" s="4" t="n">
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1154775233667968</v>
+        <v>0.1158122941496467</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04945453700575531</v>
+        <v>0.04957887035413444</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2927,16 +2927,16 @@
         <v>11.52840300107181</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>0.009015864231691571</v>
+        <v>0.009084150364760003</v>
       </c>
       <c r="AI19" s="6" t="n">
-        <v>-0.05246586081636603</v>
+        <v>-0.05659379693867067</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>0.3113917043958672</v>
+        <v>0.3096511495772121</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2879669142.357646</v>
+        <v>2835244034.580903</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -2969,13 +2969,13 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="3" t="n">
-        <v>146.92</v>
+        <v>146.64</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.03618031565538482</v>
+        <v>0.0342055641689738</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>-0.1215545590433483</v>
+        <v>-0.1232286995515696</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>167.25</v>
@@ -2984,40 +2984,40 @@
         <v>137.62</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>349259537024</v>
+        <v>348593917071</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>21.76592592592592</v>
+        <v>21.72740740740741</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.83950251127317</v>
+        <v>20.79641508838826</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>4.013001390568986</v>
+        <v>4.005899700110304</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>6.553252563937323</v>
+        <v>6.541655465743587</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.77091216931239</v>
+        <v>20.73415449735472</v>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>17.61285108798344</v>
+        <v>17.5837707113955</v>
       </c>
       <c r="R20" s="6" t="n">
-        <v>4.301217219229708</v>
+        <v>4.294115528771027</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0.04556210586428885</v>
+        <v>0.04564287872350072</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04445515981735171</v>
+        <v>0.04476696176058592</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02441244393764164</v>
+        <v>0.02463207400701717</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3053,16 +3053,16 @@
         <v>24.23489167616876</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>0.02920364824394229</v>
+        <v>0.029259410801964</v>
       </c>
       <c r="AI20" s="6" t="n">
-        <v>-0.05775603397441936</v>
+        <v>-0.06044833438413458</v>
       </c>
       <c r="AJ20" s="4" t="n">
-        <v>0.1729319476117685</v>
+        <v>0.1580980011872035</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1328230494.789775</v>
+        <v>1304549121.592146</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3095,13 +3095,13 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="3" t="n">
-        <v>318.07</v>
+        <v>319.15</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-0.08024407708198944</v>
+        <v>-0.07712106517658668</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>-0.2546690099589924</v>
+        <v>-0.2521382542472174</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>426.75</v>
@@ -3110,31 +3110,31 @@
         <v>289.1</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>317153004190</v>
+        <v>318229890550</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22.21159217877095</v>
+        <v>22.28701117318435</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.21189285149808</v>
+        <v>21.2839173878568</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1.874692652563011</v>
+        <v>1.88105813206365</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>19.02639345248841</v>
+        <v>19.09099717157128</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-7.619092665973789</v>
+        <v>-7.644963134987689</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>15.79071729834832</v>
+        <v>15.83574704369642</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2.232201991949213</v>
+        <v>2.238567471449851</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0.04761424233885955</v>
+        <v>0.04745311627987172</v>
       </c>
       <c r="T21" s="4" t="n">
         <v>0.03240467921310985</v>
@@ -3179,16 +3179,16 @@
         <v>8.712271973466004</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>0.02920740717452133</v>
+        <v>0.0291085696381012</v>
       </c>
       <c r="AI21" s="6" t="n">
-        <v>0.7033510113784245</v>
+        <v>0.6979491357779022</v>
       </c>
       <c r="AJ21" s="4" t="n">
-        <v>0.2541235475434628</v>
+        <v>0.2469017628299812</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1285111662.326097</v>
+        <v>1248847853.988887</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3221,13 +3221,13 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="3" t="n">
-        <v>456.16</v>
+        <v>469.6</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>1.041258323301694</v>
+        <v>1.101400623953165</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>-0.2198792605133993</v>
+        <v>-0.1968942930925385</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>584.73</v>
@@ -3236,40 +3236,40 @@
         <v>149.22</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>743814496000</v>
+        <v>765729760000</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>115.7766497461929</v>
+        <v>119.2365228426396</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>34.61308492998636</v>
+        <v>35.57299457741164</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>18.00785609490377</v>
+        <v>18.54600344122987</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.06743067951922</v>
+        <v>11.39817013120314</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.9347105667582545</v>
+        <v>0.9626434871699342</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>69.32305430117559</v>
+        <v>71.39696511849226</v>
       </c>
       <c r="R22" s="6" t="n">
-        <v>17.98824587822298</v>
+        <v>18.52639322454909</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>0.01129717160016198</v>
+        <v>0.01096936281176813</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.344880988804673</v>
+        <v>2.351883198451703</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8617462116679628</v>
+        <v>0.8650211849362994</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.530233599649874</v>
+        <v>2.535464031877131</v>
       </c>
       <c r="AJ22" s="4" t="n">
-        <v>0.6613200552914463</v>
+        <v>0.6658835817300017</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>11146352301.10236</v>
+        <v>10810280032.1679</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3347,55 +3347,55 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="3" t="n">
-        <v>1646.19</v>
+        <v>1709.9</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>0.4145198908376047</v>
+        <v>0.4692639132440486</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>-0.1768885377707554</v>
+        <v>-0.1450329006580131</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>735.4299999999999</v>
+        <v>766.24</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>634471242604</v>
+        <v>659026222811</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>51.64731494920174</v>
+        <v>53.5123385341074</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>34.37443160214586</v>
+        <v>35.65198634398397</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>15.52909117228788</v>
+        <v>16.08985838075154</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.13485938402045</v>
+        <v>26.04249815673481</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.515821468071722</v>
+        <v>3.642780439021532</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>39.40138856090405</v>
+        <v>40.8364643374262</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.39640417207558</v>
+        <v>15.95717138053924</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01823154876070442</v>
+        <v>0.01759613889800855</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.5024921880010842</v>
+        <v>0.5009637336276282</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2640704275990478</v>
+        <v>0.2624803193606415</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3429,16 +3429,16 @@
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="4" t="n">
-        <v>0.004726064427556965</v>
+        <v>0.004549973682671501</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.688280059650562</v>
+        <v>1.685894462757977</v>
       </c>
       <c r="AJ23" s="4" t="n">
-        <v>0.3983574561603626</v>
+        <v>0.4085822230380305</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2396109337.855273</v>
+        <v>2355176406.519214</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3475,13 +3475,13 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="3" t="n">
-        <v>210.51</v>
+        <v>210.575</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.07577821464065282</v>
+        <v>-0.07549283904781467</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>-0.1723609199921369</v>
+        <v>-0.1721053666207981</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>254.35</v>
@@ -3490,40 +3490,40 @@
         <v>176.77</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>166380788700</v>
+        <v>166432162750</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>78.84269662921345</v>
+        <v>78.86704119850184</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>87.92257775092823</v>
+        <v>87.44396782006693</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>1.770102544816214</v>
+        <v>1.770649106335443</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>27.29882554028853</v>
+        <v>27.30725470593443</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.4219719216214408</v>
+        <v>0.4221022155500209</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>29.50097679136691</v>
+        <v>29.50836874100719</v>
       </c>
       <c r="R24" s="6" t="n">
-        <v>2.181305268365338</v>
+        <v>2.181851829884568</v>
       </c>
       <c r="S24" s="4" t="n">
-        <v>-0.001262164950898565</v>
+        <v>-0.001261775347565746</v>
       </c>
       <c r="T24" s="4" t="n">
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.1032713252270281</v>
+        <v>-0.09808482889538817</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1482776801428523</v>
+        <v>0.1487023210673839</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3562,13 +3562,13 @@
         <v>0</v>
       </c>
       <c r="AI24" s="6" t="n">
-        <v>1.204834063154122</v>
+        <v>1.209805708792098</v>
       </c>
       <c r="AJ24" s="4" t="n">
-        <v>0.341210965489833</v>
+        <v>0.3343499177733284</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1271156612.602015</v>
+        <v>1252503616.502017</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3601,13 +3601,13 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="3" t="n">
-        <v>1037.93</v>
+        <v>1026.52</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.135168503526607</v>
+        <v>0.1226895573305835</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>-0.1005727952581911</v>
+        <v>-0.1104602292914151</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>1153.99</v>
@@ -3616,40 +3616,40 @@
         <v>727.15</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>306196615510</v>
+        <v>302830585640</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>15.8124619134674</v>
+        <v>15.63863497867154</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.35127124923024</v>
+        <v>14.19183809123103</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>2.596272717722174</v>
+        <v>2.567731802911724</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>2.537703418552737</v>
+        <v>2.509806358051848</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>0.3706221969631351</v>
+        <v>0.3665479344720718</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>27.42027252922626</v>
+        <v>27.3130502226611</v>
       </c>
       <c r="R25" s="6" t="n">
-        <v>7.298851213020511</v>
+        <v>7.270310298210061</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>-0.1355828180231606</v>
+        <v>-0.1370898514503167</v>
       </c>
       <c r="T25" s="4" t="n">
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1018161136293438</v>
+        <v>0.1019457013348026</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3827991531369952</v>
+        <v>-0.382756348332898</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3685,16 +3685,16 @@
         <v>0.327057203580088</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>0.01734220997562456</v>
+        <v>0.01753497252854304</v>
       </c>
       <c r="AI25" s="6" t="n">
-        <v>1.578882813963619</v>
+        <v>1.574600638425609</v>
       </c>
       <c r="AJ25" s="4" t="n">
-        <v>0.3904956600205113</v>
+        <v>0.3900886619133271</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1966192999.941805</v>
+        <v>1930788751.819092</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3727,13 +3727,13 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="3" t="n">
-        <v>234.71</v>
+        <v>234.33</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>-0.194819897084048</v>
+        <v>-0.196123499142367</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>-0.2940203332731757</v>
+        <v>-0.2951633279191481</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>332.46</v>
@@ -3742,40 +3742,40 @@
         <v>199.19</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>221128271140</v>
+        <v>220770260220</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>20.49868995633188</v>
+        <v>20.46200873362445</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.23041882450315</v>
+        <v>18.19766716538466</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>3.200258638435822</v>
+        <v>3.194531960287712</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>6.403225618251481</v>
+        <v>6.391767415534657</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>0.2498774415219527</v>
+        <v>0.2494303002606548</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>17.21399859071574</v>
+        <v>17.18960451636767</v>
       </c>
       <c r="R26" s="6" t="n">
-        <v>4.041105563772668</v>
+        <v>4.035378885624557</v>
       </c>
       <c r="S26" s="4" t="n">
-        <v>0.06164295469650729</v>
+        <v>0.0617534589475318</v>
       </c>
       <c r="T26" s="4" t="n">
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1244223269725431</v>
+        <v>0.1244303210769231</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04471020269214554</v>
+        <v>0.04463937618784009</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3811,16 +3811,16 @@
         <v>6.337467700258398</v>
       </c>
       <c r="AH26" s="4" t="n">
-        <v>0.02871628818542031</v>
+        <v>0.02876285580164725</v>
       </c>
       <c r="AI26" s="6" t="n">
-        <v>0.8945046703446532</v>
+        <v>0.8909179076988699</v>
       </c>
       <c r="AJ26" s="4" t="n">
-        <v>0.7802150538044913</v>
+        <v>0.7800852243335122</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1406683275.038429</v>
+        <v>1336569933.709947</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3853,13 +3853,13 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="3" t="n">
-        <v>1159.5</v>
+        <v>1142.95996</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.07325337454319381</v>
+        <v>0.05794362573329348</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>-0.1030054539125054</v>
+        <v>-0.1158009051173946</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1292.65</v>
@@ -3868,40 +3868,40 @@
         <v>712.05</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1091948689500</v>
+        <v>1076372256573</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>38.84422110552764</v>
+        <v>38.29011591289783</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.77901331224493</v>
+        <v>26.37991756488887</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>13.70661801550979</v>
+        <v>13.51109580990839</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>30.54215885947047</v>
+        <v>30.10648095587236</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.4117648282821975</v>
+        <v>0.4058910837971775</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>32.32125339411498</v>
+        <v>31.87884164317769</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>14.28425609860191</v>
+        <v>14.08873389300051</v>
       </c>
       <c r="S27" s="4" t="n">
-        <v>0.01836524022862523</v>
+        <v>0.01863100788555111</v>
       </c>
       <c r="T27" s="4" t="n">
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4505471375140544</v>
+        <v>0.4514873224570342</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2229077529986656</v>
+        <v>0.223375610820848</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3937,16 +3937,16 @@
         <v>33.16107129385138</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>0.005769728331177231</v>
+        <v>0.005853223414755492</v>
       </c>
       <c r="AI27" s="6" t="n">
-        <v>0.3496622436410882</v>
+        <v>0.3535963268178253</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>0.3293615887888398</v>
+        <v>0.3289385023092813</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3241610819.776656</v>
+        <v>3184520761.432145</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -3979,13 +3979,13 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="3" t="n">
-        <v>217.15</v>
+        <v>214.825</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.193787835548668</v>
+        <v>0.181006086906482</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>-0.06501614639397202</v>
+        <v>-0.07502691065662004</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>232.25</v>
@@ -3994,40 +3994,40 @@
         <v>146.29</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>342506352000</v>
+        <v>338839176000</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>17.45578778135048</v>
+        <v>17.26889067524116</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.19237291027406</v>
+        <v>16.0165047662502</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>2.706939531648871</v>
+        <v>2.677956642350765</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>3.089584484273255</v>
+        <v>3.056504659608575</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>0.4441030908474639</v>
+        <v>0.4393481302846254</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>24.08928858145637</v>
+        <v>23.9643294374212</v>
       </c>
       <c r="R28" s="6" t="n">
-        <v>5.587243651652981</v>
+        <v>5.558260762354876</v>
       </c>
       <c r="S28" s="4" t="n">
-        <v>-0.04579185147491805</v>
+        <v>-0.04628744581765835</v>
       </c>
       <c r="T28" s="4" t="n">
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07802530722811984</v>
+        <v>0.07819345901422725</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3291535514892736</v>
+        <v>-0.3290564360672744</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4063,16 +4063,16 @@
         <v>0.4478854275047432</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>0.01911121344692609</v>
+        <v>0.01931804957523566</v>
       </c>
       <c r="AI28" s="6" t="n">
-        <v>1.37951057203454</v>
+        <v>1.380365496584128</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>0.2853123854269439</v>
+        <v>0.2830584978640965</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>948020811.0540599</v>
+        <v>923971551.4352275</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4105,46 +4105,46 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="3" t="n">
-        <v>958.16</v>
+        <v>999.455</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>2.037727345159483</v>
+        <v>2.168648016778378</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>-0.2365258964143426</v>
+        <v>-0.2036215139442231</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>118.52</v>
+        <v>125.66</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>1082136322400</v>
+        <v>1128774482450</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>21.38272706985048</v>
+        <v>22.30428475786655</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.16601772337544</v>
+        <v>6.431762173036028</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>11.98724242195981</v>
+        <v>12.50387135221658</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.73035701520988</v>
+        <v>11.19281640919741</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>0.03047665586957272</v>
+        <v>0.03179014579206375</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>15.56078369472976</v>
+        <v>16.24316686345945</v>
       </c>
       <c r="R29" s="6" t="n">
-        <v>11.78099256042714</v>
+        <v>12.29762149068392</v>
       </c>
       <c r="S29" s="4" t="n">
-        <v>0.02418549258373919</v>
+        <v>0.02318620805742684</v>
       </c>
       <c r="T29" s="4" t="n">
         <v>0.4885110111106685</v>
@@ -4189,16 +4189,16 @@
         <v>21.25786163522013</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>0.0005531435250897554</v>
+        <v>0.0005302890075090925</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.885622767400017</v>
+        <v>2.881535671182869</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>0.8386657793584558</v>
+        <v>0.8444754705332586</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>31030678607.43187</v>
+        <v>30383306965.06598</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4231,13 +4231,13 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="3" t="n">
-        <v>145.59</v>
+        <v>141.02</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>-0.01261442513895117</v>
+        <v>-0.0436079829184346</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>-0.2523340488686667</v>
+        <v>-0.2758029230816634</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>194.726</v>
@@ -4246,40 +4246,40 @@
         <v>81.23999999999999</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>150519968580</v>
+        <v>145795219240</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>90.42857142857144</v>
+        <v>87.59006211180126</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>30.91229582683789</v>
+        <v>29.92550196914318</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>10.21721209475971</v>
+        <v>9.896498726581591</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>12.01617689357622</v>
+        <v>11.63899488654522</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>144.6857142857174</v>
+        <v>140.144099378885</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>44.84665192891946</v>
+        <v>43.49246753797649</v>
       </c>
       <c r="R30" s="6" t="n">
-        <v>10.62109479907684</v>
+        <v>10.30038143089872</v>
       </c>
       <c r="S30" s="4" t="n">
-        <v>0.03042785647118822</v>
+        <v>0.03141392443369942</v>
       </c>
       <c r="T30" s="4" t="n">
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.925326929294648</v>
+        <v>1.926937105419893</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2391478002190743</v>
+        <v>0.2397122868509145</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4318,13 +4318,13 @@
         <v>0</v>
       </c>
       <c r="AI30" s="6" t="n">
-        <v>0.6932180537876992</v>
+        <v>0.7155914085469055</v>
       </c>
       <c r="AJ30" s="4" t="n">
-        <v>0.6118506236410205</v>
+        <v>0.6137207924122136</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2575518048.896585</v>
+        <v>2504658146.245494</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4357,13 +4357,13 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="3" t="n">
-        <v>28.81</v>
+        <v>28.585</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>0.1441620194928301</v>
+        <v>0.1352263563763467</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>-0.01369394043135919</v>
+        <v>-0.02139678192399863</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>29.21</v>
@@ -4372,40 +4372,40 @@
         <v>23.58</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>164200866400</v>
+        <v>162918492400</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>38.06818181818182</v>
+        <v>37.77087737843552</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.867727049097358</v>
+        <v>9.791405875563322</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>2.577883484049234</v>
+        <v>2.557750759859332</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>1.927317642915835</v>
+        <v>1.912265700199554</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.6367156074014481</v>
+        <v>-0.6317429933207357</v>
       </c>
       <c r="Q31" s="6" t="n">
-        <v>17.93558827629911</v>
+        <v>17.83400605196451</v>
       </c>
       <c r="R31" s="6" t="n">
-        <v>3.554679515197186</v>
+        <v>3.534546791007284</v>
       </c>
       <c r="S31" s="4" t="n">
-        <v>0.06690585890842778</v>
+        <v>0.06743249239642485</v>
       </c>
       <c r="T31" s="4" t="n">
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857847063338064</v>
+        <v>2.857554048770599</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.0494803444525882</v>
+        <v>-0.04958914097975653</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4441,16 +4441,16 @@
         <v>3.815424934481467</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>0.05970149253731343</v>
+        <v>0.06017141857617631</v>
       </c>
       <c r="AI31" s="6" t="n">
-        <v>0.3305507131034656</v>
+        <v>0.3390656089871334</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>0.2036684369353451</v>
+        <v>0.2054653071889354</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1030479174.718319</v>
+        <v>1013938551.226678</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4483,13 +4483,13 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="3" t="n">
-        <v>163.68</v>
+        <v>170.575</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>-0.02577224360697039</v>
+        <v>0.01526698159054862</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>-0.1597535934291581</v>
+        <v>-0.1243583162217661</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>194.8</v>
@@ -4498,40 +4498,40 @@
         <v>124.8</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1161890485589</v>
+        <v>1210834980323</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6.973377601755823</v>
+        <v>7.196211096548772</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003478066430933068</v>
+        <v>0.003615363739354024</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>5.988923840185221</v>
+        <v>6.180299226055801</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>4.339938366634638</v>
+        <v>4.478620607673715</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>0.015605548321709</v>
+        <v>0.01610422185830497</v>
       </c>
       <c r="Q32" s="6" t="n">
-        <v>7.040390110614151</v>
+        <v>7.266507184860058</v>
       </c>
       <c r="R32" s="6" t="n">
-        <v>5.958671535935959</v>
+        <v>6.150046921806539</v>
       </c>
       <c r="S32" s="4" t="n">
-        <v>0.08048511319355385</v>
+        <v>0.07799286014384453</v>
       </c>
       <c r="T32" s="4" t="n">
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>2003.958139883792</v>
+        <v>1989.45286044567</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2608.178912384364</v>
+        <v>2590.833748909825</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4567,14 +4567,14 @@
         <v>55.63395918385022</v>
       </c>
       <c r="AH32" s="4" t="n">
-        <v>1.832844574780059</v>
+        <v>1.758757144950901</v>
       </c>
       <c r="AI32" s="6" t="inlineStr"/>
       <c r="AJ32" s="4" t="n">
-        <v>1.187135798893464</v>
+        <v>1.176534148093971</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3873753680.121977</v>
+        <v>3793481895.037031</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4611,22 +4611,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="n">
-        <v>552.6</v>
+        <v>564.1900000000001</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.4803107904371822</v>
+        <v>0.511358206400206</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>-0.1774704910468422</v>
+        <v>-0.1602191030469017</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>284.3</v>
+        <v>289.25</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>69650117345</v>
+        <v>71110929922</v>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
       <c r="M33" s="6" t="inlineStr"/>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.817982688236564</v>
+        <v>1.81859451685127</v>
       </c>
       <c r="AJ33" s="4" t="n">
-        <v>0.4123977515525699</v>
+        <v>0.4127445894451111</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5307148870.407312</v>
+        <v>5046306299.042116</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4691,13 +4691,13 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="3" t="n">
-        <v>149.74</v>
+        <v>149.08501</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>-0.06964894166383273</v>
+        <v>-0.07371846643810553</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>-0.3363765289842225</v>
+        <v>-0.3392793387697216</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>225.64</v>
@@ -4706,38 +4706,38 @@
         <v>104.83</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>1957980091285</v>
+        <v>1949415487210</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>-97.23376623376623</v>
+        <v>-96.80844805194806</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>143.5760632568891</v>
+        <v>141.3733824790211</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>118.128512294721</v>
+        <v>117.6117941001508</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>6.901805948563164</v>
+        <v>6.871616193799913</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-0.9723376623376623</v>
+        <v>-0.9680844805194806</v>
       </c>
       <c r="Q34" s="6" t="n">
-        <v>456.8807514482842</v>
+        <v>454.8254108975282</v>
       </c>
       <c r="R34" s="6" t="n">
-        <v>114.8610613143288</v>
+        <v>114.3443431197587</v>
       </c>
       <c r="S34" s="4" t="n">
-        <v>-0.0145164908093352</v>
+        <v>-0.01458026787336082</v>
       </c>
       <c r="T34" s="4" t="n">
         <v>0.3324295397788084</v>
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.059407012541581</v>
+        <v>4.069354325502593</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4777,10 +4777,10 @@
       </c>
       <c r="AI34" s="6" t="inlineStr"/>
       <c r="AJ34" s="4" t="n">
-        <v>0.791710326769945</v>
+        <v>0.7915464580604885</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13119625143.11764</v>
+        <v>13034631031.47679</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4817,13 +4817,13 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="n">
-        <v>773.17</v>
+        <v>769.08</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.1317388341719334</v>
+        <v>0.1257520371780472</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>-0.007955143256733077</v>
+        <v>-0.01320297163093265</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>779.37</v>
@@ -4832,7 +4832,7 @@
         <v>629.28</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>823610239196</v>
+        <v>819253414852</v>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
       <c r="M35" s="6" t="inlineStr"/>
@@ -4858,13 +4858,13 @@
       <c r="AG35" s="6" t="inlineStr"/>
       <c r="AH35" s="4" t="inlineStr"/>
       <c r="AI35" s="6" t="n">
-        <v>0.9952653864121357</v>
+        <v>0.9953985772066537</v>
       </c>
       <c r="AJ35" s="4" t="n">
-        <v>0.1145393709711229</v>
+        <v>0.1151398278706942</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32489047548.78963</v>
+        <v>31697736864.29349</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -4897,55 +4897,55 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="3" t="n">
-        <v>417.01</v>
+        <v>425.15</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.3047464694862398</v>
+        <v>0.3302150104363801</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>-0.1294154488517746</v>
+        <v>-0.1124217118997913</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>230.3</v>
+        <v>237.9</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>2162814024800</v>
+        <v>2205031972000</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>27.70372087631853</v>
+        <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.643742455565232</v>
+        <v>0.655918488201354</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>13.95756055860477</v>
+        <v>14.07436022855125</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>9.634196613208077</v>
+        <v>9.714817505368815</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>0.5204269220342786</v>
+        <v>0.5247819590387496</v>
       </c>
       <c r="Q36" s="6" t="n">
-        <v>18.35433323546673</v>
+        <v>18.51345021489235</v>
       </c>
       <c r="R36" s="6" t="n">
-        <v>13.47298114713415</v>
+        <v>13.58978081708063</v>
       </c>
       <c r="S36" s="4" t="n">
-        <v>0.01804608982065956</v>
+        <v>0.01789632973916031</v>
       </c>
       <c r="T36" s="4" t="n">
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>42.03541056957871</v>
+        <v>41.58997372241032</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>42.03984231566236</v>
+        <v>41.60168636340224</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4979,16 +4979,16 @@
       </c>
       <c r="AG36" s="6" t="inlineStr"/>
       <c r="AH36" s="4" t="n">
-        <v>0.2637826431020839</v>
+        <v>0.258732212160414</v>
       </c>
       <c r="AI36" s="6" t="n">
-        <v>2.18287447020443</v>
+        <v>2.17411419941909</v>
       </c>
       <c r="AJ36" s="4" t="n">
-        <v>0.3479026760906407</v>
+        <v>0.3503892774790344</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4528731837.996655</v>
+        <v>4438748489.58455</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -5025,53 +5025,53 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="n">
-        <v>28.37</v>
+        <v>28.295</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>-0.004910565687755053</v>
+        <v>-0.007541221576842672</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>-0.05433333333333334</v>
+        <v>-0.05683333333333329</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>11.54</v>
+        <v>11.77</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>71127468236</v>
+        <v>70939432983</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>-22.33858267716535</v>
+        <v>-22.27952755905512</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-77.62729724526305</v>
+        <v>-78.10331445565421</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.969471638820435</v>
+        <v>1.964265069444829</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>2.16934862050064</v>
+        <v>2.163613648821487</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>0.1662406152719283</v>
+        <v>0.165801135323201</v>
       </c>
       <c r="Q37" s="6" t="n">
-        <v>16.49280466710744</v>
+        <v>16.46172446</v>
       </c>
       <c r="R37" s="6" t="n">
-        <v>2.762881579288385</v>
+        <v>2.757675009912778</v>
       </c>
       <c r="S37" s="4" t="n">
-        <v>0.03064920000760872</v>
+        <v>0.03073044015621633</v>
       </c>
       <c r="T37" s="4" t="n">
         <v>-0.05149919890135046</v>
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.0219303172237848</v>
+        <v>0.02200689340269579</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2922701356886339</v>
+        <v>0.2966219527418959</v>
       </c>
       <c r="AJ37" s="4" t="n">
-        <v>0.1981179980120381</v>
+        <v>0.1984575546482785</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>565299740.3450707</v>
+        <v>536106086.608327</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -5153,13 +5153,13 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="3" t="n">
-        <v>329.82</v>
+        <v>326.43</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>-0.1151235739584761</v>
+        <v>-0.1242186290924302</v>
       </c>
       <c r="H38" s="4" t="n">
-        <v>-0.1488296472167024</v>
+        <v>-0.1575782600841312</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>387.49</v>
@@ -5168,40 +5168,40 @@
         <v>290.97</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>222730744200</v>
+        <v>220441443300</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>20.00121285627653</v>
+        <v>19.79563371740449</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>17.0777527986065</v>
+        <v>16.89628197915581</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.649254150559633</v>
+        <v>2.622024232512222</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>6.523277712952159</v>
+        <v>6.456229288214703</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>1.240249880170862</v>
+        <v>1.227502178109801</v>
       </c>
       <c r="Q38" s="6" t="n">
-        <v>9.567090446529688</v>
+        <v>9.474496169713639</v>
       </c>
       <c r="R38" s="6" t="n">
-        <v>2.813468583255029</v>
+        <v>2.786238665207617</v>
       </c>
       <c r="S38" s="4" t="n">
-        <v>0.06757935485764879</v>
+        <v>0.06828117151962051</v>
       </c>
       <c r="T38" s="4" t="n">
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1711852895486679</v>
+        <v>0.1715970260099522</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.003502196421537818</v>
+        <v>0.003736949153157587</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5237,16 +5237,16 @@
         <v>1.675370415350984</v>
       </c>
       <c r="AH38" s="4" t="n">
-        <v>0.01073312716026924</v>
+        <v>0.01084459148975278</v>
       </c>
       <c r="AI38" s="6" t="n">
-        <v>0.9722676603901</v>
+        <v>0.9674884975755212</v>
       </c>
       <c r="AJ38" s="4" t="n">
-        <v>0.251938710333756</v>
+        <v>0.235365187593823</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>875846347.6576233</v>
+        <v>811114483.4227986</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>
@@ -5279,13 +5279,13 @@
       <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="n">
-        <v>154.04</v>
+        <v>157.38</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>-0.2129170981777634</v>
+        <v>-0.1958510316230616</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>-0.554437116741872</v>
+        <v>-0.5447761194029852</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>345.72</v>
@@ -5294,40 +5294,40 @@
         <v>114.5</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>443707598800</v>
+        <v>453328368600</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>25.93265993265993</v>
+        <v>26.49494949494949</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.47537023688456</v>
+        <v>17.83827475543388</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>6.58730364321981</v>
+        <v>6.73013403901541</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>10.42926319751576</v>
+        <v>10.6553975722217</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>0.7814842114842107</v>
+        <v>0.7984288834288826</v>
       </c>
       <c r="Q39" s="6" t="n">
-        <v>17.71528799576284</v>
+        <v>18.01502846371935</v>
       </c>
       <c r="R39" s="6" t="n">
-        <v>8.441574850797233</v>
+        <v>8.584405246592832</v>
       </c>
       <c r="S39" s="4" t="n">
-        <v>-0.05338200216552162</v>
+        <v>-0.05224910162394809</v>
       </c>
       <c r="T39" s="4" t="n">
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.483954822194548</v>
+        <v>0.485286545823532</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4888090421977518</v>
+        <v>0.4904724170212567</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5363,16 +5363,16 @@
         <v>5.261852979556329</v>
       </c>
       <c r="AH39" s="4" t="n">
-        <v>0.01298364061282784</v>
+        <v>0.01270809505655102</v>
       </c>
       <c r="AI39" s="6" t="n">
-        <v>2.09189437610112</v>
+        <v>2.08829802185471</v>
       </c>
       <c r="AJ39" s="4" t="n">
-        <v>0.5897025832694764</v>
+        <v>0.5910198990571904</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3790128030.546288</v>
+        <v>3677088460.671458</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46 ET</t>
+          <t>2026-09-04 11:29 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-05)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>36.52625570776257</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.70467535643121</v>
+        <v>33.69777391889267</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.06701319198068</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08371480577969637</v>
+        <v>0.08393675486332652</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.1089653641838908</v>
+        <v>0.109217750504</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -784,13 +784,13 @@
         <v>0.003312810575991499</v>
       </c>
       <c r="AI2" s="6" t="n">
-        <v>0.3175081738012429</v>
+        <v>0.3175082681883968</v>
       </c>
       <c r="AJ2" s="4" t="n">
         <v>0.2982180051172286</v>
       </c>
       <c r="AK2" s="5" t="n">
-        <v>15054656555.68585</v>
+        <v>15068297719.42556</v>
       </c>
       <c r="AL2" s="7" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.76111111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.4917294889757</v>
+        <v>24.47938757198791</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18176987936921</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1334892100456622</v>
+        <v>0.134060687975647</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2186149345582133</v>
+        <v>0.2192426134081278</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -914,13 +914,13 @@
         <v>0.007284370622373425</v>
       </c>
       <c r="AI3" s="6" t="n">
-        <v>0.5641256900349051</v>
+        <v>0.5641257661392662</v>
       </c>
       <c r="AJ3" s="4" t="n">
         <v>0.436990889842759</v>
       </c>
       <c r="AK3" s="5" t="n">
-        <v>15142370432.28577</v>
+        <v>15152987391.87846</v>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         <v>408.61</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>231.9</v>
+        <v>233.23</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>4096080585860</v>
@@ -974,7 +974,7 @@
         <v>16.80536246276067</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.07825138230969</v>
+        <v>20.09596201330776</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.186776742526359</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1630066711104461</v>
+        <v>-0.1637443158166806</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2895004357856084</v>
+        <v>0.2902410152781847</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1040,13 +1040,13 @@
         <v>0.002540920640548366</v>
       </c>
       <c r="AI4" s="6" t="n">
-        <v>0.7792817166538825</v>
+        <v>0.7792817695885479</v>
       </c>
       <c r="AJ4" s="4" t="n">
         <v>0.380392782346809</v>
       </c>
       <c r="AK4" s="5" t="n">
-        <v>8933902284.886404</v>
+        <v>8960028124.446817</v>
       </c>
       <c r="AL4" s="7" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.51666666666667</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.88197048247476</v>
+        <v>22.89359237692626</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.585006601949257</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.103369760817569</v>
+        <v>-0.103824933681235</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.173391249565207</v>
+        <v>0.1738178611619783</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="AI5" s="6" t="n">
-        <v>0.8294919958643998</v>
+        <v>0.8294920097490567</v>
       </c>
       <c r="AJ5" s="4" t="n">
         <v>0.4620984616318468</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>11137677032.44418</v>
+        <v>11143961798.5466</v>
       </c>
       <c r="AL5" s="7" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
         <v>236.54</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>164.07</v>
+        <v>164.27</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>5579549560000</v>
@@ -1226,7 +1226,7 @@
         <v>28.97610062893081</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.57235485252426</v>
+        <v>17.51064972048581</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.41623915318069</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6489594520547941</v>
+        <v>0.6547701593865769</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9012376830240194</v>
+        <v>0.9074423675885106</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1292,13 +1292,13 @@
         <v>0.001215488800138913</v>
       </c>
       <c r="AI6" s="6" t="n">
-        <v>1.321246907143806</v>
+        <v>1.321246893536647</v>
       </c>
       <c r="AJ6" s="4" t="n">
         <v>0.4309848297610164</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>28130876056.99435</v>
+        <v>28151931598.37947</v>
       </c>
       <c r="AL6" s="7" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.91973244147157</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>18.65114751511503</v>
+        <v>18.64733463517109</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.883798726731451</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2288644665373671</v>
+        <v>0.229115736371365</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2650237051818187</v>
+        <v>0.2656378462090505</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1418,13 +1418,13 @@
         <v>0.003404834865509023</v>
       </c>
       <c r="AI7" s="6" t="n">
-        <v>0.7903980498531025</v>
+        <v>0.7903980197347575</v>
       </c>
       <c r="AJ7" s="4" t="n">
         <v>0.4311231712219439</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>9855166431.974243</v>
+        <v>9859210942.495321</v>
       </c>
       <c r="AL7" s="7" t="inlineStr">
         <is>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>300.0677966101695</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.6171253286651</v>
+        <v>170.4836248303892</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.49613238178326</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7587202693289996</v>
+        <v>0.7600974692361278</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1168689092940987</v>
+        <v>0.1172420675402921</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1544,13 +1544,13 @@
         <v>0</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>1.557031210113276</v>
+        <v>1.557031430906623</v>
       </c>
       <c r="AJ8" s="4" t="n">
         <v>0.5751750302023199</v>
       </c>
       <c r="AK8" s="5" t="n">
-        <v>12709866709.84739</v>
+        <v>12713048850.29205</v>
       </c>
       <c r="AL8" s="7" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.40384615384615</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.87055927234632</v>
+        <v>19.81248559279334</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.10928907905369</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.234655076651144</v>
+        <v>1.241205221115606</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8340731425702643</v>
+        <v>0.8361840458910876</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1670,13 +1670,13 @@
         <v>0.007097053605107644</v>
       </c>
       <c r="AI9" s="6" t="n">
-        <v>1.596165826791928</v>
+        <v>1.596166254295669</v>
       </c>
       <c r="AJ9" s="4" t="n">
-        <v>0.4045962527016247</v>
+        <v>0.4045971083689626</v>
       </c>
       <c r="AK9" s="5" t="n">
-        <v>8442914990.74994</v>
+        <v>8446407465.018311</v>
       </c>
       <c r="AL9" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v>45.99397287795078</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>40.35851711735455</v>
+        <v>40.40253408166894</v>
       </c>
       <c r="N10" s="6" t="n">
         <v>1.383274666316969</v>
@@ -1754,10 +1754,10 @@
         <v>0.08167323631476142</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>0.1396348568558514</v>
+        <v>0.1383932697137118</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>0.1141161844836454</v>
+        <v>0.113636913092201</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>0.1022561610551892</v>
@@ -1796,13 +1796,13 @@
         <v>0.006049752113045187</v>
       </c>
       <c r="AI10" s="6" t="n">
-        <v>-0.1873632514767745</v>
+        <v>-0.187363216879025</v>
       </c>
       <c r="AJ10" s="4" t="n">
         <v>0.2128794639580522</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>1772359591.536369</v>
+        <v>1773082751.406657</v>
       </c>
       <c r="AL10" s="7" t="inlineStr">
         <is>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1841,10 +1841,10 @@
         <v>-0.1400153661157778</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>-0.3824481098571541</v>
+        <v>-0.3823993685872139</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>126.71</v>
+        <v>126.7</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>65.08</v>
@@ -1856,7 +1856,7 @@
         <v>24.22600619195047</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.90309065529075</v>
+        <v>20.89979836309201</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.736058684580629</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1589676661436026</v>
+        <v>0.1591502353789391</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.139820830509469</v>
+        <v>0.1401490170986257</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1922,13 +1922,13 @@
         <v>0</v>
       </c>
       <c r="AI11" s="6" t="n">
-        <v>0.09591897935031683</v>
+        <v>0.09591916068103171</v>
       </c>
       <c r="AJ11" s="4" t="n">
         <v>0.3642770786058767</v>
       </c>
       <c r="AK11" s="5" t="n">
-        <v>2403089955.437776</v>
+        <v>2403652557.287776</v>
       </c>
       <c r="AL11" s="7" t="inlineStr">
         <is>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.72391249685693</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.81192953834584</v>
+        <v>22.81190288538</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.837196538167393</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422255041833006</v>
+        <v>-0.4422248524908636</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.0601519584450636</v>
+        <v>0.06019736237441342</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2054,7 +2054,7 @@
         <v>0.1442597908977017</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>2173477516.089017</v>
+        <v>2173551447.071838</v>
       </c>
       <c r="AL12" s="7" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.41874462596733</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.32951582906882</v>
+        <v>14.32904772789045</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.228739643789499</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07601295186044621</v>
+        <v>0.07604810304008325</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2903302039302701</v>
+        <v>-0.2902800576403256</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2180,7 +2180,7 @@
         <v>0.1763642599566969</v>
       </c>
       <c r="AK13" s="5" t="n">
-        <v>2098214693.317708</v>
+        <v>2098286839.733989</v>
       </c>
       <c r="AL13" s="7" t="inlineStr">
         <is>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.86661002548853</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.18190982644482</v>
+        <v>25.17358996145257</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.74072553115447</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2654564425460597</v>
+        <v>0.2658746755740737</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1344633994277662</v>
+        <v>0.1347694655893046</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2306,7 +2306,7 @@
         <v>0.1927988600450382</v>
       </c>
       <c r="AK14" s="5" t="n">
-        <v>2546328478.613403</v>
+        <v>2546726302.867838</v>
       </c>
       <c r="AL14" s="7" t="inlineStr">
         <is>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.80724876441516</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.23888632476035</v>
+        <v>26.22869314951558</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.47960612148334</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2122179413689604</v>
+        <v>0.2126890418481491</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1527873237135888</v>
+        <v>0.1531542493821503</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2432,7 +2432,7 @@
         <v>0.2087876204900281</v>
       </c>
       <c r="AK15" s="5" t="n">
-        <v>1707444703.905229</v>
+        <v>1707831345.901896</v>
       </c>
       <c r="AL15" s="7" t="inlineStr">
         <is>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.53790753006238</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.40417065877212</v>
+        <v>18.39786938919137</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8012380197787745</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3876152315448156</v>
+        <v>0.3880904897099517</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009596695305574166</v>
+        <v>0.009675158503585024</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2558,7 +2558,7 @@
         <v>0.2227524147564033</v>
       </c>
       <c r="AK16" s="5" t="n">
-        <v>1709417242.470483</v>
+        <v>1719200773.493347</v>
       </c>
       <c r="AL16" s="7" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.52252252252253</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.44056253331197</v>
+        <v>14.44358064113855</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.830376091508336</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4211719574760673</v>
+        <v>0.4208749916256767</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08393020134943607</v>
+        <v>0.08376876315147408</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2684,7 +2684,7 @@
         <v>0.2544364048602604</v>
       </c>
       <c r="AK17" s="5" t="n">
-        <v>2254732914.848759</v>
+        <v>2256061842.156931</v>
       </c>
       <c r="AL17" s="7" t="inlineStr">
         <is>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.81849710982659</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.19660112484208</v>
+        <v>22.1907608068986</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.773032922178313</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4334851057090825</v>
+        <v>0.4338623802359649</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.0864773700708803</v>
+        <v>0.08668675260466174</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2810,7 +2810,7 @@
         <v>0.2228567277751259</v>
       </c>
       <c r="AK18" s="5" t="n">
-        <v>1783855402.516428</v>
+        <v>1787902412.120972</v>
       </c>
       <c r="AL18" s="7" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.67870036101083</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.66416400303926</v>
+        <v>34.65470304705833</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.158714790171776</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1158122941496464</v>
+        <v>0.1161169180554869</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04957887035413444</v>
+        <v>0.04970321858612436</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2936,7 +2936,7 @@
         <v>0.3103786878848654</v>
       </c>
       <c r="AK19" s="5" t="n">
-        <v>2881156546.489607</v>
+        <v>2885935951.151047</v>
       </c>
       <c r="AL19" s="7" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.69333333333333</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.76663298822076</v>
+        <v>20.76326738947317</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.999617435483501</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04462448706240485</v>
+        <v>0.04479381430745821</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02449234083794738</v>
+        <v>0.02455680977052066</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3062,7 +3062,7 @@
         <v>0.1582296409033706</v>
       </c>
       <c r="AK20" s="5" t="n">
-        <v>1322803199.782758</v>
+        <v>1322977819.723002</v>
       </c>
       <c r="AL20" s="7" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v>22.41969273743017</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>21.41062722033973</v>
+        <v>21.39423365261975</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1.892256660814773</v>
@@ -3140,10 +3140,10 @@
         <v>0.03240467921310985</v>
       </c>
       <c r="U21" s="4" t="n">
-        <v>0.04712918994413395</v>
+        <v>0.04793156424581002</v>
       </c>
       <c r="V21" s="4" t="n">
-        <v>0.01431960424055423</v>
+        <v>0.01431952960230776</v>
       </c>
       <c r="W21" s="4" t="n">
         <v>0.1300647261025379</v>
@@ -3188,7 +3188,7 @@
         <v>0.2479791008294195</v>
       </c>
       <c r="AK21" s="5" t="n">
-        <v>1266289791.918237</v>
+        <v>1266306443.710938</v>
       </c>
       <c r="AL21" s="7" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>121.2106598984771</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.17673556289284</v>
+        <v>36.11576140682565</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.85305996852681</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.350514025450246</v>
+        <v>2.356170690494402</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8642593634459987</v>
+        <v>0.8667727034885493</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="AI22" s="6" t="n">
-        <v>2.537609502426293</v>
+        <v>2.537609377471187</v>
       </c>
       <c r="AJ22" s="4" t="n">
         <v>0.6719580495745092</v>
       </c>
       <c r="AK22" s="5" t="n">
-        <v>10982010964.43387</v>
+        <v>10986583156.008</v>
       </c>
       <c r="AL22" s="7" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
         <v>1999.96</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>766.24</v>
+        <v>786.75</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>660945604406</v>
@@ -3368,7 +3368,7 @@
         <v>53.24383164005805</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.75582100799534</v>
+        <v>35.72645155346037</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.00912490249805</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4890954854078788</v>
+        <v>0.4903196182353853</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2524977808262898</v>
+        <v>0.2532979490632601</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3432,13 +3432,13 @@
         <v>0.00453676058966225</v>
       </c>
       <c r="AI23" s="6" t="n">
-        <v>1.688292808004549</v>
+        <v>1.688292688877463</v>
       </c>
       <c r="AJ23" s="4" t="n">
         <v>0.4104047912906506</v>
       </c>
       <c r="AK23" s="5" t="n">
-        <v>2391216706.498515</v>
+        <v>2392755811.302897</v>
       </c>
       <c r="AL23" s="7" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>79.49438202247188</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>88.13953303957832</v>
+        <v>87.63889358355186</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.784733576254056</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.09808482889538805</v>
+        <v>-0.0929326150531018</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1487023210673839</v>
+        <v>0.1491269236518411</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3568,7 +3568,7 @@
         <v>0.3351860805767036</v>
       </c>
       <c r="AK24" s="5" t="n">
-        <v>1277409530.063648</v>
+        <v>1277474825.238647</v>
       </c>
       <c r="AL24" s="7" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
         <v>1153.99</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>727.15</v>
+        <v>733.5700000000001</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>306397220270</v>
@@ -3622,7 +3622,7 @@
         <v>15.82282145033516</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.35898468605917</v>
+        <v>14.3572962824658</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.597973666194663</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1019457013348026</v>
+        <v>0.1020752890402612</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3827563483328981</v>
+        <v>-0.3827135435288007</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3694,7 +3694,7 @@
         <v>0.3891830400092962</v>
       </c>
       <c r="AK25" s="5" t="n">
-        <v>1967098606.966423</v>
+        <v>1967121941.07076</v>
       </c>
       <c r="AL25" s="7" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.51441048034935</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.24115580795119</v>
+        <v>18.23791296662955</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.202712929070727</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1246222934737096</v>
+        <v>0.1248222599748761</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04481772598957101</v>
+        <v>0.04492524928699626</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3820,7 +3820,7 @@
         <v>0.7801961678822183</v>
       </c>
       <c r="AK26" s="5" t="n">
-        <v>1355088229.680336</v>
+        <v>1360299929.83846</v>
       </c>
       <c r="AL26" s="7" t="inlineStr">
         <is>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.46566164154105</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.50085952967714</v>
+        <v>26.48370500115239</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.57303907322841</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4514873224570342</v>
+        <v>0.4524275074000139</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.223375610820848</v>
+        <v>0.2238434686430302</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3946,7 +3946,7 @@
         <v>0.3278665989608857</v>
       </c>
       <c r="AK27" s="5" t="n">
-        <v>3245355284.315865</v>
+        <v>3247614504.615072</v>
       </c>
       <c r="AL27" s="7" t="inlineStr">
         <is>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.5</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.23085342773265</v>
+        <v>16.22300117136641</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.713795699009713</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07819345901422725</v>
+        <v>0.07871532616834775</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3290564360672743</v>
+        <v>-0.3289593206452751</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4072,7 +4072,7 @@
         <v>0.281987612132052</v>
       </c>
       <c r="AK28" s="5" t="n">
-        <v>940021797.8748667</v>
+        <v>941500907.732493</v>
       </c>
       <c r="AL28" s="7" t="inlineStr">
         <is>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
         <v>1255</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>125.66</v>
+        <v>128.4</v>
       </c>
       <c r="K29" s="5" t="n">
         <v>1148126580100</v>
@@ -4192,13 +4192,13 @@
         <v>0.0005213507903874719</v>
       </c>
       <c r="AI29" s="6" t="n">
-        <v>2.884292454259064</v>
+        <v>2.884292298340282</v>
       </c>
       <c r="AJ29" s="4" t="n">
         <v>0.8505963460831095</v>
       </c>
       <c r="AK29" s="5" t="n">
-        <v>30963849470.73486</v>
+        <v>30970310069.78719</v>
       </c>
       <c r="AL29" s="7" t="inlineStr">
         <is>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>87.73913043478261</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.97643176968632</v>
+        <v>29.95995010484869</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.913341441759435</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.926937105419893</v>
+        <v>1.928547281545138</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2397122868509145</v>
+        <v>0.2402767734827549</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4324,7 +4324,7 @@
         <v>0.6129734621011685</v>
       </c>
       <c r="AK30" s="5" t="n">
-        <v>2535969032.858816</v>
+        <v>2536904673.141098</v>
       </c>
       <c r="AL30" s="7" t="inlineStr">
         <is>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.59249471458774</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.745163447954399</v>
+        <v>9.745903733568273</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.545671125345391</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857554048770598</v>
+        <v>2.857261034203133</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04958914097975653</v>
+        <v>-0.04969793750692497</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4450,7 +4450,7 @@
         <v>0.2074754188779906</v>
       </c>
       <c r="AK31" s="5" t="n">
-        <v>1029179576.274991</v>
+        <v>1029419848.859768</v>
       </c>
       <c r="AL31" s="7" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.196211096548772</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003751542616829326</v>
+        <v>0.003748608100936018</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.180299226055801</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1917.200546161131</v>
+        <v>1918.702167519698</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2496.751648136735</v>
+        <v>2499.72805327578</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4574,7 +4574,7 @@
         <v>1.188436150548777</v>
       </c>
       <c r="AK32" s="5" t="n">
-        <v>3860416798.9248</v>
+        <v>3860931420.524801</v>
       </c>
       <c r="AL32" s="7" t="inlineStr">
         <is>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
         <v>671.83</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>289.25</v>
+        <v>294.8</v>
       </c>
       <c r="K33" s="5" t="n">
         <v>71466364523</v>
@@ -4652,13 +4652,13 @@
       <c r="AG33" s="6" t="inlineStr"/>
       <c r="AH33" s="4" t="inlineStr"/>
       <c r="AI33" s="6" t="n">
-        <v>1.819949615289042</v>
+        <v>1.819949549204461</v>
       </c>
       <c r="AJ33" s="4" t="n">
         <v>0.4145504822608118</v>
       </c>
       <c r="AK33" s="5" t="n">
-        <v>5122894375.495097</v>
+        <v>5128464776.332703</v>
       </c>
       <c r="AL33" s="7" t="inlineStr"/>
       <c r="AM33" s="2" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-96.07142857142857</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>140.2970824348549</v>
+        <v>139.6512710439887</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>116.7163977160784</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.069354325502593</v>
+        <v>4.104307113783343</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4780,7 +4780,7 @@
         <v>0.792031732777318</v>
       </c>
       <c r="AK34" s="5" t="n">
-        <v>13144272489.95751</v>
+        <v>13144960447.57998</v>
       </c>
       <c r="AL34" s="7" t="inlineStr">
         <is>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>0.1147149274533218</v>
       </c>
       <c r="AK35" s="5" t="n">
-        <v>32254975228.66363</v>
+        <v>32282065558.0605</v>
       </c>
       <c r="AL35" s="7" t="inlineStr"/>
       <c r="AM35" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
         <v>479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>237.9</v>
+        <v>241.62</v>
       </c>
       <c r="K36" s="5" t="n">
         <v>2224533136800</v>
@@ -4918,7 +4918,7 @@
         <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6617193902727103</v>
+        <v>0.6612684557085317</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.07436022855125</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.21661264153959</v>
+        <v>41.2454011459031</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.22822260474334</v>
+        <v>41.26055915818448</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -4988,7 +4988,7 @@
         <v>0.3541403848515018</v>
       </c>
       <c r="AK36" s="5" t="n">
-        <v>4549469512.579889</v>
+        <v>4549591637.554932</v>
       </c>
       <c r="AL36" s="7" t="inlineStr">
         <is>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
         <v>30</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>11.77</v>
+        <v>11.92</v>
       </c>
       <c r="K37" s="5" t="n">
         <v>70826611832</v>
@@ -5046,7 +5046,7 @@
         <v>-22.24409448818897</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-77.97909996014248</v>
+        <v>-78.67132773762907</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.961141127841617</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02200689340269579</v>
+        <v>0.02208346958160678</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="AI37" s="6" t="n">
-        <v>0.2961500575504797</v>
+        <v>0.2961500878968145</v>
       </c>
       <c r="AJ37" s="4" t="n">
         <v>0.1986934987575738</v>
       </c>
       <c r="AK37" s="5" t="n">
-        <v>543691092.4733177</v>
+        <v>543764745.8733177</v>
       </c>
       <c r="AL37" s="7" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>19.77926015767132</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.88230655981821</v>
+        <v>16.87637566460323</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.619855477977472</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1715970260099522</v>
+        <v>0.1720087624712363</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.003736949153157587</v>
+        <v>0.003971701884777579</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5246,7 +5246,7 @@
         <v>0.2355892750850924</v>
       </c>
       <c r="AK38" s="5" t="n">
-        <v>828214958.5648925</v>
+        <v>828758428.1069946</v>
       </c>
       <c r="AL38" s="7" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>26.73905723905724</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>18.00262536158065</v>
+        <v>17.9529854159251</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.792141246770985</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.485286545823532</v>
+        <v>0.4893933582399337</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4904724170212567</v>
+        <v>0.4924303962356122</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5372,7 +5372,7 @@
         <v>0.59317779056187</v>
       </c>
       <c r="AK39" s="5" t="n">
-        <v>3751154398.346746</v>
+        <v>3752571271.665853</v>
       </c>
       <c r="AL39" s="7" t="inlineStr">
         <is>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 18:30 ET</t>
+          <t>2026-09-05 10:17 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-06)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>36.52625570776257</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.69777391889267</v>
+        <v>33.57993253578827</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.06701319198068</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.08393675486332652</v>
+        <v>0.0877405923562895</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.109217750504</v>
+        <v>0.111542837260457</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.76111111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.47938757198791</v>
+        <v>24.46705808745777</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18176987936921</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.134060687975647</v>
+        <v>0.1346321659056318</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2192426134081278</v>
+        <v>0.2198702922580422</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.80536246276067</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.09596201330776</v>
+        <v>20.11391098360043</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.186776742526359</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.1637443158166806</v>
+        <v>-0.164490561956714</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2902410152781847</v>
+        <v>0.2909434328511566</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.51666666666667</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.89359237692626</v>
+        <v>22.90522608304126</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.585006601949257</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.103824933681235</v>
+        <v>-0.1042801065449011</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1738178611619783</v>
+        <v>0.1742444727587495</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>28.97610062893081</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.51064972048581</v>
+        <v>17.4874487372077</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.41623915318069</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6547701593865769</v>
+        <v>0.6569655793917459</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9074423675885106</v>
+        <v>0.9099517112314717</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.91973244147157</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>18.64733463517109</v>
+        <v>18.64352331385319</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.883798726731451</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.229115736371365</v>
+        <v>0.2293670062053623</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2656378462090505</v>
+        <v>0.2662519872362821</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>300.0677966101695</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.4836248303892</v>
+        <v>170.3554572187399</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.49613238178326</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7600974692361278</v>
+        <v>0.7614216856280478</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1172420675402921</v>
+        <v>0.1176152580105436</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.40384615384615</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.81248559279334</v>
+        <v>19.78946536052194</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.10928907905369</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.241205221115606</v>
+        <v>1.243812318569631</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8361840458910876</v>
+        <v>0.8382949492119105</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.22600619195047</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.89979836309201</v>
+        <v>20.89650710781945</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.736058684580629</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1591502353789391</v>
+        <v>0.1593328046142757</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1401490170986257</v>
+        <v>0.1404772036877822</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.72391249685693</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.81190288538</v>
+        <v>22.81187623247644</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.837196538167393</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422248524908636</v>
+        <v>-0.4422242007984266</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06019736237441342</v>
+        <v>0.06024276630376346</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.41874462596733</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.32904772789045</v>
+        <v>14.32857965729392</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.228739643789499</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07604810304008325</v>
+        <v>0.07608325421972029</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.2902800576403256</v>
+        <v>-0.290229911350381</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.86661002548853</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.17358996145257</v>
+        <v>25.16527559225406</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.74072553115447</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2658746755740737</v>
+        <v>0.2662929086020882</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1347694655893046</v>
+        <v>0.1350755317508432</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.80724876441516</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.22869314951558</v>
+        <v>26.21850789080149</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.47960612148334</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2126890418481491</v>
+        <v>0.2131601423273377</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1531542493821503</v>
+        <v>0.1535211750507113</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.53790753006238</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.39786938919137</v>
+        <v>18.39159523100312</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8012380197787745</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3880904897099517</v>
+        <v>0.3885640266273676</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009675158503585024</v>
+        <v>0.009753623419861635</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.52252252252253</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.44358064113855</v>
+        <v>14.44660001081058</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.830376091508336</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4208749916256767</v>
+        <v>0.4205780257752862</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08376876315147408</v>
+        <v>0.08360732495351209</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.81849710982659</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.1907608068986</v>
+        <v>22.18492356152836</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.773032922178313</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4338623802359649</v>
+        <v>0.4342396547628473</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08668675260466174</v>
+        <v>0.08689613513844319</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.67870036101083</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.65470304705833</v>
+        <v>34.64601214664498</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.158714790171776</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1161169180554869</v>
+        <v>0.1163968943177884</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04970321858612436</v>
+        <v>0.04982755194757948</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.69333333333333</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.76326738947317</v>
+        <v>20.75990288145795</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.999617435483501</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04479381430745821</v>
+        <v>0.04496314155251135</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02455680977052066</v>
+        <v>0.02463661523029792</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>121.2106598984771</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.11576140682565</v>
+        <v>36.05524592963388</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.85305996852681</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.356170690494402</v>
+        <v>2.361803720186356</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8667727034885493</v>
+        <v>0.8692858552626717</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v>53.24383164005805</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.72645155346037</v>
+        <v>35.69713030684876</v>
       </c>
       <c r="N23" s="6" t="n">
         <v>16.00912490249805</v>
@@ -3392,10 +3392,10 @@
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4903196182353853</v>
+        <v>0.4915437510628919</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2532979490632601</v>
+        <v>0.2540981173002304</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>79.49438202247188</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>87.63889358355186</v>
+        <v>87.14390934812964</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.784733576254056</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.0929326150531018</v>
+        <v>-0.08778040121081554</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1491269236518411</v>
+        <v>0.1495515262362979</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.82282145033516</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.3572962824658</v>
+        <v>14.35560827588817</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.597973666194663</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1020752890402612</v>
+        <v>0.1022048767457198</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3827135435288007</v>
+        <v>-0.3826707387247035</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.51441048034935</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.23791296662955</v>
+        <v>18.23467127810226</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.202712929070727</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1248222599748761</v>
+        <v>0.1250222264760426</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04492524928699626</v>
+        <v>0.04503277258442129</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.46566164154105</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.48370500115239</v>
+        <v>26.46657266718929</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.57303907322841</v>
@@ -3898,10 +3898,10 @@
         <v>0.4470491333778837</v>
       </c>
       <c r="U27" s="4" t="n">
-        <v>0.4524275074000139</v>
+        <v>0.4533676923429937</v>
       </c>
       <c r="V27" s="4" t="n">
-        <v>0.2238434686430302</v>
+        <v>0.2243113264652126</v>
       </c>
       <c r="W27" s="4" t="n">
         <v>0.1877209505000597</v>
@@ -3956,7 +3956,7 @@
       <c r="AM27" s="2" t="inlineStr"/>
       <c r="AN27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4000,7 +4000,7 @@
         <v>17.5</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>16.22300117136641</v>
+        <v>16.22045710401671</v>
       </c>
       <c r="N28" s="6" t="n">
         <v>2.713795699009713</v>
@@ -4024,10 +4024,10 @@
         <v>0.1147704687575744</v>
       </c>
       <c r="U28" s="4" t="n">
-        <v>0.07871532616834775</v>
+        <v>0.07888451526230011</v>
       </c>
       <c r="V28" s="4" t="n">
-        <v>-0.3289593206452751</v>
+        <v>-0.3288622052232759</v>
       </c>
       <c r="W28" s="4" t="n">
         <v>0.01207481297651363</v>
@@ -4082,7 +4082,7 @@
       <c r="AM28" s="2" t="inlineStr"/>
       <c r="AN28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
         <v>22.6866770810087</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>6.542030514116889</v>
+        <v>6.542031777108996</v>
       </c>
       <c r="N29" s="6" t="n">
         <v>12.71824201985068</v>
@@ -4150,7 +4150,7 @@
         <v>0.4885110111106685</v>
       </c>
       <c r="U29" s="4" t="n">
-        <v>2.467834188797144</v>
+        <v>2.467833519303727</v>
       </c>
       <c r="V29" s="4" t="n">
         <v>1.763697862828721</v>
@@ -4208,7 +4208,7 @@
       <c r="AM29" s="2" t="inlineStr"/>
       <c r="AN29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
         <v>87.73913043478261</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>29.95995010484869</v>
+        <v>29.94348655397498</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>9.913341441759435</v>
@@ -4276,10 +4276,10 @@
         <v>0.2088492352512745</v>
       </c>
       <c r="U30" s="4" t="n">
-        <v>1.928547281545138</v>
+        <v>1.930157457670382</v>
       </c>
       <c r="V30" s="4" t="n">
-        <v>0.2402767734827549</v>
+        <v>0.2408412601145953</v>
       </c>
       <c r="W30" s="4" t="n">
         <v>0.0527379523779448</v>
@@ -4334,7 +4334,7 @@
       <c r="AM30" s="2" t="inlineStr"/>
       <c r="AN30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
         <v>37.59249471458774</v>
       </c>
       <c r="M31" s="6" t="n">
-        <v>9.745903733568273</v>
+        <v>9.746644131661416</v>
       </c>
       <c r="N31" s="6" t="n">
         <v>2.545671125345391</v>
@@ -4402,10 +4402,10 @@
         <v>-0.01647099501783833</v>
       </c>
       <c r="U31" s="4" t="n">
-        <v>2.857261034203133</v>
+        <v>2.856968019635668</v>
       </c>
       <c r="V31" s="4" t="n">
-        <v>-0.04969793750692497</v>
+        <v>-0.04980673403409341</v>
       </c>
       <c r="W31" s="4" t="n">
         <v>0.02155311712267129</v>
@@ -4460,7 +4460,7 @@
       <c r="AM31" s="2" t="inlineStr"/>
       <c r="AN31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
         <v>7.196211096548772</v>
       </c>
       <c r="M32" s="6" t="n">
-        <v>0.003748608100936018</v>
+        <v>0.003745678172303852</v>
       </c>
       <c r="N32" s="6" t="n">
         <v>6.180299226055801</v>
@@ -4528,10 +4528,10 @@
         <v>0.4676285061130367</v>
       </c>
       <c r="U32" s="4" t="n">
-        <v>1918.702167519698</v>
+        <v>1920.203788878264</v>
       </c>
       <c r="V32" s="4" t="n">
-        <v>2499.72805327578</v>
+        <v>2502.704458414824</v>
       </c>
       <c r="W32" s="4" t="n">
         <v>0.4645609082788198</v>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="AN32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="AN33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
         <v>-96.07142857142857</v>
       </c>
       <c r="M34" s="6" t="n">
-        <v>139.6512710439887</v>
+        <v>139.0113779699848</v>
       </c>
       <c r="N34" s="6" t="n">
         <v>116.7163977160784</v>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="U34" s="4" t="inlineStr"/>
       <c r="V34" s="4" t="n">
-        <v>4.104307113783343</v>
+        <v>4.114355255273869</v>
       </c>
       <c r="W34" s="4" t="n">
         <v>-0.027727343466307</v>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="AN34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="AN35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
         <v>27.93555117653877</v>
       </c>
       <c r="M36" s="6" t="n">
-        <v>0.6612684557085317</v>
+        <v>0.660809059606603</v>
       </c>
       <c r="N36" s="6" t="n">
         <v>14.07436022855125</v>
@@ -4942,10 +4942,10 @@
         <v>0.3296825869948878</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>41.2454011459031</v>
+        <v>41.27477025386054</v>
       </c>
       <c r="V36" s="4" t="n">
-        <v>41.26055915818448</v>
+        <v>41.29289571162562</v>
       </c>
       <c r="W36" s="4" t="n">
         <v>0.2386060493906826</v>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AN36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
         <v>-22.24409448818897</v>
       </c>
       <c r="M37" s="6" t="n">
-        <v>-78.67132773762907</v>
+        <v>-76.47929971907686</v>
       </c>
       <c r="N37" s="6" t="n">
         <v>1.961141127841617</v>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="U37" s="4" t="inlineStr"/>
       <c r="V37" s="4" t="n">
-        <v>0.02208346958160678</v>
+        <v>0.019917309350306</v>
       </c>
       <c r="W37" s="4" t="n">
         <v>-0.03256622244159263</v>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="AN37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
         <v>19.77926015767132</v>
       </c>
       <c r="M38" s="6" t="n">
-        <v>16.87637566460323</v>
+        <v>16.8704489350708</v>
       </c>
       <c r="N38" s="6" t="n">
         <v>2.619855477977472</v>
@@ -5198,10 +5198,10 @@
         <v>0.08440587054082838</v>
       </c>
       <c r="U38" s="4" t="n">
-        <v>0.1720087624712363</v>
+        <v>0.1724204989325204</v>
       </c>
       <c r="V38" s="4" t="n">
-        <v>0.003971701884777579</v>
+        <v>0.00420645461639757</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0.03713461582139044</v>
@@ -5256,7 +5256,7 @@
       <c r="AM38" s="2" t="inlineStr"/>
       <c r="AN38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
         <v>26.73905723905724</v>
       </c>
       <c r="M39" s="6" t="n">
-        <v>17.9529854159251</v>
+        <v>17.93673275465103</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>6.792141246770985</v>
@@ -5324,10 +5324,10 @@
         <v>0.1735047648913743</v>
       </c>
       <c r="U39" s="4" t="n">
-        <v>0.4893933582399337</v>
+        <v>0.4907429131497625</v>
       </c>
       <c r="V39" s="4" t="n">
-        <v>0.4924303962356122</v>
+        <v>0.4940937548312492</v>
       </c>
       <c r="W39" s="4" t="n">
         <v>0.06527760268032809</v>
@@ -5382,7 +5382,7 @@
       <c r="AM39" s="2" t="inlineStr"/>
       <c r="AN39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17 ET</t>
+          <t>2026-09-06 10:40 ET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh daily snapshot (2026-09-07)
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -720,7 +720,7 @@
         <v>36.52625570776257</v>
       </c>
       <c r="M2" s="6" t="n">
-        <v>33.57993253578827</v>
+        <v>33.57276292230583</v>
       </c>
       <c r="N2" s="6" t="n">
         <v>10.06701319198068</v>
@@ -744,10 +744,10 @@
         <v>0.06425511782832749</v>
       </c>
       <c r="U2" s="4" t="n">
-        <v>0.0877405923562895</v>
+        <v>0.08797288421842753</v>
       </c>
       <c r="V2" s="4" t="n">
-        <v>0.111542837260457</v>
+        <v>0.1118010928154136</v>
       </c>
       <c r="W2" s="4" t="n">
         <v>0.3363982195133406</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v>27.76111111111111</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>24.46705808745777</v>
+        <v>24.45474101660923</v>
       </c>
       <c r="N3" s="6" t="n">
         <v>11.18176987936921</v>
@@ -872,10 +872,10 @@
         <v>0.1778868679984666</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>0.1346321659056318</v>
+        <v>0.1352036438356166</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>0.2198702922580422</v>
+        <v>0.2204979711079564</v>
       </c>
       <c r="W3" s="4" t="n">
         <v>0.1763623848855976</v>
@@ -930,7 +930,7 @@
       <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v>16.80536246276067</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>20.11391098360043</v>
+        <v>20.13183594513879</v>
       </c>
       <c r="N4" s="6" t="n">
         <v>9.186776742526359</v>
@@ -998,10 +998,10 @@
         <v>0.1509008108154437</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>-0.164490561956714</v>
+        <v>-0.1652344819142714</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0.2909434328511566</v>
+        <v>0.2916458457633306</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0.2648693088701202</v>
@@ -1056,7 +1056,7 @@
       <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v>20.51666666666667</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>22.90522608304126</v>
+        <v>22.91687161883568</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>3.585006601949257</v>
@@ -1124,10 +1124,10 @@
         <v>0.1237775468329469</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>-0.1042801065449011</v>
+        <v>-0.104735279408567</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>0.1742444727587495</v>
+        <v>0.174671084355521</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0.1234666041185044</v>
@@ -1182,7 +1182,7 @@
       <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v>28.97610062893081</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>17.4874487372077</v>
+        <v>17.46427462014875</v>
       </c>
       <c r="N6" s="6" t="n">
         <v>18.41623915318069</v>
@@ -1250,10 +1250,10 @@
         <v>0.6547353579009478</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>0.6569655793917459</v>
+        <v>0.6591642801757556</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>0.9099517112314717</v>
+        <v>0.9124610540515541</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>0.6022349752710197</v>
@@ -1308,7 +1308,7 @@
       <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v>22.91973244147157</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>18.64352331385319</v>
+        <v>18.63971355020581</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>6.883798726731451</v>
@@ -1376,10 +1376,10 @@
         <v>0.2216703849824622</v>
       </c>
       <c r="U7" s="4" t="n">
-        <v>0.2293670062053623</v>
+        <v>0.2296182760393601</v>
       </c>
       <c r="V7" s="4" t="n">
-        <v>0.2662519872362821</v>
+        <v>0.2668661282635136</v>
       </c>
       <c r="W7" s="4" t="n">
         <v>0.1513436869382784</v>
@@ -1434,7 +1434,7 @@
       <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v>300.0677966101695</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>170.3554572187399</v>
+        <v>170.2277758946151</v>
       </c>
       <c r="N8" s="6" t="n">
         <v>13.49613238178326</v>
@@ -1502,10 +1502,10 @@
         <v>-0.02930699150373628</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>0.7614216856280478</v>
+        <v>0.7627428604597173</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>0.1176152580105436</v>
+        <v>0.1179884159689601</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>0.02570628315962403</v>
@@ -1560,7 +1560,7 @@
       <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v>44.40384615384615</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>19.78946536052194</v>
+        <v>19.7664985608273</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>19.10928907905369</v>
@@ -1628,10 +1628,10 @@
         <v>0.2387443285376352</v>
       </c>
       <c r="U9" s="4" t="n">
-        <v>1.243812318569631</v>
+        <v>1.246419416023658</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0.8382949492119105</v>
+        <v>0.8404058525327336</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0.2033771286434084</v>
@@ -1686,7 +1686,7 @@
       <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       <c r="AM10" s="2" t="inlineStr"/>
       <c r="AN10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v>24.22600619195047</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>20.89650710781945</v>
+        <v>20.89321688898327</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6.736058684580629</v>
@@ -1880,10 +1880,10 @@
         <v>0.1585106891967754</v>
       </c>
       <c r="U11" s="4" t="n">
-        <v>0.1593328046142757</v>
+        <v>0.1595153738496122</v>
       </c>
       <c r="V11" s="4" t="n">
-        <v>0.1404772036877822</v>
+        <v>0.1408053902769388</v>
       </c>
       <c r="W11" s="4" t="n">
         <v>0.2335250473131588</v>
@@ -1938,7 +1938,7 @@
       <c r="AM11" s="2" t="inlineStr"/>
       <c r="AN11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v>12.72391249685693</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>22.81187623247644</v>
+        <v>22.81184957963517</v>
       </c>
       <c r="N12" s="6" t="n">
         <v>2.837196538167393</v>
@@ -2006,10 +2006,10 @@
         <v>2.961503151310829e-05</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>-0.4422242007984266</v>
+        <v>-0.4422235491059896</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>0.06024276630376346</v>
+        <v>0.0602881702331135</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>0.06790433791924602</v>
@@ -2064,7 +2064,7 @@
       <c r="AM12" s="2" t="inlineStr"/>
       <c r="AN12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v>15.41874462596733</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>14.32857965729392</v>
+        <v>14.32811161727626</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3.228739643789499</v>
@@ -2132,10 +2132,10 @@
         <v>0.03307372160612143</v>
       </c>
       <c r="U13" s="4" t="n">
-        <v>0.07608325421972029</v>
+        <v>0.0761184053993571</v>
       </c>
       <c r="V13" s="4" t="n">
-        <v>-0.290229911350381</v>
+        <v>-0.2901797650604363</v>
       </c>
       <c r="W13" s="4" t="n">
         <v>0.01297429806050525</v>
@@ -2190,7 +2190,7 @@
       <c r="AM13" s="2" t="inlineStr"/>
       <c r="AN13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v>31.86661002548853</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>25.16527559225406</v>
+        <v>25.15696671340563</v>
       </c>
       <c r="N14" s="6" t="n">
         <v>15.74072553115447</v>
@@ -2258,10 +2258,10 @@
         <v>0.1133997661860491</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>0.2662929086020882</v>
+        <v>0.2667111416301022</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>0.1350755317508432</v>
+        <v>0.1353815979123814</v>
       </c>
       <c r="W14" s="4" t="n">
         <v>0.238841315149593</v>
@@ -2316,7 +2316,7 @@
       <c r="AM14" s="2" t="inlineStr"/>
       <c r="AN14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v>31.80724876441516</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>26.21850789080149</v>
+        <v>26.20833053939909</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>14.47960612148334</v>
@@ -2384,10 +2384,10 @@
         <v>0.164163737707246</v>
       </c>
       <c r="U15" s="4" t="n">
-        <v>0.2131601423273377</v>
+        <v>0.2136312428065266</v>
       </c>
       <c r="V15" s="4" t="n">
-        <v>0.1535211750507113</v>
+        <v>0.1538881007192727</v>
       </c>
       <c r="W15" s="4" t="n">
         <v>0.2817943873394463</v>
@@ -2442,7 +2442,7 @@
       <c r="AM15" s="2" t="inlineStr"/>
       <c r="AN15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v>25.53790753006238</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>18.39159523100312</v>
+        <v>18.38532535066249</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>0.8012380197787745</v>
@@ -2510,10 +2510,10 @@
         <v>0.118140392427263</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>0.3885640266273676</v>
+        <v>0.389037563544784</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>0.009753623419861635</v>
+        <v>0.009832088336138245</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>0.0455949917185134</v>
@@ -2568,7 +2568,7 @@
       <c r="AM16" s="2" t="inlineStr"/>
       <c r="AN16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>20.52252252252253</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>14.44660001081058</v>
+        <v>14.44962064311958</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>1.830376091508336</v>
@@ -2636,10 +2636,10 @@
         <v>-0.04522368657644726</v>
       </c>
       <c r="U17" s="4" t="n">
-        <v>0.4205780257752862</v>
+        <v>0.4202810599248956</v>
       </c>
       <c r="V17" s="4" t="n">
-        <v>0.08360732495351209</v>
+        <v>0.08344588675555009</v>
       </c>
       <c r="W17" s="4" t="n">
         <v>0.07052372320132966</v>
@@ -2694,7 +2694,7 @@
       <c r="AM17" s="2" t="inlineStr"/>
       <c r="AN17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v>31.81849710982659</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>22.18492356152836</v>
+        <v>22.17908938630728</v>
       </c>
       <c r="N18" s="6" t="n">
         <v>6.773032922178313</v>
@@ -2762,10 +2762,10 @@
         <v>0.06048119251078021</v>
       </c>
       <c r="U18" s="4" t="n">
-        <v>0.4342396547628473</v>
+        <v>0.4346169292897299</v>
       </c>
       <c r="V18" s="4" t="n">
-        <v>0.08689613513844319</v>
+        <v>0.08710551767222463</v>
       </c>
       <c r="W18" s="4" t="n">
         <v>0.1046304585695812</v>
@@ -2820,7 +2820,7 @@
       <c r="AM18" s="2" t="inlineStr"/>
       <c r="AN18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v>38.67870036101083</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>34.64601214664498</v>
+        <v>34.63563403511925</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1.158714790171776</v>
@@ -2888,10 +2888,10 @@
         <v>0.04725214211766771</v>
       </c>
       <c r="U19" s="4" t="n">
-        <v>0.1163968943177884</v>
+        <v>0.1167314079422381</v>
       </c>
       <c r="V19" s="4" t="n">
-        <v>0.04982755194757948</v>
+        <v>0.0499518853090346</v>
       </c>
       <c r="W19" s="4" t="n">
         <v>0.07511040644542281</v>
@@ -2946,7 +2946,7 @@
       <c r="AM19" s="2" t="inlineStr"/>
       <c r="AN19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v>21.69333333333333</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>20.75990288145795</v>
+        <v>20.75653946364496</v>
       </c>
       <c r="N20" s="6" t="n">
         <v>3.999617435483501</v>
@@ -3014,10 +3014,10 @@
         <v>0.03260405296378899</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>0.04496314155251135</v>
+        <v>0.0451324687975645</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>0.02463661523029792</v>
+        <v>0.02471642069007518</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>0.1268247958836873</v>
@@ -3072,7 +3072,7 @@
       <c r="AM20" s="2" t="inlineStr"/>
       <c r="AN20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       <c r="AM21" s="2" t="inlineStr"/>
       <c r="AN21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>121.2106598984771</v>
       </c>
       <c r="M22" s="6" t="n">
-        <v>36.05524592963388</v>
+        <v>35.99493291235754</v>
       </c>
       <c r="N22" s="6" t="n">
         <v>18.85305996852681</v>
@@ -3266,10 +3266,10 @@
         <v>0.3433779329067288</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>2.361803720186356</v>
+        <v>2.367436749878312</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>0.8692858552626717</v>
+        <v>0.8717990070367947</v>
       </c>
       <c r="W22" s="4" t="n">
         <v>0.07617446486076908</v>
@@ -3324,7 +3324,7 @@
       <c r="AM22" s="2" t="inlineStr"/>
       <c r="AN22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3365,37 +3365,37 @@
         <v>660945604406</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>53.24383164005805</v>
+        <v>54.44121988388969</v>
       </c>
       <c r="M23" s="6" t="n">
-        <v>35.69713030684876</v>
+        <v>35.66785714956291</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>16.00912490249805</v>
+        <v>16.36915046652042</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>25.91182567100717</v>
+        <v>26.49455073941371</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>3.624502193514434</v>
+        <v>3.706012786996797</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>40.62985693020391</v>
+        <v>41.55120888884059</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>15.87643790228575</v>
+        <v>16.23646346630812</v>
       </c>
       <c r="S23" s="4" t="n">
-        <v>0.01768487563444603</v>
+        <v>0.01729591181265338</v>
       </c>
       <c r="T23" s="4" t="n">
         <v>0.1558368037250246</v>
       </c>
       <c r="U23" s="4" t="n">
-        <v>0.4915437510628919</v>
+        <v>0.5263383963776149</v>
       </c>
       <c r="V23" s="4" t="n">
-        <v>0.2540981173002304</v>
+        <v>0.2831194072907532</v>
       </c>
       <c r="W23" s="4" t="n">
         <v>0.2118578586392856</v>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="AN23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
         <v>79.49438202247188</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>87.14390934812964</v>
+        <v>86.65448504946228</v>
       </c>
       <c r="N24" s="6" t="n">
         <v>1.784733576254056</v>
@@ -3520,10 +3520,10 @@
         <v>0.3449644451794278</v>
       </c>
       <c r="U24" s="4" t="n">
-        <v>-0.08778040121081554</v>
+        <v>-0.08262818736852928</v>
       </c>
       <c r="V24" s="4" t="n">
-        <v>0.1495515262362979</v>
+        <v>0.1499761288207551</v>
       </c>
       <c r="W24" s="4" t="n">
         <v>0.01468017121842407</v>
@@ -3578,7 +3578,7 @@
       <c r="AM24" s="2" t="inlineStr"/>
       <c r="AN24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
         <v>15.82282145033516</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>14.35560827588817</v>
+        <v>14.35392066618628</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>2.597973666194663</v>
@@ -3646,10 +3646,10 @@
         <v>-0.01384279441558334</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0.1022048767457198</v>
+        <v>0.1023344644511786</v>
       </c>
       <c r="V25" s="4" t="n">
-        <v>-0.3826707387247035</v>
+        <v>-0.3826279339206061</v>
       </c>
       <c r="W25" s="4" t="n">
         <v>0.009857071754575692</v>
@@ -3704,7 +3704,7 @@
       <c r="AM25" s="2" t="inlineStr"/>
       <c r="AN25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         <v>20.51441048034935</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>18.23467127810226</v>
+        <v>18.23143074175472</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>3.202712929070727</v>
@@ -3772,10 +3772,10 @@
         <v>0.07621946361130139</v>
       </c>
       <c r="U26" s="4" t="n">
-        <v>0.1250222264760426</v>
+        <v>0.125222192977209</v>
       </c>
       <c r="V26" s="4" t="n">
-        <v>0.04503277258442129</v>
+        <v>0.04514029588184676</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0.07051328411100664</v>
@@ -3830,7 +3830,7 @@
       <c r="AM26" s="2" t="inlineStr"/>
       <c r="AN26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 10:40 ET</t>
+          <t>2026-09-07 12:55 ET</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
         <v>38.46566164154105</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>26.46657266718929</v>
+        <v>26.44946248474263</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>13.57303907322841</v>
@@ -3898,10 +3898,10 @@
         <v>0.44704913337788